<commit_message>
Inclui e formata o Patrimonio Liquido das empresas
</commit_message>
<xml_diff>
--- a/acoes_b3.xlsx
+++ b/acoes_b3.xlsx
@@ -461,21 +461,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MNSA3</t>
+          <t>PORP4</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Empresa MNSA</t>
+          <t>Empresa PORP</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.42</v>
+        <v>2.4</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -486,30 +486,30 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>-13.5</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>145.7</v>
+        <v>-2.08</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CFLU4</t>
+          <t>IVTT3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Empresa CFLU</t>
+          <t>Empresa IVTT</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -520,21 +520,21 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>17.68</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>32.15</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CSTB3</t>
+          <t>MNSA3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa MNSA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>150</v>
+        <v>0.42</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -554,21 +554,21 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>22.4</v>
+        <v>-13.5</v>
       </c>
       <c r="H4" t="n">
-        <v>20.11</v>
+        <v>145.7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>POPR4</t>
+          <t>CFLU4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Empresa POPR</t>
+          <t>Empresa CFLU</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>10.17</v>
+        <v>1000</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -588,21 +588,21 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>15.25</v>
+        <v>17.68</v>
       </c>
       <c r="H5" t="n">
-        <v>19.93</v>
+        <v>32.15</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PMET3</t>
+          <t>CSTB3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Empresa PMET</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -622,30 +622,30 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>22.4</v>
       </c>
       <c r="H6" t="n">
-        <v>4.1</v>
+        <v>20.11</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CLAN3</t>
+          <t>POPR4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Empresa CLAN</t>
+          <t>Empresa POPR</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>10.17</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -656,30 +656,30 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>15.25</v>
       </c>
       <c r="H7" t="n">
-        <v>-1.05</v>
+        <v>19.93</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MNSA4</t>
+          <t>PMET3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Empresa MNSA</t>
+          <t>Empresa PMET</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.47</v>
+        <v>0</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -690,30 +690,30 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>-13.5</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>145.7</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CSTB4</t>
+          <t>CLAN3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa CLAN</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>147.69</v>
+        <v>0</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -724,21 +724,21 @@
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>22.4</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>20.11</v>
+        <v>-1.05</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PORP4</t>
+          <t>MNSA4</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Empresa PORP</t>
+          <t>Empresa MNSA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2.4</v>
+        <v>0.47</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -758,30 +758,30 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>-13.5</v>
       </c>
       <c r="H10" t="n">
-        <v>-2.08</v>
+        <v>145.7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>IVTT3</t>
+          <t>CSTB4</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Empresa IVTT</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>147.69</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -792,10 +792,10 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>22.4</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.4</v>
+        <v>20.11</v>
       </c>
     </row>
     <row r="12">
@@ -5459,7 +5459,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>PNOR5</t>
+          <t>PNOR6</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -5493,7 +5493,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>PNOR6</t>
+          <t>PNOR5</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -5935,7 +5935,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>RNEW4</t>
+          <t>RNEW3</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -5945,7 +5945,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -5957,7 +5957,7 @@
         </is>
       </c>
       <c r="F163" t="n">
-        <v>44097</v>
+        <v>45273.4</v>
       </c>
       <c r="G163" t="n">
         <v>-0.52</v>
@@ -5969,7 +5969,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>RNEW3</t>
+          <t>RNEW4</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -5979,7 +5979,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -5991,7 +5991,7 @@
         </is>
       </c>
       <c r="F164" t="n">
-        <v>45273.4</v>
+        <v>44097</v>
       </c>
       <c r="G164" t="n">
         <v>-0.52</v>
@@ -6751,7 +6751,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>SDIA3</t>
+          <t>SDIA4</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -6761,7 +6761,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -6785,7 +6785,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>SDIA4</t>
+          <t>SDIA3</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -6795,7 +6795,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -10899,12 +10899,12 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>REPA4</t>
+          <t>CCHI4</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -10913,7 +10913,7 @@
         </is>
       </c>
       <c r="D309" t="n">
-        <v>1.08</v>
+        <v>0.02</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -10924,30 +10924,30 @@
         <v>0</v>
       </c>
       <c r="G309" t="n">
-        <v>4.05</v>
+        <v>0</v>
       </c>
       <c r="H309" t="n">
-        <v>1.91</v>
+        <v>0</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>EQMA6B</t>
+          <t>REPA3</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -10958,21 +10958,21 @@
         <v>0</v>
       </c>
       <c r="G310" t="n">
-        <v>0</v>
+        <v>4.05</v>
       </c>
       <c r="H310" t="n">
-        <v>0</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>SEBB4</t>
+          <t>EQMA5B</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -10992,21 +10992,21 @@
         <v>0</v>
       </c>
       <c r="G311" t="n">
-        <v>24.15</v>
+        <v>0</v>
       </c>
       <c r="H311" t="n">
-        <v>23.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>MSAN3</t>
+          <t>SEBB3</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -11015,7 +11015,7 @@
         </is>
       </c>
       <c r="D312" t="n">
-        <v>6.44</v>
+        <v>0</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -11026,30 +11026,30 @@
         <v>0</v>
       </c>
       <c r="G312" t="n">
-        <v>11.78</v>
+        <v>24.15</v>
       </c>
       <c r="H312" t="n">
-        <v>11.81</v>
+        <v>23.01</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>GALO3</t>
+          <t>BBTG11</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>0</v>
+        <v>15.01</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -11060,30 +11060,30 @@
         <v>0</v>
       </c>
       <c r="G313" t="n">
-        <v>39.37</v>
+        <v>0</v>
       </c>
       <c r="H313" t="n">
-        <v>7.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>SLCP3</t>
+          <t>JFAB4</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Empresa SLCP</t>
+          <t>Empresa JFAB</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>610.02</v>
+        <v>0.06</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -11097,18 +11097,18 @@
         <v>0</v>
       </c>
       <c r="H314" t="n">
-        <v>0</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>DAYC3</t>
+          <t>LECO3</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Empresa DAYC</t>
+          <t>Empresa LECO</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -11128,21 +11128,21 @@
         <v>0</v>
       </c>
       <c r="G315" t="n">
-        <v>0</v>
+        <v>-3.48</v>
       </c>
       <c r="H315" t="n">
-        <v>17.33</v>
+        <v>-14.82</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>PTIP3</t>
+          <t>VGOR3</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa VGOR</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -11151,7 +11151,7 @@
         </is>
       </c>
       <c r="D316" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -11162,21 +11162,21 @@
         <v>0</v>
       </c>
       <c r="G316" t="n">
-        <v>23.13</v>
+        <v>6</v>
       </c>
       <c r="H316" t="n">
-        <v>-121.74</v>
+        <v>-24.29</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>MLPA3</t>
+          <t>GPIV33</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Empresa MLPA</t>
+          <t>Empresa GPIV</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -11185,7 +11185,7 @@
         </is>
       </c>
       <c r="D317" t="n">
-        <v>0</v>
+        <v>4.42</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -11196,21 +11196,21 @@
         <v>0</v>
       </c>
       <c r="G317" t="n">
-        <v>0</v>
+        <v>-6.05</v>
       </c>
       <c r="H317" t="n">
-        <v>45.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>CLSC6</t>
+          <t>ECIS4</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Empresa CLSC</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -11219,7 +11219,7 @@
         </is>
       </c>
       <c r="D318" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -11230,21 +11230,21 @@
         <v>0</v>
       </c>
       <c r="G318" t="n">
-        <v>0</v>
+        <v>12.48</v>
       </c>
       <c r="H318" t="n">
-        <v>0</v>
+        <v>7.33</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>SGEN3</t>
+          <t>TNEP3</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -11253,7 +11253,7 @@
         </is>
       </c>
       <c r="D319" t="n">
-        <v>5</v>
+        <v>3.01</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -11264,21 +11264,21 @@
         <v>0</v>
       </c>
       <c r="G319" t="n">
-        <v>-1.59</v>
+        <v>20.53</v>
       </c>
       <c r="H319" t="n">
-        <v>0</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>DUFB11</t>
+          <t>CBMA4</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Empresa DUFB</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -11287,7 +11287,7 @@
         </is>
       </c>
       <c r="D320" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -11307,12 +11307,12 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>TNEP4</t>
+          <t>SALM4</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -11321,7 +11321,7 @@
         </is>
       </c>
       <c r="D321" t="n">
-        <v>3.95</v>
+        <v>5.9</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -11332,21 +11332,21 @@
         <v>0</v>
       </c>
       <c r="G321" t="n">
-        <v>20.53</v>
+        <v>25.78</v>
       </c>
       <c r="H321" t="n">
-        <v>22.8</v>
+        <v>19.53</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>CCHI3</t>
+          <t>BERG3</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa BERG</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -11355,7 +11355,7 @@
         </is>
       </c>
       <c r="D322" t="n">
-        <v>0.02</v>
+        <v>33</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -11366,21 +11366,21 @@
         <v>0</v>
       </c>
       <c r="G322" t="n">
-        <v>0</v>
+        <v>-5.58</v>
       </c>
       <c r="H322" t="n">
-        <v>0</v>
+        <v>-102.71</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>SFSA3</t>
+          <t>JBDU3</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Empresa SFSA</t>
+          <t>Empresa JBDU</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -11403,18 +11403,18 @@
         <v>0</v>
       </c>
       <c r="H323" t="n">
-        <v>6.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>PRBC3</t>
+          <t>EGGY3</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Empresa PRBC</t>
+          <t>Empresa EGGY</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -11437,18 +11437,18 @@
         <v>0</v>
       </c>
       <c r="H324" t="n">
-        <v>8.27</v>
+        <v>0</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>ECIS3</t>
+          <t>AGEI3</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa AGEI</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -11457,7 +11457,7 @@
         </is>
       </c>
       <c r="D325" t="n">
-        <v>211.65</v>
+        <v>7.8</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -11468,21 +11468,21 @@
         <v>0</v>
       </c>
       <c r="G325" t="n">
-        <v>12.48</v>
+        <v>0</v>
       </c>
       <c r="H325" t="n">
-        <v>7.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>CBMA3</t>
+          <t>SASG3</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa SASG</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -11491,7 +11491,7 @@
         </is>
       </c>
       <c r="D326" t="n">
-        <v>0.01</v>
+        <v>0.98</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -11511,12 +11511,12 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>ALBA3</t>
+          <t>BMEF3</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Empresa ALBA</t>
+          <t>Empresa BMEF</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -11525,7 +11525,7 @@
         </is>
       </c>
       <c r="D327" t="n">
-        <v>2.15</v>
+        <v>11</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -11536,16 +11536,16 @@
         <v>0</v>
       </c>
       <c r="G327" t="n">
-        <v>20.4</v>
+        <v>0</v>
       </c>
       <c r="H327" t="n">
-        <v>19.77</v>
+        <v>0</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>ARPS4</t>
+          <t>ARPS3</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
@@ -11555,11 +11555,11 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -11579,12 +11579,12 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>SALM3</t>
+          <t>ODER3</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa ODER</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -11593,7 +11593,7 @@
         </is>
       </c>
       <c r="D329" t="n">
-        <v>5.7</v>
+        <v>0</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -11604,30 +11604,30 @@
         <v>0</v>
       </c>
       <c r="G329" t="n">
-        <v>25.78</v>
+        <v>0</v>
       </c>
       <c r="H329" t="n">
-        <v>19.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>CMMA4</t>
+          <t>CCTY3</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Empresa CMMA</t>
+          <t>Empresa CCTY</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>0.8100000000000001</v>
+        <v>0</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -11641,23 +11641,23 @@
         <v>0</v>
       </c>
       <c r="H330" t="n">
-        <v>-1.92</v>
+        <v>0</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>CZRS3</t>
+          <t>VVAX4</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Empresa CZRS</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D331" t="n">
@@ -11672,21 +11672,21 @@
         <v>0</v>
       </c>
       <c r="G331" t="n">
-        <v>0</v>
+        <v>-6.52</v>
       </c>
       <c r="H331" t="n">
-        <v>3.34</v>
+        <v>-92.03</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>BPNM3</t>
+          <t>CSPC3</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Empresa BPNM</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -11695,7 +11695,7 @@
         </is>
       </c>
       <c r="D332" t="n">
-        <v>0</v>
+        <v>1.24</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -11706,21 +11706,21 @@
         <v>0</v>
       </c>
       <c r="G332" t="n">
-        <v>0</v>
+        <v>29.18</v>
       </c>
       <c r="H332" t="n">
-        <v>9.67</v>
+        <v>45.33</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>BSGR3</t>
+          <t>ABCB3</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Empresa BSGR</t>
+          <t>Empresa ABCB</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -11729,11 +11729,11 @@
         </is>
       </c>
       <c r="D333" t="n">
-        <v>1091.28</v>
+        <v>0</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="F333" t="n">
@@ -11743,23 +11743,23 @@
         <v>0</v>
       </c>
       <c r="H333" t="n">
-        <v>0</v>
+        <v>14.05</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>VNET3</t>
+          <t>ESTC4</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Empresa VNET</t>
+          <t>Empresa ESTC</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D334" t="n">
@@ -11774,21 +11774,21 @@
         <v>0</v>
       </c>
       <c r="G334" t="n">
-        <v>0</v>
+        <v>11.35</v>
       </c>
       <c r="H334" t="n">
-        <v>0</v>
+        <v>3.89</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>CSPC4</t>
+          <t>VSPT4</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -11797,7 +11797,7 @@
         </is>
       </c>
       <c r="D335" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -11808,30 +11808,30 @@
         <v>0</v>
       </c>
       <c r="G335" t="n">
-        <v>29.18</v>
+        <v>0</v>
       </c>
       <c r="H335" t="n">
-        <v>45.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>BOVH3</t>
+          <t>BAUH4</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Empresa BOVH</t>
+          <t>Empresa BAUH</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>15.71</v>
+        <v>93.39</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -11839,7 +11839,7 @@
         </is>
       </c>
       <c r="F336" t="n">
-        <v>0</v>
+        <v>207.53</v>
       </c>
       <c r="G336" t="n">
         <v>0</v>
@@ -11851,12 +11851,12 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>ARND3</t>
+          <t>ICPI3</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Empresa ARND</t>
+          <t>Empresa ICPI</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -11865,7 +11865,7 @@
         </is>
       </c>
       <c r="D337" t="n">
-        <v>0.51</v>
+        <v>0</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -11873,7 +11873,7 @@
         </is>
       </c>
       <c r="F337" t="n">
-        <v>913.58</v>
+        <v>0</v>
       </c>
       <c r="G337" t="n">
         <v>0</v>
@@ -11885,21 +11885,21 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>VVAX3</t>
+          <t>ILLS4</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa ILLS</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>0</v>
+        <v>100.01</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -11910,30 +11910,30 @@
         <v>0</v>
       </c>
       <c r="G338" t="n">
-        <v>-6.52</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="H338" t="n">
-        <v>-92.03</v>
+        <v>36.09</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>MSAN4</t>
+          <t>BPAT33</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa BPAT</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>6.44</v>
+        <v>20</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -11944,21 +11944,21 @@
         <v>0</v>
       </c>
       <c r="G339" t="n">
-        <v>11.78</v>
+        <v>0</v>
       </c>
       <c r="H339" t="n">
-        <v>11.81</v>
+        <v>0</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>GALO4</t>
+          <t>REPA4</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -11967,7 +11967,7 @@
         </is>
       </c>
       <c r="D340" t="n">
-        <v>0.25</v>
+        <v>1.08</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -11978,26 +11978,26 @@
         <v>0</v>
       </c>
       <c r="G340" t="n">
-        <v>39.37</v>
+        <v>4.05</v>
       </c>
       <c r="H340" t="n">
-        <v>7.62</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>BBTG13</t>
+          <t>EQMA6B</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D341" t="n">
@@ -12015,23 +12015,23 @@
         <v>0</v>
       </c>
       <c r="H341" t="n">
-        <v>-42.86</v>
+        <v>0</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>INHA3</t>
+          <t>SEBB4</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Empresa INHA</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D342" t="n">
@@ -12046,30 +12046,30 @@
         <v>0</v>
       </c>
       <c r="G342" t="n">
-        <v>-6.27</v>
+        <v>24.15</v>
       </c>
       <c r="H342" t="n">
-        <v>-39.87</v>
+        <v>23.01</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>PTIP4</t>
+          <t>MSAN3</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>25.15</v>
+        <v>6.44</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -12080,21 +12080,21 @@
         <v>0</v>
       </c>
       <c r="G343" t="n">
-        <v>23.13</v>
+        <v>11.78</v>
       </c>
       <c r="H343" t="n">
-        <v>-121.74</v>
+        <v>11.81</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>LATS3</t>
+          <t>GALO3</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Empresa LATS</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
@@ -12103,7 +12103,7 @@
         </is>
       </c>
       <c r="D344" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -12114,21 +12114,21 @@
         <v>0</v>
       </c>
       <c r="G344" t="n">
-        <v>11.63</v>
+        <v>39.37</v>
       </c>
       <c r="H344" t="n">
-        <v>1.84</v>
+        <v>7.62</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>VSPT3</t>
+          <t>SLCP3</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa SLCP</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -12137,7 +12137,7 @@
         </is>
       </c>
       <c r="D345" t="n">
-        <v>0</v>
+        <v>610.02</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -12157,21 +12157,21 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>SGEN4</t>
+          <t>DAYC3</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa DAYC</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -12182,30 +12182,30 @@
         <v>0</v>
       </c>
       <c r="G346" t="n">
-        <v>-1.59</v>
+        <v>0</v>
       </c>
       <c r="H346" t="n">
-        <v>0</v>
+        <v>17.33</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>CCHI4</t>
+          <t>PTIP3</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>0.02</v>
+        <v>22</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -12216,21 +12216,21 @@
         <v>0</v>
       </c>
       <c r="G347" t="n">
-        <v>0</v>
+        <v>23.13</v>
       </c>
       <c r="H347" t="n">
-        <v>0</v>
+        <v>-121.74</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>REPA3</t>
+          <t>MLPA3</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa MLPA</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
@@ -12239,7 +12239,7 @@
         </is>
       </c>
       <c r="D348" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -12250,21 +12250,21 @@
         <v>0</v>
       </c>
       <c r="G348" t="n">
-        <v>4.05</v>
+        <v>0</v>
       </c>
       <c r="H348" t="n">
-        <v>1.91</v>
+        <v>45.13</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>EQMA5B</t>
+          <t>CLSC6</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa CLSC</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
@@ -12293,12 +12293,12 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>SEBB3</t>
+          <t>SGEN3</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
@@ -12307,7 +12307,7 @@
         </is>
       </c>
       <c r="D350" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -12318,21 +12318,21 @@
         <v>0</v>
       </c>
       <c r="G350" t="n">
-        <v>24.15</v>
+        <v>-1.59</v>
       </c>
       <c r="H350" t="n">
-        <v>23.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>BBTG11</t>
+          <t>DUFB11</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa DUFB</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -12341,7 +12341,7 @@
         </is>
       </c>
       <c r="D351" t="n">
-        <v>15.01</v>
+        <v>0</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -12361,12 +12361,12 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>JFAB4</t>
+          <t>TNEP4</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Empresa JFAB</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -12375,7 +12375,7 @@
         </is>
       </c>
       <c r="D352" t="n">
-        <v>0.06</v>
+        <v>3.95</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -12386,21 +12386,21 @@
         <v>0</v>
       </c>
       <c r="G352" t="n">
-        <v>0</v>
+        <v>20.53</v>
       </c>
       <c r="H352" t="n">
-        <v>2.34</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>VGOR3</t>
+          <t>CCHI3</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Empresa VGOR</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -12409,7 +12409,7 @@
         </is>
       </c>
       <c r="D353" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -12420,21 +12420,21 @@
         <v>0</v>
       </c>
       <c r="G353" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H353" t="n">
-        <v>-24.29</v>
+        <v>0</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>GPIV33</t>
+          <t>SFSA3</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Empresa GPIV</t>
+          <t>Empresa SFSA</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -12443,7 +12443,7 @@
         </is>
       </c>
       <c r="D354" t="n">
-        <v>4.42</v>
+        <v>0</v>
       </c>
       <c r="E354" t="inlineStr">
         <is>
@@ -12454,30 +12454,30 @@
         <v>0</v>
       </c>
       <c r="G354" t="n">
-        <v>-6.05</v>
+        <v>0</v>
       </c>
       <c r="H354" t="n">
-        <v>0</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>ECIS4</t>
+          <t>PRBC3</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa PRBC</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>145</v>
+        <v>0</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -12488,21 +12488,21 @@
         <v>0</v>
       </c>
       <c r="G355" t="n">
-        <v>12.48</v>
+        <v>0</v>
       </c>
       <c r="H355" t="n">
-        <v>7.33</v>
+        <v>8.27</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>TNEP3</t>
+          <t>ECIS3</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -12511,7 +12511,7 @@
         </is>
       </c>
       <c r="D356" t="n">
-        <v>3.01</v>
+        <v>211.65</v>
       </c>
       <c r="E356" t="inlineStr">
         <is>
@@ -12522,21 +12522,21 @@
         <v>0</v>
       </c>
       <c r="G356" t="n">
-        <v>20.53</v>
+        <v>12.48</v>
       </c>
       <c r="H356" t="n">
-        <v>22.8</v>
+        <v>7.33</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>LECO3</t>
+          <t>CBMA3</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Empresa LECO</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -12545,7 +12545,7 @@
         </is>
       </c>
       <c r="D357" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -12556,30 +12556,30 @@
         <v>0</v>
       </c>
       <c r="G357" t="n">
-        <v>-3.48</v>
+        <v>0</v>
       </c>
       <c r="H357" t="n">
-        <v>-14.82</v>
+        <v>0</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>CBMA4</t>
+          <t>ALBA3</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa ALBA</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D358" t="n">
-        <v>0.01</v>
+        <v>2.15</v>
       </c>
       <c r="E358" t="inlineStr">
         <is>
@@ -12590,21 +12590,21 @@
         <v>0</v>
       </c>
       <c r="G358" t="n">
-        <v>0</v>
+        <v>20.4</v>
       </c>
       <c r="H358" t="n">
-        <v>0</v>
+        <v>19.77</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>SALM4</t>
+          <t>ARPS4</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
@@ -12613,7 +12613,7 @@
         </is>
       </c>
       <c r="D359" t="n">
-        <v>5.9</v>
+        <v>0</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -12624,21 +12624,21 @@
         <v>0</v>
       </c>
       <c r="G359" t="n">
-        <v>25.78</v>
+        <v>-6.64</v>
       </c>
       <c r="H359" t="n">
-        <v>19.53</v>
+        <v>20.34</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>BERG3</t>
+          <t>SALM3</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Empresa BERG</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
@@ -12647,7 +12647,7 @@
         </is>
       </c>
       <c r="D360" t="n">
-        <v>33</v>
+        <v>5.7</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -12658,30 +12658,30 @@
         <v>0</v>
       </c>
       <c r="G360" t="n">
-        <v>-5.58</v>
+        <v>25.78</v>
       </c>
       <c r="H360" t="n">
-        <v>-102.71</v>
+        <v>19.53</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>JBDU3</t>
+          <t>CMMA4</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Empresa JBDU</t>
+          <t>Empresa CMMA</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D361" t="n">
-        <v>0</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -12695,18 +12695,18 @@
         <v>0</v>
       </c>
       <c r="H361" t="n">
-        <v>0</v>
+        <v>-1.92</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>EGGY3</t>
+          <t>CZRS3</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>Empresa EGGY</t>
+          <t>Empresa CZRS</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -12729,18 +12729,18 @@
         <v>0</v>
       </c>
       <c r="H362" t="n">
-        <v>0</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>AGEI3</t>
+          <t>BPNM3</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Empresa AGEI</t>
+          <t>Empresa BPNM</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -12749,7 +12749,7 @@
         </is>
       </c>
       <c r="D363" t="n">
-        <v>7.8</v>
+        <v>0</v>
       </c>
       <c r="E363" t="inlineStr">
         <is>
@@ -12763,18 +12763,18 @@
         <v>0</v>
       </c>
       <c r="H363" t="n">
-        <v>0</v>
+        <v>9.67</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>SASG3</t>
+          <t>BSGR3</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Empresa SASG</t>
+          <t>Empresa BSGR</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -12783,7 +12783,7 @@
         </is>
       </c>
       <c r="D364" t="n">
-        <v>0.98</v>
+        <v>1091.28</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -12803,12 +12803,12 @@
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>BMEF3</t>
+          <t>VNET3</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Empresa BMEF</t>
+          <t>Empresa VNET</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
@@ -12817,7 +12817,7 @@
         </is>
       </c>
       <c r="D365" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="E365" t="inlineStr">
         <is>
@@ -12837,21 +12837,21 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>ARPS3</t>
+          <t>CSPC4</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D366" t="n">
-        <v>0.3</v>
+        <v>1.2</v>
       </c>
       <c r="E366" t="inlineStr">
         <is>
@@ -12862,21 +12862,21 @@
         <v>0</v>
       </c>
       <c r="G366" t="n">
-        <v>-6.64</v>
+        <v>29.18</v>
       </c>
       <c r="H366" t="n">
-        <v>20.34</v>
+        <v>45.33</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>ODER3</t>
+          <t>BOVH3</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Empresa ODER</t>
+          <t>Empresa BOVH</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -12885,7 +12885,7 @@
         </is>
       </c>
       <c r="D367" t="n">
-        <v>0</v>
+        <v>15.71</v>
       </c>
       <c r="E367" t="inlineStr">
         <is>
@@ -12905,12 +12905,12 @@
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>CCTY3</t>
+          <t>ARND3</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Empresa CCTY</t>
+          <t>Empresa ARND</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -12919,7 +12919,7 @@
         </is>
       </c>
       <c r="D368" t="n">
-        <v>0</v>
+        <v>0.51</v>
       </c>
       <c r="E368" t="inlineStr">
         <is>
@@ -12927,7 +12927,7 @@
         </is>
       </c>
       <c r="F368" t="n">
-        <v>0</v>
+        <v>913.58</v>
       </c>
       <c r="G368" t="n">
         <v>0</v>
@@ -12939,7 +12939,7 @@
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>VVAX4</t>
+          <t>VVAX3</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
@@ -12949,7 +12949,7 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D369" t="n">
@@ -12973,21 +12973,21 @@
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>CSPC3</t>
+          <t>MSAN4</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D370" t="n">
-        <v>1.24</v>
+        <v>6.44</v>
       </c>
       <c r="E370" t="inlineStr">
         <is>
@@ -12998,60 +12998,60 @@
         <v>0</v>
       </c>
       <c r="G370" t="n">
-        <v>29.18</v>
+        <v>11.78</v>
       </c>
       <c r="H370" t="n">
-        <v>45.33</v>
+        <v>11.81</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>ABCB3</t>
+          <t>GALO4</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Empresa ABCB</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D371" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t>Bancos</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="F371" t="n">
         <v>0</v>
       </c>
       <c r="G371" t="n">
-        <v>0</v>
+        <v>39.37</v>
       </c>
       <c r="H371" t="n">
-        <v>14.05</v>
+        <v>7.62</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>ESTC4</t>
+          <t>BBTG13</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Empresa ESTC</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D372" t="n">
@@ -13066,26 +13066,26 @@
         <v>0</v>
       </c>
       <c r="G372" t="n">
-        <v>11.35</v>
+        <v>0</v>
       </c>
       <c r="H372" t="n">
-        <v>3.89</v>
+        <v>-42.86</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>VSPT4</t>
+          <t>INHA3</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa INHA</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D373" t="n">
@@ -13100,21 +13100,21 @@
         <v>0</v>
       </c>
       <c r="G373" t="n">
-        <v>0</v>
+        <v>-6.27</v>
       </c>
       <c r="H373" t="n">
-        <v>0</v>
+        <v>-39.87</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>BAUH4</t>
+          <t>PTIP4</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>Empresa BAUH</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
@@ -13123,7 +13123,7 @@
         </is>
       </c>
       <c r="D374" t="n">
-        <v>93.39</v>
+        <v>25.15</v>
       </c>
       <c r="E374" t="inlineStr">
         <is>
@@ -13131,24 +13131,24 @@
         </is>
       </c>
       <c r="F374" t="n">
-        <v>207.53</v>
+        <v>0</v>
       </c>
       <c r="G374" t="n">
-        <v>0</v>
+        <v>23.13</v>
       </c>
       <c r="H374" t="n">
-        <v>0</v>
+        <v>-121.74</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>ICPI3</t>
+          <t>LATS3</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>Empresa ICPI</t>
+          <t>Empresa LATS</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
@@ -13157,7 +13157,7 @@
         </is>
       </c>
       <c r="D375" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="E375" t="inlineStr">
         <is>
@@ -13168,30 +13168,30 @@
         <v>0</v>
       </c>
       <c r="G375" t="n">
-        <v>0</v>
+        <v>11.63</v>
       </c>
       <c r="H375" t="n">
-        <v>0</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>ILLS4</t>
+          <t>VSPT3</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>Empresa ILLS</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D376" t="n">
-        <v>100.01</v>
+        <v>0</v>
       </c>
       <c r="E376" t="inlineStr">
         <is>
@@ -13202,30 +13202,30 @@
         <v>0</v>
       </c>
       <c r="G376" t="n">
-        <v>8.140000000000001</v>
+        <v>0</v>
       </c>
       <c r="H376" t="n">
-        <v>36.09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>BPAT33</t>
+          <t>SGEN4</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>Empresa BPAT</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D377" t="n">
-        <v>20</v>
+        <v>0.6</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -13236,7 +13236,7 @@
         <v>0</v>
       </c>
       <c r="G377" t="n">
-        <v>0</v>
+        <v>-1.59</v>
       </c>
       <c r="H377" t="n">
         <v>0</v>
@@ -15421,7 +15421,7 @@
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>MMAQ4</t>
+          <t>MMAQ3</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
@@ -15431,7 +15431,7 @@
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D442" t="n">
@@ -15455,7 +15455,7 @@
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>MMAQ3</t>
+          <t>MMAQ4</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
@@ -15465,7 +15465,7 @@
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D443" t="n">
@@ -19535,7 +19535,7 @@
     <row r="563">
       <c r="A563" t="inlineStr">
         <is>
-          <t>CIQU4</t>
+          <t>CIQU3</t>
         </is>
       </c>
       <c r="B563" t="inlineStr">
@@ -19545,7 +19545,7 @@
       </c>
       <c r="C563" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D563" t="n">
@@ -19569,7 +19569,7 @@
     <row r="564">
       <c r="A564" t="inlineStr">
         <is>
-          <t>CIQU3</t>
+          <t>CIQU4</t>
         </is>
       </c>
       <c r="B564" t="inlineStr">
@@ -19579,7 +19579,7 @@
       </c>
       <c r="C564" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D564" t="n">
@@ -20521,7 +20521,7 @@
     <row r="592">
       <c r="A592" t="inlineStr">
         <is>
-          <t>GETT4</t>
+          <t>GETT3</t>
         </is>
       </c>
       <c r="B592" t="inlineStr">
@@ -20531,7 +20531,7 @@
       </c>
       <c r="C592" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D592" t="n">
@@ -20555,7 +20555,7 @@
     <row r="593">
       <c r="A593" t="inlineStr">
         <is>
-          <t>GETT3</t>
+          <t>GETT4</t>
         </is>
       </c>
       <c r="B593" t="inlineStr">
@@ -20565,7 +20565,7 @@
       </c>
       <c r="C593" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D593" t="n">
@@ -21439,7 +21439,7 @@
     <row r="619">
       <c r="A619" t="inlineStr">
         <is>
-          <t>AESL4</t>
+          <t>AESL3</t>
         </is>
       </c>
       <c r="B619" t="inlineStr">
@@ -21449,7 +21449,7 @@
       </c>
       <c r="C619" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D619" t="n">
@@ -21473,7 +21473,7 @@
     <row r="620">
       <c r="A620" t="inlineStr">
         <is>
-          <t>AESL3</t>
+          <t>AESL4</t>
         </is>
       </c>
       <c r="B620" t="inlineStr">
@@ -21483,7 +21483,7 @@
       </c>
       <c r="C620" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D620" t="n">
@@ -29769,7 +29769,7 @@
     <row r="864">
       <c r="A864" t="inlineStr">
         <is>
-          <t>RSIP3</t>
+          <t>RSIP4</t>
         </is>
       </c>
       <c r="B864" t="inlineStr">
@@ -29779,7 +29779,7 @@
       </c>
       <c r="C864" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D864" t="n">
@@ -29803,7 +29803,7 @@
     <row r="865">
       <c r="A865" t="inlineStr">
         <is>
-          <t>RSIP4</t>
+          <t>RSIP3</t>
         </is>
       </c>
       <c r="B865" t="inlineStr">
@@ -29813,7 +29813,7 @@
       </c>
       <c r="C865" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D865" t="n">
@@ -31163,7 +31163,7 @@
     <row r="905">
       <c r="A905" t="inlineStr">
         <is>
-          <t>BRGE5</t>
+          <t>BRGE11</t>
         </is>
       </c>
       <c r="B905" t="inlineStr">
@@ -31197,7 +31197,7 @@
     <row r="906">
       <c r="A906" t="inlineStr">
         <is>
-          <t>BRGE11</t>
+          <t>BRGE5</t>
         </is>
       </c>
       <c r="B906" t="inlineStr">
@@ -33475,7 +33475,7 @@
     <row r="973">
       <c r="A973" t="inlineStr">
         <is>
-          <t>PQUN3</t>
+          <t>PQUN4</t>
         </is>
       </c>
       <c r="B973" t="inlineStr">
@@ -33485,7 +33485,7 @@
       </c>
       <c r="C973" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D973" t="n">
@@ -33509,7 +33509,7 @@
     <row r="974">
       <c r="A974" t="inlineStr">
         <is>
-          <t>PQUN4</t>
+          <t>PQUN3</t>
         </is>
       </c>
       <c r="B974" t="inlineStr">
@@ -33519,7 +33519,7 @@
       </c>
       <c r="C974" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D974" t="n">

</xml_diff>

<commit_message>
Corrige Mapeamento e Chave de Patrimonio Liquido
</commit_message>
<xml_diff>
--- a/acoes_b3.xlsx
+++ b/acoes_b3.xlsx
@@ -461,21 +461,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PORP4</t>
+          <t>CLAN3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Empresa PORP</t>
+          <t>Empresa CLAN</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2.4</v>
+        <v>0</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -489,27 +489,27 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>-2.08</v>
+        <v>-1.05</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>IVTT3</t>
+          <t>MNSA4</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Empresa IVTT</t>
+          <t>Empresa MNSA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>0.47</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -520,30 +520,30 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>-13.5</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.4</v>
+        <v>145.7</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MNSA3</t>
+          <t>CSTB4</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Empresa MNSA</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.42</v>
+        <v>147.69</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -554,21 +554,21 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>-13.5</v>
+        <v>22.4</v>
       </c>
       <c r="H4" t="n">
-        <v>145.7</v>
+        <v>20.11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CFLU4</t>
+          <t>PORP4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Empresa CFLU</t>
+          <t>Empresa PORP</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1000</v>
+        <v>2.4</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -588,21 +588,21 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>17.68</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>32.15</v>
+        <v>-2.08</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CSTB3</t>
+          <t>IVTT3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa IVTT</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -622,30 +622,30 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>22.4</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>20.11</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>POPR4</t>
+          <t>MNSA3</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Empresa POPR</t>
+          <t>Empresa MNSA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>10.17</v>
+        <v>0.42</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -656,21 +656,21 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>15.25</v>
+        <v>-13.5</v>
       </c>
       <c r="H7" t="n">
-        <v>19.93</v>
+        <v>145.7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PMET3</t>
+          <t>CSTB3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Empresa PMET</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -690,30 +690,30 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>22.4</v>
       </c>
       <c r="H8" t="n">
-        <v>4.1</v>
+        <v>20.11</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CLAN3</t>
+          <t>CFLU4</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Empresa CLAN</t>
+          <t>Empresa CFLU</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -724,21 +724,21 @@
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>17.68</v>
       </c>
       <c r="H9" t="n">
-        <v>-1.05</v>
+        <v>32.15</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MNSA4</t>
+          <t>POPR4</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Empresa MNSA</t>
+          <t>Empresa POPR</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.47</v>
+        <v>10.17</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -758,30 +758,30 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>-13.5</v>
+        <v>15.25</v>
       </c>
       <c r="H10" t="n">
-        <v>145.7</v>
+        <v>19.93</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CSTB4</t>
+          <t>PMET3</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa PMET</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>147.69</v>
+        <v>0</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -792,10 +792,10 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>22.4</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>20.11</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="12">
@@ -5459,7 +5459,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>PNOR6</t>
+          <t>PNOR5</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -5493,7 +5493,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>PNOR5</t>
+          <t>PNOR6</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -10899,12 +10899,12 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>CCHI4</t>
+          <t>CSPC4</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -10913,7 +10913,7 @@
         </is>
       </c>
       <c r="D309" t="n">
-        <v>0.02</v>
+        <v>1.2</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -10924,21 +10924,21 @@
         <v>0</v>
       </c>
       <c r="G309" t="n">
-        <v>0</v>
+        <v>29.18</v>
       </c>
       <c r="H309" t="n">
-        <v>0</v>
+        <v>45.33</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>REPA3</t>
+          <t>BOVH3</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa BOVH</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -10947,7 +10947,7 @@
         </is>
       </c>
       <c r="D310" t="n">
-        <v>1</v>
+        <v>15.71</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -10958,26 +10958,26 @@
         <v>0</v>
       </c>
       <c r="G310" t="n">
-        <v>4.05</v>
+        <v>0</v>
       </c>
       <c r="H310" t="n">
-        <v>1.91</v>
+        <v>0</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>EQMA5B</t>
+          <t>VNET3</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa VNET</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D311" t="n">
@@ -11001,12 +11001,12 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>SEBB3</t>
+          <t>ARND3</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa ARND</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -11015,7 +11015,7 @@
         </is>
       </c>
       <c r="D312" t="n">
-        <v>0</v>
+        <v>0.51</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -11023,24 +11023,24 @@
         </is>
       </c>
       <c r="F312" t="n">
-        <v>0</v>
+        <v>913.58</v>
       </c>
       <c r="G312" t="n">
-        <v>24.15</v>
+        <v>0</v>
       </c>
       <c r="H312" t="n">
-        <v>23.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>BBTG11</t>
+          <t>MSAN4</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -11049,7 +11049,7 @@
         </is>
       </c>
       <c r="D313" t="n">
-        <v>15.01</v>
+        <v>6.44</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -11060,21 +11060,21 @@
         <v>0</v>
       </c>
       <c r="G313" t="n">
-        <v>0</v>
+        <v>11.78</v>
       </c>
       <c r="H313" t="n">
-        <v>0</v>
+        <v>11.81</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>JFAB4</t>
+          <t>GALO4</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Empresa JFAB</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -11083,7 +11083,7 @@
         </is>
       </c>
       <c r="D314" t="n">
-        <v>0.06</v>
+        <v>0.25</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -11094,21 +11094,21 @@
         <v>0</v>
       </c>
       <c r="G314" t="n">
-        <v>0</v>
+        <v>39.37</v>
       </c>
       <c r="H314" t="n">
-        <v>2.34</v>
+        <v>7.62</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>LECO3</t>
+          <t>BBTG13</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Empresa LECO</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -11128,21 +11128,21 @@
         <v>0</v>
       </c>
       <c r="G315" t="n">
-        <v>-3.48</v>
+        <v>0</v>
       </c>
       <c r="H315" t="n">
-        <v>-14.82</v>
+        <v>-42.86</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>VGOR3</t>
+          <t>INHA3</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Empresa VGOR</t>
+          <t>Empresa INHA</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -11162,30 +11162,30 @@
         <v>0</v>
       </c>
       <c r="G316" t="n">
-        <v>6</v>
+        <v>-6.27</v>
       </c>
       <c r="H316" t="n">
-        <v>-24.29</v>
+        <v>-39.87</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>GPIV33</t>
+          <t>PTIP4</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Empresa GPIV</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D317" t="n">
-        <v>4.42</v>
+        <v>25.15</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -11196,30 +11196,30 @@
         <v>0</v>
       </c>
       <c r="G317" t="n">
-        <v>-6.05</v>
+        <v>23.13</v>
       </c>
       <c r="H317" t="n">
-        <v>0</v>
+        <v>-121.74</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>ECIS4</t>
+          <t>LATS3</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa LATS</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>145</v>
+        <v>22</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -11230,21 +11230,21 @@
         <v>0</v>
       </c>
       <c r="G318" t="n">
-        <v>12.48</v>
+        <v>11.63</v>
       </c>
       <c r="H318" t="n">
-        <v>7.33</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>TNEP3</t>
+          <t>VVAX3</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -11253,7 +11253,7 @@
         </is>
       </c>
       <c r="D319" t="n">
-        <v>3.01</v>
+        <v>0</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -11264,21 +11264,21 @@
         <v>0</v>
       </c>
       <c r="G319" t="n">
-        <v>20.53</v>
+        <v>-6.52</v>
       </c>
       <c r="H319" t="n">
-        <v>22.8</v>
+        <v>-92.03</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>CBMA4</t>
+          <t>SGEN4</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -11287,7 +11287,7 @@
         </is>
       </c>
       <c r="D320" t="n">
-        <v>0.01</v>
+        <v>0.6</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -11298,7 +11298,7 @@
         <v>0</v>
       </c>
       <c r="G320" t="n">
-        <v>0</v>
+        <v>-1.59</v>
       </c>
       <c r="H320" t="n">
         <v>0</v>
@@ -11307,21 +11307,21 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>SALM4</t>
+          <t>VSPT3</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>5.9</v>
+        <v>0</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -11332,30 +11332,30 @@
         <v>0</v>
       </c>
       <c r="G321" t="n">
-        <v>25.78</v>
+        <v>0</v>
       </c>
       <c r="H321" t="n">
-        <v>19.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>BERG3</t>
+          <t>BBTG11</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Empresa BERG</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>33</v>
+        <v>15.01</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -11366,30 +11366,30 @@
         <v>0</v>
       </c>
       <c r="G322" t="n">
-        <v>-5.58</v>
+        <v>0</v>
       </c>
       <c r="H322" t="n">
-        <v>-102.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>JBDU3</t>
+          <t>JFAB4</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Empresa JBDU</t>
+          <t>Empresa JFAB</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D323" t="n">
-        <v>0</v>
+        <v>0.06</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -11403,27 +11403,27 @@
         <v>0</v>
       </c>
       <c r="H323" t="n">
-        <v>0</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>EGGY3</t>
+          <t>CCHI4</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Empresa EGGY</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D324" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -11443,12 +11443,12 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>AGEI3</t>
+          <t>REPA3</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Empresa AGEI</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -11457,7 +11457,7 @@
         </is>
       </c>
       <c r="D325" t="n">
-        <v>7.8</v>
+        <v>1</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -11468,30 +11468,30 @@
         <v>0</v>
       </c>
       <c r="G325" t="n">
-        <v>0</v>
+        <v>4.05</v>
       </c>
       <c r="H325" t="n">
-        <v>0</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>SASG3</t>
+          <t>EQMA5B</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Empresa SASG</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>0.98</v>
+        <v>0</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -11511,12 +11511,12 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>BMEF3</t>
+          <t>SEBB3</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Empresa BMEF</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -11525,7 +11525,7 @@
         </is>
       </c>
       <c r="D327" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -11536,21 +11536,21 @@
         <v>0</v>
       </c>
       <c r="G327" t="n">
-        <v>0</v>
+        <v>24.15</v>
       </c>
       <c r="H327" t="n">
-        <v>0</v>
+        <v>23.01</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>ARPS3</t>
+          <t>GPIV33</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa GPIV</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -11559,7 +11559,7 @@
         </is>
       </c>
       <c r="D328" t="n">
-        <v>0.3</v>
+        <v>4.42</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -11570,30 +11570,30 @@
         <v>0</v>
       </c>
       <c r="G328" t="n">
-        <v>-6.64</v>
+        <v>-6.05</v>
       </c>
       <c r="H328" t="n">
-        <v>20.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>ODER3</t>
+          <t>ECIS4</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Empresa ODER</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D329" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -11604,21 +11604,21 @@
         <v>0</v>
       </c>
       <c r="G329" t="n">
-        <v>0</v>
+        <v>12.48</v>
       </c>
       <c r="H329" t="n">
-        <v>0</v>
+        <v>7.33</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>CCTY3</t>
+          <t>TNEP3</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Empresa CCTY</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -11627,7 +11627,7 @@
         </is>
       </c>
       <c r="D330" t="n">
-        <v>0</v>
+        <v>3.01</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -11638,26 +11638,26 @@
         <v>0</v>
       </c>
       <c r="G330" t="n">
-        <v>0</v>
+        <v>20.53</v>
       </c>
       <c r="H330" t="n">
-        <v>0</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>VVAX4</t>
+          <t>LECO3</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa LECO</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D331" t="n">
@@ -11672,21 +11672,21 @@
         <v>0</v>
       </c>
       <c r="G331" t="n">
-        <v>-6.52</v>
+        <v>-3.48</v>
       </c>
       <c r="H331" t="n">
-        <v>-92.03</v>
+        <v>-14.82</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>CSPC3</t>
+          <t>VGOR3</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa VGOR</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -11695,7 +11695,7 @@
         </is>
       </c>
       <c r="D332" t="n">
-        <v>1.24</v>
+        <v>0</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -11706,21 +11706,21 @@
         <v>0</v>
       </c>
       <c r="G332" t="n">
-        <v>29.18</v>
+        <v>6</v>
       </c>
       <c r="H332" t="n">
-        <v>45.33</v>
+        <v>-24.29</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>ABCB3</t>
+          <t>BERG3</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Empresa ABCB</t>
+          <t>Empresa BERG</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -11729,37 +11729,37 @@
         </is>
       </c>
       <c r="D333" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>Bancos</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="F333" t="n">
         <v>0</v>
       </c>
       <c r="G333" t="n">
-        <v>0</v>
+        <v>-5.58</v>
       </c>
       <c r="H333" t="n">
-        <v>14.05</v>
+        <v>-102.71</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>ESTC4</t>
+          <t>JBDU3</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Empresa ESTC</t>
+          <t>Empresa JBDU</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D334" t="n">
@@ -11774,26 +11774,26 @@
         <v>0</v>
       </c>
       <c r="G334" t="n">
-        <v>11.35</v>
+        <v>0</v>
       </c>
       <c r="H334" t="n">
-        <v>3.89</v>
+        <v>0</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>VSPT4</t>
+          <t>EGGY3</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa EGGY</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D335" t="n">
@@ -11817,12 +11817,12 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>BAUH4</t>
+          <t>CBMA4</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Empresa BAUH</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -11831,7 +11831,7 @@
         </is>
       </c>
       <c r="D336" t="n">
-        <v>93.39</v>
+        <v>0.01</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -11839,7 +11839,7 @@
         </is>
       </c>
       <c r="F336" t="n">
-        <v>207.53</v>
+        <v>0</v>
       </c>
       <c r="G336" t="n">
         <v>0</v>
@@ -11851,21 +11851,21 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>ICPI3</t>
+          <t>SALM4</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Empresa ICPI</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -11876,30 +11876,30 @@
         <v>0</v>
       </c>
       <c r="G337" t="n">
-        <v>0</v>
+        <v>25.78</v>
       </c>
       <c r="H337" t="n">
-        <v>0</v>
+        <v>19.53</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>ILLS4</t>
+          <t>BMEF3</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Empresa ILLS</t>
+          <t>Empresa BMEF</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>100.01</v>
+        <v>11</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -11910,21 +11910,21 @@
         <v>0</v>
       </c>
       <c r="G338" t="n">
-        <v>8.140000000000001</v>
+        <v>0</v>
       </c>
       <c r="H338" t="n">
-        <v>36.09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>BPAT33</t>
+          <t>AGEI3</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Empresa BPAT</t>
+          <t>Empresa AGEI</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -11933,7 +11933,7 @@
         </is>
       </c>
       <c r="D339" t="n">
-        <v>20</v>
+        <v>7.8</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -11953,21 +11953,21 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>REPA4</t>
+          <t>SASG3</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa SASG</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D340" t="n">
-        <v>1.08</v>
+        <v>0.98</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -11978,26 +11978,26 @@
         <v>0</v>
       </c>
       <c r="G340" t="n">
-        <v>4.05</v>
+        <v>0</v>
       </c>
       <c r="H340" t="n">
-        <v>1.91</v>
+        <v>0</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>EQMA6B</t>
+          <t>ODER3</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa ODER</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D341" t="n">
@@ -12021,21 +12021,21 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>SEBB4</t>
+          <t>ARPS3</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -12046,21 +12046,21 @@
         <v>0</v>
       </c>
       <c r="G342" t="n">
-        <v>24.15</v>
+        <v>-6.64</v>
       </c>
       <c r="H342" t="n">
-        <v>23.01</v>
+        <v>20.34</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>MSAN3</t>
+          <t>CSPC3</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -12069,7 +12069,7 @@
         </is>
       </c>
       <c r="D343" t="n">
-        <v>6.44</v>
+        <v>1.24</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -12080,21 +12080,21 @@
         <v>0</v>
       </c>
       <c r="G343" t="n">
-        <v>11.78</v>
+        <v>29.18</v>
       </c>
       <c r="H343" t="n">
-        <v>11.81</v>
+        <v>45.33</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>GALO3</t>
+          <t>ABCB3</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa ABCB</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
@@ -12107,28 +12107,28 @@
       </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="F344" t="n">
         <v>0</v>
       </c>
       <c r="G344" t="n">
-        <v>39.37</v>
+        <v>0</v>
       </c>
       <c r="H344" t="n">
-        <v>7.62</v>
+        <v>14.05</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>SLCP3</t>
+          <t>CCTY3</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Empresa SLCP</t>
+          <t>Empresa CCTY</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -12137,7 +12137,7 @@
         </is>
       </c>
       <c r="D345" t="n">
-        <v>610.02</v>
+        <v>0</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -12157,17 +12157,17 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>DAYC3</t>
+          <t>VVAX4</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Empresa DAYC</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D346" t="n">
@@ -12182,30 +12182,30 @@
         <v>0</v>
       </c>
       <c r="G346" t="n">
-        <v>0</v>
+        <v>-6.52</v>
       </c>
       <c r="H346" t="n">
-        <v>17.33</v>
+        <v>-92.03</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>PTIP3</t>
+          <t>BAUH4</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa BAUH</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>22</v>
+        <v>93.39</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -12213,24 +12213,24 @@
         </is>
       </c>
       <c r="F347" t="n">
-        <v>0</v>
+        <v>207.53</v>
       </c>
       <c r="G347" t="n">
-        <v>23.13</v>
+        <v>0</v>
       </c>
       <c r="H347" t="n">
-        <v>-121.74</v>
+        <v>0</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>MLPA3</t>
+          <t>ICPI3</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Empresa MLPA</t>
+          <t>Empresa ICPI</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
@@ -12253,18 +12253,18 @@
         <v>0</v>
       </c>
       <c r="H348" t="n">
-        <v>45.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>CLSC6</t>
+          <t>ILLS4</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Empresa CLSC</t>
+          <t>Empresa ILLS</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
@@ -12273,7 +12273,7 @@
         </is>
       </c>
       <c r="D349" t="n">
-        <v>0</v>
+        <v>100.01</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -12284,21 +12284,21 @@
         <v>0</v>
       </c>
       <c r="G349" t="n">
-        <v>0</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="H349" t="n">
-        <v>0</v>
+        <v>36.09</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>SGEN3</t>
+          <t>BPAT33</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa BPAT</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
@@ -12307,7 +12307,7 @@
         </is>
       </c>
       <c r="D350" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -12318,7 +12318,7 @@
         <v>0</v>
       </c>
       <c r="G350" t="n">
-        <v>-1.59</v>
+        <v>0</v>
       </c>
       <c r="H350" t="n">
         <v>0</v>
@@ -12327,12 +12327,12 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>DUFB11</t>
+          <t>ESTC4</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Empresa DUFB</t>
+          <t>Empresa ESTC</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -12352,21 +12352,21 @@
         <v>0</v>
       </c>
       <c r="G351" t="n">
-        <v>0</v>
+        <v>11.35</v>
       </c>
       <c r="H351" t="n">
-        <v>0</v>
+        <v>3.89</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>TNEP4</t>
+          <t>VSPT4</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -12375,7 +12375,7 @@
         </is>
       </c>
       <c r="D352" t="n">
-        <v>3.95</v>
+        <v>0</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -12386,21 +12386,21 @@
         <v>0</v>
       </c>
       <c r="G352" t="n">
-        <v>20.53</v>
+        <v>0</v>
       </c>
       <c r="H352" t="n">
-        <v>22.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>CCHI3</t>
+          <t>MSAN3</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -12409,7 +12409,7 @@
         </is>
       </c>
       <c r="D353" t="n">
-        <v>0.02</v>
+        <v>6.44</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -12420,21 +12420,21 @@
         <v>0</v>
       </c>
       <c r="G353" t="n">
-        <v>0</v>
+        <v>11.78</v>
       </c>
       <c r="H353" t="n">
-        <v>0</v>
+        <v>11.81</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>SFSA3</t>
+          <t>GALO3</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Empresa SFSA</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -12454,21 +12454,21 @@
         <v>0</v>
       </c>
       <c r="G354" t="n">
-        <v>0</v>
+        <v>39.37</v>
       </c>
       <c r="H354" t="n">
-        <v>6.25</v>
+        <v>7.62</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>PRBC3</t>
+          <t>SLCP3</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Empresa PRBC</t>
+          <t>Empresa SLCP</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -12477,7 +12477,7 @@
         </is>
       </c>
       <c r="D355" t="n">
-        <v>0</v>
+        <v>610.02</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -12491,18 +12491,18 @@
         <v>0</v>
       </c>
       <c r="H355" t="n">
-        <v>8.27</v>
+        <v>0</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>ECIS3</t>
+          <t>DAYC3</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa DAYC</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -12511,7 +12511,7 @@
         </is>
       </c>
       <c r="D356" t="n">
-        <v>211.65</v>
+        <v>0</v>
       </c>
       <c r="E356" t="inlineStr">
         <is>
@@ -12522,21 +12522,21 @@
         <v>0</v>
       </c>
       <c r="G356" t="n">
-        <v>12.48</v>
+        <v>0</v>
       </c>
       <c r="H356" t="n">
-        <v>7.33</v>
+        <v>17.33</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>CBMA3</t>
+          <t>PTIP3</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -12545,7 +12545,7 @@
         </is>
       </c>
       <c r="D357" t="n">
-        <v>0.01</v>
+        <v>22</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -12556,30 +12556,30 @@
         <v>0</v>
       </c>
       <c r="G357" t="n">
-        <v>0</v>
+        <v>23.13</v>
       </c>
       <c r="H357" t="n">
-        <v>0</v>
+        <v>-121.74</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>ALBA3</t>
+          <t>REPA4</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Empresa ALBA</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D358" t="n">
-        <v>2.15</v>
+        <v>1.08</v>
       </c>
       <c r="E358" t="inlineStr">
         <is>
@@ -12590,21 +12590,21 @@
         <v>0</v>
       </c>
       <c r="G358" t="n">
-        <v>20.4</v>
+        <v>4.05</v>
       </c>
       <c r="H358" t="n">
-        <v>19.77</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>ARPS4</t>
+          <t>EQMA6B</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
@@ -12624,30 +12624,30 @@
         <v>0</v>
       </c>
       <c r="G359" t="n">
-        <v>-6.64</v>
+        <v>0</v>
       </c>
       <c r="H359" t="n">
-        <v>20.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>SALM3</t>
+          <t>SEBB4</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>5.7</v>
+        <v>0</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -12658,30 +12658,30 @@
         <v>0</v>
       </c>
       <c r="G360" t="n">
-        <v>25.78</v>
+        <v>24.15</v>
       </c>
       <c r="H360" t="n">
-        <v>19.53</v>
+        <v>23.01</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>CMMA4</t>
+          <t>SGEN3</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Empresa CMMA</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D361" t="n">
-        <v>0.8100000000000001</v>
+        <v>5</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -12692,26 +12692,26 @@
         <v>0</v>
       </c>
       <c r="G361" t="n">
-        <v>0</v>
+        <v>-1.59</v>
       </c>
       <c r="H361" t="n">
-        <v>-1.92</v>
+        <v>0</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>CZRS3</t>
+          <t>DUFB11</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>Empresa CZRS</t>
+          <t>Empresa DUFB</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D362" t="n">
@@ -12729,27 +12729,27 @@
         <v>0</v>
       </c>
       <c r="H362" t="n">
-        <v>3.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>BPNM3</t>
+          <t>TNEP4</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Empresa BPNM</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D363" t="n">
-        <v>0</v>
+        <v>3.95</v>
       </c>
       <c r="E363" t="inlineStr">
         <is>
@@ -12760,21 +12760,21 @@
         <v>0</v>
       </c>
       <c r="G363" t="n">
-        <v>0</v>
+        <v>20.53</v>
       </c>
       <c r="H363" t="n">
-        <v>9.67</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>BSGR3</t>
+          <t>MLPA3</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Empresa BSGR</t>
+          <t>Empresa MLPA</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -12783,7 +12783,7 @@
         </is>
       </c>
       <c r="D364" t="n">
-        <v>1091.28</v>
+        <v>0</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -12797,23 +12797,23 @@
         <v>0</v>
       </c>
       <c r="H364" t="n">
-        <v>0</v>
+        <v>45.13</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>VNET3</t>
+          <t>CLSC6</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Empresa VNET</t>
+          <t>Empresa CLSC</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D365" t="n">
@@ -12837,21 +12837,21 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>CSPC4</t>
+          <t>CCHI3</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D366" t="n">
-        <v>1.2</v>
+        <v>0.02</v>
       </c>
       <c r="E366" t="inlineStr">
         <is>
@@ -12862,21 +12862,21 @@
         <v>0</v>
       </c>
       <c r="G366" t="n">
-        <v>29.18</v>
+        <v>0</v>
       </c>
       <c r="H366" t="n">
-        <v>45.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>BOVH3</t>
+          <t>SFSA3</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Empresa BOVH</t>
+          <t>Empresa SFSA</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -12885,7 +12885,7 @@
         </is>
       </c>
       <c r="D367" t="n">
-        <v>15.71</v>
+        <v>0</v>
       </c>
       <c r="E367" t="inlineStr">
         <is>
@@ -12899,18 +12899,18 @@
         <v>0</v>
       </c>
       <c r="H367" t="n">
-        <v>0</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>ARND3</t>
+          <t>PRBC3</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Empresa ARND</t>
+          <t>Empresa PRBC</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -12919,7 +12919,7 @@
         </is>
       </c>
       <c r="D368" t="n">
-        <v>0.51</v>
+        <v>0</v>
       </c>
       <c r="E368" t="inlineStr">
         <is>
@@ -12927,24 +12927,24 @@
         </is>
       </c>
       <c r="F368" t="n">
-        <v>913.58</v>
+        <v>0</v>
       </c>
       <c r="G368" t="n">
         <v>0</v>
       </c>
       <c r="H368" t="n">
-        <v>0</v>
+        <v>8.27</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>VVAX3</t>
+          <t>ECIS3</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -12953,7 +12953,7 @@
         </is>
       </c>
       <c r="D369" t="n">
-        <v>0</v>
+        <v>211.65</v>
       </c>
       <c r="E369" t="inlineStr">
         <is>
@@ -12964,30 +12964,30 @@
         <v>0</v>
       </c>
       <c r="G369" t="n">
-        <v>-6.52</v>
+        <v>12.48</v>
       </c>
       <c r="H369" t="n">
-        <v>-92.03</v>
+        <v>7.33</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>MSAN4</t>
+          <t>CZRS3</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa CZRS</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D370" t="n">
-        <v>6.44</v>
+        <v>0</v>
       </c>
       <c r="E370" t="inlineStr">
         <is>
@@ -12998,30 +12998,30 @@
         <v>0</v>
       </c>
       <c r="G370" t="n">
-        <v>11.78</v>
+        <v>0</v>
       </c>
       <c r="H370" t="n">
-        <v>11.81</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>GALO4</t>
+          <t>BPNM3</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa BPNM</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D371" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="E371" t="inlineStr">
         <is>
@@ -13032,21 +13032,21 @@
         <v>0</v>
       </c>
       <c r="G371" t="n">
-        <v>39.37</v>
+        <v>0</v>
       </c>
       <c r="H371" t="n">
-        <v>7.62</v>
+        <v>9.67</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>BBTG13</t>
+          <t>BSGR3</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa BSGR</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
@@ -13055,7 +13055,7 @@
         </is>
       </c>
       <c r="D372" t="n">
-        <v>0</v>
+        <v>1091.28</v>
       </c>
       <c r="E372" t="inlineStr">
         <is>
@@ -13069,18 +13069,18 @@
         <v>0</v>
       </c>
       <c r="H372" t="n">
-        <v>-42.86</v>
+        <v>0</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>INHA3</t>
+          <t>CBMA3</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Empresa INHA</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
@@ -13089,7 +13089,7 @@
         </is>
       </c>
       <c r="D373" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="E373" t="inlineStr">
         <is>
@@ -13100,30 +13100,30 @@
         <v>0</v>
       </c>
       <c r="G373" t="n">
-        <v>-6.27</v>
+        <v>0</v>
       </c>
       <c r="H373" t="n">
-        <v>-39.87</v>
+        <v>0</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>PTIP4</t>
+          <t>ALBA3</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa ALBA</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D374" t="n">
-        <v>25.15</v>
+        <v>2.15</v>
       </c>
       <c r="E374" t="inlineStr">
         <is>
@@ -13134,30 +13134,30 @@
         <v>0</v>
       </c>
       <c r="G374" t="n">
-        <v>23.13</v>
+        <v>20.4</v>
       </c>
       <c r="H374" t="n">
-        <v>-121.74</v>
+        <v>19.77</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>LATS3</t>
+          <t>ARPS4</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>Empresa LATS</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D375" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="E375" t="inlineStr">
         <is>
@@ -13168,21 +13168,21 @@
         <v>0</v>
       </c>
       <c r="G375" t="n">
-        <v>11.63</v>
+        <v>-6.64</v>
       </c>
       <c r="H375" t="n">
-        <v>1.84</v>
+        <v>20.34</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>VSPT3</t>
+          <t>SALM3</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
@@ -13191,7 +13191,7 @@
         </is>
       </c>
       <c r="D376" t="n">
-        <v>0</v>
+        <v>5.7</v>
       </c>
       <c r="E376" t="inlineStr">
         <is>
@@ -13202,21 +13202,21 @@
         <v>0</v>
       </c>
       <c r="G376" t="n">
-        <v>0</v>
+        <v>25.78</v>
       </c>
       <c r="H376" t="n">
-        <v>0</v>
+        <v>19.53</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>SGEN4</t>
+          <t>CMMA4</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa CMMA</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
@@ -13225,7 +13225,7 @@
         </is>
       </c>
       <c r="D377" t="n">
-        <v>0.6</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -13236,10 +13236,10 @@
         <v>0</v>
       </c>
       <c r="G377" t="n">
-        <v>-1.59</v>
+        <v>0</v>
       </c>
       <c r="H377" t="n">
-        <v>0</v>
+        <v>-1.92</v>
       </c>
     </row>
     <row r="378">
@@ -15421,7 +15421,7 @@
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>MMAQ3</t>
+          <t>MMAQ4</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
@@ -15431,7 +15431,7 @@
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D442" t="n">
@@ -15455,7 +15455,7 @@
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>MMAQ4</t>
+          <t>MMAQ3</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
@@ -15465,7 +15465,7 @@
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D443" t="n">
@@ -20521,7 +20521,7 @@
     <row r="592">
       <c r="A592" t="inlineStr">
         <is>
-          <t>GETT3</t>
+          <t>GETT4</t>
         </is>
       </c>
       <c r="B592" t="inlineStr">
@@ -20531,7 +20531,7 @@
       </c>
       <c r="C592" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D592" t="n">
@@ -20555,7 +20555,7 @@
     <row r="593">
       <c r="A593" t="inlineStr">
         <is>
-          <t>GETT4</t>
+          <t>GETT3</t>
         </is>
       </c>
       <c r="B593" t="inlineStr">
@@ -20565,7 +20565,7 @@
       </c>
       <c r="C593" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D593" t="n">
@@ -29769,7 +29769,7 @@
     <row r="864">
       <c r="A864" t="inlineStr">
         <is>
-          <t>RSIP4</t>
+          <t>RSIP3</t>
         </is>
       </c>
       <c r="B864" t="inlineStr">
@@ -29779,7 +29779,7 @@
       </c>
       <c r="C864" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D864" t="n">
@@ -29803,7 +29803,7 @@
     <row r="865">
       <c r="A865" t="inlineStr">
         <is>
-          <t>RSIP3</t>
+          <t>RSIP4</t>
         </is>
       </c>
       <c r="B865" t="inlineStr">
@@ -29813,7 +29813,7 @@
       </c>
       <c r="C865" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D865" t="n">
@@ -33475,7 +33475,7 @@
     <row r="973">
       <c r="A973" t="inlineStr">
         <is>
-          <t>PQUN4</t>
+          <t>PQUN3</t>
         </is>
       </c>
       <c r="B973" t="inlineStr">
@@ -33485,7 +33485,7 @@
       </c>
       <c r="C973" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D973" t="n">
@@ -33509,7 +33509,7 @@
     <row r="974">
       <c r="A974" t="inlineStr">
         <is>
-          <t>PQUN3</t>
+          <t>PQUN4</t>
         </is>
       </c>
       <c r="B974" t="inlineStr">
@@ -33519,7 +33519,7 @@
       </c>
       <c r="C974" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D974" t="n">

</xml_diff>

<commit_message>
Corrige tratamento e mapeamento da Margem Liquida
</commit_message>
<xml_diff>
--- a/acoes_b3.xlsx
+++ b/acoes_b3.xlsx
@@ -471,21 +471,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CLAN3</t>
+          <t>PORP4</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Empresa CLAN</t>
+          <t>Empresa PORP</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1012240000</v>
+        <v>22399000</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -505,27 +505,27 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>-1.05</v>
+        <v>-2.08</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MNSA4</t>
+          <t>IVTT3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Empresa MNSA</t>
+          <t>Empresa IVTT</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.47</v>
+        <v>0</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -533,39 +533,39 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>-9105000</v>
+        <v>1083050000</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>-208.15</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>-13.5</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>145.7</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CSTB4</t>
+          <t>MNSA3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa MNSA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>147.69</v>
+        <v>0.42</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -573,30 +573,30 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>8420670000</v>
+        <v>-9105000</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>40.85</v>
+        <v>-208.15</v>
       </c>
       <c r="I4" t="n">
-        <v>22.4</v>
+        <v>-13.5</v>
       </c>
       <c r="J4" t="n">
-        <v>20.11</v>
+        <v>145.7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PORP4</t>
+          <t>CFLU4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Empresa PORP</t>
+          <t>Empresa CFLU</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2.4</v>
+        <v>1000</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -613,30 +613,30 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>22399000</v>
+        <v>60351000</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>17.68</v>
       </c>
       <c r="J5" t="n">
-        <v>-2.08</v>
+        <v>32.15</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>IVTT3</t>
+          <t>CSTB3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Empresa IVTT</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -653,39 +653,39 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>1083050000</v>
+        <v>8420670000</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>40.85</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>22.4</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.4</v>
+        <v>20.11</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MNSA3</t>
+          <t>POPR4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Empresa MNSA</t>
+          <t>Empresa POPR</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.42</v>
+        <v>10.17</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -693,39 +693,39 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>-9105000</v>
+        <v>545803000</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>-208.15</v>
+        <v>8.66</v>
       </c>
       <c r="I7" t="n">
-        <v>-13.5</v>
+        <v>15.25</v>
       </c>
       <c r="J7" t="n">
-        <v>145.7</v>
+        <v>19.93</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CFLU4</t>
+          <t>PMET3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Empresa CFLU</t>
+          <t>Empresa PMET</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -733,30 +733,30 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>60351000</v>
+        <v>-290863000</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>8.880000000000001</v>
+        <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>17.68</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>32.15</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CSTB3</t>
+          <t>CLAN3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa CLAN</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -773,30 +773,30 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>8420670000</v>
+        <v>1012240000</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>40.85</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>22.4</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>20.11</v>
+        <v>-1.05</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>POPR4</t>
+          <t>MNSA4</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Empresa POPR</t>
+          <t>Empresa MNSA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>10.17</v>
+        <v>0.47</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -813,39 +813,39 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>545803000</v>
+        <v>-9105000</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>8.66</v>
+        <v>-208.15</v>
       </c>
       <c r="I10" t="n">
-        <v>15.25</v>
+        <v>-13.5</v>
       </c>
       <c r="J10" t="n">
-        <v>19.93</v>
+        <v>145.7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PMET3</t>
+          <t>CSTB4</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Empresa PMET</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>147.69</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -853,19 +853,19 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>-290863000</v>
+        <v>8420670000</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>40.85</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>22.4</v>
       </c>
       <c r="J11" t="n">
-        <v>4.1</v>
+        <v>20.11</v>
       </c>
     </row>
     <row r="12">
@@ -6351,7 +6351,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>PNOR5</t>
+          <t>PNOR6</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -6391,7 +6391,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>PNOR6</t>
+          <t>PNOR5</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -12751,21 +12751,21 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>VVAX3</t>
+          <t>CCHI4</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -12773,39 +12773,39 @@
         </is>
       </c>
       <c r="F309" t="n">
-        <v>144676000</v>
+        <v>-160477000</v>
       </c>
       <c r="G309" t="n">
         <v>0</v>
       </c>
       <c r="H309" t="n">
-        <v>-7.36</v>
+        <v>0</v>
       </c>
       <c r="I309" t="n">
-        <v>-6.52</v>
+        <v>0</v>
       </c>
       <c r="J309" t="n">
-        <v>-92.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>MSAN4</t>
+          <t>REPA3</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>6.44</v>
+        <v>1</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -12813,30 +12813,30 @@
         </is>
       </c>
       <c r="F310" t="n">
-        <v>2533030000</v>
+        <v>378378000</v>
       </c>
       <c r="G310" t="n">
         <v>0</v>
       </c>
       <c r="H310" t="n">
-        <v>6.27</v>
+        <v>5.18</v>
       </c>
       <c r="I310" t="n">
-        <v>11.78</v>
+        <v>4.05</v>
       </c>
       <c r="J310" t="n">
-        <v>11.81</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>GALO4</t>
+          <t>EQMA5B</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -12845,7 +12845,7 @@
         </is>
       </c>
       <c r="D311" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -12853,30 +12853,30 @@
         </is>
       </c>
       <c r="F311" t="n">
-        <v>-60607000</v>
+        <v>4940330000</v>
       </c>
       <c r="G311" t="n">
         <v>0</v>
       </c>
       <c r="H311" t="n">
-        <v>13.98</v>
+        <v>0</v>
       </c>
       <c r="I311" t="n">
-        <v>39.37</v>
+        <v>0</v>
       </c>
       <c r="J311" t="n">
-        <v>7.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>BBTG13</t>
+          <t>SEBB3</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -12893,39 +12893,39 @@
         </is>
       </c>
       <c r="F312" t="n">
-        <v>7000</v>
+        <v>145783000</v>
       </c>
       <c r="G312" t="n">
         <v>0</v>
       </c>
       <c r="H312" t="n">
-        <v>0</v>
+        <v>9.24</v>
       </c>
       <c r="I312" t="n">
-        <v>0</v>
+        <v>24.15</v>
       </c>
       <c r="J312" t="n">
-        <v>-42.86</v>
+        <v>23.01</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>INHA3</t>
+          <t>BBTG11</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Empresa INHA</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>0</v>
+        <v>15.01</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -12933,30 +12933,30 @@
         </is>
       </c>
       <c r="F313" t="n">
-        <v>1533210000</v>
+        <v>0</v>
       </c>
       <c r="G313" t="n">
         <v>0</v>
       </c>
       <c r="H313" t="n">
-        <v>-56.05</v>
+        <v>0</v>
       </c>
       <c r="I313" t="n">
-        <v>-6.27</v>
+        <v>0</v>
       </c>
       <c r="J313" t="n">
-        <v>-39.87</v>
+        <v>0</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>PTIP4</t>
+          <t>JFAB4</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa JFAB</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -12965,7 +12965,7 @@
         </is>
       </c>
       <c r="D314" t="n">
-        <v>25.15</v>
+        <v>0.06</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -12973,30 +12973,30 @@
         </is>
       </c>
       <c r="F314" t="n">
-        <v>-155957000</v>
+        <v>-10183000</v>
       </c>
       <c r="G314" t="n">
         <v>0</v>
       </c>
       <c r="H314" t="n">
-        <v>13.73</v>
+        <v>0</v>
       </c>
       <c r="I314" t="n">
-        <v>23.13</v>
+        <v>0</v>
       </c>
       <c r="J314" t="n">
-        <v>-121.74</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>LATS3</t>
+          <t>LECO3</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Empresa LATS</t>
+          <t>Empresa LECO</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -13005,7 +13005,7 @@
         </is>
       </c>
       <c r="D315" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -13013,30 +13013,30 @@
         </is>
       </c>
       <c r="F315" t="n">
-        <v>680646000</v>
+        <v>105928000</v>
       </c>
       <c r="G315" t="n">
         <v>0</v>
       </c>
       <c r="H315" t="n">
-        <v>11.74</v>
+        <v>-2.14</v>
       </c>
       <c r="I315" t="n">
-        <v>11.63</v>
+        <v>-3.48</v>
       </c>
       <c r="J315" t="n">
-        <v>1.84</v>
+        <v>-14.82</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>VSPT3</t>
+          <t>VGOR3</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa VGOR</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -13053,39 +13053,39 @@
         </is>
       </c>
       <c r="F316" t="n">
-        <v>5031600000</v>
+        <v>135178000</v>
       </c>
       <c r="G316" t="n">
         <v>0</v>
       </c>
       <c r="H316" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="I316" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J316" t="n">
-        <v>0</v>
+        <v>-24.29</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>SGEN4</t>
+          <t>GPIV33</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa GPIV</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D317" t="n">
-        <v>0.6</v>
+        <v>4.42</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -13093,16 +13093,16 @@
         </is>
       </c>
       <c r="F317" t="n">
-        <v>156981000</v>
+        <v>1318490000</v>
       </c>
       <c r="G317" t="n">
         <v>0</v>
       </c>
       <c r="H317" t="n">
-        <v>-1871.17</v>
+        <v>257.32</v>
       </c>
       <c r="I317" t="n">
-        <v>-1.59</v>
+        <v>-6.05</v>
       </c>
       <c r="J317" t="n">
         <v>0</v>
@@ -13111,21 +13111,21 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>REPA3</t>
+          <t>ECIS4</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>1</v>
+        <v>145</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -13133,39 +13133,39 @@
         </is>
       </c>
       <c r="F318" t="n">
-        <v>378378000</v>
+        <v>129346000</v>
       </c>
       <c r="G318" t="n">
         <v>0</v>
       </c>
       <c r="H318" t="n">
-        <v>5.18</v>
+        <v>34.9</v>
       </c>
       <c r="I318" t="n">
-        <v>4.05</v>
+        <v>12.48</v>
       </c>
       <c r="J318" t="n">
-        <v>1.91</v>
+        <v>7.33</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>EQMA5B</t>
+          <t>TNEP3</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>0</v>
+        <v>3.01</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -13173,39 +13173,39 @@
         </is>
       </c>
       <c r="F319" t="n">
-        <v>4940330000</v>
+        <v>955105000</v>
       </c>
       <c r="G319" t="n">
         <v>0</v>
       </c>
       <c r="H319" t="n">
-        <v>0</v>
+        <v>20.92</v>
       </c>
       <c r="I319" t="n">
-        <v>0</v>
+        <v>20.53</v>
       </c>
       <c r="J319" t="n">
-        <v>0</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>SEBB3</t>
+          <t>CBMA4</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -13213,30 +13213,30 @@
         </is>
       </c>
       <c r="F320" t="n">
-        <v>145783000</v>
+        <v>-34022300000</v>
       </c>
       <c r="G320" t="n">
         <v>0</v>
       </c>
       <c r="H320" t="n">
-        <v>9.24</v>
+        <v>0</v>
       </c>
       <c r="I320" t="n">
-        <v>24.15</v>
+        <v>0</v>
       </c>
       <c r="J320" t="n">
-        <v>23.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>BBTG11</t>
+          <t>SALM4</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -13245,7 +13245,7 @@
         </is>
       </c>
       <c r="D321" t="n">
-        <v>15.01</v>
+        <v>5.9</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -13253,39 +13253,39 @@
         </is>
       </c>
       <c r="F321" t="n">
-        <v>0</v>
+        <v>475600000</v>
       </c>
       <c r="G321" t="n">
         <v>0</v>
       </c>
       <c r="H321" t="n">
-        <v>0</v>
+        <v>10.22</v>
       </c>
       <c r="I321" t="n">
-        <v>0</v>
+        <v>25.78</v>
       </c>
       <c r="J321" t="n">
-        <v>0</v>
+        <v>19.53</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>JFAB4</t>
+          <t>BERG3</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Empresa JFAB</t>
+          <t>Empresa BERG</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>0.06</v>
+        <v>33</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -13293,39 +13293,39 @@
         </is>
       </c>
       <c r="F322" t="n">
-        <v>-10183000</v>
+        <v>9538000</v>
       </c>
       <c r="G322" t="n">
         <v>0</v>
       </c>
       <c r="H322" t="n">
-        <v>0</v>
+        <v>-8.6</v>
       </c>
       <c r="I322" t="n">
-        <v>0</v>
+        <v>-5.58</v>
       </c>
       <c r="J322" t="n">
-        <v>2.34</v>
+        <v>-102.71</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>CCHI4</t>
+          <t>JBDU3</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa JBDU</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D323" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -13333,7 +13333,7 @@
         </is>
       </c>
       <c r="F323" t="n">
-        <v>-160477000</v>
+        <v>56569000</v>
       </c>
       <c r="G323" t="n">
         <v>0</v>
@@ -13351,12 +13351,12 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>VGOR3</t>
+          <t>EGGY3</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Empresa VGOR</t>
+          <t>Empresa EGGY</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -13373,30 +13373,30 @@
         </is>
       </c>
       <c r="F324" t="n">
-        <v>135178000</v>
+        <v>954480000</v>
       </c>
       <c r="G324" t="n">
         <v>0</v>
       </c>
       <c r="H324" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="I324" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J324" t="n">
-        <v>-24.29</v>
+        <v>0</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>GPIV33</t>
+          <t>AGEI3</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Empresa GPIV</t>
+          <t>Empresa AGEI</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -13405,7 +13405,7 @@
         </is>
       </c>
       <c r="D325" t="n">
-        <v>4.42</v>
+        <v>7.8</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -13413,16 +13413,16 @@
         </is>
       </c>
       <c r="F325" t="n">
-        <v>1318490000</v>
+        <v>1878210000</v>
       </c>
       <c r="G325" t="n">
         <v>0</v>
       </c>
       <c r="H325" t="n">
-        <v>257.32</v>
+        <v>0</v>
       </c>
       <c r="I325" t="n">
-        <v>-6.05</v>
+        <v>0</v>
       </c>
       <c r="J325" t="n">
         <v>0</v>
@@ -13431,21 +13431,21 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>ECIS4</t>
+          <t>SASG3</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa SASG</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>145</v>
+        <v>0.98</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -13453,30 +13453,30 @@
         </is>
       </c>
       <c r="F326" t="n">
-        <v>129346000</v>
+        <v>0</v>
       </c>
       <c r="G326" t="n">
         <v>0</v>
       </c>
       <c r="H326" t="n">
-        <v>34.9</v>
+        <v>0</v>
       </c>
       <c r="I326" t="n">
-        <v>12.48</v>
+        <v>0</v>
       </c>
       <c r="J326" t="n">
-        <v>7.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>TNEP3</t>
+          <t>BMEF3</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa BMEF</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -13485,7 +13485,7 @@
         </is>
       </c>
       <c r="D327" t="n">
-        <v>3.01</v>
+        <v>11</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -13493,30 +13493,30 @@
         </is>
       </c>
       <c r="F327" t="n">
-        <v>955105000</v>
+        <v>2674780000</v>
       </c>
       <c r="G327" t="n">
         <v>0</v>
       </c>
       <c r="H327" t="n">
-        <v>20.92</v>
+        <v>0</v>
       </c>
       <c r="I327" t="n">
-        <v>20.53</v>
+        <v>0</v>
       </c>
       <c r="J327" t="n">
-        <v>22.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>LECO3</t>
+          <t>ARPS3</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Empresa LECO</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -13525,7 +13525,7 @@
         </is>
       </c>
       <c r="D328" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -13533,39 +13533,39 @@
         </is>
       </c>
       <c r="F328" t="n">
-        <v>105928000</v>
+        <v>-12690000</v>
       </c>
       <c r="G328" t="n">
         <v>0</v>
       </c>
       <c r="H328" t="n">
-        <v>-2.14</v>
+        <v>-4.92</v>
       </c>
       <c r="I328" t="n">
-        <v>-3.48</v>
+        <v>-6.64</v>
       </c>
       <c r="J328" t="n">
-        <v>-14.82</v>
+        <v>20.34</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>SALM4</t>
+          <t>ODER3</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa ODER</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D329" t="n">
-        <v>5.9</v>
+        <v>0</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -13573,30 +13573,30 @@
         </is>
       </c>
       <c r="F329" t="n">
-        <v>475600000</v>
+        <v>609518000</v>
       </c>
       <c r="G329" t="n">
         <v>0</v>
       </c>
       <c r="H329" t="n">
-        <v>10.22</v>
+        <v>0</v>
       </c>
       <c r="I329" t="n">
-        <v>25.78</v>
+        <v>0</v>
       </c>
       <c r="J329" t="n">
-        <v>19.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>BERG3</t>
+          <t>CCTY3</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Empresa BERG</t>
+          <t>Empresa CCTY</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -13605,7 +13605,7 @@
         </is>
       </c>
       <c r="D330" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -13613,35 +13613,35 @@
         </is>
       </c>
       <c r="F330" t="n">
-        <v>9538000</v>
+        <v>0</v>
       </c>
       <c r="G330" t="n">
         <v>0</v>
       </c>
       <c r="H330" t="n">
-        <v>-8.6</v>
+        <v>0</v>
       </c>
       <c r="I330" t="n">
-        <v>-5.58</v>
+        <v>0</v>
       </c>
       <c r="J330" t="n">
-        <v>-102.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>JBDU3</t>
+          <t>VVAX4</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Empresa JBDU</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D331" t="n">
@@ -13653,30 +13653,30 @@
         </is>
       </c>
       <c r="F331" t="n">
-        <v>56569000</v>
+        <v>144676000</v>
       </c>
       <c r="G331" t="n">
         <v>0</v>
       </c>
       <c r="H331" t="n">
-        <v>0</v>
+        <v>-7.36</v>
       </c>
       <c r="I331" t="n">
-        <v>0</v>
+        <v>-6.52</v>
       </c>
       <c r="J331" t="n">
-        <v>0</v>
+        <v>-92.03</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>EGGY3</t>
+          <t>CSPC3</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Empresa EGGY</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -13685,7 +13685,7 @@
         </is>
       </c>
       <c r="D332" t="n">
-        <v>0</v>
+        <v>1.24</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -13693,47 +13693,47 @@
         </is>
       </c>
       <c r="F332" t="n">
-        <v>954480000</v>
+        <v>2126670000</v>
       </c>
       <c r="G332" t="n">
         <v>0</v>
       </c>
       <c r="H332" t="n">
-        <v>0</v>
+        <v>38.62</v>
       </c>
       <c r="I332" t="n">
-        <v>0</v>
+        <v>29.18</v>
       </c>
       <c r="J332" t="n">
-        <v>0</v>
+        <v>45.33</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>CBMA4</t>
+          <t>ABCB3</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa ABCB</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="F333" t="n">
-        <v>-34022300000</v>
+        <v>7258910000</v>
       </c>
       <c r="G333" t="n">
         <v>0</v>
@@ -13745,27 +13745,27 @@
         <v>0</v>
       </c>
       <c r="J333" t="n">
-        <v>0</v>
+        <v>14.05</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>SASG3</t>
+          <t>ESTC4</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Empresa SASG</t>
+          <t>Empresa ESTC</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>0.98</v>
+        <v>0</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -13773,39 +13773,39 @@
         </is>
       </c>
       <c r="F334" t="n">
-        <v>0</v>
+        <v>2916530000</v>
       </c>
       <c r="G334" t="n">
         <v>0</v>
       </c>
       <c r="H334" t="n">
-        <v>0</v>
+        <v>16.91</v>
       </c>
       <c r="I334" t="n">
-        <v>0</v>
+        <v>11.35</v>
       </c>
       <c r="J334" t="n">
-        <v>0</v>
+        <v>3.89</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>BMEF3</t>
+          <t>VSPT4</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Empresa BMEF</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -13813,7 +13813,7 @@
         </is>
       </c>
       <c r="F335" t="n">
-        <v>2674780000</v>
+        <v>5031600000</v>
       </c>
       <c r="G335" t="n">
         <v>0</v>
@@ -13831,21 +13831,21 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>AGEI3</t>
+          <t>BAUH4</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Empresa AGEI</t>
+          <t>Empresa BAUH</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>7.8</v>
+        <v>93.39</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -13853,10 +13853,10 @@
         </is>
       </c>
       <c r="F336" t="n">
-        <v>1878210000</v>
+        <v>153407000</v>
       </c>
       <c r="G336" t="n">
-        <v>0</v>
+        <v>207.53</v>
       </c>
       <c r="H336" t="n">
         <v>0</v>
@@ -13871,12 +13871,12 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>ARPS3</t>
+          <t>ICPI3</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa ICPI</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -13885,7 +13885,7 @@
         </is>
       </c>
       <c r="D337" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -13893,39 +13893,39 @@
         </is>
       </c>
       <c r="F337" t="n">
-        <v>-12690000</v>
+        <v>0</v>
       </c>
       <c r="G337" t="n">
         <v>0</v>
       </c>
       <c r="H337" t="n">
-        <v>-4.92</v>
+        <v>0</v>
       </c>
       <c r="I337" t="n">
-        <v>-6.64</v>
+        <v>0</v>
       </c>
       <c r="J337" t="n">
-        <v>20.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>ODER3</t>
+          <t>ILLS4</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Empresa ODER</t>
+          <t>Empresa ILLS</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>0</v>
+        <v>100.01</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -13933,30 +13933,30 @@
         </is>
       </c>
       <c r="F338" t="n">
-        <v>609518000</v>
+        <v>-18567000</v>
       </c>
       <c r="G338" t="n">
         <v>0</v>
       </c>
       <c r="H338" t="n">
-        <v>0</v>
+        <v>8.43</v>
       </c>
       <c r="I338" t="n">
-        <v>0</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="J338" t="n">
-        <v>0</v>
+        <v>36.09</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>CCTY3</t>
+          <t>BPAT33</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Empresa CCTY</t>
+          <t>Empresa BPAT</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -13965,7 +13965,7 @@
         </is>
       </c>
       <c r="D339" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -13973,7 +13973,7 @@
         </is>
       </c>
       <c r="F339" t="n">
-        <v>0</v>
+        <v>876492000</v>
       </c>
       <c r="G339" t="n">
         <v>0</v>
@@ -13991,12 +13991,12 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>VVAX4</t>
+          <t>REPA4</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -14005,7 +14005,7 @@
         </is>
       </c>
       <c r="D340" t="n">
-        <v>0</v>
+        <v>1.08</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -14013,39 +14013,39 @@
         </is>
       </c>
       <c r="F340" t="n">
-        <v>144676000</v>
+        <v>378378000</v>
       </c>
       <c r="G340" t="n">
         <v>0</v>
       </c>
       <c r="H340" t="n">
-        <v>-7.36</v>
+        <v>5.18</v>
       </c>
       <c r="I340" t="n">
-        <v>-6.52</v>
+        <v>4.05</v>
       </c>
       <c r="J340" t="n">
-        <v>-92.03</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>CSPC3</t>
+          <t>EQMA6B</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>1.24</v>
+        <v>0</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -14053,35 +14053,35 @@
         </is>
       </c>
       <c r="F341" t="n">
-        <v>2126670000</v>
+        <v>4940330000</v>
       </c>
       <c r="G341" t="n">
         <v>0</v>
       </c>
       <c r="H341" t="n">
-        <v>38.62</v>
+        <v>0</v>
       </c>
       <c r="I341" t="n">
-        <v>29.18</v>
+        <v>0</v>
       </c>
       <c r="J341" t="n">
-        <v>45.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>ABCB3</t>
+          <t>SEBB4</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Empresa ABCB</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D342" t="n">
@@ -14089,43 +14089,43 @@
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>Bancos</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="F342" t="n">
-        <v>7258910000</v>
+        <v>145783000</v>
       </c>
       <c r="G342" t="n">
         <v>0</v>
       </c>
       <c r="H342" t="n">
-        <v>0</v>
+        <v>9.24</v>
       </c>
       <c r="I342" t="n">
-        <v>0</v>
+        <v>24.15</v>
       </c>
       <c r="J342" t="n">
-        <v>14.05</v>
+        <v>23.01</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>ESTC4</t>
+          <t>MSAN3</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Empresa ESTC</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>0</v>
+        <v>6.44</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -14133,35 +14133,35 @@
         </is>
       </c>
       <c r="F343" t="n">
-        <v>2916530000</v>
+        <v>2533030000</v>
       </c>
       <c r="G343" t="n">
         <v>0</v>
       </c>
       <c r="H343" t="n">
-        <v>16.91</v>
+        <v>6.27</v>
       </c>
       <c r="I343" t="n">
-        <v>11.35</v>
+        <v>11.78</v>
       </c>
       <c r="J343" t="n">
-        <v>3.89</v>
+        <v>11.81</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>VSPT4</t>
+          <t>GALO3</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D344" t="n">
@@ -14173,39 +14173,39 @@
         </is>
       </c>
       <c r="F344" t="n">
-        <v>5031600000</v>
+        <v>-60607000</v>
       </c>
       <c r="G344" t="n">
         <v>0</v>
       </c>
       <c r="H344" t="n">
-        <v>0</v>
+        <v>13.98</v>
       </c>
       <c r="I344" t="n">
-        <v>0</v>
+        <v>39.37</v>
       </c>
       <c r="J344" t="n">
-        <v>0</v>
+        <v>7.62</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>BAUH4</t>
+          <t>SLCP3</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Empresa BAUH</t>
+          <t>Empresa SLCP</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>93.39</v>
+        <v>610.02</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -14213,10 +14213,10 @@
         </is>
       </c>
       <c r="F345" t="n">
-        <v>153407000</v>
+        <v>0</v>
       </c>
       <c r="G345" t="n">
-        <v>207.53</v>
+        <v>0</v>
       </c>
       <c r="H345" t="n">
         <v>0</v>
@@ -14231,12 +14231,12 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>ICPI3</t>
+          <t>DAYC3</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Empresa ICPI</t>
+          <t>Empresa DAYC</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
@@ -14253,7 +14253,7 @@
         </is>
       </c>
       <c r="F346" t="n">
-        <v>0</v>
+        <v>3009030000</v>
       </c>
       <c r="G346" t="n">
         <v>0</v>
@@ -14265,27 +14265,27 @@
         <v>0</v>
       </c>
       <c r="J346" t="n">
-        <v>0</v>
+        <v>17.33</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>ILLS4</t>
+          <t>PTIP3</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Empresa ILLS</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>100.01</v>
+        <v>22</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -14293,30 +14293,30 @@
         </is>
       </c>
       <c r="F347" t="n">
-        <v>-18567000</v>
+        <v>-155957000</v>
       </c>
       <c r="G347" t="n">
         <v>0</v>
       </c>
       <c r="H347" t="n">
-        <v>8.43</v>
+        <v>13.73</v>
       </c>
       <c r="I347" t="n">
-        <v>8.140000000000001</v>
+        <v>23.13</v>
       </c>
       <c r="J347" t="n">
-        <v>36.09</v>
+        <v>-121.74</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>BPAT33</t>
+          <t>MLPA3</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Empresa BPAT</t>
+          <t>Empresa MLPA</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
@@ -14325,7 +14325,7 @@
         </is>
       </c>
       <c r="D348" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -14333,30 +14333,30 @@
         </is>
       </c>
       <c r="F348" t="n">
-        <v>876492000</v>
+        <v>44578000</v>
       </c>
       <c r="G348" t="n">
         <v>0</v>
       </c>
       <c r="H348" t="n">
-        <v>0</v>
+        <v>6.66</v>
       </c>
       <c r="I348" t="n">
         <v>0</v>
       </c>
       <c r="J348" t="n">
-        <v>0</v>
+        <v>45.13</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>REPA4</t>
+          <t>CLSC6</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa CLSC</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
@@ -14365,7 +14365,7 @@
         </is>
       </c>
       <c r="D349" t="n">
-        <v>1.08</v>
+        <v>0</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -14373,39 +14373,39 @@
         </is>
       </c>
       <c r="F349" t="n">
-        <v>378378000</v>
+        <v>4228180000</v>
       </c>
       <c r="G349" t="n">
         <v>0</v>
       </c>
       <c r="H349" t="n">
-        <v>5.18</v>
+        <v>0</v>
       </c>
       <c r="I349" t="n">
-        <v>4.05</v>
+        <v>0</v>
       </c>
       <c r="J349" t="n">
-        <v>1.91</v>
+        <v>0</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>EQMA6B</t>
+          <t>SGEN3</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -14413,16 +14413,16 @@
         </is>
       </c>
       <c r="F350" t="n">
-        <v>4940330000</v>
+        <v>156981000</v>
       </c>
       <c r="G350" t="n">
         <v>0</v>
       </c>
       <c r="H350" t="n">
-        <v>0</v>
+        <v>-1871.17</v>
       </c>
       <c r="I350" t="n">
-        <v>0</v>
+        <v>-1.59</v>
       </c>
       <c r="J350" t="n">
         <v>0</v>
@@ -14431,12 +14431,12 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>SEBB4</t>
+          <t>DUFB11</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa DUFB</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -14453,39 +14453,39 @@
         </is>
       </c>
       <c r="F351" t="n">
-        <v>145783000</v>
+        <v>0</v>
       </c>
       <c r="G351" t="n">
         <v>0</v>
       </c>
       <c r="H351" t="n">
-        <v>9.24</v>
+        <v>0</v>
       </c>
       <c r="I351" t="n">
-        <v>24.15</v>
+        <v>0</v>
       </c>
       <c r="J351" t="n">
-        <v>23.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>MSAN3</t>
+          <t>TNEP4</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>6.44</v>
+        <v>3.95</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -14493,30 +14493,30 @@
         </is>
       </c>
       <c r="F352" t="n">
-        <v>2533030000</v>
+        <v>955105000</v>
       </c>
       <c r="G352" t="n">
         <v>0</v>
       </c>
       <c r="H352" t="n">
-        <v>6.27</v>
+        <v>20.92</v>
       </c>
       <c r="I352" t="n">
-        <v>11.78</v>
+        <v>20.53</v>
       </c>
       <c r="J352" t="n">
-        <v>11.81</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>GALO3</t>
+          <t>CCHI3</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -14525,7 +14525,7 @@
         </is>
       </c>
       <c r="D353" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -14533,30 +14533,30 @@
         </is>
       </c>
       <c r="F353" t="n">
-        <v>-60607000</v>
+        <v>-160477000</v>
       </c>
       <c r="G353" t="n">
         <v>0</v>
       </c>
       <c r="H353" t="n">
-        <v>13.98</v>
+        <v>0</v>
       </c>
       <c r="I353" t="n">
-        <v>39.37</v>
+        <v>0</v>
       </c>
       <c r="J353" t="n">
-        <v>7.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>SLCP3</t>
+          <t>SFSA3</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Empresa SLCP</t>
+          <t>Empresa SFSA</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -14565,7 +14565,7 @@
         </is>
       </c>
       <c r="D354" t="n">
-        <v>610.02</v>
+        <v>0</v>
       </c>
       <c r="E354" t="inlineStr">
         <is>
@@ -14573,7 +14573,7 @@
         </is>
       </c>
       <c r="F354" t="n">
-        <v>0</v>
+        <v>739524000</v>
       </c>
       <c r="G354" t="n">
         <v>0</v>
@@ -14585,18 +14585,18 @@
         <v>0</v>
       </c>
       <c r="J354" t="n">
-        <v>0</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>DAYC3</t>
+          <t>PRBC3</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Empresa DAYC</t>
+          <t>Empresa PRBC</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -14613,7 +14613,7 @@
         </is>
       </c>
       <c r="F355" t="n">
-        <v>3009030000</v>
+        <v>1319270000</v>
       </c>
       <c r="G355" t="n">
         <v>0</v>
@@ -14625,18 +14625,18 @@
         <v>0</v>
       </c>
       <c r="J355" t="n">
-        <v>17.33</v>
+        <v>8.27</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>PTIP3</t>
+          <t>ECIS3</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -14645,7 +14645,7 @@
         </is>
       </c>
       <c r="D356" t="n">
-        <v>22</v>
+        <v>211.65</v>
       </c>
       <c r="E356" t="inlineStr">
         <is>
@@ -14653,30 +14653,30 @@
         </is>
       </c>
       <c r="F356" t="n">
-        <v>-155957000</v>
+        <v>129346000</v>
       </c>
       <c r="G356" t="n">
         <v>0</v>
       </c>
       <c r="H356" t="n">
-        <v>13.73</v>
+        <v>34.9</v>
       </c>
       <c r="I356" t="n">
-        <v>23.13</v>
+        <v>12.48</v>
       </c>
       <c r="J356" t="n">
-        <v>-121.74</v>
+        <v>7.33</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>MLPA3</t>
+          <t>CBMA3</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Empresa MLPA</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -14685,7 +14685,7 @@
         </is>
       </c>
       <c r="D357" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -14693,39 +14693,39 @@
         </is>
       </c>
       <c r="F357" t="n">
-        <v>44578000</v>
+        <v>-34022300000</v>
       </c>
       <c r="G357" t="n">
         <v>0</v>
       </c>
       <c r="H357" t="n">
-        <v>6.66</v>
+        <v>0</v>
       </c>
       <c r="I357" t="n">
         <v>0</v>
       </c>
       <c r="J357" t="n">
-        <v>45.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>CLSC6</t>
+          <t>ALBA3</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Empresa CLSC</t>
+          <t>Empresa ALBA</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D358" t="n">
-        <v>0</v>
+        <v>2.15</v>
       </c>
       <c r="E358" t="inlineStr">
         <is>
@@ -14733,39 +14733,39 @@
         </is>
       </c>
       <c r="F358" t="n">
-        <v>4228180000</v>
+        <v>354860000</v>
       </c>
       <c r="G358" t="n">
         <v>0</v>
       </c>
       <c r="H358" t="n">
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="I358" t="n">
-        <v>0</v>
+        <v>20.4</v>
       </c>
       <c r="J358" t="n">
-        <v>0</v>
+        <v>19.77</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>SGEN3</t>
+          <t>ARPS4</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -14773,39 +14773,39 @@
         </is>
       </c>
       <c r="F359" t="n">
-        <v>156981000</v>
+        <v>-12690000</v>
       </c>
       <c r="G359" t="n">
         <v>0</v>
       </c>
       <c r="H359" t="n">
-        <v>-1871.17</v>
+        <v>-4.92</v>
       </c>
       <c r="I359" t="n">
-        <v>-1.59</v>
+        <v>-6.64</v>
       </c>
       <c r="J359" t="n">
-        <v>0</v>
+        <v>20.34</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>DUFB11</t>
+          <t>SALM3</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Empresa DUFB</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>0</v>
+        <v>5.7</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -14813,30 +14813,30 @@
         </is>
       </c>
       <c r="F360" t="n">
-        <v>0</v>
+        <v>475600000</v>
       </c>
       <c r="G360" t="n">
         <v>0</v>
       </c>
       <c r="H360" t="n">
-        <v>0</v>
+        <v>10.22</v>
       </c>
       <c r="I360" t="n">
-        <v>0</v>
+        <v>25.78</v>
       </c>
       <c r="J360" t="n">
-        <v>0</v>
+        <v>19.53</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>TNEP4</t>
+          <t>CMMA4</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa CMMA</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -14845,7 +14845,7 @@
         </is>
       </c>
       <c r="D361" t="n">
-        <v>3.95</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -14853,30 +14853,30 @@
         </is>
       </c>
       <c r="F361" t="n">
-        <v>955105000</v>
+        <v>-79623000</v>
       </c>
       <c r="G361" t="n">
         <v>0</v>
       </c>
       <c r="H361" t="n">
-        <v>20.92</v>
+        <v>0</v>
       </c>
       <c r="I361" t="n">
-        <v>20.53</v>
+        <v>0</v>
       </c>
       <c r="J361" t="n">
-        <v>22.8</v>
+        <v>-1.92</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>CCHI3</t>
+          <t>CZRS3</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa CZRS</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -14885,7 +14885,7 @@
         </is>
       </c>
       <c r="D362" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -14893,7 +14893,7 @@
         </is>
       </c>
       <c r="F362" t="n">
-        <v>-160477000</v>
+        <v>1145670000</v>
       </c>
       <c r="G362" t="n">
         <v>0</v>
@@ -14905,18 +14905,18 @@
         <v>0</v>
       </c>
       <c r="J362" t="n">
-        <v>0</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>SFSA3</t>
+          <t>BPNM3</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Empresa SFSA</t>
+          <t>Empresa BPNM</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -14933,7 +14933,7 @@
         </is>
       </c>
       <c r="F363" t="n">
-        <v>739524000</v>
+        <v>7792670000</v>
       </c>
       <c r="G363" t="n">
         <v>0</v>
@@ -14945,18 +14945,18 @@
         <v>0</v>
       </c>
       <c r="J363" t="n">
-        <v>6.25</v>
+        <v>9.67</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>PRBC3</t>
+          <t>BSGR3</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Empresa PRBC</t>
+          <t>Empresa BSGR</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -14965,7 +14965,7 @@
         </is>
       </c>
       <c r="D364" t="n">
-        <v>0</v>
+        <v>1091.28</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -14973,7 +14973,7 @@
         </is>
       </c>
       <c r="F364" t="n">
-        <v>1319270000</v>
+        <v>0</v>
       </c>
       <c r="G364" t="n">
         <v>0</v>
@@ -14985,18 +14985,18 @@
         <v>0</v>
       </c>
       <c r="J364" t="n">
-        <v>8.27</v>
+        <v>0</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>ECIS3</t>
+          <t>VNET3</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa VNET</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
@@ -15005,7 +15005,7 @@
         </is>
       </c>
       <c r="D365" t="n">
-        <v>211.65</v>
+        <v>0</v>
       </c>
       <c r="E365" t="inlineStr">
         <is>
@@ -15013,30 +15013,30 @@
         </is>
       </c>
       <c r="F365" t="n">
-        <v>129346000</v>
+        <v>14163000000</v>
       </c>
       <c r="G365" t="n">
         <v>0</v>
       </c>
       <c r="H365" t="n">
-        <v>34.9</v>
+        <v>0</v>
       </c>
       <c r="I365" t="n">
-        <v>12.48</v>
+        <v>0</v>
       </c>
       <c r="J365" t="n">
-        <v>7.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>ARPS4</t>
+          <t>CSPC4</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -15045,7 +15045,7 @@
         </is>
       </c>
       <c r="D366" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="E366" t="inlineStr">
         <is>
@@ -15053,30 +15053,30 @@
         </is>
       </c>
       <c r="F366" t="n">
-        <v>-12690000</v>
+        <v>2126670000</v>
       </c>
       <c r="G366" t="n">
         <v>0</v>
       </c>
       <c r="H366" t="n">
-        <v>-4.92</v>
+        <v>38.62</v>
       </c>
       <c r="I366" t="n">
-        <v>-6.64</v>
+        <v>29.18</v>
       </c>
       <c r="J366" t="n">
-        <v>20.34</v>
+        <v>45.33</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>SALM3</t>
+          <t>BOVH3</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa BOVH</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -15085,7 +15085,7 @@
         </is>
       </c>
       <c r="D367" t="n">
-        <v>5.7</v>
+        <v>15.71</v>
       </c>
       <c r="E367" t="inlineStr">
         <is>
@@ -15093,39 +15093,39 @@
         </is>
       </c>
       <c r="F367" t="n">
-        <v>475600000</v>
+        <v>1843320000</v>
       </c>
       <c r="G367" t="n">
         <v>0</v>
       </c>
       <c r="H367" t="n">
-        <v>10.22</v>
+        <v>0</v>
       </c>
       <c r="I367" t="n">
-        <v>25.78</v>
+        <v>0</v>
       </c>
       <c r="J367" t="n">
-        <v>19.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>CMMA4</t>
+          <t>ARND3</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Empresa CMMA</t>
+          <t>Empresa ARND</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D368" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.51</v>
       </c>
       <c r="E368" t="inlineStr">
         <is>
@@ -15133,10 +15133,10 @@
         </is>
       </c>
       <c r="F368" t="n">
-        <v>-79623000</v>
+        <v>125211000</v>
       </c>
       <c r="G368" t="n">
-        <v>0</v>
+        <v>913.58</v>
       </c>
       <c r="H368" t="n">
         <v>0</v>
@@ -15145,18 +15145,18 @@
         <v>0</v>
       </c>
       <c r="J368" t="n">
-        <v>-1.92</v>
+        <v>0</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>CZRS3</t>
+          <t>VVAX3</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Empresa CZRS</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -15173,39 +15173,39 @@
         </is>
       </c>
       <c r="F369" t="n">
-        <v>1145670000</v>
+        <v>144676000</v>
       </c>
       <c r="G369" t="n">
         <v>0</v>
       </c>
       <c r="H369" t="n">
-        <v>0</v>
+        <v>-7.36</v>
       </c>
       <c r="I369" t="n">
-        <v>0</v>
+        <v>-6.52</v>
       </c>
       <c r="J369" t="n">
-        <v>3.34</v>
+        <v>-92.03</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>BPNM3</t>
+          <t>MSAN4</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Empresa BPNM</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D370" t="n">
-        <v>0</v>
+        <v>6.44</v>
       </c>
       <c r="E370" t="inlineStr">
         <is>
@@ -15213,39 +15213,39 @@
         </is>
       </c>
       <c r="F370" t="n">
-        <v>7792670000</v>
+        <v>2533030000</v>
       </c>
       <c r="G370" t="n">
         <v>0</v>
       </c>
       <c r="H370" t="n">
-        <v>0</v>
+        <v>6.27</v>
       </c>
       <c r="I370" t="n">
-        <v>0</v>
+        <v>11.78</v>
       </c>
       <c r="J370" t="n">
-        <v>9.67</v>
+        <v>11.81</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>BSGR3</t>
+          <t>GALO4</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Empresa BSGR</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D371" t="n">
-        <v>1091.28</v>
+        <v>0.25</v>
       </c>
       <c r="E371" t="inlineStr">
         <is>
@@ -15253,30 +15253,30 @@
         </is>
       </c>
       <c r="F371" t="n">
-        <v>0</v>
+        <v>-60607000</v>
       </c>
       <c r="G371" t="n">
         <v>0</v>
       </c>
       <c r="H371" t="n">
-        <v>0</v>
+        <v>13.98</v>
       </c>
       <c r="I371" t="n">
-        <v>0</v>
+        <v>39.37</v>
       </c>
       <c r="J371" t="n">
-        <v>0</v>
+        <v>7.62</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>CBMA3</t>
+          <t>BBTG13</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
@@ -15285,7 +15285,7 @@
         </is>
       </c>
       <c r="D372" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="E372" t="inlineStr">
         <is>
@@ -15293,7 +15293,7 @@
         </is>
       </c>
       <c r="F372" t="n">
-        <v>-34022300000</v>
+        <v>7000</v>
       </c>
       <c r="G372" t="n">
         <v>0</v>
@@ -15305,18 +15305,18 @@
         <v>0</v>
       </c>
       <c r="J372" t="n">
-        <v>0</v>
+        <v>-42.86</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>ALBA3</t>
+          <t>INHA3</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Empresa ALBA</t>
+          <t>Empresa INHA</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
@@ -15325,7 +15325,7 @@
         </is>
       </c>
       <c r="D373" t="n">
-        <v>2.15</v>
+        <v>0</v>
       </c>
       <c r="E373" t="inlineStr">
         <is>
@@ -15333,39 +15333,39 @@
         </is>
       </c>
       <c r="F373" t="n">
-        <v>354860000</v>
+        <v>1533210000</v>
       </c>
       <c r="G373" t="n">
         <v>0</v>
       </c>
       <c r="H373" t="n">
-        <v>9.5</v>
+        <v>-56.05</v>
       </c>
       <c r="I373" t="n">
-        <v>20.4</v>
+        <v>-6.27</v>
       </c>
       <c r="J373" t="n">
-        <v>19.77</v>
+        <v>-39.87</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>VNET3</t>
+          <t>PTIP4</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>Empresa VNET</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D374" t="n">
-        <v>0</v>
+        <v>25.15</v>
       </c>
       <c r="E374" t="inlineStr">
         <is>
@@ -15373,39 +15373,39 @@
         </is>
       </c>
       <c r="F374" t="n">
-        <v>14163000000</v>
+        <v>-155957000</v>
       </c>
       <c r="G374" t="n">
         <v>0</v>
       </c>
       <c r="H374" t="n">
-        <v>0</v>
+        <v>13.73</v>
       </c>
       <c r="I374" t="n">
-        <v>0</v>
+        <v>23.13</v>
       </c>
       <c r="J374" t="n">
-        <v>0</v>
+        <v>-121.74</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>CSPC4</t>
+          <t>LATS3</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa LATS</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D375" t="n">
-        <v>1.2</v>
+        <v>22</v>
       </c>
       <c r="E375" t="inlineStr">
         <is>
@@ -15413,30 +15413,30 @@
         </is>
       </c>
       <c r="F375" t="n">
-        <v>2126670000</v>
+        <v>680646000</v>
       </c>
       <c r="G375" t="n">
         <v>0</v>
       </c>
       <c r="H375" t="n">
-        <v>38.62</v>
+        <v>11.74</v>
       </c>
       <c r="I375" t="n">
-        <v>29.18</v>
+        <v>11.63</v>
       </c>
       <c r="J375" t="n">
-        <v>45.33</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>BOVH3</t>
+          <t>VSPT3</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>Empresa BOVH</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
@@ -15445,7 +15445,7 @@
         </is>
       </c>
       <c r="D376" t="n">
-        <v>15.71</v>
+        <v>0</v>
       </c>
       <c r="E376" t="inlineStr">
         <is>
@@ -15453,7 +15453,7 @@
         </is>
       </c>
       <c r="F376" t="n">
-        <v>1843320000</v>
+        <v>5031600000</v>
       </c>
       <c r="G376" t="n">
         <v>0</v>
@@ -15471,21 +15471,21 @@
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>ARND3</t>
+          <t>SGEN4</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>Empresa ARND</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D377" t="n">
-        <v>0.51</v>
+        <v>0.6</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -15493,16 +15493,16 @@
         </is>
       </c>
       <c r="F377" t="n">
-        <v>125211000</v>
+        <v>156981000</v>
       </c>
       <c r="G377" t="n">
-        <v>913.58</v>
+        <v>0</v>
       </c>
       <c r="H377" t="n">
-        <v>0</v>
+        <v>-1871.17</v>
       </c>
       <c r="I377" t="n">
-        <v>0</v>
+        <v>-1.59</v>
       </c>
       <c r="J377" t="n">
         <v>0</v>
@@ -24591,7 +24591,7 @@
     <row r="605">
       <c r="A605" t="inlineStr">
         <is>
-          <t>RPAD3</t>
+          <t>RPAD6</t>
         </is>
       </c>
       <c r="B605" t="inlineStr">
@@ -24601,7 +24601,7 @@
       </c>
       <c r="C605" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D605" t="n">
@@ -24616,7 +24616,7 @@
         <v>1046150000</v>
       </c>
       <c r="G605" t="n">
-        <v>2695.56</v>
+        <v>2752.22</v>
       </c>
       <c r="H605" t="n">
         <v>0</v>
@@ -24631,7 +24631,7 @@
     <row r="606">
       <c r="A606" t="inlineStr">
         <is>
-          <t>RPAD6</t>
+          <t>RPAD3</t>
         </is>
       </c>
       <c r="B606" t="inlineStr">
@@ -24641,7 +24641,7 @@
       </c>
       <c r="C606" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D606" t="n">
@@ -24656,7 +24656,7 @@
         <v>1046150000</v>
       </c>
       <c r="G606" t="n">
-        <v>2752.22</v>
+        <v>2695.56</v>
       </c>
       <c r="H606" t="n">
         <v>0</v>
@@ -26529,7 +26529,7 @@
       </c>
       <c r="E653" t="inlineStr">
         <is>
-          <t>Seguradoras</t>
+          <t>Porto Seguro</t>
         </is>
       </c>
       <c r="F653" t="n">
@@ -26769,7 +26769,7 @@
       </c>
       <c r="E659" t="inlineStr">
         <is>
-          <t>Agro e Alimentos</t>
+          <t>M. Dias Branco</t>
         </is>
       </c>
       <c r="F659" t="n">
@@ -34449,7 +34449,7 @@
       </c>
       <c r="E851" t="inlineStr">
         <is>
-          <t>Agro e Alimentos</t>
+          <t>SLC Agrícola</t>
         </is>
       </c>
       <c r="F851" t="n">
@@ -34951,7 +34951,7 @@
     <row r="864">
       <c r="A864" t="inlineStr">
         <is>
-          <t>RSIP3</t>
+          <t>RSIP4</t>
         </is>
       </c>
       <c r="B864" t="inlineStr">
@@ -34961,7 +34961,7 @@
       </c>
       <c r="C864" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D864" t="n">
@@ -34991,7 +34991,7 @@
     <row r="865">
       <c r="A865" t="inlineStr">
         <is>
-          <t>RSIP4</t>
+          <t>RSIP3</t>
         </is>
       </c>
       <c r="B865" t="inlineStr">
@@ -35001,7 +35001,7 @@
       </c>
       <c r="C865" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D865" t="n">

</xml_diff>

<commit_message>
Adiciona checagem condicional no print e valida reordenacao de colunas
</commit_message>
<xml_diff>
--- a/acoes_b3.xlsx
+++ b/acoes_b3.xlsx
@@ -471,12 +471,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PORP4</t>
+          <t>CFLU4</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Empresa PORP</t>
+          <t>Empresa CFLU</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -485,7 +485,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2.4</v>
+        <v>1000</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -493,30 +493,30 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>22399000</v>
+        <v>60351000</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>17.68</v>
       </c>
       <c r="J2" t="n">
-        <v>-2.08</v>
+        <v>32.15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>IVTT3</t>
+          <t>CSTB3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Empresa IVTT</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -533,39 +533,39 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1083050000</v>
+        <v>8420670000</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>40.85</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>22.4</v>
       </c>
       <c r="J3" t="n">
-        <v>-0.4</v>
+        <v>20.11</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MNSA3</t>
+          <t>POPR4</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Empresa MNSA</t>
+          <t>Empresa POPR</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.42</v>
+        <v>10.17</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -573,39 +573,39 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>-9105000</v>
+        <v>545803000</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>-208.15</v>
+        <v>8.66</v>
       </c>
       <c r="I4" t="n">
-        <v>-13.5</v>
+        <v>15.25</v>
       </c>
       <c r="J4" t="n">
-        <v>145.7</v>
+        <v>19.93</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CFLU4</t>
+          <t>PMET3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Empresa CFLU</t>
+          <t>Empresa PMET</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -613,30 +613,30 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>60351000</v>
+        <v>-290863000</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>8.880000000000001</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>17.68</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>32.15</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CSTB3</t>
+          <t>CLAN3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa CLAN</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -653,30 +653,30 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>8420670000</v>
+        <v>1012240000</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>40.85</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>22.4</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>20.11</v>
+        <v>-1.05</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>POPR4</t>
+          <t>MNSA4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Empresa POPR</t>
+          <t>Empresa MNSA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>10.17</v>
+        <v>0.47</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -693,39 +693,39 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>545803000</v>
+        <v>-9105000</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>8.66</v>
+        <v>-208.15</v>
       </c>
       <c r="I7" t="n">
-        <v>15.25</v>
+        <v>-13.5</v>
       </c>
       <c r="J7" t="n">
-        <v>19.93</v>
+        <v>145.7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PMET3</t>
+          <t>CSTB4</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Empresa PMET</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>147.69</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -733,39 +733,39 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>-290863000</v>
+        <v>8420670000</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>40.85</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>22.4</v>
       </c>
       <c r="J8" t="n">
-        <v>4.1</v>
+        <v>20.11</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CLAN3</t>
+          <t>PORP4</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Empresa CLAN</t>
+          <t>Empresa PORP</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>1012240000</v>
+        <v>22399000</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -785,27 +785,27 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>-1.05</v>
+        <v>-2.08</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MNSA4</t>
+          <t>IVTT3</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Empresa MNSA</t>
+          <t>Empresa IVTT</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.47</v>
+        <v>0</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -813,39 +813,39 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>-9105000</v>
+        <v>1083050000</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>-208.15</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>-13.5</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>145.7</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CSTB4</t>
+          <t>MNSA3</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa MNSA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>147.69</v>
+        <v>0.42</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -853,19 +853,19 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>8420670000</v>
+        <v>-9105000</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>40.85</v>
+        <v>-208.15</v>
       </c>
       <c r="I11" t="n">
-        <v>22.4</v>
+        <v>-13.5</v>
       </c>
       <c r="J11" t="n">
-        <v>20.11</v>
+        <v>145.7</v>
       </c>
     </row>
     <row r="12">
@@ -6249,7 +6249,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Mineração e Siderurgia</t>
+          <t>Siderúrgica Nacional</t>
         </is>
       </c>
       <c r="F146" t="n">
@@ -6351,7 +6351,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>PNOR6</t>
+          <t>PNOR5</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -6391,7 +6391,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>PNOR5</t>
+          <t>PNOR6</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -6911,7 +6911,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>RNEW3</t>
+          <t>RNEW4</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -6921,7 +6921,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -6936,7 +6936,7 @@
         <v>1150280000</v>
       </c>
       <c r="G163" t="n">
-        <v>45273.4</v>
+        <v>44097</v>
       </c>
       <c r="H163" t="n">
         <v>-2.89</v>
@@ -6951,7 +6951,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>RNEW4</t>
+          <t>RNEW3</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -6961,7 +6961,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -6976,7 +6976,7 @@
         <v>1150280000</v>
       </c>
       <c r="G164" t="n">
-        <v>44097</v>
+        <v>45273.4</v>
       </c>
       <c r="H164" t="n">
         <v>-2.89</v>
@@ -7871,7 +7871,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>SDIA4</t>
+          <t>SDIA3</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -7881,7 +7881,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -7911,7 +7911,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>SDIA3</t>
+          <t>SDIA4</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -7921,7 +7921,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -12751,21 +12751,21 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>CCHI4</t>
+          <t>MLPA3</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa MLPA</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -12773,39 +12773,39 @@
         </is>
       </c>
       <c r="F309" t="n">
-        <v>-160477000</v>
+        <v>44578000</v>
       </c>
       <c r="G309" t="n">
         <v>0</v>
       </c>
       <c r="H309" t="n">
-        <v>0</v>
+        <v>6.66</v>
       </c>
       <c r="I309" t="n">
         <v>0</v>
       </c>
       <c r="J309" t="n">
-        <v>0</v>
+        <v>45.13</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>REPA3</t>
+          <t>CLSC6</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa CLSC</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -12813,39 +12813,39 @@
         </is>
       </c>
       <c r="F310" t="n">
-        <v>378378000</v>
+        <v>4228180000</v>
       </c>
       <c r="G310" t="n">
         <v>0</v>
       </c>
       <c r="H310" t="n">
-        <v>5.18</v>
+        <v>0</v>
       </c>
       <c r="I310" t="n">
-        <v>4.05</v>
+        <v>0</v>
       </c>
       <c r="J310" t="n">
-        <v>1.91</v>
+        <v>0</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>EQMA5B</t>
+          <t>SGEN3</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -12853,16 +12853,16 @@
         </is>
       </c>
       <c r="F311" t="n">
-        <v>4940330000</v>
+        <v>156981000</v>
       </c>
       <c r="G311" t="n">
         <v>0</v>
       </c>
       <c r="H311" t="n">
-        <v>0</v>
+        <v>-1871.17</v>
       </c>
       <c r="I311" t="n">
-        <v>0</v>
+        <v>-1.59</v>
       </c>
       <c r="J311" t="n">
         <v>0</v>
@@ -12871,17 +12871,17 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>SEBB3</t>
+          <t>DUFB11</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa DUFB</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D312" t="n">
@@ -12893,30 +12893,30 @@
         </is>
       </c>
       <c r="F312" t="n">
-        <v>145783000</v>
+        <v>0</v>
       </c>
       <c r="G312" t="n">
         <v>0</v>
       </c>
       <c r="H312" t="n">
-        <v>9.24</v>
+        <v>0</v>
       </c>
       <c r="I312" t="n">
-        <v>24.15</v>
+        <v>0</v>
       </c>
       <c r="J312" t="n">
-        <v>23.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>BBTG11</t>
+          <t>TNEP4</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -12925,7 +12925,7 @@
         </is>
       </c>
       <c r="D313" t="n">
-        <v>15.01</v>
+        <v>3.95</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -12933,39 +12933,39 @@
         </is>
       </c>
       <c r="F313" t="n">
-        <v>0</v>
+        <v>955105000</v>
       </c>
       <c r="G313" t="n">
         <v>0</v>
       </c>
       <c r="H313" t="n">
-        <v>0</v>
+        <v>20.92</v>
       </c>
       <c r="I313" t="n">
-        <v>0</v>
+        <v>20.53</v>
       </c>
       <c r="J313" t="n">
-        <v>0</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>JFAB4</t>
+          <t>CCHI3</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Empresa JFAB</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>0.06</v>
+        <v>0.02</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -12973,7 +12973,7 @@
         </is>
       </c>
       <c r="F314" t="n">
-        <v>-10183000</v>
+        <v>-160477000</v>
       </c>
       <c r="G314" t="n">
         <v>0</v>
@@ -12985,18 +12985,18 @@
         <v>0</v>
       </c>
       <c r="J314" t="n">
-        <v>2.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>LECO3</t>
+          <t>SFSA3</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Empresa LECO</t>
+          <t>Empresa SFSA</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -13013,30 +13013,30 @@
         </is>
       </c>
       <c r="F315" t="n">
-        <v>105928000</v>
+        <v>739524000</v>
       </c>
       <c r="G315" t="n">
         <v>0</v>
       </c>
       <c r="H315" t="n">
-        <v>-2.14</v>
+        <v>0</v>
       </c>
       <c r="I315" t="n">
-        <v>-3.48</v>
+        <v>0</v>
       </c>
       <c r="J315" t="n">
-        <v>-14.82</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>VGOR3</t>
+          <t>PRBC3</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Empresa VGOR</t>
+          <t>Empresa PRBC</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -13053,30 +13053,30 @@
         </is>
       </c>
       <c r="F316" t="n">
-        <v>135178000</v>
+        <v>1319270000</v>
       </c>
       <c r="G316" t="n">
         <v>0</v>
       </c>
       <c r="H316" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="I316" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J316" t="n">
-        <v>-24.29</v>
+        <v>8.27</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>GPIV33</t>
+          <t>ECIS3</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Empresa GPIV</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -13085,7 +13085,7 @@
         </is>
       </c>
       <c r="D317" t="n">
-        <v>4.42</v>
+        <v>211.65</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -13093,39 +13093,39 @@
         </is>
       </c>
       <c r="F317" t="n">
-        <v>1318490000</v>
+        <v>129346000</v>
       </c>
       <c r="G317" t="n">
         <v>0</v>
       </c>
       <c r="H317" t="n">
-        <v>257.32</v>
+        <v>34.9</v>
       </c>
       <c r="I317" t="n">
-        <v>-6.05</v>
+        <v>12.48</v>
       </c>
       <c r="J317" t="n">
-        <v>0</v>
+        <v>7.33</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>ECIS4</t>
+          <t>CBMA3</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>145</v>
+        <v>0.01</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -13133,30 +13133,30 @@
         </is>
       </c>
       <c r="F318" t="n">
-        <v>129346000</v>
+        <v>-34022300000</v>
       </c>
       <c r="G318" t="n">
         <v>0</v>
       </c>
       <c r="H318" t="n">
-        <v>34.9</v>
+        <v>0</v>
       </c>
       <c r="I318" t="n">
-        <v>12.48</v>
+        <v>0</v>
       </c>
       <c r="J318" t="n">
-        <v>7.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>TNEP3</t>
+          <t>ALBA3</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa ALBA</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -13165,7 +13165,7 @@
         </is>
       </c>
       <c r="D319" t="n">
-        <v>3.01</v>
+        <v>2.15</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -13173,30 +13173,30 @@
         </is>
       </c>
       <c r="F319" t="n">
-        <v>955105000</v>
+        <v>354860000</v>
       </c>
       <c r="G319" t="n">
         <v>0</v>
       </c>
       <c r="H319" t="n">
-        <v>20.92</v>
+        <v>9.5</v>
       </c>
       <c r="I319" t="n">
-        <v>20.53</v>
+        <v>20.4</v>
       </c>
       <c r="J319" t="n">
-        <v>22.8</v>
+        <v>19.77</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>CBMA4</t>
+          <t>ARPS4</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -13205,7 +13205,7 @@
         </is>
       </c>
       <c r="D320" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -13213,25 +13213,25 @@
         </is>
       </c>
       <c r="F320" t="n">
-        <v>-34022300000</v>
+        <v>-12690000</v>
       </c>
       <c r="G320" t="n">
         <v>0</v>
       </c>
       <c r="H320" t="n">
-        <v>0</v>
+        <v>-4.92</v>
       </c>
       <c r="I320" t="n">
-        <v>0</v>
+        <v>-6.64</v>
       </c>
       <c r="J320" t="n">
-        <v>0</v>
+        <v>20.34</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>SALM4</t>
+          <t>SALM3</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
@@ -13241,11 +13241,11 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -13271,21 +13271,21 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>BERG3</t>
+          <t>CMMA4</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Empresa BERG</t>
+          <t>Empresa CMMA</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>33</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -13293,30 +13293,30 @@
         </is>
       </c>
       <c r="F322" t="n">
-        <v>9538000</v>
+        <v>-79623000</v>
       </c>
       <c r="G322" t="n">
         <v>0</v>
       </c>
       <c r="H322" t="n">
-        <v>-8.6</v>
+        <v>0</v>
       </c>
       <c r="I322" t="n">
-        <v>-5.58</v>
+        <v>0</v>
       </c>
       <c r="J322" t="n">
-        <v>-102.71</v>
+        <v>-1.92</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>JBDU3</t>
+          <t>CZRS3</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Empresa JBDU</t>
+          <t>Empresa CZRS</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -13333,7 +13333,7 @@
         </is>
       </c>
       <c r="F323" t="n">
-        <v>56569000</v>
+        <v>1145670000</v>
       </c>
       <c r="G323" t="n">
         <v>0</v>
@@ -13345,18 +13345,18 @@
         <v>0</v>
       </c>
       <c r="J323" t="n">
-        <v>0</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>EGGY3</t>
+          <t>BPNM3</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Empresa EGGY</t>
+          <t>Empresa BPNM</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -13373,7 +13373,7 @@
         </is>
       </c>
       <c r="F324" t="n">
-        <v>954480000</v>
+        <v>7792670000</v>
       </c>
       <c r="G324" t="n">
         <v>0</v>
@@ -13385,18 +13385,18 @@
         <v>0</v>
       </c>
       <c r="J324" t="n">
-        <v>0</v>
+        <v>9.67</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>AGEI3</t>
+          <t>BSGR3</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Empresa AGEI</t>
+          <t>Empresa BSGR</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -13405,7 +13405,7 @@
         </is>
       </c>
       <c r="D325" t="n">
-        <v>7.8</v>
+        <v>1091.28</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -13413,7 +13413,7 @@
         </is>
       </c>
       <c r="F325" t="n">
-        <v>1878210000</v>
+        <v>0</v>
       </c>
       <c r="G325" t="n">
         <v>0</v>
@@ -13431,12 +13431,12 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>SASG3</t>
+          <t>VNET3</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Empresa SASG</t>
+          <t>Empresa VNET</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -13445,7 +13445,7 @@
         </is>
       </c>
       <c r="D326" t="n">
-        <v>0.98</v>
+        <v>0</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -13453,7 +13453,7 @@
         </is>
       </c>
       <c r="F326" t="n">
-        <v>0</v>
+        <v>14163000000</v>
       </c>
       <c r="G326" t="n">
         <v>0</v>
@@ -13471,21 +13471,21 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>BMEF3</t>
+          <t>CSPC4</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Empresa BMEF</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>11</v>
+        <v>1.2</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -13493,30 +13493,30 @@
         </is>
       </c>
       <c r="F327" t="n">
-        <v>2674780000</v>
+        <v>2126670000</v>
       </c>
       <c r="G327" t="n">
         <v>0</v>
       </c>
       <c r="H327" t="n">
-        <v>0</v>
+        <v>38.62</v>
       </c>
       <c r="I327" t="n">
-        <v>0</v>
+        <v>29.18</v>
       </c>
       <c r="J327" t="n">
-        <v>0</v>
+        <v>45.33</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>ARPS3</t>
+          <t>BOVH3</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa BOVH</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -13525,7 +13525,7 @@
         </is>
       </c>
       <c r="D328" t="n">
-        <v>0.3</v>
+        <v>15.71</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -13533,30 +13533,30 @@
         </is>
       </c>
       <c r="F328" t="n">
-        <v>-12690000</v>
+        <v>1843320000</v>
       </c>
       <c r="G328" t="n">
         <v>0</v>
       </c>
       <c r="H328" t="n">
-        <v>-4.92</v>
+        <v>0</v>
       </c>
       <c r="I328" t="n">
-        <v>-6.64</v>
+        <v>0</v>
       </c>
       <c r="J328" t="n">
-        <v>20.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>ODER3</t>
+          <t>ARND3</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Empresa ODER</t>
+          <t>Empresa ARND</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -13565,7 +13565,7 @@
         </is>
       </c>
       <c r="D329" t="n">
-        <v>0</v>
+        <v>0.51</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -13573,10 +13573,10 @@
         </is>
       </c>
       <c r="F329" t="n">
-        <v>609518000</v>
+        <v>125211000</v>
       </c>
       <c r="G329" t="n">
-        <v>0</v>
+        <v>913.58</v>
       </c>
       <c r="H329" t="n">
         <v>0</v>
@@ -13591,12 +13591,12 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>CCTY3</t>
+          <t>VVAX3</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Empresa CCTY</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -13613,30 +13613,30 @@
         </is>
       </c>
       <c r="F330" t="n">
-        <v>0</v>
+        <v>144676000</v>
       </c>
       <c r="G330" t="n">
         <v>0</v>
       </c>
       <c r="H330" t="n">
-        <v>0</v>
+        <v>-7.36</v>
       </c>
       <c r="I330" t="n">
-        <v>0</v>
+        <v>-6.52</v>
       </c>
       <c r="J330" t="n">
-        <v>0</v>
+        <v>-92.03</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>VVAX4</t>
+          <t>MSAN4</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -13645,7 +13645,7 @@
         </is>
       </c>
       <c r="D331" t="n">
-        <v>0</v>
+        <v>6.44</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -13653,39 +13653,39 @@
         </is>
       </c>
       <c r="F331" t="n">
-        <v>144676000</v>
+        <v>2533030000</v>
       </c>
       <c r="G331" t="n">
         <v>0</v>
       </c>
       <c r="H331" t="n">
-        <v>-7.36</v>
+        <v>6.27</v>
       </c>
       <c r="I331" t="n">
-        <v>-6.52</v>
+        <v>11.78</v>
       </c>
       <c r="J331" t="n">
-        <v>-92.03</v>
+        <v>11.81</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>CSPC3</t>
+          <t>GALO4</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>1.24</v>
+        <v>0.25</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -13693,30 +13693,30 @@
         </is>
       </c>
       <c r="F332" t="n">
-        <v>2126670000</v>
+        <v>-60607000</v>
       </c>
       <c r="G332" t="n">
         <v>0</v>
       </c>
       <c r="H332" t="n">
-        <v>38.62</v>
+        <v>13.98</v>
       </c>
       <c r="I332" t="n">
-        <v>29.18</v>
+        <v>39.37</v>
       </c>
       <c r="J332" t="n">
-        <v>45.33</v>
+        <v>7.62</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>ABCB3</t>
+          <t>BBTG13</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Empresa ABCB</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -13729,11 +13729,11 @@
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>Bancos</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="F333" t="n">
-        <v>7258910000</v>
+        <v>7000</v>
       </c>
       <c r="G333" t="n">
         <v>0</v>
@@ -13745,23 +13745,23 @@
         <v>0</v>
       </c>
       <c r="J333" t="n">
-        <v>14.05</v>
+        <v>-42.86</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>ESTC4</t>
+          <t>INHA3</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Empresa ESTC</t>
+          <t>Empresa INHA</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D334" t="n">
@@ -13773,30 +13773,30 @@
         </is>
       </c>
       <c r="F334" t="n">
-        <v>2916530000</v>
+        <v>1533210000</v>
       </c>
       <c r="G334" t="n">
         <v>0</v>
       </c>
       <c r="H334" t="n">
-        <v>16.91</v>
+        <v>-56.05</v>
       </c>
       <c r="I334" t="n">
-        <v>11.35</v>
+        <v>-6.27</v>
       </c>
       <c r="J334" t="n">
-        <v>3.89</v>
+        <v>-39.87</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>VSPT4</t>
+          <t>PTIP4</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -13805,7 +13805,7 @@
         </is>
       </c>
       <c r="D335" t="n">
-        <v>0</v>
+        <v>25.15</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -13813,39 +13813,39 @@
         </is>
       </c>
       <c r="F335" t="n">
-        <v>5031600000</v>
+        <v>-155957000</v>
       </c>
       <c r="G335" t="n">
         <v>0</v>
       </c>
       <c r="H335" t="n">
-        <v>0</v>
+        <v>13.73</v>
       </c>
       <c r="I335" t="n">
-        <v>0</v>
+        <v>23.13</v>
       </c>
       <c r="J335" t="n">
-        <v>0</v>
+        <v>-121.74</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>BAUH4</t>
+          <t>LATS3</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Empresa BAUH</t>
+          <t>Empresa LATS</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>93.39</v>
+        <v>22</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -13853,30 +13853,30 @@
         </is>
       </c>
       <c r="F336" t="n">
-        <v>153407000</v>
+        <v>680646000</v>
       </c>
       <c r="G336" t="n">
-        <v>207.53</v>
+        <v>0</v>
       </c>
       <c r="H336" t="n">
-        <v>0</v>
+        <v>11.74</v>
       </c>
       <c r="I336" t="n">
-        <v>0</v>
+        <v>11.63</v>
       </c>
       <c r="J336" t="n">
-        <v>0</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>ICPI3</t>
+          <t>VSPT3</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Empresa ICPI</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -13893,7 +13893,7 @@
         </is>
       </c>
       <c r="F337" t="n">
-        <v>0</v>
+        <v>5031600000</v>
       </c>
       <c r="G337" t="n">
         <v>0</v>
@@ -13911,12 +13911,12 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>ILLS4</t>
+          <t>SGEN4</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Empresa ILLS</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -13925,7 +13925,7 @@
         </is>
       </c>
       <c r="D338" t="n">
-        <v>100.01</v>
+        <v>0.6</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -13933,39 +13933,39 @@
         </is>
       </c>
       <c r="F338" t="n">
-        <v>-18567000</v>
+        <v>156981000</v>
       </c>
       <c r="G338" t="n">
         <v>0</v>
       </c>
       <c r="H338" t="n">
-        <v>8.43</v>
+        <v>-1871.17</v>
       </c>
       <c r="I338" t="n">
-        <v>8.140000000000001</v>
+        <v>-1.59</v>
       </c>
       <c r="J338" t="n">
-        <v>36.09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>BPAT33</t>
+          <t>CCHI4</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Empresa BPAT</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>20</v>
+        <v>0.02</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -13973,7 +13973,7 @@
         </is>
       </c>
       <c r="F339" t="n">
-        <v>876492000</v>
+        <v>-160477000</v>
       </c>
       <c r="G339" t="n">
         <v>0</v>
@@ -13991,7 +13991,7 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>REPA4</t>
+          <t>REPA3</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
@@ -14001,11 +14001,11 @@
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D340" t="n">
-        <v>1.08</v>
+        <v>1</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -14031,7 +14031,7 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>EQMA6B</t>
+          <t>EQMA5B</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
@@ -14071,7 +14071,7 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>SEBB4</t>
+          <t>SEBB3</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
@@ -14081,7 +14081,7 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D342" t="n">
@@ -14111,21 +14111,21 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>MSAN3</t>
+          <t>BBTG11</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>6.44</v>
+        <v>15.01</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -14133,39 +14133,39 @@
         </is>
       </c>
       <c r="F343" t="n">
-        <v>2533030000</v>
+        <v>0</v>
       </c>
       <c r="G343" t="n">
         <v>0</v>
       </c>
       <c r="H343" t="n">
-        <v>6.27</v>
+        <v>0</v>
       </c>
       <c r="I343" t="n">
-        <v>11.78</v>
+        <v>0</v>
       </c>
       <c r="J343" t="n">
-        <v>11.81</v>
+        <v>0</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>GALO3</t>
+          <t>JFAB4</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa JFAB</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>0</v>
+        <v>0.06</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -14173,30 +14173,30 @@
         </is>
       </c>
       <c r="F344" t="n">
-        <v>-60607000</v>
+        <v>-10183000</v>
       </c>
       <c r="G344" t="n">
         <v>0</v>
       </c>
       <c r="H344" t="n">
-        <v>13.98</v>
+        <v>0</v>
       </c>
       <c r="I344" t="n">
-        <v>39.37</v>
+        <v>0</v>
       </c>
       <c r="J344" t="n">
-        <v>7.62</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>SLCP3</t>
+          <t>LECO3</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Empresa SLCP</t>
+          <t>Empresa LECO</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -14205,7 +14205,7 @@
         </is>
       </c>
       <c r="D345" t="n">
-        <v>610.02</v>
+        <v>0</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -14213,30 +14213,30 @@
         </is>
       </c>
       <c r="F345" t="n">
-        <v>0</v>
+        <v>105928000</v>
       </c>
       <c r="G345" t="n">
         <v>0</v>
       </c>
       <c r="H345" t="n">
-        <v>0</v>
+        <v>-2.14</v>
       </c>
       <c r="I345" t="n">
-        <v>0</v>
+        <v>-3.48</v>
       </c>
       <c r="J345" t="n">
-        <v>0</v>
+        <v>-14.82</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>DAYC3</t>
+          <t>VGOR3</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Empresa DAYC</t>
+          <t>Empresa VGOR</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
@@ -14253,30 +14253,30 @@
         </is>
       </c>
       <c r="F346" t="n">
-        <v>3009030000</v>
+        <v>135178000</v>
       </c>
       <c r="G346" t="n">
         <v>0</v>
       </c>
       <c r="H346" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="I346" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J346" t="n">
-        <v>17.33</v>
+        <v>-24.29</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>PTIP3</t>
+          <t>GPIV33</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa GPIV</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
@@ -14285,7 +14285,7 @@
         </is>
       </c>
       <c r="D347" t="n">
-        <v>22</v>
+        <v>4.42</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -14293,39 +14293,39 @@
         </is>
       </c>
       <c r="F347" t="n">
-        <v>-155957000</v>
+        <v>1318490000</v>
       </c>
       <c r="G347" t="n">
         <v>0</v>
       </c>
       <c r="H347" t="n">
-        <v>13.73</v>
+        <v>257.32</v>
       </c>
       <c r="I347" t="n">
-        <v>23.13</v>
+        <v>-6.05</v>
       </c>
       <c r="J347" t="n">
-        <v>-121.74</v>
+        <v>0</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>MLPA3</t>
+          <t>ECIS4</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Empresa MLPA</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -14333,39 +14333,39 @@
         </is>
       </c>
       <c r="F348" t="n">
-        <v>44578000</v>
+        <v>129346000</v>
       </c>
       <c r="G348" t="n">
         <v>0</v>
       </c>
       <c r="H348" t="n">
-        <v>6.66</v>
+        <v>34.9</v>
       </c>
       <c r="I348" t="n">
-        <v>0</v>
+        <v>12.48</v>
       </c>
       <c r="J348" t="n">
-        <v>45.13</v>
+        <v>7.33</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>CLSC6</t>
+          <t>TNEP3</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Empresa CLSC</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>0</v>
+        <v>3.01</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -14373,39 +14373,39 @@
         </is>
       </c>
       <c r="F349" t="n">
-        <v>4228180000</v>
+        <v>955105000</v>
       </c>
       <c r="G349" t="n">
         <v>0</v>
       </c>
       <c r="H349" t="n">
-        <v>0</v>
+        <v>20.92</v>
       </c>
       <c r="I349" t="n">
-        <v>0</v>
+        <v>20.53</v>
       </c>
       <c r="J349" t="n">
-        <v>0</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>SGEN3</t>
+          <t>CBMA4</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>5</v>
+        <v>0.01</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -14413,16 +14413,16 @@
         </is>
       </c>
       <c r="F350" t="n">
-        <v>156981000</v>
+        <v>-34022300000</v>
       </c>
       <c r="G350" t="n">
         <v>0</v>
       </c>
       <c r="H350" t="n">
-        <v>-1871.17</v>
+        <v>0</v>
       </c>
       <c r="I350" t="n">
-        <v>-1.59</v>
+        <v>0</v>
       </c>
       <c r="J350" t="n">
         <v>0</v>
@@ -14431,12 +14431,12 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>DUFB11</t>
+          <t>SALM4</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Empresa DUFB</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -14445,7 +14445,7 @@
         </is>
       </c>
       <c r="D351" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -14453,39 +14453,39 @@
         </is>
       </c>
       <c r="F351" t="n">
-        <v>0</v>
+        <v>475600000</v>
       </c>
       <c r="G351" t="n">
         <v>0</v>
       </c>
       <c r="H351" t="n">
-        <v>0</v>
+        <v>10.22</v>
       </c>
       <c r="I351" t="n">
-        <v>0</v>
+        <v>25.78</v>
       </c>
       <c r="J351" t="n">
-        <v>0</v>
+        <v>19.53</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>TNEP4</t>
+          <t>BERG3</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa BERG</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>3.95</v>
+        <v>33</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -14493,30 +14493,30 @@
         </is>
       </c>
       <c r="F352" t="n">
-        <v>955105000</v>
+        <v>9538000</v>
       </c>
       <c r="G352" t="n">
         <v>0</v>
       </c>
       <c r="H352" t="n">
-        <v>20.92</v>
+        <v>-8.6</v>
       </c>
       <c r="I352" t="n">
-        <v>20.53</v>
+        <v>-5.58</v>
       </c>
       <c r="J352" t="n">
-        <v>22.8</v>
+        <v>-102.71</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>CCHI3</t>
+          <t>JBDU3</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa JBDU</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -14525,7 +14525,7 @@
         </is>
       </c>
       <c r="D353" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -14533,7 +14533,7 @@
         </is>
       </c>
       <c r="F353" t="n">
-        <v>-160477000</v>
+        <v>56569000</v>
       </c>
       <c r="G353" t="n">
         <v>0</v>
@@ -14551,12 +14551,12 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>SFSA3</t>
+          <t>EGGY3</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Empresa SFSA</t>
+          <t>Empresa EGGY</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -14573,7 +14573,7 @@
         </is>
       </c>
       <c r="F354" t="n">
-        <v>739524000</v>
+        <v>954480000</v>
       </c>
       <c r="G354" t="n">
         <v>0</v>
@@ -14585,18 +14585,18 @@
         <v>0</v>
       </c>
       <c r="J354" t="n">
-        <v>6.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>PRBC3</t>
+          <t>AGEI3</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Empresa PRBC</t>
+          <t>Empresa AGEI</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -14605,7 +14605,7 @@
         </is>
       </c>
       <c r="D355" t="n">
-        <v>0</v>
+        <v>7.8</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -14613,7 +14613,7 @@
         </is>
       </c>
       <c r="F355" t="n">
-        <v>1319270000</v>
+        <v>1878210000</v>
       </c>
       <c r="G355" t="n">
         <v>0</v>
@@ -14625,18 +14625,18 @@
         <v>0</v>
       </c>
       <c r="J355" t="n">
-        <v>8.27</v>
+        <v>0</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>ECIS3</t>
+          <t>SASG3</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa SASG</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -14645,7 +14645,7 @@
         </is>
       </c>
       <c r="D356" t="n">
-        <v>211.65</v>
+        <v>0.98</v>
       </c>
       <c r="E356" t="inlineStr">
         <is>
@@ -14653,30 +14653,30 @@
         </is>
       </c>
       <c r="F356" t="n">
-        <v>129346000</v>
+        <v>0</v>
       </c>
       <c r="G356" t="n">
         <v>0</v>
       </c>
       <c r="H356" t="n">
-        <v>34.9</v>
+        <v>0</v>
       </c>
       <c r="I356" t="n">
-        <v>12.48</v>
+        <v>0</v>
       </c>
       <c r="J356" t="n">
-        <v>7.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>CBMA3</t>
+          <t>BMEF3</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa BMEF</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -14685,7 +14685,7 @@
         </is>
       </c>
       <c r="D357" t="n">
-        <v>0.01</v>
+        <v>11</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -14693,7 +14693,7 @@
         </is>
       </c>
       <c r="F357" t="n">
-        <v>-34022300000</v>
+        <v>2674780000</v>
       </c>
       <c r="G357" t="n">
         <v>0</v>
@@ -14711,12 +14711,12 @@
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>ALBA3</t>
+          <t>ARPS3</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Empresa ALBA</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -14725,7 +14725,7 @@
         </is>
       </c>
       <c r="D358" t="n">
-        <v>2.15</v>
+        <v>0.3</v>
       </c>
       <c r="E358" t="inlineStr">
         <is>
@@ -14733,35 +14733,35 @@
         </is>
       </c>
       <c r="F358" t="n">
-        <v>354860000</v>
+        <v>-12690000</v>
       </c>
       <c r="G358" t="n">
         <v>0</v>
       </c>
       <c r="H358" t="n">
-        <v>9.5</v>
+        <v>-4.92</v>
       </c>
       <c r="I358" t="n">
-        <v>20.4</v>
+        <v>-6.64</v>
       </c>
       <c r="J358" t="n">
-        <v>19.77</v>
+        <v>20.34</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>ARPS4</t>
+          <t>ODER3</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa ODER</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D359" t="n">
@@ -14773,30 +14773,30 @@
         </is>
       </c>
       <c r="F359" t="n">
-        <v>-12690000</v>
+        <v>609518000</v>
       </c>
       <c r="G359" t="n">
         <v>0</v>
       </c>
       <c r="H359" t="n">
-        <v>-4.92</v>
+        <v>0</v>
       </c>
       <c r="I359" t="n">
-        <v>-6.64</v>
+        <v>0</v>
       </c>
       <c r="J359" t="n">
-        <v>20.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>SALM3</t>
+          <t>CCTY3</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa CCTY</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
@@ -14805,7 +14805,7 @@
         </is>
       </c>
       <c r="D360" t="n">
-        <v>5.7</v>
+        <v>0</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -14813,30 +14813,30 @@
         </is>
       </c>
       <c r="F360" t="n">
-        <v>475600000</v>
+        <v>0</v>
       </c>
       <c r="G360" t="n">
         <v>0</v>
       </c>
       <c r="H360" t="n">
-        <v>10.22</v>
+        <v>0</v>
       </c>
       <c r="I360" t="n">
-        <v>25.78</v>
+        <v>0</v>
       </c>
       <c r="J360" t="n">
-        <v>19.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>CMMA4</t>
+          <t>VVAX4</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Empresa CMMA</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -14845,7 +14845,7 @@
         </is>
       </c>
       <c r="D361" t="n">
-        <v>0.8100000000000001</v>
+        <v>0</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -14853,30 +14853,30 @@
         </is>
       </c>
       <c r="F361" t="n">
-        <v>-79623000</v>
+        <v>144676000</v>
       </c>
       <c r="G361" t="n">
         <v>0</v>
       </c>
       <c r="H361" t="n">
-        <v>0</v>
+        <v>-7.36</v>
       </c>
       <c r="I361" t="n">
-        <v>0</v>
+        <v>-6.52</v>
       </c>
       <c r="J361" t="n">
-        <v>-1.92</v>
+        <v>-92.03</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>CZRS3</t>
+          <t>CSPC3</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>Empresa CZRS</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -14885,7 +14885,7 @@
         </is>
       </c>
       <c r="D362" t="n">
-        <v>0</v>
+        <v>1.24</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -14893,30 +14893,30 @@
         </is>
       </c>
       <c r="F362" t="n">
-        <v>1145670000</v>
+        <v>2126670000</v>
       </c>
       <c r="G362" t="n">
         <v>0</v>
       </c>
       <c r="H362" t="n">
-        <v>0</v>
+        <v>38.62</v>
       </c>
       <c r="I362" t="n">
-        <v>0</v>
+        <v>29.18</v>
       </c>
       <c r="J362" t="n">
-        <v>3.34</v>
+        <v>45.33</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>BPNM3</t>
+          <t>ABCB3</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Empresa BPNM</t>
+          <t>Empresa ABCB</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -14929,11 +14929,11 @@
       </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="F363" t="n">
-        <v>7792670000</v>
+        <v>7258910000</v>
       </c>
       <c r="G363" t="n">
         <v>0</v>
@@ -14945,27 +14945,27 @@
         <v>0</v>
       </c>
       <c r="J363" t="n">
-        <v>9.67</v>
+        <v>14.05</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>BSGR3</t>
+          <t>ESTC4</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Empresa BSGR</t>
+          <t>Empresa ESTC</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D364" t="n">
-        <v>1091.28</v>
+        <v>0</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -14973,35 +14973,35 @@
         </is>
       </c>
       <c r="F364" t="n">
-        <v>0</v>
+        <v>2916530000</v>
       </c>
       <c r="G364" t="n">
         <v>0</v>
       </c>
       <c r="H364" t="n">
-        <v>0</v>
+        <v>16.91</v>
       </c>
       <c r="I364" t="n">
-        <v>0</v>
+        <v>11.35</v>
       </c>
       <c r="J364" t="n">
-        <v>0</v>
+        <v>3.89</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>VNET3</t>
+          <t>VSPT4</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Empresa VNET</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D365" t="n">
@@ -15013,7 +15013,7 @@
         </is>
       </c>
       <c r="F365" t="n">
-        <v>14163000000</v>
+        <v>5031600000</v>
       </c>
       <c r="G365" t="n">
         <v>0</v>
@@ -15031,12 +15031,12 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>CSPC4</t>
+          <t>BAUH4</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa BAUH</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -15045,7 +15045,7 @@
         </is>
       </c>
       <c r="D366" t="n">
-        <v>1.2</v>
+        <v>93.39</v>
       </c>
       <c r="E366" t="inlineStr">
         <is>
@@ -15053,30 +15053,30 @@
         </is>
       </c>
       <c r="F366" t="n">
-        <v>2126670000</v>
+        <v>153407000</v>
       </c>
       <c r="G366" t="n">
-        <v>0</v>
+        <v>207.53</v>
       </c>
       <c r="H366" t="n">
-        <v>38.62</v>
+        <v>0</v>
       </c>
       <c r="I366" t="n">
-        <v>29.18</v>
+        <v>0</v>
       </c>
       <c r="J366" t="n">
-        <v>45.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>BOVH3</t>
+          <t>ICPI3</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Empresa BOVH</t>
+          <t>Empresa ICPI</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -15085,7 +15085,7 @@
         </is>
       </c>
       <c r="D367" t="n">
-        <v>15.71</v>
+        <v>0</v>
       </c>
       <c r="E367" t="inlineStr">
         <is>
@@ -15093,7 +15093,7 @@
         </is>
       </c>
       <c r="F367" t="n">
-        <v>1843320000</v>
+        <v>0</v>
       </c>
       <c r="G367" t="n">
         <v>0</v>
@@ -15111,21 +15111,21 @@
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>ARND3</t>
+          <t>ILLS4</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Empresa ARND</t>
+          <t>Empresa ILLS</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D368" t="n">
-        <v>0.51</v>
+        <v>100.01</v>
       </c>
       <c r="E368" t="inlineStr">
         <is>
@@ -15133,30 +15133,30 @@
         </is>
       </c>
       <c r="F368" t="n">
-        <v>125211000</v>
+        <v>-18567000</v>
       </c>
       <c r="G368" t="n">
-        <v>913.58</v>
+        <v>0</v>
       </c>
       <c r="H368" t="n">
-        <v>0</v>
+        <v>8.43</v>
       </c>
       <c r="I368" t="n">
-        <v>0</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="J368" t="n">
-        <v>0</v>
+        <v>36.09</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>VVAX3</t>
+          <t>BPAT33</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa BPAT</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -15165,7 +15165,7 @@
         </is>
       </c>
       <c r="D369" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="E369" t="inlineStr">
         <is>
@@ -15173,30 +15173,30 @@
         </is>
       </c>
       <c r="F369" t="n">
-        <v>144676000</v>
+        <v>876492000</v>
       </c>
       <c r="G369" t="n">
         <v>0</v>
       </c>
       <c r="H369" t="n">
-        <v>-7.36</v>
+        <v>0</v>
       </c>
       <c r="I369" t="n">
-        <v>-6.52</v>
+        <v>0</v>
       </c>
       <c r="J369" t="n">
-        <v>-92.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>MSAN4</t>
+          <t>REPA4</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -15205,7 +15205,7 @@
         </is>
       </c>
       <c r="D370" t="n">
-        <v>6.44</v>
+        <v>1.08</v>
       </c>
       <c r="E370" t="inlineStr">
         <is>
@@ -15213,30 +15213,30 @@
         </is>
       </c>
       <c r="F370" t="n">
-        <v>2533030000</v>
+        <v>378378000</v>
       </c>
       <c r="G370" t="n">
         <v>0</v>
       </c>
       <c r="H370" t="n">
-        <v>6.27</v>
+        <v>5.18</v>
       </c>
       <c r="I370" t="n">
-        <v>11.78</v>
+        <v>4.05</v>
       </c>
       <c r="J370" t="n">
-        <v>11.81</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>GALO4</t>
+          <t>EQMA6B</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
@@ -15245,7 +15245,7 @@
         </is>
       </c>
       <c r="D371" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="E371" t="inlineStr">
         <is>
@@ -15253,35 +15253,35 @@
         </is>
       </c>
       <c r="F371" t="n">
-        <v>-60607000</v>
+        <v>4940330000</v>
       </c>
       <c r="G371" t="n">
         <v>0</v>
       </c>
       <c r="H371" t="n">
-        <v>13.98</v>
+        <v>0</v>
       </c>
       <c r="I371" t="n">
-        <v>39.37</v>
+        <v>0</v>
       </c>
       <c r="J371" t="n">
-        <v>7.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>BBTG13</t>
+          <t>SEBB4</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D372" t="n">
@@ -15293,30 +15293,30 @@
         </is>
       </c>
       <c r="F372" t="n">
-        <v>7000</v>
+        <v>145783000</v>
       </c>
       <c r="G372" t="n">
         <v>0</v>
       </c>
       <c r="H372" t="n">
-        <v>0</v>
+        <v>9.24</v>
       </c>
       <c r="I372" t="n">
-        <v>0</v>
+        <v>24.15</v>
       </c>
       <c r="J372" t="n">
-        <v>-42.86</v>
+        <v>23.01</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>INHA3</t>
+          <t>MSAN3</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Empresa INHA</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
@@ -15325,7 +15325,7 @@
         </is>
       </c>
       <c r="D373" t="n">
-        <v>0</v>
+        <v>6.44</v>
       </c>
       <c r="E373" t="inlineStr">
         <is>
@@ -15333,39 +15333,39 @@
         </is>
       </c>
       <c r="F373" t="n">
-        <v>1533210000</v>
+        <v>2533030000</v>
       </c>
       <c r="G373" t="n">
         <v>0</v>
       </c>
       <c r="H373" t="n">
-        <v>-56.05</v>
+        <v>6.27</v>
       </c>
       <c r="I373" t="n">
-        <v>-6.27</v>
+        <v>11.78</v>
       </c>
       <c r="J373" t="n">
-        <v>-39.87</v>
+        <v>11.81</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>PTIP4</t>
+          <t>GALO3</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D374" t="n">
-        <v>25.15</v>
+        <v>0</v>
       </c>
       <c r="E374" t="inlineStr">
         <is>
@@ -15373,30 +15373,30 @@
         </is>
       </c>
       <c r="F374" t="n">
-        <v>-155957000</v>
+        <v>-60607000</v>
       </c>
       <c r="G374" t="n">
         <v>0</v>
       </c>
       <c r="H374" t="n">
-        <v>13.73</v>
+        <v>13.98</v>
       </c>
       <c r="I374" t="n">
-        <v>23.13</v>
+        <v>39.37</v>
       </c>
       <c r="J374" t="n">
-        <v>-121.74</v>
+        <v>7.62</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>LATS3</t>
+          <t>SLCP3</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>Empresa LATS</t>
+          <t>Empresa SLCP</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
@@ -15405,7 +15405,7 @@
         </is>
       </c>
       <c r="D375" t="n">
-        <v>22</v>
+        <v>610.02</v>
       </c>
       <c r="E375" t="inlineStr">
         <is>
@@ -15413,30 +15413,30 @@
         </is>
       </c>
       <c r="F375" t="n">
-        <v>680646000</v>
+        <v>0</v>
       </c>
       <c r="G375" t="n">
         <v>0</v>
       </c>
       <c r="H375" t="n">
-        <v>11.74</v>
+        <v>0</v>
       </c>
       <c r="I375" t="n">
-        <v>11.63</v>
+        <v>0</v>
       </c>
       <c r="J375" t="n">
-        <v>1.84</v>
+        <v>0</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>VSPT3</t>
+          <t>DAYC3</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa DAYC</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
@@ -15453,7 +15453,7 @@
         </is>
       </c>
       <c r="F376" t="n">
-        <v>5031600000</v>
+        <v>3009030000</v>
       </c>
       <c r="G376" t="n">
         <v>0</v>
@@ -15465,27 +15465,27 @@
         <v>0</v>
       </c>
       <c r="J376" t="n">
-        <v>0</v>
+        <v>17.33</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>SGEN4</t>
+          <t>PTIP3</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D377" t="n">
-        <v>0.6</v>
+        <v>22</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -15493,19 +15493,19 @@
         </is>
       </c>
       <c r="F377" t="n">
-        <v>156981000</v>
+        <v>-155957000</v>
       </c>
       <c r="G377" t="n">
         <v>0</v>
       </c>
       <c r="H377" t="n">
-        <v>-1871.17</v>
+        <v>13.73</v>
       </c>
       <c r="I377" t="n">
-        <v>-1.59</v>
+        <v>23.13</v>
       </c>
       <c r="J377" t="n">
-        <v>0</v>
+        <v>-121.74</v>
       </c>
     </row>
     <row r="378">
@@ -18071,7 +18071,7 @@
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>MMAQ3</t>
+          <t>MMAQ4</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
@@ -18081,7 +18081,7 @@
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D442" t="n">
@@ -18111,7 +18111,7 @@
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>MMAQ4</t>
+          <t>MMAQ3</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
@@ -18121,7 +18121,7 @@
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D443" t="n">
@@ -24071,7 +24071,7 @@
     <row r="592">
       <c r="A592" t="inlineStr">
         <is>
-          <t>GETT3</t>
+          <t>GETT4</t>
         </is>
       </c>
       <c r="B592" t="inlineStr">
@@ -24081,7 +24081,7 @@
       </c>
       <c r="C592" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D592" t="n">
@@ -24111,7 +24111,7 @@
     <row r="593">
       <c r="A593" t="inlineStr">
         <is>
-          <t>GETT4</t>
+          <t>GETT3</t>
         </is>
       </c>
       <c r="B593" t="inlineStr">
@@ -24121,7 +24121,7 @@
       </c>
       <c r="C593" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D593" t="n">
@@ -32329,7 +32329,7 @@
       </c>
       <c r="E798" t="inlineStr">
         <is>
-          <t>Mineração e Siderurgia</t>
+          <t>CSN Mineração</t>
         </is>
       </c>
       <c r="F798" t="n">
@@ -34951,7 +34951,7 @@
     <row r="864">
       <c r="A864" t="inlineStr">
         <is>
-          <t>RSIP4</t>
+          <t>RSIP3</t>
         </is>
       </c>
       <c r="B864" t="inlineStr">
@@ -34961,7 +34961,7 @@
       </c>
       <c r="C864" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D864" t="n">
@@ -34991,7 +34991,7 @@
     <row r="865">
       <c r="A865" t="inlineStr">
         <is>
-          <t>RSIP3</t>
+          <t>RSIP4</t>
         </is>
       </c>
       <c r="B865" t="inlineStr">
@@ -35001,7 +35001,7 @@
       </c>
       <c r="C865" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D865" t="n">
@@ -36591,7 +36591,7 @@
     <row r="905">
       <c r="A905" t="inlineStr">
         <is>
-          <t>BRGE11</t>
+          <t>BRGE5</t>
         </is>
       </c>
       <c r="B905" t="inlineStr">
@@ -36631,7 +36631,7 @@
     <row r="906">
       <c r="A906" t="inlineStr">
         <is>
-          <t>BRGE5</t>
+          <t>BRGE11</t>
         </is>
       </c>
       <c r="B906" t="inlineStr">
@@ -39311,7 +39311,7 @@
     <row r="973">
       <c r="A973" t="inlineStr">
         <is>
-          <t>PQUN4</t>
+          <t>PQUN3</t>
         </is>
       </c>
       <c r="B973" t="inlineStr">
@@ -39321,7 +39321,7 @@
       </c>
       <c r="C973" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D973" t="n">
@@ -39351,7 +39351,7 @@
     <row r="974">
       <c r="A974" t="inlineStr">
         <is>
-          <t>PQUN3</t>
+          <t>PQUN4</t>
         </is>
       </c>
       <c r="B974" t="inlineStr">
@@ -39361,7 +39361,7 @@
       </c>
       <c r="C974" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D974" t="n">

</xml_diff>

<commit_message>
Corrige extracao da Margem Liquida e sanitiza valores numéricos
</commit_message>
<xml_diff>
--- a/acoes_b3.xlsx
+++ b/acoes_b3.xlsx
@@ -471,12 +471,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CFLU4</t>
+          <t>PORP4</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Empresa CFLU</t>
+          <t>Empresa PORP</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -485,7 +485,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1000</v>
+        <v>2.4</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -493,30 +493,30 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>60351000</v>
+        <v>22399000</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>8.880000000000001</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>17.68</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>32.15</v>
+        <v>-2.08</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CSTB3</t>
+          <t>IVTT3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa IVTT</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -533,39 +533,39 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>8420670000</v>
+        <v>1083050000</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>40.85</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>22.4</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>20.11</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>POPR4</t>
+          <t>MNSA3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Empresa POPR</t>
+          <t>Empresa MNSA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>10.17</v>
+        <v>0.42</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -573,39 +573,39 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>545803000</v>
+        <v>-9105000</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>8.66</v>
+        <v>-208.15</v>
       </c>
       <c r="I4" t="n">
-        <v>15.25</v>
+        <v>-13.5</v>
       </c>
       <c r="J4" t="n">
-        <v>19.93</v>
+        <v>145.7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PMET3</t>
+          <t>CFLU4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Empresa PMET</t>
+          <t>Empresa CFLU</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -613,30 +613,30 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>-290863000</v>
+        <v>60351000</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>17.68</v>
       </c>
       <c r="J5" t="n">
-        <v>4.1</v>
+        <v>32.15</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CLAN3</t>
+          <t>CSTB3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Empresa CLAN</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -653,30 +653,30 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>1012240000</v>
+        <v>8420670000</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>40.85</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>22.4</v>
       </c>
       <c r="J6" t="n">
-        <v>-1.05</v>
+        <v>20.11</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MNSA4</t>
+          <t>POPR4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Empresa MNSA</t>
+          <t>Empresa POPR</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.47</v>
+        <v>10.17</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -693,39 +693,39 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>-9105000</v>
+        <v>545803000</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>-208.15</v>
+        <v>8.66</v>
       </c>
       <c r="I7" t="n">
-        <v>-13.5</v>
+        <v>15.25</v>
       </c>
       <c r="J7" t="n">
-        <v>145.7</v>
+        <v>19.93</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CSTB4</t>
+          <t>PMET3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa PMET</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>147.69</v>
+        <v>0</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -733,39 +733,39 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>8420670000</v>
+        <v>-290863000</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>40.85</v>
+        <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>22.4</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>20.11</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PORP4</t>
+          <t>CLAN3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Empresa PORP</t>
+          <t>Empresa CLAN</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2.4</v>
+        <v>0</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>22399000</v>
+        <v>1012240000</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -785,27 +785,27 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>-2.08</v>
+        <v>-1.05</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>IVTT3</t>
+          <t>MNSA4</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Empresa IVTT</t>
+          <t>Empresa MNSA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>0.47</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -813,39 +813,39 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>1083050000</v>
+        <v>-9105000</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>-208.15</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>-13.5</v>
       </c>
       <c r="J10" t="n">
-        <v>-0.4</v>
+        <v>145.7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MNSA3</t>
+          <t>CSTB4</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Empresa MNSA</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.42</v>
+        <v>147.69</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -853,19 +853,19 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>-9105000</v>
+        <v>8420670000</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>-208.15</v>
+        <v>40.85</v>
       </c>
       <c r="I11" t="n">
-        <v>-13.5</v>
+        <v>22.4</v>
       </c>
       <c r="J11" t="n">
-        <v>145.7</v>
+        <v>20.11</v>
       </c>
     </row>
     <row r="12">
@@ -6351,7 +6351,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>PNOR5</t>
+          <t>PNOR6</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -6391,7 +6391,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>PNOR6</t>
+          <t>PNOR5</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -6911,7 +6911,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>RNEW4</t>
+          <t>RNEW3</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -6921,7 +6921,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -6936,7 +6936,7 @@
         <v>1150280000</v>
       </c>
       <c r="G163" t="n">
-        <v>44097</v>
+        <v>45273.4</v>
       </c>
       <c r="H163" t="n">
         <v>-2.89</v>
@@ -6951,7 +6951,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>RNEW3</t>
+          <t>RNEW4</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -6961,7 +6961,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -6976,7 +6976,7 @@
         <v>1150280000</v>
       </c>
       <c r="G164" t="n">
-        <v>45273.4</v>
+        <v>44097</v>
       </c>
       <c r="H164" t="n">
         <v>-2.89</v>
@@ -7871,7 +7871,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>SDIA3</t>
+          <t>SDIA4</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -7881,7 +7881,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -7911,7 +7911,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>SDIA4</t>
+          <t>SDIA3</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -7921,7 +7921,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -12751,21 +12751,21 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>MLPA3</t>
+          <t>JFAB4</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Empresa MLPA</t>
+          <t>Empresa JFAB</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>0</v>
+        <v>0.06</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -12773,30 +12773,30 @@
         </is>
       </c>
       <c r="F309" t="n">
-        <v>44578000</v>
+        <v>-10183000</v>
       </c>
       <c r="G309" t="n">
         <v>0</v>
       </c>
       <c r="H309" t="n">
-        <v>6.66</v>
+        <v>0</v>
       </c>
       <c r="I309" t="n">
         <v>0</v>
       </c>
       <c r="J309" t="n">
-        <v>45.13</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>CLSC6</t>
+          <t>CCHI4</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Empresa CLSC</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -12805,7 +12805,7 @@
         </is>
       </c>
       <c r="D310" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -12813,7 +12813,7 @@
         </is>
       </c>
       <c r="F310" t="n">
-        <v>4228180000</v>
+        <v>-160477000</v>
       </c>
       <c r="G310" t="n">
         <v>0</v>
@@ -12831,12 +12831,12 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>SGEN3</t>
+          <t>REPA3</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -12845,7 +12845,7 @@
         </is>
       </c>
       <c r="D311" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -12853,30 +12853,30 @@
         </is>
       </c>
       <c r="F311" t="n">
-        <v>156981000</v>
+        <v>378378000</v>
       </c>
       <c r="G311" t="n">
         <v>0</v>
       </c>
       <c r="H311" t="n">
-        <v>-1871.17</v>
+        <v>5.18</v>
       </c>
       <c r="I311" t="n">
-        <v>-1.59</v>
+        <v>4.05</v>
       </c>
       <c r="J311" t="n">
-        <v>0</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>DUFB11</t>
+          <t>EQMA5B</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Empresa DUFB</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -12893,7 +12893,7 @@
         </is>
       </c>
       <c r="F312" t="n">
-        <v>0</v>
+        <v>4940330000</v>
       </c>
       <c r="G312" t="n">
         <v>0</v>
@@ -12911,21 +12911,21 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>TNEP4</t>
+          <t>SEBB3</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>3.95</v>
+        <v>0</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -12933,39 +12933,39 @@
         </is>
       </c>
       <c r="F313" t="n">
-        <v>955105000</v>
+        <v>145783000</v>
       </c>
       <c r="G313" t="n">
         <v>0</v>
       </c>
       <c r="H313" t="n">
-        <v>20.92</v>
+        <v>9.24</v>
       </c>
       <c r="I313" t="n">
-        <v>20.53</v>
+        <v>24.15</v>
       </c>
       <c r="J313" t="n">
-        <v>22.8</v>
+        <v>23.01</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>CCHI3</t>
+          <t>BBTG11</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>0.02</v>
+        <v>15.01</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -12973,7 +12973,7 @@
         </is>
       </c>
       <c r="F314" t="n">
-        <v>-160477000</v>
+        <v>0</v>
       </c>
       <c r="G314" t="n">
         <v>0</v>
@@ -12991,21 +12991,21 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>SFSA3</t>
+          <t>ECIS4</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Empresa SFSA</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -13013,30 +13013,30 @@
         </is>
       </c>
       <c r="F315" t="n">
-        <v>739524000</v>
+        <v>129346000</v>
       </c>
       <c r="G315" t="n">
         <v>0</v>
       </c>
       <c r="H315" t="n">
-        <v>0</v>
+        <v>34.9</v>
       </c>
       <c r="I315" t="n">
-        <v>0</v>
+        <v>12.48</v>
       </c>
       <c r="J315" t="n">
-        <v>6.25</v>
+        <v>7.33</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>PRBC3</t>
+          <t>TNEP3</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Empresa PRBC</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -13045,7 +13045,7 @@
         </is>
       </c>
       <c r="D316" t="n">
-        <v>0</v>
+        <v>3.01</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -13053,30 +13053,30 @@
         </is>
       </c>
       <c r="F316" t="n">
-        <v>1319270000</v>
+        <v>955105000</v>
       </c>
       <c r="G316" t="n">
         <v>0</v>
       </c>
       <c r="H316" t="n">
-        <v>0</v>
+        <v>20.92</v>
       </c>
       <c r="I316" t="n">
-        <v>0</v>
+        <v>20.53</v>
       </c>
       <c r="J316" t="n">
-        <v>8.27</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>ECIS3</t>
+          <t>LECO3</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa LECO</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -13085,7 +13085,7 @@
         </is>
       </c>
       <c r="D317" t="n">
-        <v>211.65</v>
+        <v>0</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -13093,30 +13093,30 @@
         </is>
       </c>
       <c r="F317" t="n">
-        <v>129346000</v>
+        <v>105928000</v>
       </c>
       <c r="G317" t="n">
         <v>0</v>
       </c>
       <c r="H317" t="n">
-        <v>34.9</v>
+        <v>-2.14</v>
       </c>
       <c r="I317" t="n">
-        <v>12.48</v>
+        <v>-3.48</v>
       </c>
       <c r="J317" t="n">
-        <v>7.33</v>
+        <v>-14.82</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>CBMA3</t>
+          <t>VGOR3</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa VGOR</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -13125,7 +13125,7 @@
         </is>
       </c>
       <c r="D318" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -13133,30 +13133,30 @@
         </is>
       </c>
       <c r="F318" t="n">
-        <v>-34022300000</v>
+        <v>135178000</v>
       </c>
       <c r="G318" t="n">
         <v>0</v>
       </c>
       <c r="H318" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="I318" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J318" t="n">
-        <v>0</v>
+        <v>-24.29</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>ALBA3</t>
+          <t>GPIV33</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Empresa ALBA</t>
+          <t>Empresa GPIV</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -13165,7 +13165,7 @@
         </is>
       </c>
       <c r="D319" t="n">
-        <v>2.15</v>
+        <v>4.42</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -13173,35 +13173,35 @@
         </is>
       </c>
       <c r="F319" t="n">
-        <v>354860000</v>
+        <v>1318490000</v>
       </c>
       <c r="G319" t="n">
         <v>0</v>
       </c>
       <c r="H319" t="n">
-        <v>9.5</v>
+        <v>257.32</v>
       </c>
       <c r="I319" t="n">
-        <v>20.4</v>
+        <v>-6.05</v>
       </c>
       <c r="J319" t="n">
-        <v>19.77</v>
+        <v>0</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>ARPS4</t>
+          <t>JBDU3</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa JBDU</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D320" t="n">
@@ -13213,30 +13213,30 @@
         </is>
       </c>
       <c r="F320" t="n">
-        <v>-12690000</v>
+        <v>56569000</v>
       </c>
       <c r="G320" t="n">
         <v>0</v>
       </c>
       <c r="H320" t="n">
-        <v>-4.92</v>
+        <v>0</v>
       </c>
       <c r="I320" t="n">
-        <v>-6.64</v>
+        <v>0</v>
       </c>
       <c r="J320" t="n">
-        <v>20.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>SALM3</t>
+          <t>EGGY3</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa EGGY</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -13245,7 +13245,7 @@
         </is>
       </c>
       <c r="D321" t="n">
-        <v>5.7</v>
+        <v>0</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -13253,30 +13253,30 @@
         </is>
       </c>
       <c r="F321" t="n">
-        <v>475600000</v>
+        <v>954480000</v>
       </c>
       <c r="G321" t="n">
         <v>0</v>
       </c>
       <c r="H321" t="n">
-        <v>10.22</v>
+        <v>0</v>
       </c>
       <c r="I321" t="n">
-        <v>25.78</v>
+        <v>0</v>
       </c>
       <c r="J321" t="n">
-        <v>19.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>CMMA4</t>
+          <t>CBMA4</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Empresa CMMA</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -13285,7 +13285,7 @@
         </is>
       </c>
       <c r="D322" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -13293,7 +13293,7 @@
         </is>
       </c>
       <c r="F322" t="n">
-        <v>-79623000</v>
+        <v>-34022300000</v>
       </c>
       <c r="G322" t="n">
         <v>0</v>
@@ -13305,27 +13305,27 @@
         <v>0</v>
       </c>
       <c r="J322" t="n">
-        <v>-1.92</v>
+        <v>0</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>CZRS3</t>
+          <t>SALM4</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Empresa CZRS</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D323" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -13333,30 +13333,30 @@
         </is>
       </c>
       <c r="F323" t="n">
-        <v>1145670000</v>
+        <v>475600000</v>
       </c>
       <c r="G323" t="n">
         <v>0</v>
       </c>
       <c r="H323" t="n">
-        <v>0</v>
+        <v>10.22</v>
       </c>
       <c r="I323" t="n">
-        <v>0</v>
+        <v>25.78</v>
       </c>
       <c r="J323" t="n">
-        <v>3.34</v>
+        <v>19.53</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>BPNM3</t>
+          <t>BERG3</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Empresa BPNM</t>
+          <t>Empresa BERG</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -13365,7 +13365,7 @@
         </is>
       </c>
       <c r="D324" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -13373,30 +13373,30 @@
         </is>
       </c>
       <c r="F324" t="n">
-        <v>7792670000</v>
+        <v>9538000</v>
       </c>
       <c r="G324" t="n">
         <v>0</v>
       </c>
       <c r="H324" t="n">
-        <v>0</v>
+        <v>-8.6</v>
       </c>
       <c r="I324" t="n">
-        <v>0</v>
+        <v>-5.58</v>
       </c>
       <c r="J324" t="n">
-        <v>9.67</v>
+        <v>-102.71</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>BSGR3</t>
+          <t>AGEI3</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Empresa BSGR</t>
+          <t>Empresa AGEI</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -13405,7 +13405,7 @@
         </is>
       </c>
       <c r="D325" t="n">
-        <v>1091.28</v>
+        <v>7.8</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -13413,7 +13413,7 @@
         </is>
       </c>
       <c r="F325" t="n">
-        <v>0</v>
+        <v>1878210000</v>
       </c>
       <c r="G325" t="n">
         <v>0</v>
@@ -13431,12 +13431,12 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>VNET3</t>
+          <t>SASG3</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Empresa VNET</t>
+          <t>Empresa SASG</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -13445,7 +13445,7 @@
         </is>
       </c>
       <c r="D326" t="n">
-        <v>0</v>
+        <v>0.98</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -13453,7 +13453,7 @@
         </is>
       </c>
       <c r="F326" t="n">
-        <v>14163000000</v>
+        <v>0</v>
       </c>
       <c r="G326" t="n">
         <v>0</v>
@@ -13471,21 +13471,21 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>CSPC4</t>
+          <t>BMEF3</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa BMEF</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>1.2</v>
+        <v>11</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -13493,30 +13493,30 @@
         </is>
       </c>
       <c r="F327" t="n">
-        <v>2126670000</v>
+        <v>2674780000</v>
       </c>
       <c r="G327" t="n">
         <v>0</v>
       </c>
       <c r="H327" t="n">
-        <v>38.62</v>
+        <v>0</v>
       </c>
       <c r="I327" t="n">
-        <v>29.18</v>
+        <v>0</v>
       </c>
       <c r="J327" t="n">
-        <v>45.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>BOVH3</t>
+          <t>ARPS3</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Empresa BOVH</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -13525,7 +13525,7 @@
         </is>
       </c>
       <c r="D328" t="n">
-        <v>15.71</v>
+        <v>0.3</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -13533,30 +13533,30 @@
         </is>
       </c>
       <c r="F328" t="n">
-        <v>1843320000</v>
+        <v>-12690000</v>
       </c>
       <c r="G328" t="n">
         <v>0</v>
       </c>
       <c r="H328" t="n">
-        <v>0</v>
+        <v>-4.92</v>
       </c>
       <c r="I328" t="n">
-        <v>0</v>
+        <v>-6.64</v>
       </c>
       <c r="J328" t="n">
-        <v>0</v>
+        <v>20.34</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>ARND3</t>
+          <t>ODER3</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Empresa ARND</t>
+          <t>Empresa ODER</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -13565,7 +13565,7 @@
         </is>
       </c>
       <c r="D329" t="n">
-        <v>0.51</v>
+        <v>0</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -13573,10 +13573,10 @@
         </is>
       </c>
       <c r="F329" t="n">
-        <v>125211000</v>
+        <v>609518000</v>
       </c>
       <c r="G329" t="n">
-        <v>913.58</v>
+        <v>0</v>
       </c>
       <c r="H329" t="n">
         <v>0</v>
@@ -13591,12 +13591,12 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>VVAX3</t>
+          <t>ABCB3</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa ABCB</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -13609,43 +13609,43 @@
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="F330" t="n">
-        <v>144676000</v>
+        <v>7258910000</v>
       </c>
       <c r="G330" t="n">
         <v>0</v>
       </c>
       <c r="H330" t="n">
-        <v>-7.36</v>
+        <v>0</v>
       </c>
       <c r="I330" t="n">
-        <v>-6.52</v>
+        <v>0</v>
       </c>
       <c r="J330" t="n">
-        <v>-92.03</v>
+        <v>14.05</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>MSAN4</t>
+          <t>CCTY3</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa CCTY</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>6.44</v>
+        <v>0</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -13653,30 +13653,30 @@
         </is>
       </c>
       <c r="F331" t="n">
-        <v>2533030000</v>
+        <v>0</v>
       </c>
       <c r="G331" t="n">
         <v>0</v>
       </c>
       <c r="H331" t="n">
-        <v>6.27</v>
+        <v>0</v>
       </c>
       <c r="I331" t="n">
-        <v>11.78</v>
+        <v>0</v>
       </c>
       <c r="J331" t="n">
-        <v>11.81</v>
+        <v>0</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>GALO4</t>
+          <t>VVAX4</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -13685,7 +13685,7 @@
         </is>
       </c>
       <c r="D332" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -13693,30 +13693,30 @@
         </is>
       </c>
       <c r="F332" t="n">
-        <v>-60607000</v>
+        <v>144676000</v>
       </c>
       <c r="G332" t="n">
         <v>0</v>
       </c>
       <c r="H332" t="n">
-        <v>13.98</v>
+        <v>-7.36</v>
       </c>
       <c r="I332" t="n">
-        <v>39.37</v>
+        <v>-6.52</v>
       </c>
       <c r="J332" t="n">
-        <v>7.62</v>
+        <v>-92.03</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>BBTG13</t>
+          <t>CSPC3</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -13725,7 +13725,7 @@
         </is>
       </c>
       <c r="D333" t="n">
-        <v>0</v>
+        <v>1.24</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -13733,39 +13733,39 @@
         </is>
       </c>
       <c r="F333" t="n">
-        <v>7000</v>
+        <v>2126670000</v>
       </c>
       <c r="G333" t="n">
         <v>0</v>
       </c>
       <c r="H333" t="n">
-        <v>0</v>
+        <v>38.62</v>
       </c>
       <c r="I333" t="n">
-        <v>0</v>
+        <v>29.18</v>
       </c>
       <c r="J333" t="n">
-        <v>-42.86</v>
+        <v>45.33</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>INHA3</t>
+          <t>ILLS4</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Empresa INHA</t>
+          <t>Empresa ILLS</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>0</v>
+        <v>100.01</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -13773,39 +13773,39 @@
         </is>
       </c>
       <c r="F334" t="n">
-        <v>1533210000</v>
+        <v>-18567000</v>
       </c>
       <c r="G334" t="n">
         <v>0</v>
       </c>
       <c r="H334" t="n">
-        <v>-56.05</v>
+        <v>8.43</v>
       </c>
       <c r="I334" t="n">
-        <v>-6.27</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="J334" t="n">
-        <v>-39.87</v>
+        <v>36.09</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>PTIP4</t>
+          <t>BPAT33</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa BPAT</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>25.15</v>
+        <v>20</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -13813,39 +13813,39 @@
         </is>
       </c>
       <c r="F335" t="n">
-        <v>-155957000</v>
+        <v>876492000</v>
       </c>
       <c r="G335" t="n">
         <v>0</v>
       </c>
       <c r="H335" t="n">
-        <v>13.73</v>
+        <v>0</v>
       </c>
       <c r="I335" t="n">
-        <v>23.13</v>
+        <v>0</v>
       </c>
       <c r="J335" t="n">
-        <v>-121.74</v>
+        <v>0</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>LATS3</t>
+          <t>ESTC4</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Empresa LATS</t>
+          <t>Empresa ESTC</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -13853,25 +13853,25 @@
         </is>
       </c>
       <c r="F336" t="n">
-        <v>680646000</v>
+        <v>2916530000</v>
       </c>
       <c r="G336" t="n">
         <v>0</v>
       </c>
       <c r="H336" t="n">
-        <v>11.74</v>
+        <v>16.91</v>
       </c>
       <c r="I336" t="n">
-        <v>11.63</v>
+        <v>11.35</v>
       </c>
       <c r="J336" t="n">
-        <v>1.84</v>
+        <v>3.89</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>VSPT3</t>
+          <t>VSPT4</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
@@ -13881,7 +13881,7 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D337" t="n">
@@ -13911,12 +13911,12 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>SGEN4</t>
+          <t>BAUH4</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa BAUH</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -13925,7 +13925,7 @@
         </is>
       </c>
       <c r="D338" t="n">
-        <v>0.6</v>
+        <v>93.39</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -13933,16 +13933,16 @@
         </is>
       </c>
       <c r="F338" t="n">
-        <v>156981000</v>
+        <v>153407000</v>
       </c>
       <c r="G338" t="n">
-        <v>0</v>
+        <v>207.53</v>
       </c>
       <c r="H338" t="n">
-        <v>-1871.17</v>
+        <v>0</v>
       </c>
       <c r="I338" t="n">
-        <v>-1.59</v>
+        <v>0</v>
       </c>
       <c r="J338" t="n">
         <v>0</v>
@@ -13951,21 +13951,21 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>CCHI4</t>
+          <t>ICPI3</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa ICPI</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -13973,7 +13973,7 @@
         </is>
       </c>
       <c r="F339" t="n">
-        <v>-160477000</v>
+        <v>0</v>
       </c>
       <c r="G339" t="n">
         <v>0</v>
@@ -13991,12 +13991,12 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>REPA3</t>
+          <t>DAYC3</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa DAYC</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -14005,7 +14005,7 @@
         </is>
       </c>
       <c r="D340" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -14013,39 +14013,39 @@
         </is>
       </c>
       <c r="F340" t="n">
-        <v>378378000</v>
+        <v>3009030000</v>
       </c>
       <c r="G340" t="n">
         <v>0</v>
       </c>
       <c r="H340" t="n">
-        <v>5.18</v>
+        <v>0</v>
       </c>
       <c r="I340" t="n">
-        <v>4.05</v>
+        <v>0</v>
       </c>
       <c r="J340" t="n">
-        <v>1.91</v>
+        <v>17.33</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>EQMA5B</t>
+          <t>PTIP3</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -14053,39 +14053,39 @@
         </is>
       </c>
       <c r="F341" t="n">
-        <v>4940330000</v>
+        <v>-155957000</v>
       </c>
       <c r="G341" t="n">
         <v>0</v>
       </c>
       <c r="H341" t="n">
-        <v>0</v>
+        <v>13.73</v>
       </c>
       <c r="I341" t="n">
-        <v>0</v>
+        <v>23.13</v>
       </c>
       <c r="J341" t="n">
-        <v>0</v>
+        <v>-121.74</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>SEBB3</t>
+          <t>REPA4</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>0</v>
+        <v>1.08</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -14093,30 +14093,30 @@
         </is>
       </c>
       <c r="F342" t="n">
-        <v>145783000</v>
+        <v>378378000</v>
       </c>
       <c r="G342" t="n">
         <v>0</v>
       </c>
       <c r="H342" t="n">
-        <v>9.24</v>
+        <v>5.18</v>
       </c>
       <c r="I342" t="n">
-        <v>24.15</v>
+        <v>4.05</v>
       </c>
       <c r="J342" t="n">
-        <v>23.01</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>BBTG11</t>
+          <t>EQMA6B</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -14125,7 +14125,7 @@
         </is>
       </c>
       <c r="D343" t="n">
-        <v>15.01</v>
+        <v>0</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -14133,7 +14133,7 @@
         </is>
       </c>
       <c r="F343" t="n">
-        <v>0</v>
+        <v>4940330000</v>
       </c>
       <c r="G343" t="n">
         <v>0</v>
@@ -14151,12 +14151,12 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>JFAB4</t>
+          <t>SEBB4</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Empresa JFAB</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
@@ -14165,7 +14165,7 @@
         </is>
       </c>
       <c r="D344" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -14173,30 +14173,30 @@
         </is>
       </c>
       <c r="F344" t="n">
-        <v>-10183000</v>
+        <v>145783000</v>
       </c>
       <c r="G344" t="n">
         <v>0</v>
       </c>
       <c r="H344" t="n">
-        <v>0</v>
+        <v>9.24</v>
       </c>
       <c r="I344" t="n">
-        <v>0</v>
+        <v>24.15</v>
       </c>
       <c r="J344" t="n">
-        <v>2.34</v>
+        <v>23.01</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>LECO3</t>
+          <t>MSAN3</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Empresa LECO</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -14205,7 +14205,7 @@
         </is>
       </c>
       <c r="D345" t="n">
-        <v>0</v>
+        <v>6.44</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -14213,30 +14213,30 @@
         </is>
       </c>
       <c r="F345" t="n">
-        <v>105928000</v>
+        <v>2533030000</v>
       </c>
       <c r="G345" t="n">
         <v>0</v>
       </c>
       <c r="H345" t="n">
-        <v>-2.14</v>
+        <v>6.27</v>
       </c>
       <c r="I345" t="n">
-        <v>-3.48</v>
+        <v>11.78</v>
       </c>
       <c r="J345" t="n">
-        <v>-14.82</v>
+        <v>11.81</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>VGOR3</t>
+          <t>GALO3</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Empresa VGOR</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
@@ -14253,30 +14253,30 @@
         </is>
       </c>
       <c r="F346" t="n">
-        <v>135178000</v>
+        <v>-60607000</v>
       </c>
       <c r="G346" t="n">
         <v>0</v>
       </c>
       <c r="H346" t="n">
-        <v>4.5</v>
+        <v>13.98</v>
       </c>
       <c r="I346" t="n">
-        <v>6</v>
+        <v>39.37</v>
       </c>
       <c r="J346" t="n">
-        <v>-24.29</v>
+        <v>7.62</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>GPIV33</t>
+          <t>SLCP3</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Empresa GPIV</t>
+          <t>Empresa SLCP</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
@@ -14285,7 +14285,7 @@
         </is>
       </c>
       <c r="D347" t="n">
-        <v>4.42</v>
+        <v>610.02</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -14293,16 +14293,16 @@
         </is>
       </c>
       <c r="F347" t="n">
-        <v>1318490000</v>
+        <v>0</v>
       </c>
       <c r="G347" t="n">
         <v>0</v>
       </c>
       <c r="H347" t="n">
-        <v>257.32</v>
+        <v>0</v>
       </c>
       <c r="I347" t="n">
-        <v>-6.05</v>
+        <v>0</v>
       </c>
       <c r="J347" t="n">
         <v>0</v>
@@ -14311,12 +14311,12 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>ECIS4</t>
+          <t>DUFB11</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa DUFB</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
@@ -14325,7 +14325,7 @@
         </is>
       </c>
       <c r="D348" t="n">
-        <v>145</v>
+        <v>0</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -14333,25 +14333,25 @@
         </is>
       </c>
       <c r="F348" t="n">
-        <v>129346000</v>
+        <v>0</v>
       </c>
       <c r="G348" t="n">
         <v>0</v>
       </c>
       <c r="H348" t="n">
-        <v>34.9</v>
+        <v>0</v>
       </c>
       <c r="I348" t="n">
-        <v>12.48</v>
+        <v>0</v>
       </c>
       <c r="J348" t="n">
-        <v>7.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>TNEP3</t>
+          <t>TNEP4</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
@@ -14361,11 +14361,11 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>3.01</v>
+        <v>3.95</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -14391,21 +14391,21 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>CBMA4</t>
+          <t>MLPA3</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa MLPA</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -14413,30 +14413,30 @@
         </is>
       </c>
       <c r="F350" t="n">
-        <v>-34022300000</v>
+        <v>44578000</v>
       </c>
       <c r="G350" t="n">
         <v>0</v>
       </c>
       <c r="H350" t="n">
-        <v>0</v>
+        <v>6.66</v>
       </c>
       <c r="I350" t="n">
         <v>0</v>
       </c>
       <c r="J350" t="n">
-        <v>0</v>
+        <v>45.13</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>SALM4</t>
+          <t>CLSC6</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa CLSC</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -14445,7 +14445,7 @@
         </is>
       </c>
       <c r="D351" t="n">
-        <v>5.9</v>
+        <v>0</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -14453,30 +14453,30 @@
         </is>
       </c>
       <c r="F351" t="n">
-        <v>475600000</v>
+        <v>4228180000</v>
       </c>
       <c r="G351" t="n">
         <v>0</v>
       </c>
       <c r="H351" t="n">
-        <v>10.22</v>
+        <v>0</v>
       </c>
       <c r="I351" t="n">
-        <v>25.78</v>
+        <v>0</v>
       </c>
       <c r="J351" t="n">
-        <v>19.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>BERG3</t>
+          <t>SGEN3</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Empresa BERG</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -14485,7 +14485,7 @@
         </is>
       </c>
       <c r="D352" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -14493,30 +14493,30 @@
         </is>
       </c>
       <c r="F352" t="n">
-        <v>9538000</v>
+        <v>156981000</v>
       </c>
       <c r="G352" t="n">
         <v>0</v>
       </c>
       <c r="H352" t="n">
-        <v>-8.6</v>
+        <v>-1871.17</v>
       </c>
       <c r="I352" t="n">
-        <v>-5.58</v>
+        <v>-1.59</v>
       </c>
       <c r="J352" t="n">
-        <v>-102.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>JBDU3</t>
+          <t>CCHI3</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Empresa JBDU</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -14525,7 +14525,7 @@
         </is>
       </c>
       <c r="D353" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -14533,7 +14533,7 @@
         </is>
       </c>
       <c r="F353" t="n">
-        <v>56569000</v>
+        <v>-160477000</v>
       </c>
       <c r="G353" t="n">
         <v>0</v>
@@ -14551,12 +14551,12 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>EGGY3</t>
+          <t>PRBC3</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Empresa EGGY</t>
+          <t>Empresa PRBC</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -14573,7 +14573,7 @@
         </is>
       </c>
       <c r="F354" t="n">
-        <v>954480000</v>
+        <v>1319270000</v>
       </c>
       <c r="G354" t="n">
         <v>0</v>
@@ -14585,18 +14585,18 @@
         <v>0</v>
       </c>
       <c r="J354" t="n">
-        <v>0</v>
+        <v>8.27</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>AGEI3</t>
+          <t>ECIS3</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Empresa AGEI</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -14605,7 +14605,7 @@
         </is>
       </c>
       <c r="D355" t="n">
-        <v>7.8</v>
+        <v>211.65</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -14613,30 +14613,30 @@
         </is>
       </c>
       <c r="F355" t="n">
-        <v>1878210000</v>
+        <v>129346000</v>
       </c>
       <c r="G355" t="n">
         <v>0</v>
       </c>
       <c r="H355" t="n">
-        <v>0</v>
+        <v>34.9</v>
       </c>
       <c r="I355" t="n">
-        <v>0</v>
+        <v>12.48</v>
       </c>
       <c r="J355" t="n">
-        <v>0</v>
+        <v>7.33</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>SASG3</t>
+          <t>SFSA3</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Empresa SASG</t>
+          <t>Empresa SFSA</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -14645,7 +14645,7 @@
         </is>
       </c>
       <c r="D356" t="n">
-        <v>0.98</v>
+        <v>0</v>
       </c>
       <c r="E356" t="inlineStr">
         <is>
@@ -14653,7 +14653,7 @@
         </is>
       </c>
       <c r="F356" t="n">
-        <v>0</v>
+        <v>739524000</v>
       </c>
       <c r="G356" t="n">
         <v>0</v>
@@ -14665,18 +14665,18 @@
         <v>0</v>
       </c>
       <c r="J356" t="n">
-        <v>0</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>BMEF3</t>
+          <t>CZRS3</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Empresa BMEF</t>
+          <t>Empresa CZRS</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -14685,7 +14685,7 @@
         </is>
       </c>
       <c r="D357" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -14693,7 +14693,7 @@
         </is>
       </c>
       <c r="F357" t="n">
-        <v>2674780000</v>
+        <v>1145670000</v>
       </c>
       <c r="G357" t="n">
         <v>0</v>
@@ -14705,18 +14705,18 @@
         <v>0</v>
       </c>
       <c r="J357" t="n">
-        <v>0</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>ARPS3</t>
+          <t>BPNM3</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa BPNM</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -14725,7 +14725,7 @@
         </is>
       </c>
       <c r="D358" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="E358" t="inlineStr">
         <is>
@@ -14733,30 +14733,30 @@
         </is>
       </c>
       <c r="F358" t="n">
-        <v>-12690000</v>
+        <v>7792670000</v>
       </c>
       <c r="G358" t="n">
         <v>0</v>
       </c>
       <c r="H358" t="n">
-        <v>-4.92</v>
+        <v>0</v>
       </c>
       <c r="I358" t="n">
-        <v>-6.64</v>
+        <v>0</v>
       </c>
       <c r="J358" t="n">
-        <v>20.34</v>
+        <v>9.67</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>ODER3</t>
+          <t>BSGR3</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Empresa ODER</t>
+          <t>Empresa BSGR</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
@@ -14765,7 +14765,7 @@
         </is>
       </c>
       <c r="D359" t="n">
-        <v>0</v>
+        <v>1091.28</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -14773,7 +14773,7 @@
         </is>
       </c>
       <c r="F359" t="n">
-        <v>609518000</v>
+        <v>0</v>
       </c>
       <c r="G359" t="n">
         <v>0</v>
@@ -14791,12 +14791,12 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>CCTY3</t>
+          <t>CBMA3</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Empresa CCTY</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
@@ -14805,7 +14805,7 @@
         </is>
       </c>
       <c r="D360" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -14813,7 +14813,7 @@
         </is>
       </c>
       <c r="F360" t="n">
-        <v>0</v>
+        <v>-34022300000</v>
       </c>
       <c r="G360" t="n">
         <v>0</v>
@@ -14831,21 +14831,21 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>VVAX4</t>
+          <t>ALBA3</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa ALBA</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D361" t="n">
-        <v>0</v>
+        <v>2.15</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -14853,39 +14853,39 @@
         </is>
       </c>
       <c r="F361" t="n">
-        <v>144676000</v>
+        <v>354860000</v>
       </c>
       <c r="G361" t="n">
         <v>0</v>
       </c>
       <c r="H361" t="n">
-        <v>-7.36</v>
+        <v>9.5</v>
       </c>
       <c r="I361" t="n">
-        <v>-6.52</v>
+        <v>20.4</v>
       </c>
       <c r="J361" t="n">
-        <v>-92.03</v>
+        <v>19.77</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>CSPC3</t>
+          <t>ARPS4</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>1.24</v>
+        <v>0</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -14893,30 +14893,30 @@
         </is>
       </c>
       <c r="F362" t="n">
-        <v>2126670000</v>
+        <v>-12690000</v>
       </c>
       <c r="G362" t="n">
         <v>0</v>
       </c>
       <c r="H362" t="n">
-        <v>38.62</v>
+        <v>-4.92</v>
       </c>
       <c r="I362" t="n">
-        <v>29.18</v>
+        <v>-6.64</v>
       </c>
       <c r="J362" t="n">
-        <v>45.33</v>
+        <v>20.34</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>ABCB3</t>
+          <t>SALM3</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Empresa ABCB</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -14925,38 +14925,38 @@
         </is>
       </c>
       <c r="D363" t="n">
-        <v>0</v>
+        <v>5.7</v>
       </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t>Bancos</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="F363" t="n">
-        <v>7258910000</v>
+        <v>475600000</v>
       </c>
       <c r="G363" t="n">
         <v>0</v>
       </c>
       <c r="H363" t="n">
-        <v>0</v>
+        <v>10.22</v>
       </c>
       <c r="I363" t="n">
-        <v>0</v>
+        <v>25.78</v>
       </c>
       <c r="J363" t="n">
-        <v>14.05</v>
+        <v>19.53</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>ESTC4</t>
+          <t>CMMA4</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Empresa ESTC</t>
+          <t>Empresa CMMA</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -14965,7 +14965,7 @@
         </is>
       </c>
       <c r="D364" t="n">
-        <v>0</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -14973,39 +14973,39 @@
         </is>
       </c>
       <c r="F364" t="n">
-        <v>2916530000</v>
+        <v>-79623000</v>
       </c>
       <c r="G364" t="n">
         <v>0</v>
       </c>
       <c r="H364" t="n">
-        <v>16.91</v>
+        <v>0</v>
       </c>
       <c r="I364" t="n">
-        <v>11.35</v>
+        <v>0</v>
       </c>
       <c r="J364" t="n">
-        <v>3.89</v>
+        <v>-1.92</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>VSPT4</t>
+          <t>BOVH3</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa BOVH</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D365" t="n">
-        <v>0</v>
+        <v>15.71</v>
       </c>
       <c r="E365" t="inlineStr">
         <is>
@@ -15013,7 +15013,7 @@
         </is>
       </c>
       <c r="F365" t="n">
-        <v>5031600000</v>
+        <v>1843320000</v>
       </c>
       <c r="G365" t="n">
         <v>0</v>
@@ -15031,21 +15031,21 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>BAUH4</t>
+          <t>VNET3</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Empresa BAUH</t>
+          <t>Empresa VNET</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D366" t="n">
-        <v>93.39</v>
+        <v>0</v>
       </c>
       <c r="E366" t="inlineStr">
         <is>
@@ -15053,10 +15053,10 @@
         </is>
       </c>
       <c r="F366" t="n">
-        <v>153407000</v>
+        <v>14163000000</v>
       </c>
       <c r="G366" t="n">
-        <v>207.53</v>
+        <v>0</v>
       </c>
       <c r="H366" t="n">
         <v>0</v>
@@ -15071,21 +15071,21 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>ICPI3</t>
+          <t>CSPC4</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Empresa ICPI</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D367" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="E367" t="inlineStr">
         <is>
@@ -15093,39 +15093,39 @@
         </is>
       </c>
       <c r="F367" t="n">
-        <v>0</v>
+        <v>2126670000</v>
       </c>
       <c r="G367" t="n">
         <v>0</v>
       </c>
       <c r="H367" t="n">
-        <v>0</v>
+        <v>38.62</v>
       </c>
       <c r="I367" t="n">
-        <v>0</v>
+        <v>29.18</v>
       </c>
       <c r="J367" t="n">
-        <v>0</v>
+        <v>45.33</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>ILLS4</t>
+          <t>ARND3</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Empresa ILLS</t>
+          <t>Empresa ARND</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D368" t="n">
-        <v>100.01</v>
+        <v>0.51</v>
       </c>
       <c r="E368" t="inlineStr">
         <is>
@@ -15133,30 +15133,30 @@
         </is>
       </c>
       <c r="F368" t="n">
-        <v>-18567000</v>
+        <v>125211000</v>
       </c>
       <c r="G368" t="n">
-        <v>0</v>
+        <v>913.58</v>
       </c>
       <c r="H368" t="n">
-        <v>8.43</v>
+        <v>0</v>
       </c>
       <c r="I368" t="n">
-        <v>8.140000000000001</v>
+        <v>0</v>
       </c>
       <c r="J368" t="n">
-        <v>36.09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>BPAT33</t>
+          <t>INHA3</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Empresa BPAT</t>
+          <t>Empresa INHA</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -15165,7 +15165,7 @@
         </is>
       </c>
       <c r="D369" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="E369" t="inlineStr">
         <is>
@@ -15173,30 +15173,30 @@
         </is>
       </c>
       <c r="F369" t="n">
-        <v>876492000</v>
+        <v>1533210000</v>
       </c>
       <c r="G369" t="n">
         <v>0</v>
       </c>
       <c r="H369" t="n">
-        <v>0</v>
+        <v>-56.05</v>
       </c>
       <c r="I369" t="n">
-        <v>0</v>
+        <v>-6.27</v>
       </c>
       <c r="J369" t="n">
-        <v>0</v>
+        <v>-39.87</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>REPA4</t>
+          <t>PTIP4</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -15205,7 +15205,7 @@
         </is>
       </c>
       <c r="D370" t="n">
-        <v>1.08</v>
+        <v>25.15</v>
       </c>
       <c r="E370" t="inlineStr">
         <is>
@@ -15213,39 +15213,39 @@
         </is>
       </c>
       <c r="F370" t="n">
-        <v>378378000</v>
+        <v>-155957000</v>
       </c>
       <c r="G370" t="n">
         <v>0</v>
       </c>
       <c r="H370" t="n">
-        <v>5.18</v>
+        <v>13.73</v>
       </c>
       <c r="I370" t="n">
-        <v>4.05</v>
+        <v>23.13</v>
       </c>
       <c r="J370" t="n">
-        <v>1.91</v>
+        <v>-121.74</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>EQMA6B</t>
+          <t>LATS3</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa LATS</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D371" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="E371" t="inlineStr">
         <is>
@@ -15253,35 +15253,35 @@
         </is>
       </c>
       <c r="F371" t="n">
-        <v>4940330000</v>
+        <v>680646000</v>
       </c>
       <c r="G371" t="n">
         <v>0</v>
       </c>
       <c r="H371" t="n">
-        <v>0</v>
+        <v>11.74</v>
       </c>
       <c r="I371" t="n">
-        <v>0</v>
+        <v>11.63</v>
       </c>
       <c r="J371" t="n">
-        <v>0</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>SEBB4</t>
+          <t>VVAX3</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D372" t="n">
@@ -15293,25 +15293,25 @@
         </is>
       </c>
       <c r="F372" t="n">
-        <v>145783000</v>
+        <v>144676000</v>
       </c>
       <c r="G372" t="n">
         <v>0</v>
       </c>
       <c r="H372" t="n">
-        <v>9.24</v>
+        <v>-7.36</v>
       </c>
       <c r="I372" t="n">
-        <v>24.15</v>
+        <v>-6.52</v>
       </c>
       <c r="J372" t="n">
-        <v>23.01</v>
+        <v>-92.03</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>MSAN3</t>
+          <t>MSAN4</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
@@ -15321,7 +15321,7 @@
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D373" t="n">
@@ -15351,7 +15351,7 @@
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>GALO3</t>
+          <t>GALO4</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
@@ -15361,11 +15361,11 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D374" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E374" t="inlineStr">
         <is>
@@ -15391,12 +15391,12 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>SLCP3</t>
+          <t>BBTG13</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>Empresa SLCP</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
@@ -15405,7 +15405,7 @@
         </is>
       </c>
       <c r="D375" t="n">
-        <v>610.02</v>
+        <v>0</v>
       </c>
       <c r="E375" t="inlineStr">
         <is>
@@ -15413,7 +15413,7 @@
         </is>
       </c>
       <c r="F375" t="n">
-        <v>0</v>
+        <v>7000</v>
       </c>
       <c r="G375" t="n">
         <v>0</v>
@@ -15425,18 +15425,18 @@
         <v>0</v>
       </c>
       <c r="J375" t="n">
-        <v>0</v>
+        <v>-42.86</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>DAYC3</t>
+          <t>VSPT3</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>Empresa DAYC</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
@@ -15453,7 +15453,7 @@
         </is>
       </c>
       <c r="F376" t="n">
-        <v>3009030000</v>
+        <v>5031600000</v>
       </c>
       <c r="G376" t="n">
         <v>0</v>
@@ -15465,27 +15465,27 @@
         <v>0</v>
       </c>
       <c r="J376" t="n">
-        <v>17.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>PTIP3</t>
+          <t>SGEN4</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D377" t="n">
-        <v>22</v>
+        <v>0.6</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -15493,19 +15493,19 @@
         </is>
       </c>
       <c r="F377" t="n">
-        <v>-155957000</v>
+        <v>156981000</v>
       </c>
       <c r="G377" t="n">
         <v>0</v>
       </c>
       <c r="H377" t="n">
-        <v>13.73</v>
+        <v>-1871.17</v>
       </c>
       <c r="I377" t="n">
-        <v>23.13</v>
+        <v>-1.59</v>
       </c>
       <c r="J377" t="n">
-        <v>-121.74</v>
+        <v>0</v>
       </c>
     </row>
     <row r="378">
@@ -18071,7 +18071,7 @@
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>MMAQ4</t>
+          <t>MMAQ3</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
@@ -18081,7 +18081,7 @@
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D442" t="n">
@@ -18111,7 +18111,7 @@
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>MMAQ3</t>
+          <t>MMAQ4</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
@@ -18121,7 +18121,7 @@
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D443" t="n">
@@ -24071,7 +24071,7 @@
     <row r="592">
       <c r="A592" t="inlineStr">
         <is>
-          <t>GETT4</t>
+          <t>GETT3</t>
         </is>
       </c>
       <c r="B592" t="inlineStr">
@@ -24081,7 +24081,7 @@
       </c>
       <c r="C592" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D592" t="n">
@@ -24111,7 +24111,7 @@
     <row r="593">
       <c r="A593" t="inlineStr">
         <is>
-          <t>GETT3</t>
+          <t>GETT4</t>
         </is>
       </c>
       <c r="B593" t="inlineStr">
@@ -24121,7 +24121,7 @@
       </c>
       <c r="C593" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D593" t="n">
@@ -34951,7 +34951,7 @@
     <row r="864">
       <c r="A864" t="inlineStr">
         <is>
-          <t>RSIP3</t>
+          <t>RSIP4</t>
         </is>
       </c>
       <c r="B864" t="inlineStr">
@@ -34961,7 +34961,7 @@
       </c>
       <c r="C864" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D864" t="n">
@@ -34991,7 +34991,7 @@
     <row r="865">
       <c r="A865" t="inlineStr">
         <is>
-          <t>RSIP4</t>
+          <t>RSIP3</t>
         </is>
       </c>
       <c r="B865" t="inlineStr">
@@ -35001,7 +35001,7 @@
       </c>
       <c r="C865" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D865" t="n">
@@ -36591,7 +36591,7 @@
     <row r="905">
       <c r="A905" t="inlineStr">
         <is>
-          <t>BRGE5</t>
+          <t>BRGE11</t>
         </is>
       </c>
       <c r="B905" t="inlineStr">
@@ -36631,7 +36631,7 @@
     <row r="906">
       <c r="A906" t="inlineStr">
         <is>
-          <t>BRGE11</t>
+          <t>BRGE5</t>
         </is>
       </c>
       <c r="B906" t="inlineStr">
@@ -39311,7 +39311,7 @@
     <row r="973">
       <c r="A973" t="inlineStr">
         <is>
-          <t>PQUN3</t>
+          <t>PQUN4</t>
         </is>
       </c>
       <c r="B973" t="inlineStr">
@@ -39321,7 +39321,7 @@
       </c>
       <c r="C973" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D973" t="n">
@@ -39351,7 +39351,7 @@
     <row r="974">
       <c r="A974" t="inlineStr">
         <is>
-          <t>PQUN4</t>
+          <t>PQUN3</t>
         </is>
       </c>
       <c r="B974" t="inlineStr">
@@ -39361,7 +39361,7 @@
       </c>
       <c r="C974" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D974" t="n">

</xml_diff>

<commit_message>
Ajusta condicao de captura da Margem Liquida por substrings
</commit_message>
<xml_diff>
--- a/acoes_b3.xlsx
+++ b/acoes_b3.xlsx
@@ -471,21 +471,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PORP4</t>
+          <t>IVTT3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Empresa PORP</t>
+          <t>Empresa IVTT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2.4</v>
+        <v>0</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>22399000</v>
+        <v>1083050000</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -505,18 +505,18 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>-2.08</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>IVTT3</t>
+          <t>MNSA3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Empresa IVTT</t>
+          <t>Empresa MNSA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>0.42</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -533,30 +533,30 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1083050000</v>
+        <v>-9105000</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>-208.15</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>-13.5</v>
       </c>
       <c r="J3" t="n">
-        <v>-0.4</v>
+        <v>145.7</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MNSA3</t>
+          <t>CSTB3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Empresa MNSA</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.42</v>
+        <v>150</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -573,19 +573,19 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>-9105000</v>
+        <v>8420670000</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>-208.15</v>
+        <v>40.85</v>
       </c>
       <c r="I4" t="n">
-        <v>-13.5</v>
+        <v>22.4</v>
       </c>
       <c r="J4" t="n">
-        <v>145.7</v>
+        <v>20.11</v>
       </c>
     </row>
     <row r="5">
@@ -631,21 +631,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CSTB3</t>
+          <t>POPR4</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa POPR</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>150</v>
+        <v>10.17</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -653,39 +653,39 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>8420670000</v>
+        <v>545803000</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>40.85</v>
+        <v>8.66</v>
       </c>
       <c r="I6" t="n">
-        <v>22.4</v>
+        <v>15.25</v>
       </c>
       <c r="J6" t="n">
-        <v>20.11</v>
+        <v>19.93</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>POPR4</t>
+          <t>PMET3</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Empresa POPR</t>
+          <t>Empresa PMET</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>10.17</v>
+        <v>0</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -693,30 +693,30 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>545803000</v>
+        <v>-290863000</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>8.66</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>15.25</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>19.93</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PMET3</t>
+          <t>CLAN3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Empresa PMET</t>
+          <t>Empresa CLAN</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>-290863000</v>
+        <v>1012240000</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -745,27 +745,27 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>4.1</v>
+        <v>-1.05</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CLAN3</t>
+          <t>MNSA4</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Empresa CLAN</t>
+          <t>Empresa MNSA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>0.47</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -773,30 +773,30 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>1012240000</v>
+        <v>-9105000</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>-208.15</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>-13.5</v>
       </c>
       <c r="J9" t="n">
-        <v>-1.05</v>
+        <v>145.7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MNSA4</t>
+          <t>CSTB4</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Empresa MNSA</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.47</v>
+        <v>147.69</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -813,30 +813,30 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>-9105000</v>
+        <v>8420670000</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>-208.15</v>
+        <v>40.85</v>
       </c>
       <c r="I10" t="n">
-        <v>-13.5</v>
+        <v>22.4</v>
       </c>
       <c r="J10" t="n">
-        <v>145.7</v>
+        <v>20.11</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CSTB4</t>
+          <t>PORP4</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa PORP</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>147.69</v>
+        <v>2.4</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -853,19 +853,19 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>8420670000</v>
+        <v>22399000</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>40.85</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>22.4</v>
+        <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>20.11</v>
+        <v>-2.08</v>
       </c>
     </row>
     <row r="12">
@@ -12751,21 +12751,21 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>JFAB4</t>
+          <t>BERG3</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Empresa JFAB</t>
+          <t>Empresa BERG</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>0.06</v>
+        <v>33</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -12773,39 +12773,39 @@
         </is>
       </c>
       <c r="F309" t="n">
-        <v>-10183000</v>
+        <v>9538000</v>
       </c>
       <c r="G309" t="n">
         <v>0</v>
       </c>
       <c r="H309" t="n">
-        <v>0</v>
+        <v>-8.6</v>
       </c>
       <c r="I309" t="n">
-        <v>0</v>
+        <v>-5.58</v>
       </c>
       <c r="J309" t="n">
-        <v>2.34</v>
+        <v>-102.71</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>CCHI4</t>
+          <t>JBDU3</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa JBDU</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -12813,7 +12813,7 @@
         </is>
       </c>
       <c r="F310" t="n">
-        <v>-160477000</v>
+        <v>56569000</v>
       </c>
       <c r="G310" t="n">
         <v>0</v>
@@ -12831,12 +12831,12 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>REPA3</t>
+          <t>EGGY3</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa EGGY</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -12845,7 +12845,7 @@
         </is>
       </c>
       <c r="D311" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -12853,30 +12853,30 @@
         </is>
       </c>
       <c r="F311" t="n">
-        <v>378378000</v>
+        <v>954480000</v>
       </c>
       <c r="G311" t="n">
         <v>0</v>
       </c>
       <c r="H311" t="n">
-        <v>5.18</v>
+        <v>0</v>
       </c>
       <c r="I311" t="n">
-        <v>4.05</v>
+        <v>0</v>
       </c>
       <c r="J311" t="n">
-        <v>1.91</v>
+        <v>0</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>EQMA5B</t>
+          <t>CBMA4</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -12885,7 +12885,7 @@
         </is>
       </c>
       <c r="D312" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -12893,7 +12893,7 @@
         </is>
       </c>
       <c r="F312" t="n">
-        <v>4940330000</v>
+        <v>-34022300000</v>
       </c>
       <c r="G312" t="n">
         <v>0</v>
@@ -12911,21 +12911,21 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>SEBB3</t>
+          <t>SALM4</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -12933,39 +12933,39 @@
         </is>
       </c>
       <c r="F313" t="n">
-        <v>145783000</v>
+        <v>475600000</v>
       </c>
       <c r="G313" t="n">
         <v>0</v>
       </c>
       <c r="H313" t="n">
-        <v>9.24</v>
+        <v>10.22</v>
       </c>
       <c r="I313" t="n">
-        <v>24.15</v>
+        <v>25.78</v>
       </c>
       <c r="J313" t="n">
-        <v>23.01</v>
+        <v>19.53</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>BBTG11</t>
+          <t>BMEF3</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa BMEF</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>15.01</v>
+        <v>11</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -12973,7 +12973,7 @@
         </is>
       </c>
       <c r="F314" t="n">
-        <v>0</v>
+        <v>2674780000</v>
       </c>
       <c r="G314" t="n">
         <v>0</v>
@@ -12991,21 +12991,21 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>ECIS4</t>
+          <t>AGEI3</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa AGEI</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>145</v>
+        <v>7.8</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -13013,30 +13013,30 @@
         </is>
       </c>
       <c r="F315" t="n">
-        <v>129346000</v>
+        <v>1878210000</v>
       </c>
       <c r="G315" t="n">
         <v>0</v>
       </c>
       <c r="H315" t="n">
-        <v>34.9</v>
+        <v>0</v>
       </c>
       <c r="I315" t="n">
-        <v>12.48</v>
+        <v>0</v>
       </c>
       <c r="J315" t="n">
-        <v>7.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>TNEP3</t>
+          <t>SASG3</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa SASG</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -13045,7 +13045,7 @@
         </is>
       </c>
       <c r="D316" t="n">
-        <v>3.01</v>
+        <v>0.98</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -13053,30 +13053,30 @@
         </is>
       </c>
       <c r="F316" t="n">
-        <v>955105000</v>
+        <v>0</v>
       </c>
       <c r="G316" t="n">
         <v>0</v>
       </c>
       <c r="H316" t="n">
-        <v>20.92</v>
+        <v>0</v>
       </c>
       <c r="I316" t="n">
-        <v>20.53</v>
+        <v>0</v>
       </c>
       <c r="J316" t="n">
-        <v>22.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>LECO3</t>
+          <t>ODER3</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Empresa LECO</t>
+          <t>Empresa ODER</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -13093,30 +13093,30 @@
         </is>
       </c>
       <c r="F317" t="n">
-        <v>105928000</v>
+        <v>609518000</v>
       </c>
       <c r="G317" t="n">
         <v>0</v>
       </c>
       <c r="H317" t="n">
-        <v>-2.14</v>
+        <v>0</v>
       </c>
       <c r="I317" t="n">
-        <v>-3.48</v>
+        <v>0</v>
       </c>
       <c r="J317" t="n">
-        <v>-14.82</v>
+        <v>0</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>VGOR3</t>
+          <t>ARPS3</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Empresa VGOR</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -13125,7 +13125,7 @@
         </is>
       </c>
       <c r="D318" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -13133,39 +13133,39 @@
         </is>
       </c>
       <c r="F318" t="n">
-        <v>135178000</v>
+        <v>-12690000</v>
       </c>
       <c r="G318" t="n">
         <v>0</v>
       </c>
       <c r="H318" t="n">
-        <v>4.5</v>
+        <v>-4.92</v>
       </c>
       <c r="I318" t="n">
-        <v>6</v>
+        <v>-6.64</v>
       </c>
       <c r="J318" t="n">
-        <v>-24.29</v>
+        <v>20.34</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>GPIV33</t>
+          <t>VVAX4</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Empresa GPIV</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>4.42</v>
+        <v>0</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -13173,30 +13173,30 @@
         </is>
       </c>
       <c r="F319" t="n">
-        <v>1318490000</v>
+        <v>144676000</v>
       </c>
       <c r="G319" t="n">
         <v>0</v>
       </c>
       <c r="H319" t="n">
-        <v>257.32</v>
+        <v>-7.36</v>
       </c>
       <c r="I319" t="n">
-        <v>-6.05</v>
+        <v>-6.52</v>
       </c>
       <c r="J319" t="n">
-        <v>0</v>
+        <v>-92.03</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>JBDU3</t>
+          <t>CSPC3</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Empresa JBDU</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -13205,7 +13205,7 @@
         </is>
       </c>
       <c r="D320" t="n">
-        <v>0</v>
+        <v>1.24</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -13213,30 +13213,30 @@
         </is>
       </c>
       <c r="F320" t="n">
-        <v>56569000</v>
+        <v>2126670000</v>
       </c>
       <c r="G320" t="n">
         <v>0</v>
       </c>
       <c r="H320" t="n">
-        <v>0</v>
+        <v>38.62</v>
       </c>
       <c r="I320" t="n">
-        <v>0</v>
+        <v>29.18</v>
       </c>
       <c r="J320" t="n">
-        <v>0</v>
+        <v>45.33</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>EGGY3</t>
+          <t>ABCB3</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Empresa EGGY</t>
+          <t>Empresa ABCB</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -13249,11 +13249,11 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="F321" t="n">
-        <v>954480000</v>
+        <v>7258910000</v>
       </c>
       <c r="G321" t="n">
         <v>0</v>
@@ -13265,27 +13265,27 @@
         <v>0</v>
       </c>
       <c r="J321" t="n">
-        <v>0</v>
+        <v>14.05</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>CBMA4</t>
+          <t>CCTY3</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa CCTY</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -13293,7 +13293,7 @@
         </is>
       </c>
       <c r="F322" t="n">
-        <v>-34022300000</v>
+        <v>0</v>
       </c>
       <c r="G322" t="n">
         <v>0</v>
@@ -13311,12 +13311,12 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>SALM4</t>
+          <t>BAUH4</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa BAUH</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -13325,7 +13325,7 @@
         </is>
       </c>
       <c r="D323" t="n">
-        <v>5.9</v>
+        <v>93.39</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -13333,30 +13333,30 @@
         </is>
       </c>
       <c r="F323" t="n">
-        <v>475600000</v>
+        <v>153407000</v>
       </c>
       <c r="G323" t="n">
-        <v>0</v>
+        <v>207.53</v>
       </c>
       <c r="H323" t="n">
-        <v>10.22</v>
+        <v>0</v>
       </c>
       <c r="I323" t="n">
-        <v>25.78</v>
+        <v>0</v>
       </c>
       <c r="J323" t="n">
-        <v>19.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>BERG3</t>
+          <t>ICPI3</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Empresa BERG</t>
+          <t>Empresa ICPI</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -13365,7 +13365,7 @@
         </is>
       </c>
       <c r="D324" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -13373,39 +13373,39 @@
         </is>
       </c>
       <c r="F324" t="n">
-        <v>9538000</v>
+        <v>0</v>
       </c>
       <c r="G324" t="n">
         <v>0</v>
       </c>
       <c r="H324" t="n">
-        <v>-8.6</v>
+        <v>0</v>
       </c>
       <c r="I324" t="n">
-        <v>-5.58</v>
+        <v>0</v>
       </c>
       <c r="J324" t="n">
-        <v>-102.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>AGEI3</t>
+          <t>ILLS4</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Empresa AGEI</t>
+          <t>Empresa ILLS</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D325" t="n">
-        <v>7.8</v>
+        <v>100.01</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -13413,30 +13413,30 @@
         </is>
       </c>
       <c r="F325" t="n">
-        <v>1878210000</v>
+        <v>-18567000</v>
       </c>
       <c r="G325" t="n">
         <v>0</v>
       </c>
       <c r="H325" t="n">
-        <v>0</v>
+        <v>8.43</v>
       </c>
       <c r="I325" t="n">
-        <v>0</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="J325" t="n">
-        <v>0</v>
+        <v>36.09</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>SASG3</t>
+          <t>BPAT33</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Empresa SASG</t>
+          <t>Empresa BPAT</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -13445,7 +13445,7 @@
         </is>
       </c>
       <c r="D326" t="n">
-        <v>0.98</v>
+        <v>20</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -13453,7 +13453,7 @@
         </is>
       </c>
       <c r="F326" t="n">
-        <v>0</v>
+        <v>876492000</v>
       </c>
       <c r="G326" t="n">
         <v>0</v>
@@ -13471,21 +13471,21 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>BMEF3</t>
+          <t>ESTC4</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Empresa BMEF</t>
+          <t>Empresa ESTC</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -13493,39 +13493,39 @@
         </is>
       </c>
       <c r="F327" t="n">
-        <v>2674780000</v>
+        <v>2916530000</v>
       </c>
       <c r="G327" t="n">
         <v>0</v>
       </c>
       <c r="H327" t="n">
-        <v>0</v>
+        <v>16.91</v>
       </c>
       <c r="I327" t="n">
-        <v>0</v>
+        <v>11.35</v>
       </c>
       <c r="J327" t="n">
-        <v>0</v>
+        <v>3.89</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>ARPS3</t>
+          <t>VSPT4</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -13533,35 +13533,35 @@
         </is>
       </c>
       <c r="F328" t="n">
-        <v>-12690000</v>
+        <v>5031600000</v>
       </c>
       <c r="G328" t="n">
         <v>0</v>
       </c>
       <c r="H328" t="n">
-        <v>-4.92</v>
+        <v>0</v>
       </c>
       <c r="I328" t="n">
-        <v>-6.64</v>
+        <v>0</v>
       </c>
       <c r="J328" t="n">
-        <v>20.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>ODER3</t>
+          <t>SEBB4</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Empresa ODER</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D329" t="n">
@@ -13573,30 +13573,30 @@
         </is>
       </c>
       <c r="F329" t="n">
-        <v>609518000</v>
+        <v>145783000</v>
       </c>
       <c r="G329" t="n">
         <v>0</v>
       </c>
       <c r="H329" t="n">
-        <v>0</v>
+        <v>9.24</v>
       </c>
       <c r="I329" t="n">
-        <v>0</v>
+        <v>24.15</v>
       </c>
       <c r="J329" t="n">
-        <v>0</v>
+        <v>23.01</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>ABCB3</t>
+          <t>MSAN3</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Empresa ABCB</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -13605,38 +13605,38 @@
         </is>
       </c>
       <c r="D330" t="n">
-        <v>0</v>
+        <v>6.44</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>Bancos</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="F330" t="n">
-        <v>7258910000</v>
+        <v>2533030000</v>
       </c>
       <c r="G330" t="n">
         <v>0</v>
       </c>
       <c r="H330" t="n">
-        <v>0</v>
+        <v>6.27</v>
       </c>
       <c r="I330" t="n">
-        <v>0</v>
+        <v>11.78</v>
       </c>
       <c r="J330" t="n">
-        <v>14.05</v>
+        <v>11.81</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>CCTY3</t>
+          <t>GALO3</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Empresa CCTY</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -13653,39 +13653,39 @@
         </is>
       </c>
       <c r="F331" t="n">
-        <v>0</v>
+        <v>-60607000</v>
       </c>
       <c r="G331" t="n">
         <v>0</v>
       </c>
       <c r="H331" t="n">
-        <v>0</v>
+        <v>13.98</v>
       </c>
       <c r="I331" t="n">
-        <v>0</v>
+        <v>39.37</v>
       </c>
       <c r="J331" t="n">
-        <v>0</v>
+        <v>7.62</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>VVAX4</t>
+          <t>SLCP3</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa SLCP</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>0</v>
+        <v>610.02</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -13693,30 +13693,30 @@
         </is>
       </c>
       <c r="F332" t="n">
-        <v>144676000</v>
+        <v>0</v>
       </c>
       <c r="G332" t="n">
         <v>0</v>
       </c>
       <c r="H332" t="n">
-        <v>-7.36</v>
+        <v>0</v>
       </c>
       <c r="I332" t="n">
-        <v>-6.52</v>
+        <v>0</v>
       </c>
       <c r="J332" t="n">
-        <v>-92.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>CSPC3</t>
+          <t>DAYC3</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa DAYC</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -13725,7 +13725,7 @@
         </is>
       </c>
       <c r="D333" t="n">
-        <v>1.24</v>
+        <v>0</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -13733,39 +13733,39 @@
         </is>
       </c>
       <c r="F333" t="n">
-        <v>2126670000</v>
+        <v>3009030000</v>
       </c>
       <c r="G333" t="n">
         <v>0</v>
       </c>
       <c r="H333" t="n">
-        <v>38.62</v>
+        <v>0</v>
       </c>
       <c r="I333" t="n">
-        <v>29.18</v>
+        <v>0</v>
       </c>
       <c r="J333" t="n">
-        <v>45.33</v>
+        <v>17.33</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>ILLS4</t>
+          <t>PTIP3</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Empresa ILLS</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>100.01</v>
+        <v>22</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -13773,39 +13773,39 @@
         </is>
       </c>
       <c r="F334" t="n">
-        <v>-18567000</v>
+        <v>-155957000</v>
       </c>
       <c r="G334" t="n">
         <v>0</v>
       </c>
       <c r="H334" t="n">
-        <v>8.43</v>
+        <v>13.73</v>
       </c>
       <c r="I334" t="n">
-        <v>8.140000000000001</v>
+        <v>23.13</v>
       </c>
       <c r="J334" t="n">
-        <v>36.09</v>
+        <v>-121.74</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>BPAT33</t>
+          <t>REPA4</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Empresa BPAT</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>20</v>
+        <v>1.08</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -13813,30 +13813,30 @@
         </is>
       </c>
       <c r="F335" t="n">
-        <v>876492000</v>
+        <v>378378000</v>
       </c>
       <c r="G335" t="n">
         <v>0</v>
       </c>
       <c r="H335" t="n">
-        <v>0</v>
+        <v>5.18</v>
       </c>
       <c r="I335" t="n">
-        <v>0</v>
+        <v>4.05</v>
       </c>
       <c r="J335" t="n">
-        <v>0</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>ESTC4</t>
+          <t>EQMA6B</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Empresa ESTC</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -13853,39 +13853,39 @@
         </is>
       </c>
       <c r="F336" t="n">
-        <v>2916530000</v>
+        <v>4940330000</v>
       </c>
       <c r="G336" t="n">
         <v>0</v>
       </c>
       <c r="H336" t="n">
-        <v>16.91</v>
+        <v>0</v>
       </c>
       <c r="I336" t="n">
-        <v>11.35</v>
+        <v>0</v>
       </c>
       <c r="J336" t="n">
-        <v>3.89</v>
+        <v>0</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>VSPT4</t>
+          <t>SGEN3</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -13893,16 +13893,16 @@
         </is>
       </c>
       <c r="F337" t="n">
-        <v>5031600000</v>
+        <v>156981000</v>
       </c>
       <c r="G337" t="n">
         <v>0</v>
       </c>
       <c r="H337" t="n">
-        <v>0</v>
+        <v>-1871.17</v>
       </c>
       <c r="I337" t="n">
-        <v>0</v>
+        <v>-1.59</v>
       </c>
       <c r="J337" t="n">
         <v>0</v>
@@ -13911,12 +13911,12 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>BAUH4</t>
+          <t>DUFB11</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Empresa BAUH</t>
+          <t>Empresa DUFB</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -13925,7 +13925,7 @@
         </is>
       </c>
       <c r="D338" t="n">
-        <v>93.39</v>
+        <v>0</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -13933,10 +13933,10 @@
         </is>
       </c>
       <c r="F338" t="n">
-        <v>153407000</v>
+        <v>0</v>
       </c>
       <c r="G338" t="n">
-        <v>207.53</v>
+        <v>0</v>
       </c>
       <c r="H338" t="n">
         <v>0</v>
@@ -13951,21 +13951,21 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>ICPI3</t>
+          <t>TNEP4</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Empresa ICPI</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>0</v>
+        <v>3.95</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -13973,30 +13973,30 @@
         </is>
       </c>
       <c r="F339" t="n">
-        <v>0</v>
+        <v>955105000</v>
       </c>
       <c r="G339" t="n">
         <v>0</v>
       </c>
       <c r="H339" t="n">
-        <v>0</v>
+        <v>20.92</v>
       </c>
       <c r="I339" t="n">
-        <v>0</v>
+        <v>20.53</v>
       </c>
       <c r="J339" t="n">
-        <v>0</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>DAYC3</t>
+          <t>MLPA3</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Empresa DAYC</t>
+          <t>Empresa MLPA</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -14013,39 +14013,39 @@
         </is>
       </c>
       <c r="F340" t="n">
-        <v>3009030000</v>
+        <v>44578000</v>
       </c>
       <c r="G340" t="n">
         <v>0</v>
       </c>
       <c r="H340" t="n">
-        <v>0</v>
+        <v>6.66</v>
       </c>
       <c r="I340" t="n">
         <v>0</v>
       </c>
       <c r="J340" t="n">
-        <v>17.33</v>
+        <v>45.13</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>PTIP3</t>
+          <t>CLSC6</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa CLSC</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -14053,39 +14053,39 @@
         </is>
       </c>
       <c r="F341" t="n">
-        <v>-155957000</v>
+        <v>4228180000</v>
       </c>
       <c r="G341" t="n">
         <v>0</v>
       </c>
       <c r="H341" t="n">
-        <v>13.73</v>
+        <v>0</v>
       </c>
       <c r="I341" t="n">
-        <v>23.13</v>
+        <v>0</v>
       </c>
       <c r="J341" t="n">
-        <v>-121.74</v>
+        <v>0</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>REPA4</t>
+          <t>CCHI3</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>1.08</v>
+        <v>0.02</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -14093,35 +14093,35 @@
         </is>
       </c>
       <c r="F342" t="n">
-        <v>378378000</v>
+        <v>-160477000</v>
       </c>
       <c r="G342" t="n">
         <v>0</v>
       </c>
       <c r="H342" t="n">
-        <v>5.18</v>
+        <v>0</v>
       </c>
       <c r="I342" t="n">
-        <v>4.05</v>
+        <v>0</v>
       </c>
       <c r="J342" t="n">
-        <v>1.91</v>
+        <v>0</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>EQMA6B</t>
+          <t>SFSA3</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa SFSA</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D343" t="n">
@@ -14133,7 +14133,7 @@
         </is>
       </c>
       <c r="F343" t="n">
-        <v>4940330000</v>
+        <v>739524000</v>
       </c>
       <c r="G343" t="n">
         <v>0</v>
@@ -14145,23 +14145,23 @@
         <v>0</v>
       </c>
       <c r="J343" t="n">
-        <v>0</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>SEBB4</t>
+          <t>PRBC3</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa PRBC</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D344" t="n">
@@ -14173,30 +14173,30 @@
         </is>
       </c>
       <c r="F344" t="n">
-        <v>145783000</v>
+        <v>1319270000</v>
       </c>
       <c r="G344" t="n">
         <v>0</v>
       </c>
       <c r="H344" t="n">
-        <v>9.24</v>
+        <v>0</v>
       </c>
       <c r="I344" t="n">
-        <v>24.15</v>
+        <v>0</v>
       </c>
       <c r="J344" t="n">
-        <v>23.01</v>
+        <v>8.27</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>MSAN3</t>
+          <t>ECIS3</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -14205,7 +14205,7 @@
         </is>
       </c>
       <c r="D345" t="n">
-        <v>6.44</v>
+        <v>211.65</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -14213,30 +14213,30 @@
         </is>
       </c>
       <c r="F345" t="n">
-        <v>2533030000</v>
+        <v>129346000</v>
       </c>
       <c r="G345" t="n">
         <v>0</v>
       </c>
       <c r="H345" t="n">
-        <v>6.27</v>
+        <v>34.9</v>
       </c>
       <c r="I345" t="n">
-        <v>11.78</v>
+        <v>12.48</v>
       </c>
       <c r="J345" t="n">
-        <v>11.81</v>
+        <v>7.33</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>GALO3</t>
+          <t>CZRS3</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa CZRS</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
@@ -14253,30 +14253,30 @@
         </is>
       </c>
       <c r="F346" t="n">
-        <v>-60607000</v>
+        <v>1145670000</v>
       </c>
       <c r="G346" t="n">
         <v>0</v>
       </c>
       <c r="H346" t="n">
-        <v>13.98</v>
+        <v>0</v>
       </c>
       <c r="I346" t="n">
-        <v>39.37</v>
+        <v>0</v>
       </c>
       <c r="J346" t="n">
-        <v>7.62</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>SLCP3</t>
+          <t>BPNM3</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Empresa SLCP</t>
+          <t>Empresa BPNM</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
@@ -14285,7 +14285,7 @@
         </is>
       </c>
       <c r="D347" t="n">
-        <v>610.02</v>
+        <v>0</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -14293,7 +14293,7 @@
         </is>
       </c>
       <c r="F347" t="n">
-        <v>0</v>
+        <v>7792670000</v>
       </c>
       <c r="G347" t="n">
         <v>0</v>
@@ -14305,27 +14305,27 @@
         <v>0</v>
       </c>
       <c r="J347" t="n">
-        <v>0</v>
+        <v>9.67</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>DUFB11</t>
+          <t>BSGR3</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Empresa DUFB</t>
+          <t>Empresa BSGR</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>0</v>
+        <v>1091.28</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -14351,21 +14351,21 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>TNEP4</t>
+          <t>CBMA3</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>3.95</v>
+        <v>0.01</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -14373,30 +14373,30 @@
         </is>
       </c>
       <c r="F349" t="n">
-        <v>955105000</v>
+        <v>-34022300000</v>
       </c>
       <c r="G349" t="n">
         <v>0</v>
       </c>
       <c r="H349" t="n">
-        <v>20.92</v>
+        <v>0</v>
       </c>
       <c r="I349" t="n">
-        <v>20.53</v>
+        <v>0</v>
       </c>
       <c r="J349" t="n">
-        <v>22.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>MLPA3</t>
+          <t>ALBA3</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Empresa MLPA</t>
+          <t>Empresa ALBA</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
@@ -14405,7 +14405,7 @@
         </is>
       </c>
       <c r="D350" t="n">
-        <v>0</v>
+        <v>2.15</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -14413,30 +14413,30 @@
         </is>
       </c>
       <c r="F350" t="n">
-        <v>44578000</v>
+        <v>354860000</v>
       </c>
       <c r="G350" t="n">
         <v>0</v>
       </c>
       <c r="H350" t="n">
-        <v>6.66</v>
+        <v>9.5</v>
       </c>
       <c r="I350" t="n">
-        <v>0</v>
+        <v>20.4</v>
       </c>
       <c r="J350" t="n">
-        <v>45.13</v>
+        <v>19.77</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>CLSC6</t>
+          <t>ARPS4</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Empresa CLSC</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -14453,30 +14453,30 @@
         </is>
       </c>
       <c r="F351" t="n">
-        <v>4228180000</v>
+        <v>-12690000</v>
       </c>
       <c r="G351" t="n">
         <v>0</v>
       </c>
       <c r="H351" t="n">
-        <v>0</v>
+        <v>-4.92</v>
       </c>
       <c r="I351" t="n">
-        <v>0</v>
+        <v>-6.64</v>
       </c>
       <c r="J351" t="n">
-        <v>0</v>
+        <v>20.34</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>SGEN3</t>
+          <t>SALM3</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -14485,7 +14485,7 @@
         </is>
       </c>
       <c r="D352" t="n">
-        <v>5</v>
+        <v>5.7</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -14493,39 +14493,39 @@
         </is>
       </c>
       <c r="F352" t="n">
-        <v>156981000</v>
+        <v>475600000</v>
       </c>
       <c r="G352" t="n">
         <v>0</v>
       </c>
       <c r="H352" t="n">
-        <v>-1871.17</v>
+        <v>10.22</v>
       </c>
       <c r="I352" t="n">
-        <v>-1.59</v>
+        <v>25.78</v>
       </c>
       <c r="J352" t="n">
-        <v>0</v>
+        <v>19.53</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>CCHI3</t>
+          <t>CMMA4</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa CMMA</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>0.02</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -14533,7 +14533,7 @@
         </is>
       </c>
       <c r="F353" t="n">
-        <v>-160477000</v>
+        <v>-79623000</v>
       </c>
       <c r="G353" t="n">
         <v>0</v>
@@ -14545,27 +14545,27 @@
         <v>0</v>
       </c>
       <c r="J353" t="n">
-        <v>0</v>
+        <v>-1.92</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>PRBC3</t>
+          <t>CSPC4</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Empresa PRBC</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D354" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="E354" t="inlineStr">
         <is>
@@ -14573,30 +14573,30 @@
         </is>
       </c>
       <c r="F354" t="n">
-        <v>1319270000</v>
+        <v>2126670000</v>
       </c>
       <c r="G354" t="n">
         <v>0</v>
       </c>
       <c r="H354" t="n">
-        <v>0</v>
+        <v>38.62</v>
       </c>
       <c r="I354" t="n">
-        <v>0</v>
+        <v>29.18</v>
       </c>
       <c r="J354" t="n">
-        <v>8.27</v>
+        <v>45.33</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>ECIS3</t>
+          <t>BOVH3</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa BOVH</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -14605,7 +14605,7 @@
         </is>
       </c>
       <c r="D355" t="n">
-        <v>211.65</v>
+        <v>15.71</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -14613,30 +14613,30 @@
         </is>
       </c>
       <c r="F355" t="n">
-        <v>129346000</v>
+        <v>1843320000</v>
       </c>
       <c r="G355" t="n">
         <v>0</v>
       </c>
       <c r="H355" t="n">
-        <v>34.9</v>
+        <v>0</v>
       </c>
       <c r="I355" t="n">
-        <v>12.48</v>
+        <v>0</v>
       </c>
       <c r="J355" t="n">
-        <v>7.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>SFSA3</t>
+          <t>VNET3</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Empresa SFSA</t>
+          <t>Empresa VNET</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -14653,7 +14653,7 @@
         </is>
       </c>
       <c r="F356" t="n">
-        <v>739524000</v>
+        <v>14163000000</v>
       </c>
       <c r="G356" t="n">
         <v>0</v>
@@ -14665,18 +14665,18 @@
         <v>0</v>
       </c>
       <c r="J356" t="n">
-        <v>6.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>CZRS3</t>
+          <t>ARND3</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Empresa CZRS</t>
+          <t>Empresa ARND</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -14685,7 +14685,7 @@
         </is>
       </c>
       <c r="D357" t="n">
-        <v>0</v>
+        <v>0.51</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -14693,10 +14693,10 @@
         </is>
       </c>
       <c r="F357" t="n">
-        <v>1145670000</v>
+        <v>125211000</v>
       </c>
       <c r="G357" t="n">
-        <v>0</v>
+        <v>913.58</v>
       </c>
       <c r="H357" t="n">
         <v>0</v>
@@ -14705,18 +14705,18 @@
         <v>0</v>
       </c>
       <c r="J357" t="n">
-        <v>3.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>BPNM3</t>
+          <t>VVAX3</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Empresa BPNM</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -14733,39 +14733,39 @@
         </is>
       </c>
       <c r="F358" t="n">
-        <v>7792670000</v>
+        <v>144676000</v>
       </c>
       <c r="G358" t="n">
         <v>0</v>
       </c>
       <c r="H358" t="n">
-        <v>0</v>
+        <v>-7.36</v>
       </c>
       <c r="I358" t="n">
-        <v>0</v>
+        <v>-6.52</v>
       </c>
       <c r="J358" t="n">
-        <v>9.67</v>
+        <v>-92.03</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>BSGR3</t>
+          <t>MSAN4</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Empresa BSGR</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>1091.28</v>
+        <v>6.44</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -14773,39 +14773,39 @@
         </is>
       </c>
       <c r="F359" t="n">
-        <v>0</v>
+        <v>2533030000</v>
       </c>
       <c r="G359" t="n">
         <v>0</v>
       </c>
       <c r="H359" t="n">
-        <v>0</v>
+        <v>6.27</v>
       </c>
       <c r="I359" t="n">
-        <v>0</v>
+        <v>11.78</v>
       </c>
       <c r="J359" t="n">
-        <v>0</v>
+        <v>11.81</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>CBMA3</t>
+          <t>GALO4</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>0.01</v>
+        <v>0.25</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -14813,30 +14813,30 @@
         </is>
       </c>
       <c r="F360" t="n">
-        <v>-34022300000</v>
+        <v>-60607000</v>
       </c>
       <c r="G360" t="n">
         <v>0</v>
       </c>
       <c r="H360" t="n">
-        <v>0</v>
+        <v>13.98</v>
       </c>
       <c r="I360" t="n">
-        <v>0</v>
+        <v>39.37</v>
       </c>
       <c r="J360" t="n">
-        <v>0</v>
+        <v>7.62</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>ALBA3</t>
+          <t>BBTG13</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Empresa ALBA</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -14845,7 +14845,7 @@
         </is>
       </c>
       <c r="D361" t="n">
-        <v>2.15</v>
+        <v>0</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -14853,35 +14853,35 @@
         </is>
       </c>
       <c r="F361" t="n">
-        <v>354860000</v>
+        <v>7000</v>
       </c>
       <c r="G361" t="n">
         <v>0</v>
       </c>
       <c r="H361" t="n">
-        <v>9.5</v>
+        <v>0</v>
       </c>
       <c r="I361" t="n">
-        <v>20.4</v>
+        <v>0</v>
       </c>
       <c r="J361" t="n">
-        <v>19.77</v>
+        <v>-42.86</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>ARPS4</t>
+          <t>INHA3</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa INHA</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D362" t="n">
@@ -14893,39 +14893,39 @@
         </is>
       </c>
       <c r="F362" t="n">
-        <v>-12690000</v>
+        <v>1533210000</v>
       </c>
       <c r="G362" t="n">
         <v>0</v>
       </c>
       <c r="H362" t="n">
-        <v>-4.92</v>
+        <v>-56.05</v>
       </c>
       <c r="I362" t="n">
-        <v>-6.64</v>
+        <v>-6.27</v>
       </c>
       <c r="J362" t="n">
-        <v>20.34</v>
+        <v>-39.87</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>SALM3</t>
+          <t>PTIP4</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D363" t="n">
-        <v>5.7</v>
+        <v>25.15</v>
       </c>
       <c r="E363" t="inlineStr">
         <is>
@@ -14933,39 +14933,39 @@
         </is>
       </c>
       <c r="F363" t="n">
-        <v>475600000</v>
+        <v>-155957000</v>
       </c>
       <c r="G363" t="n">
         <v>0</v>
       </c>
       <c r="H363" t="n">
-        <v>10.22</v>
+        <v>13.73</v>
       </c>
       <c r="I363" t="n">
-        <v>25.78</v>
+        <v>23.13</v>
       </c>
       <c r="J363" t="n">
-        <v>19.53</v>
+        <v>-121.74</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>CMMA4</t>
+          <t>LATS3</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Empresa CMMA</t>
+          <t>Empresa LATS</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D364" t="n">
-        <v>0.8100000000000001</v>
+        <v>22</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -14973,39 +14973,39 @@
         </is>
       </c>
       <c r="F364" t="n">
-        <v>-79623000</v>
+        <v>680646000</v>
       </c>
       <c r="G364" t="n">
         <v>0</v>
       </c>
       <c r="H364" t="n">
-        <v>0</v>
+        <v>11.74</v>
       </c>
       <c r="I364" t="n">
-        <v>0</v>
+        <v>11.63</v>
       </c>
       <c r="J364" t="n">
-        <v>-1.92</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>BOVH3</t>
+          <t>SGEN4</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Empresa BOVH</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D365" t="n">
-        <v>15.71</v>
+        <v>0.6</v>
       </c>
       <c r="E365" t="inlineStr">
         <is>
@@ -15013,16 +15013,16 @@
         </is>
       </c>
       <c r="F365" t="n">
-        <v>1843320000</v>
+        <v>156981000</v>
       </c>
       <c r="G365" t="n">
         <v>0</v>
       </c>
       <c r="H365" t="n">
-        <v>0</v>
+        <v>-1871.17</v>
       </c>
       <c r="I365" t="n">
-        <v>0</v>
+        <v>-1.59</v>
       </c>
       <c r="J365" t="n">
         <v>0</v>
@@ -15031,12 +15031,12 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>VNET3</t>
+          <t>VSPT3</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Empresa VNET</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -15053,7 +15053,7 @@
         </is>
       </c>
       <c r="F366" t="n">
-        <v>14163000000</v>
+        <v>5031600000</v>
       </c>
       <c r="G366" t="n">
         <v>0</v>
@@ -15071,21 +15071,21 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>CSPC4</t>
+          <t>SEBB3</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D367" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="E367" t="inlineStr">
         <is>
@@ -15093,39 +15093,39 @@
         </is>
       </c>
       <c r="F367" t="n">
-        <v>2126670000</v>
+        <v>145783000</v>
       </c>
       <c r="G367" t="n">
         <v>0</v>
       </c>
       <c r="H367" t="n">
-        <v>38.62</v>
+        <v>9.24</v>
       </c>
       <c r="I367" t="n">
-        <v>29.18</v>
+        <v>24.15</v>
       </c>
       <c r="J367" t="n">
-        <v>45.33</v>
+        <v>23.01</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>ARND3</t>
+          <t>BBTG11</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Empresa ARND</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D368" t="n">
-        <v>0.51</v>
+        <v>15.01</v>
       </c>
       <c r="E368" t="inlineStr">
         <is>
@@ -15133,10 +15133,10 @@
         </is>
       </c>
       <c r="F368" t="n">
-        <v>125211000</v>
+        <v>0</v>
       </c>
       <c r="G368" t="n">
-        <v>913.58</v>
+        <v>0</v>
       </c>
       <c r="H368" t="n">
         <v>0</v>
@@ -15151,21 +15151,21 @@
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>INHA3</t>
+          <t>JFAB4</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Empresa INHA</t>
+          <t>Empresa JFAB</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D369" t="n">
-        <v>0</v>
+        <v>0.06</v>
       </c>
       <c r="E369" t="inlineStr">
         <is>
@@ -15173,30 +15173,30 @@
         </is>
       </c>
       <c r="F369" t="n">
-        <v>1533210000</v>
+        <v>-10183000</v>
       </c>
       <c r="G369" t="n">
         <v>0</v>
       </c>
       <c r="H369" t="n">
-        <v>-56.05</v>
+        <v>0</v>
       </c>
       <c r="I369" t="n">
-        <v>-6.27</v>
+        <v>0</v>
       </c>
       <c r="J369" t="n">
-        <v>-39.87</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>PTIP4</t>
+          <t>CCHI4</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -15205,7 +15205,7 @@
         </is>
       </c>
       <c r="D370" t="n">
-        <v>25.15</v>
+        <v>0.02</v>
       </c>
       <c r="E370" t="inlineStr">
         <is>
@@ -15213,30 +15213,30 @@
         </is>
       </c>
       <c r="F370" t="n">
-        <v>-155957000</v>
+        <v>-160477000</v>
       </c>
       <c r="G370" t="n">
         <v>0</v>
       </c>
       <c r="H370" t="n">
-        <v>13.73</v>
+        <v>0</v>
       </c>
       <c r="I370" t="n">
-        <v>23.13</v>
+        <v>0</v>
       </c>
       <c r="J370" t="n">
-        <v>-121.74</v>
+        <v>0</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>LATS3</t>
+          <t>REPA3</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Empresa LATS</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
@@ -15245,7 +15245,7 @@
         </is>
       </c>
       <c r="D371" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E371" t="inlineStr">
         <is>
@@ -15253,35 +15253,35 @@
         </is>
       </c>
       <c r="F371" t="n">
-        <v>680646000</v>
+        <v>378378000</v>
       </c>
       <c r="G371" t="n">
         <v>0</v>
       </c>
       <c r="H371" t="n">
-        <v>11.74</v>
+        <v>5.18</v>
       </c>
       <c r="I371" t="n">
-        <v>11.63</v>
+        <v>4.05</v>
       </c>
       <c r="J371" t="n">
-        <v>1.84</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>VVAX3</t>
+          <t>EQMA5B</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D372" t="n">
@@ -15293,39 +15293,39 @@
         </is>
       </c>
       <c r="F372" t="n">
-        <v>144676000</v>
+        <v>4940330000</v>
       </c>
       <c r="G372" t="n">
         <v>0</v>
       </c>
       <c r="H372" t="n">
-        <v>-7.36</v>
+        <v>0</v>
       </c>
       <c r="I372" t="n">
-        <v>-6.52</v>
+        <v>0</v>
       </c>
       <c r="J372" t="n">
-        <v>-92.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>MSAN4</t>
+          <t>GPIV33</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa GPIV</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D373" t="n">
-        <v>6.44</v>
+        <v>4.42</v>
       </c>
       <c r="E373" t="inlineStr">
         <is>
@@ -15333,30 +15333,30 @@
         </is>
       </c>
       <c r="F373" t="n">
-        <v>2533030000</v>
+        <v>1318490000</v>
       </c>
       <c r="G373" t="n">
         <v>0</v>
       </c>
       <c r="H373" t="n">
-        <v>6.27</v>
+        <v>257.32</v>
       </c>
       <c r="I373" t="n">
-        <v>11.78</v>
+        <v>-6.05</v>
       </c>
       <c r="J373" t="n">
-        <v>11.81</v>
+        <v>0</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>GALO4</t>
+          <t>ECIS4</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
@@ -15365,7 +15365,7 @@
         </is>
       </c>
       <c r="D374" t="n">
-        <v>0.25</v>
+        <v>145</v>
       </c>
       <c r="E374" t="inlineStr">
         <is>
@@ -15373,30 +15373,30 @@
         </is>
       </c>
       <c r="F374" t="n">
-        <v>-60607000</v>
+        <v>129346000</v>
       </c>
       <c r="G374" t="n">
         <v>0</v>
       </c>
       <c r="H374" t="n">
-        <v>13.98</v>
+        <v>34.9</v>
       </c>
       <c r="I374" t="n">
-        <v>39.37</v>
+        <v>12.48</v>
       </c>
       <c r="J374" t="n">
-        <v>7.62</v>
+        <v>7.33</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>BBTG13</t>
+          <t>TNEP3</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
@@ -15405,7 +15405,7 @@
         </is>
       </c>
       <c r="D375" t="n">
-        <v>0</v>
+        <v>3.01</v>
       </c>
       <c r="E375" t="inlineStr">
         <is>
@@ -15413,30 +15413,30 @@
         </is>
       </c>
       <c r="F375" t="n">
-        <v>7000</v>
+        <v>955105000</v>
       </c>
       <c r="G375" t="n">
         <v>0</v>
       </c>
       <c r="H375" t="n">
-        <v>0</v>
+        <v>20.92</v>
       </c>
       <c r="I375" t="n">
-        <v>0</v>
+        <v>20.53</v>
       </c>
       <c r="J375" t="n">
-        <v>-42.86</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>VSPT3</t>
+          <t>LECO3</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa LECO</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
@@ -15453,39 +15453,39 @@
         </is>
       </c>
       <c r="F376" t="n">
-        <v>5031600000</v>
+        <v>105928000</v>
       </c>
       <c r="G376" t="n">
         <v>0</v>
       </c>
       <c r="H376" t="n">
-        <v>0</v>
+        <v>-2.14</v>
       </c>
       <c r="I376" t="n">
-        <v>0</v>
+        <v>-3.48</v>
       </c>
       <c r="J376" t="n">
-        <v>0</v>
+        <v>-14.82</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>SGEN4</t>
+          <t>VGOR3</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa VGOR</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D377" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -15493,19 +15493,19 @@
         </is>
       </c>
       <c r="F377" t="n">
-        <v>156981000</v>
+        <v>135178000</v>
       </c>
       <c r="G377" t="n">
         <v>0</v>
       </c>
       <c r="H377" t="n">
-        <v>-1871.17</v>
+        <v>4.5</v>
       </c>
       <c r="I377" t="n">
-        <v>-1.59</v>
+        <v>6</v>
       </c>
       <c r="J377" t="n">
-        <v>0</v>
+        <v>-24.29</v>
       </c>
     </row>
     <row r="378">
@@ -22911,7 +22911,7 @@
     <row r="563">
       <c r="A563" t="inlineStr">
         <is>
-          <t>CIQU3</t>
+          <t>CIQU4</t>
         </is>
       </c>
       <c r="B563" t="inlineStr">
@@ -22921,7 +22921,7 @@
       </c>
       <c r="C563" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D563" t="n">
@@ -22951,7 +22951,7 @@
     <row r="564">
       <c r="A564" t="inlineStr">
         <is>
-          <t>CIQU4</t>
+          <t>CIQU3</t>
         </is>
       </c>
       <c r="B564" t="inlineStr">
@@ -22961,7 +22961,7 @@
       </c>
       <c r="C564" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D564" t="n">
@@ -25151,7 +25151,7 @@
     <row r="619">
       <c r="A619" t="inlineStr">
         <is>
-          <t>AESL3</t>
+          <t>AESL4</t>
         </is>
       </c>
       <c r="B619" t="inlineStr">
@@ -25161,7 +25161,7 @@
       </c>
       <c r="C619" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D619" t="n">
@@ -25191,7 +25191,7 @@
     <row r="620">
       <c r="A620" t="inlineStr">
         <is>
-          <t>AESL4</t>
+          <t>AESL3</t>
         </is>
       </c>
       <c r="B620" t="inlineStr">
@@ -25201,7 +25201,7 @@
       </c>
       <c r="C620" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D620" t="n">

</xml_diff>

<commit_message>
Padroniza mapeamento de setores B3 para relatorios graficos
</commit_message>
<xml_diff>
--- a/acoes_b3.xlsx
+++ b/acoes_b3.xlsx
@@ -491,12 +491,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>IVTT3</t>
+          <t>CLAN3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Empresa IVTT</t>
+          <t>Empresa CLAN</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -522,7 +522,7 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>1083050000</v>
+        <v>1012240000</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -537,13 +537,13 @@
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>-0.4</v>
+        <v>-1.05</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MNSA3</t>
+          <t>MNSA4</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -553,11 +553,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.42</v>
+        <v>0.47</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -595,7 +595,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CSTB3</t>
+          <t>CSTB4</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -605,11 +605,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>150</v>
+        <v>147.69</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -647,12 +647,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CFLU4</t>
+          <t>PORP4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Empresa CFLU</t>
+          <t>Empresa PORP</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -661,7 +661,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1000</v>
+        <v>2.4</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -678,42 +678,42 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>60351000</v>
+        <v>22399000</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>8.880000000000001</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>10.72</v>
+        <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>17.68</v>
+        <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>32.15</v>
+        <v>-2.08</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>POPR4</t>
+          <t>IVTT3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Empresa POPR</t>
+          <t>Empresa IVTT</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>10.17</v>
+        <v>0</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -730,33 +730,33 @@
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>545803000</v>
+        <v>1083050000</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>8.66</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>5.65</v>
+        <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>15.25</v>
+        <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>19.93</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PMET3</t>
+          <t>MNSA3</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Empresa PMET</t>
+          <t>Empresa MNSA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>0.42</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -782,42 +782,42 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>-290863000</v>
+        <v>-9105000</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>-208.15</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>-362.66</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>-13.5</v>
       </c>
       <c r="N7" t="n">
-        <v>4.1</v>
+        <v>145.7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CLAN3</t>
+          <t>CFLU4</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Empresa CLAN</t>
+          <t>Empresa CFLU</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -834,42 +834,42 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>1012240000</v>
+        <v>60351000</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>10.72</v>
       </c>
       <c r="M8" t="n">
-        <v>0</v>
+        <v>17.68</v>
       </c>
       <c r="N8" t="n">
-        <v>-1.05</v>
+        <v>32.15</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MNSA4</t>
+          <t>CSTB3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Empresa MNSA</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.47</v>
+        <v>150</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -886,33 +886,33 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>-9105000</v>
+        <v>8420670000</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>-208.15</v>
+        <v>40.85</v>
       </c>
       <c r="L9" t="n">
-        <v>-362.66</v>
+        <v>28.98</v>
       </c>
       <c r="M9" t="n">
-        <v>-13.5</v>
+        <v>22.4</v>
       </c>
       <c r="N9" t="n">
-        <v>145.7</v>
+        <v>20.11</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CSTB4</t>
+          <t>POPR4</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa POPR</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -921,7 +921,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>147.69</v>
+        <v>10.17</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -938,42 +938,42 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>8420670000</v>
+        <v>545803000</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>40.85</v>
+        <v>8.66</v>
       </c>
       <c r="L10" t="n">
-        <v>28.98</v>
+        <v>5.65</v>
       </c>
       <c r="M10" t="n">
-        <v>22.4</v>
+        <v>15.25</v>
       </c>
       <c r="N10" t="n">
-        <v>20.11</v>
+        <v>19.93</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PORP4</t>
+          <t>PMET3</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Empresa PORP</t>
+          <t>Empresa PMET</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2.4</v>
+        <v>0</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -990,7 +990,7 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>22399000</v>
+        <v>-290863000</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -1005,7 +1005,7 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>-2.08</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="12">
@@ -7997,7 +7997,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Siderúrgica Nacional</t>
+          <t>Mineração e Siderurgia</t>
         </is>
       </c>
       <c r="F146" t="n">
@@ -8135,7 +8135,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>PNOR6</t>
+          <t>PNOR5</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -8187,7 +8187,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>PNOR5</t>
+          <t>PNOR6</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -8863,7 +8863,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>RNEW3</t>
+          <t>RNEW4</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -8873,7 +8873,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8897,7 +8897,7 @@
         <v>1150280000</v>
       </c>
       <c r="J163" t="n">
-        <v>45273.4</v>
+        <v>44097</v>
       </c>
       <c r="K163" t="n">
         <v>-2.89</v>
@@ -8915,7 +8915,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>RNEW4</t>
+          <t>RNEW3</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -8925,7 +8925,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8949,7 +8949,7 @@
         <v>1150280000</v>
       </c>
       <c r="J164" t="n">
-        <v>44097</v>
+        <v>45273.4</v>
       </c>
       <c r="K164" t="n">
         <v>-2.89</v>
@@ -10111,7 +10111,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>SDIA4</t>
+          <t>SDIA3</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -10121,7 +10121,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -10163,7 +10163,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>SDIA3</t>
+          <t>SDIA4</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -10173,7 +10173,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -12937,7 +12937,7 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Saúde e Farmácia</t>
         </is>
       </c>
       <c r="F241" t="n">
@@ -16455,12 +16455,12 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>BERG3</t>
+          <t>BPNM3</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Empresa BERG</t>
+          <t>Empresa BPNM</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -16469,7 +16469,7 @@
         </is>
       </c>
       <c r="D309" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -16486,33 +16486,33 @@
         <v>0</v>
       </c>
       <c r="I309" t="n">
-        <v>9538000</v>
+        <v>7792670000</v>
       </c>
       <c r="J309" t="n">
         <v>0</v>
       </c>
       <c r="K309" t="n">
-        <v>-8.6</v>
+        <v>0</v>
       </c>
       <c r="L309" t="n">
-        <v>-32.6</v>
+        <v>0</v>
       </c>
       <c r="M309" t="n">
-        <v>-5.58</v>
+        <v>0</v>
       </c>
       <c r="N309" t="n">
-        <v>-102.71</v>
+        <v>9.67</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>JBDU3</t>
+          <t>BSGR3</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Empresa JBDU</t>
+          <t>Empresa BSGR</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -16521,7 +16521,7 @@
         </is>
       </c>
       <c r="D310" t="n">
-        <v>0</v>
+        <v>1091.28</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -16538,7 +16538,7 @@
         <v>0</v>
       </c>
       <c r="I310" t="n">
-        <v>56569000</v>
+        <v>0</v>
       </c>
       <c r="J310" t="n">
         <v>0</v>
@@ -16559,12 +16559,12 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>EGGY3</t>
+          <t>CBMA3</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Empresa EGGY</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -16573,7 +16573,7 @@
         </is>
       </c>
       <c r="D311" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -16590,7 +16590,7 @@
         <v>0</v>
       </c>
       <c r="I311" t="n">
-        <v>954480000</v>
+        <v>-34022300000</v>
       </c>
       <c r="J311" t="n">
         <v>0</v>
@@ -16611,21 +16611,21 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>CBMA4</t>
+          <t>ALBA3</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa ALBA</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>0.01</v>
+        <v>2.15</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -16642,33 +16642,33 @@
         <v>0</v>
       </c>
       <c r="I312" t="n">
-        <v>-34022300000</v>
+        <v>354860000</v>
       </c>
       <c r="J312" t="n">
         <v>0</v>
       </c>
       <c r="K312" t="n">
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="L312" t="n">
-        <v>0</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="M312" t="n">
-        <v>0</v>
+        <v>20.4</v>
       </c>
       <c r="N312" t="n">
-        <v>0</v>
+        <v>19.77</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>SALM4</t>
+          <t>ARPS4</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -16677,7 +16677,7 @@
         </is>
       </c>
       <c r="D313" t="n">
-        <v>5.9</v>
+        <v>0</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -16694,33 +16694,33 @@
         <v>0</v>
       </c>
       <c r="I313" t="n">
-        <v>475600000</v>
+        <v>-12690000</v>
       </c>
       <c r="J313" t="n">
         <v>0</v>
       </c>
       <c r="K313" t="n">
-        <v>10.22</v>
+        <v>-4.92</v>
       </c>
       <c r="L313" t="n">
-        <v>4.13</v>
+        <v>-11.59</v>
       </c>
       <c r="M313" t="n">
-        <v>25.78</v>
+        <v>-6.64</v>
       </c>
       <c r="N313" t="n">
-        <v>19.53</v>
+        <v>20.34</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>BMEF3</t>
+          <t>SALM3</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Empresa BMEF</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -16729,7 +16729,7 @@
         </is>
       </c>
       <c r="D314" t="n">
-        <v>11</v>
+        <v>5.7</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -16740,48 +16740,48 @@
         <v>0</v>
       </c>
       <c r="G314" t="n">
-        <v>4.16</v>
+        <v>0</v>
       </c>
       <c r="H314" t="n">
         <v>0</v>
       </c>
       <c r="I314" t="n">
-        <v>2674780000</v>
+        <v>475600000</v>
       </c>
       <c r="J314" t="n">
         <v>0</v>
       </c>
       <c r="K314" t="n">
-        <v>0</v>
+        <v>10.22</v>
       </c>
       <c r="L314" t="n">
-        <v>0</v>
+        <v>4.13</v>
       </c>
       <c r="M314" t="n">
-        <v>0</v>
+        <v>25.78</v>
       </c>
       <c r="N314" t="n">
-        <v>0</v>
+        <v>19.53</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>AGEI3</t>
+          <t>CMMA4</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Empresa AGEI</t>
+          <t>Empresa CMMA</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>7.8</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -16792,13 +16792,13 @@
         <v>0</v>
       </c>
       <c r="G315" t="n">
-        <v>1.25</v>
+        <v>0</v>
       </c>
       <c r="H315" t="n">
         <v>0</v>
       </c>
       <c r="I315" t="n">
-        <v>1878210000</v>
+        <v>-79623000</v>
       </c>
       <c r="J315" t="n">
         <v>0</v>
@@ -16813,18 +16813,18 @@
         <v>0</v>
       </c>
       <c r="N315" t="n">
-        <v>0</v>
+        <v>-1.92</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>SASG3</t>
+          <t>CZRS3</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Empresa SASG</t>
+          <t>Empresa CZRS</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -16833,7 +16833,7 @@
         </is>
       </c>
       <c r="D316" t="n">
-        <v>0.98</v>
+        <v>0</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -16850,7 +16850,7 @@
         <v>0</v>
       </c>
       <c r="I316" t="n">
-        <v>0</v>
+        <v>1145670000</v>
       </c>
       <c r="J316" t="n">
         <v>0</v>
@@ -16865,18 +16865,18 @@
         <v>0</v>
       </c>
       <c r="N316" t="n">
-        <v>0</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>ODER3</t>
+          <t>VNET3</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Empresa ODER</t>
+          <t>Empresa VNET</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -16902,7 +16902,7 @@
         <v>0</v>
       </c>
       <c r="I317" t="n">
-        <v>609518000</v>
+        <v>14163000000</v>
       </c>
       <c r="J317" t="n">
         <v>0</v>
@@ -16923,21 +16923,21 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>ARPS3</t>
+          <t>CSPC4</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>0.3</v>
+        <v>1.2</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -16954,42 +16954,42 @@
         <v>0</v>
       </c>
       <c r="I318" t="n">
-        <v>-12690000</v>
+        <v>2126670000</v>
       </c>
       <c r="J318" t="n">
         <v>0</v>
       </c>
       <c r="K318" t="n">
-        <v>-4.92</v>
+        <v>38.62</v>
       </c>
       <c r="L318" t="n">
-        <v>-11.59</v>
+        <v>18.85</v>
       </c>
       <c r="M318" t="n">
-        <v>-6.64</v>
+        <v>29.18</v>
       </c>
       <c r="N318" t="n">
-        <v>20.34</v>
+        <v>45.33</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>VVAX4</t>
+          <t>BOVH3</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa BOVH</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>0</v>
+        <v>15.71</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -17000,39 +17000,39 @@
         <v>0</v>
       </c>
       <c r="G319" t="n">
-        <v>0</v>
+        <v>6.16</v>
       </c>
       <c r="H319" t="n">
         <v>0</v>
       </c>
       <c r="I319" t="n">
-        <v>144676000</v>
+        <v>1843320000</v>
       </c>
       <c r="J319" t="n">
         <v>0</v>
       </c>
       <c r="K319" t="n">
-        <v>-7.36</v>
+        <v>0</v>
       </c>
       <c r="L319" t="n">
-        <v>-37.76</v>
+        <v>0</v>
       </c>
       <c r="M319" t="n">
-        <v>-6.52</v>
+        <v>0</v>
       </c>
       <c r="N319" t="n">
-        <v>-92.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>CSPC3</t>
+          <t>ARND3</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa ARND</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -17041,7 +17041,7 @@
         </is>
       </c>
       <c r="D320" t="n">
-        <v>1.24</v>
+        <v>0.51</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -17052,39 +17052,39 @@
         <v>0</v>
       </c>
       <c r="G320" t="n">
-        <v>0</v>
+        <v>0.57</v>
       </c>
       <c r="H320" t="n">
         <v>0</v>
       </c>
       <c r="I320" t="n">
-        <v>2126670000</v>
+        <v>125211000</v>
       </c>
       <c r="J320" t="n">
-        <v>0</v>
+        <v>913.58</v>
       </c>
       <c r="K320" t="n">
-        <v>38.62</v>
+        <v>0</v>
       </c>
       <c r="L320" t="n">
-        <v>18.85</v>
+        <v>0</v>
       </c>
       <c r="M320" t="n">
-        <v>29.18</v>
+        <v>0</v>
       </c>
       <c r="N320" t="n">
-        <v>45.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>ABCB3</t>
+          <t>INHA3</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Empresa ABCB</t>
+          <t>Empresa INHA</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -17097,7 +17097,7 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>Bancos</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="F321" t="n">
@@ -17110,42 +17110,42 @@
         <v>0</v>
       </c>
       <c r="I321" t="n">
-        <v>7258910000</v>
+        <v>1533210000</v>
       </c>
       <c r="J321" t="n">
         <v>0</v>
       </c>
       <c r="K321" t="n">
-        <v>0</v>
+        <v>-56.05</v>
       </c>
       <c r="L321" t="n">
-        <v>0</v>
+        <v>-124.06</v>
       </c>
       <c r="M321" t="n">
-        <v>0</v>
+        <v>-6.27</v>
       </c>
       <c r="N321" t="n">
-        <v>14.05</v>
+        <v>-39.87</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>CCTY3</t>
+          <t>PTIP4</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Empresa CCTY</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>0</v>
+        <v>25.15</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -17162,42 +17162,42 @@
         <v>0</v>
       </c>
       <c r="I322" t="n">
-        <v>0</v>
+        <v>-155957000</v>
       </c>
       <c r="J322" t="n">
         <v>0</v>
       </c>
       <c r="K322" t="n">
-        <v>0</v>
+        <v>13.73</v>
       </c>
       <c r="L322" t="n">
-        <v>0</v>
+        <v>7.55</v>
       </c>
       <c r="M322" t="n">
-        <v>0</v>
+        <v>23.13</v>
       </c>
       <c r="N322" t="n">
-        <v>0</v>
+        <v>-121.74</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>BAUH4</t>
+          <t>LATS3</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Empresa BAUH</t>
+          <t>Empresa LATS</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D323" t="n">
-        <v>93.39</v>
+        <v>22</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -17208,39 +17208,39 @@
         <v>0</v>
       </c>
       <c r="G323" t="n">
-        <v>3.18</v>
+        <v>0</v>
       </c>
       <c r="H323" t="n">
-        <v>1.16</v>
+        <v>0</v>
       </c>
       <c r="I323" t="n">
-        <v>153407000</v>
+        <v>680646000</v>
       </c>
       <c r="J323" t="n">
-        <v>207.53</v>
+        <v>0</v>
       </c>
       <c r="K323" t="n">
-        <v>0</v>
+        <v>11.74</v>
       </c>
       <c r="L323" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="M323" t="n">
-        <v>0</v>
+        <v>11.63</v>
       </c>
       <c r="N323" t="n">
-        <v>0</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>ICPI3</t>
+          <t>VVAX3</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Empresa ICPI</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -17266,33 +17266,33 @@
         <v>0</v>
       </c>
       <c r="I324" t="n">
-        <v>0</v>
+        <v>144676000</v>
       </c>
       <c r="J324" t="n">
         <v>0</v>
       </c>
       <c r="K324" t="n">
-        <v>0</v>
+        <v>-7.36</v>
       </c>
       <c r="L324" t="n">
-        <v>0</v>
+        <v>-37.76</v>
       </c>
       <c r="M324" t="n">
-        <v>0</v>
+        <v>-6.52</v>
       </c>
       <c r="N324" t="n">
-        <v>0</v>
+        <v>-92.03</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>ILLS4</t>
+          <t>MSAN4</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Empresa ILLS</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -17301,7 +17301,7 @@
         </is>
       </c>
       <c r="D325" t="n">
-        <v>100.01</v>
+        <v>6.44</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -17318,42 +17318,42 @@
         <v>0</v>
       </c>
       <c r="I325" t="n">
-        <v>-18567000</v>
+        <v>2533030000</v>
       </c>
       <c r="J325" t="n">
         <v>0</v>
       </c>
       <c r="K325" t="n">
-        <v>8.43</v>
+        <v>6.27</v>
       </c>
       <c r="L325" t="n">
-        <v>-10.22</v>
+        <v>2.42</v>
       </c>
       <c r="M325" t="n">
-        <v>8.140000000000001</v>
+        <v>11.78</v>
       </c>
       <c r="N325" t="n">
-        <v>36.09</v>
+        <v>11.81</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>BPAT33</t>
+          <t>GALO4</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Empresa BPAT</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>20</v>
+        <v>0.25</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -17364,44 +17364,44 @@
         <v>0</v>
       </c>
       <c r="G326" t="n">
-        <v>0.82</v>
+        <v>0</v>
       </c>
       <c r="H326" t="n">
-        <v>35.72</v>
+        <v>0</v>
       </c>
       <c r="I326" t="n">
-        <v>876492000</v>
+        <v>-60607000</v>
       </c>
       <c r="J326" t="n">
         <v>0</v>
       </c>
       <c r="K326" t="n">
-        <v>0</v>
+        <v>13.98</v>
       </c>
       <c r="L326" t="n">
-        <v>0</v>
+        <v>-184.58</v>
       </c>
       <c r="M326" t="n">
-        <v>0</v>
+        <v>39.37</v>
       </c>
       <c r="N326" t="n">
-        <v>0</v>
+        <v>7.62</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>ESTC4</t>
+          <t>BBTG13</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Empresa ESTC</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D327" t="n">
@@ -17422,28 +17422,28 @@
         <v>0</v>
       </c>
       <c r="I327" t="n">
-        <v>2916530000</v>
+        <v>7000</v>
       </c>
       <c r="J327" t="n">
         <v>0</v>
       </c>
       <c r="K327" t="n">
-        <v>16.91</v>
+        <v>0</v>
       </c>
       <c r="L327" t="n">
-        <v>2.02</v>
+        <v>0</v>
       </c>
       <c r="M327" t="n">
-        <v>11.35</v>
+        <v>0</v>
       </c>
       <c r="N327" t="n">
-        <v>3.89</v>
+        <v>-42.86</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>VSPT4</t>
+          <t>VSPT3</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
@@ -17453,7 +17453,7 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D328" t="n">
@@ -17495,12 +17495,12 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>SEBB4</t>
+          <t>SGEN4</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -17509,7 +17509,7 @@
         </is>
       </c>
       <c r="D329" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -17520,48 +17520,48 @@
         <v>0</v>
       </c>
       <c r="G329" t="n">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="H329" t="n">
         <v>0</v>
       </c>
       <c r="I329" t="n">
-        <v>145783000</v>
+        <v>156981000</v>
       </c>
       <c r="J329" t="n">
         <v>0</v>
       </c>
       <c r="K329" t="n">
-        <v>9.24</v>
+        <v>-1871.17</v>
       </c>
       <c r="L329" t="n">
-        <v>7.4</v>
+        <v>0</v>
       </c>
       <c r="M329" t="n">
-        <v>24.15</v>
+        <v>-1.59</v>
       </c>
       <c r="N329" t="n">
-        <v>23.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>MSAN3</t>
+          <t>JFAB4</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa JFAB</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>6.44</v>
+        <v>0.06</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -17578,42 +17578,42 @@
         <v>0</v>
       </c>
       <c r="I330" t="n">
-        <v>2533030000</v>
+        <v>-10183000</v>
       </c>
       <c r="J330" t="n">
         <v>0</v>
       </c>
       <c r="K330" t="n">
-        <v>6.27</v>
+        <v>0</v>
       </c>
       <c r="L330" t="n">
-        <v>2.42</v>
+        <v>0</v>
       </c>
       <c r="M330" t="n">
-        <v>11.78</v>
+        <v>0</v>
       </c>
       <c r="N330" t="n">
-        <v>11.81</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>GALO3</t>
+          <t>CCHI4</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -17624,39 +17624,39 @@
         <v>0</v>
       </c>
       <c r="G331" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="H331" t="n">
         <v>0</v>
       </c>
       <c r="I331" t="n">
-        <v>-60607000</v>
+        <v>-160477000</v>
       </c>
       <c r="J331" t="n">
         <v>0</v>
       </c>
       <c r="K331" t="n">
-        <v>13.98</v>
+        <v>0</v>
       </c>
       <c r="L331" t="n">
-        <v>-184.58</v>
+        <v>0</v>
       </c>
       <c r="M331" t="n">
-        <v>39.37</v>
+        <v>0</v>
       </c>
       <c r="N331" t="n">
-        <v>7.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>SLCP3</t>
+          <t>REPA3</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Empresa SLCP</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -17665,7 +17665,7 @@
         </is>
       </c>
       <c r="D332" t="n">
-        <v>610.02</v>
+        <v>1</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -17682,38 +17682,38 @@
         <v>0</v>
       </c>
       <c r="I332" t="n">
-        <v>0</v>
+        <v>378378000</v>
       </c>
       <c r="J332" t="n">
         <v>0</v>
       </c>
       <c r="K332" t="n">
-        <v>0</v>
+        <v>5.18</v>
       </c>
       <c r="L332" t="n">
-        <v>0</v>
+        <v>1.22</v>
       </c>
       <c r="M332" t="n">
-        <v>0</v>
+        <v>4.05</v>
       </c>
       <c r="N332" t="n">
-        <v>0</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>DAYC3</t>
+          <t>EQMA5B</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Empresa DAYC</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D333" t="n">
@@ -17734,7 +17734,7 @@
         <v>0</v>
       </c>
       <c r="I333" t="n">
-        <v>3009030000</v>
+        <v>4940330000</v>
       </c>
       <c r="J333" t="n">
         <v>0</v>
@@ -17749,18 +17749,18 @@
         <v>0</v>
       </c>
       <c r="N333" t="n">
-        <v>17.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>PTIP3</t>
+          <t>SEBB3</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -17769,7 +17769,7 @@
         </is>
       </c>
       <c r="D334" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -17786,33 +17786,33 @@
         <v>0</v>
       </c>
       <c r="I334" t="n">
-        <v>-155957000</v>
+        <v>145783000</v>
       </c>
       <c r="J334" t="n">
         <v>0</v>
       </c>
       <c r="K334" t="n">
-        <v>13.73</v>
+        <v>9.24</v>
       </c>
       <c r="L334" t="n">
-        <v>7.55</v>
+        <v>7.4</v>
       </c>
       <c r="M334" t="n">
-        <v>23.13</v>
+        <v>24.15</v>
       </c>
       <c r="N334" t="n">
-        <v>-121.74</v>
+        <v>23.01</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>REPA4</t>
+          <t>BBTG11</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -17821,7 +17821,7 @@
         </is>
       </c>
       <c r="D335" t="n">
-        <v>1.08</v>
+        <v>15.01</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -17838,33 +17838,33 @@
         <v>0</v>
       </c>
       <c r="I335" t="n">
-        <v>378378000</v>
+        <v>0</v>
       </c>
       <c r="J335" t="n">
         <v>0</v>
       </c>
       <c r="K335" t="n">
-        <v>5.18</v>
+        <v>0</v>
       </c>
       <c r="L335" t="n">
-        <v>1.22</v>
+        <v>0</v>
       </c>
       <c r="M335" t="n">
-        <v>4.05</v>
+        <v>0</v>
       </c>
       <c r="N335" t="n">
-        <v>1.91</v>
+        <v>0</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>EQMA6B</t>
+          <t>ECIS4</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -17873,7 +17873,7 @@
         </is>
       </c>
       <c r="D336" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -17890,33 +17890,33 @@
         <v>0</v>
       </c>
       <c r="I336" t="n">
-        <v>4940330000</v>
+        <v>129346000</v>
       </c>
       <c r="J336" t="n">
         <v>0</v>
       </c>
       <c r="K336" t="n">
-        <v>0</v>
+        <v>34.9</v>
       </c>
       <c r="L336" t="n">
-        <v>0</v>
+        <v>14.18</v>
       </c>
       <c r="M336" t="n">
-        <v>0</v>
+        <v>12.48</v>
       </c>
       <c r="N336" t="n">
-        <v>0</v>
+        <v>7.33</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>SGEN3</t>
+          <t>TNEP3</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -17925,7 +17925,7 @@
         </is>
       </c>
       <c r="D337" t="n">
-        <v>5</v>
+        <v>3.01</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -17936,44 +17936,44 @@
         <v>0</v>
       </c>
       <c r="G337" t="n">
-        <v>0.77</v>
+        <v>0</v>
       </c>
       <c r="H337" t="n">
         <v>0</v>
       </c>
       <c r="I337" t="n">
-        <v>156981000</v>
+        <v>955105000</v>
       </c>
       <c r="J337" t="n">
         <v>0</v>
       </c>
       <c r="K337" t="n">
-        <v>-1871.17</v>
+        <v>20.92</v>
       </c>
       <c r="L337" t="n">
-        <v>0</v>
+        <v>25.42</v>
       </c>
       <c r="M337" t="n">
-        <v>-1.59</v>
+        <v>20.53</v>
       </c>
       <c r="N337" t="n">
-        <v>0</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>DUFB11</t>
+          <t>LECO3</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Empresa DUFB</t>
+          <t>Empresa LECO</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D338" t="n">
@@ -17994,42 +17994,42 @@
         <v>0</v>
       </c>
       <c r="I338" t="n">
-        <v>0</v>
+        <v>105928000</v>
       </c>
       <c r="J338" t="n">
         <v>0</v>
       </c>
       <c r="K338" t="n">
-        <v>0</v>
+        <v>-2.14</v>
       </c>
       <c r="L338" t="n">
-        <v>0</v>
+        <v>-4.72</v>
       </c>
       <c r="M338" t="n">
-        <v>0</v>
+        <v>-3.48</v>
       </c>
       <c r="N338" t="n">
-        <v>0</v>
+        <v>-14.82</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>TNEP4</t>
+          <t>VGOR3</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa VGOR</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>3.95</v>
+        <v>0</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -18046,33 +18046,33 @@
         <v>0</v>
       </c>
       <c r="I339" t="n">
-        <v>955105000</v>
+        <v>135178000</v>
       </c>
       <c r="J339" t="n">
         <v>0</v>
       </c>
       <c r="K339" t="n">
-        <v>20.92</v>
+        <v>4.5</v>
       </c>
       <c r="L339" t="n">
-        <v>25.42</v>
+        <v>-4.59</v>
       </c>
       <c r="M339" t="n">
-        <v>20.53</v>
+        <v>6</v>
       </c>
       <c r="N339" t="n">
-        <v>22.8</v>
+        <v>-24.29</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>MLPA3</t>
+          <t>GPIV33</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Empresa MLPA</t>
+          <t>Empresa GPIV</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -18081,7 +18081,7 @@
         </is>
       </c>
       <c r="D340" t="n">
-        <v>0</v>
+        <v>4.42</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -18092,44 +18092,44 @@
         <v>0</v>
       </c>
       <c r="G340" t="n">
-        <v>0</v>
+        <v>0.23</v>
       </c>
       <c r="H340" t="n">
         <v>0</v>
       </c>
       <c r="I340" t="n">
-        <v>44578000</v>
+        <v>1318490000</v>
       </c>
       <c r="J340" t="n">
         <v>0</v>
       </c>
       <c r="K340" t="n">
-        <v>6.66</v>
+        <v>257.32</v>
       </c>
       <c r="L340" t="n">
-        <v>8.92</v>
+        <v>0</v>
       </c>
       <c r="M340" t="n">
-        <v>0</v>
+        <v>-6.05</v>
       </c>
       <c r="N340" t="n">
-        <v>45.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>CLSC6</t>
+          <t>JBDU3</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Empresa CLSC</t>
+          <t>Empresa JBDU</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D341" t="n">
@@ -18150,7 +18150,7 @@
         <v>0</v>
       </c>
       <c r="I341" t="n">
-        <v>4228180000</v>
+        <v>56569000</v>
       </c>
       <c r="J341" t="n">
         <v>0</v>
@@ -18171,12 +18171,12 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>CCHI3</t>
+          <t>EGGY3</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa EGGY</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -18185,7 +18185,7 @@
         </is>
       </c>
       <c r="D342" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -18196,13 +18196,13 @@
         <v>0</v>
       </c>
       <c r="G342" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="H342" t="n">
         <v>0</v>
       </c>
       <c r="I342" t="n">
-        <v>-160477000</v>
+        <v>954480000</v>
       </c>
       <c r="J342" t="n">
         <v>0</v>
@@ -18223,21 +18223,21 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>SFSA3</t>
+          <t>CBMA4</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Empresa SFSA</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -18254,7 +18254,7 @@
         <v>0</v>
       </c>
       <c r="I343" t="n">
-        <v>739524000</v>
+        <v>-34022300000</v>
       </c>
       <c r="J343" t="n">
         <v>0</v>
@@ -18269,27 +18269,27 @@
         <v>0</v>
       </c>
       <c r="N343" t="n">
-        <v>6.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>PRBC3</t>
+          <t>SALM4</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Empresa PRBC</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -18306,33 +18306,33 @@
         <v>0</v>
       </c>
       <c r="I344" t="n">
-        <v>1319270000</v>
+        <v>475600000</v>
       </c>
       <c r="J344" t="n">
         <v>0</v>
       </c>
       <c r="K344" t="n">
-        <v>0</v>
+        <v>10.22</v>
       </c>
       <c r="L344" t="n">
-        <v>0</v>
+        <v>4.13</v>
       </c>
       <c r="M344" t="n">
-        <v>0</v>
+        <v>25.78</v>
       </c>
       <c r="N344" t="n">
-        <v>8.27</v>
+        <v>19.53</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>ECIS3</t>
+          <t>BERG3</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa BERG</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -18341,7 +18341,7 @@
         </is>
       </c>
       <c r="D345" t="n">
-        <v>211.65</v>
+        <v>33</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -18358,33 +18358,33 @@
         <v>0</v>
       </c>
       <c r="I345" t="n">
-        <v>129346000</v>
+        <v>9538000</v>
       </c>
       <c r="J345" t="n">
         <v>0</v>
       </c>
       <c r="K345" t="n">
-        <v>34.9</v>
+        <v>-8.6</v>
       </c>
       <c r="L345" t="n">
-        <v>14.18</v>
+        <v>-32.6</v>
       </c>
       <c r="M345" t="n">
-        <v>12.48</v>
+        <v>-5.58</v>
       </c>
       <c r="N345" t="n">
-        <v>7.33</v>
+        <v>-102.71</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>CZRS3</t>
+          <t>AGEI3</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Empresa CZRS</t>
+          <t>Empresa AGEI</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
@@ -18393,7 +18393,7 @@
         </is>
       </c>
       <c r="D346" t="n">
-        <v>0</v>
+        <v>7.8</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -18404,13 +18404,13 @@
         <v>0</v>
       </c>
       <c r="G346" t="n">
-        <v>0</v>
+        <v>1.25</v>
       </c>
       <c r="H346" t="n">
         <v>0</v>
       </c>
       <c r="I346" t="n">
-        <v>1145670000</v>
+        <v>1878210000</v>
       </c>
       <c r="J346" t="n">
         <v>0</v>
@@ -18425,18 +18425,18 @@
         <v>0</v>
       </c>
       <c r="N346" t="n">
-        <v>3.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>BPNM3</t>
+          <t>SASG3</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Empresa BPNM</t>
+          <t>Empresa SASG</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
@@ -18445,7 +18445,7 @@
         </is>
       </c>
       <c r="D347" t="n">
-        <v>0</v>
+        <v>0.98</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -18462,7 +18462,7 @@
         <v>0</v>
       </c>
       <c r="I347" t="n">
-        <v>7792670000</v>
+        <v>0</v>
       </c>
       <c r="J347" t="n">
         <v>0</v>
@@ -18477,18 +18477,18 @@
         <v>0</v>
       </c>
       <c r="N347" t="n">
-        <v>9.67</v>
+        <v>0</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>BSGR3</t>
+          <t>BMEF3</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Empresa BSGR</t>
+          <t>Empresa BMEF</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
@@ -18497,7 +18497,7 @@
         </is>
       </c>
       <c r="D348" t="n">
-        <v>1091.28</v>
+        <v>11</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -18508,13 +18508,13 @@
         <v>0</v>
       </c>
       <c r="G348" t="n">
-        <v>0</v>
+        <v>4.16</v>
       </c>
       <c r="H348" t="n">
         <v>0</v>
       </c>
       <c r="I348" t="n">
-        <v>0</v>
+        <v>2674780000</v>
       </c>
       <c r="J348" t="n">
         <v>0</v>
@@ -18535,12 +18535,12 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>CBMA3</t>
+          <t>ARPS3</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
@@ -18549,7 +18549,7 @@
         </is>
       </c>
       <c r="D349" t="n">
-        <v>0.01</v>
+        <v>0.3</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -18566,33 +18566,33 @@
         <v>0</v>
       </c>
       <c r="I349" t="n">
-        <v>-34022300000</v>
+        <v>-12690000</v>
       </c>
       <c r="J349" t="n">
         <v>0</v>
       </c>
       <c r="K349" t="n">
-        <v>0</v>
+        <v>-4.92</v>
       </c>
       <c r="L349" t="n">
-        <v>0</v>
+        <v>-11.59</v>
       </c>
       <c r="M349" t="n">
-        <v>0</v>
+        <v>-6.64</v>
       </c>
       <c r="N349" t="n">
-        <v>0</v>
+        <v>20.34</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>ALBA3</t>
+          <t>ODER3</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Empresa ALBA</t>
+          <t>Empresa ODER</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
@@ -18601,7 +18601,7 @@
         </is>
       </c>
       <c r="D350" t="n">
-        <v>2.15</v>
+        <v>0</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -18618,38 +18618,38 @@
         <v>0</v>
       </c>
       <c r="I350" t="n">
-        <v>354860000</v>
+        <v>609518000</v>
       </c>
       <c r="J350" t="n">
         <v>0</v>
       </c>
       <c r="K350" t="n">
-        <v>9.5</v>
+        <v>0</v>
       </c>
       <c r="L350" t="n">
-        <v>9.619999999999999</v>
+        <v>0</v>
       </c>
       <c r="M350" t="n">
-        <v>20.4</v>
+        <v>0</v>
       </c>
       <c r="N350" t="n">
-        <v>19.77</v>
+        <v>0</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>ARPS4</t>
+          <t>ABCB3</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa ABCB</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D351" t="n">
@@ -18657,7 +18657,7 @@
       </c>
       <c r="E351" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="F351" t="n">
@@ -18670,33 +18670,33 @@
         <v>0</v>
       </c>
       <c r="I351" t="n">
-        <v>-12690000</v>
+        <v>7258910000</v>
       </c>
       <c r="J351" t="n">
         <v>0</v>
       </c>
       <c r="K351" t="n">
-        <v>-4.92</v>
+        <v>0</v>
       </c>
       <c r="L351" t="n">
-        <v>-11.59</v>
+        <v>0</v>
       </c>
       <c r="M351" t="n">
-        <v>-6.64</v>
+        <v>0</v>
       </c>
       <c r="N351" t="n">
-        <v>20.34</v>
+        <v>14.05</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>SALM3</t>
+          <t>CCTY3</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa CCTY</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -18705,7 +18705,7 @@
         </is>
       </c>
       <c r="D352" t="n">
-        <v>5.7</v>
+        <v>0</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -18722,33 +18722,33 @@
         <v>0</v>
       </c>
       <c r="I352" t="n">
-        <v>475600000</v>
+        <v>0</v>
       </c>
       <c r="J352" t="n">
         <v>0</v>
       </c>
       <c r="K352" t="n">
-        <v>10.22</v>
+        <v>0</v>
       </c>
       <c r="L352" t="n">
-        <v>4.13</v>
+        <v>0</v>
       </c>
       <c r="M352" t="n">
-        <v>25.78</v>
+        <v>0</v>
       </c>
       <c r="N352" t="n">
-        <v>19.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>CMMA4</t>
+          <t>VVAX4</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Empresa CMMA</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -18757,7 +18757,7 @@
         </is>
       </c>
       <c r="D353" t="n">
-        <v>0.8100000000000001</v>
+        <v>0</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -18774,28 +18774,28 @@
         <v>0</v>
       </c>
       <c r="I353" t="n">
-        <v>-79623000</v>
+        <v>144676000</v>
       </c>
       <c r="J353" t="n">
         <v>0</v>
       </c>
       <c r="K353" t="n">
-        <v>0</v>
+        <v>-7.36</v>
       </c>
       <c r="L353" t="n">
-        <v>0</v>
+        <v>-37.76</v>
       </c>
       <c r="M353" t="n">
-        <v>0</v>
+        <v>-6.52</v>
       </c>
       <c r="N353" t="n">
-        <v>-1.92</v>
+        <v>-92.03</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>CSPC4</t>
+          <t>CSPC3</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
@@ -18805,11 +18805,11 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D354" t="n">
-        <v>1.2</v>
+        <v>1.24</v>
       </c>
       <c r="E354" t="inlineStr">
         <is>
@@ -18847,12 +18847,12 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>BOVH3</t>
+          <t>BPAT33</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Empresa BOVH</t>
+          <t>Empresa BPAT</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -18861,7 +18861,7 @@
         </is>
       </c>
       <c r="D355" t="n">
-        <v>15.71</v>
+        <v>20</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -18872,13 +18872,13 @@
         <v>0</v>
       </c>
       <c r="G355" t="n">
-        <v>6.16</v>
+        <v>0.82</v>
       </c>
       <c r="H355" t="n">
-        <v>0</v>
+        <v>35.72</v>
       </c>
       <c r="I355" t="n">
-        <v>1843320000</v>
+        <v>876492000</v>
       </c>
       <c r="J355" t="n">
         <v>0</v>
@@ -18899,17 +18899,17 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>VNET3</t>
+          <t>ESTC4</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Empresa VNET</t>
+          <t>Empresa ESTC</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D356" t="n">
@@ -18930,42 +18930,42 @@
         <v>0</v>
       </c>
       <c r="I356" t="n">
-        <v>14163000000</v>
+        <v>2916530000</v>
       </c>
       <c r="J356" t="n">
         <v>0</v>
       </c>
       <c r="K356" t="n">
-        <v>0</v>
+        <v>16.91</v>
       </c>
       <c r="L356" t="n">
-        <v>0</v>
+        <v>2.02</v>
       </c>
       <c r="M356" t="n">
-        <v>0</v>
+        <v>11.35</v>
       </c>
       <c r="N356" t="n">
-        <v>0</v>
+        <v>3.89</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>ARND3</t>
+          <t>VSPT4</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Empresa ARND</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D357" t="n">
-        <v>0.51</v>
+        <v>0</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -18976,16 +18976,16 @@
         <v>0</v>
       </c>
       <c r="G357" t="n">
-        <v>0.57</v>
+        <v>0</v>
       </c>
       <c r="H357" t="n">
         <v>0</v>
       </c>
       <c r="I357" t="n">
-        <v>125211000</v>
+        <v>5031600000</v>
       </c>
       <c r="J357" t="n">
-        <v>913.58</v>
+        <v>0</v>
       </c>
       <c r="K357" t="n">
         <v>0</v>
@@ -19003,21 +19003,21 @@
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>VVAX3</t>
+          <t>BAUH4</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa BAUH</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D358" t="n">
-        <v>0</v>
+        <v>93.39</v>
       </c>
       <c r="E358" t="inlineStr">
         <is>
@@ -19028,48 +19028,48 @@
         <v>0</v>
       </c>
       <c r="G358" t="n">
-        <v>0</v>
+        <v>3.18</v>
       </c>
       <c r="H358" t="n">
-        <v>0</v>
+        <v>1.16</v>
       </c>
       <c r="I358" t="n">
-        <v>144676000</v>
+        <v>153407000</v>
       </c>
       <c r="J358" t="n">
-        <v>0</v>
+        <v>207.53</v>
       </c>
       <c r="K358" t="n">
-        <v>-7.36</v>
+        <v>0</v>
       </c>
       <c r="L358" t="n">
-        <v>-37.76</v>
+        <v>0</v>
       </c>
       <c r="M358" t="n">
-        <v>-6.52</v>
+        <v>0</v>
       </c>
       <c r="N358" t="n">
-        <v>-92.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>MSAN4</t>
+          <t>ICPI3</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa ICPI</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>6.44</v>
+        <v>0</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -19086,33 +19086,33 @@
         <v>0</v>
       </c>
       <c r="I359" t="n">
-        <v>2533030000</v>
+        <v>0</v>
       </c>
       <c r="J359" t="n">
         <v>0</v>
       </c>
       <c r="K359" t="n">
-        <v>6.27</v>
+        <v>0</v>
       </c>
       <c r="L359" t="n">
-        <v>2.42</v>
+        <v>0</v>
       </c>
       <c r="M359" t="n">
-        <v>11.78</v>
+        <v>0</v>
       </c>
       <c r="N359" t="n">
-        <v>11.81</v>
+        <v>0</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>GALO4</t>
+          <t>ILLS4</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa ILLS</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
@@ -19121,7 +19121,7 @@
         </is>
       </c>
       <c r="D360" t="n">
-        <v>0.25</v>
+        <v>100.01</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -19138,33 +19138,33 @@
         <v>0</v>
       </c>
       <c r="I360" t="n">
-        <v>-60607000</v>
+        <v>-18567000</v>
       </c>
       <c r="J360" t="n">
         <v>0</v>
       </c>
       <c r="K360" t="n">
-        <v>13.98</v>
+        <v>8.43</v>
       </c>
       <c r="L360" t="n">
-        <v>-184.58</v>
+        <v>-10.22</v>
       </c>
       <c r="M360" t="n">
-        <v>39.37</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="N360" t="n">
-        <v>7.62</v>
+        <v>36.09</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>BBTG13</t>
+          <t>PTIP3</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -19173,7 +19173,7 @@
         </is>
       </c>
       <c r="D361" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -19190,42 +19190,42 @@
         <v>0</v>
       </c>
       <c r="I361" t="n">
-        <v>7000</v>
+        <v>-155957000</v>
       </c>
       <c r="J361" t="n">
         <v>0</v>
       </c>
       <c r="K361" t="n">
-        <v>0</v>
+        <v>13.73</v>
       </c>
       <c r="L361" t="n">
-        <v>0</v>
+        <v>7.55</v>
       </c>
       <c r="M361" t="n">
-        <v>0</v>
+        <v>23.13</v>
       </c>
       <c r="N361" t="n">
-        <v>-42.86</v>
+        <v>-121.74</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>INHA3</t>
+          <t>REPA4</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>Empresa INHA</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>0</v>
+        <v>1.08</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -19242,33 +19242,33 @@
         <v>0</v>
       </c>
       <c r="I362" t="n">
-        <v>1533210000</v>
+        <v>378378000</v>
       </c>
       <c r="J362" t="n">
         <v>0</v>
       </c>
       <c r="K362" t="n">
-        <v>-56.05</v>
+        <v>5.18</v>
       </c>
       <c r="L362" t="n">
-        <v>-124.06</v>
+        <v>1.22</v>
       </c>
       <c r="M362" t="n">
-        <v>-6.27</v>
+        <v>4.05</v>
       </c>
       <c r="N362" t="n">
-        <v>-39.87</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>PTIP4</t>
+          <t>EQMA6B</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -19277,7 +19277,7 @@
         </is>
       </c>
       <c r="D363" t="n">
-        <v>25.15</v>
+        <v>0</v>
       </c>
       <c r="E363" t="inlineStr">
         <is>
@@ -19294,42 +19294,42 @@
         <v>0</v>
       </c>
       <c r="I363" t="n">
-        <v>-155957000</v>
+        <v>4940330000</v>
       </c>
       <c r="J363" t="n">
         <v>0</v>
       </c>
       <c r="K363" t="n">
-        <v>13.73</v>
+        <v>0</v>
       </c>
       <c r="L363" t="n">
-        <v>7.55</v>
+        <v>0</v>
       </c>
       <c r="M363" t="n">
-        <v>23.13</v>
+        <v>0</v>
       </c>
       <c r="N363" t="n">
-        <v>-121.74</v>
+        <v>0</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>LATS3</t>
+          <t>SEBB4</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Empresa LATS</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D364" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -19346,42 +19346,42 @@
         <v>0</v>
       </c>
       <c r="I364" t="n">
-        <v>680646000</v>
+        <v>145783000</v>
       </c>
       <c r="J364" t="n">
         <v>0</v>
       </c>
       <c r="K364" t="n">
-        <v>11.74</v>
+        <v>9.24</v>
       </c>
       <c r="L364" t="n">
-        <v>1.3</v>
+        <v>7.4</v>
       </c>
       <c r="M364" t="n">
-        <v>11.63</v>
+        <v>24.15</v>
       </c>
       <c r="N364" t="n">
-        <v>1.84</v>
+        <v>23.01</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>SGEN4</t>
+          <t>MSAN3</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D365" t="n">
-        <v>0.6</v>
+        <v>6.44</v>
       </c>
       <c r="E365" t="inlineStr">
         <is>
@@ -19392,39 +19392,39 @@
         <v>0</v>
       </c>
       <c r="G365" t="n">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="H365" t="n">
         <v>0</v>
       </c>
       <c r="I365" t="n">
-        <v>156981000</v>
+        <v>2533030000</v>
       </c>
       <c r="J365" t="n">
         <v>0</v>
       </c>
       <c r="K365" t="n">
-        <v>-1871.17</v>
+        <v>6.27</v>
       </c>
       <c r="L365" t="n">
-        <v>0</v>
+        <v>2.42</v>
       </c>
       <c r="M365" t="n">
-        <v>-1.59</v>
+        <v>11.78</v>
       </c>
       <c r="N365" t="n">
-        <v>0</v>
+        <v>11.81</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>VSPT3</t>
+          <t>GALO3</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -19450,33 +19450,33 @@
         <v>0</v>
       </c>
       <c r="I366" t="n">
-        <v>5031600000</v>
+        <v>-60607000</v>
       </c>
       <c r="J366" t="n">
         <v>0</v>
       </c>
       <c r="K366" t="n">
-        <v>0</v>
+        <v>13.98</v>
       </c>
       <c r="L366" t="n">
-        <v>0</v>
+        <v>-184.58</v>
       </c>
       <c r="M366" t="n">
-        <v>0</v>
+        <v>39.37</v>
       </c>
       <c r="N366" t="n">
-        <v>0</v>
+        <v>7.62</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>SEBB3</t>
+          <t>SLCP3</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa SLCP</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -19485,7 +19485,7 @@
         </is>
       </c>
       <c r="D367" t="n">
-        <v>0</v>
+        <v>610.02</v>
       </c>
       <c r="E367" t="inlineStr">
         <is>
@@ -19502,42 +19502,42 @@
         <v>0</v>
       </c>
       <c r="I367" t="n">
-        <v>145783000</v>
+        <v>0</v>
       </c>
       <c r="J367" t="n">
         <v>0</v>
       </c>
       <c r="K367" t="n">
-        <v>9.24</v>
+        <v>0</v>
       </c>
       <c r="L367" t="n">
-        <v>7.4</v>
+        <v>0</v>
       </c>
       <c r="M367" t="n">
-        <v>24.15</v>
+        <v>0</v>
       </c>
       <c r="N367" t="n">
-        <v>23.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>BBTG11</t>
+          <t>DAYC3</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa DAYC</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D368" t="n">
-        <v>15.01</v>
+        <v>0</v>
       </c>
       <c r="E368" t="inlineStr">
         <is>
@@ -19554,7 +19554,7 @@
         <v>0</v>
       </c>
       <c r="I368" t="n">
-        <v>0</v>
+        <v>3009030000</v>
       </c>
       <c r="J368" t="n">
         <v>0</v>
@@ -19569,18 +19569,18 @@
         <v>0</v>
       </c>
       <c r="N368" t="n">
-        <v>0</v>
+        <v>17.33</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>JFAB4</t>
+          <t>DUFB11</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Empresa JFAB</t>
+          <t>Empresa DUFB</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -19589,7 +19589,7 @@
         </is>
       </c>
       <c r="D369" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="E369" t="inlineStr">
         <is>
@@ -19606,7 +19606,7 @@
         <v>0</v>
       </c>
       <c r="I369" t="n">
-        <v>-10183000</v>
+        <v>0</v>
       </c>
       <c r="J369" t="n">
         <v>0</v>
@@ -19621,18 +19621,18 @@
         <v>0</v>
       </c>
       <c r="N369" t="n">
-        <v>2.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>CCHI4</t>
+          <t>TNEP4</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -19641,7 +19641,7 @@
         </is>
       </c>
       <c r="D370" t="n">
-        <v>0.02</v>
+        <v>3.95</v>
       </c>
       <c r="E370" t="inlineStr">
         <is>
@@ -19652,39 +19652,39 @@
         <v>0</v>
       </c>
       <c r="G370" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="H370" t="n">
         <v>0</v>
       </c>
       <c r="I370" t="n">
-        <v>-160477000</v>
+        <v>955105000</v>
       </c>
       <c r="J370" t="n">
         <v>0</v>
       </c>
       <c r="K370" t="n">
-        <v>0</v>
+        <v>20.92</v>
       </c>
       <c r="L370" t="n">
-        <v>0</v>
+        <v>25.42</v>
       </c>
       <c r="M370" t="n">
-        <v>0</v>
+        <v>20.53</v>
       </c>
       <c r="N370" t="n">
-        <v>0</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>REPA3</t>
+          <t>MLPA3</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa MLPA</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
@@ -19693,7 +19693,7 @@
         </is>
       </c>
       <c r="D371" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E371" t="inlineStr">
         <is>
@@ -19710,33 +19710,33 @@
         <v>0</v>
       </c>
       <c r="I371" t="n">
-        <v>378378000</v>
+        <v>44578000</v>
       </c>
       <c r="J371" t="n">
         <v>0</v>
       </c>
       <c r="K371" t="n">
-        <v>5.18</v>
+        <v>6.66</v>
       </c>
       <c r="L371" t="n">
-        <v>1.22</v>
+        <v>8.92</v>
       </c>
       <c r="M371" t="n">
-        <v>4.05</v>
+        <v>0</v>
       </c>
       <c r="N371" t="n">
-        <v>1.91</v>
+        <v>45.13</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>EQMA5B</t>
+          <t>CLSC6</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa CLSC</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
@@ -19762,7 +19762,7 @@
         <v>0</v>
       </c>
       <c r="I372" t="n">
-        <v>4940330000</v>
+        <v>4228180000</v>
       </c>
       <c r="J372" t="n">
         <v>0</v>
@@ -19783,12 +19783,12 @@
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>GPIV33</t>
+          <t>SGEN3</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Empresa GPIV</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
@@ -19797,7 +19797,7 @@
         </is>
       </c>
       <c r="D373" t="n">
-        <v>4.42</v>
+        <v>5</v>
       </c>
       <c r="E373" t="inlineStr">
         <is>
@@ -19808,25 +19808,25 @@
         <v>0</v>
       </c>
       <c r="G373" t="n">
-        <v>0.23</v>
+        <v>0.77</v>
       </c>
       <c r="H373" t="n">
         <v>0</v>
       </c>
       <c r="I373" t="n">
-        <v>1318490000</v>
+        <v>156981000</v>
       </c>
       <c r="J373" t="n">
         <v>0</v>
       </c>
       <c r="K373" t="n">
-        <v>257.32</v>
+        <v>-1871.17</v>
       </c>
       <c r="L373" t="n">
         <v>0</v>
       </c>
       <c r="M373" t="n">
-        <v>-6.05</v>
+        <v>-1.59</v>
       </c>
       <c r="N373" t="n">
         <v>0</v>
@@ -19835,21 +19835,21 @@
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>ECIS4</t>
+          <t>CCHI3</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D374" t="n">
-        <v>145</v>
+        <v>0.02</v>
       </c>
       <c r="E374" t="inlineStr">
         <is>
@@ -19860,39 +19860,39 @@
         <v>0</v>
       </c>
       <c r="G374" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="H374" t="n">
         <v>0</v>
       </c>
       <c r="I374" t="n">
-        <v>129346000</v>
+        <v>-160477000</v>
       </c>
       <c r="J374" t="n">
         <v>0</v>
       </c>
       <c r="K374" t="n">
-        <v>34.9</v>
+        <v>0</v>
       </c>
       <c r="L374" t="n">
-        <v>14.18</v>
+        <v>0</v>
       </c>
       <c r="M374" t="n">
-        <v>12.48</v>
+        <v>0</v>
       </c>
       <c r="N374" t="n">
-        <v>7.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>TNEP3</t>
+          <t>PRBC3</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa PRBC</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
@@ -19901,7 +19901,7 @@
         </is>
       </c>
       <c r="D375" t="n">
-        <v>3.01</v>
+        <v>0</v>
       </c>
       <c r="E375" t="inlineStr">
         <is>
@@ -19918,33 +19918,33 @@
         <v>0</v>
       </c>
       <c r="I375" t="n">
-        <v>955105000</v>
+        <v>1319270000</v>
       </c>
       <c r="J375" t="n">
         <v>0</v>
       </c>
       <c r="K375" t="n">
-        <v>20.92</v>
+        <v>0</v>
       </c>
       <c r="L375" t="n">
-        <v>25.42</v>
+        <v>0</v>
       </c>
       <c r="M375" t="n">
-        <v>20.53</v>
+        <v>0</v>
       </c>
       <c r="N375" t="n">
-        <v>22.8</v>
+        <v>8.27</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>LECO3</t>
+          <t>ECIS3</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>Empresa LECO</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
@@ -19953,7 +19953,7 @@
         </is>
       </c>
       <c r="D376" t="n">
-        <v>0</v>
+        <v>211.65</v>
       </c>
       <c r="E376" t="inlineStr">
         <is>
@@ -19970,33 +19970,33 @@
         <v>0</v>
       </c>
       <c r="I376" t="n">
-        <v>105928000</v>
+        <v>129346000</v>
       </c>
       <c r="J376" t="n">
         <v>0</v>
       </c>
       <c r="K376" t="n">
-        <v>-2.14</v>
+        <v>34.9</v>
       </c>
       <c r="L376" t="n">
-        <v>-4.72</v>
+        <v>14.18</v>
       </c>
       <c r="M376" t="n">
-        <v>-3.48</v>
+        <v>12.48</v>
       </c>
       <c r="N376" t="n">
-        <v>-14.82</v>
+        <v>7.33</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>VGOR3</t>
+          <t>SFSA3</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>Empresa VGOR</t>
+          <t>Empresa SFSA</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
@@ -20022,22 +20022,22 @@
         <v>0</v>
       </c>
       <c r="I377" t="n">
-        <v>135178000</v>
+        <v>739524000</v>
       </c>
       <c r="J377" t="n">
         <v>0</v>
       </c>
       <c r="K377" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="L377" t="n">
-        <v>-4.59</v>
+        <v>0</v>
       </c>
       <c r="M377" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N377" t="n">
-        <v>-24.29</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="378">
@@ -20828,7 +20828,7 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>Empresa BRSR</t>
+          <t>Banrisul</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
@@ -22856,7 +22856,7 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>Empresa ALLD</t>
+          <t>Allos</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
@@ -22869,7 +22869,7 @@
       </c>
       <c r="E432" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Shoppings e Imóveis</t>
         </is>
       </c>
       <c r="F432" t="n">
@@ -23371,7 +23371,7 @@
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>MMAQ3</t>
+          <t>MMAQ4</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
@@ -23381,7 +23381,7 @@
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D442" t="n">
@@ -23399,7 +23399,7 @@
         <v>0.36</v>
       </c>
       <c r="H442" t="n">
-        <v>0</v>
+        <v>41.68</v>
       </c>
       <c r="I442" t="n">
         <v>259016000</v>
@@ -23423,7 +23423,7 @@
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>MMAQ4</t>
+          <t>MMAQ3</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
@@ -23433,7 +23433,7 @@
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D443" t="n">
@@ -23451,7 +23451,7 @@
         <v>0.36</v>
       </c>
       <c r="H443" t="n">
-        <v>41.68</v>
+        <v>0</v>
       </c>
       <c r="I443" t="n">
         <v>259016000</v>
@@ -23532,7 +23532,7 @@
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>Empresa RIAA</t>
+          <t>Riauto</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
@@ -24260,7 +24260,7 @@
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>Empresa JHSF</t>
+          <t>JHSF Participações</t>
         </is>
       </c>
       <c r="C459" t="inlineStr">
@@ -24416,7 +24416,7 @@
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>Empresa RSUL</t>
+          <t>Riosulense</t>
         </is>
       </c>
       <c r="C462" t="inlineStr">
@@ -24832,7 +24832,7 @@
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>Empresa BRSR</t>
+          <t>Banrisul</t>
         </is>
       </c>
       <c r="C470" t="inlineStr">
@@ -25144,7 +25144,7 @@
       </c>
       <c r="B476" t="inlineStr">
         <is>
-          <t>Empresa EVEN</t>
+          <t>Even Construtora</t>
         </is>
       </c>
       <c r="C476" t="inlineStr">
@@ -25157,7 +25157,7 @@
       </c>
       <c r="E476" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Construção Civil</t>
         </is>
       </c>
       <c r="F476" t="n">
@@ -25404,7 +25404,7 @@
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>Empresa BAZA</t>
+          <t>Banco da Amazônia</t>
         </is>
       </c>
       <c r="C481" t="inlineStr">
@@ -25417,7 +25417,7 @@
       </c>
       <c r="E481" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="F481" t="n">
@@ -25612,7 +25612,7 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>Empresa POMO</t>
+          <t>Marcopolo</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
@@ -25625,7 +25625,7 @@
       </c>
       <c r="E485" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Transporte e Logística</t>
         </is>
       </c>
       <c r="F485" t="n">
@@ -25664,7 +25664,7 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>Empresa VULC</t>
+          <t>Vulcabras</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
@@ -25677,7 +25677,7 @@
       </c>
       <c r="E486" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Varejo e Comércio</t>
         </is>
       </c>
       <c r="F486" t="n">
@@ -26132,7 +26132,7 @@
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>Empresa BRSR</t>
+          <t>Banrisul</t>
         </is>
       </c>
       <c r="C495" t="inlineStr">
@@ -26236,7 +26236,7 @@
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>Empresa POMO</t>
+          <t>Marcopolo</t>
         </is>
       </c>
       <c r="C497" t="inlineStr">
@@ -26249,7 +26249,7 @@
       </c>
       <c r="E497" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Transporte e Logística</t>
         </is>
       </c>
       <c r="F497" t="n">
@@ -26392,7 +26392,7 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>Empresa BRSR</t>
+          <t>Banrisul</t>
         </is>
       </c>
       <c r="C500" t="inlineStr">
@@ -28680,7 +28680,7 @@
       </c>
       <c r="B544" t="inlineStr">
         <is>
-          <t>Empresa VULC</t>
+          <t>Vulcabras</t>
         </is>
       </c>
       <c r="C544" t="inlineStr">
@@ -28693,7 +28693,7 @@
       </c>
       <c r="E544" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Varejo e Comércio</t>
         </is>
       </c>
       <c r="F544" t="n">
@@ -29663,7 +29663,7 @@
     <row r="563">
       <c r="A563" t="inlineStr">
         <is>
-          <t>CIQU4</t>
+          <t>CIQU3</t>
         </is>
       </c>
       <c r="B563" t="inlineStr">
@@ -29673,7 +29673,7 @@
       </c>
       <c r="C563" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D563" t="n">
@@ -29715,7 +29715,7 @@
     <row r="564">
       <c r="A564" t="inlineStr">
         <is>
-          <t>CIQU3</t>
+          <t>CIQU4</t>
         </is>
       </c>
       <c r="B564" t="inlineStr">
@@ -29725,7 +29725,7 @@
       </c>
       <c r="C564" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D564" t="n">
@@ -31171,7 +31171,7 @@
     <row r="592">
       <c r="A592" t="inlineStr">
         <is>
-          <t>GETT3</t>
+          <t>GETT4</t>
         </is>
       </c>
       <c r="B592" t="inlineStr">
@@ -31181,7 +31181,7 @@
       </c>
       <c r="C592" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D592" t="n">
@@ -31223,7 +31223,7 @@
     <row r="593">
       <c r="A593" t="inlineStr">
         <is>
-          <t>GETT4</t>
+          <t>GETT3</t>
         </is>
       </c>
       <c r="B593" t="inlineStr">
@@ -31233,7 +31233,7 @@
       </c>
       <c r="C593" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D593" t="n">
@@ -32575,7 +32575,7 @@
     <row r="619">
       <c r="A619" t="inlineStr">
         <is>
-          <t>AESL4</t>
+          <t>AESL3</t>
         </is>
       </c>
       <c r="B619" t="inlineStr">
@@ -32585,7 +32585,7 @@
       </c>
       <c r="C619" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D619" t="n">
@@ -32627,7 +32627,7 @@
     <row r="620">
       <c r="A620" t="inlineStr">
         <is>
-          <t>AESL3</t>
+          <t>AESL4</t>
         </is>
       </c>
       <c r="B620" t="inlineStr">
@@ -32637,7 +32637,7 @@
       </c>
       <c r="C620" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D620" t="n">
@@ -33529,7 +33529,7 @@
       </c>
       <c r="E637" t="inlineStr">
         <is>
-          <t>Ultrapar</t>
+          <t>Petróleo e Gás</t>
         </is>
       </c>
       <c r="F637" t="n">
@@ -34361,7 +34361,7 @@
       </c>
       <c r="E653" t="inlineStr">
         <is>
-          <t>Porto Seguro</t>
+          <t>Seguradoras</t>
         </is>
       </c>
       <c r="F653" t="n">
@@ -34673,7 +34673,7 @@
       </c>
       <c r="E659" t="inlineStr">
         <is>
-          <t>M. Dias Branco</t>
+          <t>Agro e Alimentos</t>
         </is>
       </c>
       <c r="F659" t="n">
@@ -38261,7 +38261,7 @@
       </c>
       <c r="E728" t="inlineStr">
         <is>
-          <t>Ultrapar</t>
+          <t>Petróleo e Gás</t>
         </is>
       </c>
       <c r="F728" t="n">
@@ -41901,7 +41901,7 @@
       </c>
       <c r="E798" t="inlineStr">
         <is>
-          <t>CSN Mineração</t>
+          <t>Mineração e Siderurgia</t>
         </is>
       </c>
       <c r="F798" t="n">
@@ -44657,7 +44657,7 @@
       </c>
       <c r="E851" t="inlineStr">
         <is>
-          <t>SLC Agrícola</t>
+          <t>Agro e Alimentos</t>
         </is>
       </c>
       <c r="F851" t="n">
@@ -45315,7 +45315,7 @@
     <row r="864">
       <c r="A864" t="inlineStr">
         <is>
-          <t>RSIP4</t>
+          <t>RSIP3</t>
         </is>
       </c>
       <c r="B864" t="inlineStr">
@@ -45325,7 +45325,7 @@
       </c>
       <c r="C864" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D864" t="n">
@@ -45367,7 +45367,7 @@
     <row r="865">
       <c r="A865" t="inlineStr">
         <is>
-          <t>RSIP3</t>
+          <t>RSIP4</t>
         </is>
       </c>
       <c r="B865" t="inlineStr">
@@ -45377,7 +45377,7 @@
       </c>
       <c r="C865" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D865" t="n">
@@ -45437,7 +45437,7 @@
       </c>
       <c r="E866" t="inlineStr">
         <is>
-          <t>Sanepar</t>
+          <t>Saneamento</t>
         </is>
       </c>
       <c r="F866" t="n">
@@ -45541,7 +45541,7 @@
       </c>
       <c r="E868" t="inlineStr">
         <is>
-          <t>Sanepar</t>
+          <t>Saneamento</t>
         </is>
       </c>
       <c r="F868" t="n">
@@ -46321,7 +46321,7 @@
       </c>
       <c r="E883" t="inlineStr">
         <is>
-          <t>Sanepar</t>
+          <t>Saneamento</t>
         </is>
       </c>
       <c r="F883" t="n">
@@ -50983,7 +50983,7 @@
     <row r="973">
       <c r="A973" t="inlineStr">
         <is>
-          <t>PQUN4</t>
+          <t>PQUN3</t>
         </is>
       </c>
       <c r="B973" t="inlineStr">
@@ -50993,7 +50993,7 @@
       </c>
       <c r="C973" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D973" t="n">
@@ -51035,7 +51035,7 @@
     <row r="974">
       <c r="A974" t="inlineStr">
         <is>
-          <t>PQUN3</t>
+          <t>PQUN4</t>
         </is>
       </c>
       <c r="B974" t="inlineStr">
@@ -51045,7 +51045,7 @@
       </c>
       <c r="C974" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D974" t="n">

</xml_diff>

<commit_message>
Corrige categorizacao de setores associando por prefixo de ticker
</commit_message>
<xml_diff>
--- a/acoes_b3.xlsx
+++ b/acoes_b3.xlsx
@@ -496,12 +496,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MNSA4</t>
+          <t>CSTB4</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Empresa MNSA</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -510,7 +510,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.47</v>
+        <v>147.69</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -527,45 +527,45 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>-9105000</v>
+        <v>8420670000</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>-208.15</v>
+        <v>40.85</v>
       </c>
       <c r="L2" t="n">
-        <v>-362.66</v>
+        <v>28.98</v>
       </c>
       <c r="M2" t="n">
-        <v>-13.5</v>
+        <v>22.4</v>
       </c>
       <c r="N2" t="n">
-        <v>145.7</v>
+        <v>20.11</v>
       </c>
       <c r="O2" t="n">
-        <v>-41.11</v>
+        <v>31.91</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CLAN3</t>
+          <t>PORP4</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Empresa CLAN</t>
+          <t>Empresa PORP</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -582,7 +582,7 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>1012240000</v>
+        <v>22399000</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -597,30 +597,30 @@
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>-1.05</v>
+        <v>-2.08</v>
       </c>
       <c r="O3" t="n">
-        <v>-63.96</v>
+        <v>13.66</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CSTB4</t>
+          <t>IVTT3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa IVTT</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>147.69</v>
+        <v>0</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -637,45 +637,45 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>8420670000</v>
+        <v>1083050000</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>40.85</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>28.98</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>22.4</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>20.11</v>
+        <v>-0.4</v>
       </c>
       <c r="O4" t="n">
-        <v>31.91</v>
+        <v>20.67</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PORP4</t>
+          <t>MNSA3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Empresa PORP</t>
+          <t>Empresa MNSA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2.4</v>
+        <v>0.42</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -692,45 +692,45 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>22399000</v>
+        <v>-9105000</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>-208.15</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>-362.66</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>-13.5</v>
       </c>
       <c r="N5" t="n">
-        <v>-2.08</v>
+        <v>145.7</v>
       </c>
       <c r="O5" t="n">
-        <v>13.66</v>
+        <v>-41.11</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>IVTT3</t>
+          <t>CFLU4</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Empresa IVTT</t>
+          <t>Empresa CFLU</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -747,36 +747,36 @@
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>1083050000</v>
+        <v>60351000</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="L6" t="n">
-        <v>0</v>
+        <v>10.72</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>17.68</v>
       </c>
       <c r="N6" t="n">
-        <v>-0.4</v>
+        <v>32.15</v>
       </c>
       <c r="O6" t="n">
-        <v>20.67</v>
+        <v>8.140000000000001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MNSA3</t>
+          <t>CSTB3</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Empresa MNSA</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -785,7 +785,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.42</v>
+        <v>150</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -802,45 +802,45 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>-9105000</v>
+        <v>8420670000</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>-208.15</v>
+        <v>40.85</v>
       </c>
       <c r="L7" t="n">
-        <v>-362.66</v>
+        <v>28.98</v>
       </c>
       <c r="M7" t="n">
-        <v>-13.5</v>
+        <v>22.4</v>
       </c>
       <c r="N7" t="n">
-        <v>145.7</v>
+        <v>20.11</v>
       </c>
       <c r="O7" t="n">
-        <v>-41.11</v>
+        <v>31.91</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CSTB3</t>
+          <t>POPR4</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa POPR</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>150</v>
+        <v>10.17</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -857,45 +857,45 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>8420670000</v>
+        <v>545803000</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>40.85</v>
+        <v>8.66</v>
       </c>
       <c r="L8" t="n">
-        <v>28.98</v>
+        <v>5.65</v>
       </c>
       <c r="M8" t="n">
-        <v>22.4</v>
+        <v>15.25</v>
       </c>
       <c r="N8" t="n">
-        <v>20.11</v>
+        <v>19.93</v>
       </c>
       <c r="O8" t="n">
-        <v>31.91</v>
+        <v>30.93</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CFLU4</t>
+          <t>PMET3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Empresa CFLU</t>
+          <t>Empresa PMET</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -912,45 +912,45 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>60351000</v>
+        <v>-290863000</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>8.880000000000001</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>10.72</v>
+        <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>17.68</v>
+        <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>32.15</v>
+        <v>4.1</v>
       </c>
       <c r="O9" t="n">
-        <v>8.140000000000001</v>
+        <v>37.74</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>POPR4</t>
+          <t>CLAN3</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Empresa POPR</t>
+          <t>Empresa CLAN</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>10.17</v>
+        <v>0</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -967,45 +967,45 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>545803000</v>
+        <v>1012240000</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>8.66</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>5.65</v>
+        <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>15.25</v>
+        <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>19.93</v>
+        <v>-1.05</v>
       </c>
       <c r="O10" t="n">
-        <v>30.93</v>
+        <v>-63.96</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PMET3</t>
+          <t>MNSA4</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Empresa PMET</t>
+          <t>Empresa MNSA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>0.47</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1022,25 +1022,25 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>-290863000</v>
+        <v>-9105000</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>-208.15</v>
       </c>
       <c r="L11" t="n">
-        <v>0</v>
+        <v>-362.66</v>
       </c>
       <c r="M11" t="n">
-        <v>0</v>
+        <v>-13.5</v>
       </c>
       <c r="N11" t="n">
-        <v>4.1</v>
+        <v>145.7</v>
       </c>
       <c r="O11" t="n">
-        <v>37.74</v>
+        <v>-41.11</v>
       </c>
     </row>
     <row r="12">
@@ -17381,12 +17381,12 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>ARND3</t>
+          <t>VSPT3</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Empresa ARND</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -17395,7 +17395,7 @@
         </is>
       </c>
       <c r="D309" t="n">
-        <v>0.51</v>
+        <v>0</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -17406,16 +17406,16 @@
         <v>0</v>
       </c>
       <c r="G309" t="n">
-        <v>0.57</v>
+        <v>0</v>
       </c>
       <c r="H309" t="n">
         <v>0</v>
       </c>
       <c r="I309" t="n">
-        <v>125211000</v>
+        <v>5031600000</v>
       </c>
       <c r="J309" t="n">
-        <v>913.58</v>
+        <v>0</v>
       </c>
       <c r="K309" t="n">
         <v>0</v>
@@ -17430,27 +17430,27 @@
         <v>0</v>
       </c>
       <c r="O309" t="n">
-        <v>-0.88</v>
+        <v>4.92</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>VVAX3</t>
+          <t>SGEN4</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -17461,42 +17461,42 @@
         <v>0</v>
       </c>
       <c r="G310" t="n">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="H310" t="n">
         <v>0</v>
       </c>
       <c r="I310" t="n">
-        <v>144676000</v>
+        <v>156981000</v>
       </c>
       <c r="J310" t="n">
         <v>0</v>
       </c>
       <c r="K310" t="n">
-        <v>-7.36</v>
+        <v>-1871.17</v>
       </c>
       <c r="L310" t="n">
-        <v>-37.76</v>
+        <v>0</v>
       </c>
       <c r="M310" t="n">
-        <v>-6.52</v>
+        <v>-1.59</v>
       </c>
       <c r="N310" t="n">
-        <v>-92.03</v>
+        <v>0</v>
       </c>
       <c r="O310" t="n">
-        <v>0</v>
+        <v>-59.85</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>MSAN4</t>
+          <t>CCHI4</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -17505,7 +17505,7 @@
         </is>
       </c>
       <c r="D311" t="n">
-        <v>6.44</v>
+        <v>0.02</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -17516,51 +17516,51 @@
         <v>0</v>
       </c>
       <c r="G311" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="H311" t="n">
         <v>0</v>
       </c>
       <c r="I311" t="n">
-        <v>2533030000</v>
+        <v>-160477000</v>
       </c>
       <c r="J311" t="n">
         <v>0</v>
       </c>
       <c r="K311" t="n">
-        <v>6.27</v>
+        <v>0</v>
       </c>
       <c r="L311" t="n">
-        <v>2.42</v>
+        <v>0</v>
       </c>
       <c r="M311" t="n">
-        <v>11.78</v>
+        <v>0</v>
       </c>
       <c r="N311" t="n">
-        <v>11.81</v>
+        <v>0</v>
       </c>
       <c r="O311" t="n">
-        <v>101.35</v>
+        <v>20.36</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>GALO4</t>
+          <t>REPA3</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -17577,41 +17577,41 @@
         <v>0</v>
       </c>
       <c r="I312" t="n">
-        <v>-60607000</v>
+        <v>378378000</v>
       </c>
       <c r="J312" t="n">
         <v>0</v>
       </c>
       <c r="K312" t="n">
-        <v>13.98</v>
+        <v>5.18</v>
       </c>
       <c r="L312" t="n">
-        <v>-184.58</v>
+        <v>1.22</v>
       </c>
       <c r="M312" t="n">
-        <v>39.37</v>
+        <v>4.05</v>
       </c>
       <c r="N312" t="n">
-        <v>7.62</v>
+        <v>1.91</v>
       </c>
       <c r="O312" t="n">
-        <v>-28.97</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>BBTG13</t>
+          <t>EQMA5B</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D313" t="n">
@@ -17632,7 +17632,7 @@
         <v>0</v>
       </c>
       <c r="I313" t="n">
-        <v>7000</v>
+        <v>4940330000</v>
       </c>
       <c r="J313" t="n">
         <v>0</v>
@@ -17647,21 +17647,21 @@
         <v>0</v>
       </c>
       <c r="N313" t="n">
-        <v>-42.86</v>
+        <v>0</v>
       </c>
       <c r="O313" t="n">
-        <v>0</v>
+        <v>9.050000000000001</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>INHA3</t>
+          <t>SEBB3</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Empresa INHA</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -17687,36 +17687,36 @@
         <v>0</v>
       </c>
       <c r="I314" t="n">
-        <v>1533210000</v>
+        <v>145783000</v>
       </c>
       <c r="J314" t="n">
         <v>0</v>
       </c>
       <c r="K314" t="n">
-        <v>-56.05</v>
+        <v>9.24</v>
       </c>
       <c r="L314" t="n">
-        <v>-124.06</v>
+        <v>7.4</v>
       </c>
       <c r="M314" t="n">
-        <v>-6.27</v>
+        <v>24.15</v>
       </c>
       <c r="N314" t="n">
-        <v>-39.87</v>
+        <v>23.01</v>
       </c>
       <c r="O314" t="n">
-        <v>-12.18</v>
+        <v>50.04</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>PTIP4</t>
+          <t>BBTG11</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -17725,7 +17725,7 @@
         </is>
       </c>
       <c r="D315" t="n">
-        <v>25.15</v>
+        <v>15.01</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -17742,45 +17742,45 @@
         <v>0</v>
       </c>
       <c r="I315" t="n">
-        <v>-155957000</v>
+        <v>0</v>
       </c>
       <c r="J315" t="n">
         <v>0</v>
       </c>
       <c r="K315" t="n">
-        <v>13.73</v>
+        <v>0</v>
       </c>
       <c r="L315" t="n">
-        <v>7.55</v>
+        <v>0</v>
       </c>
       <c r="M315" t="n">
-        <v>23.13</v>
+        <v>0</v>
       </c>
       <c r="N315" t="n">
-        <v>-121.74</v>
+        <v>0</v>
       </c>
       <c r="O315" t="n">
-        <v>62.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>LATS3</t>
+          <t>JFAB4</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Empresa LATS</t>
+          <t>Empresa JFAB</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D316" t="n">
-        <v>22</v>
+        <v>0.06</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -17797,36 +17797,36 @@
         <v>0</v>
       </c>
       <c r="I316" t="n">
-        <v>680646000</v>
+        <v>-10183000</v>
       </c>
       <c r="J316" t="n">
         <v>0</v>
       </c>
       <c r="K316" t="n">
-        <v>11.74</v>
+        <v>0</v>
       </c>
       <c r="L316" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="M316" t="n">
-        <v>11.63</v>
+        <v>0</v>
       </c>
       <c r="N316" t="n">
-        <v>1.84</v>
+        <v>2.34</v>
       </c>
       <c r="O316" t="n">
-        <v>15.37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>VSPT3</t>
+          <t>TNEP3</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -17835,7 +17835,7 @@
         </is>
       </c>
       <c r="D317" t="n">
-        <v>0</v>
+        <v>3.01</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -17852,45 +17852,45 @@
         <v>0</v>
       </c>
       <c r="I317" t="n">
-        <v>5031600000</v>
+        <v>955105000</v>
       </c>
       <c r="J317" t="n">
         <v>0</v>
       </c>
       <c r="K317" t="n">
-        <v>0</v>
+        <v>20.92</v>
       </c>
       <c r="L317" t="n">
-        <v>0</v>
+        <v>25.42</v>
       </c>
       <c r="M317" t="n">
-        <v>0</v>
+        <v>20.53</v>
       </c>
       <c r="N317" t="n">
-        <v>0</v>
+        <v>22.8</v>
       </c>
       <c r="O317" t="n">
-        <v>4.92</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>SGEN4</t>
+          <t>LECO3</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa LECO</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -17901,42 +17901,42 @@
         <v>0</v>
       </c>
       <c r="G318" t="n">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="H318" t="n">
         <v>0</v>
       </c>
       <c r="I318" t="n">
-        <v>156981000</v>
+        <v>105928000</v>
       </c>
       <c r="J318" t="n">
         <v>0</v>
       </c>
       <c r="K318" t="n">
-        <v>-1871.17</v>
+        <v>-2.14</v>
       </c>
       <c r="L318" t="n">
-        <v>0</v>
+        <v>-4.72</v>
       </c>
       <c r="M318" t="n">
-        <v>-1.59</v>
+        <v>-3.48</v>
       </c>
       <c r="N318" t="n">
-        <v>0</v>
+        <v>-14.82</v>
       </c>
       <c r="O318" t="n">
-        <v>-59.85</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>SEBB3</t>
+          <t>VGOR3</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa VGOR</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -17962,45 +17962,45 @@
         <v>0</v>
       </c>
       <c r="I319" t="n">
-        <v>145783000</v>
+        <v>135178000</v>
       </c>
       <c r="J319" t="n">
         <v>0</v>
       </c>
       <c r="K319" t="n">
-        <v>9.24</v>
+        <v>4.5</v>
       </c>
       <c r="L319" t="n">
-        <v>7.4</v>
+        <v>-4.59</v>
       </c>
       <c r="M319" t="n">
-        <v>24.15</v>
+        <v>6</v>
       </c>
       <c r="N319" t="n">
-        <v>23.01</v>
+        <v>-24.29</v>
       </c>
       <c r="O319" t="n">
-        <v>50.04</v>
+        <v>4.77</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>BBTG11</t>
+          <t>GPIV33</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa GPIV</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>15.01</v>
+        <v>4.42</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -18011,42 +18011,42 @@
         <v>0</v>
       </c>
       <c r="G320" t="n">
-        <v>0</v>
+        <v>0.23</v>
       </c>
       <c r="H320" t="n">
         <v>0</v>
       </c>
       <c r="I320" t="n">
-        <v>0</v>
+        <v>1318490000</v>
       </c>
       <c r="J320" t="n">
         <v>0</v>
       </c>
       <c r="K320" t="n">
-        <v>0</v>
+        <v>257.32</v>
       </c>
       <c r="L320" t="n">
         <v>0</v>
       </c>
       <c r="M320" t="n">
-        <v>0</v>
+        <v>-6.05</v>
       </c>
       <c r="N320" t="n">
         <v>0</v>
       </c>
       <c r="O320" t="n">
-        <v>0</v>
+        <v>-40.99</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>JFAB4</t>
+          <t>ECIS4</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Empresa JFAB</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -18055,7 +18055,7 @@
         </is>
       </c>
       <c r="D321" t="n">
-        <v>0.06</v>
+        <v>145</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -18072,45 +18072,45 @@
         <v>0</v>
       </c>
       <c r="I321" t="n">
-        <v>-10183000</v>
+        <v>129346000</v>
       </c>
       <c r="J321" t="n">
         <v>0</v>
       </c>
       <c r="K321" t="n">
-        <v>0</v>
+        <v>34.9</v>
       </c>
       <c r="L321" t="n">
-        <v>0</v>
+        <v>14.18</v>
       </c>
       <c r="M321" t="n">
-        <v>0</v>
+        <v>12.48</v>
       </c>
       <c r="N321" t="n">
-        <v>2.34</v>
+        <v>7.33</v>
       </c>
       <c r="O321" t="n">
-        <v>0</v>
+        <v>4.66</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>CCHI4</t>
+          <t>EGGY3</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa EGGY</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -18121,13 +18121,13 @@
         <v>0</v>
       </c>
       <c r="G322" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="H322" t="n">
         <v>0</v>
       </c>
       <c r="I322" t="n">
-        <v>-160477000</v>
+        <v>954480000</v>
       </c>
       <c r="J322" t="n">
         <v>0</v>
@@ -18145,27 +18145,27 @@
         <v>0</v>
       </c>
       <c r="O322" t="n">
-        <v>20.36</v>
+        <v>-0.82</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>REPA3</t>
+          <t>CBMA4</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D323" t="n">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -18182,36 +18182,36 @@
         <v>0</v>
       </c>
       <c r="I323" t="n">
-        <v>378378000</v>
+        <v>-34022300000</v>
       </c>
       <c r="J323" t="n">
         <v>0</v>
       </c>
       <c r="K323" t="n">
-        <v>5.18</v>
+        <v>0</v>
       </c>
       <c r="L323" t="n">
-        <v>1.22</v>
+        <v>0</v>
       </c>
       <c r="M323" t="n">
-        <v>4.05</v>
+        <v>0</v>
       </c>
       <c r="N323" t="n">
-        <v>1.91</v>
+        <v>0</v>
       </c>
       <c r="O323" t="n">
-        <v>1.09</v>
+        <v>252.65</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>EQMA5B</t>
+          <t>SALM4</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -18220,7 +18220,7 @@
         </is>
       </c>
       <c r="D324" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -18237,36 +18237,36 @@
         <v>0</v>
       </c>
       <c r="I324" t="n">
-        <v>4940330000</v>
+        <v>475600000</v>
       </c>
       <c r="J324" t="n">
         <v>0</v>
       </c>
       <c r="K324" t="n">
-        <v>0</v>
+        <v>10.22</v>
       </c>
       <c r="L324" t="n">
-        <v>0</v>
+        <v>4.13</v>
       </c>
       <c r="M324" t="n">
-        <v>0</v>
+        <v>25.78</v>
       </c>
       <c r="N324" t="n">
-        <v>0</v>
+        <v>19.53</v>
       </c>
       <c r="O324" t="n">
-        <v>9.050000000000001</v>
+        <v>24.53</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>GPIV33</t>
+          <t>BERG3</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Empresa GPIV</t>
+          <t>Empresa BERG</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -18275,7 +18275,7 @@
         </is>
       </c>
       <c r="D325" t="n">
-        <v>4.42</v>
+        <v>33</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -18286,51 +18286,51 @@
         <v>0</v>
       </c>
       <c r="G325" t="n">
-        <v>0.23</v>
+        <v>0</v>
       </c>
       <c r="H325" t="n">
         <v>0</v>
       </c>
       <c r="I325" t="n">
-        <v>1318490000</v>
+        <v>9538000</v>
       </c>
       <c r="J325" t="n">
         <v>0</v>
       </c>
       <c r="K325" t="n">
-        <v>257.32</v>
+        <v>-8.6</v>
       </c>
       <c r="L325" t="n">
-        <v>0</v>
+        <v>-32.6</v>
       </c>
       <c r="M325" t="n">
-        <v>-6.05</v>
+        <v>-5.58</v>
       </c>
       <c r="N325" t="n">
-        <v>0</v>
+        <v>-102.71</v>
       </c>
       <c r="O325" t="n">
-        <v>-40.99</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>ECIS4</t>
+          <t>JBDU3</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa JBDU</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>145</v>
+        <v>0</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -18347,36 +18347,36 @@
         <v>0</v>
       </c>
       <c r="I326" t="n">
-        <v>129346000</v>
+        <v>56569000</v>
       </c>
       <c r="J326" t="n">
         <v>0</v>
       </c>
       <c r="K326" t="n">
-        <v>34.9</v>
+        <v>0</v>
       </c>
       <c r="L326" t="n">
-        <v>14.18</v>
+        <v>0</v>
       </c>
       <c r="M326" t="n">
-        <v>12.48</v>
+        <v>0</v>
       </c>
       <c r="N326" t="n">
-        <v>7.33</v>
+        <v>0</v>
       </c>
       <c r="O326" t="n">
-        <v>4.66</v>
+        <v>0</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>TNEP3</t>
+          <t>AGEI3</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa AGEI</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -18385,7 +18385,7 @@
         </is>
       </c>
       <c r="D327" t="n">
-        <v>3.01</v>
+        <v>7.8</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -18396,42 +18396,42 @@
         <v>0</v>
       </c>
       <c r="G327" t="n">
-        <v>0</v>
+        <v>1.25</v>
       </c>
       <c r="H327" t="n">
         <v>0</v>
       </c>
       <c r="I327" t="n">
-        <v>955105000</v>
+        <v>1878210000</v>
       </c>
       <c r="J327" t="n">
         <v>0</v>
       </c>
       <c r="K327" t="n">
-        <v>20.92</v>
+        <v>0</v>
       </c>
       <c r="L327" t="n">
-        <v>25.42</v>
+        <v>0</v>
       </c>
       <c r="M327" t="n">
-        <v>20.53</v>
+        <v>0</v>
       </c>
       <c r="N327" t="n">
-        <v>22.8</v>
+        <v>0</v>
       </c>
       <c r="O327" t="n">
-        <v>8.15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>LECO3</t>
+          <t>SASG3</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Empresa LECO</t>
+          <t>Empresa SASG</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -18440,7 +18440,7 @@
         </is>
       </c>
       <c r="D328" t="n">
-        <v>0</v>
+        <v>0.98</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -18457,36 +18457,36 @@
         <v>0</v>
       </c>
       <c r="I328" t="n">
-        <v>105928000</v>
+        <v>0</v>
       </c>
       <c r="J328" t="n">
         <v>0</v>
       </c>
       <c r="K328" t="n">
-        <v>-2.14</v>
+        <v>0</v>
       </c>
       <c r="L328" t="n">
-        <v>-4.72</v>
+        <v>0</v>
       </c>
       <c r="M328" t="n">
-        <v>-3.48</v>
+        <v>0</v>
       </c>
       <c r="N328" t="n">
-        <v>-14.82</v>
+        <v>0</v>
       </c>
       <c r="O328" t="n">
-        <v>3.58</v>
+        <v>0</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>VGOR3</t>
+          <t>BMEF3</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Empresa VGOR</t>
+          <t>Empresa BMEF</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -18495,7 +18495,7 @@
         </is>
       </c>
       <c r="D329" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -18506,42 +18506,42 @@
         <v>0</v>
       </c>
       <c r="G329" t="n">
-        <v>0</v>
+        <v>4.16</v>
       </c>
       <c r="H329" t="n">
         <v>0</v>
       </c>
       <c r="I329" t="n">
-        <v>135178000</v>
+        <v>2674780000</v>
       </c>
       <c r="J329" t="n">
         <v>0</v>
       </c>
       <c r="K329" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="L329" t="n">
-        <v>-4.59</v>
+        <v>0</v>
       </c>
       <c r="M329" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N329" t="n">
-        <v>-24.29</v>
+        <v>0</v>
       </c>
       <c r="O329" t="n">
-        <v>4.77</v>
+        <v>0</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>BERG3</t>
+          <t>ARPS3</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Empresa BERG</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -18550,7 +18550,7 @@
         </is>
       </c>
       <c r="D330" t="n">
-        <v>33</v>
+        <v>0.3</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -18567,36 +18567,36 @@
         <v>0</v>
       </c>
       <c r="I330" t="n">
-        <v>9538000</v>
+        <v>-12690000</v>
       </c>
       <c r="J330" t="n">
         <v>0</v>
       </c>
       <c r="K330" t="n">
-        <v>-8.6</v>
+        <v>-4.92</v>
       </c>
       <c r="L330" t="n">
-        <v>-32.6</v>
+        <v>-11.59</v>
       </c>
       <c r="M330" t="n">
-        <v>-5.58</v>
+        <v>-6.64</v>
       </c>
       <c r="N330" t="n">
-        <v>-102.71</v>
+        <v>20.34</v>
       </c>
       <c r="O330" t="n">
-        <v>-8</v>
+        <v>-17.53</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>JBDU3</t>
+          <t>ODER3</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Empresa JBDU</t>
+          <t>Empresa ODER</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -18622,7 +18622,7 @@
         <v>0</v>
       </c>
       <c r="I331" t="n">
-        <v>56569000</v>
+        <v>609518000</v>
       </c>
       <c r="J331" t="n">
         <v>0</v>
@@ -18640,18 +18640,18 @@
         <v>0</v>
       </c>
       <c r="O331" t="n">
-        <v>0</v>
+        <v>3.17</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>EGGY3</t>
+          <t>CCTY3</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Empresa EGGY</t>
+          <t>Empresa CCTY</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -18677,7 +18677,7 @@
         <v>0</v>
       </c>
       <c r="I332" t="n">
-        <v>954480000</v>
+        <v>0</v>
       </c>
       <c r="J332" t="n">
         <v>0</v>
@@ -18695,18 +18695,18 @@
         <v>0</v>
       </c>
       <c r="O332" t="n">
-        <v>-0.82</v>
+        <v>0</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>CBMA4</t>
+          <t>VVAX4</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -18715,7 +18715,7 @@
         </is>
       </c>
       <c r="D333" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -18732,45 +18732,45 @@
         <v>0</v>
       </c>
       <c r="I333" t="n">
-        <v>-34022300000</v>
+        <v>144676000</v>
       </c>
       <c r="J333" t="n">
         <v>0</v>
       </c>
       <c r="K333" t="n">
-        <v>0</v>
+        <v>-7.36</v>
       </c>
       <c r="L333" t="n">
-        <v>0</v>
+        <v>-37.76</v>
       </c>
       <c r="M333" t="n">
-        <v>0</v>
+        <v>-6.52</v>
       </c>
       <c r="N333" t="n">
-        <v>0</v>
+        <v>-92.03</v>
       </c>
       <c r="O333" t="n">
-        <v>252.65</v>
+        <v>0</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>SALM4</t>
+          <t>CSPC3</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>5.9</v>
+        <v>1.24</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -18787,36 +18787,36 @@
         <v>0</v>
       </c>
       <c r="I334" t="n">
-        <v>475600000</v>
+        <v>2126670000</v>
       </c>
       <c r="J334" t="n">
         <v>0</v>
       </c>
       <c r="K334" t="n">
-        <v>10.22</v>
+        <v>38.62</v>
       </c>
       <c r="L334" t="n">
-        <v>4.13</v>
+        <v>18.85</v>
       </c>
       <c r="M334" t="n">
-        <v>25.78</v>
+        <v>29.18</v>
       </c>
       <c r="N334" t="n">
-        <v>19.53</v>
+        <v>45.33</v>
       </c>
       <c r="O334" t="n">
-        <v>24.53</v>
+        <v>41.15</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>SASG3</t>
+          <t>ABCB3</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Empresa SASG</t>
+          <t>Empresa ABCB</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -18825,7 +18825,7 @@
         </is>
       </c>
       <c r="D335" t="n">
-        <v>0.98</v>
+        <v>0</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -18842,7 +18842,7 @@
         <v>0</v>
       </c>
       <c r="I335" t="n">
-        <v>0</v>
+        <v>7258910000</v>
       </c>
       <c r="J335" t="n">
         <v>0</v>
@@ -18857,30 +18857,30 @@
         <v>0</v>
       </c>
       <c r="N335" t="n">
-        <v>0</v>
+        <v>14.05</v>
       </c>
       <c r="O335" t="n">
-        <v>0</v>
+        <v>7.57</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>BMEF3</t>
+          <t>ESTC4</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Empresa BMEF</t>
+          <t>Empresa ESTC</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -18891,51 +18891,51 @@
         <v>0</v>
       </c>
       <c r="G336" t="n">
-        <v>4.16</v>
+        <v>0</v>
       </c>
       <c r="H336" t="n">
         <v>0</v>
       </c>
       <c r="I336" t="n">
-        <v>2674780000</v>
+        <v>2916530000</v>
       </c>
       <c r="J336" t="n">
         <v>0</v>
       </c>
       <c r="K336" t="n">
-        <v>0</v>
+        <v>16.91</v>
       </c>
       <c r="L336" t="n">
-        <v>0</v>
+        <v>2.02</v>
       </c>
       <c r="M336" t="n">
-        <v>0</v>
+        <v>11.35</v>
       </c>
       <c r="N336" t="n">
-        <v>0</v>
+        <v>3.89</v>
       </c>
       <c r="O336" t="n">
-        <v>0</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>AGEI3</t>
+          <t>VSPT4</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Empresa AGEI</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>7.8</v>
+        <v>0</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -18946,13 +18946,13 @@
         <v>0</v>
       </c>
       <c r="G337" t="n">
-        <v>1.25</v>
+        <v>0</v>
       </c>
       <c r="H337" t="n">
         <v>0</v>
       </c>
       <c r="I337" t="n">
-        <v>1878210000</v>
+        <v>5031600000</v>
       </c>
       <c r="J337" t="n">
         <v>0</v>
@@ -18970,27 +18970,27 @@
         <v>0</v>
       </c>
       <c r="O337" t="n">
-        <v>0</v>
+        <v>4.92</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>ODER3</t>
+          <t>BAUH4</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Empresa ODER</t>
+          <t>Empresa BAUH</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>0</v>
+        <v>93.39</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -19001,16 +19001,16 @@
         <v>0</v>
       </c>
       <c r="G338" t="n">
-        <v>0</v>
+        <v>3.18</v>
       </c>
       <c r="H338" t="n">
-        <v>0</v>
+        <v>1.16</v>
       </c>
       <c r="I338" t="n">
-        <v>609518000</v>
+        <v>153407000</v>
       </c>
       <c r="J338" t="n">
-        <v>0</v>
+        <v>207.53</v>
       </c>
       <c r="K338" t="n">
         <v>0</v>
@@ -19025,18 +19025,18 @@
         <v>0</v>
       </c>
       <c r="O338" t="n">
-        <v>3.17</v>
+        <v>13.32</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>ARPS3</t>
+          <t>ICPI3</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa ICPI</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -19045,7 +19045,7 @@
         </is>
       </c>
       <c r="D339" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -19062,36 +19062,36 @@
         <v>0</v>
       </c>
       <c r="I339" t="n">
-        <v>-12690000</v>
+        <v>0</v>
       </c>
       <c r="J339" t="n">
         <v>0</v>
       </c>
       <c r="K339" t="n">
-        <v>-4.92</v>
+        <v>0</v>
       </c>
       <c r="L339" t="n">
-        <v>-11.59</v>
+        <v>0</v>
       </c>
       <c r="M339" t="n">
-        <v>-6.64</v>
+        <v>0</v>
       </c>
       <c r="N339" t="n">
-        <v>20.34</v>
+        <v>0</v>
       </c>
       <c r="O339" t="n">
-        <v>-17.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>VVAX4</t>
+          <t>ILLS4</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa ILLS</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -19100,7 +19100,7 @@
         </is>
       </c>
       <c r="D340" t="n">
-        <v>0</v>
+        <v>100.01</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -19117,36 +19117,36 @@
         <v>0</v>
       </c>
       <c r="I340" t="n">
-        <v>144676000</v>
+        <v>-18567000</v>
       </c>
       <c r="J340" t="n">
         <v>0</v>
       </c>
       <c r="K340" t="n">
-        <v>-7.36</v>
+        <v>8.43</v>
       </c>
       <c r="L340" t="n">
-        <v>-37.76</v>
+        <v>-10.22</v>
       </c>
       <c r="M340" t="n">
-        <v>-6.52</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="N340" t="n">
-        <v>-92.03</v>
+        <v>36.09</v>
       </c>
       <c r="O340" t="n">
-        <v>0</v>
+        <v>9.33</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>CSPC3</t>
+          <t>BPAT33</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa BPAT</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -19155,7 +19155,7 @@
         </is>
       </c>
       <c r="D341" t="n">
-        <v>1.24</v>
+        <v>20</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -19166,42 +19166,42 @@
         <v>0</v>
       </c>
       <c r="G341" t="n">
-        <v>0</v>
+        <v>0.82</v>
       </c>
       <c r="H341" t="n">
-        <v>0</v>
+        <v>35.72</v>
       </c>
       <c r="I341" t="n">
-        <v>2126670000</v>
+        <v>876492000</v>
       </c>
       <c r="J341" t="n">
         <v>0</v>
       </c>
       <c r="K341" t="n">
-        <v>38.62</v>
+        <v>0</v>
       </c>
       <c r="L341" t="n">
-        <v>18.85</v>
+        <v>0</v>
       </c>
       <c r="M341" t="n">
-        <v>29.18</v>
+        <v>0</v>
       </c>
       <c r="N341" t="n">
-        <v>45.33</v>
+        <v>0</v>
       </c>
       <c r="O341" t="n">
-        <v>41.15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>ABCB3</t>
+          <t>PTIP3</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Empresa ABCB</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -19210,7 +19210,7 @@
         </is>
       </c>
       <c r="D342" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -19227,45 +19227,45 @@
         <v>0</v>
       </c>
       <c r="I342" t="n">
-        <v>7258910000</v>
+        <v>-155957000</v>
       </c>
       <c r="J342" t="n">
         <v>0</v>
       </c>
       <c r="K342" t="n">
-        <v>0</v>
+        <v>13.73</v>
       </c>
       <c r="L342" t="n">
-        <v>0</v>
+        <v>7.55</v>
       </c>
       <c r="M342" t="n">
-        <v>0</v>
+        <v>23.13</v>
       </c>
       <c r="N342" t="n">
-        <v>14.05</v>
+        <v>-121.74</v>
       </c>
       <c r="O342" t="n">
-        <v>7.57</v>
+        <v>62.11</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>CCTY3</t>
+          <t>REPA4</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Empresa CCTY</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>0</v>
+        <v>1.08</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -19282,36 +19282,36 @@
         <v>0</v>
       </c>
       <c r="I343" t="n">
-        <v>0</v>
+        <v>378378000</v>
       </c>
       <c r="J343" t="n">
         <v>0</v>
       </c>
       <c r="K343" t="n">
-        <v>0</v>
+        <v>5.18</v>
       </c>
       <c r="L343" t="n">
-        <v>0</v>
+        <v>1.22</v>
       </c>
       <c r="M343" t="n">
-        <v>0</v>
+        <v>4.05</v>
       </c>
       <c r="N343" t="n">
-        <v>0</v>
+        <v>1.91</v>
       </c>
       <c r="O343" t="n">
-        <v>0</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>VSPT4</t>
+          <t>EQMA6B</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
@@ -19337,7 +19337,7 @@
         <v>0</v>
       </c>
       <c r="I344" t="n">
-        <v>5031600000</v>
+        <v>4940330000</v>
       </c>
       <c r="J344" t="n">
         <v>0</v>
@@ -19355,18 +19355,18 @@
         <v>0</v>
       </c>
       <c r="O344" t="n">
-        <v>4.92</v>
+        <v>9.050000000000001</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>BAUH4</t>
+          <t>SEBB4</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Empresa BAUH</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -19375,7 +19375,7 @@
         </is>
       </c>
       <c r="D345" t="n">
-        <v>93.39</v>
+        <v>0</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -19386,42 +19386,42 @@
         <v>0</v>
       </c>
       <c r="G345" t="n">
-        <v>3.18</v>
+        <v>0</v>
       </c>
       <c r="H345" t="n">
-        <v>1.16</v>
+        <v>0</v>
       </c>
       <c r="I345" t="n">
-        <v>153407000</v>
+        <v>145783000</v>
       </c>
       <c r="J345" t="n">
-        <v>207.53</v>
+        <v>0</v>
       </c>
       <c r="K345" t="n">
-        <v>0</v>
+        <v>9.24</v>
       </c>
       <c r="L345" t="n">
-        <v>0</v>
+        <v>7.4</v>
       </c>
       <c r="M345" t="n">
-        <v>0</v>
+        <v>24.15</v>
       </c>
       <c r="N345" t="n">
-        <v>0</v>
+        <v>23.01</v>
       </c>
       <c r="O345" t="n">
-        <v>13.32</v>
+        <v>50.04</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>ICPI3</t>
+          <t>MSAN3</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Empresa ICPI</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
@@ -19430,7 +19430,7 @@
         </is>
       </c>
       <c r="D346" t="n">
-        <v>0</v>
+        <v>6.44</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -19447,45 +19447,45 @@
         <v>0</v>
       </c>
       <c r="I346" t="n">
-        <v>0</v>
+        <v>2533030000</v>
       </c>
       <c r="J346" t="n">
         <v>0</v>
       </c>
       <c r="K346" t="n">
-        <v>0</v>
+        <v>6.27</v>
       </c>
       <c r="L346" t="n">
-        <v>0</v>
+        <v>2.42</v>
       </c>
       <c r="M346" t="n">
-        <v>0</v>
+        <v>11.78</v>
       </c>
       <c r="N346" t="n">
-        <v>0</v>
+        <v>11.81</v>
       </c>
       <c r="O346" t="n">
-        <v>0</v>
+        <v>101.35</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>ILLS4</t>
+          <t>GALO3</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Empresa ILLS</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>100.01</v>
+        <v>0</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -19502,36 +19502,36 @@
         <v>0</v>
       </c>
       <c r="I347" t="n">
-        <v>-18567000</v>
+        <v>-60607000</v>
       </c>
       <c r="J347" t="n">
         <v>0</v>
       </c>
       <c r="K347" t="n">
-        <v>8.43</v>
+        <v>13.98</v>
       </c>
       <c r="L347" t="n">
-        <v>-10.22</v>
+        <v>-184.58</v>
       </c>
       <c r="M347" t="n">
-        <v>8.140000000000001</v>
+        <v>39.37</v>
       </c>
       <c r="N347" t="n">
-        <v>36.09</v>
+        <v>7.62</v>
       </c>
       <c r="O347" t="n">
-        <v>9.33</v>
+        <v>-28.97</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>BPAT33</t>
+          <t>SLCP3</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Empresa BPAT</t>
+          <t>Empresa SLCP</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
@@ -19540,7 +19540,7 @@
         </is>
       </c>
       <c r="D348" t="n">
-        <v>20</v>
+        <v>610.02</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -19551,13 +19551,13 @@
         <v>0</v>
       </c>
       <c r="G348" t="n">
-        <v>0.82</v>
+        <v>0</v>
       </c>
       <c r="H348" t="n">
-        <v>35.72</v>
+        <v>0</v>
       </c>
       <c r="I348" t="n">
-        <v>876492000</v>
+        <v>0</v>
       </c>
       <c r="J348" t="n">
         <v>0</v>
@@ -19581,17 +19581,17 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>ESTC4</t>
+          <t>DAYC3</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Empresa ESTC</t>
+          <t>Empresa DAYC</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D349" t="n">
@@ -19612,36 +19612,36 @@
         <v>0</v>
       </c>
       <c r="I349" t="n">
-        <v>2916530000</v>
+        <v>3009030000</v>
       </c>
       <c r="J349" t="n">
         <v>0</v>
       </c>
       <c r="K349" t="n">
-        <v>16.91</v>
+        <v>0</v>
       </c>
       <c r="L349" t="n">
-        <v>2.02</v>
+        <v>0</v>
       </c>
       <c r="M349" t="n">
-        <v>11.35</v>
+        <v>0</v>
       </c>
       <c r="N349" t="n">
-        <v>3.89</v>
+        <v>17.33</v>
       </c>
       <c r="O349" t="n">
-        <v>5.6</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>SEBB4</t>
+          <t>TNEP4</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
@@ -19650,7 +19650,7 @@
         </is>
       </c>
       <c r="D350" t="n">
-        <v>0</v>
+        <v>3.95</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -19667,36 +19667,36 @@
         <v>0</v>
       </c>
       <c r="I350" t="n">
-        <v>145783000</v>
+        <v>955105000</v>
       </c>
       <c r="J350" t="n">
         <v>0</v>
       </c>
       <c r="K350" t="n">
-        <v>9.24</v>
+        <v>20.92</v>
       </c>
       <c r="L350" t="n">
-        <v>7.4</v>
+        <v>25.42</v>
       </c>
       <c r="M350" t="n">
-        <v>24.15</v>
+        <v>20.53</v>
       </c>
       <c r="N350" t="n">
-        <v>23.01</v>
+        <v>22.8</v>
       </c>
       <c r="O350" t="n">
-        <v>50.04</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>MSAN3</t>
+          <t>MLPA3</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa MLPA</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -19705,7 +19705,7 @@
         </is>
       </c>
       <c r="D351" t="n">
-        <v>6.44</v>
+        <v>0</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -19722,41 +19722,41 @@
         <v>0</v>
       </c>
       <c r="I351" t="n">
-        <v>2533030000</v>
+        <v>44578000</v>
       </c>
       <c r="J351" t="n">
         <v>0</v>
       </c>
       <c r="K351" t="n">
-        <v>6.27</v>
+        <v>6.66</v>
       </c>
       <c r="L351" t="n">
-        <v>2.42</v>
+        <v>8.92</v>
       </c>
       <c r="M351" t="n">
-        <v>11.78</v>
+        <v>0</v>
       </c>
       <c r="N351" t="n">
-        <v>11.81</v>
+        <v>45.13</v>
       </c>
       <c r="O351" t="n">
-        <v>101.35</v>
+        <v>-7.51</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>GALO3</t>
+          <t>CLSC6</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa CLSC</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D352" t="n">
@@ -19777,36 +19777,36 @@
         <v>0</v>
       </c>
       <c r="I352" t="n">
-        <v>-60607000</v>
+        <v>4228180000</v>
       </c>
       <c r="J352" t="n">
         <v>0</v>
       </c>
       <c r="K352" t="n">
-        <v>13.98</v>
+        <v>0</v>
       </c>
       <c r="L352" t="n">
-        <v>-184.58</v>
+        <v>0</v>
       </c>
       <c r="M352" t="n">
-        <v>39.37</v>
+        <v>0</v>
       </c>
       <c r="N352" t="n">
-        <v>7.62</v>
+        <v>0</v>
       </c>
       <c r="O352" t="n">
-        <v>-28.97</v>
+        <v>2.82</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>SLCP3</t>
+          <t>SGEN3</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Empresa SLCP</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -19815,7 +19815,7 @@
         </is>
       </c>
       <c r="D353" t="n">
-        <v>610.02</v>
+        <v>5</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -19826,47 +19826,47 @@
         <v>0</v>
       </c>
       <c r="G353" t="n">
-        <v>0</v>
+        <v>0.77</v>
       </c>
       <c r="H353" t="n">
         <v>0</v>
       </c>
       <c r="I353" t="n">
-        <v>0</v>
+        <v>156981000</v>
       </c>
       <c r="J353" t="n">
         <v>0</v>
       </c>
       <c r="K353" t="n">
-        <v>0</v>
+        <v>-1871.17</v>
       </c>
       <c r="L353" t="n">
         <v>0</v>
       </c>
       <c r="M353" t="n">
-        <v>0</v>
+        <v>-1.59</v>
       </c>
       <c r="N353" t="n">
         <v>0</v>
       </c>
       <c r="O353" t="n">
-        <v>0</v>
+        <v>-59.85</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>DAYC3</t>
+          <t>DUFB11</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Empresa DAYC</t>
+          <t>Empresa DUFB</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D354" t="n">
@@ -19887,7 +19887,7 @@
         <v>0</v>
       </c>
       <c r="I354" t="n">
-        <v>3009030000</v>
+        <v>0</v>
       </c>
       <c r="J354" t="n">
         <v>0</v>
@@ -19902,21 +19902,21 @@
         <v>0</v>
       </c>
       <c r="N354" t="n">
-        <v>17.33</v>
+        <v>0</v>
       </c>
       <c r="O354" t="n">
-        <v>8.15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>PTIP3</t>
+          <t>CCHI3</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -19925,7 +19925,7 @@
         </is>
       </c>
       <c r="D355" t="n">
-        <v>22</v>
+        <v>0.02</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -19936,51 +19936,51 @@
         <v>0</v>
       </c>
       <c r="G355" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="H355" t="n">
         <v>0</v>
       </c>
       <c r="I355" t="n">
-        <v>-155957000</v>
+        <v>-160477000</v>
       </c>
       <c r="J355" t="n">
         <v>0</v>
       </c>
       <c r="K355" t="n">
-        <v>13.73</v>
+        <v>0</v>
       </c>
       <c r="L355" t="n">
-        <v>7.55</v>
+        <v>0</v>
       </c>
       <c r="M355" t="n">
-        <v>23.13</v>
+        <v>0</v>
       </c>
       <c r="N355" t="n">
-        <v>-121.74</v>
+        <v>0</v>
       </c>
       <c r="O355" t="n">
-        <v>62.11</v>
+        <v>20.36</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>REPA4</t>
+          <t>SFSA3</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa SFSA</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D356" t="n">
-        <v>1.08</v>
+        <v>0</v>
       </c>
       <c r="E356" t="inlineStr">
         <is>
@@ -19997,41 +19997,41 @@
         <v>0</v>
       </c>
       <c r="I356" t="n">
-        <v>378378000</v>
+        <v>739524000</v>
       </c>
       <c r="J356" t="n">
         <v>0</v>
       </c>
       <c r="K356" t="n">
-        <v>5.18</v>
+        <v>0</v>
       </c>
       <c r="L356" t="n">
-        <v>1.22</v>
+        <v>0</v>
       </c>
       <c r="M356" t="n">
-        <v>4.05</v>
+        <v>0</v>
       </c>
       <c r="N356" t="n">
-        <v>1.91</v>
+        <v>6.25</v>
       </c>
       <c r="O356" t="n">
-        <v>1.09</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>EQMA6B</t>
+          <t>PRBC3</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa PRBC</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D357" t="n">
@@ -20052,7 +20052,7 @@
         <v>0</v>
       </c>
       <c r="I357" t="n">
-        <v>4940330000</v>
+        <v>1319270000</v>
       </c>
       <c r="J357" t="n">
         <v>0</v>
@@ -20067,21 +20067,21 @@
         <v>0</v>
       </c>
       <c r="N357" t="n">
-        <v>0</v>
+        <v>8.27</v>
       </c>
       <c r="O357" t="n">
-        <v>9.050000000000001</v>
+        <v>-1.98</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>SGEN3</t>
+          <t>ECIS3</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -20090,7 +20090,7 @@
         </is>
       </c>
       <c r="D358" t="n">
-        <v>5</v>
+        <v>211.65</v>
       </c>
       <c r="E358" t="inlineStr">
         <is>
@@ -20101,51 +20101,51 @@
         <v>0</v>
       </c>
       <c r="G358" t="n">
-        <v>0.77</v>
+        <v>0</v>
       </c>
       <c r="H358" t="n">
         <v>0</v>
       </c>
       <c r="I358" t="n">
-        <v>156981000</v>
+        <v>129346000</v>
       </c>
       <c r="J358" t="n">
         <v>0</v>
       </c>
       <c r="K358" t="n">
-        <v>-1871.17</v>
+        <v>34.9</v>
       </c>
       <c r="L358" t="n">
-        <v>0</v>
+        <v>14.18</v>
       </c>
       <c r="M358" t="n">
-        <v>-1.59</v>
+        <v>12.48</v>
       </c>
       <c r="N358" t="n">
-        <v>0</v>
+        <v>7.33</v>
       </c>
       <c r="O358" t="n">
-        <v>-59.85</v>
+        <v>4.66</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>DUFB11</t>
+          <t>BSGR3</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Empresa DUFB</t>
+          <t>Empresa BSGR</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>0</v>
+        <v>1091.28</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -20186,21 +20186,21 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>TNEP4</t>
+          <t>CBMA3</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>3.95</v>
+        <v>0.01</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -20217,36 +20217,36 @@
         <v>0</v>
       </c>
       <c r="I360" t="n">
-        <v>955105000</v>
+        <v>-34022300000</v>
       </c>
       <c r="J360" t="n">
         <v>0</v>
       </c>
       <c r="K360" t="n">
-        <v>20.92</v>
+        <v>0</v>
       </c>
       <c r="L360" t="n">
-        <v>25.42</v>
+        <v>0</v>
       </c>
       <c r="M360" t="n">
-        <v>20.53</v>
+        <v>0</v>
       </c>
       <c r="N360" t="n">
-        <v>22.8</v>
+        <v>0</v>
       </c>
       <c r="O360" t="n">
-        <v>8.15</v>
+        <v>252.65</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>MLPA3</t>
+          <t>ALBA3</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Empresa MLPA</t>
+          <t>Empresa ALBA</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -20255,7 +20255,7 @@
         </is>
       </c>
       <c r="D361" t="n">
-        <v>0</v>
+        <v>2.15</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -20272,36 +20272,36 @@
         <v>0</v>
       </c>
       <c r="I361" t="n">
-        <v>44578000</v>
+        <v>354860000</v>
       </c>
       <c r="J361" t="n">
         <v>0</v>
       </c>
       <c r="K361" t="n">
-        <v>6.66</v>
+        <v>9.5</v>
       </c>
       <c r="L361" t="n">
-        <v>8.92</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="M361" t="n">
-        <v>0</v>
+        <v>20.4</v>
       </c>
       <c r="N361" t="n">
-        <v>45.13</v>
+        <v>19.77</v>
       </c>
       <c r="O361" t="n">
-        <v>-7.51</v>
+        <v>14.69</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>CLSC6</t>
+          <t>ARPS4</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>Empresa CLSC</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -20327,36 +20327,36 @@
         <v>0</v>
       </c>
       <c r="I362" t="n">
-        <v>4228180000</v>
+        <v>-12690000</v>
       </c>
       <c r="J362" t="n">
         <v>0</v>
       </c>
       <c r="K362" t="n">
-        <v>0</v>
+        <v>-4.92</v>
       </c>
       <c r="L362" t="n">
-        <v>0</v>
+        <v>-11.59</v>
       </c>
       <c r="M362" t="n">
-        <v>0</v>
+        <v>-6.64</v>
       </c>
       <c r="N362" t="n">
-        <v>0</v>
+        <v>20.34</v>
       </c>
       <c r="O362" t="n">
-        <v>2.82</v>
+        <v>-17.53</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>CCHI3</t>
+          <t>SALM3</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -20365,7 +20365,7 @@
         </is>
       </c>
       <c r="D363" t="n">
-        <v>0.02</v>
+        <v>5.7</v>
       </c>
       <c r="E363" t="inlineStr">
         <is>
@@ -20376,51 +20376,51 @@
         <v>0</v>
       </c>
       <c r="G363" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="H363" t="n">
         <v>0</v>
       </c>
       <c r="I363" t="n">
-        <v>-160477000</v>
+        <v>475600000</v>
       </c>
       <c r="J363" t="n">
         <v>0</v>
       </c>
       <c r="K363" t="n">
-        <v>0</v>
+        <v>10.22</v>
       </c>
       <c r="L363" t="n">
-        <v>0</v>
+        <v>4.13</v>
       </c>
       <c r="M363" t="n">
-        <v>0</v>
+        <v>25.78</v>
       </c>
       <c r="N363" t="n">
-        <v>0</v>
+        <v>19.53</v>
       </c>
       <c r="O363" t="n">
-        <v>20.36</v>
+        <v>24.53</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>SFSA3</t>
+          <t>CMMA4</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Empresa SFSA</t>
+          <t>Empresa CMMA</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D364" t="n">
-        <v>0</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -20437,7 +20437,7 @@
         <v>0</v>
       </c>
       <c r="I364" t="n">
-        <v>739524000</v>
+        <v>-79623000</v>
       </c>
       <c r="J364" t="n">
         <v>0</v>
@@ -20452,21 +20452,21 @@
         <v>0</v>
       </c>
       <c r="N364" t="n">
-        <v>6.25</v>
+        <v>-1.92</v>
       </c>
       <c r="O364" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>PRBC3</t>
+          <t>CZRS3</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Empresa PRBC</t>
+          <t>Empresa CZRS</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
@@ -20492,7 +20492,7 @@
         <v>0</v>
       </c>
       <c r="I365" t="n">
-        <v>1319270000</v>
+        <v>1145670000</v>
       </c>
       <c r="J365" t="n">
         <v>0</v>
@@ -20507,21 +20507,21 @@
         <v>0</v>
       </c>
       <c r="N365" t="n">
-        <v>8.27</v>
+        <v>3.34</v>
       </c>
       <c r="O365" t="n">
-        <v>-1.98</v>
+        <v>14.44</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>ECIS3</t>
+          <t>BPNM3</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa BPNM</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -20530,7 +20530,7 @@
         </is>
       </c>
       <c r="D366" t="n">
-        <v>211.65</v>
+        <v>0</v>
       </c>
       <c r="E366" t="inlineStr">
         <is>
@@ -20547,45 +20547,45 @@
         <v>0</v>
       </c>
       <c r="I366" t="n">
-        <v>129346000</v>
+        <v>7792670000</v>
       </c>
       <c r="J366" t="n">
         <v>0</v>
       </c>
       <c r="K366" t="n">
-        <v>34.9</v>
+        <v>0</v>
       </c>
       <c r="L366" t="n">
-        <v>14.18</v>
+        <v>0</v>
       </c>
       <c r="M366" t="n">
-        <v>12.48</v>
+        <v>0</v>
       </c>
       <c r="N366" t="n">
-        <v>7.33</v>
+        <v>9.67</v>
       </c>
       <c r="O366" t="n">
-        <v>4.66</v>
+        <v>-1.53</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>CMMA4</t>
+          <t>VNET3</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Empresa CMMA</t>
+          <t>Empresa VNET</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D367" t="n">
-        <v>0.8100000000000001</v>
+        <v>0</v>
       </c>
       <c r="E367" t="inlineStr">
         <is>
@@ -20602,7 +20602,7 @@
         <v>0</v>
       </c>
       <c r="I367" t="n">
-        <v>-79623000</v>
+        <v>14163000000</v>
       </c>
       <c r="J367" t="n">
         <v>0</v>
@@ -20617,30 +20617,30 @@
         <v>0</v>
       </c>
       <c r="N367" t="n">
-        <v>-1.92</v>
+        <v>0</v>
       </c>
       <c r="O367" t="n">
-        <v>0</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>CZRS3</t>
+          <t>CSPC4</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Empresa CZRS</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D368" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="E368" t="inlineStr">
         <is>
@@ -20657,36 +20657,36 @@
         <v>0</v>
       </c>
       <c r="I368" t="n">
-        <v>1145670000</v>
+        <v>2126670000</v>
       </c>
       <c r="J368" t="n">
         <v>0</v>
       </c>
       <c r="K368" t="n">
-        <v>0</v>
+        <v>38.62</v>
       </c>
       <c r="L368" t="n">
-        <v>0</v>
+        <v>18.85</v>
       </c>
       <c r="M368" t="n">
-        <v>0</v>
+        <v>29.18</v>
       </c>
       <c r="N368" t="n">
-        <v>3.34</v>
+        <v>45.33</v>
       </c>
       <c r="O368" t="n">
-        <v>14.44</v>
+        <v>41.15</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>BPNM3</t>
+          <t>BOVH3</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Empresa BPNM</t>
+          <t>Empresa BOVH</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -20695,7 +20695,7 @@
         </is>
       </c>
       <c r="D369" t="n">
-        <v>0</v>
+        <v>15.71</v>
       </c>
       <c r="E369" t="inlineStr">
         <is>
@@ -20706,13 +20706,13 @@
         <v>0</v>
       </c>
       <c r="G369" t="n">
-        <v>0</v>
+        <v>6.16</v>
       </c>
       <c r="H369" t="n">
         <v>0</v>
       </c>
       <c r="I369" t="n">
-        <v>7792670000</v>
+        <v>1843320000</v>
       </c>
       <c r="J369" t="n">
         <v>0</v>
@@ -20727,21 +20727,21 @@
         <v>0</v>
       </c>
       <c r="N369" t="n">
-        <v>9.67</v>
+        <v>0</v>
       </c>
       <c r="O369" t="n">
-        <v>-1.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>BSGR3</t>
+          <t>ARND3</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Empresa BSGR</t>
+          <t>Empresa ARND</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -20750,7 +20750,7 @@
         </is>
       </c>
       <c r="D370" t="n">
-        <v>1091.28</v>
+        <v>0.51</v>
       </c>
       <c r="E370" t="inlineStr">
         <is>
@@ -20761,16 +20761,16 @@
         <v>0</v>
       </c>
       <c r="G370" t="n">
-        <v>0</v>
+        <v>0.57</v>
       </c>
       <c r="H370" t="n">
         <v>0</v>
       </c>
       <c r="I370" t="n">
-        <v>0</v>
+        <v>125211000</v>
       </c>
       <c r="J370" t="n">
-        <v>0</v>
+        <v>913.58</v>
       </c>
       <c r="K370" t="n">
         <v>0</v>
@@ -20785,27 +20785,27 @@
         <v>0</v>
       </c>
       <c r="O370" t="n">
-        <v>0</v>
+        <v>-0.88</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>CBMA3</t>
+          <t>PTIP4</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D371" t="n">
-        <v>0.01</v>
+        <v>25.15</v>
       </c>
       <c r="E371" t="inlineStr">
         <is>
@@ -20822,36 +20822,36 @@
         <v>0</v>
       </c>
       <c r="I371" t="n">
-        <v>-34022300000</v>
+        <v>-155957000</v>
       </c>
       <c r="J371" t="n">
         <v>0</v>
       </c>
       <c r="K371" t="n">
-        <v>0</v>
+        <v>13.73</v>
       </c>
       <c r="L371" t="n">
-        <v>0</v>
+        <v>7.55</v>
       </c>
       <c r="M371" t="n">
-        <v>0</v>
+        <v>23.13</v>
       </c>
       <c r="N371" t="n">
-        <v>0</v>
+        <v>-121.74</v>
       </c>
       <c r="O371" t="n">
-        <v>252.65</v>
+        <v>62.11</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>ALBA3</t>
+          <t>LATS3</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Empresa ALBA</t>
+          <t>Empresa LATS</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
@@ -20860,7 +20860,7 @@
         </is>
       </c>
       <c r="D372" t="n">
-        <v>2.15</v>
+        <v>22</v>
       </c>
       <c r="E372" t="inlineStr">
         <is>
@@ -20877,41 +20877,41 @@
         <v>0</v>
       </c>
       <c r="I372" t="n">
-        <v>354860000</v>
+        <v>680646000</v>
       </c>
       <c r="J372" t="n">
         <v>0</v>
       </c>
       <c r="K372" t="n">
-        <v>9.5</v>
+        <v>11.74</v>
       </c>
       <c r="L372" t="n">
-        <v>9.619999999999999</v>
+        <v>1.3</v>
       </c>
       <c r="M372" t="n">
-        <v>20.4</v>
+        <v>11.63</v>
       </c>
       <c r="N372" t="n">
-        <v>19.77</v>
+        <v>1.84</v>
       </c>
       <c r="O372" t="n">
-        <v>14.69</v>
+        <v>15.37</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>ARPS4</t>
+          <t>VVAX3</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D373" t="n">
@@ -20932,45 +20932,45 @@
         <v>0</v>
       </c>
       <c r="I373" t="n">
-        <v>-12690000</v>
+        <v>144676000</v>
       </c>
       <c r="J373" t="n">
         <v>0</v>
       </c>
       <c r="K373" t="n">
-        <v>-4.92</v>
+        <v>-7.36</v>
       </c>
       <c r="L373" t="n">
-        <v>-11.59</v>
+        <v>-37.76</v>
       </c>
       <c r="M373" t="n">
-        <v>-6.64</v>
+        <v>-6.52</v>
       </c>
       <c r="N373" t="n">
-        <v>20.34</v>
+        <v>-92.03</v>
       </c>
       <c r="O373" t="n">
-        <v>-17.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>SALM3</t>
+          <t>MSAN4</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D374" t="n">
-        <v>5.7</v>
+        <v>6.44</v>
       </c>
       <c r="E374" t="inlineStr">
         <is>
@@ -20987,45 +20987,45 @@
         <v>0</v>
       </c>
       <c r="I374" t="n">
-        <v>475600000</v>
+        <v>2533030000</v>
       </c>
       <c r="J374" t="n">
         <v>0</v>
       </c>
       <c r="K374" t="n">
-        <v>10.22</v>
+        <v>6.27</v>
       </c>
       <c r="L374" t="n">
-        <v>4.13</v>
+        <v>2.42</v>
       </c>
       <c r="M374" t="n">
-        <v>25.78</v>
+        <v>11.78</v>
       </c>
       <c r="N374" t="n">
-        <v>19.53</v>
+        <v>11.81</v>
       </c>
       <c r="O374" t="n">
-        <v>24.53</v>
+        <v>101.35</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>VNET3</t>
+          <t>GALO4</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>Empresa VNET</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D375" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E375" t="inlineStr">
         <is>
@@ -21042,45 +21042,45 @@
         <v>0</v>
       </c>
       <c r="I375" t="n">
-        <v>14163000000</v>
+        <v>-60607000</v>
       </c>
       <c r="J375" t="n">
         <v>0</v>
       </c>
       <c r="K375" t="n">
-        <v>0</v>
+        <v>13.98</v>
       </c>
       <c r="L375" t="n">
-        <v>0</v>
+        <v>-184.58</v>
       </c>
       <c r="M375" t="n">
-        <v>0</v>
+        <v>39.37</v>
       </c>
       <c r="N375" t="n">
-        <v>0</v>
+        <v>7.62</v>
       </c>
       <c r="O375" t="n">
-        <v>1.08</v>
+        <v>-28.97</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>CSPC4</t>
+          <t>BBTG13</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D376" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="E376" t="inlineStr">
         <is>
@@ -21097,36 +21097,36 @@
         <v>0</v>
       </c>
       <c r="I376" t="n">
-        <v>2126670000</v>
+        <v>7000</v>
       </c>
       <c r="J376" t="n">
         <v>0</v>
       </c>
       <c r="K376" t="n">
-        <v>38.62</v>
+        <v>0</v>
       </c>
       <c r="L376" t="n">
-        <v>18.85</v>
+        <v>0</v>
       </c>
       <c r="M376" t="n">
-        <v>29.18</v>
+        <v>0</v>
       </c>
       <c r="N376" t="n">
-        <v>45.33</v>
+        <v>-42.86</v>
       </c>
       <c r="O376" t="n">
-        <v>41.15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>BOVH3</t>
+          <t>INHA3</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>Empresa BOVH</t>
+          <t>Empresa INHA</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
@@ -21135,7 +21135,7 @@
         </is>
       </c>
       <c r="D377" t="n">
-        <v>15.71</v>
+        <v>0</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -21146,31 +21146,31 @@
         <v>0</v>
       </c>
       <c r="G377" t="n">
-        <v>6.16</v>
+        <v>0</v>
       </c>
       <c r="H377" t="n">
         <v>0</v>
       </c>
       <c r="I377" t="n">
-        <v>1843320000</v>
+        <v>1533210000</v>
       </c>
       <c r="J377" t="n">
         <v>0</v>
       </c>
       <c r="K377" t="n">
-        <v>0</v>
+        <v>-56.05</v>
       </c>
       <c r="L377" t="n">
-        <v>0</v>
+        <v>-124.06</v>
       </c>
       <c r="M377" t="n">
-        <v>0</v>
+        <v>-6.27</v>
       </c>
       <c r="N377" t="n">
-        <v>0</v>
+        <v>-39.87</v>
       </c>
       <c r="O377" t="n">
-        <v>0</v>
+        <v>-12.18</v>
       </c>
     </row>
     <row r="378">
@@ -24696,7 +24696,7 @@
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>MMAQ4</t>
+          <t>MMAQ3</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
@@ -24706,7 +24706,7 @@
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D442" t="n">
@@ -24724,7 +24724,7 @@
         <v>0.36</v>
       </c>
       <c r="H442" t="n">
-        <v>41.68</v>
+        <v>0</v>
       </c>
       <c r="I442" t="n">
         <v>259016000</v>
@@ -24751,7 +24751,7 @@
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>MMAQ3</t>
+          <t>MMAQ4</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
@@ -24761,7 +24761,7 @@
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D443" t="n">
@@ -24779,7 +24779,7 @@
         <v>0.36</v>
       </c>
       <c r="H443" t="n">
-        <v>0</v>
+        <v>41.68</v>
       </c>
       <c r="I443" t="n">
         <v>259016000</v>
@@ -32946,7 +32946,7 @@
     <row r="592">
       <c r="A592" t="inlineStr">
         <is>
-          <t>GETT4</t>
+          <t>GETT3</t>
         </is>
       </c>
       <c r="B592" t="inlineStr">
@@ -32956,7 +32956,7 @@
       </c>
       <c r="C592" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D592" t="n">
@@ -33001,7 +33001,7 @@
     <row r="593">
       <c r="A593" t="inlineStr">
         <is>
-          <t>GETT3</t>
+          <t>GETT4</t>
         </is>
       </c>
       <c r="B593" t="inlineStr">
@@ -33011,7 +33011,7 @@
       </c>
       <c r="C593" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D593" t="n">
@@ -33661,7 +33661,7 @@
     <row r="605">
       <c r="A605" t="inlineStr">
         <is>
-          <t>RPAD3</t>
+          <t>RPAD6</t>
         </is>
       </c>
       <c r="B605" t="inlineStr">
@@ -33671,7 +33671,7 @@
       </c>
       <c r="C605" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D605" t="n">
@@ -33689,13 +33689,13 @@
         <v>0.57</v>
       </c>
       <c r="H605" t="n">
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="I605" t="n">
         <v>1046150000</v>
       </c>
       <c r="J605" t="n">
-        <v>2695.56</v>
+        <v>2752.22</v>
       </c>
       <c r="K605" t="n">
         <v>0</v>
@@ -33716,7 +33716,7 @@
     <row r="606">
       <c r="A606" t="inlineStr">
         <is>
-          <t>RPAD6</t>
+          <t>RPAD3</t>
         </is>
       </c>
       <c r="B606" t="inlineStr">
@@ -33726,7 +33726,7 @@
       </c>
       <c r="C606" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D606" t="n">
@@ -33744,13 +33744,13 @@
         <v>0.57</v>
       </c>
       <c r="H606" t="n">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="I606" t="n">
         <v>1046150000</v>
       </c>
       <c r="J606" t="n">
-        <v>2752.22</v>
+        <v>2695.56</v>
       </c>
       <c r="K606" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atualiza nomenclatura setorial oficial da B3 e ajustes nos graficos
</commit_message>
<xml_diff>
--- a/acoes_b3.xlsx
+++ b/acoes_b3.xlsx
@@ -2879,7 +2879,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Exploração de Imóveis</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -3374,7 +3374,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Seguradoras</t>
+          <t>Previdência e Seguros</t>
         </is>
       </c>
       <c r="F54" t="n">
@@ -4309,7 +4309,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Agro e Alimentos</t>
+          <t>Agropecuária</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Saúde e Farmácia</t>
+          <t>Serviços Médico-Hospitalares</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -4969,7 +4969,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Agro e Alimentos</t>
+          <t>Agropecuária</t>
         </is>
       </c>
       <c r="F83" t="n">
@@ -5684,7 +5684,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Tecnologia</t>
+          <t>Tecnologia da Informação</t>
         </is>
       </c>
       <c r="F96" t="n">
@@ -6619,7 +6619,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Serviços Financeiros</t>
+          <t>Serviços Financeiros Diversos</t>
         </is>
       </c>
       <c r="F113" t="n">
@@ -7499,7 +7499,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Mineração e Siderurgia</t>
+          <t>Siderurgia e Metalurgia</t>
         </is>
       </c>
       <c r="F129" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Varejo e Comércio</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F132" t="n">
@@ -7884,7 +7884,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Mineração e Siderurgia</t>
+          <t>Siderurgia e Metalurgia</t>
         </is>
       </c>
       <c r="F136" t="n">
@@ -8159,7 +8159,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Mineração e Siderurgia</t>
+          <t>Siderurgia e Metalurgia</t>
         </is>
       </c>
       <c r="F141" t="n">
@@ -8434,7 +8434,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Mineração e Siderurgia</t>
+          <t>Siderurgia e Metalurgia</t>
         </is>
       </c>
       <c r="F146" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Varejo e Comércio</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F152" t="n">
@@ -9351,7 +9351,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>RNEW4</t>
+          <t>RNEW3</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -9361,7 +9361,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -9385,7 +9385,7 @@
         <v>1150280000</v>
       </c>
       <c r="J163" t="n">
-        <v>44097</v>
+        <v>45273.4</v>
       </c>
       <c r="K163" t="n">
         <v>-2.89</v>
@@ -9406,7 +9406,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>RNEW3</t>
+          <t>RNEW4</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -9416,7 +9416,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -9440,7 +9440,7 @@
         <v>1150280000</v>
       </c>
       <c r="J164" t="n">
-        <v>45273.4</v>
+        <v>44097</v>
       </c>
       <c r="K164" t="n">
         <v>-2.89</v>
@@ -10414,7 +10414,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Petróleo e Gás</t>
+          <t>Petróleo, Gás e Biocombustíveis</t>
         </is>
       </c>
       <c r="F182" t="n">
@@ -10671,7 +10671,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>SDIA3</t>
+          <t>SDIA4</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -10681,7 +10681,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -10726,7 +10726,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>SDIA4</t>
+          <t>SDIA3</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -10736,7 +10736,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -11404,7 +11404,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Varejo e Comércio</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F200" t="n">
@@ -12119,7 +12119,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Saneamento</t>
+          <t>Água e Saneamento</t>
         </is>
       </c>
       <c r="F213" t="n">
@@ -13659,7 +13659,7 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>Saúde e Farmácia</t>
+          <t>Serviços Médico-Hospitalares</t>
         </is>
       </c>
       <c r="F241" t="n">
@@ -15254,7 +15254,7 @@
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>Agro e Alimentos</t>
+          <t>Petróleo, Gás e Biocombustíveis</t>
         </is>
       </c>
       <c r="F270" t="n">
@@ -15914,7 +15914,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Varejo e Comércio</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F282" t="n">
@@ -16409,7 +16409,7 @@
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Exploração de Imóveis</t>
         </is>
       </c>
       <c r="F291" t="n">
@@ -17381,17 +17381,17 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>ARPS4</t>
+          <t>VVAX3</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -17412,45 +17412,45 @@
         <v>0</v>
       </c>
       <c r="I309" t="n">
-        <v>-12690000</v>
+        <v>144676000</v>
       </c>
       <c r="J309" t="n">
         <v>0</v>
       </c>
       <c r="K309" t="n">
-        <v>-4.92</v>
+        <v>-7.36</v>
       </c>
       <c r="L309" t="n">
-        <v>-11.59</v>
+        <v>-37.76</v>
       </c>
       <c r="M309" t="n">
-        <v>-6.64</v>
+        <v>-6.52</v>
       </c>
       <c r="N309" t="n">
-        <v>20.34</v>
+        <v>-92.03</v>
       </c>
       <c r="O309" t="n">
-        <v>-17.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>SALM3</t>
+          <t>MSAN4</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>5.7</v>
+        <v>6.44</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -17467,36 +17467,36 @@
         <v>0</v>
       </c>
       <c r="I310" t="n">
-        <v>475600000</v>
+        <v>2533030000</v>
       </c>
       <c r="J310" t="n">
         <v>0</v>
       </c>
       <c r="K310" t="n">
-        <v>10.22</v>
+        <v>6.27</v>
       </c>
       <c r="L310" t="n">
-        <v>4.13</v>
+        <v>2.42</v>
       </c>
       <c r="M310" t="n">
-        <v>25.78</v>
+        <v>11.78</v>
       </c>
       <c r="N310" t="n">
-        <v>19.53</v>
+        <v>11.81</v>
       </c>
       <c r="O310" t="n">
-        <v>24.53</v>
+        <v>101.35</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>CMMA4</t>
+          <t>GALO4</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Empresa CMMA</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -17505,7 +17505,7 @@
         </is>
       </c>
       <c r="D311" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.25</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -17522,36 +17522,36 @@
         <v>0</v>
       </c>
       <c r="I311" t="n">
-        <v>-79623000</v>
+        <v>-60607000</v>
       </c>
       <c r="J311" t="n">
         <v>0</v>
       </c>
       <c r="K311" t="n">
-        <v>0</v>
+        <v>13.98</v>
       </c>
       <c r="L311" t="n">
-        <v>0</v>
+        <v>-184.58</v>
       </c>
       <c r="M311" t="n">
-        <v>0</v>
+        <v>39.37</v>
       </c>
       <c r="N311" t="n">
-        <v>-1.92</v>
+        <v>7.62</v>
       </c>
       <c r="O311" t="n">
-        <v>0</v>
+        <v>-28.97</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>CZRS3</t>
+          <t>BBTG13</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Empresa CZRS</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -17577,7 +17577,7 @@
         <v>0</v>
       </c>
       <c r="I312" t="n">
-        <v>1145670000</v>
+        <v>7000</v>
       </c>
       <c r="J312" t="n">
         <v>0</v>
@@ -17592,21 +17592,21 @@
         <v>0</v>
       </c>
       <c r="N312" t="n">
-        <v>3.34</v>
+        <v>-42.86</v>
       </c>
       <c r="O312" t="n">
-        <v>14.44</v>
+        <v>0</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>BPNM3</t>
+          <t>INHA3</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Empresa BPNM</t>
+          <t>Empresa INHA</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -17632,45 +17632,45 @@
         <v>0</v>
       </c>
       <c r="I313" t="n">
-        <v>7792670000</v>
+        <v>1533210000</v>
       </c>
       <c r="J313" t="n">
         <v>0</v>
       </c>
       <c r="K313" t="n">
-        <v>0</v>
+        <v>-56.05</v>
       </c>
       <c r="L313" t="n">
-        <v>0</v>
+        <v>-124.06</v>
       </c>
       <c r="M313" t="n">
-        <v>0</v>
+        <v>-6.27</v>
       </c>
       <c r="N313" t="n">
-        <v>9.67</v>
+        <v>-39.87</v>
       </c>
       <c r="O313" t="n">
-        <v>-1.53</v>
+        <v>-12.18</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>BSGR3</t>
+          <t>PTIP4</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Empresa BSGR</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>1091.28</v>
+        <v>25.15</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -17687,36 +17687,36 @@
         <v>0</v>
       </c>
       <c r="I314" t="n">
-        <v>0</v>
+        <v>-155957000</v>
       </c>
       <c r="J314" t="n">
         <v>0</v>
       </c>
       <c r="K314" t="n">
-        <v>0</v>
+        <v>13.73</v>
       </c>
       <c r="L314" t="n">
-        <v>0</v>
+        <v>7.55</v>
       </c>
       <c r="M314" t="n">
-        <v>0</v>
+        <v>23.13</v>
       </c>
       <c r="N314" t="n">
-        <v>0</v>
+        <v>-121.74</v>
       </c>
       <c r="O314" t="n">
-        <v>0</v>
+        <v>62.11</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>CBMA3</t>
+          <t>LATS3</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa LATS</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -17725,7 +17725,7 @@
         </is>
       </c>
       <c r="D315" t="n">
-        <v>0.01</v>
+        <v>22</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -17742,36 +17742,36 @@
         <v>0</v>
       </c>
       <c r="I315" t="n">
-        <v>-34022300000</v>
+        <v>680646000</v>
       </c>
       <c r="J315" t="n">
         <v>0</v>
       </c>
       <c r="K315" t="n">
-        <v>0</v>
+        <v>11.74</v>
       </c>
       <c r="L315" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="M315" t="n">
-        <v>0</v>
+        <v>11.63</v>
       </c>
       <c r="N315" t="n">
-        <v>0</v>
+        <v>1.84</v>
       </c>
       <c r="O315" t="n">
-        <v>252.65</v>
+        <v>15.37</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>ALBA3</t>
+          <t>VSPT3</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Empresa ALBA</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -17780,7 +17780,7 @@
         </is>
       </c>
       <c r="D316" t="n">
-        <v>2.15</v>
+        <v>0</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -17797,45 +17797,45 @@
         <v>0</v>
       </c>
       <c r="I316" t="n">
-        <v>354860000</v>
+        <v>5031600000</v>
       </c>
       <c r="J316" t="n">
         <v>0</v>
       </c>
       <c r="K316" t="n">
-        <v>9.5</v>
+        <v>0</v>
       </c>
       <c r="L316" t="n">
-        <v>9.619999999999999</v>
+        <v>0</v>
       </c>
       <c r="M316" t="n">
-        <v>20.4</v>
+        <v>0</v>
       </c>
       <c r="N316" t="n">
-        <v>19.77</v>
+        <v>0</v>
       </c>
       <c r="O316" t="n">
-        <v>14.69</v>
+        <v>4.92</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>VNET3</t>
+          <t>SGEN4</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Empresa VNET</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D317" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -17846,51 +17846,51 @@
         <v>0</v>
       </c>
       <c r="G317" t="n">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="H317" t="n">
         <v>0</v>
       </c>
       <c r="I317" t="n">
-        <v>14163000000</v>
+        <v>156981000</v>
       </c>
       <c r="J317" t="n">
         <v>0</v>
       </c>
       <c r="K317" t="n">
-        <v>0</v>
+        <v>-1871.17</v>
       </c>
       <c r="L317" t="n">
         <v>0</v>
       </c>
       <c r="M317" t="n">
-        <v>0</v>
+        <v>-1.59</v>
       </c>
       <c r="N317" t="n">
         <v>0</v>
       </c>
       <c r="O317" t="n">
-        <v>1.08</v>
+        <v>-59.85</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>CSPC4</t>
+          <t>SEBB3</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -17907,45 +17907,45 @@
         <v>0</v>
       </c>
       <c r="I318" t="n">
-        <v>2126670000</v>
+        <v>145783000</v>
       </c>
       <c r="J318" t="n">
         <v>0</v>
       </c>
       <c r="K318" t="n">
-        <v>38.62</v>
+        <v>9.24</v>
       </c>
       <c r="L318" t="n">
-        <v>18.85</v>
+        <v>7.4</v>
       </c>
       <c r="M318" t="n">
-        <v>29.18</v>
+        <v>24.15</v>
       </c>
       <c r="N318" t="n">
-        <v>45.33</v>
+        <v>23.01</v>
       </c>
       <c r="O318" t="n">
-        <v>41.15</v>
+        <v>50.04</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>BOVH3</t>
+          <t>BBTG11</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Empresa BOVH</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>15.71</v>
+        <v>15.01</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -17956,13 +17956,13 @@
         <v>0</v>
       </c>
       <c r="G319" t="n">
-        <v>6.16</v>
+        <v>0</v>
       </c>
       <c r="H319" t="n">
         <v>0</v>
       </c>
       <c r="I319" t="n">
-        <v>1843320000</v>
+        <v>0</v>
       </c>
       <c r="J319" t="n">
         <v>0</v>
@@ -17986,21 +17986,21 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>ARND3</t>
+          <t>JFAB4</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Empresa ARND</t>
+          <t>Empresa JFAB</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>0.51</v>
+        <v>0.06</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -18011,16 +18011,16 @@
         <v>0</v>
       </c>
       <c r="G320" t="n">
-        <v>0.57</v>
+        <v>0</v>
       </c>
       <c r="H320" t="n">
         <v>0</v>
       </c>
       <c r="I320" t="n">
-        <v>125211000</v>
+        <v>-10183000</v>
       </c>
       <c r="J320" t="n">
-        <v>913.58</v>
+        <v>0</v>
       </c>
       <c r="K320" t="n">
         <v>0</v>
@@ -18032,30 +18032,30 @@
         <v>0</v>
       </c>
       <c r="N320" t="n">
-        <v>0</v>
+        <v>2.34</v>
       </c>
       <c r="O320" t="n">
-        <v>-0.88</v>
+        <v>0</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>VVAX3</t>
+          <t>CCHI4</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -18066,51 +18066,51 @@
         <v>0</v>
       </c>
       <c r="G321" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="H321" t="n">
         <v>0</v>
       </c>
       <c r="I321" t="n">
-        <v>144676000</v>
+        <v>-160477000</v>
       </c>
       <c r="J321" t="n">
         <v>0</v>
       </c>
       <c r="K321" t="n">
-        <v>-7.36</v>
+        <v>0</v>
       </c>
       <c r="L321" t="n">
-        <v>-37.76</v>
+        <v>0</v>
       </c>
       <c r="M321" t="n">
-        <v>-6.52</v>
+        <v>0</v>
       </c>
       <c r="N321" t="n">
-        <v>-92.03</v>
+        <v>0</v>
       </c>
       <c r="O321" t="n">
-        <v>0</v>
+        <v>20.36</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>MSAN4</t>
+          <t>REPA3</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>6.44</v>
+        <v>1</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -18127,36 +18127,36 @@
         <v>0</v>
       </c>
       <c r="I322" t="n">
-        <v>2533030000</v>
+        <v>378378000</v>
       </c>
       <c r="J322" t="n">
         <v>0</v>
       </c>
       <c r="K322" t="n">
-        <v>6.27</v>
+        <v>5.18</v>
       </c>
       <c r="L322" t="n">
-        <v>2.42</v>
+        <v>1.22</v>
       </c>
       <c r="M322" t="n">
-        <v>11.78</v>
+        <v>4.05</v>
       </c>
       <c r="N322" t="n">
-        <v>11.81</v>
+        <v>1.91</v>
       </c>
       <c r="O322" t="n">
-        <v>101.35</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>GALO4</t>
+          <t>EQMA5B</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -18165,7 +18165,7 @@
         </is>
       </c>
       <c r="D323" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -18182,36 +18182,36 @@
         <v>0</v>
       </c>
       <c r="I323" t="n">
-        <v>-60607000</v>
+        <v>4940330000</v>
       </c>
       <c r="J323" t="n">
         <v>0</v>
       </c>
       <c r="K323" t="n">
-        <v>13.98</v>
+        <v>0</v>
       </c>
       <c r="L323" t="n">
-        <v>-184.58</v>
+        <v>0</v>
       </c>
       <c r="M323" t="n">
-        <v>39.37</v>
+        <v>0</v>
       </c>
       <c r="N323" t="n">
-        <v>7.62</v>
+        <v>0</v>
       </c>
       <c r="O323" t="n">
-        <v>-28.97</v>
+        <v>9.050000000000001</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>BBTG13</t>
+          <t>VGOR3</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa VGOR</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -18237,36 +18237,36 @@
         <v>0</v>
       </c>
       <c r="I324" t="n">
-        <v>7000</v>
+        <v>135178000</v>
       </c>
       <c r="J324" t="n">
         <v>0</v>
       </c>
       <c r="K324" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="L324" t="n">
-        <v>0</v>
+        <v>-4.59</v>
       </c>
       <c r="M324" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N324" t="n">
-        <v>-42.86</v>
+        <v>-24.29</v>
       </c>
       <c r="O324" t="n">
-        <v>0</v>
+        <v>4.77</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>INHA3</t>
+          <t>GPIV33</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Empresa INHA</t>
+          <t>Empresa GPIV</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -18275,7 +18275,7 @@
         </is>
       </c>
       <c r="D325" t="n">
-        <v>0</v>
+        <v>4.42</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -18286,42 +18286,42 @@
         <v>0</v>
       </c>
       <c r="G325" t="n">
-        <v>0</v>
+        <v>0.23</v>
       </c>
       <c r="H325" t="n">
         <v>0</v>
       </c>
       <c r="I325" t="n">
-        <v>1533210000</v>
+        <v>1318490000</v>
       </c>
       <c r="J325" t="n">
         <v>0</v>
       </c>
       <c r="K325" t="n">
-        <v>-56.05</v>
+        <v>257.32</v>
       </c>
       <c r="L325" t="n">
-        <v>-124.06</v>
+        <v>0</v>
       </c>
       <c r="M325" t="n">
-        <v>-6.27</v>
+        <v>-6.05</v>
       </c>
       <c r="N325" t="n">
-        <v>-39.87</v>
+        <v>0</v>
       </c>
       <c r="O325" t="n">
-        <v>-12.18</v>
+        <v>-40.99</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>PTIP4</t>
+          <t>ECIS4</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -18330,7 +18330,7 @@
         </is>
       </c>
       <c r="D326" t="n">
-        <v>25.15</v>
+        <v>145</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -18347,36 +18347,36 @@
         <v>0</v>
       </c>
       <c r="I326" t="n">
-        <v>-155957000</v>
+        <v>129346000</v>
       </c>
       <c r="J326" t="n">
         <v>0</v>
       </c>
       <c r="K326" t="n">
-        <v>13.73</v>
+        <v>34.9</v>
       </c>
       <c r="L326" t="n">
-        <v>7.55</v>
+        <v>14.18</v>
       </c>
       <c r="M326" t="n">
-        <v>23.13</v>
+        <v>12.48</v>
       </c>
       <c r="N326" t="n">
-        <v>-121.74</v>
+        <v>7.33</v>
       </c>
       <c r="O326" t="n">
-        <v>62.11</v>
+        <v>4.66</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>LATS3</t>
+          <t>TNEP3</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Empresa LATS</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -18385,7 +18385,7 @@
         </is>
       </c>
       <c r="D327" t="n">
-        <v>22</v>
+        <v>3.01</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -18402,36 +18402,36 @@
         <v>0</v>
       </c>
       <c r="I327" t="n">
-        <v>680646000</v>
+        <v>955105000</v>
       </c>
       <c r="J327" t="n">
         <v>0</v>
       </c>
       <c r="K327" t="n">
-        <v>11.74</v>
+        <v>20.92</v>
       </c>
       <c r="L327" t="n">
-        <v>1.3</v>
+        <v>25.42</v>
       </c>
       <c r="M327" t="n">
-        <v>11.63</v>
+        <v>20.53</v>
       </c>
       <c r="N327" t="n">
-        <v>1.84</v>
+        <v>22.8</v>
       </c>
       <c r="O327" t="n">
-        <v>15.37</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>VSPT3</t>
+          <t>LECO3</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa LECO</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -18457,36 +18457,36 @@
         <v>0</v>
       </c>
       <c r="I328" t="n">
-        <v>5031600000</v>
+        <v>105928000</v>
       </c>
       <c r="J328" t="n">
         <v>0</v>
       </c>
       <c r="K328" t="n">
-        <v>0</v>
+        <v>-2.14</v>
       </c>
       <c r="L328" t="n">
-        <v>0</v>
+        <v>-4.72</v>
       </c>
       <c r="M328" t="n">
-        <v>0</v>
+        <v>-3.48</v>
       </c>
       <c r="N328" t="n">
-        <v>0</v>
+        <v>-14.82</v>
       </c>
       <c r="O328" t="n">
-        <v>4.92</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>SGEN4</t>
+          <t>SALM4</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -18495,7 +18495,7 @@
         </is>
       </c>
       <c r="D329" t="n">
-        <v>0.6</v>
+        <v>5.9</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -18506,42 +18506,42 @@
         <v>0</v>
       </c>
       <c r="G329" t="n">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="H329" t="n">
         <v>0</v>
       </c>
       <c r="I329" t="n">
-        <v>156981000</v>
+        <v>475600000</v>
       </c>
       <c r="J329" t="n">
         <v>0</v>
       </c>
       <c r="K329" t="n">
-        <v>-1871.17</v>
+        <v>10.22</v>
       </c>
       <c r="L329" t="n">
-        <v>0</v>
+        <v>4.13</v>
       </c>
       <c r="M329" t="n">
-        <v>-1.59</v>
+        <v>25.78</v>
       </c>
       <c r="N329" t="n">
-        <v>0</v>
+        <v>19.53</v>
       </c>
       <c r="O329" t="n">
-        <v>-59.85</v>
+        <v>24.53</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>SEBB3</t>
+          <t>BERG3</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa BERG</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -18550,7 +18550,7 @@
         </is>
       </c>
       <c r="D330" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -18567,45 +18567,45 @@
         <v>0</v>
       </c>
       <c r="I330" t="n">
-        <v>145783000</v>
+        <v>9538000</v>
       </c>
       <c r="J330" t="n">
         <v>0</v>
       </c>
       <c r="K330" t="n">
-        <v>9.24</v>
+        <v>-8.6</v>
       </c>
       <c r="L330" t="n">
-        <v>7.4</v>
+        <v>-32.6</v>
       </c>
       <c r="M330" t="n">
-        <v>24.15</v>
+        <v>-5.58</v>
       </c>
       <c r="N330" t="n">
-        <v>23.01</v>
+        <v>-102.71</v>
       </c>
       <c r="O330" t="n">
-        <v>50.04</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>BBTG11</t>
+          <t>JBDU3</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa JBDU</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>15.01</v>
+        <v>0</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -18622,7 +18622,7 @@
         <v>0</v>
       </c>
       <c r="I331" t="n">
-        <v>0</v>
+        <v>56569000</v>
       </c>
       <c r="J331" t="n">
         <v>0</v>
@@ -18646,21 +18646,21 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>JFAB4</t>
+          <t>EGGY3</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Empresa JFAB</t>
+          <t>Empresa EGGY</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -18677,7 +18677,7 @@
         <v>0</v>
       </c>
       <c r="I332" t="n">
-        <v>-10183000</v>
+        <v>954480000</v>
       </c>
       <c r="J332" t="n">
         <v>0</v>
@@ -18692,21 +18692,21 @@
         <v>0</v>
       </c>
       <c r="N332" t="n">
-        <v>2.34</v>
+        <v>0</v>
       </c>
       <c r="O332" t="n">
-        <v>0</v>
+        <v>-0.82</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>CCHI4</t>
+          <t>CBMA4</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -18715,7 +18715,7 @@
         </is>
       </c>
       <c r="D333" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -18726,13 +18726,13 @@
         <v>0</v>
       </c>
       <c r="G333" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="H333" t="n">
         <v>0</v>
       </c>
       <c r="I333" t="n">
-        <v>-160477000</v>
+        <v>-34022300000</v>
       </c>
       <c r="J333" t="n">
         <v>0</v>
@@ -18750,18 +18750,18 @@
         <v>0</v>
       </c>
       <c r="O333" t="n">
-        <v>20.36</v>
+        <v>252.65</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>REPA3</t>
+          <t>SASG3</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa SASG</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -18770,7 +18770,7 @@
         </is>
       </c>
       <c r="D334" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -18787,45 +18787,45 @@
         <v>0</v>
       </c>
       <c r="I334" t="n">
-        <v>378378000</v>
+        <v>0</v>
       </c>
       <c r="J334" t="n">
         <v>0</v>
       </c>
       <c r="K334" t="n">
-        <v>5.18</v>
+        <v>0</v>
       </c>
       <c r="L334" t="n">
-        <v>1.22</v>
+        <v>0</v>
       </c>
       <c r="M334" t="n">
-        <v>4.05</v>
+        <v>0</v>
       </c>
       <c r="N334" t="n">
-        <v>1.91</v>
+        <v>0</v>
       </c>
       <c r="O334" t="n">
-        <v>1.09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>EQMA5B</t>
+          <t>BMEF3</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa BMEF</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -18836,13 +18836,13 @@
         <v>0</v>
       </c>
       <c r="G335" t="n">
-        <v>0</v>
+        <v>4.16</v>
       </c>
       <c r="H335" t="n">
         <v>0</v>
       </c>
       <c r="I335" t="n">
-        <v>4940330000</v>
+        <v>2674780000</v>
       </c>
       <c r="J335" t="n">
         <v>0</v>
@@ -18860,18 +18860,18 @@
         <v>0</v>
       </c>
       <c r="O335" t="n">
-        <v>9.050000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>VGOR3</t>
+          <t>AGEI3</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Empresa VGOR</t>
+          <t>Empresa AGEI</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -18880,7 +18880,7 @@
         </is>
       </c>
       <c r="D336" t="n">
-        <v>0</v>
+        <v>7.8</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -18891,42 +18891,42 @@
         <v>0</v>
       </c>
       <c r="G336" t="n">
-        <v>0</v>
+        <v>1.25</v>
       </c>
       <c r="H336" t="n">
         <v>0</v>
       </c>
       <c r="I336" t="n">
-        <v>135178000</v>
+        <v>1878210000</v>
       </c>
       <c r="J336" t="n">
         <v>0</v>
       </c>
       <c r="K336" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="L336" t="n">
-        <v>-4.59</v>
+        <v>0</v>
       </c>
       <c r="M336" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N336" t="n">
-        <v>-24.29</v>
+        <v>0</v>
       </c>
       <c r="O336" t="n">
-        <v>4.77</v>
+        <v>0</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>GPIV33</t>
+          <t>ARPS3</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Empresa GPIV</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -18935,7 +18935,7 @@
         </is>
       </c>
       <c r="D337" t="n">
-        <v>4.42</v>
+        <v>0.3</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -18946,51 +18946,51 @@
         <v>0</v>
       </c>
       <c r="G337" t="n">
-        <v>0.23</v>
+        <v>0</v>
       </c>
       <c r="H337" t="n">
         <v>0</v>
       </c>
       <c r="I337" t="n">
-        <v>1318490000</v>
+        <v>-12690000</v>
       </c>
       <c r="J337" t="n">
         <v>0</v>
       </c>
       <c r="K337" t="n">
-        <v>257.32</v>
+        <v>-4.92</v>
       </c>
       <c r="L337" t="n">
-        <v>0</v>
+        <v>-11.59</v>
       </c>
       <c r="M337" t="n">
-        <v>-6.05</v>
+        <v>-6.64</v>
       </c>
       <c r="N337" t="n">
-        <v>0</v>
+        <v>20.34</v>
       </c>
       <c r="O337" t="n">
-        <v>-40.99</v>
+        <v>-17.53</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>ECIS4</t>
+          <t>ODER3</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa ODER</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>145</v>
+        <v>0</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -19007,45 +19007,45 @@
         <v>0</v>
       </c>
       <c r="I338" t="n">
-        <v>129346000</v>
+        <v>609518000</v>
       </c>
       <c r="J338" t="n">
         <v>0</v>
       </c>
       <c r="K338" t="n">
-        <v>34.9</v>
+        <v>0</v>
       </c>
       <c r="L338" t="n">
-        <v>14.18</v>
+        <v>0</v>
       </c>
       <c r="M338" t="n">
-        <v>12.48</v>
+        <v>0</v>
       </c>
       <c r="N338" t="n">
-        <v>7.33</v>
+        <v>0</v>
       </c>
       <c r="O338" t="n">
-        <v>4.66</v>
+        <v>3.17</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>TNEP3</t>
+          <t>VVAX4</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>3.01</v>
+        <v>0</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -19062,36 +19062,36 @@
         <v>0</v>
       </c>
       <c r="I339" t="n">
-        <v>955105000</v>
+        <v>144676000</v>
       </c>
       <c r="J339" t="n">
         <v>0</v>
       </c>
       <c r="K339" t="n">
-        <v>20.92</v>
+        <v>-7.36</v>
       </c>
       <c r="L339" t="n">
-        <v>25.42</v>
+        <v>-37.76</v>
       </c>
       <c r="M339" t="n">
-        <v>20.53</v>
+        <v>-6.52</v>
       </c>
       <c r="N339" t="n">
-        <v>22.8</v>
+        <v>-92.03</v>
       </c>
       <c r="O339" t="n">
-        <v>8.15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>LECO3</t>
+          <t>CSPC3</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Empresa LECO</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -19100,7 +19100,7 @@
         </is>
       </c>
       <c r="D340" t="n">
-        <v>0</v>
+        <v>1.24</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -19117,49 +19117,49 @@
         <v>0</v>
       </c>
       <c r="I340" t="n">
-        <v>105928000</v>
+        <v>2126670000</v>
       </c>
       <c r="J340" t="n">
         <v>0</v>
       </c>
       <c r="K340" t="n">
-        <v>-2.14</v>
+        <v>38.62</v>
       </c>
       <c r="L340" t="n">
-        <v>-4.72</v>
+        <v>18.85</v>
       </c>
       <c r="M340" t="n">
-        <v>-3.48</v>
+        <v>29.18</v>
       </c>
       <c r="N340" t="n">
-        <v>-14.82</v>
+        <v>45.33</v>
       </c>
       <c r="O340" t="n">
-        <v>3.58</v>
+        <v>41.15</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>SALM4</t>
+          <t>ABCB3</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa ABCB</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>5.9</v>
+        <v>0</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="F341" t="n">
@@ -19172,36 +19172,36 @@
         <v>0</v>
       </c>
       <c r="I341" t="n">
-        <v>475600000</v>
+        <v>7258910000</v>
       </c>
       <c r="J341" t="n">
         <v>0</v>
       </c>
       <c r="K341" t="n">
-        <v>10.22</v>
+        <v>0</v>
       </c>
       <c r="L341" t="n">
-        <v>4.13</v>
+        <v>0</v>
       </c>
       <c r="M341" t="n">
-        <v>25.78</v>
+        <v>0</v>
       </c>
       <c r="N341" t="n">
-        <v>19.53</v>
+        <v>14.05</v>
       </c>
       <c r="O341" t="n">
-        <v>24.53</v>
+        <v>7.57</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>BERG3</t>
+          <t>CCTY3</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Empresa BERG</t>
+          <t>Empresa CCTY</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -19210,7 +19210,7 @@
         </is>
       </c>
       <c r="D342" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -19227,41 +19227,41 @@
         <v>0</v>
       </c>
       <c r="I342" t="n">
-        <v>9538000</v>
+        <v>0</v>
       </c>
       <c r="J342" t="n">
         <v>0</v>
       </c>
       <c r="K342" t="n">
-        <v>-8.6</v>
+        <v>0</v>
       </c>
       <c r="L342" t="n">
-        <v>-32.6</v>
+        <v>0</v>
       </c>
       <c r="M342" t="n">
-        <v>-5.58</v>
+        <v>0</v>
       </c>
       <c r="N342" t="n">
-        <v>-102.71</v>
+        <v>0</v>
       </c>
       <c r="O342" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>JBDU3</t>
+          <t>ESTC4</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Empresa JBDU</t>
+          <t>Empresa ESTC</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D343" t="n">
@@ -19282,41 +19282,41 @@
         <v>0</v>
       </c>
       <c r="I343" t="n">
-        <v>56569000</v>
+        <v>2916530000</v>
       </c>
       <c r="J343" t="n">
         <v>0</v>
       </c>
       <c r="K343" t="n">
-        <v>0</v>
+        <v>16.91</v>
       </c>
       <c r="L343" t="n">
-        <v>0</v>
+        <v>2.02</v>
       </c>
       <c r="M343" t="n">
-        <v>0</v>
+        <v>11.35</v>
       </c>
       <c r="N343" t="n">
-        <v>0</v>
+        <v>3.89</v>
       </c>
       <c r="O343" t="n">
-        <v>0</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>EGGY3</t>
+          <t>VSPT4</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Empresa EGGY</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D344" t="n">
@@ -19337,7 +19337,7 @@
         <v>0</v>
       </c>
       <c r="I344" t="n">
-        <v>954480000</v>
+        <v>5031600000</v>
       </c>
       <c r="J344" t="n">
         <v>0</v>
@@ -19355,18 +19355,18 @@
         <v>0</v>
       </c>
       <c r="O344" t="n">
-        <v>-0.82</v>
+        <v>4.92</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>CBMA4</t>
+          <t>BAUH4</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa BAUH</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -19375,7 +19375,7 @@
         </is>
       </c>
       <c r="D345" t="n">
-        <v>0.01</v>
+        <v>93.39</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -19386,16 +19386,16 @@
         <v>0</v>
       </c>
       <c r="G345" t="n">
-        <v>0</v>
+        <v>3.18</v>
       </c>
       <c r="H345" t="n">
-        <v>0</v>
+        <v>1.16</v>
       </c>
       <c r="I345" t="n">
-        <v>-34022300000</v>
+        <v>153407000</v>
       </c>
       <c r="J345" t="n">
-        <v>0</v>
+        <v>207.53</v>
       </c>
       <c r="K345" t="n">
         <v>0</v>
@@ -19410,18 +19410,18 @@
         <v>0</v>
       </c>
       <c r="O345" t="n">
-        <v>252.65</v>
+        <v>13.32</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>SASG3</t>
+          <t>ICPI3</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Empresa SASG</t>
+          <t>Empresa ICPI</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
@@ -19430,7 +19430,7 @@
         </is>
       </c>
       <c r="D346" t="n">
-        <v>0.98</v>
+        <v>0</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -19471,21 +19471,21 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>BMEF3</t>
+          <t>ILLS4</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Empresa BMEF</t>
+          <t>Empresa ILLS</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>11</v>
+        <v>100.01</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -19496,42 +19496,42 @@
         <v>0</v>
       </c>
       <c r="G347" t="n">
-        <v>4.16</v>
+        <v>0</v>
       </c>
       <c r="H347" t="n">
         <v>0</v>
       </c>
       <c r="I347" t="n">
-        <v>2674780000</v>
+        <v>-18567000</v>
       </c>
       <c r="J347" t="n">
         <v>0</v>
       </c>
       <c r="K347" t="n">
-        <v>0</v>
+        <v>8.43</v>
       </c>
       <c r="L347" t="n">
-        <v>0</v>
+        <v>-10.22</v>
       </c>
       <c r="M347" t="n">
-        <v>0</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="N347" t="n">
-        <v>0</v>
+        <v>36.09</v>
       </c>
       <c r="O347" t="n">
-        <v>0</v>
+        <v>9.33</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>AGEI3</t>
+          <t>BPAT33</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Empresa AGEI</t>
+          <t>Empresa BPAT</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
@@ -19540,7 +19540,7 @@
         </is>
       </c>
       <c r="D348" t="n">
-        <v>7.8</v>
+        <v>20</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -19551,13 +19551,13 @@
         <v>0</v>
       </c>
       <c r="G348" t="n">
-        <v>1.25</v>
+        <v>0.82</v>
       </c>
       <c r="H348" t="n">
-        <v>0</v>
+        <v>35.72</v>
       </c>
       <c r="I348" t="n">
-        <v>1878210000</v>
+        <v>876492000</v>
       </c>
       <c r="J348" t="n">
         <v>0</v>
@@ -19581,21 +19581,21 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>ARPS3</t>
+          <t>SEBB4</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -19612,36 +19612,36 @@
         <v>0</v>
       </c>
       <c r="I349" t="n">
-        <v>-12690000</v>
+        <v>145783000</v>
       </c>
       <c r="J349" t="n">
         <v>0</v>
       </c>
       <c r="K349" t="n">
-        <v>-4.92</v>
+        <v>9.24</v>
       </c>
       <c r="L349" t="n">
-        <v>-11.59</v>
+        <v>7.4</v>
       </c>
       <c r="M349" t="n">
-        <v>-6.64</v>
+        <v>24.15</v>
       </c>
       <c r="N349" t="n">
-        <v>20.34</v>
+        <v>23.01</v>
       </c>
       <c r="O349" t="n">
-        <v>-17.53</v>
+        <v>50.04</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>ODER3</t>
+          <t>MSAN3</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Empresa ODER</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
@@ -19650,7 +19650,7 @@
         </is>
       </c>
       <c r="D350" t="n">
-        <v>0</v>
+        <v>6.44</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -19667,41 +19667,41 @@
         <v>0</v>
       </c>
       <c r="I350" t="n">
-        <v>609518000</v>
+        <v>2533030000</v>
       </c>
       <c r="J350" t="n">
         <v>0</v>
       </c>
       <c r="K350" t="n">
-        <v>0</v>
+        <v>6.27</v>
       </c>
       <c r="L350" t="n">
-        <v>0</v>
+        <v>2.42</v>
       </c>
       <c r="M350" t="n">
-        <v>0</v>
+        <v>11.78</v>
       </c>
       <c r="N350" t="n">
-        <v>0</v>
+        <v>11.81</v>
       </c>
       <c r="O350" t="n">
-        <v>3.17</v>
+        <v>101.35</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>VVAX4</t>
+          <t>GALO3</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D351" t="n">
@@ -19722,36 +19722,36 @@
         <v>0</v>
       </c>
       <c r="I351" t="n">
-        <v>144676000</v>
+        <v>-60607000</v>
       </c>
       <c r="J351" t="n">
         <v>0</v>
       </c>
       <c r="K351" t="n">
-        <v>-7.36</v>
+        <v>13.98</v>
       </c>
       <c r="L351" t="n">
-        <v>-37.76</v>
+        <v>-184.58</v>
       </c>
       <c r="M351" t="n">
-        <v>-6.52</v>
+        <v>39.37</v>
       </c>
       <c r="N351" t="n">
-        <v>-92.03</v>
+        <v>7.62</v>
       </c>
       <c r="O351" t="n">
-        <v>0</v>
+        <v>-28.97</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>CSPC3</t>
+          <t>SLCP3</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa SLCP</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -19760,7 +19760,7 @@
         </is>
       </c>
       <c r="D352" t="n">
-        <v>1.24</v>
+        <v>610.02</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -19777,36 +19777,36 @@
         <v>0</v>
       </c>
       <c r="I352" t="n">
-        <v>2126670000</v>
+        <v>0</v>
       </c>
       <c r="J352" t="n">
         <v>0</v>
       </c>
       <c r="K352" t="n">
-        <v>38.62</v>
+        <v>0</v>
       </c>
       <c r="L352" t="n">
-        <v>18.85</v>
+        <v>0</v>
       </c>
       <c r="M352" t="n">
-        <v>29.18</v>
+        <v>0</v>
       </c>
       <c r="N352" t="n">
-        <v>45.33</v>
+        <v>0</v>
       </c>
       <c r="O352" t="n">
-        <v>41.15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>ABCB3</t>
+          <t>DAYC3</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Empresa ABCB</t>
+          <t>Empresa DAYC</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -19819,7 +19819,7 @@
       </c>
       <c r="E353" t="inlineStr">
         <is>
-          <t>Bancos</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="F353" t="n">
@@ -19832,7 +19832,7 @@
         <v>0</v>
       </c>
       <c r="I353" t="n">
-        <v>7258910000</v>
+        <v>3009030000</v>
       </c>
       <c r="J353" t="n">
         <v>0</v>
@@ -19847,21 +19847,21 @@
         <v>0</v>
       </c>
       <c r="N353" t="n">
-        <v>14.05</v>
+        <v>17.33</v>
       </c>
       <c r="O353" t="n">
-        <v>7.57</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>CCTY3</t>
+          <t>PTIP3</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Empresa CCTY</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -19870,7 +19870,7 @@
         </is>
       </c>
       <c r="D354" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="E354" t="inlineStr">
         <is>
@@ -19887,36 +19887,36 @@
         <v>0</v>
       </c>
       <c r="I354" t="n">
-        <v>0</v>
+        <v>-155957000</v>
       </c>
       <c r="J354" t="n">
         <v>0</v>
       </c>
       <c r="K354" t="n">
-        <v>0</v>
+        <v>13.73</v>
       </c>
       <c r="L354" t="n">
-        <v>0</v>
+        <v>7.55</v>
       </c>
       <c r="M354" t="n">
-        <v>0</v>
+        <v>23.13</v>
       </c>
       <c r="N354" t="n">
-        <v>0</v>
+        <v>-121.74</v>
       </c>
       <c r="O354" t="n">
-        <v>0</v>
+        <v>62.11</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>ESTC4</t>
+          <t>REPA4</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Empresa ESTC</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -19925,7 +19925,7 @@
         </is>
       </c>
       <c r="D355" t="n">
-        <v>0</v>
+        <v>1.08</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -19942,36 +19942,36 @@
         <v>0</v>
       </c>
       <c r="I355" t="n">
-        <v>2916530000</v>
+        <v>378378000</v>
       </c>
       <c r="J355" t="n">
         <v>0</v>
       </c>
       <c r="K355" t="n">
-        <v>16.91</v>
+        <v>5.18</v>
       </c>
       <c r="L355" t="n">
-        <v>2.02</v>
+        <v>1.22</v>
       </c>
       <c r="M355" t="n">
-        <v>11.35</v>
+        <v>4.05</v>
       </c>
       <c r="N355" t="n">
-        <v>3.89</v>
+        <v>1.91</v>
       </c>
       <c r="O355" t="n">
-        <v>5.6</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>VSPT4</t>
+          <t>EQMA6B</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -19997,7 +19997,7 @@
         <v>0</v>
       </c>
       <c r="I356" t="n">
-        <v>5031600000</v>
+        <v>4940330000</v>
       </c>
       <c r="J356" t="n">
         <v>0</v>
@@ -20015,27 +20015,27 @@
         <v>0</v>
       </c>
       <c r="O356" t="n">
-        <v>4.92</v>
+        <v>9.050000000000001</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>BAUH4</t>
+          <t>MLPA3</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Empresa BAUH</t>
+          <t>Empresa MLPA</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D357" t="n">
-        <v>93.39</v>
+        <v>0</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -20046,47 +20046,47 @@
         <v>0</v>
       </c>
       <c r="G357" t="n">
-        <v>3.18</v>
+        <v>0</v>
       </c>
       <c r="H357" t="n">
-        <v>1.16</v>
+        <v>0</v>
       </c>
       <c r="I357" t="n">
-        <v>153407000</v>
+        <v>44578000</v>
       </c>
       <c r="J357" t="n">
-        <v>207.53</v>
+        <v>0</v>
       </c>
       <c r="K357" t="n">
-        <v>0</v>
+        <v>6.66</v>
       </c>
       <c r="L357" t="n">
-        <v>0</v>
+        <v>8.92</v>
       </c>
       <c r="M357" t="n">
         <v>0</v>
       </c>
       <c r="N357" t="n">
-        <v>0</v>
+        <v>45.13</v>
       </c>
       <c r="O357" t="n">
-        <v>13.32</v>
+        <v>-7.51</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>ICPI3</t>
+          <t>CLSC6</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Empresa ICPI</t>
+          <t>Empresa CLSC</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D358" t="n">
@@ -20107,7 +20107,7 @@
         <v>0</v>
       </c>
       <c r="I358" t="n">
-        <v>0</v>
+        <v>4228180000</v>
       </c>
       <c r="J358" t="n">
         <v>0</v>
@@ -20125,27 +20125,27 @@
         <v>0</v>
       </c>
       <c r="O358" t="n">
-        <v>0</v>
+        <v>2.82</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>ILLS4</t>
+          <t>SGEN3</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Empresa ILLS</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>100.01</v>
+        <v>5</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -20156,51 +20156,51 @@
         <v>0</v>
       </c>
       <c r="G359" t="n">
-        <v>0</v>
+        <v>0.77</v>
       </c>
       <c r="H359" t="n">
         <v>0</v>
       </c>
       <c r="I359" t="n">
-        <v>-18567000</v>
+        <v>156981000</v>
       </c>
       <c r="J359" t="n">
         <v>0</v>
       </c>
       <c r="K359" t="n">
-        <v>8.43</v>
+        <v>-1871.17</v>
       </c>
       <c r="L359" t="n">
-        <v>-10.22</v>
+        <v>0</v>
       </c>
       <c r="M359" t="n">
-        <v>8.140000000000001</v>
+        <v>-1.59</v>
       </c>
       <c r="N359" t="n">
-        <v>36.09</v>
+        <v>0</v>
       </c>
       <c r="O359" t="n">
-        <v>9.33</v>
+        <v>-59.85</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>BPAT33</t>
+          <t>DUFB11</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Empresa BPAT</t>
+          <t>Empresa DUFB</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -20211,13 +20211,13 @@
         <v>0</v>
       </c>
       <c r="G360" t="n">
-        <v>0.82</v>
+        <v>0</v>
       </c>
       <c r="H360" t="n">
-        <v>35.72</v>
+        <v>0</v>
       </c>
       <c r="I360" t="n">
-        <v>876492000</v>
+        <v>0</v>
       </c>
       <c r="J360" t="n">
         <v>0</v>
@@ -20241,12 +20241,12 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>SEBB4</t>
+          <t>TNEP4</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -20255,7 +20255,7 @@
         </is>
       </c>
       <c r="D361" t="n">
-        <v>0</v>
+        <v>3.95</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -20272,36 +20272,36 @@
         <v>0</v>
       </c>
       <c r="I361" t="n">
-        <v>145783000</v>
+        <v>955105000</v>
       </c>
       <c r="J361" t="n">
         <v>0</v>
       </c>
       <c r="K361" t="n">
-        <v>9.24</v>
+        <v>20.92</v>
       </c>
       <c r="L361" t="n">
-        <v>7.4</v>
+        <v>25.42</v>
       </c>
       <c r="M361" t="n">
-        <v>24.15</v>
+        <v>20.53</v>
       </c>
       <c r="N361" t="n">
-        <v>23.01</v>
+        <v>22.8</v>
       </c>
       <c r="O361" t="n">
-        <v>50.04</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>MSAN3</t>
+          <t>CCHI3</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -20310,7 +20310,7 @@
         </is>
       </c>
       <c r="D362" t="n">
-        <v>6.44</v>
+        <v>0.02</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -20321,42 +20321,42 @@
         <v>0</v>
       </c>
       <c r="G362" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="H362" t="n">
         <v>0</v>
       </c>
       <c r="I362" t="n">
-        <v>2533030000</v>
+        <v>-160477000</v>
       </c>
       <c r="J362" t="n">
         <v>0</v>
       </c>
       <c r="K362" t="n">
-        <v>6.27</v>
+        <v>0</v>
       </c>
       <c r="L362" t="n">
-        <v>2.42</v>
+        <v>0</v>
       </c>
       <c r="M362" t="n">
-        <v>11.78</v>
+        <v>0</v>
       </c>
       <c r="N362" t="n">
-        <v>11.81</v>
+        <v>0</v>
       </c>
       <c r="O362" t="n">
-        <v>101.35</v>
+        <v>20.36</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>GALO3</t>
+          <t>SFSA3</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa SFSA</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -20382,36 +20382,36 @@
         <v>0</v>
       </c>
       <c r="I363" t="n">
-        <v>-60607000</v>
+        <v>739524000</v>
       </c>
       <c r="J363" t="n">
         <v>0</v>
       </c>
       <c r="K363" t="n">
-        <v>13.98</v>
+        <v>0</v>
       </c>
       <c r="L363" t="n">
-        <v>-184.58</v>
+        <v>0</v>
       </c>
       <c r="M363" t="n">
-        <v>39.37</v>
+        <v>0</v>
       </c>
       <c r="N363" t="n">
-        <v>7.62</v>
+        <v>6.25</v>
       </c>
       <c r="O363" t="n">
-        <v>-28.97</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>SLCP3</t>
+          <t>PRBC3</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Empresa SLCP</t>
+          <t>Empresa PRBC</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -20420,7 +20420,7 @@
         </is>
       </c>
       <c r="D364" t="n">
-        <v>610.02</v>
+        <v>0</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -20437,7 +20437,7 @@
         <v>0</v>
       </c>
       <c r="I364" t="n">
-        <v>0</v>
+        <v>1319270000</v>
       </c>
       <c r="J364" t="n">
         <v>0</v>
@@ -20452,21 +20452,21 @@
         <v>0</v>
       </c>
       <c r="N364" t="n">
-        <v>0</v>
+        <v>8.27</v>
       </c>
       <c r="O364" t="n">
-        <v>0</v>
+        <v>-1.98</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>DAYC3</t>
+          <t>ECIS3</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Empresa DAYC</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
@@ -20475,7 +20475,7 @@
         </is>
       </c>
       <c r="D365" t="n">
-        <v>0</v>
+        <v>211.65</v>
       </c>
       <c r="E365" t="inlineStr">
         <is>
@@ -20492,45 +20492,45 @@
         <v>0</v>
       </c>
       <c r="I365" t="n">
-        <v>3009030000</v>
+        <v>129346000</v>
       </c>
       <c r="J365" t="n">
         <v>0</v>
       </c>
       <c r="K365" t="n">
-        <v>0</v>
+        <v>34.9</v>
       </c>
       <c r="L365" t="n">
-        <v>0</v>
+        <v>14.18</v>
       </c>
       <c r="M365" t="n">
-        <v>0</v>
+        <v>12.48</v>
       </c>
       <c r="N365" t="n">
-        <v>17.33</v>
+        <v>7.33</v>
       </c>
       <c r="O365" t="n">
-        <v>8.15</v>
+        <v>4.66</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>PTIP3</t>
+          <t>ARPS4</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D366" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="E366" t="inlineStr">
         <is>
@@ -20547,45 +20547,45 @@
         <v>0</v>
       </c>
       <c r="I366" t="n">
-        <v>-155957000</v>
+        <v>-12690000</v>
       </c>
       <c r="J366" t="n">
         <v>0</v>
       </c>
       <c r="K366" t="n">
-        <v>13.73</v>
+        <v>-4.92</v>
       </c>
       <c r="L366" t="n">
-        <v>7.55</v>
+        <v>-11.59</v>
       </c>
       <c r="M366" t="n">
-        <v>23.13</v>
+        <v>-6.64</v>
       </c>
       <c r="N366" t="n">
-        <v>-121.74</v>
+        <v>20.34</v>
       </c>
       <c r="O366" t="n">
-        <v>62.11</v>
+        <v>-17.53</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>REPA4</t>
+          <t>SALM3</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D367" t="n">
-        <v>1.08</v>
+        <v>5.7</v>
       </c>
       <c r="E367" t="inlineStr">
         <is>
@@ -20602,36 +20602,36 @@
         <v>0</v>
       </c>
       <c r="I367" t="n">
-        <v>378378000</v>
+        <v>475600000</v>
       </c>
       <c r="J367" t="n">
         <v>0</v>
       </c>
       <c r="K367" t="n">
-        <v>5.18</v>
+        <v>10.22</v>
       </c>
       <c r="L367" t="n">
-        <v>1.22</v>
+        <v>4.13</v>
       </c>
       <c r="M367" t="n">
-        <v>4.05</v>
+        <v>25.78</v>
       </c>
       <c r="N367" t="n">
-        <v>1.91</v>
+        <v>19.53</v>
       </c>
       <c r="O367" t="n">
-        <v>1.09</v>
+        <v>24.53</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>EQMA6B</t>
+          <t>CMMA4</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa CMMA</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -20640,7 +20640,7 @@
         </is>
       </c>
       <c r="D368" t="n">
-        <v>0</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E368" t="inlineStr">
         <is>
@@ -20657,7 +20657,7 @@
         <v>0</v>
       </c>
       <c r="I368" t="n">
-        <v>4940330000</v>
+        <v>-79623000</v>
       </c>
       <c r="J368" t="n">
         <v>0</v>
@@ -20672,21 +20672,21 @@
         <v>0</v>
       </c>
       <c r="N368" t="n">
-        <v>0</v>
+        <v>-1.92</v>
       </c>
       <c r="O368" t="n">
-        <v>9.050000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>MLPA3</t>
+          <t>CZRS3</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Empresa MLPA</t>
+          <t>Empresa CZRS</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -20712,41 +20712,41 @@
         <v>0</v>
       </c>
       <c r="I369" t="n">
-        <v>44578000</v>
+        <v>1145670000</v>
       </c>
       <c r="J369" t="n">
         <v>0</v>
       </c>
       <c r="K369" t="n">
-        <v>6.66</v>
+        <v>0</v>
       </c>
       <c r="L369" t="n">
-        <v>8.92</v>
+        <v>0</v>
       </c>
       <c r="M369" t="n">
         <v>0</v>
       </c>
       <c r="N369" t="n">
-        <v>45.13</v>
+        <v>3.34</v>
       </c>
       <c r="O369" t="n">
-        <v>-7.51</v>
+        <v>14.44</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>CLSC6</t>
+          <t>BPNM3</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Empresa CLSC</t>
+          <t>Empresa BPNM</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D370" t="n">
@@ -20767,7 +20767,7 @@
         <v>0</v>
       </c>
       <c r="I370" t="n">
-        <v>4228180000</v>
+        <v>7792670000</v>
       </c>
       <c r="J370" t="n">
         <v>0</v>
@@ -20782,21 +20782,21 @@
         <v>0</v>
       </c>
       <c r="N370" t="n">
-        <v>0</v>
+        <v>9.67</v>
       </c>
       <c r="O370" t="n">
-        <v>2.82</v>
+        <v>-1.53</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>SGEN3</t>
+          <t>BSGR3</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa BSGR</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
@@ -20805,7 +20805,7 @@
         </is>
       </c>
       <c r="D371" t="n">
-        <v>5</v>
+        <v>1091.28</v>
       </c>
       <c r="E371" t="inlineStr">
         <is>
@@ -20816,51 +20816,51 @@
         <v>0</v>
       </c>
       <c r="G371" t="n">
-        <v>0.77</v>
+        <v>0</v>
       </c>
       <c r="H371" t="n">
         <v>0</v>
       </c>
       <c r="I371" t="n">
-        <v>156981000</v>
+        <v>0</v>
       </c>
       <c r="J371" t="n">
         <v>0</v>
       </c>
       <c r="K371" t="n">
-        <v>-1871.17</v>
+        <v>0</v>
       </c>
       <c r="L371" t="n">
         <v>0</v>
       </c>
       <c r="M371" t="n">
-        <v>-1.59</v>
+        <v>0</v>
       </c>
       <c r="N371" t="n">
         <v>0</v>
       </c>
       <c r="O371" t="n">
-        <v>-59.85</v>
+        <v>0</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>DUFB11</t>
+          <t>CBMA3</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Empresa DUFB</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D372" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="E372" t="inlineStr">
         <is>
@@ -20877,7 +20877,7 @@
         <v>0</v>
       </c>
       <c r="I372" t="n">
-        <v>0</v>
+        <v>-34022300000</v>
       </c>
       <c r="J372" t="n">
         <v>0</v>
@@ -20895,27 +20895,27 @@
         <v>0</v>
       </c>
       <c r="O372" t="n">
-        <v>0</v>
+        <v>252.65</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>TNEP4</t>
+          <t>ALBA3</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa ALBA</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D373" t="n">
-        <v>3.95</v>
+        <v>2.15</v>
       </c>
       <c r="E373" t="inlineStr">
         <is>
@@ -20932,36 +20932,36 @@
         <v>0</v>
       </c>
       <c r="I373" t="n">
-        <v>955105000</v>
+        <v>354860000</v>
       </c>
       <c r="J373" t="n">
         <v>0</v>
       </c>
       <c r="K373" t="n">
-        <v>20.92</v>
+        <v>9.5</v>
       </c>
       <c r="L373" t="n">
-        <v>25.42</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="M373" t="n">
-        <v>20.53</v>
+        <v>20.4</v>
       </c>
       <c r="N373" t="n">
-        <v>22.8</v>
+        <v>19.77</v>
       </c>
       <c r="O373" t="n">
-        <v>8.15</v>
+        <v>14.69</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>CCHI3</t>
+          <t>VNET3</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa VNET</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
@@ -20970,7 +20970,7 @@
         </is>
       </c>
       <c r="D374" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="E374" t="inlineStr">
         <is>
@@ -20981,13 +20981,13 @@
         <v>0</v>
       </c>
       <c r="G374" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="H374" t="n">
         <v>0</v>
       </c>
       <c r="I374" t="n">
-        <v>-160477000</v>
+        <v>14163000000</v>
       </c>
       <c r="J374" t="n">
         <v>0</v>
@@ -21005,27 +21005,27 @@
         <v>0</v>
       </c>
       <c r="O374" t="n">
-        <v>20.36</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>SFSA3</t>
+          <t>CSPC4</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>Empresa SFSA</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D375" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="E375" t="inlineStr">
         <is>
@@ -21042,36 +21042,36 @@
         <v>0</v>
       </c>
       <c r="I375" t="n">
-        <v>739524000</v>
+        <v>2126670000</v>
       </c>
       <c r="J375" t="n">
         <v>0</v>
       </c>
       <c r="K375" t="n">
-        <v>0</v>
+        <v>38.62</v>
       </c>
       <c r="L375" t="n">
-        <v>0</v>
+        <v>18.85</v>
       </c>
       <c r="M375" t="n">
-        <v>0</v>
+        <v>29.18</v>
       </c>
       <c r="N375" t="n">
-        <v>6.25</v>
+        <v>45.33</v>
       </c>
       <c r="O375" t="n">
-        <v>0.15</v>
+        <v>41.15</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>PRBC3</t>
+          <t>BOVH3</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>Empresa PRBC</t>
+          <t>Empresa BOVH</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
@@ -21080,7 +21080,7 @@
         </is>
       </c>
       <c r="D376" t="n">
-        <v>0</v>
+        <v>15.71</v>
       </c>
       <c r="E376" t="inlineStr">
         <is>
@@ -21091,13 +21091,13 @@
         <v>0</v>
       </c>
       <c r="G376" t="n">
-        <v>0</v>
+        <v>6.16</v>
       </c>
       <c r="H376" t="n">
         <v>0</v>
       </c>
       <c r="I376" t="n">
-        <v>1319270000</v>
+        <v>1843320000</v>
       </c>
       <c r="J376" t="n">
         <v>0</v>
@@ -21112,21 +21112,21 @@
         <v>0</v>
       </c>
       <c r="N376" t="n">
-        <v>8.27</v>
+        <v>0</v>
       </c>
       <c r="O376" t="n">
-        <v>-1.98</v>
+        <v>0</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>ECIS3</t>
+          <t>ARND3</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa ARND</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
@@ -21135,7 +21135,7 @@
         </is>
       </c>
       <c r="D377" t="n">
-        <v>211.65</v>
+        <v>0.51</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -21146,31 +21146,31 @@
         <v>0</v>
       </c>
       <c r="G377" t="n">
-        <v>0</v>
+        <v>0.57</v>
       </c>
       <c r="H377" t="n">
         <v>0</v>
       </c>
       <c r="I377" t="n">
-        <v>129346000</v>
+        <v>125211000</v>
       </c>
       <c r="J377" t="n">
-        <v>0</v>
+        <v>913.58</v>
       </c>
       <c r="K377" t="n">
-        <v>34.9</v>
+        <v>0</v>
       </c>
       <c r="L377" t="n">
-        <v>14.18</v>
+        <v>0</v>
       </c>
       <c r="M377" t="n">
-        <v>12.48</v>
+        <v>0</v>
       </c>
       <c r="N377" t="n">
-        <v>7.33</v>
+        <v>0</v>
       </c>
       <c r="O377" t="n">
-        <v>4.66</v>
+        <v>-0.88</v>
       </c>
     </row>
     <row r="378">
@@ -22349,7 +22349,7 @@
       </c>
       <c r="E399" t="inlineStr">
         <is>
-          <t>Varejo e Comércio</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F399" t="n">
@@ -24164,7 +24164,7 @@
       </c>
       <c r="E432" t="inlineStr">
         <is>
-          <t>Shoppings e Imóveis</t>
+          <t>Exploração de Imóveis</t>
         </is>
       </c>
       <c r="F432" t="n">
@@ -24696,7 +24696,7 @@
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>MMAQ4</t>
+          <t>MMAQ3</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
@@ -24706,7 +24706,7 @@
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D442" t="n">
@@ -24724,7 +24724,7 @@
         <v>0.36</v>
       </c>
       <c r="H442" t="n">
-        <v>41.68</v>
+        <v>0</v>
       </c>
       <c r="I442" t="n">
         <v>259016000</v>
@@ -24751,7 +24751,7 @@
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>MMAQ3</t>
+          <t>MMAQ4</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
@@ -24761,7 +24761,7 @@
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D443" t="n">
@@ -24779,7 +24779,7 @@
         <v>0.36</v>
       </c>
       <c r="H443" t="n">
-        <v>0</v>
+        <v>41.68</v>
       </c>
       <c r="I443" t="n">
         <v>259016000</v>
@@ -26749,7 +26749,7 @@
       </c>
       <c r="E479" t="inlineStr">
         <is>
-          <t>Saúde e Farmácia</t>
+          <t>Serviços Médico-Hospitalares</t>
         </is>
       </c>
       <c r="F479" t="n">
@@ -27134,7 +27134,7 @@
       </c>
       <c r="E486" t="inlineStr">
         <is>
-          <t>Varejo e Comércio</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F486" t="n">
@@ -27244,7 +27244,7 @@
       </c>
       <c r="E488" t="inlineStr">
         <is>
-          <t>Petróleo e Gás</t>
+          <t>Petróleo, Gás e Biocombustíveis</t>
         </is>
       </c>
       <c r="F488" t="n">
@@ -28234,7 +28234,7 @@
       </c>
       <c r="E506" t="inlineStr">
         <is>
-          <t>Varejo e Comércio</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F506" t="n">
@@ -28399,7 +28399,7 @@
       </c>
       <c r="E509" t="inlineStr">
         <is>
-          <t>Petróleo e Gás</t>
+          <t>Petróleo, Gás e Biocombustíveis</t>
         </is>
       </c>
       <c r="F509" t="n">
@@ -28564,7 +28564,7 @@
       </c>
       <c r="E512" t="inlineStr">
         <is>
-          <t>Varejo e Comércio</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F512" t="n">
@@ -29554,7 +29554,7 @@
       </c>
       <c r="E530" t="inlineStr">
         <is>
-          <t>Shoppings e Imóveis</t>
+          <t>Exploração de Imóveis</t>
         </is>
       </c>
       <c r="F530" t="n">
@@ -29664,7 +29664,7 @@
       </c>
       <c r="E532" t="inlineStr">
         <is>
-          <t>Agro e Alimentos</t>
+          <t>Alimentos Processados</t>
         </is>
       </c>
       <c r="F532" t="n">
@@ -30324,7 +30324,7 @@
       </c>
       <c r="E544" t="inlineStr">
         <is>
-          <t>Varejo e Comércio</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F544" t="n">
@@ -30764,7 +30764,7 @@
       </c>
       <c r="E552" t="inlineStr">
         <is>
-          <t>Varejo e Comércio</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F552" t="n">
@@ -31149,7 +31149,7 @@
       </c>
       <c r="E559" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Exploração de Imóveis</t>
         </is>
       </c>
       <c r="F559" t="n">
@@ -31204,7 +31204,7 @@
       </c>
       <c r="E560" t="inlineStr">
         <is>
-          <t>Seguradoras</t>
+          <t>Previdência e Seguros</t>
         </is>
       </c>
       <c r="F560" t="n">
@@ -31259,7 +31259,7 @@
       </c>
       <c r="E561" t="inlineStr">
         <is>
-          <t>Petróleo e Gás</t>
+          <t>Petróleo, Gás e Biocombustíveis</t>
         </is>
       </c>
       <c r="F561" t="n">
@@ -31699,7 +31699,7 @@
       </c>
       <c r="E569" t="inlineStr">
         <is>
-          <t>Varejo e Comércio</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F569" t="n">
@@ -32946,7 +32946,7 @@
     <row r="592">
       <c r="A592" t="inlineStr">
         <is>
-          <t>GETT4</t>
+          <t>GETT3</t>
         </is>
       </c>
       <c r="B592" t="inlineStr">
@@ -32956,7 +32956,7 @@
       </c>
       <c r="C592" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D592" t="n">
@@ -33001,7 +33001,7 @@
     <row r="593">
       <c r="A593" t="inlineStr">
         <is>
-          <t>GETT3</t>
+          <t>GETT4</t>
         </is>
       </c>
       <c r="B593" t="inlineStr">
@@ -33011,7 +33011,7 @@
       </c>
       <c r="C593" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D593" t="n">
@@ -33239,7 +33239,7 @@
       </c>
       <c r="E597" t="inlineStr">
         <is>
-          <t>Varejo e Comércio</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F597" t="n">
@@ -33661,7 +33661,7 @@
     <row r="605">
       <c r="A605" t="inlineStr">
         <is>
-          <t>RPAD6</t>
+          <t>RPAD3</t>
         </is>
       </c>
       <c r="B605" t="inlineStr">
@@ -33671,7 +33671,7 @@
       </c>
       <c r="C605" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D605" t="n">
@@ -33689,13 +33689,13 @@
         <v>0.57</v>
       </c>
       <c r="H605" t="n">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="I605" t="n">
         <v>1046150000</v>
       </c>
       <c r="J605" t="n">
-        <v>2752.22</v>
+        <v>2695.56</v>
       </c>
       <c r="K605" t="n">
         <v>0</v>
@@ -33716,7 +33716,7 @@
     <row r="606">
       <c r="A606" t="inlineStr">
         <is>
-          <t>RPAD3</t>
+          <t>RPAD6</t>
         </is>
       </c>
       <c r="B606" t="inlineStr">
@@ -33726,7 +33726,7 @@
       </c>
       <c r="C606" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D606" t="n">
@@ -33744,13 +33744,13 @@
         <v>0.57</v>
       </c>
       <c r="H606" t="n">
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="I606" t="n">
         <v>1046150000</v>
       </c>
       <c r="J606" t="n">
-        <v>2695.56</v>
+        <v>2752.22</v>
       </c>
       <c r="K606" t="n">
         <v>0</v>
@@ -34064,7 +34064,7 @@
       </c>
       <c r="E612" t="inlineStr">
         <is>
-          <t>Tecnologia</t>
+          <t>Tecnologia da Informação</t>
         </is>
       </c>
       <c r="F612" t="n">
@@ -34559,7 +34559,7 @@
       </c>
       <c r="E621" t="inlineStr">
         <is>
-          <t>Agro e Alimentos</t>
+          <t>Agropecuária</t>
         </is>
       </c>
       <c r="F621" t="n">
@@ -34944,7 +34944,7 @@
       </c>
       <c r="E628" t="inlineStr">
         <is>
-          <t>Agro e Alimentos</t>
+          <t>Alimentos Processados</t>
         </is>
       </c>
       <c r="F628" t="n">
@@ -35439,7 +35439,7 @@
       </c>
       <c r="E637" t="inlineStr">
         <is>
-          <t>Petróleo e Gás</t>
+          <t>Petróleo, Gás e Biocombustíveis</t>
         </is>
       </c>
       <c r="F637" t="n">
@@ -35494,7 +35494,7 @@
       </c>
       <c r="E638" t="inlineStr">
         <is>
-          <t>Petróleo e Gás</t>
+          <t>Petróleo, Gás e Biocombustíveis</t>
         </is>
       </c>
       <c r="F638" t="n">
@@ -35769,7 +35769,7 @@
       </c>
       <c r="E643" t="inlineStr">
         <is>
-          <t>Serviços Financeiros</t>
+          <t>Serviços Financeiros Diversos</t>
         </is>
       </c>
       <c r="F643" t="n">
@@ -35879,7 +35879,7 @@
       </c>
       <c r="E645" t="inlineStr">
         <is>
-          <t>Seguradoras</t>
+          <t>Previdência e Seguros</t>
         </is>
       </c>
       <c r="F645" t="n">
@@ -36319,7 +36319,7 @@
       </c>
       <c r="E653" t="inlineStr">
         <is>
-          <t>Seguradoras</t>
+          <t>Previdência e Seguros</t>
         </is>
       </c>
       <c r="F653" t="n">
@@ -36649,7 +36649,7 @@
       </c>
       <c r="E659" t="inlineStr">
         <is>
-          <t>Agro e Alimentos</t>
+          <t>Alimentos Processados</t>
         </is>
       </c>
       <c r="F659" t="n">
@@ -36814,7 +36814,7 @@
       </c>
       <c r="E662" t="inlineStr">
         <is>
-          <t>Saúde e Farmácia</t>
+          <t>Medicamentos</t>
         </is>
       </c>
       <c r="F662" t="n">
@@ -37199,7 +37199,7 @@
       </c>
       <c r="E669" t="inlineStr">
         <is>
-          <t>Agro e Alimentos</t>
+          <t>Agropecuária</t>
         </is>
       </c>
       <c r="F669" t="n">
@@ -37309,7 +37309,7 @@
       </c>
       <c r="E671" t="inlineStr">
         <is>
-          <t>Saúde e Farmácia</t>
+          <t>Medicamentos</t>
         </is>
       </c>
       <c r="F671" t="n">
@@ -37584,7 +37584,7 @@
       </c>
       <c r="E676" t="inlineStr">
         <is>
-          <t>Varejo e Comércio</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F676" t="n">
@@ -37804,7 +37804,7 @@
       </c>
       <c r="E680" t="inlineStr">
         <is>
-          <t>Varejo e Comércio</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F680" t="n">
@@ -38409,7 +38409,7 @@
       </c>
       <c r="E691" t="inlineStr">
         <is>
-          <t>Shoppings e Imóveis</t>
+          <t>Exploração de Imóveis</t>
         </is>
       </c>
       <c r="F691" t="n">
@@ -39124,7 +39124,7 @@
       </c>
       <c r="E704" t="inlineStr">
         <is>
-          <t>Shoppings e Imóveis</t>
+          <t>Exploração de Imóveis</t>
         </is>
       </c>
       <c r="F704" t="n">
@@ -39344,7 +39344,7 @@
       </c>
       <c r="E708" t="inlineStr">
         <is>
-          <t>Shoppings e Imóveis</t>
+          <t>Exploração de Imóveis</t>
         </is>
       </c>
       <c r="F708" t="n">
@@ -39399,7 +39399,7 @@
       </c>
       <c r="E709" t="inlineStr">
         <is>
-          <t>Agro e Alimentos</t>
+          <t>Alimentos Processados</t>
         </is>
       </c>
       <c r="F709" t="n">
@@ -39839,7 +39839,7 @@
       </c>
       <c r="E717" t="inlineStr">
         <is>
-          <t>Saneamento</t>
+          <t>Água e Saneamento</t>
         </is>
       </c>
       <c r="F717" t="n">
@@ -40444,7 +40444,7 @@
       </c>
       <c r="E728" t="inlineStr">
         <is>
-          <t>Petróleo e Gás</t>
+          <t>Petróleo, Gás e Biocombustíveis</t>
         </is>
       </c>
       <c r="F728" t="n">
@@ -40554,7 +40554,7 @@
       </c>
       <c r="E730" t="inlineStr">
         <is>
-          <t>Saúde e Farmácia</t>
+          <t>Serviços Médico-Hospitalares</t>
         </is>
       </c>
       <c r="F730" t="n">
@@ -40774,7 +40774,7 @@
       </c>
       <c r="E734" t="inlineStr">
         <is>
-          <t>Shoppings e Imóveis</t>
+          <t>Exploração de Imóveis</t>
         </is>
       </c>
       <c r="F734" t="n">
@@ -41214,7 +41214,7 @@
       </c>
       <c r="E742" t="inlineStr">
         <is>
-          <t>Varejo e Comércio</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F742" t="n">
@@ -41489,7 +41489,7 @@
       </c>
       <c r="E747" t="inlineStr">
         <is>
-          <t>Mineração e Siderurgia</t>
+          <t>Mineração</t>
         </is>
       </c>
       <c r="F747" t="n">
@@ -41929,7 +41929,7 @@
       </c>
       <c r="E755" t="inlineStr">
         <is>
-          <t>Varejo e Comércio</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F755" t="n">
@@ -42039,7 +42039,7 @@
       </c>
       <c r="E757" t="inlineStr">
         <is>
-          <t>Seguradoras</t>
+          <t>Previdência e Seguros</t>
         </is>
       </c>
       <c r="F757" t="n">
@@ -42149,7 +42149,7 @@
       </c>
       <c r="E759" t="inlineStr">
         <is>
-          <t>Mineração e Siderurgia</t>
+          <t>Siderurgia e Metalurgia</t>
         </is>
       </c>
       <c r="F759" t="n">
@@ -42314,7 +42314,7 @@
       </c>
       <c r="E762" t="inlineStr">
         <is>
-          <t>Petróleo e Gás</t>
+          <t>Petróleo, Gás e Biocombustíveis</t>
         </is>
       </c>
       <c r="F762" t="n">
@@ -42479,7 +42479,7 @@
       </c>
       <c r="E765" t="inlineStr">
         <is>
-          <t>Petróleo e Gás</t>
+          <t>Petróleo, Gás e Biocombustíveis</t>
         </is>
       </c>
       <c r="F765" t="n">
@@ -42974,7 +42974,7 @@
       </c>
       <c r="E774" t="inlineStr">
         <is>
-          <t>Tecnologia</t>
+          <t>Tecnologia da Informação</t>
         </is>
       </c>
       <c r="F774" t="n">
@@ -43139,7 +43139,7 @@
       </c>
       <c r="E777" t="inlineStr">
         <is>
-          <t>Mineração e Siderurgia</t>
+          <t>Mineração</t>
         </is>
       </c>
       <c r="F777" t="n">
@@ -43249,7 +43249,7 @@
       </c>
       <c r="E779" t="inlineStr">
         <is>
-          <t>Saúde e Farmácia</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F779" t="n">
@@ -43799,7 +43799,7 @@
       </c>
       <c r="E789" t="inlineStr">
         <is>
-          <t>Varejo e Comércio</t>
+          <t>Bebidas</t>
         </is>
       </c>
       <c r="F789" t="n">
@@ -44074,7 +44074,7 @@
       </c>
       <c r="E794" t="inlineStr">
         <is>
-          <t>Mineração e Siderurgia</t>
+          <t>Mineração</t>
         </is>
       </c>
       <c r="F794" t="n">
@@ -44294,7 +44294,7 @@
       </c>
       <c r="E798" t="inlineStr">
         <is>
-          <t>Mineração e Siderurgia</t>
+          <t>Mineração</t>
         </is>
       </c>
       <c r="F798" t="n">
@@ -44349,7 +44349,7 @@
       </c>
       <c r="E799" t="inlineStr">
         <is>
-          <t>Shoppings e Imóveis</t>
+          <t>Exploração de Imóveis</t>
         </is>
       </c>
       <c r="F799" t="n">
@@ -44404,7 +44404,7 @@
       </c>
       <c r="E800" t="inlineStr">
         <is>
-          <t>Saúde e Farmácia</t>
+          <t>Serviços Médico-Hospitalares</t>
         </is>
       </c>
       <c r="F800" t="n">
@@ -44459,7 +44459,7 @@
       </c>
       <c r="E801" t="inlineStr">
         <is>
-          <t>Agro e Alimentos</t>
+          <t>Alimentos Processados</t>
         </is>
       </c>
       <c r="F801" t="n">
@@ -44844,7 +44844,7 @@
       </c>
       <c r="E808" t="inlineStr">
         <is>
-          <t>Saúde e Farmácia</t>
+          <t>Serviços Médico-Hospitalares</t>
         </is>
       </c>
       <c r="F808" t="n">
@@ -45009,7 +45009,7 @@
       </c>
       <c r="E811" t="inlineStr">
         <is>
-          <t>Saneamento</t>
+          <t>Água e Saneamento</t>
         </is>
       </c>
       <c r="F811" t="n">
@@ -45064,7 +45064,7 @@
       </c>
       <c r="E812" t="inlineStr">
         <is>
-          <t>Serviços Financeiros</t>
+          <t>Serviços Financeiros Diversos</t>
         </is>
       </c>
       <c r="F812" t="n">
@@ -45174,7 +45174,7 @@
       </c>
       <c r="E814" t="inlineStr">
         <is>
-          <t>Mineração e Siderurgia</t>
+          <t>Siderurgia e Metalurgia</t>
         </is>
       </c>
       <c r="F814" t="n">
@@ -45614,7 +45614,7 @@
       </c>
       <c r="E822" t="inlineStr">
         <is>
-          <t>Saúde e Farmácia</t>
+          <t>Serviços Médico-Hospitalares</t>
         </is>
       </c>
       <c r="F822" t="n">
@@ -46054,7 +46054,7 @@
       </c>
       <c r="E830" t="inlineStr">
         <is>
-          <t>Mineração e Siderurgia</t>
+          <t>Siderurgia e Metalurgia</t>
         </is>
       </c>
       <c r="F830" t="n">
@@ -46329,7 +46329,7 @@
       </c>
       <c r="E835" t="inlineStr">
         <is>
-          <t>Mineração e Siderurgia</t>
+          <t>Siderurgia e Metalurgia</t>
         </is>
       </c>
       <c r="F835" t="n">
@@ -46824,7 +46824,7 @@
       </c>
       <c r="E844" t="inlineStr">
         <is>
-          <t>Saúde e Farmácia</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F844" t="n">
@@ -47209,7 +47209,7 @@
       </c>
       <c r="E851" t="inlineStr">
         <is>
-          <t>Agro e Alimentos</t>
+          <t>Agropecuária</t>
         </is>
       </c>
       <c r="F851" t="n">
@@ -47814,7 +47814,7 @@
       </c>
       <c r="E862" t="inlineStr">
         <is>
-          <t>Mineração e Siderurgia</t>
+          <t>Siderurgia e Metalurgia</t>
         </is>
       </c>
       <c r="F862" t="n">
@@ -48034,7 +48034,7 @@
       </c>
       <c r="E866" t="inlineStr">
         <is>
-          <t>Saneamento</t>
+          <t>Água e Saneamento</t>
         </is>
       </c>
       <c r="F866" t="n">
@@ -48144,7 +48144,7 @@
       </c>
       <c r="E868" t="inlineStr">
         <is>
-          <t>Saneamento</t>
+          <t>Água e Saneamento</t>
         </is>
       </c>
       <c r="F868" t="n">
@@ -48694,7 +48694,7 @@
       </c>
       <c r="E878" t="inlineStr">
         <is>
-          <t>Mineração e Siderurgia</t>
+          <t>Siderurgia e Metalurgia</t>
         </is>
       </c>
       <c r="F878" t="n">
@@ -48969,7 +48969,7 @@
       </c>
       <c r="E883" t="inlineStr">
         <is>
-          <t>Saneamento</t>
+          <t>Água e Saneamento</t>
         </is>
       </c>
       <c r="F883" t="n">
@@ -49079,7 +49079,7 @@
       </c>
       <c r="E885" t="inlineStr">
         <is>
-          <t>Saúde e Farmácia</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F885" t="n">
@@ -50344,7 +50344,7 @@
       </c>
       <c r="E908" t="inlineStr">
         <is>
-          <t>Mineração e Siderurgia</t>
+          <t>Mineração</t>
         </is>
       </c>
       <c r="F908" t="n">
@@ -50729,7 +50729,7 @@
       </c>
       <c r="E915" t="inlineStr">
         <is>
-          <t>Saúde e Farmácia</t>
+          <t>Serviços Médico-Hospitalares</t>
         </is>
       </c>
       <c r="F915" t="n">
@@ -50894,7 +50894,7 @@
       </c>
       <c r="E918" t="inlineStr">
         <is>
-          <t>Tecnologia</t>
+          <t>Tecnologia da Informação</t>
         </is>
       </c>
       <c r="F918" t="n">
@@ -51224,7 +51224,7 @@
       </c>
       <c r="E924" t="inlineStr">
         <is>
-          <t>Varejo e Comércio</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F924" t="n">
@@ -51829,7 +51829,7 @@
       </c>
       <c r="E935" t="inlineStr">
         <is>
-          <t>Agro e Alimentos</t>
+          <t>Agropecuária</t>
         </is>
       </c>
       <c r="F935" t="n">
@@ -51884,7 +51884,7 @@
       </c>
       <c r="E936" t="inlineStr">
         <is>
-          <t>Varejo e Comércio</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F936" t="n">
@@ -51994,7 +51994,7 @@
       </c>
       <c r="E938" t="inlineStr">
         <is>
-          <t>Varejo e Comércio</t>
+          <t>Comércio / Varejo</t>
         </is>
       </c>
       <c r="F938" t="n">
@@ -53039,7 +53039,7 @@
       </c>
       <c r="E957" t="inlineStr">
         <is>
-          <t>Shoppings e Imóveis</t>
+          <t>Exploração de Imóveis</t>
         </is>
       </c>
       <c r="F957" t="n">
@@ -53901,7 +53901,7 @@
     <row r="973">
       <c r="A973" t="inlineStr">
         <is>
-          <t>PQUN3</t>
+          <t>PQUN4</t>
         </is>
       </c>
       <c r="B973" t="inlineStr">
@@ -53911,7 +53911,7 @@
       </c>
       <c r="C973" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D973" t="n">
@@ -53956,7 +53956,7 @@
     <row r="974">
       <c r="A974" t="inlineStr">
         <is>
-          <t>PQUN4</t>
+          <t>PQUN3</t>
         </is>
       </c>
       <c r="B974" t="inlineStr">
@@ -53966,7 +53966,7 @@
       </c>
       <c r="C974" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D974" t="n">
@@ -54359,7 +54359,7 @@
       </c>
       <c r="E981" t="inlineStr">
         <is>
-          <t>Saneamento</t>
+          <t>Água e Saneamento</t>
         </is>
       </c>
       <c r="F981" t="n">

</xml_diff>

<commit_message>
Atualizacao completa dos codigos com tipo de acao e setores oficiais B3
</commit_message>
<xml_diff>
--- a/acoes_b3.xlsx
+++ b/acoes_b3.xlsx
@@ -496,25 +496,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CFLU4</t>
+          <t>MNSA3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Empresa CFLU</t>
+          <t>Empresa MNSA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1000</v>
+        <v>0.42</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Mineração</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -527,45 +527,45 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>60351000</v>
+        <v>-9105000</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>8.880000000000001</v>
+        <v>-208.15</v>
       </c>
       <c r="L2" t="n">
-        <v>10.72</v>
+        <v>-362.66</v>
       </c>
       <c r="M2" t="n">
-        <v>17.68</v>
+        <v>-13.5</v>
       </c>
       <c r="N2" t="n">
-        <v>32.15</v>
+        <v>145.7</v>
       </c>
       <c r="O2" t="n">
-        <v>8.140000000000001</v>
+        <v>-41.11</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CSTB3</t>
+          <t>CFLU4</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa CFLU</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>150</v>
+        <v>1000</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -582,45 +582,45 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>8420670000</v>
+        <v>60351000</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>40.85</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="L3" t="n">
-        <v>28.98</v>
+        <v>10.72</v>
       </c>
       <c r="M3" t="n">
-        <v>22.4</v>
+        <v>17.68</v>
       </c>
       <c r="N3" t="n">
-        <v>20.11</v>
+        <v>32.15</v>
       </c>
       <c r="O3" t="n">
-        <v>31.91</v>
+        <v>8.140000000000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>POPR4</t>
+          <t>CSTB3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Empresa POPR</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>10.17</v>
+        <v>150</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -637,45 +637,45 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>545803000</v>
+        <v>8420670000</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>8.66</v>
+        <v>40.85</v>
       </c>
       <c r="L4" t="n">
-        <v>5.65</v>
+        <v>28.98</v>
       </c>
       <c r="M4" t="n">
-        <v>15.25</v>
+        <v>22.4</v>
       </c>
       <c r="N4" t="n">
-        <v>19.93</v>
+        <v>20.11</v>
       </c>
       <c r="O4" t="n">
-        <v>30.93</v>
+        <v>31.91</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PMET3</t>
+          <t>POPR4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Empresa PMET</t>
+          <t>Empresa POPR</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>10.17</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -692,36 +692,36 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>-290863000</v>
+        <v>545803000</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>8.66</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>5.65</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>15.25</v>
       </c>
       <c r="N5" t="n">
-        <v>4.1</v>
+        <v>19.93</v>
       </c>
       <c r="O5" t="n">
-        <v>37.74</v>
+        <v>30.93</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CLAN3</t>
+          <t>PMET3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Empresa CLAN</t>
+          <t>Empresa PMET</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -747,7 +747,7 @@
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>1012240000</v>
+        <v>-290863000</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -762,34 +762,34 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>-1.05</v>
+        <v>4.1</v>
       </c>
       <c r="O6" t="n">
-        <v>-63.96</v>
+        <v>37.74</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MNSA4</t>
+          <t>CLAN3</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Empresa MNSA</t>
+          <t>Empresa CLAN</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.47</v>
+        <v>0</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Mineração</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -802,36 +802,36 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>-9105000</v>
+        <v>1012240000</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>-208.15</v>
+        <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>-362.66</v>
+        <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>-13.5</v>
+        <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>145.7</v>
+        <v>-1.05</v>
       </c>
       <c r="O7" t="n">
-        <v>-41.11</v>
+        <v>-63.96</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CSTB4</t>
+          <t>MNSA4</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa MNSA</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -840,11 +840,11 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>147.69</v>
+        <v>0.47</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Mineração</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -857,36 +857,36 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>8420670000</v>
+        <v>-9105000</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>40.85</v>
+        <v>-208.15</v>
       </c>
       <c r="L8" t="n">
-        <v>28.98</v>
+        <v>-362.66</v>
       </c>
       <c r="M8" t="n">
-        <v>22.4</v>
+        <v>-13.5</v>
       </c>
       <c r="N8" t="n">
-        <v>20.11</v>
+        <v>145.7</v>
       </c>
       <c r="O8" t="n">
-        <v>31.91</v>
+        <v>-41.11</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PORP4</t>
+          <t>CSTB4</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Empresa PORP</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -895,7 +895,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2.4</v>
+        <v>147.69</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -912,45 +912,45 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>22399000</v>
+        <v>8420670000</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>40.85</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>28.98</v>
       </c>
       <c r="M9" t="n">
-        <v>0</v>
+        <v>22.4</v>
       </c>
       <c r="N9" t="n">
-        <v>-2.08</v>
+        <v>20.11</v>
       </c>
       <c r="O9" t="n">
-        <v>13.66</v>
+        <v>31.91</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>IVTT3</t>
+          <t>PORP4</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Empresa IVTT</t>
+          <t>Empresa PORP</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -967,7 +967,7 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>1083050000</v>
+        <v>22399000</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -982,21 +982,21 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>-0.4</v>
+        <v>-2.08</v>
       </c>
       <c r="O10" t="n">
-        <v>20.67</v>
+        <v>13.66</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MNSA3</t>
+          <t>IVTT3</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Empresa MNSA</t>
+          <t>Empresa IVTT</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1005,11 +1005,11 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.42</v>
+        <v>0</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Mineração</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -1022,25 +1022,25 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>-9105000</v>
+        <v>1083050000</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>-208.15</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>-362.66</v>
+        <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>-13.5</v>
+        <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>145.7</v>
+        <v>-0.4</v>
       </c>
       <c r="O11" t="n">
-        <v>-41.11</v>
+        <v>20.67</v>
       </c>
     </row>
     <row r="12">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -2431,7 +2431,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -4356,7 +4356,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -8811,7 +8811,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -11616,7 +11616,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D204" t="n">
@@ -12661,7 +12661,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D223" t="n">
@@ -13486,7 +13486,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D238" t="n">
@@ -17381,21 +17381,21 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>MLPA3</t>
+          <t>REPA4</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Empresa MLPA</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>0</v>
+        <v>1.08</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -17412,41 +17412,41 @@
         <v>0</v>
       </c>
       <c r="I309" t="n">
-        <v>44578000</v>
+        <v>378378000</v>
       </c>
       <c r="J309" t="n">
         <v>0</v>
       </c>
       <c r="K309" t="n">
-        <v>6.66</v>
+        <v>5.18</v>
       </c>
       <c r="L309" t="n">
-        <v>8.92</v>
+        <v>1.22</v>
       </c>
       <c r="M309" t="n">
-        <v>0</v>
+        <v>4.05</v>
       </c>
       <c r="N309" t="n">
-        <v>45.13</v>
+        <v>1.91</v>
       </c>
       <c r="O309" t="n">
-        <v>-7.51</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>CLSC6</t>
+          <t>EQMA6B</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Empresa CLSC</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -17467,7 +17467,7 @@
         <v>0</v>
       </c>
       <c r="I310" t="n">
-        <v>4228180000</v>
+        <v>4940330000</v>
       </c>
       <c r="J310" t="n">
         <v>0</v>
@@ -17485,27 +17485,27 @@
         <v>0</v>
       </c>
       <c r="O310" t="n">
-        <v>2.82</v>
+        <v>9.050000000000001</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>SGEN3</t>
+          <t>SEBB4</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -17516,51 +17516,51 @@
         <v>0</v>
       </c>
       <c r="G311" t="n">
-        <v>0.77</v>
+        <v>0</v>
       </c>
       <c r="H311" t="n">
         <v>0</v>
       </c>
       <c r="I311" t="n">
-        <v>156981000</v>
+        <v>145783000</v>
       </c>
       <c r="J311" t="n">
         <v>0</v>
       </c>
       <c r="K311" t="n">
-        <v>-1871.17</v>
+        <v>9.24</v>
       </c>
       <c r="L311" t="n">
-        <v>0</v>
+        <v>7.4</v>
       </c>
       <c r="M311" t="n">
-        <v>-1.59</v>
+        <v>24.15</v>
       </c>
       <c r="N311" t="n">
-        <v>0</v>
+        <v>23.01</v>
       </c>
       <c r="O311" t="n">
-        <v>-59.85</v>
+        <v>50.04</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>DUFB11</t>
+          <t>MSAN3</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Empresa DUFB</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>0</v>
+        <v>6.44</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -17577,45 +17577,45 @@
         <v>0</v>
       </c>
       <c r="I312" t="n">
-        <v>0</v>
+        <v>2533030000</v>
       </c>
       <c r="J312" t="n">
         <v>0</v>
       </c>
       <c r="K312" t="n">
-        <v>0</v>
+        <v>6.27</v>
       </c>
       <c r="L312" t="n">
-        <v>0</v>
+        <v>2.42</v>
       </c>
       <c r="M312" t="n">
-        <v>0</v>
+        <v>11.78</v>
       </c>
       <c r="N312" t="n">
-        <v>0</v>
+        <v>11.81</v>
       </c>
       <c r="O312" t="n">
-        <v>0</v>
+        <v>101.35</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>TNEP4</t>
+          <t>GALO3</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>3.95</v>
+        <v>0</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -17632,36 +17632,36 @@
         <v>0</v>
       </c>
       <c r="I313" t="n">
-        <v>955105000</v>
+        <v>-60607000</v>
       </c>
       <c r="J313" t="n">
         <v>0</v>
       </c>
       <c r="K313" t="n">
-        <v>20.92</v>
+        <v>13.98</v>
       </c>
       <c r="L313" t="n">
-        <v>25.42</v>
+        <v>-184.58</v>
       </c>
       <c r="M313" t="n">
-        <v>20.53</v>
+        <v>39.37</v>
       </c>
       <c r="N313" t="n">
-        <v>22.8</v>
+        <v>7.62</v>
       </c>
       <c r="O313" t="n">
-        <v>8.15</v>
+        <v>-28.97</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>CCHI3</t>
+          <t>SLCP3</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa SLCP</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -17670,7 +17670,7 @@
         </is>
       </c>
       <c r="D314" t="n">
-        <v>0.02</v>
+        <v>610.02</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -17681,13 +17681,13 @@
         <v>0</v>
       </c>
       <c r="G314" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="H314" t="n">
         <v>0</v>
       </c>
       <c r="I314" t="n">
-        <v>-160477000</v>
+        <v>0</v>
       </c>
       <c r="J314" t="n">
         <v>0</v>
@@ -17705,18 +17705,18 @@
         <v>0</v>
       </c>
       <c r="O314" t="n">
-        <v>20.36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>SFSA3</t>
+          <t>DAYC3</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Empresa SFSA</t>
+          <t>Empresa DAYC</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -17742,7 +17742,7 @@
         <v>0</v>
       </c>
       <c r="I315" t="n">
-        <v>739524000</v>
+        <v>3009030000</v>
       </c>
       <c r="J315" t="n">
         <v>0</v>
@@ -17757,21 +17757,21 @@
         <v>0</v>
       </c>
       <c r="N315" t="n">
-        <v>6.25</v>
+        <v>17.33</v>
       </c>
       <c r="O315" t="n">
-        <v>0.15</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>PRBC3</t>
+          <t>PTIP3</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Empresa PRBC</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -17780,7 +17780,7 @@
         </is>
       </c>
       <c r="D316" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -17797,36 +17797,36 @@
         <v>0</v>
       </c>
       <c r="I316" t="n">
-        <v>1319270000</v>
+        <v>-155957000</v>
       </c>
       <c r="J316" t="n">
         <v>0</v>
       </c>
       <c r="K316" t="n">
-        <v>0</v>
+        <v>13.73</v>
       </c>
       <c r="L316" t="n">
-        <v>0</v>
+        <v>7.55</v>
       </c>
       <c r="M316" t="n">
-        <v>0</v>
+        <v>23.13</v>
       </c>
       <c r="N316" t="n">
-        <v>8.27</v>
+        <v>-121.74</v>
       </c>
       <c r="O316" t="n">
-        <v>-1.98</v>
+        <v>62.11</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>ECIS3</t>
+          <t>MLPA3</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa MLPA</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -17835,7 +17835,7 @@
         </is>
       </c>
       <c r="D317" t="n">
-        <v>211.65</v>
+        <v>0</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -17852,45 +17852,45 @@
         <v>0</v>
       </c>
       <c r="I317" t="n">
-        <v>129346000</v>
+        <v>44578000</v>
       </c>
       <c r="J317" t="n">
         <v>0</v>
       </c>
       <c r="K317" t="n">
-        <v>34.9</v>
+        <v>6.66</v>
       </c>
       <c r="L317" t="n">
-        <v>14.18</v>
+        <v>8.92</v>
       </c>
       <c r="M317" t="n">
-        <v>12.48</v>
+        <v>0</v>
       </c>
       <c r="N317" t="n">
-        <v>7.33</v>
+        <v>45.13</v>
       </c>
       <c r="O317" t="n">
-        <v>4.66</v>
+        <v>-7.51</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>CBMA3</t>
+          <t>CLSC6</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa CLSC</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -17907,7 +17907,7 @@
         <v>0</v>
       </c>
       <c r="I318" t="n">
-        <v>-34022300000</v>
+        <v>4228180000</v>
       </c>
       <c r="J318" t="n">
         <v>0</v>
@@ -17925,18 +17925,18 @@
         <v>0</v>
       </c>
       <c r="O318" t="n">
-        <v>252.65</v>
+        <v>2.82</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>ALBA3</t>
+          <t>SGEN3</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Empresa ALBA</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -17945,7 +17945,7 @@
         </is>
       </c>
       <c r="D319" t="n">
-        <v>2.15</v>
+        <v>5</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -17956,47 +17956,47 @@
         <v>0</v>
       </c>
       <c r="G319" t="n">
-        <v>0</v>
+        <v>0.77</v>
       </c>
       <c r="H319" t="n">
         <v>0</v>
       </c>
       <c r="I319" t="n">
-        <v>354860000</v>
+        <v>156981000</v>
       </c>
       <c r="J319" t="n">
         <v>0</v>
       </c>
       <c r="K319" t="n">
-        <v>9.5</v>
+        <v>-1871.17</v>
       </c>
       <c r="L319" t="n">
-        <v>9.619999999999999</v>
+        <v>0</v>
       </c>
       <c r="M319" t="n">
-        <v>20.4</v>
+        <v>-1.59</v>
       </c>
       <c r="N319" t="n">
-        <v>19.77</v>
+        <v>0</v>
       </c>
       <c r="O319" t="n">
-        <v>14.69</v>
+        <v>-59.85</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>ARPS4</t>
+          <t>DUFB11</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa DUFB</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D320" t="n">
@@ -18017,45 +18017,45 @@
         <v>0</v>
       </c>
       <c r="I320" t="n">
-        <v>-12690000</v>
+        <v>0</v>
       </c>
       <c r="J320" t="n">
         <v>0</v>
       </c>
       <c r="K320" t="n">
-        <v>-4.92</v>
+        <v>0</v>
       </c>
       <c r="L320" t="n">
-        <v>-11.59</v>
+        <v>0</v>
       </c>
       <c r="M320" t="n">
-        <v>-6.64</v>
+        <v>0</v>
       </c>
       <c r="N320" t="n">
-        <v>20.34</v>
+        <v>0</v>
       </c>
       <c r="O320" t="n">
-        <v>-17.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>SALM3</t>
+          <t>TNEP4</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>5.7</v>
+        <v>3.95</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -18072,45 +18072,45 @@
         <v>0</v>
       </c>
       <c r="I321" t="n">
-        <v>475600000</v>
+        <v>955105000</v>
       </c>
       <c r="J321" t="n">
         <v>0</v>
       </c>
       <c r="K321" t="n">
-        <v>10.22</v>
+        <v>20.92</v>
       </c>
       <c r="L321" t="n">
-        <v>4.13</v>
+        <v>25.42</v>
       </c>
       <c r="M321" t="n">
-        <v>25.78</v>
+        <v>20.53</v>
       </c>
       <c r="N321" t="n">
-        <v>19.53</v>
+        <v>22.8</v>
       </c>
       <c r="O321" t="n">
-        <v>24.53</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>CMMA4</t>
+          <t>CCHI3</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Empresa CMMA</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.02</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -18121,13 +18121,13 @@
         <v>0</v>
       </c>
       <c r="G322" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="H322" t="n">
         <v>0</v>
       </c>
       <c r="I322" t="n">
-        <v>-79623000</v>
+        <v>-160477000</v>
       </c>
       <c r="J322" t="n">
         <v>0</v>
@@ -18142,21 +18142,21 @@
         <v>0</v>
       </c>
       <c r="N322" t="n">
-        <v>-1.92</v>
+        <v>0</v>
       </c>
       <c r="O322" t="n">
-        <v>0</v>
+        <v>20.36</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>CZRS3</t>
+          <t>SFSA3</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Empresa CZRS</t>
+          <t>Empresa SFSA</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -18182,7 +18182,7 @@
         <v>0</v>
       </c>
       <c r="I323" t="n">
-        <v>1145670000</v>
+        <v>739524000</v>
       </c>
       <c r="J323" t="n">
         <v>0</v>
@@ -18197,21 +18197,21 @@
         <v>0</v>
       </c>
       <c r="N323" t="n">
-        <v>3.34</v>
+        <v>6.25</v>
       </c>
       <c r="O323" t="n">
-        <v>14.44</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>BPNM3</t>
+          <t>PRBC3</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Empresa BPNM</t>
+          <t>Empresa PRBC</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -18237,7 +18237,7 @@
         <v>0</v>
       </c>
       <c r="I324" t="n">
-        <v>7792670000</v>
+        <v>1319270000</v>
       </c>
       <c r="J324" t="n">
         <v>0</v>
@@ -18252,21 +18252,21 @@
         <v>0</v>
       </c>
       <c r="N324" t="n">
-        <v>9.67</v>
+        <v>8.27</v>
       </c>
       <c r="O324" t="n">
-        <v>-1.53</v>
+        <v>-1.98</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>BSGR3</t>
+          <t>ECIS3</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Empresa BSGR</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -18275,7 +18275,7 @@
         </is>
       </c>
       <c r="D325" t="n">
-        <v>1091.28</v>
+        <v>211.65</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -18292,36 +18292,36 @@
         <v>0</v>
       </c>
       <c r="I325" t="n">
-        <v>0</v>
+        <v>129346000</v>
       </c>
       <c r="J325" t="n">
         <v>0</v>
       </c>
       <c r="K325" t="n">
-        <v>0</v>
+        <v>34.9</v>
       </c>
       <c r="L325" t="n">
-        <v>0</v>
+        <v>14.18</v>
       </c>
       <c r="M325" t="n">
-        <v>0</v>
+        <v>12.48</v>
       </c>
       <c r="N325" t="n">
-        <v>0</v>
+        <v>7.33</v>
       </c>
       <c r="O325" t="n">
-        <v>0</v>
+        <v>4.66</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>VNET3</t>
+          <t>CBMA3</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Empresa VNET</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -18330,7 +18330,7 @@
         </is>
       </c>
       <c r="D326" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -18347,7 +18347,7 @@
         <v>0</v>
       </c>
       <c r="I326" t="n">
-        <v>14163000000</v>
+        <v>-34022300000</v>
       </c>
       <c r="J326" t="n">
         <v>0</v>
@@ -18365,27 +18365,27 @@
         <v>0</v>
       </c>
       <c r="O326" t="n">
-        <v>1.08</v>
+        <v>252.65</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>CSPC4</t>
+          <t>ALBA3</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa ALBA</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>1.2</v>
+        <v>2.15</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -18402,45 +18402,45 @@
         <v>0</v>
       </c>
       <c r="I327" t="n">
-        <v>2126670000</v>
+        <v>354860000</v>
       </c>
       <c r="J327" t="n">
         <v>0</v>
       </c>
       <c r="K327" t="n">
-        <v>38.62</v>
+        <v>9.5</v>
       </c>
       <c r="L327" t="n">
-        <v>18.85</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="M327" t="n">
-        <v>29.18</v>
+        <v>20.4</v>
       </c>
       <c r="N327" t="n">
-        <v>45.33</v>
+        <v>19.77</v>
       </c>
       <c r="O327" t="n">
-        <v>41.15</v>
+        <v>14.69</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>BOVH3</t>
+          <t>ARPS4</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Empresa BOVH</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>15.71</v>
+        <v>0</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -18451,42 +18451,42 @@
         <v>0</v>
       </c>
       <c r="G328" t="n">
-        <v>6.16</v>
+        <v>0</v>
       </c>
       <c r="H328" t="n">
         <v>0</v>
       </c>
       <c r="I328" t="n">
-        <v>1843320000</v>
+        <v>-12690000</v>
       </c>
       <c r="J328" t="n">
         <v>0</v>
       </c>
       <c r="K328" t="n">
-        <v>0</v>
+        <v>-4.92</v>
       </c>
       <c r="L328" t="n">
-        <v>0</v>
+        <v>-11.59</v>
       </c>
       <c r="M328" t="n">
-        <v>0</v>
+        <v>-6.64</v>
       </c>
       <c r="N328" t="n">
-        <v>0</v>
+        <v>20.34</v>
       </c>
       <c r="O328" t="n">
-        <v>0</v>
+        <v>-17.53</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>ARND3</t>
+          <t>SALM3</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Empresa ARND</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -18495,7 +18495,7 @@
         </is>
       </c>
       <c r="D329" t="n">
-        <v>0.51</v>
+        <v>5.7</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -18506,51 +18506,51 @@
         <v>0</v>
       </c>
       <c r="G329" t="n">
-        <v>0.57</v>
+        <v>0</v>
       </c>
       <c r="H329" t="n">
         <v>0</v>
       </c>
       <c r="I329" t="n">
-        <v>125211000</v>
+        <v>475600000</v>
       </c>
       <c r="J329" t="n">
-        <v>913.58</v>
+        <v>0</v>
       </c>
       <c r="K329" t="n">
-        <v>0</v>
+        <v>10.22</v>
       </c>
       <c r="L329" t="n">
-        <v>0</v>
+        <v>4.13</v>
       </c>
       <c r="M329" t="n">
-        <v>0</v>
+        <v>25.78</v>
       </c>
       <c r="N329" t="n">
-        <v>0</v>
+        <v>19.53</v>
       </c>
       <c r="O329" t="n">
-        <v>-0.88</v>
+        <v>24.53</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>VVAX3</t>
+          <t>CMMA4</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa CMMA</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>0</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -18567,22 +18567,22 @@
         <v>0</v>
       </c>
       <c r="I330" t="n">
-        <v>144676000</v>
+        <v>-79623000</v>
       </c>
       <c r="J330" t="n">
         <v>0</v>
       </c>
       <c r="K330" t="n">
-        <v>-7.36</v>
+        <v>0</v>
       </c>
       <c r="L330" t="n">
-        <v>-37.76</v>
+        <v>0</v>
       </c>
       <c r="M330" t="n">
-        <v>-6.52</v>
+        <v>0</v>
       </c>
       <c r="N330" t="n">
-        <v>-92.03</v>
+        <v>-1.92</v>
       </c>
       <c r="O330" t="n">
         <v>0</v>
@@ -18591,21 +18591,21 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>MSAN4</t>
+          <t>CZRS3</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa CZRS</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>6.44</v>
+        <v>0</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -18622,45 +18622,45 @@
         <v>0</v>
       </c>
       <c r="I331" t="n">
-        <v>2533030000</v>
+        <v>1145670000</v>
       </c>
       <c r="J331" t="n">
         <v>0</v>
       </c>
       <c r="K331" t="n">
-        <v>6.27</v>
+        <v>0</v>
       </c>
       <c r="L331" t="n">
-        <v>2.42</v>
+        <v>0</v>
       </c>
       <c r="M331" t="n">
-        <v>11.78</v>
+        <v>0</v>
       </c>
       <c r="N331" t="n">
-        <v>11.81</v>
+        <v>3.34</v>
       </c>
       <c r="O331" t="n">
-        <v>101.35</v>
+        <v>14.44</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>GALO4</t>
+          <t>BPNM3</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa BPNM</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -18677,36 +18677,36 @@
         <v>0</v>
       </c>
       <c r="I332" t="n">
-        <v>-60607000</v>
+        <v>7792670000</v>
       </c>
       <c r="J332" t="n">
         <v>0</v>
       </c>
       <c r="K332" t="n">
-        <v>13.98</v>
+        <v>0</v>
       </c>
       <c r="L332" t="n">
-        <v>-184.58</v>
+        <v>0</v>
       </c>
       <c r="M332" t="n">
-        <v>39.37</v>
+        <v>0</v>
       </c>
       <c r="N332" t="n">
-        <v>7.62</v>
+        <v>9.67</v>
       </c>
       <c r="O332" t="n">
-        <v>-28.97</v>
+        <v>-1.53</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>BBTG13</t>
+          <t>BSGR3</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa BSGR</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -18715,7 +18715,7 @@
         </is>
       </c>
       <c r="D333" t="n">
-        <v>0</v>
+        <v>1091.28</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -18732,7 +18732,7 @@
         <v>0</v>
       </c>
       <c r="I333" t="n">
-        <v>7000</v>
+        <v>0</v>
       </c>
       <c r="J333" t="n">
         <v>0</v>
@@ -18747,7 +18747,7 @@
         <v>0</v>
       </c>
       <c r="N333" t="n">
-        <v>-42.86</v>
+        <v>0</v>
       </c>
       <c r="O333" t="n">
         <v>0</v>
@@ -18756,12 +18756,12 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>INHA3</t>
+          <t>VNET3</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Empresa INHA</t>
+          <t>Empresa VNET</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -18787,36 +18787,36 @@
         <v>0</v>
       </c>
       <c r="I334" t="n">
-        <v>1533210000</v>
+        <v>14163000000</v>
       </c>
       <c r="J334" t="n">
         <v>0</v>
       </c>
       <c r="K334" t="n">
-        <v>-56.05</v>
+        <v>0</v>
       </c>
       <c r="L334" t="n">
-        <v>-124.06</v>
+        <v>0</v>
       </c>
       <c r="M334" t="n">
-        <v>-6.27</v>
+        <v>0</v>
       </c>
       <c r="N334" t="n">
-        <v>-39.87</v>
+        <v>0</v>
       </c>
       <c r="O334" t="n">
-        <v>-12.18</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>PTIP4</t>
+          <t>CSPC4</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -18825,7 +18825,7 @@
         </is>
       </c>
       <c r="D335" t="n">
-        <v>25.15</v>
+        <v>1.2</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -18842,36 +18842,36 @@
         <v>0</v>
       </c>
       <c r="I335" t="n">
-        <v>-155957000</v>
+        <v>2126670000</v>
       </c>
       <c r="J335" t="n">
         <v>0</v>
       </c>
       <c r="K335" t="n">
-        <v>13.73</v>
+        <v>38.62</v>
       </c>
       <c r="L335" t="n">
-        <v>7.55</v>
+        <v>18.85</v>
       </c>
       <c r="M335" t="n">
-        <v>23.13</v>
+        <v>29.18</v>
       </c>
       <c r="N335" t="n">
-        <v>-121.74</v>
+        <v>45.33</v>
       </c>
       <c r="O335" t="n">
-        <v>62.11</v>
+        <v>41.15</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>LATS3</t>
+          <t>BOVH3</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Empresa LATS</t>
+          <t>Empresa BOVH</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -18880,7 +18880,7 @@
         </is>
       </c>
       <c r="D336" t="n">
-        <v>22</v>
+        <v>15.71</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -18891,42 +18891,42 @@
         <v>0</v>
       </c>
       <c r="G336" t="n">
-        <v>0</v>
+        <v>6.16</v>
       </c>
       <c r="H336" t="n">
         <v>0</v>
       </c>
       <c r="I336" t="n">
-        <v>680646000</v>
+        <v>1843320000</v>
       </c>
       <c r="J336" t="n">
         <v>0</v>
       </c>
       <c r="K336" t="n">
-        <v>11.74</v>
+        <v>0</v>
       </c>
       <c r="L336" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="M336" t="n">
-        <v>11.63</v>
+        <v>0</v>
       </c>
       <c r="N336" t="n">
-        <v>1.84</v>
+        <v>0</v>
       </c>
       <c r="O336" t="n">
-        <v>15.37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>VSPT3</t>
+          <t>ARND3</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa ARND</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -18935,7 +18935,7 @@
         </is>
       </c>
       <c r="D337" t="n">
-        <v>0</v>
+        <v>0.51</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -18946,16 +18946,16 @@
         <v>0</v>
       </c>
       <c r="G337" t="n">
-        <v>0</v>
+        <v>0.57</v>
       </c>
       <c r="H337" t="n">
         <v>0</v>
       </c>
       <c r="I337" t="n">
-        <v>5031600000</v>
+        <v>125211000</v>
       </c>
       <c r="J337" t="n">
-        <v>0</v>
+        <v>913.58</v>
       </c>
       <c r="K337" t="n">
         <v>0</v>
@@ -18970,27 +18970,27 @@
         <v>0</v>
       </c>
       <c r="O337" t="n">
-        <v>4.92</v>
+        <v>-0.88</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>SGEN4</t>
+          <t>VVAX3</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -19001,42 +19001,42 @@
         <v>0</v>
       </c>
       <c r="G338" t="n">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="H338" t="n">
         <v>0</v>
       </c>
       <c r="I338" t="n">
-        <v>156981000</v>
+        <v>144676000</v>
       </c>
       <c r="J338" t="n">
         <v>0</v>
       </c>
       <c r="K338" t="n">
-        <v>-1871.17</v>
+        <v>-7.36</v>
       </c>
       <c r="L338" t="n">
-        <v>0</v>
+        <v>-37.76</v>
       </c>
       <c r="M338" t="n">
-        <v>-1.59</v>
+        <v>-6.52</v>
       </c>
       <c r="N338" t="n">
-        <v>0</v>
+        <v>-92.03</v>
       </c>
       <c r="O338" t="n">
-        <v>-59.85</v>
+        <v>0</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>CCHI4</t>
+          <t>MSAN4</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -19045,7 +19045,7 @@
         </is>
       </c>
       <c r="D339" t="n">
-        <v>0.02</v>
+        <v>6.44</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -19056,51 +19056,51 @@
         <v>0</v>
       </c>
       <c r="G339" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="H339" t="n">
         <v>0</v>
       </c>
       <c r="I339" t="n">
-        <v>-160477000</v>
+        <v>2533030000</v>
       </c>
       <c r="J339" t="n">
         <v>0</v>
       </c>
       <c r="K339" t="n">
-        <v>0</v>
+        <v>6.27</v>
       </c>
       <c r="L339" t="n">
-        <v>0</v>
+        <v>2.42</v>
       </c>
       <c r="M339" t="n">
-        <v>0</v>
+        <v>11.78</v>
       </c>
       <c r="N339" t="n">
-        <v>0</v>
+        <v>11.81</v>
       </c>
       <c r="O339" t="n">
-        <v>20.36</v>
+        <v>101.35</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>REPA3</t>
+          <t>GALO4</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D340" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -19117,41 +19117,41 @@
         <v>0</v>
       </c>
       <c r="I340" t="n">
-        <v>378378000</v>
+        <v>-60607000</v>
       </c>
       <c r="J340" t="n">
         <v>0</v>
       </c>
       <c r="K340" t="n">
-        <v>5.18</v>
+        <v>13.98</v>
       </c>
       <c r="L340" t="n">
-        <v>1.22</v>
+        <v>-184.58</v>
       </c>
       <c r="M340" t="n">
-        <v>4.05</v>
+        <v>39.37</v>
       </c>
       <c r="N340" t="n">
-        <v>1.91</v>
+        <v>7.62</v>
       </c>
       <c r="O340" t="n">
-        <v>1.09</v>
+        <v>-28.97</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>EQMA5B</t>
+          <t>BBTG13</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D341" t="n">
@@ -19172,7 +19172,7 @@
         <v>0</v>
       </c>
       <c r="I341" t="n">
-        <v>4940330000</v>
+        <v>7000</v>
       </c>
       <c r="J341" t="n">
         <v>0</v>
@@ -19187,21 +19187,21 @@
         <v>0</v>
       </c>
       <c r="N341" t="n">
-        <v>0</v>
+        <v>-42.86</v>
       </c>
       <c r="O341" t="n">
-        <v>9.050000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>SEBB3</t>
+          <t>INHA3</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa INHA</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -19227,36 +19227,36 @@
         <v>0</v>
       </c>
       <c r="I342" t="n">
-        <v>145783000</v>
+        <v>1533210000</v>
       </c>
       <c r="J342" t="n">
         <v>0</v>
       </c>
       <c r="K342" t="n">
-        <v>9.24</v>
+        <v>-56.05</v>
       </c>
       <c r="L342" t="n">
-        <v>7.4</v>
+        <v>-124.06</v>
       </c>
       <c r="M342" t="n">
-        <v>24.15</v>
+        <v>-6.27</v>
       </c>
       <c r="N342" t="n">
-        <v>23.01</v>
+        <v>-39.87</v>
       </c>
       <c r="O342" t="n">
-        <v>50.04</v>
+        <v>-12.18</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>BBTG11</t>
+          <t>PTIP4</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -19265,7 +19265,7 @@
         </is>
       </c>
       <c r="D343" t="n">
-        <v>15.01</v>
+        <v>25.15</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -19282,45 +19282,45 @@
         <v>0</v>
       </c>
       <c r="I343" t="n">
-        <v>0</v>
+        <v>-155957000</v>
       </c>
       <c r="J343" t="n">
         <v>0</v>
       </c>
       <c r="K343" t="n">
-        <v>0</v>
+        <v>13.73</v>
       </c>
       <c r="L343" t="n">
-        <v>0</v>
+        <v>7.55</v>
       </c>
       <c r="M343" t="n">
-        <v>0</v>
+        <v>23.13</v>
       </c>
       <c r="N343" t="n">
-        <v>0</v>
+        <v>-121.74</v>
       </c>
       <c r="O343" t="n">
-        <v>0</v>
+        <v>62.11</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>JFAB4</t>
+          <t>LATS3</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Empresa JFAB</t>
+          <t>Empresa LATS</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>0.06</v>
+        <v>22</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -19337,36 +19337,36 @@
         <v>0</v>
       </c>
       <c r="I344" t="n">
-        <v>-10183000</v>
+        <v>680646000</v>
       </c>
       <c r="J344" t="n">
         <v>0</v>
       </c>
       <c r="K344" t="n">
-        <v>0</v>
+        <v>11.74</v>
       </c>
       <c r="L344" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="M344" t="n">
-        <v>0</v>
+        <v>11.63</v>
       </c>
       <c r="N344" t="n">
-        <v>2.34</v>
+        <v>1.84</v>
       </c>
       <c r="O344" t="n">
-        <v>0</v>
+        <v>15.37</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>LECO3</t>
+          <t>VSPT3</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Empresa LECO</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -19392,45 +19392,45 @@
         <v>0</v>
       </c>
       <c r="I345" t="n">
-        <v>105928000</v>
+        <v>5031600000</v>
       </c>
       <c r="J345" t="n">
         <v>0</v>
       </c>
       <c r="K345" t="n">
-        <v>-2.14</v>
+        <v>0</v>
       </c>
       <c r="L345" t="n">
-        <v>-4.72</v>
+        <v>0</v>
       </c>
       <c r="M345" t="n">
-        <v>-3.48</v>
+        <v>0</v>
       </c>
       <c r="N345" t="n">
-        <v>-14.82</v>
+        <v>0</v>
       </c>
       <c r="O345" t="n">
-        <v>3.58</v>
+        <v>4.92</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>VGOR3</t>
+          <t>SGEN4</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Empresa VGOR</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -19441,51 +19441,51 @@
         <v>0</v>
       </c>
       <c r="G346" t="n">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="H346" t="n">
         <v>0</v>
       </c>
       <c r="I346" t="n">
-        <v>135178000</v>
+        <v>156981000</v>
       </c>
       <c r="J346" t="n">
         <v>0</v>
       </c>
       <c r="K346" t="n">
-        <v>4.5</v>
+        <v>-1871.17</v>
       </c>
       <c r="L346" t="n">
-        <v>-4.59</v>
+        <v>0</v>
       </c>
       <c r="M346" t="n">
-        <v>6</v>
+        <v>-1.59</v>
       </c>
       <c r="N346" t="n">
-        <v>-24.29</v>
+        <v>0</v>
       </c>
       <c r="O346" t="n">
-        <v>4.77</v>
+        <v>-59.85</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>GPIV33</t>
+          <t>CCHI4</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Empresa GPIV</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>4.42</v>
+        <v>0.02</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -19496,51 +19496,51 @@
         <v>0</v>
       </c>
       <c r="G347" t="n">
-        <v>0.23</v>
+        <v>-0.01</v>
       </c>
       <c r="H347" t="n">
         <v>0</v>
       </c>
       <c r="I347" t="n">
-        <v>1318490000</v>
+        <v>-160477000</v>
       </c>
       <c r="J347" t="n">
         <v>0</v>
       </c>
       <c r="K347" t="n">
-        <v>257.32</v>
+        <v>0</v>
       </c>
       <c r="L347" t="n">
         <v>0</v>
       </c>
       <c r="M347" t="n">
-        <v>-6.05</v>
+        <v>0</v>
       </c>
       <c r="N347" t="n">
         <v>0</v>
       </c>
       <c r="O347" t="n">
-        <v>-40.99</v>
+        <v>20.36</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>ECIS4</t>
+          <t>REPA3</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>145</v>
+        <v>1</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -19557,45 +19557,45 @@
         <v>0</v>
       </c>
       <c r="I348" t="n">
-        <v>129346000</v>
+        <v>378378000</v>
       </c>
       <c r="J348" t="n">
         <v>0</v>
       </c>
       <c r="K348" t="n">
-        <v>34.9</v>
+        <v>5.18</v>
       </c>
       <c r="L348" t="n">
-        <v>14.18</v>
+        <v>1.22</v>
       </c>
       <c r="M348" t="n">
-        <v>12.48</v>
+        <v>4.05</v>
       </c>
       <c r="N348" t="n">
-        <v>7.33</v>
+        <v>1.91</v>
       </c>
       <c r="O348" t="n">
-        <v>4.66</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>TNEP3</t>
+          <t>EQMA5B</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>3.01</v>
+        <v>0</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -19612,45 +19612,45 @@
         <v>0</v>
       </c>
       <c r="I349" t="n">
-        <v>955105000</v>
+        <v>4940330000</v>
       </c>
       <c r="J349" t="n">
         <v>0</v>
       </c>
       <c r="K349" t="n">
-        <v>20.92</v>
+        <v>0</v>
       </c>
       <c r="L349" t="n">
-        <v>25.42</v>
+        <v>0</v>
       </c>
       <c r="M349" t="n">
-        <v>20.53</v>
+        <v>0</v>
       </c>
       <c r="N349" t="n">
-        <v>22.8</v>
+        <v>0</v>
       </c>
       <c r="O349" t="n">
-        <v>8.15</v>
+        <v>9.050000000000001</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>CBMA4</t>
+          <t>SEBB3</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -19667,45 +19667,45 @@
         <v>0</v>
       </c>
       <c r="I350" t="n">
-        <v>-34022300000</v>
+        <v>145783000</v>
       </c>
       <c r="J350" t="n">
         <v>0</v>
       </c>
       <c r="K350" t="n">
-        <v>0</v>
+        <v>9.24</v>
       </c>
       <c r="L350" t="n">
-        <v>0</v>
+        <v>7.4</v>
       </c>
       <c r="M350" t="n">
-        <v>0</v>
+        <v>24.15</v>
       </c>
       <c r="N350" t="n">
-        <v>0</v>
+        <v>23.01</v>
       </c>
       <c r="O350" t="n">
-        <v>252.65</v>
+        <v>50.04</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>SALM4</t>
+          <t>BBTG11</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>5.9</v>
+        <v>15.01</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -19722,45 +19722,45 @@
         <v>0</v>
       </c>
       <c r="I351" t="n">
-        <v>475600000</v>
+        <v>0</v>
       </c>
       <c r="J351" t="n">
         <v>0</v>
       </c>
       <c r="K351" t="n">
-        <v>10.22</v>
+        <v>0</v>
       </c>
       <c r="L351" t="n">
-        <v>4.13</v>
+        <v>0</v>
       </c>
       <c r="M351" t="n">
-        <v>25.78</v>
+        <v>0</v>
       </c>
       <c r="N351" t="n">
-        <v>19.53</v>
+        <v>0</v>
       </c>
       <c r="O351" t="n">
-        <v>24.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>BERG3</t>
+          <t>JFAB4</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Empresa BERG</t>
+          <t>Empresa JFAB</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>33</v>
+        <v>0.06</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -19777,36 +19777,36 @@
         <v>0</v>
       </c>
       <c r="I352" t="n">
-        <v>9538000</v>
+        <v>-10183000</v>
       </c>
       <c r="J352" t="n">
         <v>0</v>
       </c>
       <c r="K352" t="n">
-        <v>-8.6</v>
+        <v>0</v>
       </c>
       <c r="L352" t="n">
-        <v>-32.6</v>
+        <v>0</v>
       </c>
       <c r="M352" t="n">
-        <v>-5.58</v>
+        <v>0</v>
       </c>
       <c r="N352" t="n">
-        <v>-102.71</v>
+        <v>2.34</v>
       </c>
       <c r="O352" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>JBDU3</t>
+          <t>VGOR3</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Empresa JBDU</t>
+          <t>Empresa VGOR</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -19832,36 +19832,36 @@
         <v>0</v>
       </c>
       <c r="I353" t="n">
-        <v>56569000</v>
+        <v>135178000</v>
       </c>
       <c r="J353" t="n">
         <v>0</v>
       </c>
       <c r="K353" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="L353" t="n">
-        <v>0</v>
+        <v>-4.59</v>
       </c>
       <c r="M353" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N353" t="n">
-        <v>0</v>
+        <v>-24.29</v>
       </c>
       <c r="O353" t="n">
-        <v>0</v>
+        <v>4.77</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>EGGY3</t>
+          <t>GPIV33</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Empresa EGGY</t>
+          <t>Empresa GPIV</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -19870,7 +19870,7 @@
         </is>
       </c>
       <c r="D354" t="n">
-        <v>0</v>
+        <v>4.42</v>
       </c>
       <c r="E354" t="inlineStr">
         <is>
@@ -19881,51 +19881,51 @@
         <v>0</v>
       </c>
       <c r="G354" t="n">
-        <v>0</v>
+        <v>0.23</v>
       </c>
       <c r="H354" t="n">
         <v>0</v>
       </c>
       <c r="I354" t="n">
-        <v>954480000</v>
+        <v>1318490000</v>
       </c>
       <c r="J354" t="n">
         <v>0</v>
       </c>
       <c r="K354" t="n">
-        <v>0</v>
+        <v>257.32</v>
       </c>
       <c r="L354" t="n">
         <v>0</v>
       </c>
       <c r="M354" t="n">
-        <v>0</v>
+        <v>-6.05</v>
       </c>
       <c r="N354" t="n">
         <v>0</v>
       </c>
       <c r="O354" t="n">
-        <v>-0.82</v>
+        <v>-40.99</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>AGEI3</t>
+          <t>ECIS4</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Empresa AGEI</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>7.8</v>
+        <v>145</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -19936,42 +19936,42 @@
         <v>0</v>
       </c>
       <c r="G355" t="n">
-        <v>1.25</v>
+        <v>0</v>
       </c>
       <c r="H355" t="n">
         <v>0</v>
       </c>
       <c r="I355" t="n">
-        <v>1878210000</v>
+        <v>129346000</v>
       </c>
       <c r="J355" t="n">
         <v>0</v>
       </c>
       <c r="K355" t="n">
-        <v>0</v>
+        <v>34.9</v>
       </c>
       <c r="L355" t="n">
-        <v>0</v>
+        <v>14.18</v>
       </c>
       <c r="M355" t="n">
-        <v>0</v>
+        <v>12.48</v>
       </c>
       <c r="N355" t="n">
-        <v>0</v>
+        <v>7.33</v>
       </c>
       <c r="O355" t="n">
-        <v>0</v>
+        <v>4.66</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>SASG3</t>
+          <t>TNEP3</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Empresa SASG</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -19980,7 +19980,7 @@
         </is>
       </c>
       <c r="D356" t="n">
-        <v>0.98</v>
+        <v>3.01</v>
       </c>
       <c r="E356" t="inlineStr">
         <is>
@@ -19997,36 +19997,36 @@
         <v>0</v>
       </c>
       <c r="I356" t="n">
-        <v>0</v>
+        <v>955105000</v>
       </c>
       <c r="J356" t="n">
         <v>0</v>
       </c>
       <c r="K356" t="n">
-        <v>0</v>
+        <v>20.92</v>
       </c>
       <c r="L356" t="n">
-        <v>0</v>
+        <v>25.42</v>
       </c>
       <c r="M356" t="n">
-        <v>0</v>
+        <v>20.53</v>
       </c>
       <c r="N356" t="n">
-        <v>0</v>
+        <v>22.8</v>
       </c>
       <c r="O356" t="n">
-        <v>0</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>BMEF3</t>
+          <t>LECO3</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Empresa BMEF</t>
+          <t>Empresa LECO</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -20035,7 +20035,7 @@
         </is>
       </c>
       <c r="D357" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -20046,51 +20046,51 @@
         <v>0</v>
       </c>
       <c r="G357" t="n">
-        <v>4.16</v>
+        <v>0</v>
       </c>
       <c r="H357" t="n">
         <v>0</v>
       </c>
       <c r="I357" t="n">
-        <v>2674780000</v>
+        <v>105928000</v>
       </c>
       <c r="J357" t="n">
         <v>0</v>
       </c>
       <c r="K357" t="n">
-        <v>0</v>
+        <v>-2.14</v>
       </c>
       <c r="L357" t="n">
-        <v>0</v>
+        <v>-4.72</v>
       </c>
       <c r="M357" t="n">
-        <v>0</v>
+        <v>-3.48</v>
       </c>
       <c r="N357" t="n">
-        <v>0</v>
+        <v>-14.82</v>
       </c>
       <c r="O357" t="n">
-        <v>0</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>ARPS3</t>
+          <t>CBMA4</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D358" t="n">
-        <v>0.3</v>
+        <v>0.01</v>
       </c>
       <c r="E358" t="inlineStr">
         <is>
@@ -20107,45 +20107,45 @@
         <v>0</v>
       </c>
       <c r="I358" t="n">
-        <v>-12690000</v>
+        <v>-34022300000</v>
       </c>
       <c r="J358" t="n">
         <v>0</v>
       </c>
       <c r="K358" t="n">
-        <v>-4.92</v>
+        <v>0</v>
       </c>
       <c r="L358" t="n">
-        <v>-11.59</v>
+        <v>0</v>
       </c>
       <c r="M358" t="n">
-        <v>-6.64</v>
+        <v>0</v>
       </c>
       <c r="N358" t="n">
-        <v>20.34</v>
+        <v>0</v>
       </c>
       <c r="O358" t="n">
-        <v>-17.53</v>
+        <v>252.65</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>ODER3</t>
+          <t>SALM4</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Empresa ODER</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -20162,36 +20162,36 @@
         <v>0</v>
       </c>
       <c r="I359" t="n">
-        <v>609518000</v>
+        <v>475600000</v>
       </c>
       <c r="J359" t="n">
         <v>0</v>
       </c>
       <c r="K359" t="n">
-        <v>0</v>
+        <v>10.22</v>
       </c>
       <c r="L359" t="n">
-        <v>0</v>
+        <v>4.13</v>
       </c>
       <c r="M359" t="n">
-        <v>0</v>
+        <v>25.78</v>
       </c>
       <c r="N359" t="n">
-        <v>0</v>
+        <v>19.53</v>
       </c>
       <c r="O359" t="n">
-        <v>3.17</v>
+        <v>24.53</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>CCTY3</t>
+          <t>BERG3</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Empresa CCTY</t>
+          <t>Empresa BERG</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
@@ -20200,7 +20200,7 @@
         </is>
       </c>
       <c r="D360" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -20217,41 +20217,41 @@
         <v>0</v>
       </c>
       <c r="I360" t="n">
-        <v>0</v>
+        <v>9538000</v>
       </c>
       <c r="J360" t="n">
         <v>0</v>
       </c>
       <c r="K360" t="n">
-        <v>0</v>
+        <v>-8.6</v>
       </c>
       <c r="L360" t="n">
-        <v>0</v>
+        <v>-32.6</v>
       </c>
       <c r="M360" t="n">
-        <v>0</v>
+        <v>-5.58</v>
       </c>
       <c r="N360" t="n">
-        <v>0</v>
+        <v>-102.71</v>
       </c>
       <c r="O360" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>VVAX4</t>
+          <t>JBDU3</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa JBDU</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D361" t="n">
@@ -20272,22 +20272,22 @@
         <v>0</v>
       </c>
       <c r="I361" t="n">
-        <v>144676000</v>
+        <v>56569000</v>
       </c>
       <c r="J361" t="n">
         <v>0</v>
       </c>
       <c r="K361" t="n">
-        <v>-7.36</v>
+        <v>0</v>
       </c>
       <c r="L361" t="n">
-        <v>-37.76</v>
+        <v>0</v>
       </c>
       <c r="M361" t="n">
-        <v>-6.52</v>
+        <v>0</v>
       </c>
       <c r="N361" t="n">
-        <v>-92.03</v>
+        <v>0</v>
       </c>
       <c r="O361" t="n">
         <v>0</v>
@@ -20296,12 +20296,12 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>CSPC3</t>
+          <t>EGGY3</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa EGGY</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -20310,7 +20310,7 @@
         </is>
       </c>
       <c r="D362" t="n">
-        <v>1.24</v>
+        <v>0</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -20327,36 +20327,36 @@
         <v>0</v>
       </c>
       <c r="I362" t="n">
-        <v>2126670000</v>
+        <v>954480000</v>
       </c>
       <c r="J362" t="n">
         <v>0</v>
       </c>
       <c r="K362" t="n">
-        <v>38.62</v>
+        <v>0</v>
       </c>
       <c r="L362" t="n">
-        <v>18.85</v>
+        <v>0</v>
       </c>
       <c r="M362" t="n">
-        <v>29.18</v>
+        <v>0</v>
       </c>
       <c r="N362" t="n">
-        <v>45.33</v>
+        <v>0</v>
       </c>
       <c r="O362" t="n">
-        <v>41.15</v>
+        <v>-0.82</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>ABCB3</t>
+          <t>AGEI3</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Empresa ABCB</t>
+          <t>Empresa AGEI</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -20365,24 +20365,24 @@
         </is>
       </c>
       <c r="D363" t="n">
-        <v>0</v>
+        <v>7.8</v>
       </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t>Bancos</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="F363" t="n">
         <v>0</v>
       </c>
       <c r="G363" t="n">
-        <v>0</v>
+        <v>1.25</v>
       </c>
       <c r="H363" t="n">
         <v>0</v>
       </c>
       <c r="I363" t="n">
-        <v>7258910000</v>
+        <v>1878210000</v>
       </c>
       <c r="J363" t="n">
         <v>0</v>
@@ -20397,30 +20397,30 @@
         <v>0</v>
       </c>
       <c r="N363" t="n">
-        <v>14.05</v>
+        <v>0</v>
       </c>
       <c r="O363" t="n">
-        <v>7.57</v>
+        <v>0</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>ESTC4</t>
+          <t>SASG3</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Empresa ESTC</t>
+          <t>Empresa SASG</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D364" t="n">
-        <v>0</v>
+        <v>0.98</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -20437,45 +20437,45 @@
         <v>0</v>
       </c>
       <c r="I364" t="n">
-        <v>2916530000</v>
+        <v>0</v>
       </c>
       <c r="J364" t="n">
         <v>0</v>
       </c>
       <c r="K364" t="n">
-        <v>16.91</v>
+        <v>0</v>
       </c>
       <c r="L364" t="n">
-        <v>2.02</v>
+        <v>0</v>
       </c>
       <c r="M364" t="n">
-        <v>11.35</v>
+        <v>0</v>
       </c>
       <c r="N364" t="n">
-        <v>3.89</v>
+        <v>0</v>
       </c>
       <c r="O364" t="n">
-        <v>5.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>VSPT4</t>
+          <t>BMEF3</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa BMEF</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D365" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E365" t="inlineStr">
         <is>
@@ -20486,13 +20486,13 @@
         <v>0</v>
       </c>
       <c r="G365" t="n">
-        <v>0</v>
+        <v>4.16</v>
       </c>
       <c r="H365" t="n">
         <v>0</v>
       </c>
       <c r="I365" t="n">
-        <v>5031600000</v>
+        <v>2674780000</v>
       </c>
       <c r="J365" t="n">
         <v>0</v>
@@ -20510,27 +20510,27 @@
         <v>0</v>
       </c>
       <c r="O365" t="n">
-        <v>4.92</v>
+        <v>0</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>BAUH4</t>
+          <t>ARPS3</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Empresa BAUH</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D366" t="n">
-        <v>93.39</v>
+        <v>0.3</v>
       </c>
       <c r="E366" t="inlineStr">
         <is>
@@ -20541,42 +20541,42 @@
         <v>0</v>
       </c>
       <c r="G366" t="n">
-        <v>3.18</v>
+        <v>0</v>
       </c>
       <c r="H366" t="n">
-        <v>1.16</v>
+        <v>0</v>
       </c>
       <c r="I366" t="n">
-        <v>153407000</v>
+        <v>-12690000</v>
       </c>
       <c r="J366" t="n">
-        <v>207.53</v>
+        <v>0</v>
       </c>
       <c r="K366" t="n">
-        <v>0</v>
+        <v>-4.92</v>
       </c>
       <c r="L366" t="n">
-        <v>0</v>
+        <v>-11.59</v>
       </c>
       <c r="M366" t="n">
-        <v>0</v>
+        <v>-6.64</v>
       </c>
       <c r="N366" t="n">
-        <v>0</v>
+        <v>20.34</v>
       </c>
       <c r="O366" t="n">
-        <v>13.32</v>
+        <v>-17.53</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>ICPI3</t>
+          <t>ODER3</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Empresa ICPI</t>
+          <t>Empresa ODER</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -20602,7 +20602,7 @@
         <v>0</v>
       </c>
       <c r="I367" t="n">
-        <v>0</v>
+        <v>609518000</v>
       </c>
       <c r="J367" t="n">
         <v>0</v>
@@ -20620,27 +20620,27 @@
         <v>0</v>
       </c>
       <c r="O367" t="n">
-        <v>0</v>
+        <v>3.17</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>ILLS4</t>
+          <t>CCTY3</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Empresa ILLS</t>
+          <t>Empresa CCTY</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D368" t="n">
-        <v>100.01</v>
+        <v>0</v>
       </c>
       <c r="E368" t="inlineStr">
         <is>
@@ -20657,45 +20657,45 @@
         <v>0</v>
       </c>
       <c r="I368" t="n">
-        <v>-18567000</v>
+        <v>0</v>
       </c>
       <c r="J368" t="n">
         <v>0</v>
       </c>
       <c r="K368" t="n">
-        <v>8.43</v>
+        <v>0</v>
       </c>
       <c r="L368" t="n">
-        <v>-10.22</v>
+        <v>0</v>
       </c>
       <c r="M368" t="n">
-        <v>8.140000000000001</v>
+        <v>0</v>
       </c>
       <c r="N368" t="n">
-        <v>36.09</v>
+        <v>0</v>
       </c>
       <c r="O368" t="n">
-        <v>9.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>BPAT33</t>
+          <t>VVAX4</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Empresa BPAT</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D369" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="E369" t="inlineStr">
         <is>
@@ -20706,28 +20706,28 @@
         <v>0</v>
       </c>
       <c r="G369" t="n">
-        <v>0.82</v>
+        <v>0</v>
       </c>
       <c r="H369" t="n">
-        <v>35.72</v>
+        <v>0</v>
       </c>
       <c r="I369" t="n">
-        <v>876492000</v>
+        <v>144676000</v>
       </c>
       <c r="J369" t="n">
         <v>0</v>
       </c>
       <c r="K369" t="n">
-        <v>0</v>
+        <v>-7.36</v>
       </c>
       <c r="L369" t="n">
-        <v>0</v>
+        <v>-37.76</v>
       </c>
       <c r="M369" t="n">
-        <v>0</v>
+        <v>-6.52</v>
       </c>
       <c r="N369" t="n">
-        <v>0</v>
+        <v>-92.03</v>
       </c>
       <c r="O369" t="n">
         <v>0</v>
@@ -20736,21 +20736,21 @@
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>REPA4</t>
+          <t>CSPC3</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D370" t="n">
-        <v>1.08</v>
+        <v>1.24</v>
       </c>
       <c r="E370" t="inlineStr">
         <is>
@@ -20767,41 +20767,41 @@
         <v>0</v>
       </c>
       <c r="I370" t="n">
-        <v>378378000</v>
+        <v>2126670000</v>
       </c>
       <c r="J370" t="n">
         <v>0</v>
       </c>
       <c r="K370" t="n">
-        <v>5.18</v>
+        <v>38.62</v>
       </c>
       <c r="L370" t="n">
-        <v>1.22</v>
+        <v>18.85</v>
       </c>
       <c r="M370" t="n">
-        <v>4.05</v>
+        <v>29.18</v>
       </c>
       <c r="N370" t="n">
-        <v>1.91</v>
+        <v>45.33</v>
       </c>
       <c r="O370" t="n">
-        <v>1.09</v>
+        <v>41.15</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>EQMA6B</t>
+          <t>ABCB3</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa ABCB</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D371" t="n">
@@ -20809,7 +20809,7 @@
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="F371" t="n">
@@ -20822,7 +20822,7 @@
         <v>0</v>
       </c>
       <c r="I371" t="n">
-        <v>4940330000</v>
+        <v>7258910000</v>
       </c>
       <c r="J371" t="n">
         <v>0</v>
@@ -20837,21 +20837,21 @@
         <v>0</v>
       </c>
       <c r="N371" t="n">
-        <v>0</v>
+        <v>14.05</v>
       </c>
       <c r="O371" t="n">
-        <v>9.050000000000001</v>
+        <v>7.57</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>SEBB4</t>
+          <t>ESTC4</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa ESTC</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
@@ -20877,45 +20877,45 @@
         <v>0</v>
       </c>
       <c r="I372" t="n">
-        <v>145783000</v>
+        <v>2916530000</v>
       </c>
       <c r="J372" t="n">
         <v>0</v>
       </c>
       <c r="K372" t="n">
-        <v>9.24</v>
+        <v>16.91</v>
       </c>
       <c r="L372" t="n">
-        <v>7.4</v>
+        <v>2.02</v>
       </c>
       <c r="M372" t="n">
-        <v>24.15</v>
+        <v>11.35</v>
       </c>
       <c r="N372" t="n">
-        <v>23.01</v>
+        <v>3.89</v>
       </c>
       <c r="O372" t="n">
-        <v>50.04</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>MSAN3</t>
+          <t>VSPT4</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D373" t="n">
-        <v>6.44</v>
+        <v>0</v>
       </c>
       <c r="E373" t="inlineStr">
         <is>
@@ -20932,45 +20932,45 @@
         <v>0</v>
       </c>
       <c r="I373" t="n">
-        <v>2533030000</v>
+        <v>5031600000</v>
       </c>
       <c r="J373" t="n">
         <v>0</v>
       </c>
       <c r="K373" t="n">
-        <v>6.27</v>
+        <v>0</v>
       </c>
       <c r="L373" t="n">
-        <v>2.42</v>
+        <v>0</v>
       </c>
       <c r="M373" t="n">
-        <v>11.78</v>
+        <v>0</v>
       </c>
       <c r="N373" t="n">
-        <v>11.81</v>
+        <v>0</v>
       </c>
       <c r="O373" t="n">
-        <v>101.35</v>
+        <v>4.92</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>GALO3</t>
+          <t>BAUH4</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa BAUH</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D374" t="n">
-        <v>0</v>
+        <v>93.39</v>
       </c>
       <c r="E374" t="inlineStr">
         <is>
@@ -20981,42 +20981,42 @@
         <v>0</v>
       </c>
       <c r="G374" t="n">
-        <v>0</v>
+        <v>3.18</v>
       </c>
       <c r="H374" t="n">
-        <v>0</v>
+        <v>1.16</v>
       </c>
       <c r="I374" t="n">
-        <v>-60607000</v>
+        <v>153407000</v>
       </c>
       <c r="J374" t="n">
-        <v>0</v>
+        <v>207.53</v>
       </c>
       <c r="K374" t="n">
-        <v>13.98</v>
+        <v>0</v>
       </c>
       <c r="L374" t="n">
-        <v>-184.58</v>
+        <v>0</v>
       </c>
       <c r="M374" t="n">
-        <v>39.37</v>
+        <v>0</v>
       </c>
       <c r="N374" t="n">
-        <v>7.62</v>
+        <v>0</v>
       </c>
       <c r="O374" t="n">
-        <v>-28.97</v>
+        <v>13.32</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>SLCP3</t>
+          <t>ICPI3</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>Empresa SLCP</t>
+          <t>Empresa ICPI</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
@@ -21025,7 +21025,7 @@
         </is>
       </c>
       <c r="D375" t="n">
-        <v>610.02</v>
+        <v>0</v>
       </c>
       <c r="E375" t="inlineStr">
         <is>
@@ -21066,21 +21066,21 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>DAYC3</t>
+          <t>ILLS4</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>Empresa DAYC</t>
+          <t>Empresa ILLS</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D376" t="n">
-        <v>0</v>
+        <v>100.01</v>
       </c>
       <c r="E376" t="inlineStr">
         <is>
@@ -21097,36 +21097,36 @@
         <v>0</v>
       </c>
       <c r="I376" t="n">
-        <v>3009030000</v>
+        <v>-18567000</v>
       </c>
       <c r="J376" t="n">
         <v>0</v>
       </c>
       <c r="K376" t="n">
-        <v>0</v>
+        <v>8.43</v>
       </c>
       <c r="L376" t="n">
-        <v>0</v>
+        <v>-10.22</v>
       </c>
       <c r="M376" t="n">
-        <v>0</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="N376" t="n">
-        <v>17.33</v>
+        <v>36.09</v>
       </c>
       <c r="O376" t="n">
-        <v>8.15</v>
+        <v>9.33</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>PTIP3</t>
+          <t>BPAT33</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa BPAT</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
@@ -21135,7 +21135,7 @@
         </is>
       </c>
       <c r="D377" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -21146,31 +21146,31 @@
         <v>0</v>
       </c>
       <c r="G377" t="n">
-        <v>0</v>
+        <v>0.82</v>
       </c>
       <c r="H377" t="n">
-        <v>0</v>
+        <v>35.72</v>
       </c>
       <c r="I377" t="n">
-        <v>-155957000</v>
+        <v>876492000</v>
       </c>
       <c r="J377" t="n">
         <v>0</v>
       </c>
       <c r="K377" t="n">
-        <v>13.73</v>
+        <v>0</v>
       </c>
       <c r="L377" t="n">
-        <v>7.55</v>
+        <v>0</v>
       </c>
       <c r="M377" t="n">
-        <v>23.13</v>
+        <v>0</v>
       </c>
       <c r="N377" t="n">
-        <v>-121.74</v>
+        <v>0</v>
       </c>
       <c r="O377" t="n">
-        <v>62.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="378">
@@ -21351,7 +21351,7 @@
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D381" t="n">
@@ -21461,7 +21461,7 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D383" t="n">
@@ -21571,7 +21571,7 @@
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D385" t="n">
@@ -21736,7 +21736,7 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D388" t="n">
@@ -21791,7 +21791,7 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D389" t="n">
@@ -22066,7 +22066,7 @@
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D394" t="n">
@@ -23936,7 +23936,7 @@
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D428" t="n">
@@ -24981,7 +24981,7 @@
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D447" t="n">
@@ -28336,7 +28336,7 @@
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D508" t="n">
@@ -29051,7 +29051,7 @@
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D521" t="n">
@@ -29986,7 +29986,7 @@
       </c>
       <c r="C538" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D538" t="n">
@@ -31351,7 +31351,7 @@
     <row r="563">
       <c r="A563" t="inlineStr">
         <is>
-          <t>CIQU3</t>
+          <t>CIQU4</t>
         </is>
       </c>
       <c r="B563" t="inlineStr">
@@ -31361,7 +31361,7 @@
       </c>
       <c r="C563" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D563" t="n">
@@ -31406,7 +31406,7 @@
     <row r="564">
       <c r="A564" t="inlineStr">
         <is>
-          <t>CIQU4</t>
+          <t>CIQU3</t>
         </is>
       </c>
       <c r="B564" t="inlineStr">
@@ -31416,7 +31416,7 @@
       </c>
       <c r="C564" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D564" t="n">
@@ -32736,7 +32736,7 @@
       </c>
       <c r="C588" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D588" t="n">
@@ -33781,7 +33781,7 @@
       </c>
       <c r="C607" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D607" t="n">
@@ -34431,7 +34431,7 @@
     <row r="619">
       <c r="A619" t="inlineStr">
         <is>
-          <t>AESL3</t>
+          <t>AESL4</t>
         </is>
       </c>
       <c r="B619" t="inlineStr">
@@ -34441,7 +34441,7 @@
       </c>
       <c r="C619" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D619" t="n">
@@ -34486,7 +34486,7 @@
     <row r="620">
       <c r="A620" t="inlineStr">
         <is>
-          <t>AESL4</t>
+          <t>AESL3</t>
         </is>
       </c>
       <c r="B620" t="inlineStr">
@@ -34496,7 +34496,7 @@
       </c>
       <c r="C620" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D620" t="n">
@@ -35101,7 +35101,7 @@
       </c>
       <c r="C631" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D631" t="n">
@@ -35156,7 +35156,7 @@
       </c>
       <c r="C632" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D632" t="n">
@@ -35651,7 +35651,7 @@
       </c>
       <c r="C641" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D641" t="n">
@@ -36366,7 +36366,7 @@
       </c>
       <c r="C654" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D654" t="n">
@@ -36916,7 +36916,7 @@
       </c>
       <c r="C664" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D664" t="n">
@@ -37081,7 +37081,7 @@
       </c>
       <c r="C667" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D667" t="n">
@@ -37686,7 +37686,7 @@
       </c>
       <c r="C678" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D678" t="n">
@@ -39171,7 +39171,7 @@
       </c>
       <c r="C705" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D705" t="n">
@@ -40766,7 +40766,7 @@
       </c>
       <c r="C734" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D734" t="n">
@@ -41041,7 +41041,7 @@
       </c>
       <c r="C739" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D739" t="n">
@@ -43076,7 +43076,7 @@
       </c>
       <c r="C776" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D776" t="n">
@@ -45386,7 +45386,7 @@
       </c>
       <c r="C818" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D818" t="n">
@@ -45496,7 +45496,7 @@
       </c>
       <c r="C820" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D820" t="n">
@@ -46211,7 +46211,7 @@
       </c>
       <c r="C833" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D833" t="n">
@@ -46761,7 +46761,7 @@
       </c>
       <c r="C843" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D843" t="n">
@@ -48136,7 +48136,7 @@
       </c>
       <c r="C868" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D868" t="n">
@@ -49346,7 +49346,7 @@
       </c>
       <c r="C890" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D890" t="n">
@@ -50226,7 +50226,7 @@
       </c>
       <c r="C906" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D906" t="n">
@@ -50391,7 +50391,7 @@
       </c>
       <c r="C909" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D909" t="n">
@@ -51546,7 +51546,7 @@
       </c>
       <c r="C930" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D930" t="n">
@@ -52151,7 +52151,7 @@
       </c>
       <c r="C941" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D941" t="n">
@@ -54571,7 +54571,7 @@
       </c>
       <c r="C985" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D985" t="n">
@@ -55011,7 +55011,7 @@
       </c>
       <c r="C993" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D993" t="n">

</xml_diff>

<commit_message>
Atualização automática dos dados da B3
</commit_message>
<xml_diff>
--- a/acoes_b3.xlsx
+++ b/acoes_b3.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,102 +429,102 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Empresa</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Segmento de Listagem</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Cotação</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Setor</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Tag Along (%)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Free Float (%)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Governo Majoritário</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/EBIT</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>P/L</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>P/VP</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Dividend Yield</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Patrimônio Líquido</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Liquidez Diária</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Margem EBIT</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Margem Líquida</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>ROIC</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>ROE</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Cresc. 5 Anos (%)</t>
         </is>
@@ -965,17 +977,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CSTB3</t>
+          <t>CFLU4</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa CFLU</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -984,7 +996,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>150</v>
+        <v>1000</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1015,41 +1027,41 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>8420670000</v>
+        <v>60351000</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>40.85</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="Q8" t="n">
-        <v>28.98</v>
+        <v>10.72</v>
       </c>
       <c r="R8" t="n">
-        <v>22.4</v>
+        <v>17.68</v>
       </c>
       <c r="S8" t="n">
-        <v>20.11</v>
+        <v>32.15</v>
       </c>
       <c r="T8" t="n">
-        <v>31.91</v>
+        <v>8.140000000000001</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CFLU4</t>
+          <t>CSTB3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Empresa CFLU</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1058,7 +1070,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>1000</v>
+        <v>150</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1089,25 +1101,25 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>60351000</v>
+        <v>8420670000</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>8.880000000000001</v>
+        <v>40.85</v>
       </c>
       <c r="Q9" t="n">
-        <v>10.72</v>
+        <v>28.98</v>
       </c>
       <c r="R9" t="n">
-        <v>17.68</v>
+        <v>22.4</v>
       </c>
       <c r="S9" t="n">
-        <v>32.15</v>
+        <v>20.11</v>
       </c>
       <c r="T9" t="n">
-        <v>8.140000000000001</v>
+        <v>31.91</v>
       </c>
     </row>
     <row r="10">
@@ -12361,7 +12373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>RNEW3</t>
+          <t>RNEW4</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -12371,7 +12383,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -12414,7 +12426,7 @@
         <v>1150280000</v>
       </c>
       <c r="O162" t="n">
-        <v>45273.4</v>
+        <v>44097</v>
       </c>
       <c r="P162" t="n">
         <v>-2.89</v>
@@ -12435,7 +12447,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>RNEW4</t>
+          <t>RNEW3</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -12445,7 +12457,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -12488,7 +12500,7 @@
         <v>1150280000</v>
       </c>
       <c r="O163" t="n">
-        <v>44097</v>
+        <v>45273.4</v>
       </c>
       <c r="P163" t="n">
         <v>-2.89</v>
@@ -14137,7 +14149,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>SDIA4</t>
+          <t>SDIA3</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -14147,7 +14159,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -14211,7 +14223,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>SDIA3</t>
+          <t>SDIA4</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -14221,7 +14233,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -23091,12 +23103,12 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>ARND3</t>
+          <t>BPNM3</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Empresa ARND</t>
+          <t>Empresa BPNM</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -23106,22 +23118,22 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Novo Mercado</t>
+          <t>Tradicional</t>
         </is>
       </c>
       <c r="E307" t="n">
-        <v>0.51</v>
+        <v>0</v>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G307" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="H307" t="n">
-        <v>12.49</v>
+        <v>0</v>
       </c>
       <c r="I307" t="inlineStr">
         <is>
@@ -23135,16 +23147,16 @@
         <v>0</v>
       </c>
       <c r="L307" t="n">
-        <v>0.57</v>
+        <v>0</v>
       </c>
       <c r="M307" t="n">
         <v>0</v>
       </c>
       <c r="N307" t="n">
-        <v>125211000</v>
+        <v>7792670000</v>
       </c>
       <c r="O307" t="n">
-        <v>913.58</v>
+        <v>0</v>
       </c>
       <c r="P307" t="n">
         <v>0</v>
@@ -23156,21 +23168,21 @@
         <v>0</v>
       </c>
       <c r="S307" t="n">
-        <v>0</v>
+        <v>9.67</v>
       </c>
       <c r="T307" t="n">
-        <v>-0.88</v>
+        <v>-1.53</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>VVAX3</t>
+          <t>BSGR3</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa BSGR</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -23184,7 +23196,7 @@
         </is>
       </c>
       <c r="E308" t="n">
-        <v>0</v>
+        <v>1091.28</v>
       </c>
       <c r="F308" t="inlineStr">
         <is>
@@ -23215,22 +23227,22 @@
         <v>0</v>
       </c>
       <c r="N308" t="n">
-        <v>144676000</v>
+        <v>0</v>
       </c>
       <c r="O308" t="n">
         <v>0</v>
       </c>
       <c r="P308" t="n">
-        <v>-7.36</v>
+        <v>0</v>
       </c>
       <c r="Q308" t="n">
-        <v>-37.76</v>
+        <v>0</v>
       </c>
       <c r="R308" t="n">
-        <v>-6.52</v>
+        <v>0</v>
       </c>
       <c r="S308" t="n">
-        <v>-92.03</v>
+        <v>0</v>
       </c>
       <c r="T308" t="n">
         <v>0</v>
@@ -23239,17 +23251,17 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>MSAN4</t>
+          <t>CBMA3</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
@@ -23258,7 +23270,7 @@
         </is>
       </c>
       <c r="E309" t="n">
-        <v>6.44</v>
+        <v>0.01</v>
       </c>
       <c r="F309" t="inlineStr">
         <is>
@@ -23289,41 +23301,41 @@
         <v>0</v>
       </c>
       <c r="N309" t="n">
-        <v>2533030000</v>
+        <v>-34022300000</v>
       </c>
       <c r="O309" t="n">
         <v>0</v>
       </c>
       <c r="P309" t="n">
-        <v>6.27</v>
+        <v>0</v>
       </c>
       <c r="Q309" t="n">
-        <v>2.42</v>
+        <v>0</v>
       </c>
       <c r="R309" t="n">
-        <v>11.78</v>
+        <v>0</v>
       </c>
       <c r="S309" t="n">
-        <v>11.81</v>
+        <v>0</v>
       </c>
       <c r="T309" t="n">
-        <v>101.35</v>
+        <v>252.65</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>GALO4</t>
+          <t>ALBA3</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa ALBA</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D310" t="inlineStr">
@@ -23332,7 +23344,7 @@
         </is>
       </c>
       <c r="E310" t="n">
-        <v>0.25</v>
+        <v>2.15</v>
       </c>
       <c r="F310" t="inlineStr">
         <is>
@@ -23363,41 +23375,41 @@
         <v>0</v>
       </c>
       <c r="N310" t="n">
-        <v>-60607000</v>
+        <v>354860000</v>
       </c>
       <c r="O310" t="n">
         <v>0</v>
       </c>
       <c r="P310" t="n">
-        <v>13.98</v>
+        <v>9.5</v>
       </c>
       <c r="Q310" t="n">
-        <v>-184.58</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="R310" t="n">
-        <v>39.37</v>
+        <v>20.4</v>
       </c>
       <c r="S310" t="n">
-        <v>7.62</v>
+        <v>19.77</v>
       </c>
       <c r="T310" t="n">
-        <v>-28.97</v>
+        <v>14.69</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>BBTG13</t>
+          <t>ARPS4</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D311" t="inlineStr">
@@ -23437,36 +23449,36 @@
         <v>0</v>
       </c>
       <c r="N311" t="n">
-        <v>7000</v>
+        <v>-12690000</v>
       </c>
       <c r="O311" t="n">
         <v>0</v>
       </c>
       <c r="P311" t="n">
-        <v>0</v>
+        <v>-4.92</v>
       </c>
       <c r="Q311" t="n">
-        <v>0</v>
+        <v>-11.59</v>
       </c>
       <c r="R311" t="n">
-        <v>0</v>
+        <v>-6.64</v>
       </c>
       <c r="S311" t="n">
-        <v>-42.86</v>
+        <v>20.34</v>
       </c>
       <c r="T311" t="n">
-        <v>0</v>
+        <v>-17.53</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>INHA3</t>
+          <t>SALM3</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Empresa INHA</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -23480,7 +23492,7 @@
         </is>
       </c>
       <c r="E312" t="n">
-        <v>0</v>
+        <v>5.7</v>
       </c>
       <c r="F312" t="inlineStr">
         <is>
@@ -23511,36 +23523,36 @@
         <v>0</v>
       </c>
       <c r="N312" t="n">
-        <v>1533210000</v>
+        <v>475600000</v>
       </c>
       <c r="O312" t="n">
         <v>0</v>
       </c>
       <c r="P312" t="n">
-        <v>-56.05</v>
+        <v>10.22</v>
       </c>
       <c r="Q312" t="n">
-        <v>-124.06</v>
+        <v>4.13</v>
       </c>
       <c r="R312" t="n">
-        <v>-6.27</v>
+        <v>25.78</v>
       </c>
       <c r="S312" t="n">
-        <v>-39.87</v>
+        <v>19.53</v>
       </c>
       <c r="T312" t="n">
-        <v>-12.18</v>
+        <v>24.53</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>PTIP4</t>
+          <t>CMMA4</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa CMMA</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -23554,7 +23566,7 @@
         </is>
       </c>
       <c r="E313" t="n">
-        <v>25.15</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="F313" t="inlineStr">
         <is>
@@ -23585,36 +23597,36 @@
         <v>0</v>
       </c>
       <c r="N313" t="n">
-        <v>-155957000</v>
+        <v>-79623000</v>
       </c>
       <c r="O313" t="n">
         <v>0</v>
       </c>
       <c r="P313" t="n">
-        <v>13.73</v>
+        <v>0</v>
       </c>
       <c r="Q313" t="n">
-        <v>7.55</v>
+        <v>0</v>
       </c>
       <c r="R313" t="n">
-        <v>23.13</v>
+        <v>0</v>
       </c>
       <c r="S313" t="n">
-        <v>-121.74</v>
+        <v>-1.92</v>
       </c>
       <c r="T313" t="n">
-        <v>62.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>LATS3</t>
+          <t>CZRS3</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Empresa LATS</t>
+          <t>Empresa CZRS</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -23628,7 +23640,7 @@
         </is>
       </c>
       <c r="E314" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="F314" t="inlineStr">
         <is>
@@ -23659,36 +23671,36 @@
         <v>0</v>
       </c>
       <c r="N314" t="n">
-        <v>680646000</v>
+        <v>1145670000</v>
       </c>
       <c r="O314" t="n">
         <v>0</v>
       </c>
       <c r="P314" t="n">
-        <v>11.74</v>
+        <v>0</v>
       </c>
       <c r="Q314" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="R314" t="n">
-        <v>11.63</v>
+        <v>0</v>
       </c>
       <c r="S314" t="n">
-        <v>1.84</v>
+        <v>3.34</v>
       </c>
       <c r="T314" t="n">
-        <v>15.37</v>
+        <v>14.44</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>VSPT3</t>
+          <t>VNET3</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa VNET</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -23706,7 +23718,7 @@
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>Bens Industriais</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G315" t="n">
@@ -23721,7 +23733,7 @@
         </is>
       </c>
       <c r="J315" t="n">
-        <v>-0.43</v>
+        <v>0</v>
       </c>
       <c r="K315" t="n">
         <v>0</v>
@@ -23733,7 +23745,7 @@
         <v>0</v>
       </c>
       <c r="N315" t="n">
-        <v>5031600000</v>
+        <v>14163000000</v>
       </c>
       <c r="O315" t="n">
         <v>0</v>
@@ -23751,18 +23763,18 @@
         <v>0</v>
       </c>
       <c r="T315" t="n">
-        <v>4.92</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>SGEN4</t>
+          <t>CSPC4</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -23776,7 +23788,7 @@
         </is>
       </c>
       <c r="E316" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="F316" t="inlineStr">
         <is>
@@ -23801,42 +23813,42 @@
         <v>0</v>
       </c>
       <c r="L316" t="n">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="M316" t="n">
         <v>0</v>
       </c>
       <c r="N316" t="n">
-        <v>156981000</v>
+        <v>2126670000</v>
       </c>
       <c r="O316" t="n">
         <v>0</v>
       </c>
       <c r="P316" t="n">
-        <v>-1871.17</v>
+        <v>38.62</v>
       </c>
       <c r="Q316" t="n">
-        <v>0</v>
+        <v>18.85</v>
       </c>
       <c r="R316" t="n">
-        <v>-1.59</v>
+        <v>29.18</v>
       </c>
       <c r="S316" t="n">
-        <v>0</v>
+        <v>45.33</v>
       </c>
       <c r="T316" t="n">
-        <v>-59.85</v>
+        <v>41.15</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>SEBB3</t>
+          <t>BOVH3</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa BOVH</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -23850,7 +23862,7 @@
         </is>
       </c>
       <c r="E317" t="n">
-        <v>0</v>
+        <v>15.71</v>
       </c>
       <c r="F317" t="inlineStr">
         <is>
@@ -23875,67 +23887,67 @@
         <v>0</v>
       </c>
       <c r="L317" t="n">
-        <v>0</v>
+        <v>6.16</v>
       </c>
       <c r="M317" t="n">
         <v>0</v>
       </c>
       <c r="N317" t="n">
-        <v>145783000</v>
+        <v>1843320000</v>
       </c>
       <c r="O317" t="n">
         <v>0</v>
       </c>
       <c r="P317" t="n">
-        <v>9.24</v>
+        <v>0</v>
       </c>
       <c r="Q317" t="n">
-        <v>7.4</v>
+        <v>0</v>
       </c>
       <c r="R317" t="n">
-        <v>24.15</v>
+        <v>0</v>
       </c>
       <c r="S317" t="n">
-        <v>23.01</v>
+        <v>0</v>
       </c>
       <c r="T317" t="n">
-        <v>50.04</v>
+        <v>0</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>BBTG11</t>
+          <t>ARND3</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa ARND</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>UNT</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Tradicional</t>
+          <t>Novo Mercado</t>
         </is>
       </c>
       <c r="E318" t="n">
-        <v>15.01</v>
+        <v>0.51</v>
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Tecnologia da Informação</t>
         </is>
       </c>
       <c r="G318" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="H318" t="n">
-        <v>0</v>
+        <v>12.49</v>
       </c>
       <c r="I318" t="inlineStr">
         <is>
@@ -23949,16 +23961,16 @@
         <v>0</v>
       </c>
       <c r="L318" t="n">
-        <v>0</v>
+        <v>0.57</v>
       </c>
       <c r="M318" t="n">
         <v>0</v>
       </c>
       <c r="N318" t="n">
-        <v>0</v>
+        <v>125211000</v>
       </c>
       <c r="O318" t="n">
-        <v>0</v>
+        <v>913.58</v>
       </c>
       <c r="P318" t="n">
         <v>0</v>
@@ -23973,23 +23985,23 @@
         <v>0</v>
       </c>
       <c r="T318" t="n">
-        <v>0</v>
+        <v>-0.88</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>JFAB4</t>
+          <t>INHA3</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Empresa JFAB</t>
+          <t>Empresa INHA</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
@@ -23998,7 +24010,7 @@
         </is>
       </c>
       <c r="E319" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="F319" t="inlineStr">
         <is>
@@ -24029,36 +24041,36 @@
         <v>0</v>
       </c>
       <c r="N319" t="n">
-        <v>-10183000</v>
+        <v>1533210000</v>
       </c>
       <c r="O319" t="n">
         <v>0</v>
       </c>
       <c r="P319" t="n">
-        <v>0</v>
+        <v>-56.05</v>
       </c>
       <c r="Q319" t="n">
-        <v>0</v>
+        <v>-124.06</v>
       </c>
       <c r="R319" t="n">
-        <v>0</v>
+        <v>-6.27</v>
       </c>
       <c r="S319" t="n">
-        <v>2.34</v>
+        <v>-39.87</v>
       </c>
       <c r="T319" t="n">
-        <v>0</v>
+        <v>-12.18</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>CCHI4</t>
+          <t>PTIP4</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -24072,7 +24084,7 @@
         </is>
       </c>
       <c r="E320" t="n">
-        <v>0.02</v>
+        <v>25.15</v>
       </c>
       <c r="F320" t="inlineStr">
         <is>
@@ -24097,42 +24109,42 @@
         <v>0</v>
       </c>
       <c r="L320" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="M320" t="n">
         <v>0</v>
       </c>
       <c r="N320" t="n">
-        <v>-160477000</v>
+        <v>-155957000</v>
       </c>
       <c r="O320" t="n">
         <v>0</v>
       </c>
       <c r="P320" t="n">
-        <v>0</v>
+        <v>13.73</v>
       </c>
       <c r="Q320" t="n">
-        <v>0</v>
+        <v>7.55</v>
       </c>
       <c r="R320" t="n">
-        <v>0</v>
+        <v>23.13</v>
       </c>
       <c r="S320" t="n">
-        <v>0</v>
+        <v>-121.74</v>
       </c>
       <c r="T320" t="n">
-        <v>20.36</v>
+        <v>62.11</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>REPA3</t>
+          <t>LATS3</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa LATS</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -24146,7 +24158,7 @@
         </is>
       </c>
       <c r="E321" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="F321" t="inlineStr">
         <is>
@@ -24177,41 +24189,41 @@
         <v>0</v>
       </c>
       <c r="N321" t="n">
-        <v>378378000</v>
+        <v>680646000</v>
       </c>
       <c r="O321" t="n">
         <v>0</v>
       </c>
       <c r="P321" t="n">
-        <v>5.18</v>
+        <v>11.74</v>
       </c>
       <c r="Q321" t="n">
-        <v>1.22</v>
+        <v>1.3</v>
       </c>
       <c r="R321" t="n">
-        <v>4.05</v>
+        <v>11.63</v>
       </c>
       <c r="S321" t="n">
-        <v>1.91</v>
+        <v>1.84</v>
       </c>
       <c r="T321" t="n">
-        <v>1.09</v>
+        <v>15.37</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>EQMA5B</t>
+          <t>VVAX3</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
@@ -24251,41 +24263,41 @@
         <v>0</v>
       </c>
       <c r="N322" t="n">
-        <v>4940330000</v>
+        <v>144676000</v>
       </c>
       <c r="O322" t="n">
         <v>0</v>
       </c>
       <c r="P322" t="n">
-        <v>0</v>
+        <v>-7.36</v>
       </c>
       <c r="Q322" t="n">
-        <v>0</v>
+        <v>-37.76</v>
       </c>
       <c r="R322" t="n">
-        <v>0</v>
+        <v>-6.52</v>
       </c>
       <c r="S322" t="n">
-        <v>0</v>
+        <v>-92.03</v>
       </c>
       <c r="T322" t="n">
-        <v>9.050000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>VGOR3</t>
+          <t>MSAN4</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Empresa VGOR</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D323" t="inlineStr">
@@ -24294,7 +24306,7 @@
         </is>
       </c>
       <c r="E323" t="n">
-        <v>0</v>
+        <v>6.44</v>
       </c>
       <c r="F323" t="inlineStr">
         <is>
@@ -24325,36 +24337,36 @@
         <v>0</v>
       </c>
       <c r="N323" t="n">
-        <v>135178000</v>
+        <v>2533030000</v>
       </c>
       <c r="O323" t="n">
         <v>0</v>
       </c>
       <c r="P323" t="n">
-        <v>4.5</v>
+        <v>6.27</v>
       </c>
       <c r="Q323" t="n">
-        <v>-4.59</v>
+        <v>2.42</v>
       </c>
       <c r="R323" t="n">
-        <v>6</v>
+        <v>11.78</v>
       </c>
       <c r="S323" t="n">
-        <v>-24.29</v>
+        <v>11.81</v>
       </c>
       <c r="T323" t="n">
-        <v>4.77</v>
+        <v>101.35</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>ECIS4</t>
+          <t>GALO4</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -24368,7 +24380,7 @@
         </is>
       </c>
       <c r="E324" t="n">
-        <v>145</v>
+        <v>0.25</v>
       </c>
       <c r="F324" t="inlineStr">
         <is>
@@ -24399,36 +24411,36 @@
         <v>0</v>
       </c>
       <c r="N324" t="n">
-        <v>129346000</v>
+        <v>-60607000</v>
       </c>
       <c r="O324" t="n">
         <v>0</v>
       </c>
       <c r="P324" t="n">
-        <v>34.9</v>
+        <v>13.98</v>
       </c>
       <c r="Q324" t="n">
-        <v>14.18</v>
+        <v>-184.58</v>
       </c>
       <c r="R324" t="n">
-        <v>12.48</v>
+        <v>39.37</v>
       </c>
       <c r="S324" t="n">
-        <v>7.33</v>
+        <v>7.62</v>
       </c>
       <c r="T324" t="n">
-        <v>4.66</v>
+        <v>-28.97</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>TNEP3</t>
+          <t>BBTG13</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -24442,7 +24454,7 @@
         </is>
       </c>
       <c r="E325" t="n">
-        <v>3.01</v>
+        <v>0</v>
       </c>
       <c r="F325" t="inlineStr">
         <is>
@@ -24473,36 +24485,36 @@
         <v>0</v>
       </c>
       <c r="N325" t="n">
-        <v>955105000</v>
+        <v>7000</v>
       </c>
       <c r="O325" t="n">
         <v>0</v>
       </c>
       <c r="P325" t="n">
-        <v>20.92</v>
+        <v>0</v>
       </c>
       <c r="Q325" t="n">
-        <v>25.42</v>
+        <v>0</v>
       </c>
       <c r="R325" t="n">
-        <v>20.53</v>
+        <v>0</v>
       </c>
       <c r="S325" t="n">
-        <v>22.8</v>
+        <v>-42.86</v>
       </c>
       <c r="T325" t="n">
-        <v>8.15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>LECO3</t>
+          <t>VSPT3</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Empresa LECO</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -24520,7 +24532,7 @@
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bens Industriais</t>
         </is>
       </c>
       <c r="G326" t="n">
@@ -24535,7 +24547,7 @@
         </is>
       </c>
       <c r="J326" t="n">
-        <v>0</v>
+        <v>-0.43</v>
       </c>
       <c r="K326" t="n">
         <v>0</v>
@@ -24547,36 +24559,36 @@
         <v>0</v>
       </c>
       <c r="N326" t="n">
-        <v>105928000</v>
+        <v>5031600000</v>
       </c>
       <c r="O326" t="n">
         <v>0</v>
       </c>
       <c r="P326" t="n">
-        <v>-2.14</v>
+        <v>0</v>
       </c>
       <c r="Q326" t="n">
-        <v>-4.72</v>
+        <v>0</v>
       </c>
       <c r="R326" t="n">
-        <v>-3.48</v>
+        <v>0</v>
       </c>
       <c r="S326" t="n">
-        <v>-14.82</v>
+        <v>0</v>
       </c>
       <c r="T326" t="n">
-        <v>3.58</v>
+        <v>4.92</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>SALM4</t>
+          <t>SGEN4</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -24590,7 +24602,7 @@
         </is>
       </c>
       <c r="E327" t="n">
-        <v>5.9</v>
+        <v>0.6</v>
       </c>
       <c r="F327" t="inlineStr">
         <is>
@@ -24615,47 +24627,47 @@
         <v>0</v>
       </c>
       <c r="L327" t="n">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="M327" t="n">
         <v>0</v>
       </c>
       <c r="N327" t="n">
-        <v>475600000</v>
+        <v>156981000</v>
       </c>
       <c r="O327" t="n">
         <v>0</v>
       </c>
       <c r="P327" t="n">
-        <v>10.22</v>
+        <v>-1871.17</v>
       </c>
       <c r="Q327" t="n">
-        <v>4.13</v>
+        <v>0</v>
       </c>
       <c r="R327" t="n">
-        <v>25.78</v>
+        <v>-1.59</v>
       </c>
       <c r="S327" t="n">
-        <v>19.53</v>
+        <v>0</v>
       </c>
       <c r="T327" t="n">
-        <v>24.53</v>
+        <v>-59.85</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>BERG3</t>
+          <t>JFAB4</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Empresa BERG</t>
+          <t>Empresa JFAB</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D328" t="inlineStr">
@@ -24664,7 +24676,7 @@
         </is>
       </c>
       <c r="E328" t="n">
-        <v>33</v>
+        <v>0.06</v>
       </c>
       <c r="F328" t="inlineStr">
         <is>
@@ -24695,41 +24707,41 @@
         <v>0</v>
       </c>
       <c r="N328" t="n">
-        <v>9538000</v>
+        <v>-10183000</v>
       </c>
       <c r="O328" t="n">
         <v>0</v>
       </c>
       <c r="P328" t="n">
-        <v>-8.6</v>
+        <v>0</v>
       </c>
       <c r="Q328" t="n">
-        <v>-32.6</v>
+        <v>0</v>
       </c>
       <c r="R328" t="n">
-        <v>-5.58</v>
+        <v>0</v>
       </c>
       <c r="S328" t="n">
-        <v>-102.71</v>
+        <v>2.34</v>
       </c>
       <c r="T328" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>JBDU3</t>
+          <t>CCHI4</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Empresa JBDU</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D329" t="inlineStr">
@@ -24738,7 +24750,7 @@
         </is>
       </c>
       <c r="E329" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="F329" t="inlineStr">
         <is>
@@ -24763,13 +24775,13 @@
         <v>0</v>
       </c>
       <c r="L329" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="M329" t="n">
         <v>0</v>
       </c>
       <c r="N329" t="n">
-        <v>56569000</v>
+        <v>-160477000</v>
       </c>
       <c r="O329" t="n">
         <v>0</v>
@@ -24787,18 +24799,18 @@
         <v>0</v>
       </c>
       <c r="T329" t="n">
-        <v>0</v>
+        <v>20.36</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>EGGY3</t>
+          <t>REPA3</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Empresa EGGY</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -24812,7 +24824,7 @@
         </is>
       </c>
       <c r="E330" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F330" t="inlineStr">
         <is>
@@ -24843,41 +24855,41 @@
         <v>0</v>
       </c>
       <c r="N330" t="n">
-        <v>954480000</v>
+        <v>378378000</v>
       </c>
       <c r="O330" t="n">
         <v>0</v>
       </c>
       <c r="P330" t="n">
-        <v>0</v>
+        <v>5.18</v>
       </c>
       <c r="Q330" t="n">
-        <v>0</v>
+        <v>1.22</v>
       </c>
       <c r="R330" t="n">
-        <v>0</v>
+        <v>4.05</v>
       </c>
       <c r="S330" t="n">
-        <v>0</v>
+        <v>1.91</v>
       </c>
       <c r="T330" t="n">
-        <v>-0.82</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>CBMA4</t>
+          <t>EQMA5B</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
@@ -24886,7 +24898,7 @@
         </is>
       </c>
       <c r="E331" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="F331" t="inlineStr">
         <is>
@@ -24917,7 +24929,7 @@
         <v>0</v>
       </c>
       <c r="N331" t="n">
-        <v>-34022300000</v>
+        <v>4940330000</v>
       </c>
       <c r="O331" t="n">
         <v>0</v>
@@ -24935,18 +24947,18 @@
         <v>0</v>
       </c>
       <c r="T331" t="n">
-        <v>252.65</v>
+        <v>9.050000000000001</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>SASG3</t>
+          <t>SEBB3</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Empresa SASG</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -24960,7 +24972,7 @@
         </is>
       </c>
       <c r="E332" t="n">
-        <v>0.98</v>
+        <v>0</v>
       </c>
       <c r="F332" t="inlineStr">
         <is>
@@ -24991,41 +25003,41 @@
         <v>0</v>
       </c>
       <c r="N332" t="n">
-        <v>0</v>
+        <v>145783000</v>
       </c>
       <c r="O332" t="n">
         <v>0</v>
       </c>
       <c r="P332" t="n">
-        <v>0</v>
+        <v>9.24</v>
       </c>
       <c r="Q332" t="n">
-        <v>0</v>
+        <v>7.4</v>
       </c>
       <c r="R332" t="n">
-        <v>0</v>
+        <v>24.15</v>
       </c>
       <c r="S332" t="n">
-        <v>0</v>
+        <v>23.01</v>
       </c>
       <c r="T332" t="n">
-        <v>0</v>
+        <v>50.04</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>BMEF3</t>
+          <t>BBTG11</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Empresa BMEF</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">
@@ -25034,7 +25046,7 @@
         </is>
       </c>
       <c r="E333" t="n">
-        <v>11</v>
+        <v>15.01</v>
       </c>
       <c r="F333" t="inlineStr">
         <is>
@@ -25059,13 +25071,13 @@
         <v>0</v>
       </c>
       <c r="L333" t="n">
-        <v>4.16</v>
+        <v>0</v>
       </c>
       <c r="M333" t="n">
         <v>0</v>
       </c>
       <c r="N333" t="n">
-        <v>2674780000</v>
+        <v>0</v>
       </c>
       <c r="O333" t="n">
         <v>0</v>
@@ -25089,17 +25101,17 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>AGEI3</t>
+          <t>ECIS4</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Empresa AGEI</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
@@ -25108,7 +25120,7 @@
         </is>
       </c>
       <c r="E334" t="n">
-        <v>7.8</v>
+        <v>145</v>
       </c>
       <c r="F334" t="inlineStr">
         <is>
@@ -25133,42 +25145,42 @@
         <v>0</v>
       </c>
       <c r="L334" t="n">
-        <v>1.25</v>
+        <v>0</v>
       </c>
       <c r="M334" t="n">
         <v>0</v>
       </c>
       <c r="N334" t="n">
-        <v>1878210000</v>
+        <v>129346000</v>
       </c>
       <c r="O334" t="n">
         <v>0</v>
       </c>
       <c r="P334" t="n">
-        <v>0</v>
+        <v>34.9</v>
       </c>
       <c r="Q334" t="n">
-        <v>0</v>
+        <v>14.18</v>
       </c>
       <c r="R334" t="n">
-        <v>0</v>
+        <v>12.48</v>
       </c>
       <c r="S334" t="n">
-        <v>0</v>
+        <v>7.33</v>
       </c>
       <c r="T334" t="n">
-        <v>0</v>
+        <v>4.66</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>ARPS3</t>
+          <t>TNEP3</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -25182,7 +25194,7 @@
         </is>
       </c>
       <c r="E335" t="n">
-        <v>0.3</v>
+        <v>3.01</v>
       </c>
       <c r="F335" t="inlineStr">
         <is>
@@ -25213,36 +25225,36 @@
         <v>0</v>
       </c>
       <c r="N335" t="n">
-        <v>-12690000</v>
+        <v>955105000</v>
       </c>
       <c r="O335" t="n">
         <v>0</v>
       </c>
       <c r="P335" t="n">
-        <v>-4.92</v>
+        <v>20.92</v>
       </c>
       <c r="Q335" t="n">
-        <v>-11.59</v>
+        <v>25.42</v>
       </c>
       <c r="R335" t="n">
-        <v>-6.64</v>
+        <v>20.53</v>
       </c>
       <c r="S335" t="n">
-        <v>20.34</v>
+        <v>22.8</v>
       </c>
       <c r="T335" t="n">
-        <v>-17.53</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>ODER3</t>
+          <t>LECO3</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Empresa ODER</t>
+          <t>Empresa LECO</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -25260,14 +25272,14 @@
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>Consumo não Cíclico</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G336" t="n">
         <v>80</v>
       </c>
       <c r="H336" t="n">
-        <v>1.75</v>
+        <v>0</v>
       </c>
       <c r="I336" t="inlineStr">
         <is>
@@ -25287,41 +25299,41 @@
         <v>0</v>
       </c>
       <c r="N336" t="n">
-        <v>609518000</v>
+        <v>105928000</v>
       </c>
       <c r="O336" t="n">
         <v>0</v>
       </c>
       <c r="P336" t="n">
-        <v>0</v>
+        <v>-2.14</v>
       </c>
       <c r="Q336" t="n">
-        <v>0</v>
+        <v>-4.72</v>
       </c>
       <c r="R336" t="n">
-        <v>0</v>
+        <v>-3.48</v>
       </c>
       <c r="S336" t="n">
-        <v>0</v>
+        <v>-14.82</v>
       </c>
       <c r="T336" t="n">
-        <v>3.17</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>VVAX4</t>
+          <t>VGOR3</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa VGOR</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
@@ -25361,36 +25373,36 @@
         <v>0</v>
       </c>
       <c r="N337" t="n">
-        <v>144676000</v>
+        <v>135178000</v>
       </c>
       <c r="O337" t="n">
         <v>0</v>
       </c>
       <c r="P337" t="n">
-        <v>-7.36</v>
+        <v>4.5</v>
       </c>
       <c r="Q337" t="n">
-        <v>-37.76</v>
+        <v>-4.59</v>
       </c>
       <c r="R337" t="n">
-        <v>-6.52</v>
+        <v>6</v>
       </c>
       <c r="S337" t="n">
-        <v>-92.03</v>
+        <v>-24.29</v>
       </c>
       <c r="T337" t="n">
-        <v>0</v>
+        <v>4.77</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>CSPC3</t>
+          <t>JBDU3</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa JBDU</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -25404,7 +25416,7 @@
         </is>
       </c>
       <c r="E338" t="n">
-        <v>1.24</v>
+        <v>0</v>
       </c>
       <c r="F338" t="inlineStr">
         <is>
@@ -25435,36 +25447,36 @@
         <v>0</v>
       </c>
       <c r="N338" t="n">
-        <v>2126670000</v>
+        <v>56569000</v>
       </c>
       <c r="O338" t="n">
         <v>0</v>
       </c>
       <c r="P338" t="n">
-        <v>38.62</v>
+        <v>0</v>
       </c>
       <c r="Q338" t="n">
-        <v>18.85</v>
+        <v>0</v>
       </c>
       <c r="R338" t="n">
-        <v>29.18</v>
+        <v>0</v>
       </c>
       <c r="S338" t="n">
-        <v>45.33</v>
+        <v>0</v>
       </c>
       <c r="T338" t="n">
-        <v>41.15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>ABCB3</t>
+          <t>EGGY3</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Empresa ABCB</t>
+          <t>Empresa EGGY</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -25509,7 +25521,7 @@
         <v>0</v>
       </c>
       <c r="N339" t="n">
-        <v>7258910000</v>
+        <v>954480000</v>
       </c>
       <c r="O339" t="n">
         <v>0</v>
@@ -25524,26 +25536,26 @@
         <v>0</v>
       </c>
       <c r="S339" t="n">
-        <v>14.05</v>
+        <v>0</v>
       </c>
       <c r="T339" t="n">
-        <v>7.57</v>
+        <v>-0.82</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>CCTY3</t>
+          <t>CBMA4</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Empresa CCTY</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D340" t="inlineStr">
@@ -25552,7 +25564,7 @@
         </is>
       </c>
       <c r="E340" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="F340" t="inlineStr">
         <is>
@@ -25583,7 +25595,7 @@
         <v>0</v>
       </c>
       <c r="N340" t="n">
-        <v>0</v>
+        <v>-34022300000</v>
       </c>
       <c r="O340" t="n">
         <v>0</v>
@@ -25601,18 +25613,18 @@
         <v>0</v>
       </c>
       <c r="T340" t="n">
-        <v>0</v>
+        <v>252.65</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>VSPT4</t>
+          <t>SALM4</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -25626,11 +25638,11 @@
         </is>
       </c>
       <c r="E341" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t>Bens Industriais</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G341" t="n">
@@ -25645,7 +25657,7 @@
         </is>
       </c>
       <c r="J341" t="n">
-        <v>-0.43</v>
+        <v>0</v>
       </c>
       <c r="K341" t="n">
         <v>0</v>
@@ -25657,41 +25669,41 @@
         <v>0</v>
       </c>
       <c r="N341" t="n">
-        <v>5031600000</v>
+        <v>475600000</v>
       </c>
       <c r="O341" t="n">
         <v>0</v>
       </c>
       <c r="P341" t="n">
-        <v>0</v>
+        <v>10.22</v>
       </c>
       <c r="Q341" t="n">
-        <v>0</v>
+        <v>4.13</v>
       </c>
       <c r="R341" t="n">
-        <v>0</v>
+        <v>25.78</v>
       </c>
       <c r="S341" t="n">
-        <v>0</v>
+        <v>19.53</v>
       </c>
       <c r="T341" t="n">
-        <v>4.92</v>
+        <v>24.53</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>BAUH4</t>
+          <t>BERG3</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Empresa BAUH</t>
+          <t>Empresa BERG</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D342" t="inlineStr">
@@ -25700,18 +25712,18 @@
         </is>
       </c>
       <c r="E342" t="n">
-        <v>93.39</v>
+        <v>33</v>
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>Consumo não Cíclico</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G342" t="n">
         <v>80</v>
       </c>
       <c r="H342" t="n">
-        <v>28.89</v>
+        <v>0</v>
       </c>
       <c r="I342" t="inlineStr">
         <is>
@@ -25719,48 +25731,48 @@
         </is>
       </c>
       <c r="J342" t="n">
-        <v>-2.88</v>
+        <v>0</v>
       </c>
       <c r="K342" t="n">
         <v>0</v>
       </c>
       <c r="L342" t="n">
-        <v>3.18</v>
+        <v>0</v>
       </c>
       <c r="M342" t="n">
-        <v>1.16</v>
+        <v>0</v>
       </c>
       <c r="N342" t="n">
-        <v>153407000</v>
+        <v>9538000</v>
       </c>
       <c r="O342" t="n">
-        <v>207.53</v>
+        <v>0</v>
       </c>
       <c r="P342" t="n">
-        <v>0</v>
+        <v>-8.6</v>
       </c>
       <c r="Q342" t="n">
-        <v>0</v>
+        <v>-32.6</v>
       </c>
       <c r="R342" t="n">
-        <v>0</v>
+        <v>-5.58</v>
       </c>
       <c r="S342" t="n">
-        <v>0</v>
+        <v>-102.71</v>
       </c>
       <c r="T342" t="n">
-        <v>13.32</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>ICPI3</t>
+          <t>AGEI3</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Empresa ICPI</t>
+          <t>Empresa AGEI</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -25774,7 +25786,7 @@
         </is>
       </c>
       <c r="E343" t="n">
-        <v>0</v>
+        <v>7.8</v>
       </c>
       <c r="F343" t="inlineStr">
         <is>
@@ -25799,13 +25811,13 @@
         <v>0</v>
       </c>
       <c r="L343" t="n">
-        <v>0</v>
+        <v>1.25</v>
       </c>
       <c r="M343" t="n">
         <v>0</v>
       </c>
       <c r="N343" t="n">
-        <v>0</v>
+        <v>1878210000</v>
       </c>
       <c r="O343" t="n">
         <v>0</v>
@@ -25829,17 +25841,17 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>ILLS4</t>
+          <t>SASG3</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Empresa ILLS</t>
+          <t>Empresa SASG</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D344" t="inlineStr">
@@ -25848,7 +25860,7 @@
         </is>
       </c>
       <c r="E344" t="n">
-        <v>100.01</v>
+        <v>0.98</v>
       </c>
       <c r="F344" t="inlineStr">
         <is>
@@ -25879,41 +25891,41 @@
         <v>0</v>
       </c>
       <c r="N344" t="n">
-        <v>-18567000</v>
+        <v>0</v>
       </c>
       <c r="O344" t="n">
         <v>0</v>
       </c>
       <c r="P344" t="n">
-        <v>8.43</v>
+        <v>0</v>
       </c>
       <c r="Q344" t="n">
-        <v>-10.22</v>
+        <v>0</v>
       </c>
       <c r="R344" t="n">
-        <v>8.140000000000001</v>
+        <v>0</v>
       </c>
       <c r="S344" t="n">
-        <v>36.09</v>
+        <v>0</v>
       </c>
       <c r="T344" t="n">
-        <v>9.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>ESTC4</t>
+          <t>BMEF3</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Empresa ESTC</t>
+          <t>Empresa BMEF</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D345" t="inlineStr">
@@ -25922,7 +25934,7 @@
         </is>
       </c>
       <c r="E345" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F345" t="inlineStr">
         <is>
@@ -25947,47 +25959,47 @@
         <v>0</v>
       </c>
       <c r="L345" t="n">
-        <v>0</v>
+        <v>4.16</v>
       </c>
       <c r="M345" t="n">
         <v>0</v>
       </c>
       <c r="N345" t="n">
-        <v>2916530000</v>
+        <v>2674780000</v>
       </c>
       <c r="O345" t="n">
         <v>0</v>
       </c>
       <c r="P345" t="n">
-        <v>16.91</v>
+        <v>0</v>
       </c>
       <c r="Q345" t="n">
-        <v>2.02</v>
+        <v>0</v>
       </c>
       <c r="R345" t="n">
-        <v>11.35</v>
+        <v>0</v>
       </c>
       <c r="S345" t="n">
-        <v>3.89</v>
+        <v>0</v>
       </c>
       <c r="T345" t="n">
-        <v>5.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>SEBB4</t>
+          <t>ARPS3</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D346" t="inlineStr">
@@ -25996,7 +26008,7 @@
         </is>
       </c>
       <c r="E346" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="F346" t="inlineStr">
         <is>
@@ -26027,36 +26039,36 @@
         <v>0</v>
       </c>
       <c r="N346" t="n">
-        <v>145783000</v>
+        <v>-12690000</v>
       </c>
       <c r="O346" t="n">
         <v>0</v>
       </c>
       <c r="P346" t="n">
-        <v>9.24</v>
+        <v>-4.92</v>
       </c>
       <c r="Q346" t="n">
-        <v>7.4</v>
+        <v>-11.59</v>
       </c>
       <c r="R346" t="n">
-        <v>24.15</v>
+        <v>-6.64</v>
       </c>
       <c r="S346" t="n">
-        <v>23.01</v>
+        <v>20.34</v>
       </c>
       <c r="T346" t="n">
-        <v>50.04</v>
+        <v>-17.53</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>MSAN3</t>
+          <t>ODER3</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa ODER</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
@@ -26070,18 +26082,18 @@
         </is>
       </c>
       <c r="E347" t="n">
-        <v>6.44</v>
+        <v>0</v>
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Consumo não Cíclico</t>
         </is>
       </c>
       <c r="G347" t="n">
         <v>80</v>
       </c>
       <c r="H347" t="n">
-        <v>0</v>
+        <v>1.75</v>
       </c>
       <c r="I347" t="inlineStr">
         <is>
@@ -26101,36 +26113,36 @@
         <v>0</v>
       </c>
       <c r="N347" t="n">
-        <v>2533030000</v>
+        <v>609518000</v>
       </c>
       <c r="O347" t="n">
         <v>0</v>
       </c>
       <c r="P347" t="n">
-        <v>6.27</v>
+        <v>0</v>
       </c>
       <c r="Q347" t="n">
-        <v>2.42</v>
+        <v>0</v>
       </c>
       <c r="R347" t="n">
-        <v>11.78</v>
+        <v>0</v>
       </c>
       <c r="S347" t="n">
-        <v>11.81</v>
+        <v>0</v>
       </c>
       <c r="T347" t="n">
-        <v>101.35</v>
+        <v>3.17</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>GALO3</t>
+          <t>ABCB3</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa ABCB</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
@@ -26175,36 +26187,36 @@
         <v>0</v>
       </c>
       <c r="N348" t="n">
-        <v>-60607000</v>
+        <v>7258910000</v>
       </c>
       <c r="O348" t="n">
         <v>0</v>
       </c>
       <c r="P348" t="n">
-        <v>13.98</v>
+        <v>0</v>
       </c>
       <c r="Q348" t="n">
-        <v>-184.58</v>
+        <v>0</v>
       </c>
       <c r="R348" t="n">
-        <v>39.37</v>
+        <v>0</v>
       </c>
       <c r="S348" t="n">
-        <v>7.62</v>
+        <v>14.05</v>
       </c>
       <c r="T348" t="n">
-        <v>-28.97</v>
+        <v>7.57</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>SLCP3</t>
+          <t>CCTY3</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Empresa SLCP</t>
+          <t>Empresa CCTY</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
@@ -26218,7 +26230,7 @@
         </is>
       </c>
       <c r="E349" t="n">
-        <v>610.02</v>
+        <v>0</v>
       </c>
       <c r="F349" t="inlineStr">
         <is>
@@ -26273,17 +26285,17 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>DAYC3</t>
+          <t>VVAX4</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Empresa DAYC</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D350" t="inlineStr">
@@ -26323,36 +26335,36 @@
         <v>0</v>
       </c>
       <c r="N350" t="n">
-        <v>3009030000</v>
+        <v>144676000</v>
       </c>
       <c r="O350" t="n">
         <v>0</v>
       </c>
       <c r="P350" t="n">
-        <v>0</v>
+        <v>-7.36</v>
       </c>
       <c r="Q350" t="n">
-        <v>0</v>
+        <v>-37.76</v>
       </c>
       <c r="R350" t="n">
-        <v>0</v>
+        <v>-6.52</v>
       </c>
       <c r="S350" t="n">
-        <v>17.33</v>
+        <v>-92.03</v>
       </c>
       <c r="T350" t="n">
-        <v>8.15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>PTIP3</t>
+          <t>CSPC3</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -26366,7 +26378,7 @@
         </is>
       </c>
       <c r="E351" t="n">
-        <v>22</v>
+        <v>1.24</v>
       </c>
       <c r="F351" t="inlineStr">
         <is>
@@ -26397,36 +26409,36 @@
         <v>0</v>
       </c>
       <c r="N351" t="n">
-        <v>-155957000</v>
+        <v>2126670000</v>
       </c>
       <c r="O351" t="n">
         <v>0</v>
       </c>
       <c r="P351" t="n">
-        <v>13.73</v>
+        <v>38.62</v>
       </c>
       <c r="Q351" t="n">
-        <v>7.55</v>
+        <v>18.85</v>
       </c>
       <c r="R351" t="n">
-        <v>23.13</v>
+        <v>29.18</v>
       </c>
       <c r="S351" t="n">
-        <v>-121.74</v>
+        <v>45.33</v>
       </c>
       <c r="T351" t="n">
-        <v>62.11</v>
+        <v>41.15</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>REPA4</t>
+          <t>ESTC4</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa ESTC</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -26440,7 +26452,7 @@
         </is>
       </c>
       <c r="E352" t="n">
-        <v>1.08</v>
+        <v>0</v>
       </c>
       <c r="F352" t="inlineStr">
         <is>
@@ -26471,41 +26483,41 @@
         <v>0</v>
       </c>
       <c r="N352" t="n">
-        <v>378378000</v>
+        <v>2916530000</v>
       </c>
       <c r="O352" t="n">
         <v>0</v>
       </c>
       <c r="P352" t="n">
-        <v>5.18</v>
+        <v>16.91</v>
       </c>
       <c r="Q352" t="n">
-        <v>1.22</v>
+        <v>2.02</v>
       </c>
       <c r="R352" t="n">
-        <v>4.05</v>
+        <v>11.35</v>
       </c>
       <c r="S352" t="n">
-        <v>1.91</v>
+        <v>3.89</v>
       </c>
       <c r="T352" t="n">
-        <v>1.09</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>EQMA6B</t>
+          <t>VSPT4</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D353" t="inlineStr">
@@ -26518,7 +26530,7 @@
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bens Industriais</t>
         </is>
       </c>
       <c r="G353" t="n">
@@ -26533,7 +26545,7 @@
         </is>
       </c>
       <c r="J353" t="n">
-        <v>0</v>
+        <v>-0.43</v>
       </c>
       <c r="K353" t="n">
         <v>0</v>
@@ -26545,7 +26557,7 @@
         <v>0</v>
       </c>
       <c r="N353" t="n">
-        <v>4940330000</v>
+        <v>5031600000</v>
       </c>
       <c r="O353" t="n">
         <v>0</v>
@@ -26563,23 +26575,23 @@
         <v>0</v>
       </c>
       <c r="T353" t="n">
-        <v>9.050000000000001</v>
+        <v>4.92</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>MLPA3</t>
+          <t>BAUH4</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Empresa MLPA</t>
+          <t>Empresa BAUH</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D354" t="inlineStr">
@@ -26588,18 +26600,18 @@
         </is>
       </c>
       <c r="E354" t="n">
-        <v>0</v>
+        <v>93.39</v>
       </c>
       <c r="F354" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Consumo não Cíclico</t>
         </is>
       </c>
       <c r="G354" t="n">
         <v>80</v>
       </c>
       <c r="H354" t="n">
-        <v>0</v>
+        <v>28.89</v>
       </c>
       <c r="I354" t="inlineStr">
         <is>
@@ -26607,58 +26619,58 @@
         </is>
       </c>
       <c r="J354" t="n">
-        <v>0</v>
+        <v>-2.88</v>
       </c>
       <c r="K354" t="n">
         <v>0</v>
       </c>
       <c r="L354" t="n">
-        <v>0</v>
+        <v>3.18</v>
       </c>
       <c r="M354" t="n">
-        <v>0</v>
+        <v>1.16</v>
       </c>
       <c r="N354" t="n">
-        <v>44578000</v>
+        <v>153407000</v>
       </c>
       <c r="O354" t="n">
-        <v>0</v>
+        <v>207.53</v>
       </c>
       <c r="P354" t="n">
-        <v>6.66</v>
+        <v>0</v>
       </c>
       <c r="Q354" t="n">
-        <v>8.92</v>
+        <v>0</v>
       </c>
       <c r="R354" t="n">
         <v>0</v>
       </c>
       <c r="S354" t="n">
-        <v>45.13</v>
+        <v>0</v>
       </c>
       <c r="T354" t="n">
-        <v>-7.51</v>
+        <v>13.32</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>CLSC6</t>
+          <t>ICPI3</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Empresa CLSC</t>
+          <t>Empresa ICPI</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>Nível 2</t>
+          <t>Tradicional</t>
         </is>
       </c>
       <c r="E355" t="n">
@@ -26666,22 +26678,22 @@
       </c>
       <c r="F355" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G355" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="H355" t="n">
-        <v>75.73</v>
+        <v>0</v>
       </c>
       <c r="I355" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="J355" t="n">
-        <v>2.73</v>
+        <v>0</v>
       </c>
       <c r="K355" t="n">
         <v>0</v>
@@ -26693,7 +26705,7 @@
         <v>0</v>
       </c>
       <c r="N355" t="n">
-        <v>4228180000</v>
+        <v>0</v>
       </c>
       <c r="O355" t="n">
         <v>0</v>
@@ -26711,23 +26723,23 @@
         <v>0</v>
       </c>
       <c r="T355" t="n">
-        <v>2.82</v>
+        <v>0</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>SGEN3</t>
+          <t>ILLS4</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa ILLS</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D356" t="inlineStr">
@@ -26736,7 +26748,7 @@
         </is>
       </c>
       <c r="E356" t="n">
-        <v>5</v>
+        <v>100.01</v>
       </c>
       <c r="F356" t="inlineStr">
         <is>
@@ -26761,47 +26773,47 @@
         <v>0</v>
       </c>
       <c r="L356" t="n">
-        <v>0.77</v>
+        <v>0</v>
       </c>
       <c r="M356" t="n">
         <v>0</v>
       </c>
       <c r="N356" t="n">
-        <v>156981000</v>
+        <v>-18567000</v>
       </c>
       <c r="O356" t="n">
         <v>0</v>
       </c>
       <c r="P356" t="n">
-        <v>-1871.17</v>
+        <v>8.43</v>
       </c>
       <c r="Q356" t="n">
-        <v>0</v>
+        <v>-10.22</v>
       </c>
       <c r="R356" t="n">
-        <v>-1.59</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="S356" t="n">
-        <v>0</v>
+        <v>36.09</v>
       </c>
       <c r="T356" t="n">
-        <v>-59.85</v>
+        <v>9.33</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>DUFB11</t>
+          <t>PTIP3</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Empresa DUFB</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>UNT</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D357" t="inlineStr">
@@ -26810,7 +26822,7 @@
         </is>
       </c>
       <c r="E357" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F357" t="inlineStr">
         <is>
@@ -26841,36 +26853,36 @@
         <v>0</v>
       </c>
       <c r="N357" t="n">
-        <v>0</v>
+        <v>-155957000</v>
       </c>
       <c r="O357" t="n">
         <v>0</v>
       </c>
       <c r="P357" t="n">
-        <v>0</v>
+        <v>13.73</v>
       </c>
       <c r="Q357" t="n">
-        <v>0</v>
+        <v>7.55</v>
       </c>
       <c r="R357" t="n">
-        <v>0</v>
+        <v>23.13</v>
       </c>
       <c r="S357" t="n">
-        <v>0</v>
+        <v>-121.74</v>
       </c>
       <c r="T357" t="n">
-        <v>0</v>
+        <v>62.11</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>TNEP4</t>
+          <t>REPA4</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -26884,7 +26896,7 @@
         </is>
       </c>
       <c r="E358" t="n">
-        <v>3.95</v>
+        <v>1.08</v>
       </c>
       <c r="F358" t="inlineStr">
         <is>
@@ -26915,41 +26927,41 @@
         <v>0</v>
       </c>
       <c r="N358" t="n">
-        <v>955105000</v>
+        <v>378378000</v>
       </c>
       <c r="O358" t="n">
         <v>0</v>
       </c>
       <c r="P358" t="n">
-        <v>20.92</v>
+        <v>5.18</v>
       </c>
       <c r="Q358" t="n">
-        <v>25.42</v>
+        <v>1.22</v>
       </c>
       <c r="R358" t="n">
-        <v>20.53</v>
+        <v>4.05</v>
       </c>
       <c r="S358" t="n">
-        <v>22.8</v>
+        <v>1.91</v>
       </c>
       <c r="T358" t="n">
-        <v>8.15</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>CCHI3</t>
+          <t>EQMA6B</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
@@ -26958,7 +26970,7 @@
         </is>
       </c>
       <c r="E359" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="F359" t="inlineStr">
         <is>
@@ -26983,13 +26995,13 @@
         <v>0</v>
       </c>
       <c r="L359" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="M359" t="n">
         <v>0</v>
       </c>
       <c r="N359" t="n">
-        <v>-160477000</v>
+        <v>4940330000</v>
       </c>
       <c r="O359" t="n">
         <v>0</v>
@@ -27007,23 +27019,23 @@
         <v>0</v>
       </c>
       <c r="T359" t="n">
-        <v>20.36</v>
+        <v>9.050000000000001</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>SFSA3</t>
+          <t>SEBB4</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Empresa SFSA</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D360" t="inlineStr">
@@ -27063,36 +27075,36 @@
         <v>0</v>
       </c>
       <c r="N360" t="n">
-        <v>739524000</v>
+        <v>145783000</v>
       </c>
       <c r="O360" t="n">
         <v>0</v>
       </c>
       <c r="P360" t="n">
-        <v>0</v>
+        <v>9.24</v>
       </c>
       <c r="Q360" t="n">
-        <v>0</v>
+        <v>7.4</v>
       </c>
       <c r="R360" t="n">
-        <v>0</v>
+        <v>24.15</v>
       </c>
       <c r="S360" t="n">
-        <v>6.25</v>
+        <v>23.01</v>
       </c>
       <c r="T360" t="n">
-        <v>0.15</v>
+        <v>50.04</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>PRBC3</t>
+          <t>MSAN3</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Empresa PRBC</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -27106,7 +27118,7 @@
         </is>
       </c>
       <c r="E361" t="n">
-        <v>0</v>
+        <v>6.44</v>
       </c>
       <c r="F361" t="inlineStr">
         <is>
@@ -27137,36 +27149,36 @@
         <v>0</v>
       </c>
       <c r="N361" t="n">
-        <v>1319270000</v>
+        <v>2533030000</v>
       </c>
       <c r="O361" t="n">
         <v>0</v>
       </c>
       <c r="P361" t="n">
-        <v>0</v>
+        <v>6.27</v>
       </c>
       <c r="Q361" t="n">
-        <v>0</v>
+        <v>2.42</v>
       </c>
       <c r="R361" t="n">
-        <v>0</v>
+        <v>11.78</v>
       </c>
       <c r="S361" t="n">
-        <v>8.27</v>
+        <v>11.81</v>
       </c>
       <c r="T361" t="n">
-        <v>-1.98</v>
+        <v>101.35</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>ECIS3</t>
+          <t>GALO3</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -27180,7 +27192,7 @@
         </is>
       </c>
       <c r="E362" t="n">
-        <v>211.65</v>
+        <v>0</v>
       </c>
       <c r="F362" t="inlineStr">
         <is>
@@ -27211,41 +27223,41 @@
         <v>0</v>
       </c>
       <c r="N362" t="n">
-        <v>129346000</v>
+        <v>-60607000</v>
       </c>
       <c r="O362" t="n">
         <v>0</v>
       </c>
       <c r="P362" t="n">
-        <v>34.9</v>
+        <v>13.98</v>
       </c>
       <c r="Q362" t="n">
-        <v>14.18</v>
+        <v>-184.58</v>
       </c>
       <c r="R362" t="n">
-        <v>12.48</v>
+        <v>39.37</v>
       </c>
       <c r="S362" t="n">
-        <v>7.33</v>
+        <v>7.62</v>
       </c>
       <c r="T362" t="n">
-        <v>4.66</v>
+        <v>-28.97</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>ARPS4</t>
+          <t>SLCP3</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa SLCP</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D363" t="inlineStr">
@@ -27254,7 +27266,7 @@
         </is>
       </c>
       <c r="E363" t="n">
-        <v>0</v>
+        <v>610.02</v>
       </c>
       <c r="F363" t="inlineStr">
         <is>
@@ -27285,36 +27297,36 @@
         <v>0</v>
       </c>
       <c r="N363" t="n">
-        <v>-12690000</v>
+        <v>0</v>
       </c>
       <c r="O363" t="n">
         <v>0</v>
       </c>
       <c r="P363" t="n">
-        <v>-4.92</v>
+        <v>0</v>
       </c>
       <c r="Q363" t="n">
-        <v>-11.59</v>
+        <v>0</v>
       </c>
       <c r="R363" t="n">
-        <v>-6.64</v>
+        <v>0</v>
       </c>
       <c r="S363" t="n">
-        <v>20.34</v>
+        <v>0</v>
       </c>
       <c r="T363" t="n">
-        <v>-17.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>SALM3</t>
+          <t>DAYC3</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa DAYC</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -27328,7 +27340,7 @@
         </is>
       </c>
       <c r="E364" t="n">
-        <v>5.7</v>
+        <v>0</v>
       </c>
       <c r="F364" t="inlineStr">
         <is>
@@ -27359,41 +27371,41 @@
         <v>0</v>
       </c>
       <c r="N364" t="n">
-        <v>475600000</v>
+        <v>3009030000</v>
       </c>
       <c r="O364" t="n">
         <v>0</v>
       </c>
       <c r="P364" t="n">
-        <v>10.22</v>
+        <v>0</v>
       </c>
       <c r="Q364" t="n">
-        <v>4.13</v>
+        <v>0</v>
       </c>
       <c r="R364" t="n">
-        <v>25.78</v>
+        <v>0</v>
       </c>
       <c r="S364" t="n">
-        <v>19.53</v>
+        <v>17.33</v>
       </c>
       <c r="T364" t="n">
-        <v>24.53</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>CMMA4</t>
+          <t>DUFB11</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Empresa CMMA</t>
+          <t>Empresa DUFB</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
@@ -27402,7 +27414,7 @@
         </is>
       </c>
       <c r="E365" t="n">
-        <v>0.8100000000000001</v>
+        <v>0</v>
       </c>
       <c r="F365" t="inlineStr">
         <is>
@@ -27433,7 +27445,7 @@
         <v>0</v>
       </c>
       <c r="N365" t="n">
-        <v>-79623000</v>
+        <v>0</v>
       </c>
       <c r="O365" t="n">
         <v>0</v>
@@ -27448,7 +27460,7 @@
         <v>0</v>
       </c>
       <c r="S365" t="n">
-        <v>-1.92</v>
+        <v>0</v>
       </c>
       <c r="T365" t="n">
         <v>0</v>
@@ -27457,17 +27469,17 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>CZRS3</t>
+          <t>TNEP4</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Empresa CZRS</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D366" t="inlineStr">
@@ -27476,7 +27488,7 @@
         </is>
       </c>
       <c r="E366" t="n">
-        <v>0</v>
+        <v>3.95</v>
       </c>
       <c r="F366" t="inlineStr">
         <is>
@@ -27507,36 +27519,36 @@
         <v>0</v>
       </c>
       <c r="N366" t="n">
-        <v>1145670000</v>
+        <v>955105000</v>
       </c>
       <c r="O366" t="n">
         <v>0</v>
       </c>
       <c r="P366" t="n">
-        <v>0</v>
+        <v>20.92</v>
       </c>
       <c r="Q366" t="n">
-        <v>0</v>
+        <v>25.42</v>
       </c>
       <c r="R366" t="n">
-        <v>0</v>
+        <v>20.53</v>
       </c>
       <c r="S366" t="n">
-        <v>3.34</v>
+        <v>22.8</v>
       </c>
       <c r="T366" t="n">
-        <v>14.44</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>BPNM3</t>
+          <t>MLPA3</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Empresa BPNM</t>
+          <t>Empresa MLPA</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -27581,69 +27593,69 @@
         <v>0</v>
       </c>
       <c r="N367" t="n">
-        <v>7792670000</v>
+        <v>44578000</v>
       </c>
       <c r="O367" t="n">
         <v>0</v>
       </c>
       <c r="P367" t="n">
-        <v>0</v>
+        <v>6.66</v>
       </c>
       <c r="Q367" t="n">
-        <v>0</v>
+        <v>8.92</v>
       </c>
       <c r="R367" t="n">
         <v>0</v>
       </c>
       <c r="S367" t="n">
-        <v>9.67</v>
+        <v>45.13</v>
       </c>
       <c r="T367" t="n">
-        <v>-1.53</v>
+        <v>-7.51</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>BSGR3</t>
+          <t>CLSC6</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Empresa BSGR</t>
+          <t>Empresa CLSC</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>Tradicional</t>
+          <t>Nível 2</t>
         </is>
       </c>
       <c r="E368" t="n">
-        <v>1091.28</v>
+        <v>0</v>
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Utilidade Pública</t>
         </is>
       </c>
       <c r="G368" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="H368" t="n">
-        <v>0</v>
+        <v>75.73</v>
       </c>
       <c r="I368" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="J368" t="n">
-        <v>0</v>
+        <v>2.73</v>
       </c>
       <c r="K368" t="n">
         <v>0</v>
@@ -27655,7 +27667,7 @@
         <v>0</v>
       </c>
       <c r="N368" t="n">
-        <v>0</v>
+        <v>4228180000</v>
       </c>
       <c r="O368" t="n">
         <v>0</v>
@@ -27673,18 +27685,18 @@
         <v>0</v>
       </c>
       <c r="T368" t="n">
-        <v>0</v>
+        <v>2.82</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>CBMA3</t>
+          <t>SGEN3</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -27698,7 +27710,7 @@
         </is>
       </c>
       <c r="E369" t="n">
-        <v>0.01</v>
+        <v>5</v>
       </c>
       <c r="F369" t="inlineStr">
         <is>
@@ -27723,42 +27735,42 @@
         <v>0</v>
       </c>
       <c r="L369" t="n">
-        <v>0</v>
+        <v>0.77</v>
       </c>
       <c r="M369" t="n">
         <v>0</v>
       </c>
       <c r="N369" t="n">
-        <v>-34022300000</v>
+        <v>156981000</v>
       </c>
       <c r="O369" t="n">
         <v>0</v>
       </c>
       <c r="P369" t="n">
-        <v>0</v>
+        <v>-1871.17</v>
       </c>
       <c r="Q369" t="n">
         <v>0</v>
       </c>
       <c r="R369" t="n">
-        <v>0</v>
+        <v>-1.59</v>
       </c>
       <c r="S369" t="n">
         <v>0</v>
       </c>
       <c r="T369" t="n">
-        <v>252.65</v>
+        <v>-59.85</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>ALBA3</t>
+          <t>CCHI3</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Empresa ALBA</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -27772,7 +27784,7 @@
         </is>
       </c>
       <c r="E370" t="n">
-        <v>2.15</v>
+        <v>0.02</v>
       </c>
       <c r="F370" t="inlineStr">
         <is>
@@ -27797,42 +27809,42 @@
         <v>0</v>
       </c>
       <c r="L370" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="M370" t="n">
         <v>0</v>
       </c>
       <c r="N370" t="n">
-        <v>354860000</v>
+        <v>-160477000</v>
       </c>
       <c r="O370" t="n">
         <v>0</v>
       </c>
       <c r="P370" t="n">
-        <v>9.5</v>
+        <v>0</v>
       </c>
       <c r="Q370" t="n">
-        <v>9.619999999999999</v>
+        <v>0</v>
       </c>
       <c r="R370" t="n">
-        <v>20.4</v>
+        <v>0</v>
       </c>
       <c r="S370" t="n">
-        <v>19.77</v>
+        <v>0</v>
       </c>
       <c r="T370" t="n">
-        <v>14.69</v>
+        <v>20.36</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>VNET3</t>
+          <t>PRBC3</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Empresa VNET</t>
+          <t>Empresa PRBC</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
@@ -27877,7 +27889,7 @@
         <v>0</v>
       </c>
       <c r="N371" t="n">
-        <v>14163000000</v>
+        <v>1319270000</v>
       </c>
       <c r="O371" t="n">
         <v>0</v>
@@ -27892,26 +27904,26 @@
         <v>0</v>
       </c>
       <c r="S371" t="n">
-        <v>0</v>
+        <v>8.27</v>
       </c>
       <c r="T371" t="n">
-        <v>1.08</v>
+        <v>-1.98</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>CSPC4</t>
+          <t>ECIS3</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D372" t="inlineStr">
@@ -27920,7 +27932,7 @@
         </is>
       </c>
       <c r="E372" t="n">
-        <v>1.2</v>
+        <v>211.65</v>
       </c>
       <c r="F372" t="inlineStr">
         <is>
@@ -27951,36 +27963,36 @@
         <v>0</v>
       </c>
       <c r="N372" t="n">
-        <v>2126670000</v>
+        <v>129346000</v>
       </c>
       <c r="O372" t="n">
         <v>0</v>
       </c>
       <c r="P372" t="n">
-        <v>38.62</v>
+        <v>34.9</v>
       </c>
       <c r="Q372" t="n">
-        <v>18.85</v>
+        <v>14.18</v>
       </c>
       <c r="R372" t="n">
-        <v>29.18</v>
+        <v>12.48</v>
       </c>
       <c r="S372" t="n">
-        <v>45.33</v>
+        <v>7.33</v>
       </c>
       <c r="T372" t="n">
-        <v>41.15</v>
+        <v>4.66</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>BOVH3</t>
+          <t>SFSA3</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Empresa BOVH</t>
+          <t>Empresa SFSA</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
@@ -27994,7 +28006,7 @@
         </is>
       </c>
       <c r="E373" t="n">
-        <v>15.71</v>
+        <v>0</v>
       </c>
       <c r="F373" t="inlineStr">
         <is>
@@ -28019,13 +28031,13 @@
         <v>0</v>
       </c>
       <c r="L373" t="n">
-        <v>6.16</v>
+        <v>0</v>
       </c>
       <c r="M373" t="n">
         <v>0</v>
       </c>
       <c r="N373" t="n">
-        <v>1843320000</v>
+        <v>739524000</v>
       </c>
       <c r="O373" t="n">
         <v>0</v>
@@ -28040,10 +28052,10 @@
         <v>0</v>
       </c>
       <c r="S373" t="n">
-        <v>0</v>
+        <v>6.25</v>
       </c>
       <c r="T373" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="374">
@@ -44699,7 +44711,7 @@
     <row r="599">
       <c r="A599" t="inlineStr">
         <is>
-          <t>RPAD3</t>
+          <t>RPAD6</t>
         </is>
       </c>
       <c r="B599" t="inlineStr">
@@ -44709,7 +44721,7 @@
       </c>
       <c r="C599" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D599" t="inlineStr">
@@ -44746,13 +44758,13 @@
         <v>0.57</v>
       </c>
       <c r="M599" t="n">
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="N599" t="n">
         <v>1046150000</v>
       </c>
       <c r="O599" t="n">
-        <v>2695.56</v>
+        <v>2752.22</v>
       </c>
       <c r="P599" t="n">
         <v>0</v>
@@ -44773,7 +44785,7 @@
     <row r="600">
       <c r="A600" t="inlineStr">
         <is>
-          <t>RPAD6</t>
+          <t>RPAD3</t>
         </is>
       </c>
       <c r="B600" t="inlineStr">
@@ -44783,7 +44795,7 @@
       </c>
       <c r="C600" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D600" t="inlineStr">
@@ -44820,13 +44832,13 @@
         <v>0.57</v>
       </c>
       <c r="M600" t="n">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="N600" t="n">
         <v>1046150000</v>
       </c>
       <c r="O600" t="n">
-        <v>2752.22</v>
+        <v>2695.56</v>
       </c>
       <c r="P600" t="n">
         <v>0</v>
@@ -71635,7 +71647,7 @@
     <row r="963">
       <c r="A963" t="inlineStr">
         <is>
-          <t>PQUN4</t>
+          <t>PQUN3</t>
         </is>
       </c>
       <c r="B963" t="inlineStr">
@@ -71645,7 +71657,7 @@
       </c>
       <c r="C963" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D963" t="inlineStr">
@@ -71709,7 +71721,7 @@
     <row r="964">
       <c r="A964" t="inlineStr">
         <is>
-          <t>PQUN3</t>
+          <t>PQUN4</t>
         </is>
       </c>
       <c r="B964" t="inlineStr">
@@ -71719,7 +71731,7 @@
       </c>
       <c r="C964" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D964" t="inlineStr">

</xml_diff>

<commit_message>
Adiciona setores perenes B.E.S.T e botão de exportar para Excel
</commit_message>
<xml_diff>
--- a/acoes_b3.xlsx
+++ b/acoes_b3.xlsx
@@ -766,7 +766,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Seguradoras</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -965,17 +965,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CSTB3</t>
+          <t>CFLU4</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa CFLU</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -984,7 +984,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>150</v>
+        <v>1000</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1015,41 +1015,41 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>8420670000</v>
+        <v>60351000</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>40.85</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="Q8" t="n">
-        <v>28.98</v>
+        <v>10.72</v>
       </c>
       <c r="R8" t="n">
-        <v>22.4</v>
+        <v>17.68</v>
       </c>
       <c r="S8" t="n">
-        <v>20.11</v>
+        <v>32.15</v>
       </c>
       <c r="T8" t="n">
-        <v>31.91</v>
+        <v>8.140000000000001</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CFLU4</t>
+          <t>CSTB3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Empresa CFLU</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1058,7 +1058,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>1000</v>
+        <v>150</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1089,25 +1089,25 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>60351000</v>
+        <v>8420670000</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>8.880000000000001</v>
+        <v>40.85</v>
       </c>
       <c r="Q9" t="n">
-        <v>10.72</v>
+        <v>28.98</v>
       </c>
       <c r="R9" t="n">
-        <v>17.68</v>
+        <v>22.4</v>
       </c>
       <c r="S9" t="n">
-        <v>32.15</v>
+        <v>20.11</v>
       </c>
       <c r="T9" t="n">
-        <v>8.140000000000001</v>
+        <v>31.91</v>
       </c>
     </row>
     <row r="10">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -2468,7 +2468,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G28" t="n">
@@ -4022,7 +4022,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G49" t="n">
@@ -4392,7 +4392,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Seguradoras</t>
         </is>
       </c>
       <c r="G54" t="n">
@@ -5428,7 +5428,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G68" t="n">
@@ -5724,7 +5724,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G72" t="n">
@@ -5946,7 +5946,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G75" t="n">
@@ -7500,7 +7500,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G96" t="n">
@@ -7722,7 +7722,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G99" t="n">
@@ -11644,7 +11644,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G152" t="n">
@@ -12384,7 +12384,7 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G162" t="n">
@@ -12458,7 +12458,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G163" t="n">
@@ -16084,7 +16084,7 @@
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Saneamento</t>
         </is>
       </c>
       <c r="G212" t="n">
@@ -20524,7 +20524,7 @@
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>Comunicações</t>
+          <t>Telecomunicações</t>
         </is>
       </c>
       <c r="G272" t="n">
@@ -22448,7 +22448,7 @@
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>Comunicações</t>
+          <t>Telecomunicações</t>
         </is>
       </c>
       <c r="G298" t="n">
@@ -23091,12 +23091,12 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>ARND3</t>
+          <t>VNET3</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Empresa ARND</t>
+          <t>Empresa VNET</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -23106,22 +23106,22 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Novo Mercado</t>
+          <t>Tradicional</t>
         </is>
       </c>
       <c r="E307" t="n">
-        <v>0.51</v>
+        <v>0</v>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G307" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="H307" t="n">
-        <v>12.49</v>
+        <v>0</v>
       </c>
       <c r="I307" t="inlineStr">
         <is>
@@ -23135,16 +23135,16 @@
         <v>0</v>
       </c>
       <c r="L307" t="n">
-        <v>0.57</v>
+        <v>0</v>
       </c>
       <c r="M307" t="n">
         <v>0</v>
       </c>
       <c r="N307" t="n">
-        <v>125211000</v>
+        <v>14163000000</v>
       </c>
       <c r="O307" t="n">
-        <v>913.58</v>
+        <v>0</v>
       </c>
       <c r="P307" t="n">
         <v>0</v>
@@ -23159,23 +23159,23 @@
         <v>0</v>
       </c>
       <c r="T307" t="n">
-        <v>-0.88</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>VVAX3</t>
+          <t>CSPC4</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D308" t="inlineStr">
@@ -23184,7 +23184,7 @@
         </is>
       </c>
       <c r="E308" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="F308" t="inlineStr">
         <is>
@@ -23215,41 +23215,41 @@
         <v>0</v>
       </c>
       <c r="N308" t="n">
-        <v>144676000</v>
+        <v>2126670000</v>
       </c>
       <c r="O308" t="n">
         <v>0</v>
       </c>
       <c r="P308" t="n">
-        <v>-7.36</v>
+        <v>38.62</v>
       </c>
       <c r="Q308" t="n">
-        <v>-37.76</v>
+        <v>18.85</v>
       </c>
       <c r="R308" t="n">
-        <v>-6.52</v>
+        <v>29.18</v>
       </c>
       <c r="S308" t="n">
-        <v>-92.03</v>
+        <v>45.33</v>
       </c>
       <c r="T308" t="n">
-        <v>0</v>
+        <v>41.15</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>MSAN4</t>
+          <t>BOVH3</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa BOVH</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
@@ -23258,7 +23258,7 @@
         </is>
       </c>
       <c r="E309" t="n">
-        <v>6.44</v>
+        <v>15.71</v>
       </c>
       <c r="F309" t="inlineStr">
         <is>
@@ -23283,67 +23283,67 @@
         <v>0</v>
       </c>
       <c r="L309" t="n">
-        <v>0</v>
+        <v>6.16</v>
       </c>
       <c r="M309" t="n">
         <v>0</v>
       </c>
       <c r="N309" t="n">
-        <v>2533030000</v>
+        <v>1843320000</v>
       </c>
       <c r="O309" t="n">
         <v>0</v>
       </c>
       <c r="P309" t="n">
-        <v>6.27</v>
+        <v>0</v>
       </c>
       <c r="Q309" t="n">
-        <v>2.42</v>
+        <v>0</v>
       </c>
       <c r="R309" t="n">
-        <v>11.78</v>
+        <v>0</v>
       </c>
       <c r="S309" t="n">
-        <v>11.81</v>
+        <v>0</v>
       </c>
       <c r="T309" t="n">
-        <v>101.35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>GALO4</t>
+          <t>ARND3</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa ARND</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Tradicional</t>
+          <t>Novo Mercado</t>
         </is>
       </c>
       <c r="E310" t="n">
-        <v>0.25</v>
+        <v>0.51</v>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Tecnologia da Informação</t>
         </is>
       </c>
       <c r="G310" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="H310" t="n">
-        <v>0</v>
+        <v>12.49</v>
       </c>
       <c r="I310" t="inlineStr">
         <is>
@@ -23357,47 +23357,47 @@
         <v>0</v>
       </c>
       <c r="L310" t="n">
-        <v>0</v>
+        <v>0.57</v>
       </c>
       <c r="M310" t="n">
         <v>0</v>
       </c>
       <c r="N310" t="n">
-        <v>-60607000</v>
+        <v>125211000</v>
       </c>
       <c r="O310" t="n">
-        <v>0</v>
+        <v>913.58</v>
       </c>
       <c r="P310" t="n">
-        <v>13.98</v>
+        <v>0</v>
       </c>
       <c r="Q310" t="n">
-        <v>-184.58</v>
+        <v>0</v>
       </c>
       <c r="R310" t="n">
-        <v>39.37</v>
+        <v>0</v>
       </c>
       <c r="S310" t="n">
-        <v>7.62</v>
+        <v>0</v>
       </c>
       <c r="T310" t="n">
-        <v>-28.97</v>
+        <v>-0.88</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>BBTG13</t>
+          <t>PTIP4</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D311" t="inlineStr">
@@ -23406,7 +23406,7 @@
         </is>
       </c>
       <c r="E311" t="n">
-        <v>0</v>
+        <v>25.15</v>
       </c>
       <c r="F311" t="inlineStr">
         <is>
@@ -23437,36 +23437,36 @@
         <v>0</v>
       </c>
       <c r="N311" t="n">
-        <v>7000</v>
+        <v>-155957000</v>
       </c>
       <c r="O311" t="n">
         <v>0</v>
       </c>
       <c r="P311" t="n">
-        <v>0</v>
+        <v>13.73</v>
       </c>
       <c r="Q311" t="n">
-        <v>0</v>
+        <v>7.55</v>
       </c>
       <c r="R311" t="n">
-        <v>0</v>
+        <v>23.13</v>
       </c>
       <c r="S311" t="n">
-        <v>-42.86</v>
+        <v>-121.74</v>
       </c>
       <c r="T311" t="n">
-        <v>0</v>
+        <v>62.11</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>INHA3</t>
+          <t>LATS3</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Empresa INHA</t>
+          <t>Empresa LATS</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -23480,7 +23480,7 @@
         </is>
       </c>
       <c r="E312" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F312" t="inlineStr">
         <is>
@@ -23511,41 +23511,41 @@
         <v>0</v>
       </c>
       <c r="N312" t="n">
-        <v>1533210000</v>
+        <v>680646000</v>
       </c>
       <c r="O312" t="n">
         <v>0</v>
       </c>
       <c r="P312" t="n">
-        <v>-56.05</v>
+        <v>11.74</v>
       </c>
       <c r="Q312" t="n">
-        <v>-124.06</v>
+        <v>1.3</v>
       </c>
       <c r="R312" t="n">
-        <v>-6.27</v>
+        <v>11.63</v>
       </c>
       <c r="S312" t="n">
-        <v>-39.87</v>
+        <v>1.84</v>
       </c>
       <c r="T312" t="n">
-        <v>-12.18</v>
+        <v>15.37</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>PTIP4</t>
+          <t>VVAX3</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D313" t="inlineStr">
@@ -23554,7 +23554,7 @@
         </is>
       </c>
       <c r="E313" t="n">
-        <v>25.15</v>
+        <v>0</v>
       </c>
       <c r="F313" t="inlineStr">
         <is>
@@ -23585,41 +23585,41 @@
         <v>0</v>
       </c>
       <c r="N313" t="n">
-        <v>-155957000</v>
+        <v>144676000</v>
       </c>
       <c r="O313" t="n">
         <v>0</v>
       </c>
       <c r="P313" t="n">
-        <v>13.73</v>
+        <v>-7.36</v>
       </c>
       <c r="Q313" t="n">
-        <v>7.55</v>
+        <v>-37.76</v>
       </c>
       <c r="R313" t="n">
-        <v>23.13</v>
+        <v>-6.52</v>
       </c>
       <c r="S313" t="n">
-        <v>-121.74</v>
+        <v>-92.03</v>
       </c>
       <c r="T313" t="n">
-        <v>62.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>LATS3</t>
+          <t>MSAN4</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Empresa LATS</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
@@ -23628,7 +23628,7 @@
         </is>
       </c>
       <c r="E314" t="n">
-        <v>22</v>
+        <v>6.44</v>
       </c>
       <c r="F314" t="inlineStr">
         <is>
@@ -23659,41 +23659,41 @@
         <v>0</v>
       </c>
       <c r="N314" t="n">
-        <v>680646000</v>
+        <v>2533030000</v>
       </c>
       <c r="O314" t="n">
         <v>0</v>
       </c>
       <c r="P314" t="n">
-        <v>11.74</v>
+        <v>6.27</v>
       </c>
       <c r="Q314" t="n">
-        <v>1.3</v>
+        <v>2.42</v>
       </c>
       <c r="R314" t="n">
-        <v>11.63</v>
+        <v>11.78</v>
       </c>
       <c r="S314" t="n">
-        <v>1.84</v>
+        <v>11.81</v>
       </c>
       <c r="T314" t="n">
-        <v>15.37</v>
+        <v>101.35</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>VSPT3</t>
+          <t>GALO4</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
@@ -23702,11 +23702,11 @@
         </is>
       </c>
       <c r="E315" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>Bens Industriais</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G315" t="n">
@@ -23721,7 +23721,7 @@
         </is>
       </c>
       <c r="J315" t="n">
-        <v>-0.43</v>
+        <v>0</v>
       </c>
       <c r="K315" t="n">
         <v>0</v>
@@ -23733,41 +23733,41 @@
         <v>0</v>
       </c>
       <c r="N315" t="n">
-        <v>5031600000</v>
+        <v>-60607000</v>
       </c>
       <c r="O315" t="n">
         <v>0</v>
       </c>
       <c r="P315" t="n">
-        <v>0</v>
+        <v>13.98</v>
       </c>
       <c r="Q315" t="n">
-        <v>0</v>
+        <v>-184.58</v>
       </c>
       <c r="R315" t="n">
-        <v>0</v>
+        <v>39.37</v>
       </c>
       <c r="S315" t="n">
-        <v>0</v>
+        <v>7.62</v>
       </c>
       <c r="T315" t="n">
-        <v>4.92</v>
+        <v>-28.97</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>SGEN4</t>
+          <t>BBTG13</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
@@ -23776,7 +23776,7 @@
         </is>
       </c>
       <c r="E316" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="F316" t="inlineStr">
         <is>
@@ -23801,42 +23801,42 @@
         <v>0</v>
       </c>
       <c r="L316" t="n">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="M316" t="n">
         <v>0</v>
       </c>
       <c r="N316" t="n">
-        <v>156981000</v>
+        <v>7000</v>
       </c>
       <c r="O316" t="n">
         <v>0</v>
       </c>
       <c r="P316" t="n">
-        <v>-1871.17</v>
+        <v>0</v>
       </c>
       <c r="Q316" t="n">
         <v>0</v>
       </c>
       <c r="R316" t="n">
-        <v>-1.59</v>
+        <v>0</v>
       </c>
       <c r="S316" t="n">
-        <v>0</v>
+        <v>-42.86</v>
       </c>
       <c r="T316" t="n">
-        <v>-59.85</v>
+        <v>0</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>SEBB3</t>
+          <t>INHA3</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa INHA</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -23881,41 +23881,41 @@
         <v>0</v>
       </c>
       <c r="N317" t="n">
-        <v>145783000</v>
+        <v>1533210000</v>
       </c>
       <c r="O317" t="n">
         <v>0</v>
       </c>
       <c r="P317" t="n">
-        <v>9.24</v>
+        <v>-56.05</v>
       </c>
       <c r="Q317" t="n">
-        <v>7.4</v>
+        <v>-124.06</v>
       </c>
       <c r="R317" t="n">
-        <v>24.15</v>
+        <v>-6.27</v>
       </c>
       <c r="S317" t="n">
-        <v>23.01</v>
+        <v>-39.87</v>
       </c>
       <c r="T317" t="n">
-        <v>50.04</v>
+        <v>-12.18</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>BBTG11</t>
+          <t>VSPT3</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>UNT</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
@@ -23924,11 +23924,11 @@
         </is>
       </c>
       <c r="E318" t="n">
-        <v>15.01</v>
+        <v>0</v>
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bens Industriais</t>
         </is>
       </c>
       <c r="G318" t="n">
@@ -23943,7 +23943,7 @@
         </is>
       </c>
       <c r="J318" t="n">
-        <v>0</v>
+        <v>-0.43</v>
       </c>
       <c r="K318" t="n">
         <v>0</v>
@@ -23955,7 +23955,7 @@
         <v>0</v>
       </c>
       <c r="N318" t="n">
-        <v>0</v>
+        <v>5031600000</v>
       </c>
       <c r="O318" t="n">
         <v>0</v>
@@ -23973,18 +23973,18 @@
         <v>0</v>
       </c>
       <c r="T318" t="n">
-        <v>0</v>
+        <v>4.92</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>JFAB4</t>
+          <t>SGEN4</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Empresa JFAB</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -23998,7 +23998,7 @@
         </is>
       </c>
       <c r="E319" t="n">
-        <v>0.06</v>
+        <v>0.6</v>
       </c>
       <c r="F319" t="inlineStr">
         <is>
@@ -24023,31 +24023,31 @@
         <v>0</v>
       </c>
       <c r="L319" t="n">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="M319" t="n">
         <v>0</v>
       </c>
       <c r="N319" t="n">
-        <v>-10183000</v>
+        <v>156981000</v>
       </c>
       <c r="O319" t="n">
         <v>0</v>
       </c>
       <c r="P319" t="n">
-        <v>0</v>
+        <v>-1871.17</v>
       </c>
       <c r="Q319" t="n">
         <v>0</v>
       </c>
       <c r="R319" t="n">
-        <v>0</v>
+        <v>-1.59</v>
       </c>
       <c r="S319" t="n">
-        <v>2.34</v>
+        <v>0</v>
       </c>
       <c r="T319" t="n">
-        <v>0</v>
+        <v>-59.85</v>
       </c>
     </row>
     <row r="320">
@@ -24275,12 +24275,12 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>VGOR3</t>
+          <t>SEBB3</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Empresa VGOR</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -24325,41 +24325,41 @@
         <v>0</v>
       </c>
       <c r="N323" t="n">
-        <v>135178000</v>
+        <v>145783000</v>
       </c>
       <c r="O323" t="n">
         <v>0</v>
       </c>
       <c r="P323" t="n">
-        <v>4.5</v>
+        <v>9.24</v>
       </c>
       <c r="Q323" t="n">
-        <v>-4.59</v>
+        <v>7.4</v>
       </c>
       <c r="R323" t="n">
-        <v>6</v>
+        <v>24.15</v>
       </c>
       <c r="S323" t="n">
-        <v>-24.29</v>
+        <v>23.01</v>
       </c>
       <c r="T323" t="n">
-        <v>4.77</v>
+        <v>50.04</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>ECIS4</t>
+          <t>BBTG11</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D324" t="inlineStr">
@@ -24368,7 +24368,7 @@
         </is>
       </c>
       <c r="E324" t="n">
-        <v>145</v>
+        <v>15.01</v>
       </c>
       <c r="F324" t="inlineStr">
         <is>
@@ -24399,41 +24399,41 @@
         <v>0</v>
       </c>
       <c r="N324" t="n">
-        <v>129346000</v>
+        <v>0</v>
       </c>
       <c r="O324" t="n">
         <v>0</v>
       </c>
       <c r="P324" t="n">
-        <v>34.9</v>
+        <v>0</v>
       </c>
       <c r="Q324" t="n">
-        <v>14.18</v>
+        <v>0</v>
       </c>
       <c r="R324" t="n">
-        <v>12.48</v>
+        <v>0</v>
       </c>
       <c r="S324" t="n">
-        <v>7.33</v>
+        <v>0</v>
       </c>
       <c r="T324" t="n">
-        <v>4.66</v>
+        <v>0</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>TNEP3</t>
+          <t>JFAB4</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa JFAB</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D325" t="inlineStr">
@@ -24442,7 +24442,7 @@
         </is>
       </c>
       <c r="E325" t="n">
-        <v>3.01</v>
+        <v>0.06</v>
       </c>
       <c r="F325" t="inlineStr">
         <is>
@@ -24473,36 +24473,36 @@
         <v>0</v>
       </c>
       <c r="N325" t="n">
-        <v>955105000</v>
+        <v>-10183000</v>
       </c>
       <c r="O325" t="n">
         <v>0</v>
       </c>
       <c r="P325" t="n">
-        <v>20.92</v>
+        <v>0</v>
       </c>
       <c r="Q325" t="n">
-        <v>25.42</v>
+        <v>0</v>
       </c>
       <c r="R325" t="n">
-        <v>20.53</v>
+        <v>0</v>
       </c>
       <c r="S325" t="n">
-        <v>22.8</v>
+        <v>2.34</v>
       </c>
       <c r="T325" t="n">
-        <v>8.15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>LECO3</t>
+          <t>TNEP3</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Empresa LECO</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -24516,7 +24516,7 @@
         </is>
       </c>
       <c r="E326" t="n">
-        <v>0</v>
+        <v>3.01</v>
       </c>
       <c r="F326" t="inlineStr">
         <is>
@@ -24547,41 +24547,41 @@
         <v>0</v>
       </c>
       <c r="N326" t="n">
-        <v>105928000</v>
+        <v>955105000</v>
       </c>
       <c r="O326" t="n">
         <v>0</v>
       </c>
       <c r="P326" t="n">
-        <v>-2.14</v>
+        <v>20.92</v>
       </c>
       <c r="Q326" t="n">
-        <v>-4.72</v>
+        <v>25.42</v>
       </c>
       <c r="R326" t="n">
-        <v>-3.48</v>
+        <v>20.53</v>
       </c>
       <c r="S326" t="n">
-        <v>-14.82</v>
+        <v>22.8</v>
       </c>
       <c r="T326" t="n">
-        <v>3.58</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>SALM4</t>
+          <t>LECO3</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa LECO</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D327" t="inlineStr">
@@ -24590,7 +24590,7 @@
         </is>
       </c>
       <c r="E327" t="n">
-        <v>5.9</v>
+        <v>0</v>
       </c>
       <c r="F327" t="inlineStr">
         <is>
@@ -24621,36 +24621,36 @@
         <v>0</v>
       </c>
       <c r="N327" t="n">
-        <v>475600000</v>
+        <v>105928000</v>
       </c>
       <c r="O327" t="n">
         <v>0</v>
       </c>
       <c r="P327" t="n">
-        <v>10.22</v>
+        <v>-2.14</v>
       </c>
       <c r="Q327" t="n">
-        <v>4.13</v>
+        <v>-4.72</v>
       </c>
       <c r="R327" t="n">
-        <v>25.78</v>
+        <v>-3.48</v>
       </c>
       <c r="S327" t="n">
-        <v>19.53</v>
+        <v>-14.82</v>
       </c>
       <c r="T327" t="n">
-        <v>24.53</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>BERG3</t>
+          <t>VGOR3</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Empresa BERG</t>
+          <t>Empresa VGOR</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -24664,7 +24664,7 @@
         </is>
       </c>
       <c r="E328" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="F328" t="inlineStr">
         <is>
@@ -24695,41 +24695,41 @@
         <v>0</v>
       </c>
       <c r="N328" t="n">
-        <v>9538000</v>
+        <v>135178000</v>
       </c>
       <c r="O328" t="n">
         <v>0</v>
       </c>
       <c r="P328" t="n">
-        <v>-8.6</v>
+        <v>4.5</v>
       </c>
       <c r="Q328" t="n">
-        <v>-32.6</v>
+        <v>-4.59</v>
       </c>
       <c r="R328" t="n">
-        <v>-5.58</v>
+        <v>6</v>
       </c>
       <c r="S328" t="n">
-        <v>-102.71</v>
+        <v>-24.29</v>
       </c>
       <c r="T328" t="n">
-        <v>-8</v>
+        <v>4.77</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>JBDU3</t>
+          <t>ECIS4</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Empresa JBDU</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D329" t="inlineStr">
@@ -24738,7 +24738,7 @@
         </is>
       </c>
       <c r="E329" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="F329" t="inlineStr">
         <is>
@@ -24769,25 +24769,25 @@
         <v>0</v>
       </c>
       <c r="N329" t="n">
-        <v>56569000</v>
+        <v>129346000</v>
       </c>
       <c r="O329" t="n">
         <v>0</v>
       </c>
       <c r="P329" t="n">
-        <v>0</v>
+        <v>34.9</v>
       </c>
       <c r="Q329" t="n">
-        <v>0</v>
+        <v>14.18</v>
       </c>
       <c r="R329" t="n">
-        <v>0</v>
+        <v>12.48</v>
       </c>
       <c r="S329" t="n">
-        <v>0</v>
+        <v>7.33</v>
       </c>
       <c r="T329" t="n">
-        <v>0</v>
+        <v>4.66</v>
       </c>
     </row>
     <row r="330">
@@ -24941,17 +24941,17 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>SASG3</t>
+          <t>SALM4</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Empresa SASG</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D332" t="inlineStr">
@@ -24960,7 +24960,7 @@
         </is>
       </c>
       <c r="E332" t="n">
-        <v>0.98</v>
+        <v>5.9</v>
       </c>
       <c r="F332" t="inlineStr">
         <is>
@@ -24991,36 +24991,36 @@
         <v>0</v>
       </c>
       <c r="N332" t="n">
-        <v>0</v>
+        <v>475600000</v>
       </c>
       <c r="O332" t="n">
         <v>0</v>
       </c>
       <c r="P332" t="n">
-        <v>0</v>
+        <v>10.22</v>
       </c>
       <c r="Q332" t="n">
-        <v>0</v>
+        <v>4.13</v>
       </c>
       <c r="R332" t="n">
-        <v>0</v>
+        <v>25.78</v>
       </c>
       <c r="S332" t="n">
-        <v>0</v>
+        <v>19.53</v>
       </c>
       <c r="T332" t="n">
-        <v>0</v>
+        <v>24.53</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>BMEF3</t>
+          <t>BERG3</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Empresa BMEF</t>
+          <t>Empresa BERG</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -25034,7 +25034,7 @@
         </is>
       </c>
       <c r="E333" t="n">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="F333" t="inlineStr">
         <is>
@@ -25059,42 +25059,42 @@
         <v>0</v>
       </c>
       <c r="L333" t="n">
-        <v>4.16</v>
+        <v>0</v>
       </c>
       <c r="M333" t="n">
         <v>0</v>
       </c>
       <c r="N333" t="n">
-        <v>2674780000</v>
+        <v>9538000</v>
       </c>
       <c r="O333" t="n">
         <v>0</v>
       </c>
       <c r="P333" t="n">
-        <v>0</v>
+        <v>-8.6</v>
       </c>
       <c r="Q333" t="n">
-        <v>0</v>
+        <v>-32.6</v>
       </c>
       <c r="R333" t="n">
-        <v>0</v>
+        <v>-5.58</v>
       </c>
       <c r="S333" t="n">
-        <v>0</v>
+        <v>-102.71</v>
       </c>
       <c r="T333" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>AGEI3</t>
+          <t>JBDU3</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Empresa AGEI</t>
+          <t>Empresa JBDU</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -25108,7 +25108,7 @@
         </is>
       </c>
       <c r="E334" t="n">
-        <v>7.8</v>
+        <v>0</v>
       </c>
       <c r="F334" t="inlineStr">
         <is>
@@ -25133,13 +25133,13 @@
         <v>0</v>
       </c>
       <c r="L334" t="n">
-        <v>1.25</v>
+        <v>0</v>
       </c>
       <c r="M334" t="n">
         <v>0</v>
       </c>
       <c r="N334" t="n">
-        <v>1878210000</v>
+        <v>56569000</v>
       </c>
       <c r="O334" t="n">
         <v>0</v>
@@ -25163,12 +25163,12 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>ARPS3</t>
+          <t>AGEI3</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa AGEI</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -25182,7 +25182,7 @@
         </is>
       </c>
       <c r="E335" t="n">
-        <v>0.3</v>
+        <v>7.8</v>
       </c>
       <c r="F335" t="inlineStr">
         <is>
@@ -25207,42 +25207,42 @@
         <v>0</v>
       </c>
       <c r="L335" t="n">
-        <v>0</v>
+        <v>1.25</v>
       </c>
       <c r="M335" t="n">
         <v>0</v>
       </c>
       <c r="N335" t="n">
-        <v>-12690000</v>
+        <v>1878210000</v>
       </c>
       <c r="O335" t="n">
         <v>0</v>
       </c>
       <c r="P335" t="n">
-        <v>-4.92</v>
+        <v>0</v>
       </c>
       <c r="Q335" t="n">
-        <v>-11.59</v>
+        <v>0</v>
       </c>
       <c r="R335" t="n">
-        <v>-6.64</v>
+        <v>0</v>
       </c>
       <c r="S335" t="n">
-        <v>20.34</v>
+        <v>0</v>
       </c>
       <c r="T335" t="n">
-        <v>-17.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>ODER3</t>
+          <t>SASG3</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Empresa ODER</t>
+          <t>Empresa SASG</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -25256,18 +25256,18 @@
         </is>
       </c>
       <c r="E336" t="n">
-        <v>0</v>
+        <v>0.98</v>
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>Consumo não Cíclico</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G336" t="n">
         <v>80</v>
       </c>
       <c r="H336" t="n">
-        <v>1.75</v>
+        <v>0</v>
       </c>
       <c r="I336" t="inlineStr">
         <is>
@@ -25287,7 +25287,7 @@
         <v>0</v>
       </c>
       <c r="N336" t="n">
-        <v>609518000</v>
+        <v>0</v>
       </c>
       <c r="O336" t="n">
         <v>0</v>
@@ -25305,23 +25305,23 @@
         <v>0</v>
       </c>
       <c r="T336" t="n">
-        <v>3.17</v>
+        <v>0</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>VVAX4</t>
+          <t>BMEF3</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa BMEF</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
@@ -25330,7 +25330,7 @@
         </is>
       </c>
       <c r="E337" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F337" t="inlineStr">
         <is>
@@ -25355,28 +25355,28 @@
         <v>0</v>
       </c>
       <c r="L337" t="n">
-        <v>0</v>
+        <v>4.16</v>
       </c>
       <c r="M337" t="n">
         <v>0</v>
       </c>
       <c r="N337" t="n">
-        <v>144676000</v>
+        <v>2674780000</v>
       </c>
       <c r="O337" t="n">
         <v>0</v>
       </c>
       <c r="P337" t="n">
-        <v>-7.36</v>
+        <v>0</v>
       </c>
       <c r="Q337" t="n">
-        <v>-37.76</v>
+        <v>0</v>
       </c>
       <c r="R337" t="n">
-        <v>-6.52</v>
+        <v>0</v>
       </c>
       <c r="S337" t="n">
-        <v>-92.03</v>
+        <v>0</v>
       </c>
       <c r="T337" t="n">
         <v>0</v>
@@ -25385,12 +25385,12 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>CSPC3</t>
+          <t>ARPS3</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -25404,7 +25404,7 @@
         </is>
       </c>
       <c r="E338" t="n">
-        <v>1.24</v>
+        <v>0.3</v>
       </c>
       <c r="F338" t="inlineStr">
         <is>
@@ -25435,36 +25435,36 @@
         <v>0</v>
       </c>
       <c r="N338" t="n">
-        <v>2126670000</v>
+        <v>-12690000</v>
       </c>
       <c r="O338" t="n">
         <v>0</v>
       </c>
       <c r="P338" t="n">
-        <v>38.62</v>
+        <v>-4.92</v>
       </c>
       <c r="Q338" t="n">
-        <v>18.85</v>
+        <v>-11.59</v>
       </c>
       <c r="R338" t="n">
-        <v>29.18</v>
+        <v>-6.64</v>
       </c>
       <c r="S338" t="n">
-        <v>45.33</v>
+        <v>20.34</v>
       </c>
       <c r="T338" t="n">
-        <v>41.15</v>
+        <v>-17.53</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>ABCB3</t>
+          <t>ODER3</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Empresa ABCB</t>
+          <t>Empresa ODER</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -25482,14 +25482,14 @@
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Consumo não Cíclico</t>
         </is>
       </c>
       <c r="G339" t="n">
         <v>80</v>
       </c>
       <c r="H339" t="n">
-        <v>0</v>
+        <v>1.75</v>
       </c>
       <c r="I339" t="inlineStr">
         <is>
@@ -25509,7 +25509,7 @@
         <v>0</v>
       </c>
       <c r="N339" t="n">
-        <v>7258910000</v>
+        <v>609518000</v>
       </c>
       <c r="O339" t="n">
         <v>0</v>
@@ -25524,10 +25524,10 @@
         <v>0</v>
       </c>
       <c r="S339" t="n">
-        <v>14.05</v>
+        <v>0</v>
       </c>
       <c r="T339" t="n">
-        <v>7.57</v>
+        <v>3.17</v>
       </c>
     </row>
     <row r="340">
@@ -25607,12 +25607,12 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>VSPT4</t>
+          <t>VVAX4</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -25630,7 +25630,7 @@
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t>Bens Industriais</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G341" t="n">
@@ -25645,7 +25645,7 @@
         </is>
       </c>
       <c r="J341" t="n">
-        <v>-0.43</v>
+        <v>0</v>
       </c>
       <c r="K341" t="n">
         <v>0</v>
@@ -25657,41 +25657,41 @@
         <v>0</v>
       </c>
       <c r="N341" t="n">
-        <v>5031600000</v>
+        <v>144676000</v>
       </c>
       <c r="O341" t="n">
         <v>0</v>
       </c>
       <c r="P341" t="n">
-        <v>0</v>
+        <v>-7.36</v>
       </c>
       <c r="Q341" t="n">
-        <v>0</v>
+        <v>-37.76</v>
       </c>
       <c r="R341" t="n">
-        <v>0</v>
+        <v>-6.52</v>
       </c>
       <c r="S341" t="n">
-        <v>0</v>
+        <v>-92.03</v>
       </c>
       <c r="T341" t="n">
-        <v>4.92</v>
+        <v>0</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>BAUH4</t>
+          <t>CSPC3</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Empresa BAUH</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D342" t="inlineStr">
@@ -25700,18 +25700,18 @@
         </is>
       </c>
       <c r="E342" t="n">
-        <v>93.39</v>
+        <v>1.24</v>
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>Consumo não Cíclico</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G342" t="n">
         <v>80</v>
       </c>
       <c r="H342" t="n">
-        <v>28.89</v>
+        <v>0</v>
       </c>
       <c r="I342" t="inlineStr">
         <is>
@@ -25719,48 +25719,48 @@
         </is>
       </c>
       <c r="J342" t="n">
-        <v>-2.88</v>
+        <v>0</v>
       </c>
       <c r="K342" t="n">
         <v>0</v>
       </c>
       <c r="L342" t="n">
-        <v>3.18</v>
+        <v>0</v>
       </c>
       <c r="M342" t="n">
-        <v>1.16</v>
+        <v>0</v>
       </c>
       <c r="N342" t="n">
-        <v>153407000</v>
+        <v>2126670000</v>
       </c>
       <c r="O342" t="n">
-        <v>207.53</v>
+        <v>0</v>
       </c>
       <c r="P342" t="n">
-        <v>0</v>
+        <v>38.62</v>
       </c>
       <c r="Q342" t="n">
-        <v>0</v>
+        <v>18.85</v>
       </c>
       <c r="R342" t="n">
-        <v>0</v>
+        <v>29.18</v>
       </c>
       <c r="S342" t="n">
-        <v>0</v>
+        <v>45.33</v>
       </c>
       <c r="T342" t="n">
-        <v>13.32</v>
+        <v>41.15</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>ICPI3</t>
+          <t>ABCB3</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Empresa ICPI</t>
+          <t>Empresa ABCB</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -25778,7 +25778,7 @@
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G343" t="n">
@@ -25805,7 +25805,7 @@
         <v>0</v>
       </c>
       <c r="N343" t="n">
-        <v>0</v>
+        <v>7258910000</v>
       </c>
       <c r="O343" t="n">
         <v>0</v>
@@ -25820,21 +25820,21 @@
         <v>0</v>
       </c>
       <c r="S343" t="n">
-        <v>0</v>
+        <v>14.05</v>
       </c>
       <c r="T343" t="n">
-        <v>0</v>
+        <v>7.57</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>ILLS4</t>
+          <t>ESTC4</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Empresa ILLS</t>
+          <t>Empresa ESTC</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
@@ -25848,7 +25848,7 @@
         </is>
       </c>
       <c r="E344" t="n">
-        <v>100.01</v>
+        <v>0</v>
       </c>
       <c r="F344" t="inlineStr">
         <is>
@@ -25879,36 +25879,36 @@
         <v>0</v>
       </c>
       <c r="N344" t="n">
-        <v>-18567000</v>
+        <v>2916530000</v>
       </c>
       <c r="O344" t="n">
         <v>0</v>
       </c>
       <c r="P344" t="n">
-        <v>8.43</v>
+        <v>16.91</v>
       </c>
       <c r="Q344" t="n">
-        <v>-10.22</v>
+        <v>2.02</v>
       </c>
       <c r="R344" t="n">
-        <v>8.140000000000001</v>
+        <v>11.35</v>
       </c>
       <c r="S344" t="n">
-        <v>36.09</v>
+        <v>3.89</v>
       </c>
       <c r="T344" t="n">
-        <v>9.33</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>ESTC4</t>
+          <t>VSPT4</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Empresa ESTC</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -25926,7 +25926,7 @@
       </c>
       <c r="F345" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bens Industriais</t>
         </is>
       </c>
       <c r="G345" t="n">
@@ -25941,7 +25941,7 @@
         </is>
       </c>
       <c r="J345" t="n">
-        <v>0</v>
+        <v>-0.43</v>
       </c>
       <c r="K345" t="n">
         <v>0</v>
@@ -25953,36 +25953,36 @@
         <v>0</v>
       </c>
       <c r="N345" t="n">
-        <v>2916530000</v>
+        <v>5031600000</v>
       </c>
       <c r="O345" t="n">
         <v>0</v>
       </c>
       <c r="P345" t="n">
-        <v>16.91</v>
+        <v>0</v>
       </c>
       <c r="Q345" t="n">
-        <v>2.02</v>
+        <v>0</v>
       </c>
       <c r="R345" t="n">
-        <v>11.35</v>
+        <v>0</v>
       </c>
       <c r="S345" t="n">
-        <v>3.89</v>
+        <v>0</v>
       </c>
       <c r="T345" t="n">
-        <v>5.6</v>
+        <v>4.92</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>SEBB4</t>
+          <t>BAUH4</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa BAUH</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
@@ -25996,18 +25996,18 @@
         </is>
       </c>
       <c r="E346" t="n">
-        <v>0</v>
+        <v>93.39</v>
       </c>
       <c r="F346" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Consumo não Cíclico</t>
         </is>
       </c>
       <c r="G346" t="n">
         <v>80</v>
       </c>
       <c r="H346" t="n">
-        <v>0</v>
+        <v>28.89</v>
       </c>
       <c r="I346" t="inlineStr">
         <is>
@@ -26015,48 +26015,48 @@
         </is>
       </c>
       <c r="J346" t="n">
-        <v>0</v>
+        <v>-2.88</v>
       </c>
       <c r="K346" t="n">
         <v>0</v>
       </c>
       <c r="L346" t="n">
-        <v>0</v>
+        <v>3.18</v>
       </c>
       <c r="M346" t="n">
-        <v>0</v>
+        <v>1.16</v>
       </c>
       <c r="N346" t="n">
-        <v>145783000</v>
+        <v>153407000</v>
       </c>
       <c r="O346" t="n">
-        <v>0</v>
+        <v>207.53</v>
       </c>
       <c r="P346" t="n">
-        <v>9.24</v>
+        <v>0</v>
       </c>
       <c r="Q346" t="n">
-        <v>7.4</v>
+        <v>0</v>
       </c>
       <c r="R346" t="n">
-        <v>24.15</v>
+        <v>0</v>
       </c>
       <c r="S346" t="n">
-        <v>23.01</v>
+        <v>0</v>
       </c>
       <c r="T346" t="n">
-        <v>50.04</v>
+        <v>13.32</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>MSAN3</t>
+          <t>ICPI3</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa ICPI</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
@@ -26070,7 +26070,7 @@
         </is>
       </c>
       <c r="E347" t="n">
-        <v>6.44</v>
+        <v>0</v>
       </c>
       <c r="F347" t="inlineStr">
         <is>
@@ -26101,41 +26101,41 @@
         <v>0</v>
       </c>
       <c r="N347" t="n">
-        <v>2533030000</v>
+        <v>0</v>
       </c>
       <c r="O347" t="n">
         <v>0</v>
       </c>
       <c r="P347" t="n">
-        <v>6.27</v>
+        <v>0</v>
       </c>
       <c r="Q347" t="n">
-        <v>2.42</v>
+        <v>0</v>
       </c>
       <c r="R347" t="n">
-        <v>11.78</v>
+        <v>0</v>
       </c>
       <c r="S347" t="n">
-        <v>11.81</v>
+        <v>0</v>
       </c>
       <c r="T347" t="n">
-        <v>101.35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>GALO3</t>
+          <t>ILLS4</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa ILLS</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D348" t="inlineStr">
@@ -26144,7 +26144,7 @@
         </is>
       </c>
       <c r="E348" t="n">
-        <v>0</v>
+        <v>100.01</v>
       </c>
       <c r="F348" t="inlineStr">
         <is>
@@ -26175,36 +26175,36 @@
         <v>0</v>
       </c>
       <c r="N348" t="n">
-        <v>-60607000</v>
+        <v>-18567000</v>
       </c>
       <c r="O348" t="n">
         <v>0</v>
       </c>
       <c r="P348" t="n">
-        <v>13.98</v>
+        <v>8.43</v>
       </c>
       <c r="Q348" t="n">
-        <v>-184.58</v>
+        <v>-10.22</v>
       </c>
       <c r="R348" t="n">
-        <v>39.37</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="S348" t="n">
-        <v>7.62</v>
+        <v>36.09</v>
       </c>
       <c r="T348" t="n">
-        <v>-28.97</v>
+        <v>9.33</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>SLCP3</t>
+          <t>PTIP3</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Empresa SLCP</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
@@ -26218,7 +26218,7 @@
         </is>
       </c>
       <c r="E349" t="n">
-        <v>610.02</v>
+        <v>22</v>
       </c>
       <c r="F349" t="inlineStr">
         <is>
@@ -26249,41 +26249,41 @@
         <v>0</v>
       </c>
       <c r="N349" t="n">
-        <v>0</v>
+        <v>-155957000</v>
       </c>
       <c r="O349" t="n">
         <v>0</v>
       </c>
       <c r="P349" t="n">
-        <v>0</v>
+        <v>13.73</v>
       </c>
       <c r="Q349" t="n">
-        <v>0</v>
+        <v>7.55</v>
       </c>
       <c r="R349" t="n">
-        <v>0</v>
+        <v>23.13</v>
       </c>
       <c r="S349" t="n">
-        <v>0</v>
+        <v>-121.74</v>
       </c>
       <c r="T349" t="n">
-        <v>0</v>
+        <v>62.11</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>DAYC3</t>
+          <t>REPA4</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Empresa DAYC</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D350" t="inlineStr">
@@ -26292,7 +26292,7 @@
         </is>
       </c>
       <c r="E350" t="n">
-        <v>0</v>
+        <v>1.08</v>
       </c>
       <c r="F350" t="inlineStr">
         <is>
@@ -26323,41 +26323,41 @@
         <v>0</v>
       </c>
       <c r="N350" t="n">
-        <v>3009030000</v>
+        <v>378378000</v>
       </c>
       <c r="O350" t="n">
         <v>0</v>
       </c>
       <c r="P350" t="n">
-        <v>0</v>
+        <v>5.18</v>
       </c>
       <c r="Q350" t="n">
-        <v>0</v>
+        <v>1.22</v>
       </c>
       <c r="R350" t="n">
-        <v>0</v>
+        <v>4.05</v>
       </c>
       <c r="S350" t="n">
-        <v>17.33</v>
+        <v>1.91</v>
       </c>
       <c r="T350" t="n">
-        <v>8.15</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>PTIP3</t>
+          <t>EQMA6B</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D351" t="inlineStr">
@@ -26366,7 +26366,7 @@
         </is>
       </c>
       <c r="E351" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="F351" t="inlineStr">
         <is>
@@ -26397,36 +26397,36 @@
         <v>0</v>
       </c>
       <c r="N351" t="n">
-        <v>-155957000</v>
+        <v>4940330000</v>
       </c>
       <c r="O351" t="n">
         <v>0</v>
       </c>
       <c r="P351" t="n">
-        <v>13.73</v>
+        <v>0</v>
       </c>
       <c r="Q351" t="n">
-        <v>7.55</v>
+        <v>0</v>
       </c>
       <c r="R351" t="n">
-        <v>23.13</v>
+        <v>0</v>
       </c>
       <c r="S351" t="n">
-        <v>-121.74</v>
+        <v>0</v>
       </c>
       <c r="T351" t="n">
-        <v>62.11</v>
+        <v>9.050000000000001</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>REPA4</t>
+          <t>SEBB4</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -26440,7 +26440,7 @@
         </is>
       </c>
       <c r="E352" t="n">
-        <v>1.08</v>
+        <v>0</v>
       </c>
       <c r="F352" t="inlineStr">
         <is>
@@ -26471,41 +26471,41 @@
         <v>0</v>
       </c>
       <c r="N352" t="n">
-        <v>378378000</v>
+        <v>145783000</v>
       </c>
       <c r="O352" t="n">
         <v>0</v>
       </c>
       <c r="P352" t="n">
-        <v>5.18</v>
+        <v>9.24</v>
       </c>
       <c r="Q352" t="n">
-        <v>1.22</v>
+        <v>7.4</v>
       </c>
       <c r="R352" t="n">
-        <v>4.05</v>
+        <v>24.15</v>
       </c>
       <c r="S352" t="n">
-        <v>1.91</v>
+        <v>23.01</v>
       </c>
       <c r="T352" t="n">
-        <v>1.09</v>
+        <v>50.04</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>EQMA6B</t>
+          <t>MSAN3</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D353" t="inlineStr">
@@ -26514,7 +26514,7 @@
         </is>
       </c>
       <c r="E353" t="n">
-        <v>0</v>
+        <v>6.44</v>
       </c>
       <c r="F353" t="inlineStr">
         <is>
@@ -26545,36 +26545,36 @@
         <v>0</v>
       </c>
       <c r="N353" t="n">
-        <v>4940330000</v>
+        <v>2533030000</v>
       </c>
       <c r="O353" t="n">
         <v>0</v>
       </c>
       <c r="P353" t="n">
-        <v>0</v>
+        <v>6.27</v>
       </c>
       <c r="Q353" t="n">
-        <v>0</v>
+        <v>2.42</v>
       </c>
       <c r="R353" t="n">
-        <v>0</v>
+        <v>11.78</v>
       </c>
       <c r="S353" t="n">
-        <v>0</v>
+        <v>11.81</v>
       </c>
       <c r="T353" t="n">
-        <v>9.050000000000001</v>
+        <v>101.35</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>MLPA3</t>
+          <t>GALO3</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Empresa MLPA</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -26619,69 +26619,69 @@
         <v>0</v>
       </c>
       <c r="N354" t="n">
-        <v>44578000</v>
+        <v>-60607000</v>
       </c>
       <c r="O354" t="n">
         <v>0</v>
       </c>
       <c r="P354" t="n">
-        <v>6.66</v>
+        <v>13.98</v>
       </c>
       <c r="Q354" t="n">
-        <v>8.92</v>
+        <v>-184.58</v>
       </c>
       <c r="R354" t="n">
-        <v>0</v>
+        <v>39.37</v>
       </c>
       <c r="S354" t="n">
-        <v>45.13</v>
+        <v>7.62</v>
       </c>
       <c r="T354" t="n">
-        <v>-7.51</v>
+        <v>-28.97</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>CLSC6</t>
+          <t>SLCP3</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Empresa CLSC</t>
+          <t>Empresa SLCP</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>Nível 2</t>
+          <t>Tradicional</t>
         </is>
       </c>
       <c r="E355" t="n">
-        <v>0</v>
+        <v>610.02</v>
       </c>
       <c r="F355" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G355" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="H355" t="n">
-        <v>75.73</v>
+        <v>0</v>
       </c>
       <c r="I355" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="J355" t="n">
-        <v>2.73</v>
+        <v>0</v>
       </c>
       <c r="K355" t="n">
         <v>0</v>
@@ -26693,7 +26693,7 @@
         <v>0</v>
       </c>
       <c r="N355" t="n">
-        <v>4228180000</v>
+        <v>0</v>
       </c>
       <c r="O355" t="n">
         <v>0</v>
@@ -26711,18 +26711,18 @@
         <v>0</v>
       </c>
       <c r="T355" t="n">
-        <v>2.82</v>
+        <v>0</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>SGEN3</t>
+          <t>DAYC3</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa DAYC</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -26736,7 +26736,7 @@
         </is>
       </c>
       <c r="E356" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F356" t="inlineStr">
         <is>
@@ -26761,47 +26761,47 @@
         <v>0</v>
       </c>
       <c r="L356" t="n">
-        <v>0.77</v>
+        <v>0</v>
       </c>
       <c r="M356" t="n">
         <v>0</v>
       </c>
       <c r="N356" t="n">
-        <v>156981000</v>
+        <v>3009030000</v>
       </c>
       <c r="O356" t="n">
         <v>0</v>
       </c>
       <c r="P356" t="n">
-        <v>-1871.17</v>
+        <v>0</v>
       </c>
       <c r="Q356" t="n">
         <v>0</v>
       </c>
       <c r="R356" t="n">
-        <v>-1.59</v>
+        <v>0</v>
       </c>
       <c r="S356" t="n">
-        <v>0</v>
+        <v>17.33</v>
       </c>
       <c r="T356" t="n">
-        <v>-59.85</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>DUFB11</t>
+          <t>TNEP4</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Empresa DUFB</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>UNT</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D357" t="inlineStr">
@@ -26810,7 +26810,7 @@
         </is>
       </c>
       <c r="E357" t="n">
-        <v>0</v>
+        <v>3.95</v>
       </c>
       <c r="F357" t="inlineStr">
         <is>
@@ -26841,41 +26841,41 @@
         <v>0</v>
       </c>
       <c r="N357" t="n">
-        <v>0</v>
+        <v>955105000</v>
       </c>
       <c r="O357" t="n">
         <v>0</v>
       </c>
       <c r="P357" t="n">
-        <v>0</v>
+        <v>20.92</v>
       </c>
       <c r="Q357" t="n">
-        <v>0</v>
+        <v>25.42</v>
       </c>
       <c r="R357" t="n">
-        <v>0</v>
+        <v>20.53</v>
       </c>
       <c r="S357" t="n">
-        <v>0</v>
+        <v>22.8</v>
       </c>
       <c r="T357" t="n">
-        <v>0</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>TNEP4</t>
+          <t>MLPA3</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa MLPA</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D358" t="inlineStr">
@@ -26884,7 +26884,7 @@
         </is>
       </c>
       <c r="E358" t="n">
-        <v>3.95</v>
+        <v>0</v>
       </c>
       <c r="F358" t="inlineStr">
         <is>
@@ -26915,81 +26915,81 @@
         <v>0</v>
       </c>
       <c r="N358" t="n">
-        <v>955105000</v>
+        <v>44578000</v>
       </c>
       <c r="O358" t="n">
         <v>0</v>
       </c>
       <c r="P358" t="n">
-        <v>20.92</v>
+        <v>6.66</v>
       </c>
       <c r="Q358" t="n">
-        <v>25.42</v>
+        <v>8.92</v>
       </c>
       <c r="R358" t="n">
-        <v>20.53</v>
+        <v>0</v>
       </c>
       <c r="S358" t="n">
-        <v>22.8</v>
+        <v>45.13</v>
       </c>
       <c r="T358" t="n">
-        <v>8.15</v>
+        <v>-7.51</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>CCHI3</t>
+          <t>CLSC6</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa CLSC</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>Tradicional</t>
+          <t>Nível 2</t>
         </is>
       </c>
       <c r="E359" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G359" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="H359" t="n">
-        <v>0</v>
+        <v>75.73</v>
       </c>
       <c r="I359" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="J359" t="n">
-        <v>0</v>
+        <v>2.73</v>
       </c>
       <c r="K359" t="n">
         <v>0</v>
       </c>
       <c r="L359" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="M359" t="n">
         <v>0</v>
       </c>
       <c r="N359" t="n">
-        <v>-160477000</v>
+        <v>4228180000</v>
       </c>
       <c r="O359" t="n">
         <v>0</v>
@@ -27007,18 +27007,18 @@
         <v>0</v>
       </c>
       <c r="T359" t="n">
-        <v>20.36</v>
+        <v>2.82</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>SFSA3</t>
+          <t>SGEN3</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Empresa SFSA</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
@@ -27032,7 +27032,7 @@
         </is>
       </c>
       <c r="E360" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F360" t="inlineStr">
         <is>
@@ -27057,47 +27057,47 @@
         <v>0</v>
       </c>
       <c r="L360" t="n">
-        <v>0</v>
+        <v>0.77</v>
       </c>
       <c r="M360" t="n">
         <v>0</v>
       </c>
       <c r="N360" t="n">
-        <v>739524000</v>
+        <v>156981000</v>
       </c>
       <c r="O360" t="n">
         <v>0</v>
       </c>
       <c r="P360" t="n">
-        <v>0</v>
+        <v>-1871.17</v>
       </c>
       <c r="Q360" t="n">
         <v>0</v>
       </c>
       <c r="R360" t="n">
-        <v>0</v>
+        <v>-1.59</v>
       </c>
       <c r="S360" t="n">
-        <v>6.25</v>
+        <v>0</v>
       </c>
       <c r="T360" t="n">
-        <v>0.15</v>
+        <v>-59.85</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>PRBC3</t>
+          <t>DUFB11</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Empresa PRBC</t>
+          <t>Empresa DUFB</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D361" t="inlineStr">
@@ -27137,7 +27137,7 @@
         <v>0</v>
       </c>
       <c r="N361" t="n">
-        <v>1319270000</v>
+        <v>0</v>
       </c>
       <c r="O361" t="n">
         <v>0</v>
@@ -27152,21 +27152,21 @@
         <v>0</v>
       </c>
       <c r="S361" t="n">
-        <v>8.27</v>
+        <v>0</v>
       </c>
       <c r="T361" t="n">
-        <v>-1.98</v>
+        <v>0</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>ECIS3</t>
+          <t>CCHI3</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -27180,7 +27180,7 @@
         </is>
       </c>
       <c r="E362" t="n">
-        <v>211.65</v>
+        <v>0.02</v>
       </c>
       <c r="F362" t="inlineStr">
         <is>
@@ -27205,47 +27205,47 @@
         <v>0</v>
       </c>
       <c r="L362" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="M362" t="n">
         <v>0</v>
       </c>
       <c r="N362" t="n">
-        <v>129346000</v>
+        <v>-160477000</v>
       </c>
       <c r="O362" t="n">
         <v>0</v>
       </c>
       <c r="P362" t="n">
-        <v>34.9</v>
+        <v>0</v>
       </c>
       <c r="Q362" t="n">
-        <v>14.18</v>
+        <v>0</v>
       </c>
       <c r="R362" t="n">
-        <v>12.48</v>
+        <v>0</v>
       </c>
       <c r="S362" t="n">
-        <v>7.33</v>
+        <v>0</v>
       </c>
       <c r="T362" t="n">
-        <v>4.66</v>
+        <v>20.36</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>ARPS4</t>
+          <t>SFSA3</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa SFSA</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D363" t="inlineStr">
@@ -27285,36 +27285,36 @@
         <v>0</v>
       </c>
       <c r="N363" t="n">
-        <v>-12690000</v>
+        <v>739524000</v>
       </c>
       <c r="O363" t="n">
         <v>0</v>
       </c>
       <c r="P363" t="n">
-        <v>-4.92</v>
+        <v>0</v>
       </c>
       <c r="Q363" t="n">
-        <v>-11.59</v>
+        <v>0</v>
       </c>
       <c r="R363" t="n">
-        <v>-6.64</v>
+        <v>0</v>
       </c>
       <c r="S363" t="n">
-        <v>20.34</v>
+        <v>6.25</v>
       </c>
       <c r="T363" t="n">
-        <v>-17.53</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>SALM3</t>
+          <t>PRBC3</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa PRBC</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -27328,7 +27328,7 @@
         </is>
       </c>
       <c r="E364" t="n">
-        <v>5.7</v>
+        <v>0</v>
       </c>
       <c r="F364" t="inlineStr">
         <is>
@@ -27359,41 +27359,41 @@
         <v>0</v>
       </c>
       <c r="N364" t="n">
-        <v>475600000</v>
+        <v>1319270000</v>
       </c>
       <c r="O364" t="n">
         <v>0</v>
       </c>
       <c r="P364" t="n">
-        <v>10.22</v>
+        <v>0</v>
       </c>
       <c r="Q364" t="n">
-        <v>4.13</v>
+        <v>0</v>
       </c>
       <c r="R364" t="n">
-        <v>25.78</v>
+        <v>0</v>
       </c>
       <c r="S364" t="n">
-        <v>19.53</v>
+        <v>8.27</v>
       </c>
       <c r="T364" t="n">
-        <v>24.53</v>
+        <v>-1.98</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>CMMA4</t>
+          <t>ECIS3</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Empresa CMMA</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
@@ -27402,7 +27402,7 @@
         </is>
       </c>
       <c r="E365" t="n">
-        <v>0.8100000000000001</v>
+        <v>211.65</v>
       </c>
       <c r="F365" t="inlineStr">
         <is>
@@ -27433,36 +27433,36 @@
         <v>0</v>
       </c>
       <c r="N365" t="n">
-        <v>-79623000</v>
+        <v>129346000</v>
       </c>
       <c r="O365" t="n">
         <v>0</v>
       </c>
       <c r="P365" t="n">
-        <v>0</v>
+        <v>34.9</v>
       </c>
       <c r="Q365" t="n">
-        <v>0</v>
+        <v>14.18</v>
       </c>
       <c r="R365" t="n">
-        <v>0</v>
+        <v>12.48</v>
       </c>
       <c r="S365" t="n">
-        <v>-1.92</v>
+        <v>7.33</v>
       </c>
       <c r="T365" t="n">
-        <v>0</v>
+        <v>4.66</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>CZRS3</t>
+          <t>BSGR3</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Empresa CZRS</t>
+          <t>Empresa BSGR</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -27476,7 +27476,7 @@
         </is>
       </c>
       <c r="E366" t="n">
-        <v>0</v>
+        <v>1091.28</v>
       </c>
       <c r="F366" t="inlineStr">
         <is>
@@ -27507,7 +27507,7 @@
         <v>0</v>
       </c>
       <c r="N366" t="n">
-        <v>1145670000</v>
+        <v>0</v>
       </c>
       <c r="O366" t="n">
         <v>0</v>
@@ -27522,21 +27522,21 @@
         <v>0</v>
       </c>
       <c r="S366" t="n">
-        <v>3.34</v>
+        <v>0</v>
       </c>
       <c r="T366" t="n">
-        <v>14.44</v>
+        <v>0</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>BPNM3</t>
+          <t>CBMA3</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Empresa BPNM</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -27550,7 +27550,7 @@
         </is>
       </c>
       <c r="E367" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="F367" t="inlineStr">
         <is>
@@ -27581,7 +27581,7 @@
         <v>0</v>
       </c>
       <c r="N367" t="n">
-        <v>7792670000</v>
+        <v>-34022300000</v>
       </c>
       <c r="O367" t="n">
         <v>0</v>
@@ -27596,21 +27596,21 @@
         <v>0</v>
       </c>
       <c r="S367" t="n">
-        <v>9.67</v>
+        <v>0</v>
       </c>
       <c r="T367" t="n">
-        <v>-1.53</v>
+        <v>252.65</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>BSGR3</t>
+          <t>ALBA3</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Empresa BSGR</t>
+          <t>Empresa ALBA</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -27624,7 +27624,7 @@
         </is>
       </c>
       <c r="E368" t="n">
-        <v>1091.28</v>
+        <v>2.15</v>
       </c>
       <c r="F368" t="inlineStr">
         <is>
@@ -27655,41 +27655,41 @@
         <v>0</v>
       </c>
       <c r="N368" t="n">
-        <v>0</v>
+        <v>354860000</v>
       </c>
       <c r="O368" t="n">
         <v>0</v>
       </c>
       <c r="P368" t="n">
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="Q368" t="n">
-        <v>0</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="R368" t="n">
-        <v>0</v>
+        <v>20.4</v>
       </c>
       <c r="S368" t="n">
-        <v>0</v>
+        <v>19.77</v>
       </c>
       <c r="T368" t="n">
-        <v>0</v>
+        <v>14.69</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>CBMA3</t>
+          <t>ARPS4</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D369" t="inlineStr">
@@ -27698,7 +27698,7 @@
         </is>
       </c>
       <c r="E369" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="F369" t="inlineStr">
         <is>
@@ -27729,36 +27729,36 @@
         <v>0</v>
       </c>
       <c r="N369" t="n">
-        <v>-34022300000</v>
+        <v>-12690000</v>
       </c>
       <c r="O369" t="n">
         <v>0</v>
       </c>
       <c r="P369" t="n">
-        <v>0</v>
+        <v>-4.92</v>
       </c>
       <c r="Q369" t="n">
-        <v>0</v>
+        <v>-11.59</v>
       </c>
       <c r="R369" t="n">
-        <v>0</v>
+        <v>-6.64</v>
       </c>
       <c r="S369" t="n">
-        <v>0</v>
+        <v>20.34</v>
       </c>
       <c r="T369" t="n">
-        <v>252.65</v>
+        <v>-17.53</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>ALBA3</t>
+          <t>SALM3</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Empresa ALBA</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -27772,7 +27772,7 @@
         </is>
       </c>
       <c r="E370" t="n">
-        <v>2.15</v>
+        <v>5.7</v>
       </c>
       <c r="F370" t="inlineStr">
         <is>
@@ -27803,41 +27803,41 @@
         <v>0</v>
       </c>
       <c r="N370" t="n">
-        <v>354860000</v>
+        <v>475600000</v>
       </c>
       <c r="O370" t="n">
         <v>0</v>
       </c>
       <c r="P370" t="n">
-        <v>9.5</v>
+        <v>10.22</v>
       </c>
       <c r="Q370" t="n">
-        <v>9.619999999999999</v>
+        <v>4.13</v>
       </c>
       <c r="R370" t="n">
-        <v>20.4</v>
+        <v>25.78</v>
       </c>
       <c r="S370" t="n">
-        <v>19.77</v>
+        <v>19.53</v>
       </c>
       <c r="T370" t="n">
-        <v>14.69</v>
+        <v>24.53</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>VNET3</t>
+          <t>CMMA4</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Empresa VNET</t>
+          <t>Empresa CMMA</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D371" t="inlineStr">
@@ -27846,7 +27846,7 @@
         </is>
       </c>
       <c r="E371" t="n">
-        <v>0</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="F371" t="inlineStr">
         <is>
@@ -27877,7 +27877,7 @@
         <v>0</v>
       </c>
       <c r="N371" t="n">
-        <v>14163000000</v>
+        <v>-79623000</v>
       </c>
       <c r="O371" t="n">
         <v>0</v>
@@ -27892,26 +27892,26 @@
         <v>0</v>
       </c>
       <c r="S371" t="n">
-        <v>0</v>
+        <v>-1.92</v>
       </c>
       <c r="T371" t="n">
-        <v>1.08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>CSPC4</t>
+          <t>CZRS3</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa CZRS</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D372" t="inlineStr">
@@ -27920,7 +27920,7 @@
         </is>
       </c>
       <c r="E372" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="F372" t="inlineStr">
         <is>
@@ -27951,36 +27951,36 @@
         <v>0</v>
       </c>
       <c r="N372" t="n">
-        <v>2126670000</v>
+        <v>1145670000</v>
       </c>
       <c r="O372" t="n">
         <v>0</v>
       </c>
       <c r="P372" t="n">
-        <v>38.62</v>
+        <v>0</v>
       </c>
       <c r="Q372" t="n">
-        <v>18.85</v>
+        <v>0</v>
       </c>
       <c r="R372" t="n">
-        <v>29.18</v>
+        <v>0</v>
       </c>
       <c r="S372" t="n">
-        <v>45.33</v>
+        <v>3.34</v>
       </c>
       <c r="T372" t="n">
-        <v>41.15</v>
+        <v>14.44</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>BOVH3</t>
+          <t>BPNM3</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Empresa BOVH</t>
+          <t>Empresa BPNM</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
@@ -27994,7 +27994,7 @@
         </is>
       </c>
       <c r="E373" t="n">
-        <v>15.71</v>
+        <v>0</v>
       </c>
       <c r="F373" t="inlineStr">
         <is>
@@ -28019,13 +28019,13 @@
         <v>0</v>
       </c>
       <c r="L373" t="n">
-        <v>6.16</v>
+        <v>0</v>
       </c>
       <c r="M373" t="n">
         <v>0</v>
       </c>
       <c r="N373" t="n">
-        <v>1843320000</v>
+        <v>7792670000</v>
       </c>
       <c r="O373" t="n">
         <v>0</v>
@@ -28040,10 +28040,10 @@
         <v>0</v>
       </c>
       <c r="S373" t="n">
-        <v>0</v>
+        <v>9.67</v>
       </c>
       <c r="T373" t="n">
-        <v>0</v>
+        <v>-1.53</v>
       </c>
     </row>
     <row r="374">
@@ -29108,7 +29108,7 @@
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G388" t="n">
@@ -31698,7 +31698,7 @@
       </c>
       <c r="F423" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G423" t="n">
@@ -32068,7 +32068,7 @@
       </c>
       <c r="F428" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G428" t="n">
@@ -32216,7 +32216,7 @@
       </c>
       <c r="F430" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G430" t="n">
@@ -32290,7 +32290,7 @@
       </c>
       <c r="F431" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G431" t="n">
@@ -32956,7 +32956,7 @@
       </c>
       <c r="F440" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G440" t="n">
@@ -34584,7 +34584,7 @@
       </c>
       <c r="F462" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G462" t="n">
@@ -34732,7 +34732,7 @@
       </c>
       <c r="F464" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G464" t="n">
@@ -35546,7 +35546,7 @@
       </c>
       <c r="F475" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G475" t="n">
@@ -36212,7 +36212,7 @@
       </c>
       <c r="F484" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G484" t="n">
@@ -36360,7 +36360,7 @@
       </c>
       <c r="F486" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G486" t="n">
@@ -36434,7 +36434,7 @@
       </c>
       <c r="F487" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G487" t="n">
@@ -36582,7 +36582,7 @@
       </c>
       <c r="F489" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G489" t="n">
@@ -36952,7 +36952,7 @@
       </c>
       <c r="F494" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G494" t="n">
@@ -39246,7 +39246,7 @@
       </c>
       <c r="F525" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G525" t="n">
@@ -39468,7 +39468,7 @@
       </c>
       <c r="F528" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G528" t="n">
@@ -39542,7 +39542,7 @@
       </c>
       <c r="F529" t="inlineStr">
         <is>
-          <t>Comunicações</t>
+          <t>Telecomunicações</t>
         </is>
       </c>
       <c r="G529" t="n">
@@ -40578,7 +40578,7 @@
       </c>
       <c r="F543" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G543" t="n">
@@ -40726,7 +40726,7 @@
       </c>
       <c r="F545" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G545" t="n">
@@ -41022,7 +41022,7 @@
       </c>
       <c r="F549" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G549" t="n">
@@ -41392,7 +41392,7 @@
       </c>
       <c r="F554" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Seguradoras</t>
         </is>
       </c>
       <c r="G554" t="n">
@@ -41836,7 +41836,7 @@
       </c>
       <c r="F560" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G560" t="n">
@@ -41984,7 +41984,7 @@
       </c>
       <c r="F562" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G562" t="n">
@@ -42132,7 +42132,7 @@
       </c>
       <c r="F564" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G564" t="n">
@@ -42206,7 +42206,7 @@
       </c>
       <c r="F565" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G565" t="n">
@@ -42354,7 +42354,7 @@
       </c>
       <c r="F567" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G567" t="n">
@@ -42428,7 +42428,7 @@
       </c>
       <c r="F568" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G568" t="n">
@@ -42650,7 +42650,7 @@
       </c>
       <c r="F571" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G571" t="n">
@@ -42872,7 +42872,7 @@
       </c>
       <c r="F574" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G574" t="n">
@@ -43020,7 +43020,7 @@
       </c>
       <c r="F576" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G576" t="n">
@@ -43390,7 +43390,7 @@
       </c>
       <c r="F581" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G581" t="n">
@@ -43464,7 +43464,7 @@
       </c>
       <c r="F582" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G582" t="n">
@@ -44204,7 +44204,7 @@
       </c>
       <c r="F592" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G592" t="n">
@@ -44352,7 +44352,7 @@
       </c>
       <c r="F594" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G594" t="n">
@@ -44426,7 +44426,7 @@
       </c>
       <c r="F595" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G595" t="n">
@@ -44648,7 +44648,7 @@
       </c>
       <c r="F598" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G598" t="n">
@@ -44699,7 +44699,7 @@
     <row r="599">
       <c r="A599" t="inlineStr">
         <is>
-          <t>RPAD3</t>
+          <t>RPAD6</t>
         </is>
       </c>
       <c r="B599" t="inlineStr">
@@ -44709,7 +44709,7 @@
       </c>
       <c r="C599" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D599" t="inlineStr">
@@ -44722,7 +44722,7 @@
       </c>
       <c r="F599" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G599" t="n">
@@ -44746,13 +44746,13 @@
         <v>0.57</v>
       </c>
       <c r="M599" t="n">
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="N599" t="n">
         <v>1046150000</v>
       </c>
       <c r="O599" t="n">
-        <v>2695.56</v>
+        <v>2752.22</v>
       </c>
       <c r="P599" t="n">
         <v>0</v>
@@ -44773,7 +44773,7 @@
     <row r="600">
       <c r="A600" t="inlineStr">
         <is>
-          <t>RPAD6</t>
+          <t>RPAD3</t>
         </is>
       </c>
       <c r="B600" t="inlineStr">
@@ -44783,7 +44783,7 @@
       </c>
       <c r="C600" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D600" t="inlineStr">
@@ -44796,7 +44796,7 @@
       </c>
       <c r="F600" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G600" t="n">
@@ -44820,13 +44820,13 @@
         <v>0.57</v>
       </c>
       <c r="M600" t="n">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="N600" t="n">
         <v>1046150000</v>
       </c>
       <c r="O600" t="n">
-        <v>2752.22</v>
+        <v>2695.56</v>
       </c>
       <c r="P600" t="n">
         <v>0</v>
@@ -44870,7 +44870,7 @@
       </c>
       <c r="F601" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G601" t="n">
@@ -45092,7 +45092,7 @@
       </c>
       <c r="F604" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G604" t="n">
@@ -45536,7 +45536,7 @@
       </c>
       <c r="F610" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G610" t="n">
@@ -46720,7 +46720,7 @@
       </c>
       <c r="F626" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G626" t="n">
@@ -47164,7 +47164,7 @@
       </c>
       <c r="F632" t="inlineStr">
         <is>
-          <t>Comunicações</t>
+          <t>Telecomunicações</t>
         </is>
       </c>
       <c r="G632" t="n">
@@ -47312,7 +47312,7 @@
       </c>
       <c r="F634" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G634" t="n">
@@ -47386,7 +47386,7 @@
       </c>
       <c r="F635" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G635" t="n">
@@ -47608,7 +47608,7 @@
       </c>
       <c r="F638" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Seguradoras</t>
         </is>
       </c>
       <c r="G638" t="n">
@@ -47682,7 +47682,7 @@
       </c>
       <c r="F639" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G639" t="n">
@@ -47756,7 +47756,7 @@
       </c>
       <c r="F640" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G640" t="n">
@@ -47904,7 +47904,7 @@
       </c>
       <c r="F642" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G642" t="n">
@@ -47978,7 +47978,7 @@
       </c>
       <c r="F643" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G643" t="n">
@@ -48200,7 +48200,7 @@
       </c>
       <c r="F646" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Seguradoras</t>
         </is>
       </c>
       <c r="G646" t="n">
@@ -48496,7 +48496,7 @@
       </c>
       <c r="F650" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G650" t="n">
@@ -49236,7 +49236,7 @@
       </c>
       <c r="F660" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G660" t="n">
@@ -49458,7 +49458,7 @@
       </c>
       <c r="F663" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G663" t="n">
@@ -50124,7 +50124,7 @@
       </c>
       <c r="F672" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G672" t="n">
@@ -50420,7 +50420,7 @@
       </c>
       <c r="F676" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G676" t="n">
@@ -51086,7 +51086,7 @@
       </c>
       <c r="F685" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G685" t="n">
@@ -51160,7 +51160,7 @@
       </c>
       <c r="F686" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G686" t="n">
@@ -51234,7 +51234,7 @@
       </c>
       <c r="F687" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G687" t="n">
@@ -51382,7 +51382,7 @@
       </c>
       <c r="F689" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G689" t="n">
@@ -51604,7 +51604,7 @@
       </c>
       <c r="F692" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G692" t="n">
@@ -51752,7 +51752,7 @@
       </c>
       <c r="F694" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G694" t="n">
@@ -52862,7 +52862,7 @@
       </c>
       <c r="F709" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Saneamento</t>
         </is>
       </c>
       <c r="G709" t="n">
@@ -53972,7 +53972,7 @@
       </c>
       <c r="F724" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G724" t="n">
@@ -54416,7 +54416,7 @@
       </c>
       <c r="F730" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G730" t="n">
@@ -54490,7 +54490,7 @@
       </c>
       <c r="F731" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G731" t="n">
@@ -54860,7 +54860,7 @@
       </c>
       <c r="F736" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G736" t="n">
@@ -55304,7 +55304,7 @@
       </c>
       <c r="F742" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G742" t="n">
@@ -55378,7 +55378,7 @@
       </c>
       <c r="F743" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G743" t="n">
@@ -55748,7 +55748,7 @@
       </c>
       <c r="F748" t="inlineStr">
         <is>
-          <t>Comunicações</t>
+          <t>Telecomunicações</t>
         </is>
       </c>
       <c r="G748" t="n">
@@ -55822,7 +55822,7 @@
       </c>
       <c r="F749" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Seguradoras</t>
         </is>
       </c>
       <c r="G749" t="n">
@@ -56340,7 +56340,7 @@
       </c>
       <c r="F756" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G756" t="n">
@@ -56858,7 +56858,7 @@
       </c>
       <c r="F763" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G763" t="n">
@@ -57968,7 +57968,7 @@
       </c>
       <c r="F778" t="inlineStr">
         <is>
-          <t>Comunicações</t>
+          <t>Telecomunicações</t>
         </is>
       </c>
       <c r="G778" t="n">
@@ -58264,7 +58264,7 @@
       </c>
       <c r="F782" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G782" t="n">
@@ -58486,7 +58486,7 @@
       </c>
       <c r="F785" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G785" t="n">
@@ -59744,7 +59744,7 @@
       </c>
       <c r="F802" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G802" t="n">
@@ -59818,7 +59818,7 @@
       </c>
       <c r="F803" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Saneamento</t>
         </is>
       </c>
       <c r="G803" t="n">
@@ -60484,7 +60484,7 @@
       </c>
       <c r="F812" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G812" t="n">
@@ -61742,7 +61742,7 @@
       </c>
       <c r="F829" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G829" t="n">
@@ -61964,7 +61964,7 @@
       </c>
       <c r="F832" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G832" t="n">
@@ -62408,7 +62408,7 @@
       </c>
       <c r="F838" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G838" t="n">
@@ -62778,7 +62778,7 @@
       </c>
       <c r="F843" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G843" t="n">
@@ -63000,7 +63000,7 @@
       </c>
       <c r="F846" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G846" t="n">
@@ -63370,7 +63370,7 @@
       </c>
       <c r="F851" t="inlineStr">
         <is>
-          <t>Comunicações</t>
+          <t>Telecomunicações</t>
         </is>
       </c>
       <c r="G851" t="n">
@@ -63814,7 +63814,7 @@
       </c>
       <c r="F857" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Saneamento</t>
         </is>
       </c>
       <c r="G857" t="n">
@@ -63962,7 +63962,7 @@
       </c>
       <c r="F859" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Saneamento</t>
         </is>
       </c>
       <c r="G859" t="n">
@@ -65072,7 +65072,7 @@
       </c>
       <c r="F874" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Saneamento</t>
         </is>
       </c>
       <c r="G874" t="n">
@@ -65664,7 +65664,7 @@
       </c>
       <c r="F882" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Saneamento</t>
         </is>
       </c>
       <c r="G882" t="n">
@@ -66108,7 +66108,7 @@
       </c>
       <c r="F888" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G888" t="n">
@@ -67810,7 +67810,7 @@
       </c>
       <c r="F911" t="inlineStr">
         <is>
-          <t>Comunicações</t>
+          <t>Telecomunicações</t>
         </is>
       </c>
       <c r="G911" t="n">
@@ -69290,7 +69290,7 @@
       </c>
       <c r="F931" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G931" t="n">
@@ -69364,7 +69364,7 @@
       </c>
       <c r="F932" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Seguradoras</t>
         </is>
       </c>
       <c r="G932" t="n">
@@ -69438,7 +69438,7 @@
       </c>
       <c r="F933" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Seguradoras</t>
         </is>
       </c>
       <c r="G933" t="n">
@@ -69808,7 +69808,7 @@
       </c>
       <c r="F938" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Seguradoras</t>
         </is>
       </c>
       <c r="G938" t="n">
@@ -69956,7 +69956,7 @@
       </c>
       <c r="F940" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G940" t="n">
@@ -70992,7 +70992,7 @@
       </c>
       <c r="F954" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G954" t="n">
@@ -71140,7 +71140,7 @@
       </c>
       <c r="F956" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G956" t="n">
@@ -71635,7 +71635,7 @@
     <row r="963">
       <c r="A963" t="inlineStr">
         <is>
-          <t>PQUN4</t>
+          <t>PQUN3</t>
         </is>
       </c>
       <c r="B963" t="inlineStr">
@@ -71645,7 +71645,7 @@
       </c>
       <c r="C963" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D963" t="inlineStr">
@@ -71709,7 +71709,7 @@
     <row r="964">
       <c r="A964" t="inlineStr">
         <is>
-          <t>PQUN3</t>
+          <t>PQUN4</t>
         </is>
       </c>
       <c r="B964" t="inlineStr">
@@ -71719,7 +71719,7 @@
       </c>
       <c r="C964" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D964" t="inlineStr">
@@ -73286,7 +73286,7 @@
       </c>
       <c r="F985" t="inlineStr">
         <is>
-          <t>Comunicações</t>
+          <t>Telecomunicações</t>
         </is>
       </c>
       <c r="G985" t="n">

</xml_diff>

<commit_message>
Atualiza gerador com setores B.E.S.T e finaliza dashboard com download Excel
</commit_message>
<xml_diff>
--- a/acoes_b3.xlsx
+++ b/acoes_b3.xlsx
@@ -521,12 +521,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CLAN3</t>
+          <t>IVTT3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Empresa CLAN</t>
+          <t>Empresa IVTT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -571,7 +571,7 @@
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>1012240000</v>
+        <v>1083050000</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
@@ -586,16 +586,16 @@
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>-1.05</v>
+        <v>-0.4</v>
       </c>
       <c r="T2" t="n">
-        <v>-63.96</v>
+        <v>20.67</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MNSA4</t>
+          <t>MNSA3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.47</v>
+        <v>0.42</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -669,7 +669,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CSTB4</t>
+          <t>CSTB3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>147.69</v>
+        <v>150</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -743,12 +743,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PORP4</t>
+          <t>CFLU4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Empresa PORP</t>
+          <t>Empresa CFLU</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -762,11 +762,11 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>2.4</v>
+        <v>1000</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Seguradoras</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -793,41 +793,41 @@
         <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>22399000</v>
+        <v>60351000</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>10.72</v>
       </c>
       <c r="R5" t="n">
-        <v>0</v>
+        <v>17.68</v>
       </c>
       <c r="S5" t="n">
-        <v>-2.08</v>
+        <v>32.15</v>
       </c>
       <c r="T5" t="n">
-        <v>13.66</v>
+        <v>8.140000000000001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>IVTT3</t>
+          <t>POPR4</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Empresa IVTT</t>
+          <t>Empresa POPR</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -836,7 +836,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>10.17</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -867,36 +867,36 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>1083050000</v>
+        <v>545803000</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>0</v>
+        <v>8.66</v>
       </c>
       <c r="Q6" t="n">
-        <v>0</v>
+        <v>5.65</v>
       </c>
       <c r="R6" t="n">
-        <v>0</v>
+        <v>15.25</v>
       </c>
       <c r="S6" t="n">
-        <v>-0.4</v>
+        <v>19.93</v>
       </c>
       <c r="T6" t="n">
-        <v>20.67</v>
+        <v>30.93</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MNSA3</t>
+          <t>PMET3</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Empresa MNSA</t>
+          <t>Empresa PMET</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.42</v>
+        <v>0</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -941,41 +941,41 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>-9105000</v>
+        <v>-290863000</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>-208.15</v>
+        <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>-362.66</v>
+        <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>-13.5</v>
+        <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>145.7</v>
+        <v>4.1</v>
       </c>
       <c r="T7" t="n">
-        <v>-41.11</v>
+        <v>37.74</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CFLU4</t>
+          <t>CLAN3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Empresa CFLU</t>
+          <t>Empresa CLAN</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -984,7 +984,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1015,41 +1015,41 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>60351000</v>
+        <v>1012240000</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>8.880000000000001</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>10.72</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>17.68</v>
+        <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>32.15</v>
+        <v>-1.05</v>
       </c>
       <c r="T8" t="n">
-        <v>8.140000000000001</v>
+        <v>-63.96</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CSTB3</t>
+          <t>MNSA4</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa MNSA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1058,7 +1058,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>150</v>
+        <v>0.47</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1089,36 +1089,36 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>8420670000</v>
+        <v>-9105000</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>40.85</v>
+        <v>-208.15</v>
       </c>
       <c r="Q9" t="n">
-        <v>28.98</v>
+        <v>-362.66</v>
       </c>
       <c r="R9" t="n">
-        <v>22.4</v>
+        <v>-13.5</v>
       </c>
       <c r="S9" t="n">
-        <v>20.11</v>
+        <v>145.7</v>
       </c>
       <c r="T9" t="n">
-        <v>31.91</v>
+        <v>-41.11</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>POPR4</t>
+          <t>CSTB4</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Empresa POPR</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1132,7 +1132,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>10.17</v>
+        <v>147.69</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1163,41 +1163,41 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>545803000</v>
+        <v>8420670000</v>
       </c>
       <c r="O10" t="n">
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>8.66</v>
+        <v>40.85</v>
       </c>
       <c r="Q10" t="n">
-        <v>5.65</v>
+        <v>28.98</v>
       </c>
       <c r="R10" t="n">
-        <v>15.25</v>
+        <v>22.4</v>
       </c>
       <c r="S10" t="n">
-        <v>19.93</v>
+        <v>20.11</v>
       </c>
       <c r="T10" t="n">
-        <v>30.93</v>
+        <v>31.91</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PMET3</t>
+          <t>PORP4</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Empresa PMET</t>
+          <t>Empresa PORP</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1206,11 +1206,11 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Seguradoras</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -1237,7 +1237,7 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>-290863000</v>
+        <v>22399000</v>
       </c>
       <c r="O11" t="n">
         <v>0</v>
@@ -1252,10 +1252,10 @@
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>4.1</v>
+        <v>-2.08</v>
       </c>
       <c r="T11" t="n">
-        <v>37.74</v>
+        <v>13.66</v>
       </c>
     </row>
     <row r="12">
@@ -11325,7 +11325,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>PNOR5</t>
+          <t>PNOR6</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -11399,7 +11399,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>PNOR6</t>
+          <t>PNOR5</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -23091,12 +23091,12 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>VNET3</t>
+          <t>BERG3</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Empresa VNET</t>
+          <t>Empresa BERG</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -23110,7 +23110,7 @@
         </is>
       </c>
       <c r="E307" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="F307" t="inlineStr">
         <is>
@@ -23141,41 +23141,41 @@
         <v>0</v>
       </c>
       <c r="N307" t="n">
-        <v>14163000000</v>
+        <v>9538000</v>
       </c>
       <c r="O307" t="n">
         <v>0</v>
       </c>
       <c r="P307" t="n">
-        <v>0</v>
+        <v>-8.6</v>
       </c>
       <c r="Q307" t="n">
-        <v>0</v>
+        <v>-32.6</v>
       </c>
       <c r="R307" t="n">
-        <v>0</v>
+        <v>-5.58</v>
       </c>
       <c r="S307" t="n">
-        <v>0</v>
+        <v>-102.71</v>
       </c>
       <c r="T307" t="n">
-        <v>1.08</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>CSPC4</t>
+          <t>JBDU3</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa JBDU</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D308" t="inlineStr">
@@ -23184,7 +23184,7 @@
         </is>
       </c>
       <c r="E308" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="F308" t="inlineStr">
         <is>
@@ -23215,36 +23215,36 @@
         <v>0</v>
       </c>
       <c r="N308" t="n">
-        <v>2126670000</v>
+        <v>56569000</v>
       </c>
       <c r="O308" t="n">
         <v>0</v>
       </c>
       <c r="P308" t="n">
-        <v>38.62</v>
+        <v>0</v>
       </c>
       <c r="Q308" t="n">
-        <v>18.85</v>
+        <v>0</v>
       </c>
       <c r="R308" t="n">
-        <v>29.18</v>
+        <v>0</v>
       </c>
       <c r="S308" t="n">
-        <v>45.33</v>
+        <v>0</v>
       </c>
       <c r="T308" t="n">
-        <v>41.15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>BOVH3</t>
+          <t>EGGY3</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Empresa BOVH</t>
+          <t>Empresa EGGY</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -23258,7 +23258,7 @@
         </is>
       </c>
       <c r="E309" t="n">
-        <v>15.71</v>
+        <v>0</v>
       </c>
       <c r="F309" t="inlineStr">
         <is>
@@ -23283,13 +23283,13 @@
         <v>0</v>
       </c>
       <c r="L309" t="n">
-        <v>6.16</v>
+        <v>0</v>
       </c>
       <c r="M309" t="n">
         <v>0</v>
       </c>
       <c r="N309" t="n">
-        <v>1843320000</v>
+        <v>954480000</v>
       </c>
       <c r="O309" t="n">
         <v>0</v>
@@ -23307,43 +23307,43 @@
         <v>0</v>
       </c>
       <c r="T309" t="n">
-        <v>0</v>
+        <v>-0.82</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>ARND3</t>
+          <t>CBMA4</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Empresa ARND</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Novo Mercado</t>
+          <t>Tradicional</t>
         </is>
       </c>
       <c r="E310" t="n">
-        <v>0.51</v>
+        <v>0.01</v>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G310" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="H310" t="n">
-        <v>12.49</v>
+        <v>0</v>
       </c>
       <c r="I310" t="inlineStr">
         <is>
@@ -23357,16 +23357,16 @@
         <v>0</v>
       </c>
       <c r="L310" t="n">
-        <v>0.57</v>
+        <v>0</v>
       </c>
       <c r="M310" t="n">
         <v>0</v>
       </c>
       <c r="N310" t="n">
-        <v>125211000</v>
+        <v>-34022300000</v>
       </c>
       <c r="O310" t="n">
-        <v>913.58</v>
+        <v>0</v>
       </c>
       <c r="P310" t="n">
         <v>0</v>
@@ -23381,18 +23381,18 @@
         <v>0</v>
       </c>
       <c r="T310" t="n">
-        <v>-0.88</v>
+        <v>252.65</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>PTIP4</t>
+          <t>SALM4</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -23406,7 +23406,7 @@
         </is>
       </c>
       <c r="E311" t="n">
-        <v>25.15</v>
+        <v>5.9</v>
       </c>
       <c r="F311" t="inlineStr">
         <is>
@@ -23437,36 +23437,36 @@
         <v>0</v>
       </c>
       <c r="N311" t="n">
-        <v>-155957000</v>
+        <v>475600000</v>
       </c>
       <c r="O311" t="n">
         <v>0</v>
       </c>
       <c r="P311" t="n">
-        <v>13.73</v>
+        <v>10.22</v>
       </c>
       <c r="Q311" t="n">
-        <v>7.55</v>
+        <v>4.13</v>
       </c>
       <c r="R311" t="n">
-        <v>23.13</v>
+        <v>25.78</v>
       </c>
       <c r="S311" t="n">
-        <v>-121.74</v>
+        <v>19.53</v>
       </c>
       <c r="T311" t="n">
-        <v>62.11</v>
+        <v>24.53</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>LATS3</t>
+          <t>BMEF3</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Empresa LATS</t>
+          <t>Empresa BMEF</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -23480,7 +23480,7 @@
         </is>
       </c>
       <c r="E312" t="n">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="F312" t="inlineStr">
         <is>
@@ -23505,42 +23505,42 @@
         <v>0</v>
       </c>
       <c r="L312" t="n">
-        <v>0</v>
+        <v>4.16</v>
       </c>
       <c r="M312" t="n">
         <v>0</v>
       </c>
       <c r="N312" t="n">
-        <v>680646000</v>
+        <v>2674780000</v>
       </c>
       <c r="O312" t="n">
         <v>0</v>
       </c>
       <c r="P312" t="n">
-        <v>11.74</v>
+        <v>0</v>
       </c>
       <c r="Q312" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="R312" t="n">
-        <v>11.63</v>
+        <v>0</v>
       </c>
       <c r="S312" t="n">
-        <v>1.84</v>
+        <v>0</v>
       </c>
       <c r="T312" t="n">
-        <v>15.37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>VVAX3</t>
+          <t>AGEI3</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa AGEI</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -23554,7 +23554,7 @@
         </is>
       </c>
       <c r="E313" t="n">
-        <v>0</v>
+        <v>7.8</v>
       </c>
       <c r="F313" t="inlineStr">
         <is>
@@ -23579,28 +23579,28 @@
         <v>0</v>
       </c>
       <c r="L313" t="n">
-        <v>0</v>
+        <v>1.25</v>
       </c>
       <c r="M313" t="n">
         <v>0</v>
       </c>
       <c r="N313" t="n">
-        <v>144676000</v>
+        <v>1878210000</v>
       </c>
       <c r="O313" t="n">
         <v>0</v>
       </c>
       <c r="P313" t="n">
-        <v>-7.36</v>
+        <v>0</v>
       </c>
       <c r="Q313" t="n">
-        <v>-37.76</v>
+        <v>0</v>
       </c>
       <c r="R313" t="n">
-        <v>-6.52</v>
+        <v>0</v>
       </c>
       <c r="S313" t="n">
-        <v>-92.03</v>
+        <v>0</v>
       </c>
       <c r="T313" t="n">
         <v>0</v>
@@ -23609,17 +23609,17 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>MSAN4</t>
+          <t>SASG3</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa SASG</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
@@ -23628,7 +23628,7 @@
         </is>
       </c>
       <c r="E314" t="n">
-        <v>6.44</v>
+        <v>0.98</v>
       </c>
       <c r="F314" t="inlineStr">
         <is>
@@ -23659,41 +23659,41 @@
         <v>0</v>
       </c>
       <c r="N314" t="n">
-        <v>2533030000</v>
+        <v>0</v>
       </c>
       <c r="O314" t="n">
         <v>0</v>
       </c>
       <c r="P314" t="n">
-        <v>6.27</v>
+        <v>0</v>
       </c>
       <c r="Q314" t="n">
-        <v>2.42</v>
+        <v>0</v>
       </c>
       <c r="R314" t="n">
-        <v>11.78</v>
+        <v>0</v>
       </c>
       <c r="S314" t="n">
-        <v>11.81</v>
+        <v>0</v>
       </c>
       <c r="T314" t="n">
-        <v>101.35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>GALO4</t>
+          <t>ODER3</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa ODER</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
@@ -23702,18 +23702,18 @@
         </is>
       </c>
       <c r="E315" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Consumo não Cíclico</t>
         </is>
       </c>
       <c r="G315" t="n">
         <v>80</v>
       </c>
       <c r="H315" t="n">
-        <v>0</v>
+        <v>1.75</v>
       </c>
       <c r="I315" t="inlineStr">
         <is>
@@ -23733,36 +23733,36 @@
         <v>0</v>
       </c>
       <c r="N315" t="n">
-        <v>-60607000</v>
+        <v>609518000</v>
       </c>
       <c r="O315" t="n">
         <v>0</v>
       </c>
       <c r="P315" t="n">
-        <v>13.98</v>
+        <v>0</v>
       </c>
       <c r="Q315" t="n">
-        <v>-184.58</v>
+        <v>0</v>
       </c>
       <c r="R315" t="n">
-        <v>39.37</v>
+        <v>0</v>
       </c>
       <c r="S315" t="n">
-        <v>7.62</v>
+        <v>0</v>
       </c>
       <c r="T315" t="n">
-        <v>-28.97</v>
+        <v>3.17</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>BBTG13</t>
+          <t>ARPS3</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -23776,7 +23776,7 @@
         </is>
       </c>
       <c r="E316" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="F316" t="inlineStr">
         <is>
@@ -23807,41 +23807,41 @@
         <v>0</v>
       </c>
       <c r="N316" t="n">
-        <v>7000</v>
+        <v>-12690000</v>
       </c>
       <c r="O316" t="n">
         <v>0</v>
       </c>
       <c r="P316" t="n">
-        <v>0</v>
+        <v>-4.92</v>
       </c>
       <c r="Q316" t="n">
-        <v>0</v>
+        <v>-11.59</v>
       </c>
       <c r="R316" t="n">
-        <v>0</v>
+        <v>-6.64</v>
       </c>
       <c r="S316" t="n">
-        <v>-42.86</v>
+        <v>20.34</v>
       </c>
       <c r="T316" t="n">
-        <v>0</v>
+        <v>-17.53</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>INHA3</t>
+          <t>VVAX4</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Empresa INHA</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D317" t="inlineStr">
@@ -23881,36 +23881,36 @@
         <v>0</v>
       </c>
       <c r="N317" t="n">
-        <v>1533210000</v>
+        <v>144676000</v>
       </c>
       <c r="O317" t="n">
         <v>0</v>
       </c>
       <c r="P317" t="n">
-        <v>-56.05</v>
+        <v>-7.36</v>
       </c>
       <c r="Q317" t="n">
-        <v>-124.06</v>
+        <v>-37.76</v>
       </c>
       <c r="R317" t="n">
-        <v>-6.27</v>
+        <v>-6.52</v>
       </c>
       <c r="S317" t="n">
-        <v>-39.87</v>
+        <v>-92.03</v>
       </c>
       <c r="T317" t="n">
-        <v>-12.18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>VSPT3</t>
+          <t>CSPC3</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -23924,11 +23924,11 @@
         </is>
       </c>
       <c r="E318" t="n">
-        <v>0</v>
+        <v>1.24</v>
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t>Bens Industriais</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G318" t="n">
@@ -23943,7 +23943,7 @@
         </is>
       </c>
       <c r="J318" t="n">
-        <v>-0.43</v>
+        <v>0</v>
       </c>
       <c r="K318" t="n">
         <v>0</v>
@@ -23955,41 +23955,41 @@
         <v>0</v>
       </c>
       <c r="N318" t="n">
-        <v>5031600000</v>
+        <v>2126670000</v>
       </c>
       <c r="O318" t="n">
         <v>0</v>
       </c>
       <c r="P318" t="n">
-        <v>0</v>
+        <v>38.62</v>
       </c>
       <c r="Q318" t="n">
-        <v>0</v>
+        <v>18.85</v>
       </c>
       <c r="R318" t="n">
-        <v>0</v>
+        <v>29.18</v>
       </c>
       <c r="S318" t="n">
-        <v>0</v>
+        <v>45.33</v>
       </c>
       <c r="T318" t="n">
-        <v>4.92</v>
+        <v>41.15</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>SGEN4</t>
+          <t>ABCB3</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa ABCB</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
@@ -23998,11 +23998,11 @@
         </is>
       </c>
       <c r="E319" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G319" t="n">
@@ -24023,47 +24023,47 @@
         <v>0</v>
       </c>
       <c r="L319" t="n">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="M319" t="n">
         <v>0</v>
       </c>
       <c r="N319" t="n">
-        <v>156981000</v>
+        <v>7258910000</v>
       </c>
       <c r="O319" t="n">
         <v>0</v>
       </c>
       <c r="P319" t="n">
-        <v>-1871.17</v>
+        <v>0</v>
       </c>
       <c r="Q319" t="n">
         <v>0</v>
       </c>
       <c r="R319" t="n">
-        <v>-1.59</v>
+        <v>0</v>
       </c>
       <c r="S319" t="n">
-        <v>0</v>
+        <v>14.05</v>
       </c>
       <c r="T319" t="n">
-        <v>-59.85</v>
+        <v>7.57</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>CCHI4</t>
+          <t>CCTY3</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa CCTY</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D320" t="inlineStr">
@@ -24072,7 +24072,7 @@
         </is>
       </c>
       <c r="E320" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="F320" t="inlineStr">
         <is>
@@ -24097,13 +24097,13 @@
         <v>0</v>
       </c>
       <c r="L320" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="M320" t="n">
         <v>0</v>
       </c>
       <c r="N320" t="n">
-        <v>-160477000</v>
+        <v>0</v>
       </c>
       <c r="O320" t="n">
         <v>0</v>
@@ -24121,23 +24121,23 @@
         <v>0</v>
       </c>
       <c r="T320" t="n">
-        <v>20.36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>REPA3</t>
+          <t>BAUH4</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa BAUH</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D321" t="inlineStr">
@@ -24146,18 +24146,18 @@
         </is>
       </c>
       <c r="E321" t="n">
-        <v>1</v>
+        <v>93.39</v>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Consumo não Cíclico</t>
         </is>
       </c>
       <c r="G321" t="n">
         <v>80</v>
       </c>
       <c r="H321" t="n">
-        <v>0</v>
+        <v>28.89</v>
       </c>
       <c r="I321" t="inlineStr">
         <is>
@@ -24165,53 +24165,53 @@
         </is>
       </c>
       <c r="J321" t="n">
-        <v>0</v>
+        <v>-2.88</v>
       </c>
       <c r="K321" t="n">
         <v>0</v>
       </c>
       <c r="L321" t="n">
-        <v>0</v>
+        <v>3.18</v>
       </c>
       <c r="M321" t="n">
-        <v>0</v>
+        <v>1.16</v>
       </c>
       <c r="N321" t="n">
-        <v>378378000</v>
+        <v>153407000</v>
       </c>
       <c r="O321" t="n">
-        <v>0</v>
+        <v>207.53</v>
       </c>
       <c r="P321" t="n">
-        <v>5.18</v>
+        <v>0</v>
       </c>
       <c r="Q321" t="n">
-        <v>1.22</v>
+        <v>0</v>
       </c>
       <c r="R321" t="n">
-        <v>4.05</v>
+        <v>0</v>
       </c>
       <c r="S321" t="n">
-        <v>1.91</v>
+        <v>0</v>
       </c>
       <c r="T321" t="n">
-        <v>1.09</v>
+        <v>13.32</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>EQMA5B</t>
+          <t>ICPI3</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa ICPI</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
@@ -24251,7 +24251,7 @@
         <v>0</v>
       </c>
       <c r="N322" t="n">
-        <v>4940330000</v>
+        <v>0</v>
       </c>
       <c r="O322" t="n">
         <v>0</v>
@@ -24269,23 +24269,23 @@
         <v>0</v>
       </c>
       <c r="T322" t="n">
-        <v>9.050000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>SEBB3</t>
+          <t>ILLS4</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa ILLS</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D323" t="inlineStr">
@@ -24294,7 +24294,7 @@
         </is>
       </c>
       <c r="E323" t="n">
-        <v>0</v>
+        <v>100.01</v>
       </c>
       <c r="F323" t="inlineStr">
         <is>
@@ -24325,41 +24325,41 @@
         <v>0</v>
       </c>
       <c r="N323" t="n">
-        <v>145783000</v>
+        <v>-18567000</v>
       </c>
       <c r="O323" t="n">
         <v>0</v>
       </c>
       <c r="P323" t="n">
-        <v>9.24</v>
+        <v>8.43</v>
       </c>
       <c r="Q323" t="n">
-        <v>7.4</v>
+        <v>-10.22</v>
       </c>
       <c r="R323" t="n">
-        <v>24.15</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="S323" t="n">
-        <v>23.01</v>
+        <v>36.09</v>
       </c>
       <c r="T323" t="n">
-        <v>50.04</v>
+        <v>9.33</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>BBTG11</t>
+          <t>ESTC4</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa ESTC</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>UNT</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D324" t="inlineStr">
@@ -24368,7 +24368,7 @@
         </is>
       </c>
       <c r="E324" t="n">
-        <v>15.01</v>
+        <v>0</v>
       </c>
       <c r="F324" t="inlineStr">
         <is>
@@ -24399,36 +24399,36 @@
         <v>0</v>
       </c>
       <c r="N324" t="n">
-        <v>0</v>
+        <v>2916530000</v>
       </c>
       <c r="O324" t="n">
         <v>0</v>
       </c>
       <c r="P324" t="n">
-        <v>0</v>
+        <v>16.91</v>
       </c>
       <c r="Q324" t="n">
-        <v>0</v>
+        <v>2.02</v>
       </c>
       <c r="R324" t="n">
-        <v>0</v>
+        <v>11.35</v>
       </c>
       <c r="S324" t="n">
-        <v>0</v>
+        <v>3.89</v>
       </c>
       <c r="T324" t="n">
-        <v>0</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>JFAB4</t>
+          <t>VSPT4</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Empresa JFAB</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -24442,11 +24442,11 @@
         </is>
       </c>
       <c r="E325" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bens Industriais</t>
         </is>
       </c>
       <c r="G325" t="n">
@@ -24461,7 +24461,7 @@
         </is>
       </c>
       <c r="J325" t="n">
-        <v>0</v>
+        <v>-0.43</v>
       </c>
       <c r="K325" t="n">
         <v>0</v>
@@ -24473,7 +24473,7 @@
         <v>0</v>
       </c>
       <c r="N325" t="n">
-        <v>-10183000</v>
+        <v>5031600000</v>
       </c>
       <c r="O325" t="n">
         <v>0</v>
@@ -24488,26 +24488,26 @@
         <v>0</v>
       </c>
       <c r="S325" t="n">
-        <v>2.34</v>
+        <v>0</v>
       </c>
       <c r="T325" t="n">
-        <v>0</v>
+        <v>4.92</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>TNEP3</t>
+          <t>SEBB4</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D326" t="inlineStr">
@@ -24516,7 +24516,7 @@
         </is>
       </c>
       <c r="E326" t="n">
-        <v>3.01</v>
+        <v>0</v>
       </c>
       <c r="F326" t="inlineStr">
         <is>
@@ -24547,36 +24547,36 @@
         <v>0</v>
       </c>
       <c r="N326" t="n">
-        <v>955105000</v>
+        <v>145783000</v>
       </c>
       <c r="O326" t="n">
         <v>0</v>
       </c>
       <c r="P326" t="n">
-        <v>20.92</v>
+        <v>9.24</v>
       </c>
       <c r="Q326" t="n">
-        <v>25.42</v>
+        <v>7.4</v>
       </c>
       <c r="R326" t="n">
-        <v>20.53</v>
+        <v>24.15</v>
       </c>
       <c r="S326" t="n">
-        <v>22.8</v>
+        <v>23.01</v>
       </c>
       <c r="T326" t="n">
-        <v>8.15</v>
+        <v>50.04</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>LECO3</t>
+          <t>MSAN3</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Empresa LECO</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -24590,7 +24590,7 @@
         </is>
       </c>
       <c r="E327" t="n">
-        <v>0</v>
+        <v>6.44</v>
       </c>
       <c r="F327" t="inlineStr">
         <is>
@@ -24621,36 +24621,36 @@
         <v>0</v>
       </c>
       <c r="N327" t="n">
-        <v>105928000</v>
+        <v>2533030000</v>
       </c>
       <c r="O327" t="n">
         <v>0</v>
       </c>
       <c r="P327" t="n">
-        <v>-2.14</v>
+        <v>6.27</v>
       </c>
       <c r="Q327" t="n">
-        <v>-4.72</v>
+        <v>2.42</v>
       </c>
       <c r="R327" t="n">
-        <v>-3.48</v>
+        <v>11.78</v>
       </c>
       <c r="S327" t="n">
-        <v>-14.82</v>
+        <v>11.81</v>
       </c>
       <c r="T327" t="n">
-        <v>3.58</v>
+        <v>101.35</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>VGOR3</t>
+          <t>GALO3</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Empresa VGOR</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -24695,41 +24695,41 @@
         <v>0</v>
       </c>
       <c r="N328" t="n">
-        <v>135178000</v>
+        <v>-60607000</v>
       </c>
       <c r="O328" t="n">
         <v>0</v>
       </c>
       <c r="P328" t="n">
-        <v>4.5</v>
+        <v>13.98</v>
       </c>
       <c r="Q328" t="n">
-        <v>-4.59</v>
+        <v>-184.58</v>
       </c>
       <c r="R328" t="n">
-        <v>6</v>
+        <v>39.37</v>
       </c>
       <c r="S328" t="n">
-        <v>-24.29</v>
+        <v>7.62</v>
       </c>
       <c r="T328" t="n">
-        <v>4.77</v>
+        <v>-28.97</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>ECIS4</t>
+          <t>SLCP3</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa SLCP</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D329" t="inlineStr">
@@ -24738,7 +24738,7 @@
         </is>
       </c>
       <c r="E329" t="n">
-        <v>145</v>
+        <v>610.02</v>
       </c>
       <c r="F329" t="inlineStr">
         <is>
@@ -24769,36 +24769,36 @@
         <v>0</v>
       </c>
       <c r="N329" t="n">
-        <v>129346000</v>
+        <v>0</v>
       </c>
       <c r="O329" t="n">
         <v>0</v>
       </c>
       <c r="P329" t="n">
-        <v>34.9</v>
+        <v>0</v>
       </c>
       <c r="Q329" t="n">
-        <v>14.18</v>
+        <v>0</v>
       </c>
       <c r="R329" t="n">
-        <v>12.48</v>
+        <v>0</v>
       </c>
       <c r="S329" t="n">
-        <v>7.33</v>
+        <v>0</v>
       </c>
       <c r="T329" t="n">
-        <v>4.66</v>
+        <v>0</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>EGGY3</t>
+          <t>DAYC3</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Empresa EGGY</t>
+          <t>Empresa DAYC</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -24843,7 +24843,7 @@
         <v>0</v>
       </c>
       <c r="N330" t="n">
-        <v>954480000</v>
+        <v>3009030000</v>
       </c>
       <c r="O330" t="n">
         <v>0</v>
@@ -24858,26 +24858,26 @@
         <v>0</v>
       </c>
       <c r="S330" t="n">
-        <v>0</v>
+        <v>17.33</v>
       </c>
       <c r="T330" t="n">
-        <v>-0.82</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>CBMA4</t>
+          <t>PTIP3</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
@@ -24886,7 +24886,7 @@
         </is>
       </c>
       <c r="E331" t="n">
-        <v>0.01</v>
+        <v>22</v>
       </c>
       <c r="F331" t="inlineStr">
         <is>
@@ -24917,36 +24917,36 @@
         <v>0</v>
       </c>
       <c r="N331" t="n">
-        <v>-34022300000</v>
+        <v>-155957000</v>
       </c>
       <c r="O331" t="n">
         <v>0</v>
       </c>
       <c r="P331" t="n">
-        <v>0</v>
+        <v>13.73</v>
       </c>
       <c r="Q331" t="n">
-        <v>0</v>
+        <v>7.55</v>
       </c>
       <c r="R331" t="n">
-        <v>0</v>
+        <v>23.13</v>
       </c>
       <c r="S331" t="n">
-        <v>0</v>
+        <v>-121.74</v>
       </c>
       <c r="T331" t="n">
-        <v>252.65</v>
+        <v>62.11</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>SALM4</t>
+          <t>REPA4</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -24960,7 +24960,7 @@
         </is>
       </c>
       <c r="E332" t="n">
-        <v>5.9</v>
+        <v>1.08</v>
       </c>
       <c r="F332" t="inlineStr">
         <is>
@@ -24991,41 +24991,41 @@
         <v>0</v>
       </c>
       <c r="N332" t="n">
-        <v>475600000</v>
+        <v>378378000</v>
       </c>
       <c r="O332" t="n">
         <v>0</v>
       </c>
       <c r="P332" t="n">
-        <v>10.22</v>
+        <v>5.18</v>
       </c>
       <c r="Q332" t="n">
-        <v>4.13</v>
+        <v>1.22</v>
       </c>
       <c r="R332" t="n">
-        <v>25.78</v>
+        <v>4.05</v>
       </c>
       <c r="S332" t="n">
-        <v>19.53</v>
+        <v>1.91</v>
       </c>
       <c r="T332" t="n">
-        <v>24.53</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>BERG3</t>
+          <t>EQMA6B</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Empresa BERG</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">
@@ -25034,7 +25034,7 @@
         </is>
       </c>
       <c r="E333" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="F333" t="inlineStr">
         <is>
@@ -25065,36 +25065,36 @@
         <v>0</v>
       </c>
       <c r="N333" t="n">
-        <v>9538000</v>
+        <v>4940330000</v>
       </c>
       <c r="O333" t="n">
         <v>0</v>
       </c>
       <c r="P333" t="n">
-        <v>-8.6</v>
+        <v>0</v>
       </c>
       <c r="Q333" t="n">
-        <v>-32.6</v>
+        <v>0</v>
       </c>
       <c r="R333" t="n">
-        <v>-5.58</v>
+        <v>0</v>
       </c>
       <c r="S333" t="n">
-        <v>-102.71</v>
+        <v>0</v>
       </c>
       <c r="T333" t="n">
-        <v>-8</v>
+        <v>9.050000000000001</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>JBDU3</t>
+          <t>SGEN3</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Empresa JBDU</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -25108,7 +25108,7 @@
         </is>
       </c>
       <c r="E334" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F334" t="inlineStr">
         <is>
@@ -25133,47 +25133,47 @@
         <v>0</v>
       </c>
       <c r="L334" t="n">
-        <v>0</v>
+        <v>0.77</v>
       </c>
       <c r="M334" t="n">
         <v>0</v>
       </c>
       <c r="N334" t="n">
-        <v>56569000</v>
+        <v>156981000</v>
       </c>
       <c r="O334" t="n">
         <v>0</v>
       </c>
       <c r="P334" t="n">
-        <v>0</v>
+        <v>-1871.17</v>
       </c>
       <c r="Q334" t="n">
         <v>0</v>
       </c>
       <c r="R334" t="n">
-        <v>0</v>
+        <v>-1.59</v>
       </c>
       <c r="S334" t="n">
         <v>0</v>
       </c>
       <c r="T334" t="n">
-        <v>0</v>
+        <v>-59.85</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>AGEI3</t>
+          <t>DUFB11</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Empresa AGEI</t>
+          <t>Empresa DUFB</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
@@ -25182,7 +25182,7 @@
         </is>
       </c>
       <c r="E335" t="n">
-        <v>7.8</v>
+        <v>0</v>
       </c>
       <c r="F335" t="inlineStr">
         <is>
@@ -25207,13 +25207,13 @@
         <v>0</v>
       </c>
       <c r="L335" t="n">
-        <v>1.25</v>
+        <v>0</v>
       </c>
       <c r="M335" t="n">
         <v>0</v>
       </c>
       <c r="N335" t="n">
-        <v>1878210000</v>
+        <v>0</v>
       </c>
       <c r="O335" t="n">
         <v>0</v>
@@ -25237,17 +25237,17 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>SASG3</t>
+          <t>TNEP4</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Empresa SASG</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
@@ -25256,7 +25256,7 @@
         </is>
       </c>
       <c r="E336" t="n">
-        <v>0.98</v>
+        <v>3.95</v>
       </c>
       <c r="F336" t="inlineStr">
         <is>
@@ -25287,36 +25287,36 @@
         <v>0</v>
       </c>
       <c r="N336" t="n">
-        <v>0</v>
+        <v>955105000</v>
       </c>
       <c r="O336" t="n">
         <v>0</v>
       </c>
       <c r="P336" t="n">
-        <v>0</v>
+        <v>20.92</v>
       </c>
       <c r="Q336" t="n">
-        <v>0</v>
+        <v>25.42</v>
       </c>
       <c r="R336" t="n">
-        <v>0</v>
+        <v>20.53</v>
       </c>
       <c r="S336" t="n">
-        <v>0</v>
+        <v>22.8</v>
       </c>
       <c r="T336" t="n">
-        <v>0</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>BMEF3</t>
+          <t>MLPA3</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Empresa BMEF</t>
+          <t>Empresa MLPA</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -25330,7 +25330,7 @@
         </is>
       </c>
       <c r="E337" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F337" t="inlineStr">
         <is>
@@ -25355,75 +25355,75 @@
         <v>0</v>
       </c>
       <c r="L337" t="n">
-        <v>4.16</v>
+        <v>0</v>
       </c>
       <c r="M337" t="n">
         <v>0</v>
       </c>
       <c r="N337" t="n">
-        <v>2674780000</v>
+        <v>44578000</v>
       </c>
       <c r="O337" t="n">
         <v>0</v>
       </c>
       <c r="P337" t="n">
-        <v>0</v>
+        <v>6.66</v>
       </c>
       <c r="Q337" t="n">
-        <v>0</v>
+        <v>8.92</v>
       </c>
       <c r="R337" t="n">
         <v>0</v>
       </c>
       <c r="S337" t="n">
-        <v>0</v>
+        <v>45.13</v>
       </c>
       <c r="T337" t="n">
-        <v>0</v>
+        <v>-7.51</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>ARPS3</t>
+          <t>CLSC6</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa CLSC</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Tradicional</t>
+          <t>Nível 2</t>
         </is>
       </c>
       <c r="E338" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G338" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="H338" t="n">
-        <v>0</v>
+        <v>75.73</v>
       </c>
       <c r="I338" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="J338" t="n">
-        <v>0</v>
+        <v>2.73</v>
       </c>
       <c r="K338" t="n">
         <v>0</v>
@@ -25435,36 +25435,36 @@
         <v>0</v>
       </c>
       <c r="N338" t="n">
-        <v>-12690000</v>
+        <v>4228180000</v>
       </c>
       <c r="O338" t="n">
         <v>0</v>
       </c>
       <c r="P338" t="n">
-        <v>-4.92</v>
+        <v>0</v>
       </c>
       <c r="Q338" t="n">
-        <v>-11.59</v>
+        <v>0</v>
       </c>
       <c r="R338" t="n">
-        <v>-6.64</v>
+        <v>0</v>
       </c>
       <c r="S338" t="n">
-        <v>20.34</v>
+        <v>0</v>
       </c>
       <c r="T338" t="n">
-        <v>-17.53</v>
+        <v>2.82</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>ODER3</t>
+          <t>CCHI3</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Empresa ODER</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -25478,18 +25478,18 @@
         </is>
       </c>
       <c r="E339" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t>Consumo não Cíclico</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G339" t="n">
         <v>80</v>
       </c>
       <c r="H339" t="n">
-        <v>1.75</v>
+        <v>0</v>
       </c>
       <c r="I339" t="inlineStr">
         <is>
@@ -25503,13 +25503,13 @@
         <v>0</v>
       </c>
       <c r="L339" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="M339" t="n">
         <v>0</v>
       </c>
       <c r="N339" t="n">
-        <v>609518000</v>
+        <v>-160477000</v>
       </c>
       <c r="O339" t="n">
         <v>0</v>
@@ -25527,18 +25527,18 @@
         <v>0</v>
       </c>
       <c r="T339" t="n">
-        <v>3.17</v>
+        <v>20.36</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>CCTY3</t>
+          <t>SFSA3</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Empresa CCTY</t>
+          <t>Empresa SFSA</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -25583,7 +25583,7 @@
         <v>0</v>
       </c>
       <c r="N340" t="n">
-        <v>0</v>
+        <v>739524000</v>
       </c>
       <c r="O340" t="n">
         <v>0</v>
@@ -25598,26 +25598,26 @@
         <v>0</v>
       </c>
       <c r="S340" t="n">
-        <v>0</v>
+        <v>6.25</v>
       </c>
       <c r="T340" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>VVAX4</t>
+          <t>PRBC3</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa PRBC</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
@@ -25657,36 +25657,36 @@
         <v>0</v>
       </c>
       <c r="N341" t="n">
-        <v>144676000</v>
+        <v>1319270000</v>
       </c>
       <c r="O341" t="n">
         <v>0</v>
       </c>
       <c r="P341" t="n">
-        <v>-7.36</v>
+        <v>0</v>
       </c>
       <c r="Q341" t="n">
-        <v>-37.76</v>
+        <v>0</v>
       </c>
       <c r="R341" t="n">
-        <v>-6.52</v>
+        <v>0</v>
       </c>
       <c r="S341" t="n">
-        <v>-92.03</v>
+        <v>8.27</v>
       </c>
       <c r="T341" t="n">
-        <v>0</v>
+        <v>-1.98</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>CSPC3</t>
+          <t>ECIS3</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -25700,7 +25700,7 @@
         </is>
       </c>
       <c r="E342" t="n">
-        <v>1.24</v>
+        <v>211.65</v>
       </c>
       <c r="F342" t="inlineStr">
         <is>
@@ -25731,36 +25731,36 @@
         <v>0</v>
       </c>
       <c r="N342" t="n">
-        <v>2126670000</v>
+        <v>129346000</v>
       </c>
       <c r="O342" t="n">
         <v>0</v>
       </c>
       <c r="P342" t="n">
-        <v>38.62</v>
+        <v>34.9</v>
       </c>
       <c r="Q342" t="n">
-        <v>18.85</v>
+        <v>14.18</v>
       </c>
       <c r="R342" t="n">
-        <v>29.18</v>
+        <v>12.48</v>
       </c>
       <c r="S342" t="n">
-        <v>45.33</v>
+        <v>7.33</v>
       </c>
       <c r="T342" t="n">
-        <v>41.15</v>
+        <v>4.66</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>ABCB3</t>
+          <t>CZRS3</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Empresa ABCB</t>
+          <t>Empresa CZRS</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -25778,7 +25778,7 @@
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t>Bancos</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G343" t="n">
@@ -25805,7 +25805,7 @@
         <v>0</v>
       </c>
       <c r="N343" t="n">
-        <v>7258910000</v>
+        <v>1145670000</v>
       </c>
       <c r="O343" t="n">
         <v>0</v>
@@ -25820,26 +25820,26 @@
         <v>0</v>
       </c>
       <c r="S343" t="n">
-        <v>14.05</v>
+        <v>3.34</v>
       </c>
       <c r="T343" t="n">
-        <v>7.57</v>
+        <v>14.44</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>ESTC4</t>
+          <t>BPNM3</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Empresa ESTC</t>
+          <t>Empresa BPNM</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D344" t="inlineStr">
@@ -25879,41 +25879,41 @@
         <v>0</v>
       </c>
       <c r="N344" t="n">
-        <v>2916530000</v>
+        <v>7792670000</v>
       </c>
       <c r="O344" t="n">
         <v>0</v>
       </c>
       <c r="P344" t="n">
-        <v>16.91</v>
+        <v>0</v>
       </c>
       <c r="Q344" t="n">
-        <v>2.02</v>
+        <v>0</v>
       </c>
       <c r="R344" t="n">
-        <v>11.35</v>
+        <v>0</v>
       </c>
       <c r="S344" t="n">
-        <v>3.89</v>
+        <v>9.67</v>
       </c>
       <c r="T344" t="n">
-        <v>5.6</v>
+        <v>-1.53</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>VSPT4</t>
+          <t>BSGR3</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa BSGR</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D345" t="inlineStr">
@@ -25922,11 +25922,11 @@
         </is>
       </c>
       <c r="E345" t="n">
-        <v>0</v>
+        <v>1091.28</v>
       </c>
       <c r="F345" t="inlineStr">
         <is>
-          <t>Bens Industriais</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G345" t="n">
@@ -25941,7 +25941,7 @@
         </is>
       </c>
       <c r="J345" t="n">
-        <v>-0.43</v>
+        <v>0</v>
       </c>
       <c r="K345" t="n">
         <v>0</v>
@@ -25953,7 +25953,7 @@
         <v>0</v>
       </c>
       <c r="N345" t="n">
-        <v>5031600000</v>
+        <v>0</v>
       </c>
       <c r="O345" t="n">
         <v>0</v>
@@ -25971,23 +25971,23 @@
         <v>0</v>
       </c>
       <c r="T345" t="n">
-        <v>4.92</v>
+        <v>0</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>BAUH4</t>
+          <t>CBMA3</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Empresa BAUH</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D346" t="inlineStr">
@@ -25996,18 +25996,18 @@
         </is>
       </c>
       <c r="E346" t="n">
-        <v>93.39</v>
+        <v>0.01</v>
       </c>
       <c r="F346" t="inlineStr">
         <is>
-          <t>Consumo não Cíclico</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G346" t="n">
         <v>80</v>
       </c>
       <c r="H346" t="n">
-        <v>28.89</v>
+        <v>0</v>
       </c>
       <c r="I346" t="inlineStr">
         <is>
@@ -26015,22 +26015,22 @@
         </is>
       </c>
       <c r="J346" t="n">
-        <v>-2.88</v>
+        <v>0</v>
       </c>
       <c r="K346" t="n">
         <v>0</v>
       </c>
       <c r="L346" t="n">
-        <v>3.18</v>
+        <v>0</v>
       </c>
       <c r="M346" t="n">
-        <v>1.16</v>
+        <v>0</v>
       </c>
       <c r="N346" t="n">
-        <v>153407000</v>
+        <v>-34022300000</v>
       </c>
       <c r="O346" t="n">
-        <v>207.53</v>
+        <v>0</v>
       </c>
       <c r="P346" t="n">
         <v>0</v>
@@ -26045,18 +26045,18 @@
         <v>0</v>
       </c>
       <c r="T346" t="n">
-        <v>13.32</v>
+        <v>252.65</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>ICPI3</t>
+          <t>ALBA3</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Empresa ICPI</t>
+          <t>Empresa ALBA</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
@@ -26070,7 +26070,7 @@
         </is>
       </c>
       <c r="E347" t="n">
-        <v>0</v>
+        <v>2.15</v>
       </c>
       <c r="F347" t="inlineStr">
         <is>
@@ -26101,36 +26101,36 @@
         <v>0</v>
       </c>
       <c r="N347" t="n">
-        <v>0</v>
+        <v>354860000</v>
       </c>
       <c r="O347" t="n">
         <v>0</v>
       </c>
       <c r="P347" t="n">
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="Q347" t="n">
-        <v>0</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="R347" t="n">
-        <v>0</v>
+        <v>20.4</v>
       </c>
       <c r="S347" t="n">
-        <v>0</v>
+        <v>19.77</v>
       </c>
       <c r="T347" t="n">
-        <v>0</v>
+        <v>14.69</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>ILLS4</t>
+          <t>ARPS4</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Empresa ILLS</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
@@ -26144,7 +26144,7 @@
         </is>
       </c>
       <c r="E348" t="n">
-        <v>100.01</v>
+        <v>0</v>
       </c>
       <c r="F348" t="inlineStr">
         <is>
@@ -26175,36 +26175,36 @@
         <v>0</v>
       </c>
       <c r="N348" t="n">
-        <v>-18567000</v>
+        <v>-12690000</v>
       </c>
       <c r="O348" t="n">
         <v>0</v>
       </c>
       <c r="P348" t="n">
-        <v>8.43</v>
+        <v>-4.92</v>
       </c>
       <c r="Q348" t="n">
-        <v>-10.22</v>
+        <v>-11.59</v>
       </c>
       <c r="R348" t="n">
-        <v>8.140000000000001</v>
+        <v>-6.64</v>
       </c>
       <c r="S348" t="n">
-        <v>36.09</v>
+        <v>20.34</v>
       </c>
       <c r="T348" t="n">
-        <v>9.33</v>
+        <v>-17.53</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>PTIP3</t>
+          <t>SALM3</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
@@ -26218,7 +26218,7 @@
         </is>
       </c>
       <c r="E349" t="n">
-        <v>22</v>
+        <v>5.7</v>
       </c>
       <c r="F349" t="inlineStr">
         <is>
@@ -26249,36 +26249,36 @@
         <v>0</v>
       </c>
       <c r="N349" t="n">
-        <v>-155957000</v>
+        <v>475600000</v>
       </c>
       <c r="O349" t="n">
         <v>0</v>
       </c>
       <c r="P349" t="n">
-        <v>13.73</v>
+        <v>10.22</v>
       </c>
       <c r="Q349" t="n">
-        <v>7.55</v>
+        <v>4.13</v>
       </c>
       <c r="R349" t="n">
-        <v>23.13</v>
+        <v>25.78</v>
       </c>
       <c r="S349" t="n">
-        <v>-121.74</v>
+        <v>19.53</v>
       </c>
       <c r="T349" t="n">
-        <v>62.11</v>
+        <v>24.53</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>REPA4</t>
+          <t>CMMA4</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa CMMA</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
@@ -26292,7 +26292,7 @@
         </is>
       </c>
       <c r="E350" t="n">
-        <v>1.08</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="F350" t="inlineStr">
         <is>
@@ -26323,41 +26323,41 @@
         <v>0</v>
       </c>
       <c r="N350" t="n">
-        <v>378378000</v>
+        <v>-79623000</v>
       </c>
       <c r="O350" t="n">
         <v>0</v>
       </c>
       <c r="P350" t="n">
-        <v>5.18</v>
+        <v>0</v>
       </c>
       <c r="Q350" t="n">
-        <v>1.22</v>
+        <v>0</v>
       </c>
       <c r="R350" t="n">
-        <v>4.05</v>
+        <v>0</v>
       </c>
       <c r="S350" t="n">
-        <v>1.91</v>
+        <v>-1.92</v>
       </c>
       <c r="T350" t="n">
-        <v>1.09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>EQMA6B</t>
+          <t>CSPC4</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D351" t="inlineStr">
@@ -26366,7 +26366,7 @@
         </is>
       </c>
       <c r="E351" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="F351" t="inlineStr">
         <is>
@@ -26397,41 +26397,41 @@
         <v>0</v>
       </c>
       <c r="N351" t="n">
-        <v>4940330000</v>
+        <v>2126670000</v>
       </c>
       <c r="O351" t="n">
         <v>0</v>
       </c>
       <c r="P351" t="n">
-        <v>0</v>
+        <v>38.62</v>
       </c>
       <c r="Q351" t="n">
-        <v>0</v>
+        <v>18.85</v>
       </c>
       <c r="R351" t="n">
-        <v>0</v>
+        <v>29.18</v>
       </c>
       <c r="S351" t="n">
-        <v>0</v>
+        <v>45.33</v>
       </c>
       <c r="T351" t="n">
-        <v>9.050000000000001</v>
+        <v>41.15</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>SEBB4</t>
+          <t>BOVH3</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa BOVH</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D352" t="inlineStr">
@@ -26440,7 +26440,7 @@
         </is>
       </c>
       <c r="E352" t="n">
-        <v>0</v>
+        <v>15.71</v>
       </c>
       <c r="F352" t="inlineStr">
         <is>
@@ -26465,42 +26465,42 @@
         <v>0</v>
       </c>
       <c r="L352" t="n">
-        <v>0</v>
+        <v>6.16</v>
       </c>
       <c r="M352" t="n">
         <v>0</v>
       </c>
       <c r="N352" t="n">
-        <v>145783000</v>
+        <v>1843320000</v>
       </c>
       <c r="O352" t="n">
         <v>0</v>
       </c>
       <c r="P352" t="n">
-        <v>9.24</v>
+        <v>0</v>
       </c>
       <c r="Q352" t="n">
-        <v>7.4</v>
+        <v>0</v>
       </c>
       <c r="R352" t="n">
-        <v>24.15</v>
+        <v>0</v>
       </c>
       <c r="S352" t="n">
-        <v>23.01</v>
+        <v>0</v>
       </c>
       <c r="T352" t="n">
-        <v>50.04</v>
+        <v>0</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>MSAN3</t>
+          <t>VNET3</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa VNET</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -26514,7 +26514,7 @@
         </is>
       </c>
       <c r="E353" t="n">
-        <v>6.44</v>
+        <v>0</v>
       </c>
       <c r="F353" t="inlineStr">
         <is>
@@ -26545,36 +26545,36 @@
         <v>0</v>
       </c>
       <c r="N353" t="n">
-        <v>2533030000</v>
+        <v>14163000000</v>
       </c>
       <c r="O353" t="n">
         <v>0</v>
       </c>
       <c r="P353" t="n">
-        <v>6.27</v>
+        <v>0</v>
       </c>
       <c r="Q353" t="n">
-        <v>2.42</v>
+        <v>0</v>
       </c>
       <c r="R353" t="n">
-        <v>11.78</v>
+        <v>0</v>
       </c>
       <c r="S353" t="n">
-        <v>11.81</v>
+        <v>0</v>
       </c>
       <c r="T353" t="n">
-        <v>101.35</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>GALO3</t>
+          <t>ARND3</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa ARND</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -26584,22 +26584,22 @@
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>Tradicional</t>
+          <t>Novo Mercado</t>
         </is>
       </c>
       <c r="E354" t="n">
-        <v>0</v>
+        <v>0.51</v>
       </c>
       <c r="F354" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Tecnologia da Informação</t>
         </is>
       </c>
       <c r="G354" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="H354" t="n">
-        <v>0</v>
+        <v>12.49</v>
       </c>
       <c r="I354" t="inlineStr">
         <is>
@@ -26613,42 +26613,42 @@
         <v>0</v>
       </c>
       <c r="L354" t="n">
-        <v>0</v>
+        <v>0.57</v>
       </c>
       <c r="M354" t="n">
         <v>0</v>
       </c>
       <c r="N354" t="n">
-        <v>-60607000</v>
+        <v>125211000</v>
       </c>
       <c r="O354" t="n">
-        <v>0</v>
+        <v>913.58</v>
       </c>
       <c r="P354" t="n">
-        <v>13.98</v>
+        <v>0</v>
       </c>
       <c r="Q354" t="n">
-        <v>-184.58</v>
+        <v>0</v>
       </c>
       <c r="R354" t="n">
-        <v>39.37</v>
+        <v>0</v>
       </c>
       <c r="S354" t="n">
-        <v>7.62</v>
+        <v>0</v>
       </c>
       <c r="T354" t="n">
-        <v>-28.97</v>
+        <v>-0.88</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>SLCP3</t>
+          <t>VVAX3</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Empresa SLCP</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -26662,7 +26662,7 @@
         </is>
       </c>
       <c r="E355" t="n">
-        <v>610.02</v>
+        <v>0</v>
       </c>
       <c r="F355" t="inlineStr">
         <is>
@@ -26693,22 +26693,22 @@
         <v>0</v>
       </c>
       <c r="N355" t="n">
-        <v>0</v>
+        <v>144676000</v>
       </c>
       <c r="O355" t="n">
         <v>0</v>
       </c>
       <c r="P355" t="n">
-        <v>0</v>
+        <v>-7.36</v>
       </c>
       <c r="Q355" t="n">
-        <v>0</v>
+        <v>-37.76</v>
       </c>
       <c r="R355" t="n">
-        <v>0</v>
+        <v>-6.52</v>
       </c>
       <c r="S355" t="n">
-        <v>0</v>
+        <v>-92.03</v>
       </c>
       <c r="T355" t="n">
         <v>0</v>
@@ -26717,17 +26717,17 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>DAYC3</t>
+          <t>MSAN4</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Empresa DAYC</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D356" t="inlineStr">
@@ -26736,7 +26736,7 @@
         </is>
       </c>
       <c r="E356" t="n">
-        <v>0</v>
+        <v>6.44</v>
       </c>
       <c r="F356" t="inlineStr">
         <is>
@@ -26767,36 +26767,36 @@
         <v>0</v>
       </c>
       <c r="N356" t="n">
-        <v>3009030000</v>
+        <v>2533030000</v>
       </c>
       <c r="O356" t="n">
         <v>0</v>
       </c>
       <c r="P356" t="n">
-        <v>0</v>
+        <v>6.27</v>
       </c>
       <c r="Q356" t="n">
-        <v>0</v>
+        <v>2.42</v>
       </c>
       <c r="R356" t="n">
-        <v>0</v>
+        <v>11.78</v>
       </c>
       <c r="S356" t="n">
-        <v>17.33</v>
+        <v>11.81</v>
       </c>
       <c r="T356" t="n">
-        <v>8.15</v>
+        <v>101.35</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>TNEP4</t>
+          <t>GALO4</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -26810,7 +26810,7 @@
         </is>
       </c>
       <c r="E357" t="n">
-        <v>3.95</v>
+        <v>0.25</v>
       </c>
       <c r="F357" t="inlineStr">
         <is>
@@ -26841,36 +26841,36 @@
         <v>0</v>
       </c>
       <c r="N357" t="n">
-        <v>955105000</v>
+        <v>-60607000</v>
       </c>
       <c r="O357" t="n">
         <v>0</v>
       </c>
       <c r="P357" t="n">
-        <v>20.92</v>
+        <v>13.98</v>
       </c>
       <c r="Q357" t="n">
-        <v>25.42</v>
+        <v>-184.58</v>
       </c>
       <c r="R357" t="n">
-        <v>20.53</v>
+        <v>39.37</v>
       </c>
       <c r="S357" t="n">
-        <v>22.8</v>
+        <v>7.62</v>
       </c>
       <c r="T357" t="n">
-        <v>8.15</v>
+        <v>-28.97</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>MLPA3</t>
+          <t>BBTG13</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Empresa MLPA</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -26915,46 +26915,46 @@
         <v>0</v>
       </c>
       <c r="N358" t="n">
-        <v>44578000</v>
+        <v>7000</v>
       </c>
       <c r="O358" t="n">
         <v>0</v>
       </c>
       <c r="P358" t="n">
-        <v>6.66</v>
+        <v>0</v>
       </c>
       <c r="Q358" t="n">
-        <v>8.92</v>
+        <v>0</v>
       </c>
       <c r="R358" t="n">
         <v>0</v>
       </c>
       <c r="S358" t="n">
-        <v>45.13</v>
+        <v>-42.86</v>
       </c>
       <c r="T358" t="n">
-        <v>-7.51</v>
+        <v>0</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>CLSC6</t>
+          <t>INHA3</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Empresa CLSC</t>
+          <t>Empresa INHA</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>Nível 2</t>
+          <t>Tradicional</t>
         </is>
       </c>
       <c r="E359" t="n">
@@ -26962,22 +26962,22 @@
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t>Energia Elétrica</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G359" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="H359" t="n">
-        <v>75.73</v>
+        <v>0</v>
       </c>
       <c r="I359" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="J359" t="n">
-        <v>2.73</v>
+        <v>0</v>
       </c>
       <c r="K359" t="n">
         <v>0</v>
@@ -26989,41 +26989,41 @@
         <v>0</v>
       </c>
       <c r="N359" t="n">
-        <v>4228180000</v>
+        <v>1533210000</v>
       </c>
       <c r="O359" t="n">
         <v>0</v>
       </c>
       <c r="P359" t="n">
-        <v>0</v>
+        <v>-56.05</v>
       </c>
       <c r="Q359" t="n">
-        <v>0</v>
+        <v>-124.06</v>
       </c>
       <c r="R359" t="n">
-        <v>0</v>
+        <v>-6.27</v>
       </c>
       <c r="S359" t="n">
-        <v>0</v>
+        <v>-39.87</v>
       </c>
       <c r="T359" t="n">
-        <v>2.82</v>
+        <v>-12.18</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>SGEN3</t>
+          <t>PTIP4</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D360" t="inlineStr">
@@ -27032,7 +27032,7 @@
         </is>
       </c>
       <c r="E360" t="n">
-        <v>5</v>
+        <v>25.15</v>
       </c>
       <c r="F360" t="inlineStr">
         <is>
@@ -27057,47 +27057,47 @@
         <v>0</v>
       </c>
       <c r="L360" t="n">
-        <v>0.77</v>
+        <v>0</v>
       </c>
       <c r="M360" t="n">
         <v>0</v>
       </c>
       <c r="N360" t="n">
-        <v>156981000</v>
+        <v>-155957000</v>
       </c>
       <c r="O360" t="n">
         <v>0</v>
       </c>
       <c r="P360" t="n">
-        <v>-1871.17</v>
+        <v>13.73</v>
       </c>
       <c r="Q360" t="n">
-        <v>0</v>
+        <v>7.55</v>
       </c>
       <c r="R360" t="n">
-        <v>-1.59</v>
+        <v>23.13</v>
       </c>
       <c r="S360" t="n">
-        <v>0</v>
+        <v>-121.74</v>
       </c>
       <c r="T360" t="n">
-        <v>-59.85</v>
+        <v>62.11</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>DUFB11</t>
+          <t>LATS3</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Empresa DUFB</t>
+          <t>Empresa LATS</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>UNT</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D361" t="inlineStr">
@@ -27106,7 +27106,7 @@
         </is>
       </c>
       <c r="E361" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F361" t="inlineStr">
         <is>
@@ -27137,41 +27137,41 @@
         <v>0</v>
       </c>
       <c r="N361" t="n">
-        <v>0</v>
+        <v>680646000</v>
       </c>
       <c r="O361" t="n">
         <v>0</v>
       </c>
       <c r="P361" t="n">
-        <v>0</v>
+        <v>11.74</v>
       </c>
       <c r="Q361" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="R361" t="n">
-        <v>0</v>
+        <v>11.63</v>
       </c>
       <c r="S361" t="n">
-        <v>0</v>
+        <v>1.84</v>
       </c>
       <c r="T361" t="n">
-        <v>0</v>
+        <v>15.37</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>CCHI3</t>
+          <t>SGEN4</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D362" t="inlineStr">
@@ -27180,7 +27180,7 @@
         </is>
       </c>
       <c r="E362" t="n">
-        <v>0.02</v>
+        <v>0.6</v>
       </c>
       <c r="F362" t="inlineStr">
         <is>
@@ -27205,42 +27205,42 @@
         <v>0</v>
       </c>
       <c r="L362" t="n">
-        <v>-0.01</v>
+        <v>0.09</v>
       </c>
       <c r="M362" t="n">
         <v>0</v>
       </c>
       <c r="N362" t="n">
-        <v>-160477000</v>
+        <v>156981000</v>
       </c>
       <c r="O362" t="n">
         <v>0</v>
       </c>
       <c r="P362" t="n">
-        <v>0</v>
+        <v>-1871.17</v>
       </c>
       <c r="Q362" t="n">
         <v>0</v>
       </c>
       <c r="R362" t="n">
-        <v>0</v>
+        <v>-1.59</v>
       </c>
       <c r="S362" t="n">
         <v>0</v>
       </c>
       <c r="T362" t="n">
-        <v>20.36</v>
+        <v>-59.85</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>SFSA3</t>
+          <t>VSPT3</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Empresa SFSA</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -27258,7 +27258,7 @@
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bens Industriais</t>
         </is>
       </c>
       <c r="G363" t="n">
@@ -27273,7 +27273,7 @@
         </is>
       </c>
       <c r="J363" t="n">
-        <v>0</v>
+        <v>-0.43</v>
       </c>
       <c r="K363" t="n">
         <v>0</v>
@@ -27285,7 +27285,7 @@
         <v>0</v>
       </c>
       <c r="N363" t="n">
-        <v>739524000</v>
+        <v>5031600000</v>
       </c>
       <c r="O363" t="n">
         <v>0</v>
@@ -27300,21 +27300,21 @@
         <v>0</v>
       </c>
       <c r="S363" t="n">
-        <v>6.25</v>
+        <v>0</v>
       </c>
       <c r="T363" t="n">
-        <v>0.15</v>
+        <v>4.92</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>PRBC3</t>
+          <t>SEBB3</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Empresa PRBC</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -27359,41 +27359,41 @@
         <v>0</v>
       </c>
       <c r="N364" t="n">
-        <v>1319270000</v>
+        <v>145783000</v>
       </c>
       <c r="O364" t="n">
         <v>0</v>
       </c>
       <c r="P364" t="n">
-        <v>0</v>
+        <v>9.24</v>
       </c>
       <c r="Q364" t="n">
-        <v>0</v>
+        <v>7.4</v>
       </c>
       <c r="R364" t="n">
-        <v>0</v>
+        <v>24.15</v>
       </c>
       <c r="S364" t="n">
-        <v>8.27</v>
+        <v>23.01</v>
       </c>
       <c r="T364" t="n">
-        <v>-1.98</v>
+        <v>50.04</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>ECIS3</t>
+          <t>BBTG11</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
@@ -27402,7 +27402,7 @@
         </is>
       </c>
       <c r="E365" t="n">
-        <v>211.65</v>
+        <v>15.01</v>
       </c>
       <c r="F365" t="inlineStr">
         <is>
@@ -27433,41 +27433,41 @@
         <v>0</v>
       </c>
       <c r="N365" t="n">
-        <v>129346000</v>
+        <v>0</v>
       </c>
       <c r="O365" t="n">
         <v>0</v>
       </c>
       <c r="P365" t="n">
-        <v>34.9</v>
+        <v>0</v>
       </c>
       <c r="Q365" t="n">
-        <v>14.18</v>
+        <v>0</v>
       </c>
       <c r="R365" t="n">
-        <v>12.48</v>
+        <v>0</v>
       </c>
       <c r="S365" t="n">
-        <v>7.33</v>
+        <v>0</v>
       </c>
       <c r="T365" t="n">
-        <v>4.66</v>
+        <v>0</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>BSGR3</t>
+          <t>JFAB4</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Empresa BSGR</t>
+          <t>Empresa JFAB</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D366" t="inlineStr">
@@ -27476,7 +27476,7 @@
         </is>
       </c>
       <c r="E366" t="n">
-        <v>1091.28</v>
+        <v>0.06</v>
       </c>
       <c r="F366" t="inlineStr">
         <is>
@@ -27507,7 +27507,7 @@
         <v>0</v>
       </c>
       <c r="N366" t="n">
-        <v>0</v>
+        <v>-10183000</v>
       </c>
       <c r="O366" t="n">
         <v>0</v>
@@ -27522,7 +27522,7 @@
         <v>0</v>
       </c>
       <c r="S366" t="n">
-        <v>0</v>
+        <v>2.34</v>
       </c>
       <c r="T366" t="n">
         <v>0</v>
@@ -27531,17 +27531,17 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>CBMA3</t>
+          <t>CCHI4</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D367" t="inlineStr">
@@ -27550,7 +27550,7 @@
         </is>
       </c>
       <c r="E367" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="F367" t="inlineStr">
         <is>
@@ -27575,13 +27575,13 @@
         <v>0</v>
       </c>
       <c r="L367" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="M367" t="n">
         <v>0</v>
       </c>
       <c r="N367" t="n">
-        <v>-34022300000</v>
+        <v>-160477000</v>
       </c>
       <c r="O367" t="n">
         <v>0</v>
@@ -27599,18 +27599,18 @@
         <v>0</v>
       </c>
       <c r="T367" t="n">
-        <v>252.65</v>
+        <v>20.36</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>ALBA3</t>
+          <t>REPA3</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Empresa ALBA</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -27624,7 +27624,7 @@
         </is>
       </c>
       <c r="E368" t="n">
-        <v>2.15</v>
+        <v>1</v>
       </c>
       <c r="F368" t="inlineStr">
         <is>
@@ -27655,41 +27655,41 @@
         <v>0</v>
       </c>
       <c r="N368" t="n">
-        <v>354860000</v>
+        <v>378378000</v>
       </c>
       <c r="O368" t="n">
         <v>0</v>
       </c>
       <c r="P368" t="n">
-        <v>9.5</v>
+        <v>5.18</v>
       </c>
       <c r="Q368" t="n">
-        <v>9.619999999999999</v>
+        <v>1.22</v>
       </c>
       <c r="R368" t="n">
-        <v>20.4</v>
+        <v>4.05</v>
       </c>
       <c r="S368" t="n">
-        <v>19.77</v>
+        <v>1.91</v>
       </c>
       <c r="T368" t="n">
-        <v>14.69</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>ARPS4</t>
+          <t>EQMA5B</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D369" t="inlineStr">
@@ -27729,41 +27729,41 @@
         <v>0</v>
       </c>
       <c r="N369" t="n">
-        <v>-12690000</v>
+        <v>4940330000</v>
       </c>
       <c r="O369" t="n">
         <v>0</v>
       </c>
       <c r="P369" t="n">
-        <v>-4.92</v>
+        <v>0</v>
       </c>
       <c r="Q369" t="n">
-        <v>-11.59</v>
+        <v>0</v>
       </c>
       <c r="R369" t="n">
-        <v>-6.64</v>
+        <v>0</v>
       </c>
       <c r="S369" t="n">
-        <v>20.34</v>
+        <v>0</v>
       </c>
       <c r="T369" t="n">
-        <v>-17.53</v>
+        <v>9.050000000000001</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>SALM3</t>
+          <t>ECIS4</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D370" t="inlineStr">
@@ -27772,7 +27772,7 @@
         </is>
       </c>
       <c r="E370" t="n">
-        <v>5.7</v>
+        <v>145</v>
       </c>
       <c r="F370" t="inlineStr">
         <is>
@@ -27803,41 +27803,41 @@
         <v>0</v>
       </c>
       <c r="N370" t="n">
-        <v>475600000</v>
+        <v>129346000</v>
       </c>
       <c r="O370" t="n">
         <v>0</v>
       </c>
       <c r="P370" t="n">
-        <v>10.22</v>
+        <v>34.9</v>
       </c>
       <c r="Q370" t="n">
-        <v>4.13</v>
+        <v>14.18</v>
       </c>
       <c r="R370" t="n">
-        <v>25.78</v>
+        <v>12.48</v>
       </c>
       <c r="S370" t="n">
-        <v>19.53</v>
+        <v>7.33</v>
       </c>
       <c r="T370" t="n">
-        <v>24.53</v>
+        <v>4.66</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>CMMA4</t>
+          <t>TNEP3</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Empresa CMMA</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D371" t="inlineStr">
@@ -27846,7 +27846,7 @@
         </is>
       </c>
       <c r="E371" t="n">
-        <v>0.8100000000000001</v>
+        <v>3.01</v>
       </c>
       <c r="F371" t="inlineStr">
         <is>
@@ -27877,36 +27877,36 @@
         <v>0</v>
       </c>
       <c r="N371" t="n">
-        <v>-79623000</v>
+        <v>955105000</v>
       </c>
       <c r="O371" t="n">
         <v>0</v>
       </c>
       <c r="P371" t="n">
-        <v>0</v>
+        <v>20.92</v>
       </c>
       <c r="Q371" t="n">
-        <v>0</v>
+        <v>25.42</v>
       </c>
       <c r="R371" t="n">
-        <v>0</v>
+        <v>20.53</v>
       </c>
       <c r="S371" t="n">
-        <v>-1.92</v>
+        <v>22.8</v>
       </c>
       <c r="T371" t="n">
-        <v>0</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>CZRS3</t>
+          <t>LECO3</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Empresa CZRS</t>
+          <t>Empresa LECO</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
@@ -27951,36 +27951,36 @@
         <v>0</v>
       </c>
       <c r="N372" t="n">
-        <v>1145670000</v>
+        <v>105928000</v>
       </c>
       <c r="O372" t="n">
         <v>0</v>
       </c>
       <c r="P372" t="n">
-        <v>0</v>
+        <v>-2.14</v>
       </c>
       <c r="Q372" t="n">
-        <v>0</v>
+        <v>-4.72</v>
       </c>
       <c r="R372" t="n">
-        <v>0</v>
+        <v>-3.48</v>
       </c>
       <c r="S372" t="n">
-        <v>3.34</v>
+        <v>-14.82</v>
       </c>
       <c r="T372" t="n">
-        <v>14.44</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>BPNM3</t>
+          <t>VGOR3</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Empresa BPNM</t>
+          <t>Empresa VGOR</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
@@ -28025,25 +28025,25 @@
         <v>0</v>
       </c>
       <c r="N373" t="n">
-        <v>7792670000</v>
+        <v>135178000</v>
       </c>
       <c r="O373" t="n">
         <v>0</v>
       </c>
       <c r="P373" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="Q373" t="n">
-        <v>0</v>
+        <v>-4.59</v>
       </c>
       <c r="R373" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S373" t="n">
-        <v>9.67</v>
+        <v>-24.29</v>
       </c>
       <c r="T373" t="n">
-        <v>-1.53</v>
+        <v>4.77</v>
       </c>
     </row>
     <row r="374">
@@ -32637,7 +32637,7 @@
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>MMAQ4</t>
+          <t>MMAQ3</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
@@ -32647,7 +32647,7 @@
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D436" t="inlineStr">
@@ -32684,7 +32684,7 @@
         <v>0.36</v>
       </c>
       <c r="M436" t="n">
-        <v>41.68</v>
+        <v>0</v>
       </c>
       <c r="N436" t="n">
         <v>259016000</v>
@@ -32711,7 +32711,7 @@
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>MMAQ3</t>
+          <t>MMAQ4</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
@@ -32721,7 +32721,7 @@
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D437" t="inlineStr">
@@ -32758,7 +32758,7 @@
         <v>0.36</v>
       </c>
       <c r="M437" t="n">
-        <v>0</v>
+        <v>41.68</v>
       </c>
       <c r="N437" t="n">
         <v>259016000</v>
@@ -41591,7 +41591,7 @@
     <row r="557">
       <c r="A557" t="inlineStr">
         <is>
-          <t>CIQU3</t>
+          <t>CIQU4</t>
         </is>
       </c>
       <c r="B557" t="inlineStr">
@@ -41601,7 +41601,7 @@
       </c>
       <c r="C557" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D557" t="inlineStr">
@@ -41665,7 +41665,7 @@
     <row r="558">
       <c r="A558" t="inlineStr">
         <is>
-          <t>CIQU4</t>
+          <t>CIQU3</t>
         </is>
       </c>
       <c r="B558" t="inlineStr">
@@ -41675,7 +41675,7 @@
       </c>
       <c r="C558" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D558" t="inlineStr">
@@ -43737,7 +43737,7 @@
     <row r="586">
       <c r="A586" t="inlineStr">
         <is>
-          <t>GETT4</t>
+          <t>GETT3</t>
         </is>
       </c>
       <c r="B586" t="inlineStr">
@@ -43747,7 +43747,7 @@
       </c>
       <c r="C586" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D586" t="inlineStr">
@@ -43811,7 +43811,7 @@
     <row r="587">
       <c r="A587" t="inlineStr">
         <is>
-          <t>GETT3</t>
+          <t>GETT4</t>
         </is>
       </c>
       <c r="B587" t="inlineStr">
@@ -43821,7 +43821,7 @@
       </c>
       <c r="C587" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D587" t="inlineStr">
@@ -45661,7 +45661,7 @@
     <row r="612">
       <c r="A612" t="inlineStr">
         <is>
-          <t>AESL3</t>
+          <t>AESL4</t>
         </is>
       </c>
       <c r="B612" t="inlineStr">
@@ -45671,7 +45671,7 @@
       </c>
       <c r="C612" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D612" t="inlineStr">
@@ -45735,7 +45735,7 @@
     <row r="613">
       <c r="A613" t="inlineStr">
         <is>
-          <t>AESL4</t>
+          <t>AESL3</t>
         </is>
       </c>
       <c r="B613" t="inlineStr">
@@ -45745,7 +45745,7 @@
       </c>
       <c r="C613" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D613" t="inlineStr">
@@ -63643,7 +63643,7 @@
     <row r="855">
       <c r="A855" t="inlineStr">
         <is>
-          <t>RSIP3</t>
+          <t>RSIP4</t>
         </is>
       </c>
       <c r="B855" t="inlineStr">
@@ -63653,7 +63653,7 @@
       </c>
       <c r="C855" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D855" t="inlineStr">
@@ -63717,7 +63717,7 @@
     <row r="856">
       <c r="A856" t="inlineStr">
         <is>
-          <t>RSIP4</t>
+          <t>RSIP3</t>
         </is>
       </c>
       <c r="B856" t="inlineStr">
@@ -63727,7 +63727,7 @@
       </c>
       <c r="C856" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D856" t="inlineStr">
@@ -71635,7 +71635,7 @@
     <row r="963">
       <c r="A963" t="inlineStr">
         <is>
-          <t>PQUN3</t>
+          <t>PQUN4</t>
         </is>
       </c>
       <c r="B963" t="inlineStr">
@@ -71645,7 +71645,7 @@
       </c>
       <c r="C963" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D963" t="inlineStr">
@@ -71709,7 +71709,7 @@
     <row r="964">
       <c r="A964" t="inlineStr">
         <is>
-          <t>PQUN4</t>
+          <t>PQUN3</t>
         </is>
       </c>
       <c r="B964" t="inlineStr">
@@ -71719,7 +71719,7 @@
       </c>
       <c r="C964" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D964" t="inlineStr">

</xml_diff>

<commit_message>
Corrige setor da EQPA e adiciona novas de energia
</commit_message>
<xml_diff>
--- a/acoes_b3.xlsx
+++ b/acoes_b3.xlsx
@@ -521,17 +521,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>IVTT3</t>
+          <t>PORP4</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Empresa IVTT</t>
+          <t>Empresa PORP</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -540,11 +540,11 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Seguradoras</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -571,7 +571,7 @@
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>1083050000</v>
+        <v>22399000</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
@@ -586,21 +586,21 @@
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>-0.4</v>
+        <v>-2.08</v>
       </c>
       <c r="T2" t="n">
-        <v>20.67</v>
+        <v>13.66</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MNSA3</t>
+          <t>IVTT3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Empresa MNSA</t>
+          <t>Empresa IVTT</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.42</v>
+        <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -645,36 +645,36 @@
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>-9105000</v>
+        <v>1083050000</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>-208.15</v>
+        <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>-362.66</v>
+        <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>-13.5</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>145.7</v>
+        <v>-0.4</v>
       </c>
       <c r="T3" t="n">
-        <v>-41.11</v>
+        <v>20.67</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CSTB3</t>
+          <t>MNSA3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa MNSA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>150</v>
+        <v>0.42</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -719,25 +719,25 @@
         <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>8420670000</v>
+        <v>-9105000</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>40.85</v>
+        <v>-208.15</v>
       </c>
       <c r="Q4" t="n">
-        <v>28.98</v>
+        <v>-362.66</v>
       </c>
       <c r="R4" t="n">
-        <v>22.4</v>
+        <v>-13.5</v>
       </c>
       <c r="S4" t="n">
-        <v>20.11</v>
+        <v>145.7</v>
       </c>
       <c r="T4" t="n">
-        <v>31.91</v>
+        <v>-41.11</v>
       </c>
     </row>
     <row r="5">
@@ -817,17 +817,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>POPR4</t>
+          <t>CSTB3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Empresa POPR</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -836,7 +836,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>10.17</v>
+        <v>150</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -867,41 +867,41 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>545803000</v>
+        <v>8420670000</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>8.66</v>
+        <v>40.85</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.65</v>
+        <v>28.98</v>
       </c>
       <c r="R6" t="n">
-        <v>15.25</v>
+        <v>22.4</v>
       </c>
       <c r="S6" t="n">
-        <v>19.93</v>
+        <v>20.11</v>
       </c>
       <c r="T6" t="n">
-        <v>30.93</v>
+        <v>31.91</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PMET3</t>
+          <t>POPR4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Empresa PMET</t>
+          <t>Empresa POPR</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>10.17</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -941,36 +941,36 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>-290863000</v>
+        <v>545803000</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>8.66</v>
       </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>5.65</v>
       </c>
       <c r="R7" t="n">
-        <v>0</v>
+        <v>15.25</v>
       </c>
       <c r="S7" t="n">
-        <v>4.1</v>
+        <v>19.93</v>
       </c>
       <c r="T7" t="n">
-        <v>37.74</v>
+        <v>30.93</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CLAN3</t>
+          <t>PMET3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Empresa CLAN</t>
+          <t>Empresa PMET</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1015,7 +1015,7 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>1012240000</v>
+        <v>-290863000</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
@@ -1030,26 +1030,26 @@
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>-1.05</v>
+        <v>4.1</v>
       </c>
       <c r="T8" t="n">
-        <v>-63.96</v>
+        <v>37.74</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MNSA4</t>
+          <t>CLAN3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Empresa MNSA</t>
+          <t>Empresa CLAN</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1058,7 +1058,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.47</v>
+        <v>0</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1089,36 +1089,36 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>-9105000</v>
+        <v>1012240000</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>-208.15</v>
+        <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>-362.66</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>-13.5</v>
+        <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>145.7</v>
+        <v>-1.05</v>
       </c>
       <c r="T9" t="n">
-        <v>-41.11</v>
+        <v>-63.96</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CSTB4</t>
+          <t>MNSA4</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Empresa CSTB</t>
+          <t>Empresa MNSA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1132,7 +1132,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>147.69</v>
+        <v>0.47</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1163,36 +1163,36 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>8420670000</v>
+        <v>-9105000</v>
       </c>
       <c r="O10" t="n">
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>40.85</v>
+        <v>-208.15</v>
       </c>
       <c r="Q10" t="n">
-        <v>28.98</v>
+        <v>-362.66</v>
       </c>
       <c r="R10" t="n">
-        <v>22.4</v>
+        <v>-13.5</v>
       </c>
       <c r="S10" t="n">
-        <v>20.11</v>
+        <v>145.7</v>
       </c>
       <c r="T10" t="n">
-        <v>31.91</v>
+        <v>-41.11</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PORP4</t>
+          <t>CSTB4</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Empresa PORP</t>
+          <t>Empresa CSTB</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1206,11 +1206,11 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>2.4</v>
+        <v>147.69</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Seguradoras</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -1237,25 +1237,25 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>22399000</v>
+        <v>8420670000</v>
       </c>
       <c r="O11" t="n">
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>0</v>
+        <v>40.85</v>
       </c>
       <c r="Q11" t="n">
-        <v>0</v>
+        <v>28.98</v>
       </c>
       <c r="R11" t="n">
-        <v>0</v>
+        <v>22.4</v>
       </c>
       <c r="S11" t="n">
-        <v>-2.08</v>
+        <v>20.11</v>
       </c>
       <c r="T11" t="n">
-        <v>13.66</v>
+        <v>31.91</v>
       </c>
     </row>
     <row r="12">
@@ -11274,7 +11274,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G147" t="n">
@@ -14382,7 +14382,7 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G189" t="n">
@@ -23091,17 +23091,17 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>BERG3</t>
+          <t>CCHI4</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Empresa BERG</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D307" t="inlineStr">
@@ -23110,7 +23110,7 @@
         </is>
       </c>
       <c r="E307" t="n">
-        <v>33</v>
+        <v>0.02</v>
       </c>
       <c r="F307" t="inlineStr">
         <is>
@@ -23135,42 +23135,42 @@
         <v>0</v>
       </c>
       <c r="L307" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="M307" t="n">
         <v>0</v>
       </c>
       <c r="N307" t="n">
-        <v>9538000</v>
+        <v>-160477000</v>
       </c>
       <c r="O307" t="n">
         <v>0</v>
       </c>
       <c r="P307" t="n">
-        <v>-8.6</v>
+        <v>0</v>
       </c>
       <c r="Q307" t="n">
-        <v>-32.6</v>
+        <v>0</v>
       </c>
       <c r="R307" t="n">
-        <v>-5.58</v>
+        <v>0</v>
       </c>
       <c r="S307" t="n">
-        <v>-102.71</v>
+        <v>0</v>
       </c>
       <c r="T307" t="n">
-        <v>-8</v>
+        <v>20.36</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>JBDU3</t>
+          <t>REPA3</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Empresa JBDU</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -23184,7 +23184,7 @@
         </is>
       </c>
       <c r="E308" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F308" t="inlineStr">
         <is>
@@ -23215,41 +23215,41 @@
         <v>0</v>
       </c>
       <c r="N308" t="n">
-        <v>56569000</v>
+        <v>378378000</v>
       </c>
       <c r="O308" t="n">
         <v>0</v>
       </c>
       <c r="P308" t="n">
-        <v>0</v>
+        <v>5.18</v>
       </c>
       <c r="Q308" t="n">
-        <v>0</v>
+        <v>1.22</v>
       </c>
       <c r="R308" t="n">
-        <v>0</v>
+        <v>4.05</v>
       </c>
       <c r="S308" t="n">
-        <v>0</v>
+        <v>1.91</v>
       </c>
       <c r="T308" t="n">
-        <v>0</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>EGGY3</t>
+          <t>EQMA5B</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Empresa EGGY</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
@@ -23289,7 +23289,7 @@
         <v>0</v>
       </c>
       <c r="N309" t="n">
-        <v>954480000</v>
+        <v>4940330000</v>
       </c>
       <c r="O309" t="n">
         <v>0</v>
@@ -23307,23 +23307,23 @@
         <v>0</v>
       </c>
       <c r="T309" t="n">
-        <v>-0.82</v>
+        <v>9.050000000000001</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>CBMA4</t>
+          <t>SEBB3</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D310" t="inlineStr">
@@ -23332,7 +23332,7 @@
         </is>
       </c>
       <c r="E310" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="F310" t="inlineStr">
         <is>
@@ -23363,41 +23363,41 @@
         <v>0</v>
       </c>
       <c r="N310" t="n">
-        <v>-34022300000</v>
+        <v>145783000</v>
       </c>
       <c r="O310" t="n">
         <v>0</v>
       </c>
       <c r="P310" t="n">
-        <v>0</v>
+        <v>9.24</v>
       </c>
       <c r="Q310" t="n">
-        <v>0</v>
+        <v>7.4</v>
       </c>
       <c r="R310" t="n">
-        <v>0</v>
+        <v>24.15</v>
       </c>
       <c r="S310" t="n">
-        <v>0</v>
+        <v>23.01</v>
       </c>
       <c r="T310" t="n">
-        <v>252.65</v>
+        <v>50.04</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>SALM4</t>
+          <t>BBTG11</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D311" t="inlineStr">
@@ -23406,7 +23406,7 @@
         </is>
       </c>
       <c r="E311" t="n">
-        <v>5.9</v>
+        <v>15.01</v>
       </c>
       <c r="F311" t="inlineStr">
         <is>
@@ -23437,41 +23437,41 @@
         <v>0</v>
       </c>
       <c r="N311" t="n">
-        <v>475600000</v>
+        <v>0</v>
       </c>
       <c r="O311" t="n">
         <v>0</v>
       </c>
       <c r="P311" t="n">
-        <v>10.22</v>
+        <v>0</v>
       </c>
       <c r="Q311" t="n">
-        <v>4.13</v>
+        <v>0</v>
       </c>
       <c r="R311" t="n">
-        <v>25.78</v>
+        <v>0</v>
       </c>
       <c r="S311" t="n">
-        <v>19.53</v>
+        <v>0</v>
       </c>
       <c r="T311" t="n">
-        <v>24.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>BMEF3</t>
+          <t>JFAB4</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Empresa BMEF</t>
+          <t>Empresa JFAB</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
@@ -23480,7 +23480,7 @@
         </is>
       </c>
       <c r="E312" t="n">
-        <v>11</v>
+        <v>0.06</v>
       </c>
       <c r="F312" t="inlineStr">
         <is>
@@ -23505,13 +23505,13 @@
         <v>0</v>
       </c>
       <c r="L312" t="n">
-        <v>4.16</v>
+        <v>0</v>
       </c>
       <c r="M312" t="n">
         <v>0</v>
       </c>
       <c r="N312" t="n">
-        <v>2674780000</v>
+        <v>-10183000</v>
       </c>
       <c r="O312" t="n">
         <v>0</v>
@@ -23526,7 +23526,7 @@
         <v>0</v>
       </c>
       <c r="S312" t="n">
-        <v>0</v>
+        <v>2.34</v>
       </c>
       <c r="T312" t="n">
         <v>0</v>
@@ -23535,12 +23535,12 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>AGEI3</t>
+          <t>LECO3</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Empresa AGEI</t>
+          <t>Empresa LECO</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -23554,7 +23554,7 @@
         </is>
       </c>
       <c r="E313" t="n">
-        <v>7.8</v>
+        <v>0</v>
       </c>
       <c r="F313" t="inlineStr">
         <is>
@@ -23579,42 +23579,42 @@
         <v>0</v>
       </c>
       <c r="L313" t="n">
-        <v>1.25</v>
+        <v>0</v>
       </c>
       <c r="M313" t="n">
         <v>0</v>
       </c>
       <c r="N313" t="n">
-        <v>1878210000</v>
+        <v>105928000</v>
       </c>
       <c r="O313" t="n">
         <v>0</v>
       </c>
       <c r="P313" t="n">
-        <v>0</v>
+        <v>-2.14</v>
       </c>
       <c r="Q313" t="n">
-        <v>0</v>
+        <v>-4.72</v>
       </c>
       <c r="R313" t="n">
-        <v>0</v>
+        <v>-3.48</v>
       </c>
       <c r="S313" t="n">
-        <v>0</v>
+        <v>-14.82</v>
       </c>
       <c r="T313" t="n">
-        <v>0</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>SASG3</t>
+          <t>VGOR3</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Empresa SASG</t>
+          <t>Empresa VGOR</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -23628,7 +23628,7 @@
         </is>
       </c>
       <c r="E314" t="n">
-        <v>0.98</v>
+        <v>0</v>
       </c>
       <c r="F314" t="inlineStr">
         <is>
@@ -23659,41 +23659,41 @@
         <v>0</v>
       </c>
       <c r="N314" t="n">
-        <v>0</v>
+        <v>135178000</v>
       </c>
       <c r="O314" t="n">
         <v>0</v>
       </c>
       <c r="P314" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="Q314" t="n">
-        <v>0</v>
+        <v>-4.59</v>
       </c>
       <c r="R314" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S314" t="n">
-        <v>0</v>
+        <v>-24.29</v>
       </c>
       <c r="T314" t="n">
-        <v>0</v>
+        <v>4.77</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>ODER3</t>
+          <t>ECIS4</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Empresa ODER</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
@@ -23702,18 +23702,18 @@
         </is>
       </c>
       <c r="E315" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>Consumo não Cíclico</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G315" t="n">
         <v>80</v>
       </c>
       <c r="H315" t="n">
-        <v>1.75</v>
+        <v>0</v>
       </c>
       <c r="I315" t="inlineStr">
         <is>
@@ -23733,36 +23733,36 @@
         <v>0</v>
       </c>
       <c r="N315" t="n">
-        <v>609518000</v>
+        <v>129346000</v>
       </c>
       <c r="O315" t="n">
         <v>0</v>
       </c>
       <c r="P315" t="n">
-        <v>0</v>
+        <v>34.9</v>
       </c>
       <c r="Q315" t="n">
-        <v>0</v>
+        <v>14.18</v>
       </c>
       <c r="R315" t="n">
-        <v>0</v>
+        <v>12.48</v>
       </c>
       <c r="S315" t="n">
-        <v>0</v>
+        <v>7.33</v>
       </c>
       <c r="T315" t="n">
-        <v>3.17</v>
+        <v>4.66</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>ARPS3</t>
+          <t>TNEP3</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -23776,7 +23776,7 @@
         </is>
       </c>
       <c r="E316" t="n">
-        <v>0.3</v>
+        <v>3.01</v>
       </c>
       <c r="F316" t="inlineStr">
         <is>
@@ -23807,36 +23807,36 @@
         <v>0</v>
       </c>
       <c r="N316" t="n">
-        <v>-12690000</v>
+        <v>955105000</v>
       </c>
       <c r="O316" t="n">
         <v>0</v>
       </c>
       <c r="P316" t="n">
-        <v>-4.92</v>
+        <v>20.92</v>
       </c>
       <c r="Q316" t="n">
-        <v>-11.59</v>
+        <v>25.42</v>
       </c>
       <c r="R316" t="n">
-        <v>-6.64</v>
+        <v>20.53</v>
       </c>
       <c r="S316" t="n">
-        <v>20.34</v>
+        <v>22.8</v>
       </c>
       <c r="T316" t="n">
-        <v>-17.53</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>VVAX4</t>
+          <t>CBMA4</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -23850,7 +23850,7 @@
         </is>
       </c>
       <c r="E317" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="F317" t="inlineStr">
         <is>
@@ -23881,41 +23881,41 @@
         <v>0</v>
       </c>
       <c r="N317" t="n">
-        <v>144676000</v>
+        <v>-34022300000</v>
       </c>
       <c r="O317" t="n">
         <v>0</v>
       </c>
       <c r="P317" t="n">
-        <v>-7.36</v>
+        <v>0</v>
       </c>
       <c r="Q317" t="n">
-        <v>-37.76</v>
+        <v>0</v>
       </c>
       <c r="R317" t="n">
-        <v>-6.52</v>
+        <v>0</v>
       </c>
       <c r="S317" t="n">
-        <v>-92.03</v>
+        <v>0</v>
       </c>
       <c r="T317" t="n">
-        <v>0</v>
+        <v>252.65</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>CSPC3</t>
+          <t>SALM4</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
@@ -23924,7 +23924,7 @@
         </is>
       </c>
       <c r="E318" t="n">
-        <v>1.24</v>
+        <v>5.9</v>
       </c>
       <c r="F318" t="inlineStr">
         <is>
@@ -23955,36 +23955,36 @@
         <v>0</v>
       </c>
       <c r="N318" t="n">
-        <v>2126670000</v>
+        <v>475600000</v>
       </c>
       <c r="O318" t="n">
         <v>0</v>
       </c>
       <c r="P318" t="n">
-        <v>38.62</v>
+        <v>10.22</v>
       </c>
       <c r="Q318" t="n">
-        <v>18.85</v>
+        <v>4.13</v>
       </c>
       <c r="R318" t="n">
-        <v>29.18</v>
+        <v>25.78</v>
       </c>
       <c r="S318" t="n">
-        <v>45.33</v>
+        <v>19.53</v>
       </c>
       <c r="T318" t="n">
-        <v>41.15</v>
+        <v>24.53</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>ABCB3</t>
+          <t>BERG3</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Empresa ABCB</t>
+          <t>Empresa BERG</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -23998,11 +23998,11 @@
         </is>
       </c>
       <c r="E319" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>Bancos</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G319" t="n">
@@ -24029,36 +24029,36 @@
         <v>0</v>
       </c>
       <c r="N319" t="n">
-        <v>7258910000</v>
+        <v>9538000</v>
       </c>
       <c r="O319" t="n">
         <v>0</v>
       </c>
       <c r="P319" t="n">
-        <v>0</v>
+        <v>-8.6</v>
       </c>
       <c r="Q319" t="n">
-        <v>0</v>
+        <v>-32.6</v>
       </c>
       <c r="R319" t="n">
-        <v>0</v>
+        <v>-5.58</v>
       </c>
       <c r="S319" t="n">
-        <v>14.05</v>
+        <v>-102.71</v>
       </c>
       <c r="T319" t="n">
-        <v>7.57</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>CCTY3</t>
+          <t>JBDU3</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Empresa CCTY</t>
+          <t>Empresa JBDU</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -24103,7 +24103,7 @@
         <v>0</v>
       </c>
       <c r="N320" t="n">
-        <v>0</v>
+        <v>56569000</v>
       </c>
       <c r="O320" t="n">
         <v>0</v>
@@ -24127,17 +24127,17 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>BAUH4</t>
+          <t>EGGY3</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Empresa BAUH</t>
+          <t>Empresa EGGY</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D321" t="inlineStr">
@@ -24146,18 +24146,18 @@
         </is>
       </c>
       <c r="E321" t="n">
-        <v>93.39</v>
+        <v>0</v>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>Consumo não Cíclico</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G321" t="n">
         <v>80</v>
       </c>
       <c r="H321" t="n">
-        <v>28.89</v>
+        <v>0</v>
       </c>
       <c r="I321" t="inlineStr">
         <is>
@@ -24165,22 +24165,22 @@
         </is>
       </c>
       <c r="J321" t="n">
-        <v>-2.88</v>
+        <v>0</v>
       </c>
       <c r="K321" t="n">
         <v>0</v>
       </c>
       <c r="L321" t="n">
-        <v>3.18</v>
+        <v>0</v>
       </c>
       <c r="M321" t="n">
-        <v>1.16</v>
+        <v>0</v>
       </c>
       <c r="N321" t="n">
-        <v>153407000</v>
+        <v>954480000</v>
       </c>
       <c r="O321" t="n">
-        <v>207.53</v>
+        <v>0</v>
       </c>
       <c r="P321" t="n">
         <v>0</v>
@@ -24195,18 +24195,18 @@
         <v>0</v>
       </c>
       <c r="T321" t="n">
-        <v>13.32</v>
+        <v>-0.82</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>ICPI3</t>
+          <t>AGEI3</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Empresa ICPI</t>
+          <t>Empresa AGEI</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -24220,7 +24220,7 @@
         </is>
       </c>
       <c r="E322" t="n">
-        <v>0</v>
+        <v>7.8</v>
       </c>
       <c r="F322" t="inlineStr">
         <is>
@@ -24245,13 +24245,13 @@
         <v>0</v>
       </c>
       <c r="L322" t="n">
-        <v>0</v>
+        <v>1.25</v>
       </c>
       <c r="M322" t="n">
         <v>0</v>
       </c>
       <c r="N322" t="n">
-        <v>0</v>
+        <v>1878210000</v>
       </c>
       <c r="O322" t="n">
         <v>0</v>
@@ -24275,17 +24275,17 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>ILLS4</t>
+          <t>SASG3</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Empresa ILLS</t>
+          <t>Empresa SASG</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D323" t="inlineStr">
@@ -24294,7 +24294,7 @@
         </is>
       </c>
       <c r="E323" t="n">
-        <v>100.01</v>
+        <v>0.98</v>
       </c>
       <c r="F323" t="inlineStr">
         <is>
@@ -24325,41 +24325,41 @@
         <v>0</v>
       </c>
       <c r="N323" t="n">
-        <v>-18567000</v>
+        <v>0</v>
       </c>
       <c r="O323" t="n">
         <v>0</v>
       </c>
       <c r="P323" t="n">
-        <v>8.43</v>
+        <v>0</v>
       </c>
       <c r="Q323" t="n">
-        <v>-10.22</v>
+        <v>0</v>
       </c>
       <c r="R323" t="n">
-        <v>8.140000000000001</v>
+        <v>0</v>
       </c>
       <c r="S323" t="n">
-        <v>36.09</v>
+        <v>0</v>
       </c>
       <c r="T323" t="n">
-        <v>9.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>ESTC4</t>
+          <t>BMEF3</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Empresa ESTC</t>
+          <t>Empresa BMEF</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D324" t="inlineStr">
@@ -24368,7 +24368,7 @@
         </is>
       </c>
       <c r="E324" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F324" t="inlineStr">
         <is>
@@ -24393,47 +24393,47 @@
         <v>0</v>
       </c>
       <c r="L324" t="n">
-        <v>0</v>
+        <v>4.16</v>
       </c>
       <c r="M324" t="n">
         <v>0</v>
       </c>
       <c r="N324" t="n">
-        <v>2916530000</v>
+        <v>2674780000</v>
       </c>
       <c r="O324" t="n">
         <v>0</v>
       </c>
       <c r="P324" t="n">
-        <v>16.91</v>
+        <v>0</v>
       </c>
       <c r="Q324" t="n">
-        <v>2.02</v>
+        <v>0</v>
       </c>
       <c r="R324" t="n">
-        <v>11.35</v>
+        <v>0</v>
       </c>
       <c r="S324" t="n">
-        <v>3.89</v>
+        <v>0</v>
       </c>
       <c r="T324" t="n">
-        <v>5.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>VSPT4</t>
+          <t>ARPS3</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D325" t="inlineStr">
@@ -24442,11 +24442,11 @@
         </is>
       </c>
       <c r="E325" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>Bens Industriais</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G325" t="n">
@@ -24461,7 +24461,7 @@
         </is>
       </c>
       <c r="J325" t="n">
-        <v>-0.43</v>
+        <v>0</v>
       </c>
       <c r="K325" t="n">
         <v>0</v>
@@ -24473,41 +24473,41 @@
         <v>0</v>
       </c>
       <c r="N325" t="n">
-        <v>5031600000</v>
+        <v>-12690000</v>
       </c>
       <c r="O325" t="n">
         <v>0</v>
       </c>
       <c r="P325" t="n">
-        <v>0</v>
+        <v>-4.92</v>
       </c>
       <c r="Q325" t="n">
-        <v>0</v>
+        <v>-11.59</v>
       </c>
       <c r="R325" t="n">
-        <v>0</v>
+        <v>-6.64</v>
       </c>
       <c r="S325" t="n">
-        <v>0</v>
+        <v>20.34</v>
       </c>
       <c r="T325" t="n">
-        <v>4.92</v>
+        <v>-17.53</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>SEBB4</t>
+          <t>ODER3</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa ODER</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D326" t="inlineStr">
@@ -24520,14 +24520,14 @@
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Consumo não Cíclico</t>
         </is>
       </c>
       <c r="G326" t="n">
         <v>80</v>
       </c>
       <c r="H326" t="n">
-        <v>0</v>
+        <v>1.75</v>
       </c>
       <c r="I326" t="inlineStr">
         <is>
@@ -24547,36 +24547,36 @@
         <v>0</v>
       </c>
       <c r="N326" t="n">
-        <v>145783000</v>
+        <v>609518000</v>
       </c>
       <c r="O326" t="n">
         <v>0</v>
       </c>
       <c r="P326" t="n">
-        <v>9.24</v>
+        <v>0</v>
       </c>
       <c r="Q326" t="n">
-        <v>7.4</v>
+        <v>0</v>
       </c>
       <c r="R326" t="n">
-        <v>24.15</v>
+        <v>0</v>
       </c>
       <c r="S326" t="n">
-        <v>23.01</v>
+        <v>0</v>
       </c>
       <c r="T326" t="n">
-        <v>50.04</v>
+        <v>3.17</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>MSAN3</t>
+          <t>CCTY3</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa CCTY</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -24590,7 +24590,7 @@
         </is>
       </c>
       <c r="E327" t="n">
-        <v>6.44</v>
+        <v>0</v>
       </c>
       <c r="F327" t="inlineStr">
         <is>
@@ -24621,41 +24621,41 @@
         <v>0</v>
       </c>
       <c r="N327" t="n">
-        <v>2533030000</v>
+        <v>0</v>
       </c>
       <c r="O327" t="n">
         <v>0</v>
       </c>
       <c r="P327" t="n">
-        <v>6.27</v>
+        <v>0</v>
       </c>
       <c r="Q327" t="n">
-        <v>2.42</v>
+        <v>0</v>
       </c>
       <c r="R327" t="n">
-        <v>11.78</v>
+        <v>0</v>
       </c>
       <c r="S327" t="n">
-        <v>11.81</v>
+        <v>0</v>
       </c>
       <c r="T327" t="n">
-        <v>101.35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>GALO3</t>
+          <t>VVAX4</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D328" t="inlineStr">
@@ -24695,36 +24695,36 @@
         <v>0</v>
       </c>
       <c r="N328" t="n">
-        <v>-60607000</v>
+        <v>144676000</v>
       </c>
       <c r="O328" t="n">
         <v>0</v>
       </c>
       <c r="P328" t="n">
-        <v>13.98</v>
+        <v>-7.36</v>
       </c>
       <c r="Q328" t="n">
-        <v>-184.58</v>
+        <v>-37.76</v>
       </c>
       <c r="R328" t="n">
-        <v>39.37</v>
+        <v>-6.52</v>
       </c>
       <c r="S328" t="n">
-        <v>7.62</v>
+        <v>-92.03</v>
       </c>
       <c r="T328" t="n">
-        <v>-28.97</v>
+        <v>0</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>SLCP3</t>
+          <t>CSPC3</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Empresa SLCP</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -24738,7 +24738,7 @@
         </is>
       </c>
       <c r="E329" t="n">
-        <v>610.02</v>
+        <v>1.24</v>
       </c>
       <c r="F329" t="inlineStr">
         <is>
@@ -24769,36 +24769,36 @@
         <v>0</v>
       </c>
       <c r="N329" t="n">
-        <v>0</v>
+        <v>2126670000</v>
       </c>
       <c r="O329" t="n">
         <v>0</v>
       </c>
       <c r="P329" t="n">
-        <v>0</v>
+        <v>38.62</v>
       </c>
       <c r="Q329" t="n">
-        <v>0</v>
+        <v>18.85</v>
       </c>
       <c r="R329" t="n">
-        <v>0</v>
+        <v>29.18</v>
       </c>
       <c r="S329" t="n">
-        <v>0</v>
+        <v>45.33</v>
       </c>
       <c r="T329" t="n">
-        <v>0</v>
+        <v>41.15</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>DAYC3</t>
+          <t>ABCB3</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Empresa DAYC</t>
+          <t>Empresa ABCB</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -24816,7 +24816,7 @@
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bancos</t>
         </is>
       </c>
       <c r="G330" t="n">
@@ -24843,7 +24843,7 @@
         <v>0</v>
       </c>
       <c r="N330" t="n">
-        <v>3009030000</v>
+        <v>7258910000</v>
       </c>
       <c r="O330" t="n">
         <v>0</v>
@@ -24858,26 +24858,26 @@
         <v>0</v>
       </c>
       <c r="S330" t="n">
-        <v>17.33</v>
+        <v>14.05</v>
       </c>
       <c r="T330" t="n">
-        <v>8.15</v>
+        <v>7.57</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>PTIP3</t>
+          <t>ESTC4</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa ESTC</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
@@ -24886,7 +24886,7 @@
         </is>
       </c>
       <c r="E331" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="F331" t="inlineStr">
         <is>
@@ -24917,36 +24917,36 @@
         <v>0</v>
       </c>
       <c r="N331" t="n">
-        <v>-155957000</v>
+        <v>2916530000</v>
       </c>
       <c r="O331" t="n">
         <v>0</v>
       </c>
       <c r="P331" t="n">
-        <v>13.73</v>
+        <v>16.91</v>
       </c>
       <c r="Q331" t="n">
-        <v>7.55</v>
+        <v>2.02</v>
       </c>
       <c r="R331" t="n">
-        <v>23.13</v>
+        <v>11.35</v>
       </c>
       <c r="S331" t="n">
-        <v>-121.74</v>
+        <v>3.89</v>
       </c>
       <c r="T331" t="n">
-        <v>62.11</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>REPA4</t>
+          <t>VSPT4</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -24960,11 +24960,11 @@
         </is>
       </c>
       <c r="E332" t="n">
-        <v>1.08</v>
+        <v>0</v>
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bens Industriais</t>
         </is>
       </c>
       <c r="G332" t="n">
@@ -24979,7 +24979,7 @@
         </is>
       </c>
       <c r="J332" t="n">
-        <v>0</v>
+        <v>-0.43</v>
       </c>
       <c r="K332" t="n">
         <v>0</v>
@@ -24991,41 +24991,41 @@
         <v>0</v>
       </c>
       <c r="N332" t="n">
-        <v>378378000</v>
+        <v>5031600000</v>
       </c>
       <c r="O332" t="n">
         <v>0</v>
       </c>
       <c r="P332" t="n">
-        <v>5.18</v>
+        <v>0</v>
       </c>
       <c r="Q332" t="n">
-        <v>1.22</v>
+        <v>0</v>
       </c>
       <c r="R332" t="n">
-        <v>4.05</v>
+        <v>0</v>
       </c>
       <c r="S332" t="n">
-        <v>1.91</v>
+        <v>0</v>
       </c>
       <c r="T332" t="n">
-        <v>1.09</v>
+        <v>4.92</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>EQMA6B</t>
+          <t>BAUH4</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa BAUH</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">
@@ -25034,18 +25034,18 @@
         </is>
       </c>
       <c r="E333" t="n">
-        <v>0</v>
+        <v>93.39</v>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Consumo não Cíclico</t>
         </is>
       </c>
       <c r="G333" t="n">
         <v>80</v>
       </c>
       <c r="H333" t="n">
-        <v>0</v>
+        <v>28.89</v>
       </c>
       <c r="I333" t="inlineStr">
         <is>
@@ -25053,22 +25053,22 @@
         </is>
       </c>
       <c r="J333" t="n">
-        <v>0</v>
+        <v>-2.88</v>
       </c>
       <c r="K333" t="n">
         <v>0</v>
       </c>
       <c r="L333" t="n">
-        <v>0</v>
+        <v>3.18</v>
       </c>
       <c r="M333" t="n">
-        <v>0</v>
+        <v>1.16</v>
       </c>
       <c r="N333" t="n">
-        <v>4940330000</v>
+        <v>153407000</v>
       </c>
       <c r="O333" t="n">
-        <v>0</v>
+        <v>207.53</v>
       </c>
       <c r="P333" t="n">
         <v>0</v>
@@ -25083,18 +25083,18 @@
         <v>0</v>
       </c>
       <c r="T333" t="n">
-        <v>9.050000000000001</v>
+        <v>13.32</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>SGEN3</t>
+          <t>ICPI3</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa ICPI</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -25108,7 +25108,7 @@
         </is>
       </c>
       <c r="E334" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F334" t="inlineStr">
         <is>
@@ -25133,47 +25133,47 @@
         <v>0</v>
       </c>
       <c r="L334" t="n">
-        <v>0.77</v>
+        <v>0</v>
       </c>
       <c r="M334" t="n">
         <v>0</v>
       </c>
       <c r="N334" t="n">
-        <v>156981000</v>
+        <v>0</v>
       </c>
       <c r="O334" t="n">
         <v>0</v>
       </c>
       <c r="P334" t="n">
-        <v>-1871.17</v>
+        <v>0</v>
       </c>
       <c r="Q334" t="n">
         <v>0</v>
       </c>
       <c r="R334" t="n">
-        <v>-1.59</v>
+        <v>0</v>
       </c>
       <c r="S334" t="n">
         <v>0</v>
       </c>
       <c r="T334" t="n">
-        <v>-59.85</v>
+        <v>0</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>DUFB11</t>
+          <t>ILLS4</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Empresa DUFB</t>
+          <t>Empresa ILLS</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>UNT</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
@@ -25182,7 +25182,7 @@
         </is>
       </c>
       <c r="E335" t="n">
-        <v>0</v>
+        <v>100.01</v>
       </c>
       <c r="F335" t="inlineStr">
         <is>
@@ -25213,36 +25213,36 @@
         <v>0</v>
       </c>
       <c r="N335" t="n">
-        <v>0</v>
+        <v>-18567000</v>
       </c>
       <c r="O335" t="n">
         <v>0</v>
       </c>
       <c r="P335" t="n">
-        <v>0</v>
+        <v>8.43</v>
       </c>
       <c r="Q335" t="n">
-        <v>0</v>
+        <v>-10.22</v>
       </c>
       <c r="R335" t="n">
-        <v>0</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="S335" t="n">
-        <v>0</v>
+        <v>36.09</v>
       </c>
       <c r="T335" t="n">
-        <v>0</v>
+        <v>9.33</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>TNEP4</t>
+          <t>REPA4</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa REPA</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -25256,7 +25256,7 @@
         </is>
       </c>
       <c r="E336" t="n">
-        <v>3.95</v>
+        <v>1.08</v>
       </c>
       <c r="F336" t="inlineStr">
         <is>
@@ -25287,41 +25287,41 @@
         <v>0</v>
       </c>
       <c r="N336" t="n">
-        <v>955105000</v>
+        <v>378378000</v>
       </c>
       <c r="O336" t="n">
         <v>0</v>
       </c>
       <c r="P336" t="n">
-        <v>20.92</v>
+        <v>5.18</v>
       </c>
       <c r="Q336" t="n">
-        <v>25.42</v>
+        <v>1.22</v>
       </c>
       <c r="R336" t="n">
-        <v>20.53</v>
+        <v>4.05</v>
       </c>
       <c r="S336" t="n">
-        <v>22.8</v>
+        <v>1.91</v>
       </c>
       <c r="T336" t="n">
-        <v>8.15</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>MLPA3</t>
+          <t>EQMA6B</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Empresa MLPA</t>
+          <t>Empresa EQMA</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
@@ -25361,36 +25361,36 @@
         <v>0</v>
       </c>
       <c r="N337" t="n">
-        <v>44578000</v>
+        <v>4940330000</v>
       </c>
       <c r="O337" t="n">
         <v>0</v>
       </c>
       <c r="P337" t="n">
-        <v>6.66</v>
+        <v>0</v>
       </c>
       <c r="Q337" t="n">
-        <v>8.92</v>
+        <v>0</v>
       </c>
       <c r="R337" t="n">
         <v>0</v>
       </c>
       <c r="S337" t="n">
-        <v>45.13</v>
+        <v>0</v>
       </c>
       <c r="T337" t="n">
-        <v>-7.51</v>
+        <v>9.050000000000001</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>CLSC6</t>
+          <t>SEBB4</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Empresa CLSC</t>
+          <t>Empresa SEBB</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -25400,7 +25400,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Nível 2</t>
+          <t>Tradicional</t>
         </is>
       </c>
       <c r="E338" t="n">
@@ -25408,22 +25408,22 @@
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t>Energia Elétrica</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G338" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="H338" t="n">
-        <v>75.73</v>
+        <v>0</v>
       </c>
       <c r="I338" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="J338" t="n">
-        <v>2.73</v>
+        <v>0</v>
       </c>
       <c r="K338" t="n">
         <v>0</v>
@@ -25435,36 +25435,36 @@
         <v>0</v>
       </c>
       <c r="N338" t="n">
-        <v>4228180000</v>
+        <v>145783000</v>
       </c>
       <c r="O338" t="n">
         <v>0</v>
       </c>
       <c r="P338" t="n">
-        <v>0</v>
+        <v>9.24</v>
       </c>
       <c r="Q338" t="n">
-        <v>0</v>
+        <v>7.4</v>
       </c>
       <c r="R338" t="n">
-        <v>0</v>
+        <v>24.15</v>
       </c>
       <c r="S338" t="n">
-        <v>0</v>
+        <v>23.01</v>
       </c>
       <c r="T338" t="n">
-        <v>2.82</v>
+        <v>50.04</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>CCHI3</t>
+          <t>MSAN3</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -25478,7 +25478,7 @@
         </is>
       </c>
       <c r="E339" t="n">
-        <v>0.02</v>
+        <v>6.44</v>
       </c>
       <c r="F339" t="inlineStr">
         <is>
@@ -25503,42 +25503,42 @@
         <v>0</v>
       </c>
       <c r="L339" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="M339" t="n">
         <v>0</v>
       </c>
       <c r="N339" t="n">
-        <v>-160477000</v>
+        <v>2533030000</v>
       </c>
       <c r="O339" t="n">
         <v>0</v>
       </c>
       <c r="P339" t="n">
-        <v>0</v>
+        <v>6.27</v>
       </c>
       <c r="Q339" t="n">
-        <v>0</v>
+        <v>2.42</v>
       </c>
       <c r="R339" t="n">
-        <v>0</v>
+        <v>11.78</v>
       </c>
       <c r="S339" t="n">
-        <v>0</v>
+        <v>11.81</v>
       </c>
       <c r="T339" t="n">
-        <v>20.36</v>
+        <v>101.35</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>SFSA3</t>
+          <t>GALO3</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Empresa SFSA</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -25583,36 +25583,36 @@
         <v>0</v>
       </c>
       <c r="N340" t="n">
-        <v>739524000</v>
+        <v>-60607000</v>
       </c>
       <c r="O340" t="n">
         <v>0</v>
       </c>
       <c r="P340" t="n">
-        <v>0</v>
+        <v>13.98</v>
       </c>
       <c r="Q340" t="n">
-        <v>0</v>
+        <v>-184.58</v>
       </c>
       <c r="R340" t="n">
-        <v>0</v>
+        <v>39.37</v>
       </c>
       <c r="S340" t="n">
-        <v>6.25</v>
+        <v>7.62</v>
       </c>
       <c r="T340" t="n">
-        <v>0.15</v>
+        <v>-28.97</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>PRBC3</t>
+          <t>SLCP3</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Empresa PRBC</t>
+          <t>Empresa SLCP</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -25626,7 +25626,7 @@
         </is>
       </c>
       <c r="E341" t="n">
-        <v>0</v>
+        <v>610.02</v>
       </c>
       <c r="F341" t="inlineStr">
         <is>
@@ -25657,7 +25657,7 @@
         <v>0</v>
       </c>
       <c r="N341" t="n">
-        <v>1319270000</v>
+        <v>0</v>
       </c>
       <c r="O341" t="n">
         <v>0</v>
@@ -25672,21 +25672,21 @@
         <v>0</v>
       </c>
       <c r="S341" t="n">
-        <v>8.27</v>
+        <v>0</v>
       </c>
       <c r="T341" t="n">
-        <v>-1.98</v>
+        <v>0</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>ECIS3</t>
+          <t>DAYC3</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa DAYC</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -25700,7 +25700,7 @@
         </is>
       </c>
       <c r="E342" t="n">
-        <v>211.65</v>
+        <v>0</v>
       </c>
       <c r="F342" t="inlineStr">
         <is>
@@ -25731,36 +25731,36 @@
         <v>0</v>
       </c>
       <c r="N342" t="n">
-        <v>129346000</v>
+        <v>3009030000</v>
       </c>
       <c r="O342" t="n">
         <v>0</v>
       </c>
       <c r="P342" t="n">
-        <v>34.9</v>
+        <v>0</v>
       </c>
       <c r="Q342" t="n">
-        <v>14.18</v>
+        <v>0</v>
       </c>
       <c r="R342" t="n">
-        <v>12.48</v>
+        <v>0</v>
       </c>
       <c r="S342" t="n">
-        <v>7.33</v>
+        <v>17.33</v>
       </c>
       <c r="T342" t="n">
-        <v>4.66</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>CZRS3</t>
+          <t>PTIP3</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Empresa CZRS</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -25774,7 +25774,7 @@
         </is>
       </c>
       <c r="E343" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F343" t="inlineStr">
         <is>
@@ -25805,36 +25805,36 @@
         <v>0</v>
       </c>
       <c r="N343" t="n">
-        <v>1145670000</v>
+        <v>-155957000</v>
       </c>
       <c r="O343" t="n">
         <v>0</v>
       </c>
       <c r="P343" t="n">
-        <v>0</v>
+        <v>13.73</v>
       </c>
       <c r="Q343" t="n">
-        <v>0</v>
+        <v>7.55</v>
       </c>
       <c r="R343" t="n">
-        <v>0</v>
+        <v>23.13</v>
       </c>
       <c r="S343" t="n">
-        <v>3.34</v>
+        <v>-121.74</v>
       </c>
       <c r="T343" t="n">
-        <v>14.44</v>
+        <v>62.11</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>BPNM3</t>
+          <t>MLPA3</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Empresa BPNM</t>
+          <t>Empresa MLPA</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
@@ -25879,69 +25879,69 @@
         <v>0</v>
       </c>
       <c r="N344" t="n">
-        <v>7792670000</v>
+        <v>44578000</v>
       </c>
       <c r="O344" t="n">
         <v>0</v>
       </c>
       <c r="P344" t="n">
-        <v>0</v>
+        <v>6.66</v>
       </c>
       <c r="Q344" t="n">
-        <v>0</v>
+        <v>8.92</v>
       </c>
       <c r="R344" t="n">
         <v>0</v>
       </c>
       <c r="S344" t="n">
-        <v>9.67</v>
+        <v>45.13</v>
       </c>
       <c r="T344" t="n">
-        <v>-1.53</v>
+        <v>-7.51</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>BSGR3</t>
+          <t>CLSC6</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Empresa BSGR</t>
+          <t>Empresa CLSC</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>Tradicional</t>
+          <t>Nível 2</t>
         </is>
       </c>
       <c r="E345" t="n">
-        <v>1091.28</v>
+        <v>0</v>
       </c>
       <c r="F345" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G345" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="H345" t="n">
-        <v>0</v>
+        <v>75.73</v>
       </c>
       <c r="I345" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="J345" t="n">
-        <v>0</v>
+        <v>2.73</v>
       </c>
       <c r="K345" t="n">
         <v>0</v>
@@ -25953,7 +25953,7 @@
         <v>0</v>
       </c>
       <c r="N345" t="n">
-        <v>0</v>
+        <v>4228180000</v>
       </c>
       <c r="O345" t="n">
         <v>0</v>
@@ -25971,18 +25971,18 @@
         <v>0</v>
       </c>
       <c r="T345" t="n">
-        <v>0</v>
+        <v>2.82</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>CBMA3</t>
+          <t>SGEN3</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Empresa CBMA</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
@@ -25996,7 +25996,7 @@
         </is>
       </c>
       <c r="E346" t="n">
-        <v>0.01</v>
+        <v>5</v>
       </c>
       <c r="F346" t="inlineStr">
         <is>
@@ -26021,47 +26021,47 @@
         <v>0</v>
       </c>
       <c r="L346" t="n">
-        <v>0</v>
+        <v>0.77</v>
       </c>
       <c r="M346" t="n">
         <v>0</v>
       </c>
       <c r="N346" t="n">
-        <v>-34022300000</v>
+        <v>156981000</v>
       </c>
       <c r="O346" t="n">
         <v>0</v>
       </c>
       <c r="P346" t="n">
-        <v>0</v>
+        <v>-1871.17</v>
       </c>
       <c r="Q346" t="n">
         <v>0</v>
       </c>
       <c r="R346" t="n">
-        <v>0</v>
+        <v>-1.59</v>
       </c>
       <c r="S346" t="n">
         <v>0</v>
       </c>
       <c r="T346" t="n">
-        <v>252.65</v>
+        <v>-59.85</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>ALBA3</t>
+          <t>DUFB11</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Empresa ALBA</t>
+          <t>Empresa DUFB</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>UNT</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
@@ -26070,7 +26070,7 @@
         </is>
       </c>
       <c r="E347" t="n">
-        <v>2.15</v>
+        <v>0</v>
       </c>
       <c r="F347" t="inlineStr">
         <is>
@@ -26101,36 +26101,36 @@
         <v>0</v>
       </c>
       <c r="N347" t="n">
-        <v>354860000</v>
+        <v>0</v>
       </c>
       <c r="O347" t="n">
         <v>0</v>
       </c>
       <c r="P347" t="n">
-        <v>9.5</v>
+        <v>0</v>
       </c>
       <c r="Q347" t="n">
-        <v>9.619999999999999</v>
+        <v>0</v>
       </c>
       <c r="R347" t="n">
-        <v>20.4</v>
+        <v>0</v>
       </c>
       <c r="S347" t="n">
-        <v>19.77</v>
+        <v>0</v>
       </c>
       <c r="T347" t="n">
-        <v>14.69</v>
+        <v>0</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>ARPS4</t>
+          <t>TNEP4</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Empresa ARPS</t>
+          <t>Empresa TNEP</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
@@ -26144,7 +26144,7 @@
         </is>
       </c>
       <c r="E348" t="n">
-        <v>0</v>
+        <v>3.95</v>
       </c>
       <c r="F348" t="inlineStr">
         <is>
@@ -26175,36 +26175,36 @@
         <v>0</v>
       </c>
       <c r="N348" t="n">
-        <v>-12690000</v>
+        <v>955105000</v>
       </c>
       <c r="O348" t="n">
         <v>0</v>
       </c>
       <c r="P348" t="n">
-        <v>-4.92</v>
+        <v>20.92</v>
       </c>
       <c r="Q348" t="n">
-        <v>-11.59</v>
+        <v>25.42</v>
       </c>
       <c r="R348" t="n">
-        <v>-6.64</v>
+        <v>20.53</v>
       </c>
       <c r="S348" t="n">
-        <v>20.34</v>
+        <v>22.8</v>
       </c>
       <c r="T348" t="n">
-        <v>-17.53</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>SALM3</t>
+          <t>CCHI3</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Empresa SALM</t>
+          <t>Empresa CCHI</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
@@ -26218,7 +26218,7 @@
         </is>
       </c>
       <c r="E349" t="n">
-        <v>5.7</v>
+        <v>0.02</v>
       </c>
       <c r="F349" t="inlineStr">
         <is>
@@ -26243,47 +26243,47 @@
         <v>0</v>
       </c>
       <c r="L349" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="M349" t="n">
         <v>0</v>
       </c>
       <c r="N349" t="n">
-        <v>475600000</v>
+        <v>-160477000</v>
       </c>
       <c r="O349" t="n">
         <v>0</v>
       </c>
       <c r="P349" t="n">
-        <v>10.22</v>
+        <v>0</v>
       </c>
       <c r="Q349" t="n">
-        <v>4.13</v>
+        <v>0</v>
       </c>
       <c r="R349" t="n">
-        <v>25.78</v>
+        <v>0</v>
       </c>
       <c r="S349" t="n">
-        <v>19.53</v>
+        <v>0</v>
       </c>
       <c r="T349" t="n">
-        <v>24.53</v>
+        <v>20.36</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>CMMA4</t>
+          <t>SFSA3</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Empresa CMMA</t>
+          <t>Empresa SFSA</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D350" t="inlineStr">
@@ -26292,7 +26292,7 @@
         </is>
       </c>
       <c r="E350" t="n">
-        <v>0.8100000000000001</v>
+        <v>0</v>
       </c>
       <c r="F350" t="inlineStr">
         <is>
@@ -26323,7 +26323,7 @@
         <v>0</v>
       </c>
       <c r="N350" t="n">
-        <v>-79623000</v>
+        <v>739524000</v>
       </c>
       <c r="O350" t="n">
         <v>0</v>
@@ -26338,26 +26338,26 @@
         <v>0</v>
       </c>
       <c r="S350" t="n">
-        <v>-1.92</v>
+        <v>6.25</v>
       </c>
       <c r="T350" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>CSPC4</t>
+          <t>PRBC3</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Empresa CSPC</t>
+          <t>Empresa PRBC</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D351" t="inlineStr">
@@ -26366,7 +26366,7 @@
         </is>
       </c>
       <c r="E351" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="F351" t="inlineStr">
         <is>
@@ -26397,36 +26397,36 @@
         <v>0</v>
       </c>
       <c r="N351" t="n">
-        <v>2126670000</v>
+        <v>1319270000</v>
       </c>
       <c r="O351" t="n">
         <v>0</v>
       </c>
       <c r="P351" t="n">
-        <v>38.62</v>
+        <v>0</v>
       </c>
       <c r="Q351" t="n">
-        <v>18.85</v>
+        <v>0</v>
       </c>
       <c r="R351" t="n">
-        <v>29.18</v>
+        <v>0</v>
       </c>
       <c r="S351" t="n">
-        <v>45.33</v>
+        <v>8.27</v>
       </c>
       <c r="T351" t="n">
-        <v>41.15</v>
+        <v>-1.98</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>BOVH3</t>
+          <t>ECIS3</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Empresa BOVH</t>
+          <t>Empresa ECIS</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -26440,7 +26440,7 @@
         </is>
       </c>
       <c r="E352" t="n">
-        <v>15.71</v>
+        <v>211.65</v>
       </c>
       <c r="F352" t="inlineStr">
         <is>
@@ -26465,42 +26465,42 @@
         <v>0</v>
       </c>
       <c r="L352" t="n">
-        <v>6.16</v>
+        <v>0</v>
       </c>
       <c r="M352" t="n">
         <v>0</v>
       </c>
       <c r="N352" t="n">
-        <v>1843320000</v>
+        <v>129346000</v>
       </c>
       <c r="O352" t="n">
         <v>0</v>
       </c>
       <c r="P352" t="n">
-        <v>0</v>
+        <v>34.9</v>
       </c>
       <c r="Q352" t="n">
-        <v>0</v>
+        <v>14.18</v>
       </c>
       <c r="R352" t="n">
-        <v>0</v>
+        <v>12.48</v>
       </c>
       <c r="S352" t="n">
-        <v>0</v>
+        <v>7.33</v>
       </c>
       <c r="T352" t="n">
-        <v>0</v>
+        <v>4.66</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>VNET3</t>
+          <t>CBMA3</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Empresa VNET</t>
+          <t>Empresa CBMA</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -26514,7 +26514,7 @@
         </is>
       </c>
       <c r="E353" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="F353" t="inlineStr">
         <is>
@@ -26545,7 +26545,7 @@
         <v>0</v>
       </c>
       <c r="N353" t="n">
-        <v>14163000000</v>
+        <v>-34022300000</v>
       </c>
       <c r="O353" t="n">
         <v>0</v>
@@ -26563,18 +26563,18 @@
         <v>0</v>
       </c>
       <c r="T353" t="n">
-        <v>1.08</v>
+        <v>252.65</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>ARND3</t>
+          <t>ALBA3</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Empresa ARND</t>
+          <t>Empresa ALBA</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -26584,22 +26584,22 @@
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>Novo Mercado</t>
+          <t>Tradicional</t>
         </is>
       </c>
       <c r="E354" t="n">
-        <v>0.51</v>
+        <v>2.15</v>
       </c>
       <c r="F354" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G354" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="H354" t="n">
-        <v>12.49</v>
+        <v>0</v>
       </c>
       <c r="I354" t="inlineStr">
         <is>
@@ -26613,47 +26613,47 @@
         <v>0</v>
       </c>
       <c r="L354" t="n">
-        <v>0.57</v>
+        <v>0</v>
       </c>
       <c r="M354" t="n">
         <v>0</v>
       </c>
       <c r="N354" t="n">
-        <v>125211000</v>
+        <v>354860000</v>
       </c>
       <c r="O354" t="n">
-        <v>913.58</v>
+        <v>0</v>
       </c>
       <c r="P354" t="n">
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="Q354" t="n">
-        <v>0</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="R354" t="n">
-        <v>0</v>
+        <v>20.4</v>
       </c>
       <c r="S354" t="n">
-        <v>0</v>
+        <v>19.77</v>
       </c>
       <c r="T354" t="n">
-        <v>-0.88</v>
+        <v>14.69</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>VVAX3</t>
+          <t>ARPS4</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Empresa VVAX</t>
+          <t>Empresa ARPS</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D355" t="inlineStr">
@@ -26693,41 +26693,41 @@
         <v>0</v>
       </c>
       <c r="N355" t="n">
-        <v>144676000</v>
+        <v>-12690000</v>
       </c>
       <c r="O355" t="n">
         <v>0</v>
       </c>
       <c r="P355" t="n">
-        <v>-7.36</v>
+        <v>-4.92</v>
       </c>
       <c r="Q355" t="n">
-        <v>-37.76</v>
+        <v>-11.59</v>
       </c>
       <c r="R355" t="n">
-        <v>-6.52</v>
+        <v>-6.64</v>
       </c>
       <c r="S355" t="n">
-        <v>-92.03</v>
+        <v>20.34</v>
       </c>
       <c r="T355" t="n">
-        <v>0</v>
+        <v>-17.53</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>MSAN4</t>
+          <t>SALM3</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Empresa MSAN</t>
+          <t>Empresa SALM</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D356" t="inlineStr">
@@ -26736,7 +26736,7 @@
         </is>
       </c>
       <c r="E356" t="n">
-        <v>6.44</v>
+        <v>5.7</v>
       </c>
       <c r="F356" t="inlineStr">
         <is>
@@ -26767,36 +26767,36 @@
         <v>0</v>
       </c>
       <c r="N356" t="n">
-        <v>2533030000</v>
+        <v>475600000</v>
       </c>
       <c r="O356" t="n">
         <v>0</v>
       </c>
       <c r="P356" t="n">
-        <v>6.27</v>
+        <v>10.22</v>
       </c>
       <c r="Q356" t="n">
-        <v>2.42</v>
+        <v>4.13</v>
       </c>
       <c r="R356" t="n">
-        <v>11.78</v>
+        <v>25.78</v>
       </c>
       <c r="S356" t="n">
-        <v>11.81</v>
+        <v>19.53</v>
       </c>
       <c r="T356" t="n">
-        <v>101.35</v>
+        <v>24.53</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>GALO4</t>
+          <t>CMMA4</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Empresa GALO</t>
+          <t>Empresa CMMA</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -26810,7 +26810,7 @@
         </is>
       </c>
       <c r="E357" t="n">
-        <v>0.25</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="F357" t="inlineStr">
         <is>
@@ -26841,36 +26841,36 @@
         <v>0</v>
       </c>
       <c r="N357" t="n">
-        <v>-60607000</v>
+        <v>-79623000</v>
       </c>
       <c r="O357" t="n">
         <v>0</v>
       </c>
       <c r="P357" t="n">
-        <v>13.98</v>
+        <v>0</v>
       </c>
       <c r="Q357" t="n">
-        <v>-184.58</v>
+        <v>0</v>
       </c>
       <c r="R357" t="n">
-        <v>39.37</v>
+        <v>0</v>
       </c>
       <c r="S357" t="n">
-        <v>7.62</v>
+        <v>-1.92</v>
       </c>
       <c r="T357" t="n">
-        <v>-28.97</v>
+        <v>0</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>BBTG13</t>
+          <t>CZRS3</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa CZRS</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -26915,7 +26915,7 @@
         <v>0</v>
       </c>
       <c r="N358" t="n">
-        <v>7000</v>
+        <v>1145670000</v>
       </c>
       <c r="O358" t="n">
         <v>0</v>
@@ -26930,21 +26930,21 @@
         <v>0</v>
       </c>
       <c r="S358" t="n">
-        <v>-42.86</v>
+        <v>3.34</v>
       </c>
       <c r="T358" t="n">
-        <v>0</v>
+        <v>14.44</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>INHA3</t>
+          <t>BPNM3</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Empresa INHA</t>
+          <t>Empresa BPNM</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
@@ -26989,41 +26989,41 @@
         <v>0</v>
       </c>
       <c r="N359" t="n">
-        <v>1533210000</v>
+        <v>7792670000</v>
       </c>
       <c r="O359" t="n">
         <v>0</v>
       </c>
       <c r="P359" t="n">
-        <v>-56.05</v>
+        <v>0</v>
       </c>
       <c r="Q359" t="n">
-        <v>-124.06</v>
+        <v>0</v>
       </c>
       <c r="R359" t="n">
-        <v>-6.27</v>
+        <v>0</v>
       </c>
       <c r="S359" t="n">
-        <v>-39.87</v>
+        <v>9.67</v>
       </c>
       <c r="T359" t="n">
-        <v>-12.18</v>
+        <v>-1.53</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>PTIP4</t>
+          <t>BSGR3</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Empresa PTIP</t>
+          <t>Empresa BSGR</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D360" t="inlineStr">
@@ -27032,7 +27032,7 @@
         </is>
       </c>
       <c r="E360" t="n">
-        <v>25.15</v>
+        <v>1091.28</v>
       </c>
       <c r="F360" t="inlineStr">
         <is>
@@ -27063,36 +27063,36 @@
         <v>0</v>
       </c>
       <c r="N360" t="n">
-        <v>-155957000</v>
+        <v>0</v>
       </c>
       <c r="O360" t="n">
         <v>0</v>
       </c>
       <c r="P360" t="n">
-        <v>13.73</v>
+        <v>0</v>
       </c>
       <c r="Q360" t="n">
-        <v>7.55</v>
+        <v>0</v>
       </c>
       <c r="R360" t="n">
-        <v>23.13</v>
+        <v>0</v>
       </c>
       <c r="S360" t="n">
-        <v>-121.74</v>
+        <v>0</v>
       </c>
       <c r="T360" t="n">
-        <v>62.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>LATS3</t>
+          <t>VNET3</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Empresa LATS</t>
+          <t>Empresa VNET</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -27106,7 +27106,7 @@
         </is>
       </c>
       <c r="E361" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="F361" t="inlineStr">
         <is>
@@ -27137,36 +27137,36 @@
         <v>0</v>
       </c>
       <c r="N361" t="n">
-        <v>680646000</v>
+        <v>14163000000</v>
       </c>
       <c r="O361" t="n">
         <v>0</v>
       </c>
       <c r="P361" t="n">
-        <v>11.74</v>
+        <v>0</v>
       </c>
       <c r="Q361" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="R361" t="n">
-        <v>11.63</v>
+        <v>0</v>
       </c>
       <c r="S361" t="n">
-        <v>1.84</v>
+        <v>0</v>
       </c>
       <c r="T361" t="n">
-        <v>15.37</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>SGEN4</t>
+          <t>CSPC4</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>Empresa SGEN</t>
+          <t>Empresa CSPC</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -27180,7 +27180,7 @@
         </is>
       </c>
       <c r="E362" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="F362" t="inlineStr">
         <is>
@@ -27205,42 +27205,42 @@
         <v>0</v>
       </c>
       <c r="L362" t="n">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="M362" t="n">
         <v>0</v>
       </c>
       <c r="N362" t="n">
-        <v>156981000</v>
+        <v>2126670000</v>
       </c>
       <c r="O362" t="n">
         <v>0</v>
       </c>
       <c r="P362" t="n">
-        <v>-1871.17</v>
+        <v>38.62</v>
       </c>
       <c r="Q362" t="n">
-        <v>0</v>
+        <v>18.85</v>
       </c>
       <c r="R362" t="n">
-        <v>-1.59</v>
+        <v>29.18</v>
       </c>
       <c r="S362" t="n">
-        <v>0</v>
+        <v>45.33</v>
       </c>
       <c r="T362" t="n">
-        <v>-59.85</v>
+        <v>41.15</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>VSPT3</t>
+          <t>BOVH3</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Empresa VSPT</t>
+          <t>Empresa BOVH</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -27254,11 +27254,11 @@
         </is>
       </c>
       <c r="E363" t="n">
-        <v>0</v>
+        <v>15.71</v>
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t>Bens Industriais</t>
+          <t>Outros Setores</t>
         </is>
       </c>
       <c r="G363" t="n">
@@ -27273,19 +27273,19 @@
         </is>
       </c>
       <c r="J363" t="n">
-        <v>-0.43</v>
+        <v>0</v>
       </c>
       <c r="K363" t="n">
         <v>0</v>
       </c>
       <c r="L363" t="n">
-        <v>0</v>
+        <v>6.16</v>
       </c>
       <c r="M363" t="n">
         <v>0</v>
       </c>
       <c r="N363" t="n">
-        <v>5031600000</v>
+        <v>1843320000</v>
       </c>
       <c r="O363" t="n">
         <v>0</v>
@@ -27303,18 +27303,18 @@
         <v>0</v>
       </c>
       <c r="T363" t="n">
-        <v>4.92</v>
+        <v>0</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>SEBB3</t>
+          <t>ARND3</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Empresa SEBB</t>
+          <t>Empresa ARND</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -27324,22 +27324,22 @@
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>Tradicional</t>
+          <t>Novo Mercado</t>
         </is>
       </c>
       <c r="E364" t="n">
-        <v>0</v>
+        <v>0.51</v>
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Tecnologia da Informação</t>
         </is>
       </c>
       <c r="G364" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="H364" t="n">
-        <v>0</v>
+        <v>12.49</v>
       </c>
       <c r="I364" t="inlineStr">
         <is>
@@ -27353,47 +27353,47 @@
         <v>0</v>
       </c>
       <c r="L364" t="n">
-        <v>0</v>
+        <v>0.57</v>
       </c>
       <c r="M364" t="n">
         <v>0</v>
       </c>
       <c r="N364" t="n">
-        <v>145783000</v>
+        <v>125211000</v>
       </c>
       <c r="O364" t="n">
-        <v>0</v>
+        <v>913.58</v>
       </c>
       <c r="P364" t="n">
-        <v>9.24</v>
+        <v>0</v>
       </c>
       <c r="Q364" t="n">
-        <v>7.4</v>
+        <v>0</v>
       </c>
       <c r="R364" t="n">
-        <v>24.15</v>
+        <v>0</v>
       </c>
       <c r="S364" t="n">
-        <v>23.01</v>
+        <v>0</v>
       </c>
       <c r="T364" t="n">
-        <v>50.04</v>
+        <v>-0.88</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>BBTG11</t>
+          <t>VVAX3</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Empresa BBTG</t>
+          <t>Empresa VVAX</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>UNT</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
@@ -27402,7 +27402,7 @@
         </is>
       </c>
       <c r="E365" t="n">
-        <v>15.01</v>
+        <v>0</v>
       </c>
       <c r="F365" t="inlineStr">
         <is>
@@ -27433,22 +27433,22 @@
         <v>0</v>
       </c>
       <c r="N365" t="n">
-        <v>0</v>
+        <v>144676000</v>
       </c>
       <c r="O365" t="n">
         <v>0</v>
       </c>
       <c r="P365" t="n">
-        <v>0</v>
+        <v>-7.36</v>
       </c>
       <c r="Q365" t="n">
-        <v>0</v>
+        <v>-37.76</v>
       </c>
       <c r="R365" t="n">
-        <v>0</v>
+        <v>-6.52</v>
       </c>
       <c r="S365" t="n">
-        <v>0</v>
+        <v>-92.03</v>
       </c>
       <c r="T365" t="n">
         <v>0</v>
@@ -27457,12 +27457,12 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>JFAB4</t>
+          <t>MSAN4</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Empresa JFAB</t>
+          <t>Empresa MSAN</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -27476,7 +27476,7 @@
         </is>
       </c>
       <c r="E366" t="n">
-        <v>0.06</v>
+        <v>6.44</v>
       </c>
       <c r="F366" t="inlineStr">
         <is>
@@ -27507,36 +27507,36 @@
         <v>0</v>
       </c>
       <c r="N366" t="n">
-        <v>-10183000</v>
+        <v>2533030000</v>
       </c>
       <c r="O366" t="n">
         <v>0</v>
       </c>
       <c r="P366" t="n">
-        <v>0</v>
+        <v>6.27</v>
       </c>
       <c r="Q366" t="n">
-        <v>0</v>
+        <v>2.42</v>
       </c>
       <c r="R366" t="n">
-        <v>0</v>
+        <v>11.78</v>
       </c>
       <c r="S366" t="n">
-        <v>2.34</v>
+        <v>11.81</v>
       </c>
       <c r="T366" t="n">
-        <v>0</v>
+        <v>101.35</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>CCHI4</t>
+          <t>GALO4</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Empresa CCHI</t>
+          <t>Empresa GALO</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -27550,7 +27550,7 @@
         </is>
       </c>
       <c r="E367" t="n">
-        <v>0.02</v>
+        <v>0.25</v>
       </c>
       <c r="F367" t="inlineStr">
         <is>
@@ -27575,42 +27575,42 @@
         <v>0</v>
       </c>
       <c r="L367" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="M367" t="n">
         <v>0</v>
       </c>
       <c r="N367" t="n">
-        <v>-160477000</v>
+        <v>-60607000</v>
       </c>
       <c r="O367" t="n">
         <v>0</v>
       </c>
       <c r="P367" t="n">
-        <v>0</v>
+        <v>13.98</v>
       </c>
       <c r="Q367" t="n">
-        <v>0</v>
+        <v>-184.58</v>
       </c>
       <c r="R367" t="n">
-        <v>0</v>
+        <v>39.37</v>
       </c>
       <c r="S367" t="n">
-        <v>0</v>
+        <v>7.62</v>
       </c>
       <c r="T367" t="n">
-        <v>20.36</v>
+        <v>-28.97</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>REPA3</t>
+          <t>BBTG13</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Empresa REPA</t>
+          <t>Empresa BBTG</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -27624,7 +27624,7 @@
         </is>
       </c>
       <c r="E368" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F368" t="inlineStr">
         <is>
@@ -27655,41 +27655,41 @@
         <v>0</v>
       </c>
       <c r="N368" t="n">
-        <v>378378000</v>
+        <v>7000</v>
       </c>
       <c r="O368" t="n">
         <v>0</v>
       </c>
       <c r="P368" t="n">
-        <v>5.18</v>
+        <v>0</v>
       </c>
       <c r="Q368" t="n">
-        <v>1.22</v>
+        <v>0</v>
       </c>
       <c r="R368" t="n">
-        <v>4.05</v>
+        <v>0</v>
       </c>
       <c r="S368" t="n">
-        <v>1.91</v>
+        <v>-42.86</v>
       </c>
       <c r="T368" t="n">
-        <v>1.09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>EQMA5B</t>
+          <t>INHA3</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Empresa EQMA</t>
+          <t>Empresa INHA</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D369" t="inlineStr">
@@ -27729,36 +27729,36 @@
         <v>0</v>
       </c>
       <c r="N369" t="n">
-        <v>4940330000</v>
+        <v>1533210000</v>
       </c>
       <c r="O369" t="n">
         <v>0</v>
       </c>
       <c r="P369" t="n">
-        <v>0</v>
+        <v>-56.05</v>
       </c>
       <c r="Q369" t="n">
-        <v>0</v>
+        <v>-124.06</v>
       </c>
       <c r="R369" t="n">
-        <v>0</v>
+        <v>-6.27</v>
       </c>
       <c r="S369" t="n">
-        <v>0</v>
+        <v>-39.87</v>
       </c>
       <c r="T369" t="n">
-        <v>9.050000000000001</v>
+        <v>-12.18</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>ECIS4</t>
+          <t>PTIP4</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Empresa ECIS</t>
+          <t>Empresa PTIP</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -27772,7 +27772,7 @@
         </is>
       </c>
       <c r="E370" t="n">
-        <v>145</v>
+        <v>25.15</v>
       </c>
       <c r="F370" t="inlineStr">
         <is>
@@ -27803,36 +27803,36 @@
         <v>0</v>
       </c>
       <c r="N370" t="n">
-        <v>129346000</v>
+        <v>-155957000</v>
       </c>
       <c r="O370" t="n">
         <v>0</v>
       </c>
       <c r="P370" t="n">
-        <v>34.9</v>
+        <v>13.73</v>
       </c>
       <c r="Q370" t="n">
-        <v>14.18</v>
+        <v>7.55</v>
       </c>
       <c r="R370" t="n">
-        <v>12.48</v>
+        <v>23.13</v>
       </c>
       <c r="S370" t="n">
-        <v>7.33</v>
+        <v>-121.74</v>
       </c>
       <c r="T370" t="n">
-        <v>4.66</v>
+        <v>62.11</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>TNEP3</t>
+          <t>LATS3</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Empresa TNEP</t>
+          <t>Empresa LATS</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
@@ -27846,7 +27846,7 @@
         </is>
       </c>
       <c r="E371" t="n">
-        <v>3.01</v>
+        <v>22</v>
       </c>
       <c r="F371" t="inlineStr">
         <is>
@@ -27877,36 +27877,36 @@
         <v>0</v>
       </c>
       <c r="N371" t="n">
-        <v>955105000</v>
+        <v>680646000</v>
       </c>
       <c r="O371" t="n">
         <v>0</v>
       </c>
       <c r="P371" t="n">
-        <v>20.92</v>
+        <v>11.74</v>
       </c>
       <c r="Q371" t="n">
-        <v>25.42</v>
+        <v>1.3</v>
       </c>
       <c r="R371" t="n">
-        <v>20.53</v>
+        <v>11.63</v>
       </c>
       <c r="S371" t="n">
-        <v>22.8</v>
+        <v>1.84</v>
       </c>
       <c r="T371" t="n">
-        <v>8.15</v>
+        <v>15.37</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>LECO3</t>
+          <t>VSPT3</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Empresa LECO</t>
+          <t>Empresa VSPT</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
@@ -27924,7 +27924,7 @@
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t>Outros Setores</t>
+          <t>Bens Industriais</t>
         </is>
       </c>
       <c r="G372" t="n">
@@ -27939,7 +27939,7 @@
         </is>
       </c>
       <c r="J372" t="n">
-        <v>0</v>
+        <v>-0.43</v>
       </c>
       <c r="K372" t="n">
         <v>0</v>
@@ -27951,41 +27951,41 @@
         <v>0</v>
       </c>
       <c r="N372" t="n">
-        <v>105928000</v>
+        <v>5031600000</v>
       </c>
       <c r="O372" t="n">
         <v>0</v>
       </c>
       <c r="P372" t="n">
-        <v>-2.14</v>
+        <v>0</v>
       </c>
       <c r="Q372" t="n">
-        <v>-4.72</v>
+        <v>0</v>
       </c>
       <c r="R372" t="n">
-        <v>-3.48</v>
+        <v>0</v>
       </c>
       <c r="S372" t="n">
-        <v>-14.82</v>
+        <v>0</v>
       </c>
       <c r="T372" t="n">
-        <v>3.58</v>
+        <v>4.92</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>VGOR3</t>
+          <t>SGEN4</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Empresa VGOR</t>
+          <t>Empresa SGEN</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D373" t="inlineStr">
@@ -27994,7 +27994,7 @@
         </is>
       </c>
       <c r="E373" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="F373" t="inlineStr">
         <is>
@@ -28019,31 +28019,31 @@
         <v>0</v>
       </c>
       <c r="L373" t="n">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="M373" t="n">
         <v>0</v>
       </c>
       <c r="N373" t="n">
-        <v>135178000</v>
+        <v>156981000</v>
       </c>
       <c r="O373" t="n">
         <v>0</v>
       </c>
       <c r="P373" t="n">
-        <v>4.5</v>
+        <v>-1871.17</v>
       </c>
       <c r="Q373" t="n">
-        <v>-4.59</v>
+        <v>0</v>
       </c>
       <c r="R373" t="n">
-        <v>6</v>
+        <v>-1.59</v>
       </c>
       <c r="S373" t="n">
-        <v>-24.29</v>
+        <v>0</v>
       </c>
       <c r="T373" t="n">
-        <v>4.77</v>
+        <v>-59.85</v>
       </c>
     </row>
     <row r="374">
@@ -41591,7 +41591,7 @@
     <row r="557">
       <c r="A557" t="inlineStr">
         <is>
-          <t>CIQU4</t>
+          <t>CIQU3</t>
         </is>
       </c>
       <c r="B557" t="inlineStr">
@@ -41601,7 +41601,7 @@
       </c>
       <c r="C557" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D557" t="inlineStr">
@@ -41665,7 +41665,7 @@
     <row r="558">
       <c r="A558" t="inlineStr">
         <is>
-          <t>CIQU3</t>
+          <t>CIQU4</t>
         </is>
       </c>
       <c r="B558" t="inlineStr">
@@ -41675,7 +41675,7 @@
       </c>
       <c r="C558" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D558" t="inlineStr">
@@ -42502,7 +42502,7 @@
       </c>
       <c r="F569" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G569" t="n">
@@ -44574,7 +44574,7 @@
       </c>
       <c r="F597" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G597" t="n">
@@ -45462,7 +45462,7 @@
       </c>
       <c r="F609" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G609" t="n">
@@ -45661,7 +45661,7 @@
     <row r="612">
       <c r="A612" t="inlineStr">
         <is>
-          <t>AESL4</t>
+          <t>AESL3</t>
         </is>
       </c>
       <c r="B612" t="inlineStr">
@@ -45671,7 +45671,7 @@
       </c>
       <c r="C612" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D612" t="inlineStr">
@@ -45735,7 +45735,7 @@
     <row r="613">
       <c r="A613" t="inlineStr">
         <is>
-          <t>AESL3</t>
+          <t>AESL4</t>
         </is>
       </c>
       <c r="B613" t="inlineStr">
@@ -45745,7 +45745,7 @@
       </c>
       <c r="C613" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="D613" t="inlineStr">
@@ -48570,7 +48570,7 @@
       </c>
       <c r="F651" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G651" t="n">
@@ -56710,7 +56710,7 @@
       </c>
       <c r="F761" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G761" t="n">
@@ -57154,7 +57154,7 @@
       </c>
       <c r="F767" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G767" t="n">
@@ -60188,7 +60188,7 @@
       </c>
       <c r="F808" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G808" t="n">
@@ -70252,7 +70252,7 @@
       </c>
       <c r="F944" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Seguradoras</t>
         </is>
       </c>
       <c r="G944" t="n">
@@ -71066,7 +71066,7 @@
       </c>
       <c r="F955" t="inlineStr">
         <is>
-          <t>Utilidade Pública</t>
+          <t>Energia Elétrica</t>
         </is>
       </c>
       <c r="G955" t="n">
@@ -71510,7 +71510,7 @@
       </c>
       <c r="F961" t="inlineStr">
         <is>
-          <t>Financeiro e Outros</t>
+          <t>Seguradoras</t>
         </is>
       </c>
       <c r="G961" t="n">

</xml_diff>